<commit_message>
Update funding data 2026-03-01
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Recursos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$99</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$93</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$94</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -679,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M99"/>
+  <dimension ref="A1:M100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -707,7 +707,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 28/02/2026 07:09 - 92 convocatorias - 24 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 01/03/2026 07:52 - 93 convocatorias - 24 nuevas</t>
         </is>
       </c>
     </row>
@@ -1627,12 +1627,12 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-07-D1-01</t>
+          <t>HORIZON-CL5-2026-08-Two-Stage-D1-06</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Next generation climate monitoring and related capabilities</t>
+          <t>Closing knowledge gaps on Earth system science in support of global and regional assessments and climate policy</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -1652,7 +1652,7 @@
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>4,000,000</t>
+          <t>5,000,000 - 9,000,000</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -1672,7 +1672,7 @@
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Climate data are improved both spatially and temporally, physically more consistent and better exp</t>
+          <t>Expected Outcome:Project results are expected to contribute to some of the following expected outcomes:Improved quality and reduced uncertainty of global and regional climate change projections;Critic</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr"/>
@@ -1690,12 +1690,12 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-08-Two-Stage-D1-06</t>
+          <t>HORIZON-CL5-2026-07-D1-01</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Closing knowledge gaps on Earth system science in support of global and regional assessments and climate policy</t>
+          <t>Next generation climate monitoring and related capabilities</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>5,000,000 - 9,000,000</t>
+          <t>4,000,000</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="K21" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to some of the following expected outcomes:Improved quality and reduced uncertainty of global and regional climate change projections;Critic</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Climate data are improved both spatially and temporally, physically more consistent and better exp</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr"/>
@@ -1753,12 +1753,12 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-07-D1-04</t>
+          <t>HORIZON-CL5-2026-07-D1-05</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Fighting disinformation and effectively communicating on climate change</t>
+          <t>Improving climate and weather models for Africa</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Advanced knowledge and understanding on the dynamics of disinformation affecting climate policy an</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved quality and performance of weather and climate models over Africa, tailored to the contin</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr"/>
@@ -1816,12 +1816,12 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-07-D1-05</t>
+          <t>HORIZON-CL5-2026-07-D1-04</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Improving climate and weather models for Africa</t>
+          <t>Fighting disinformation and effectively communicating on climate change</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="K23" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved quality and performance of weather and climate models over Africa, tailored to the contin</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Advanced knowledge and understanding on the dynamics of disinformation affecting climate policy an</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr"/>
@@ -2686,12 +2686,12 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-13</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Next generation scenarios for informing climate and sustainability transitions</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="K37" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to some of the following expected outcomes:Strengthened collaboration and integration across research communities, better capturing interact</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorpo</t>
         </is>
       </c>
       <c r="L37" s="6" t="inlineStr"/>
@@ -2749,12 +2749,12 @@
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -2779,7 +2779,7 @@
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>Programme Cofund Actions</t>
+          <t xml:space="preserve"> Research and Innovation Actions</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="K38" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is estab</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Euro</t>
         </is>
       </c>
       <c r="L38" s="6" t="inlineStr"/>
@@ -2812,12 +2812,12 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -2857,7 +2857,7 @@
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorpo</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to info</t>
         </is>
       </c>
       <c r="L39" s="6" t="inlineStr"/>
@@ -2875,12 +2875,12 @@
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-13</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
+          <t>Next generation scenarios for informing climate and sustainability transitions</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -2920,7 +2920,7 @@
       </c>
       <c r="K40" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Euro</t>
+          <t>Expected Outcome:Project results are expected to contribute to some of the following expected outcomes:Strengthened collaboration and integration across research communities, better capturing interact</t>
         </is>
       </c>
       <c r="L40" s="6" t="inlineStr"/>
@@ -2938,12 +2938,12 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -2968,7 +2968,7 @@
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Research and Innovation Actions</t>
+          <t>Programme Cofund Actions</t>
         </is>
       </c>
       <c r="I41" s="11" t="inlineStr">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="K41" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to info</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is estab</t>
         </is>
       </c>
       <c r="L41" s="6" t="inlineStr"/>
@@ -4565,7 +4565,7 @@
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>dc0033a0-cb94-44ed-8102-0fd0a386989e-EXA</t>
+          <t>4b45d249-5739-4bf7-9595-a4715b73c2f6-EXA</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -4612,7 +4612,7 @@
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>4b45d249-5739-4bf7-9595-a4715b73c2f6-EXA</t>
+          <t>dc0033a0-cb94-44ed-8102-0fd0a386989e-EXA</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -4779,12 +4779,12 @@
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>EUS-74373</t>
+          <t>EUS-74952</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a proyectos al amparo de la estrategia de desarrollo local participativo (EDLP), aprobada al grupo de acción local del sector pesquero (GALP) para el desarrollo sostenible de las zonas de pesca</t>
+          <t>Servicio de transporte y reparto de comida desde las cocinas de elaboración a domicilios del municipio de Vitoria-Gasteiz y comedores del Departamento de Políticas Sociales</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr">
@@ -4801,12 +4801,12 @@
       <c r="G76" s="6" t="inlineStr"/>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
-        </is>
-      </c>
-      <c r="I76" s="8" t="inlineStr">
-        <is>
-          <t>ALTA</t>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I76" s="12" t="inlineStr">
+        <is>
+          <t>MUY ALTA</t>
         </is>
       </c>
       <c r="J76" s="6" t="inlineStr"/>
@@ -4834,12 +4834,12 @@
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>EUS-13151</t>
+          <t>EUS-31018</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>ReSourceEU y materias primas críticas: la UE sigue tramitando convocatorias para favorecer proyectos otorgándoles carácter estratégico, de la mano del Banco Europeo de Inversiones, de cara a ámbitos c</t>
+          <t>Ayudas a proyectos al amparo de la estrategia de desarrollo local participativo (EDLP), aprobada al grupo de acción local del sector pesquero (GALP) para el desarrollo sostenible de las zonas de pesca</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
@@ -4889,12 +4889,12 @@
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>EUS-33319</t>
+          <t>EUS-53900</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>Ciudades sostenibles: los Premios Capital Verde Europea y Hoja Verde de 2028 abren su convocatoria hasta el 01.04.26 para ciudades de más de 100.000 y de más de 20.000 habitantes, climáticamente resil</t>
+          <t>ReSourceEU y materias primas críticas: la UE sigue tramitando convocatorias para favorecer proyectos otorgándoles carácter estratégico, de la mano del Banco Europeo de Inversiones, de cara a ámbitos c</t>
         </is>
       </c>
       <c r="D78" s="6" t="inlineStr">
@@ -4944,12 +4944,12 @@
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>EUS-06487</t>
+          <t>EUS-66315</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>Presolicitud para programa de ayudas a empresas que realicen inversiones productivas que permitan diversificar líneas de negocio, productos, servicios y mercados, con un enfoque en el crecimiento sost</t>
+          <t>Ciudades sostenibles: los Premios Capital Verde Europea y Hoja Verde de 2028 abren su convocatoria hasta el 01.04.26 para ciudades de más de 100.000 y de más de 20.000 habitantes, climáticamente resil</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
@@ -4999,12 +4999,12 @@
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>EUS-05566</t>
+          <t>EUS-81441</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de aceleración de proyectos, a localidades de menos de 20.000 habitantes son objeto de convocatoria abierta hasta el 17.03.26. Transformacione</t>
+          <t>Presolicitud para programa de ayudas a empresas que realicen inversiones productivas que permitan diversificar líneas de negocio, productos, servicios y mercados, con un enfoque en el crecimiento sost</t>
         </is>
       </c>
       <c r="D80" s="6" t="inlineStr">
@@ -5024,9 +5024,9 @@
           <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
-      <c r="I80" s="10" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
+      <c r="I80" s="8" t="inlineStr">
+        <is>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="J80" s="6" t="inlineStr"/>
@@ -5054,12 +5054,12 @@
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>EUS-49036</t>
+          <t>EUS-88586</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinancia convocatorias de ayudas de las Diputaciones a explotaciones con limitaciones o desfavorecidas, y a compromisos medioambientales, climátic</t>
+          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de aceleración de proyectos, a localidades de menos de 20.000 habitantes son objeto de convocatoria abierta hasta el 17.03.26. Transformacione</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
@@ -5109,12 +5109,12 @@
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>EUS-84033</t>
+          <t>EUS-91314</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>Digital Europe, Horizon (programas de la UE). Apoyos para consorcios interestatales de I+D+i. IA, robótica, cuántica, computación, ciberseguridad, electrónica, fotónica, TICs e internet avanzadas, esp</t>
+          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinancia convocatorias de ayudas de las Diputaciones a explotaciones con limitaciones o desfavorecidas, y a compromisos medioambientales, climátic</t>
         </is>
       </c>
       <c r="D82" s="6" t="inlineStr">
@@ -5164,12 +5164,12 @@
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>EUS-55512</t>
+          <t>EUS-84020</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para consorcios internacionales de I+D+i. Jornada del Gobierno Vasco y con Enterprise Europe Network y otros socios. Digitalización, dispositivos,</t>
+          <t>Digital Europe, Horizon (programas de la UE). Apoyos para consorcios interestatales de I+D+i. IA, robótica, cuántica, computación, ciberseguridad, electrónica, fotónica, TICs e internet avanzadas, esp</t>
         </is>
       </c>
       <c r="D83" s="6" t="inlineStr">
@@ -5219,12 +5219,12 @@
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>EUS-90444</t>
+          <t>EUS-18785</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>Política Agraria Común de la UE de 2026, y sus ayudas abiertas hasta el 30.4.26: el pilar 1, con el Fondo Europeo Agrícola de Garantía Agraria FEAGA, aborda sostenibilidad de renta, ayuda redistributi</t>
+          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para consorcios internacionales de I+D+i. Jornada del Gobierno Vasco y con Enterprise Europe Network y otros socios. Digitalización, dispositivos,</t>
         </is>
       </c>
       <c r="D84" s="6" t="inlineStr">
@@ -5274,12 +5274,12 @@
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>EUS-25327</t>
+          <t>EUS-44870</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>Programa de impulso a las ciudades y territorios inteligentes para el fomento del desarrollo económico y productivo, que podrá ser cofinanciado por el Programa Plurirregional 2021-2027 del Fondo Europ</t>
+          <t>Política Agraria Común de la UE de 2026, y sus ayudas abiertas hasta el 30.4.26: el pilar 1, con el Fondo Europeo Agrícola de Garantía Agraria FEAGA, aborda sostenibilidad de renta, ayuda redistributi</t>
         </is>
       </c>
       <c r="D85" s="6" t="inlineStr">
@@ -5329,12 +5329,12 @@
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>EUS-73767</t>
+          <t>EUS-29143</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>Formación digital para empleabilidad turística: los fondos Next de la UE apoyan una convocatoria de Lanbide y el Gobierno Vasco, de cursos en línea para mejorar las competencias del sector y de sus py</t>
+          <t>Programa de impulso a las ciudades y territorios inteligentes para el fomento del desarrollo económico y productivo, que podrá ser cofinanciado por el Programa Plurirregional 2021-2027 del Fondo Europ</t>
         </is>
       </c>
       <c r="D86" s="6" t="inlineStr">
@@ -5384,12 +5384,12 @@
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>EUS-54415</t>
+          <t>EUS-05166</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Horizon Europe. Clúster digital, industrial y espacial. Apoyos a proyectos para tecnologías de inteligencia artificial, internet, mundos virtuales, robótica, cuántica, fotónica, materias primas, bajo </t>
+          <t>Formación digital para empleabilidad turística: los fondos Next de la UE apoyan una convocatoria de Lanbide y el Gobierno Vasco, de cursos en línea para mejorar las competencias del sector y de sus py</t>
         </is>
       </c>
       <c r="D87" s="6" t="inlineStr">
@@ -5439,12 +5439,12 @@
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>EUS-27582</t>
+          <t>EUS-07020</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>Horizon Europe: ayudas de la línea de energía del clúster 5 y de la Misión Ciudades. Jornada informativa sobre estas y otras iniciativas en colaboración transestatal para la doble transición ecológica</t>
+          <t xml:space="preserve">Horizon Europe. Clúster digital, industrial y espacial. Apoyos a proyectos para tecnologías de inteligencia artificial, internet, mundos virtuales, robótica, cuántica, fotónica, materias primas, bajo </t>
         </is>
       </c>
       <c r="D88" s="6" t="inlineStr">
@@ -5494,12 +5494,12 @@
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>EUS-96937</t>
+          <t>EUS-58974</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>Azpitek 2026: Programa de Ayudas para la Adquisición, Instalación, Renovación y Actualización de Infraestructuras de Investigación</t>
+          <t>Horizon Europe: ayudas de la línea de energía del clúster 5 y de la Misión Ciudades. Jornada informativa sobre estas y otras iniciativas en colaboración transestatal para la doble transición ecológica</t>
         </is>
       </c>
       <c r="D89" s="6" t="inlineStr">
@@ -5549,12 +5549,12 @@
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>EUS-68824</t>
+          <t>EUS-81341</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>Subvenciones para innovación en economía circular 2026</t>
+          <t>Azpitek 2026: Programa de Ayudas para la Adquisición, Instalación, Renovación y Actualización de Infraestructuras de Investigación</t>
         </is>
       </c>
       <c r="D90" s="6" t="inlineStr">
@@ -5604,12 +5604,12 @@
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>EUS-21415</t>
+          <t>EUS-61815</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>Horizon Europe 2026-27: convocatorias ligadas a misiones ambientales de la UE, partenariados de economía circular, azul o bio, o a la división alimentaria EIT Food del Instituto Europeo de Tecnología,</t>
+          <t>Subvenciones para innovación en economía circular 2026</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr">
@@ -5659,12 +5659,12 @@
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>EUS-12091</t>
+          <t>EUS-61141</t>
         </is>
       </c>
       <c r="C92" s="6" t="inlineStr">
         <is>
-          <t>Escudo Europeo de la Democracia: ayudas a proyectos de alfabetización mediática y fomento del diálogo y la comprensión en torno a la desinformación digital</t>
+          <t>Horizon Europe 2026-27: convocatorias ligadas a misiones ambientales de la UE, partenariados de economía circular, azul o bio, o a la división alimentaria EIT Food del Instituto Europeo de Tecnología,</t>
         </is>
       </c>
       <c r="D92" s="6" t="inlineStr">
@@ -5714,12 +5714,12 @@
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>EUS-29046</t>
+          <t>EUS-33047</t>
         </is>
       </c>
       <c r="C93" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">KSI Berritzaile Plus: ayudas del Gobierno Vasco a las Industrias Culturales y Creativas para proyectos innovadores en la triple transición tecnológico-digital, energético-climática y socio-sanitaria, </t>
+          <t>Escudo Europeo de la Democracia: ayudas a proyectos de alfabetización mediática y fomento del diálogo y la comprensión en torno a la desinformación digital</t>
         </is>
       </c>
       <c r="D93" s="6" t="inlineStr">
@@ -5769,12 +5769,12 @@
       </c>
       <c r="B94" s="6" t="inlineStr">
         <is>
-          <t>EUS-78377</t>
+          <t>EUS-49824</t>
         </is>
       </c>
       <c r="C94" s="6" t="inlineStr">
         <is>
-          <t>Desmontaje de dos depósitos de agua en local del polideportivo ipurua y tuberías que lo alimentan.</t>
+          <t xml:space="preserve">KSI Berritzaile Plus: ayudas del Gobierno Vasco a las Industrias Culturales y Creativas para proyectos innovadores en la triple transición tecnológico-digital, energético-climática y socio-sanitaria, </t>
         </is>
       </c>
       <c r="D94" s="6" t="inlineStr">
@@ -5791,7 +5791,7 @@
       <c r="G94" s="6" t="inlineStr"/>
       <c r="H94" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="I94" s="10" t="inlineStr">
@@ -5824,12 +5824,12 @@
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>EUS-16975</t>
+          <t>EUS-83207</t>
         </is>
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>Reparación del ascensor exterior de urki polonia tras entrada agua en cuadro</t>
+          <t>Desmontaje de dos depósitos de agua en local del polideportivo ipurua y tuberías que lo alimentan.</t>
         </is>
       </c>
       <c r="D95" s="6" t="inlineStr">
@@ -5879,12 +5879,12 @@
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>EUS-54763</t>
+          <t>EUS-43218</t>
         </is>
       </c>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>Desatasco tanto de la red de pluviales como de la de fecales de errebal plazia</t>
+          <t>Reparación del ascensor exterior de urki polonia tras entrada agua en cuadro</t>
         </is>
       </c>
       <c r="D96" s="6" t="inlineStr">
@@ -5934,12 +5934,12 @@
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>EUS-00010</t>
+          <t>EUS-03214</t>
         </is>
       </c>
       <c r="C97" s="6" t="inlineStr">
         <is>
-          <t>Contratación de la actuación de unos bertsolaris el 8 y 14 de septiembre en el marco de las fiestas de ntra. sra. de arrate</t>
+          <t>Desatasco tanto de la red de pluviales como de la de fecales de errebal plazia</t>
         </is>
       </c>
       <c r="D97" s="6" t="inlineStr">
@@ -5989,12 +5989,12 @@
       </c>
       <c r="B98" s="6" t="inlineStr">
         <is>
-          <t>EUS-50530</t>
+          <t>EUS-68824</t>
         </is>
       </c>
       <c r="C98" s="6" t="inlineStr">
         <is>
-          <t>Suministro de botellines de agua mineral para atender a los grupos que actúan en el teatro coliseo</t>
+          <t>Contratación de la actuación de unos bertsolaris el 8 y 14 de septiembre en el marco de las fiestas de ntra. sra. de arrate</t>
         </is>
       </c>
       <c r="D98" s="6" t="inlineStr">
@@ -6025,11 +6025,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L98" s="17" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
+      <c r="L98" s="6" t="inlineStr"/>
       <c r="M98" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
@@ -6044,12 +6040,12 @@
       </c>
       <c r="B99" s="6" t="inlineStr">
         <is>
-          <t>EUS-28619</t>
+          <t>EUS-26937</t>
         </is>
       </c>
       <c r="C99" s="6" t="inlineStr">
         <is>
-          <t>Servicio de organización de la sesión de bertsolaris de arrate del 7 de septiembre.</t>
+          <t>Suministro de botellines de agua mineral para atender a los grupos que actúan en el teatro coliseo</t>
         </is>
       </c>
       <c r="D99" s="6" t="inlineStr">
@@ -6091,8 +6087,63 @@
         </is>
       </c>
     </row>
+    <row r="100" ht="40" customHeight="1">
+      <c r="A100" s="16" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B100" s="6" t="inlineStr">
+        <is>
+          <t>EUS-27498</t>
+        </is>
+      </c>
+      <c r="C100" s="6" t="inlineStr">
+        <is>
+          <t>Servicio de organización de la sesión de bertsolaris de arrate del 7 de septiembre.</t>
+        </is>
+      </c>
+      <c r="D100" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E100" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F100" s="6" t="inlineStr"/>
+      <c r="G100" s="6" t="inlineStr"/>
+      <c r="H100" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I100" s="10" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J100" s="6" t="inlineStr"/>
+      <c r="K100" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L100" s="17" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M100" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:M99"/>
+  <autoFilter ref="A4:M100"/>
   <mergeCells count="5">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A75:M75"/>
@@ -6193,6 +6244,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M97" r:id="rId90"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M98" r:id="rId91"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M99" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M100" r:id="rId93"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6204,7 +6256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1379"/>
+  <dimension ref="A1:F1394"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -9266,7 +9318,7 @@
     <row r="211" ht="30" customHeight="1">
       <c r="A211" s="18" t="inlineStr">
         <is>
-          <t>FICHA 15: HORIZON-CL5-2026-07-D1-01</t>
+          <t>FICHA 15: HORIZON-CL5-2026-08-Two-Stage-D1-06</t>
         </is>
       </c>
       <c r="B211" s="19" t="n"/>
@@ -9291,7 +9343,7 @@
       <c r="E212" s="22" t="n"/>
       <c r="F212" s="22" t="n"/>
     </row>
-    <row r="213" ht="20" customHeight="1">
+    <row r="213" ht="45" customHeight="1">
       <c r="A213" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -9299,7 +9351,7 @@
       </c>
       <c r="B213" s="21" t="inlineStr">
         <is>
-          <t>Next generation climate monitoring and related capabilities</t>
+          <t>Closing knowledge gaps on Earth system science in support of global and regional assessments and climate policy</t>
         </is>
       </c>
       <c r="C213" s="22" t="n"/>
@@ -9315,7 +9367,7 @@
       </c>
       <c r="B214" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-07-D1-01</t>
+          <t>HORIZON-CL5-2026-08-Two-Stage-D1-06</t>
         </is>
       </c>
       <c r="C214" s="22" t="n"/>
@@ -9379,7 +9431,7 @@
       </c>
       <c r="B218" s="21" t="inlineStr">
         <is>
-          <t>4,000,000</t>
+          <t>5,000,000 - 9,000,000</t>
         </is>
       </c>
       <c r="C218" s="22" t="n"/>
@@ -9411,7 +9463,7 @@
       </c>
       <c r="B220" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-07</t>
+          <t>HORIZON-CL5-2026-08-Two-Stage</t>
         </is>
       </c>
       <c r="C220" s="22" t="n"/>
@@ -9427,7 +9479,7 @@
       </c>
       <c r="B221" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Climate data are improved both spatially and temporally, physically more consistent and better exploited across a wide range of users, stakeholders and regions;The EU climate data sovereignty is strengthened, with enhanced EU contribution to climate monitoring and climate change assessments;Climate information distillation is facilitated by innovative methods to provide useful information to policy making in a more efficient way. Scope:Climate monitoring of Essential Climate Variables[1] at gl</t>
+          <t>Expected Outcome:Project results are expected to contribute to some of the following expected outcomes:Improved quality and reduced uncertainty of global and regional climate change projections;Critical knowledge and data gaps in Earth system science as identified in the IPCC Sixth Assessment Report (AR6) and other authoritative sources, are addressed, ensuring that future climate assessments are grounded in the most comprehensive and up-to-date scientific evidence;New climate science evidence is generated that is relevant for policy needs and for informing climate action. Scope:The global com</t>
         </is>
       </c>
       <c r="C221" s="22" t="n"/>
@@ -9471,7 +9523,7 @@
       </c>
       <c r="B224" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-07-D1-01</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-08-Two-Stage-D1-06</t>
         </is>
       </c>
       <c r="C224" s="22" t="n"/>
@@ -9482,7 +9534,7 @@
     <row r="226" ht="30" customHeight="1">
       <c r="A226" s="18" t="inlineStr">
         <is>
-          <t>FICHA 16: HORIZON-CL5-2026-08-Two-Stage-D1-06</t>
+          <t>FICHA 16: HORIZON-CL5-2026-07-D1-01</t>
         </is>
       </c>
       <c r="B226" s="19" t="n"/>
@@ -9507,7 +9559,7 @@
       <c r="E227" s="22" t="n"/>
       <c r="F227" s="22" t="n"/>
     </row>
-    <row r="228" ht="45" customHeight="1">
+    <row r="228" ht="20" customHeight="1">
       <c r="A228" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -9515,7 +9567,7 @@
       </c>
       <c r="B228" s="21" t="inlineStr">
         <is>
-          <t>Closing knowledge gaps on Earth system science in support of global and regional assessments and climate policy</t>
+          <t>Next generation climate monitoring and related capabilities</t>
         </is>
       </c>
       <c r="C228" s="22" t="n"/>
@@ -9531,7 +9583,7 @@
       </c>
       <c r="B229" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-08-Two-Stage-D1-06</t>
+          <t>HORIZON-CL5-2026-07-D1-01</t>
         </is>
       </c>
       <c r="C229" s="22" t="n"/>
@@ -9595,7 +9647,7 @@
       </c>
       <c r="B233" s="21" t="inlineStr">
         <is>
-          <t>5,000,000 - 9,000,000</t>
+          <t>4,000,000</t>
         </is>
       </c>
       <c r="C233" s="22" t="n"/>
@@ -9627,7 +9679,7 @@
       </c>
       <c r="B235" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-08-Two-Stage</t>
+          <t>HORIZON-CL5-2026-07</t>
         </is>
       </c>
       <c r="C235" s="22" t="n"/>
@@ -9643,7 +9695,7 @@
       </c>
       <c r="B236" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to some of the following expected outcomes:Improved quality and reduced uncertainty of global and regional climate change projections;Critical knowledge and data gaps in Earth system science as identified in the IPCC Sixth Assessment Report (AR6) and other authoritative sources, are addressed, ensuring that future climate assessments are grounded in the most comprehensive and up-to-date scientific evidence;New climate science evidence is generated that is relevant for policy needs and for informing climate action. Scope:The global com</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Climate data are improved both spatially and temporally, physically more consistent and better exploited across a wide range of users, stakeholders and regions;The EU climate data sovereignty is strengthened, with enhanced EU contribution to climate monitoring and climate change assessments;Climate information distillation is facilitated by innovative methods to provide useful information to policy making in a more efficient way. Scope:Climate monitoring of Essential Climate Variables[1] at gl</t>
         </is>
       </c>
       <c r="C236" s="22" t="n"/>
@@ -9687,7 +9739,7 @@
       </c>
       <c r="B239" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-08-Two-Stage-D1-06</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-07-D1-01</t>
         </is>
       </c>
       <c r="C239" s="22" t="n"/>
@@ -9698,7 +9750,7 @@
     <row r="241" ht="30" customHeight="1">
       <c r="A241" s="18" t="inlineStr">
         <is>
-          <t>FICHA 17: HORIZON-CL5-2026-07-D1-04</t>
+          <t>FICHA 17: HORIZON-CL5-2026-07-D1-05</t>
         </is>
       </c>
       <c r="B241" s="19" t="n"/>
@@ -9731,7 +9783,7 @@
       </c>
       <c r="B243" s="21" t="inlineStr">
         <is>
-          <t>Fighting disinformation and effectively communicating on climate change</t>
+          <t>Improving climate and weather models for Africa</t>
         </is>
       </c>
       <c r="C243" s="22" t="n"/>
@@ -9747,7 +9799,7 @@
       </c>
       <c r="B244" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-07-D1-04</t>
+          <t>HORIZON-CL5-2026-07-D1-05</t>
         </is>
       </c>
       <c r="C244" s="22" t="n"/>
@@ -9859,7 +9911,7 @@
       </c>
       <c r="B251" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Advanced knowledge and understanding on the dynamics of disinformation affecting climate policy and climate policy backlash from a communication perspective;Tools and products are developed for public authorities, media and civil society to detect and combat the influence and spread of climate change-related disinformation at scale;Tailored, innovative and effective communication techniques, tools and materials are developed, tested and disseminated, to better communicate with and engage citiz</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved quality and performance of weather and climate models over Africa, tailored to the continent’s needs, enabling more effective adaptation actions and disaster risk response strategies, and informing the implementation of the international dimension of the EU Adaptation and Preparedness Union Strategies, the Sendai Framework for Disaster Risk Reduction, the Nairobi Declaration and the Team Europe Initiative on Adaptation and Resilience in Africa[1];Enhanced provision of weather predicti</t>
         </is>
       </c>
       <c r="C251" s="22" t="n"/>
@@ -9903,7 +9955,7 @@
       </c>
       <c r="B254" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-07-D1-04</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-07-D1-05</t>
         </is>
       </c>
       <c r="C254" s="22" t="n"/>
@@ -9914,7 +9966,7 @@
     <row r="256" ht="30" customHeight="1">
       <c r="A256" s="18" t="inlineStr">
         <is>
-          <t>FICHA 18: HORIZON-CL5-2026-07-D1-05</t>
+          <t>FICHA 18: HORIZON-CL5-2026-07-D1-04</t>
         </is>
       </c>
       <c r="B256" s="19" t="n"/>
@@ -9947,7 +9999,7 @@
       </c>
       <c r="B258" s="21" t="inlineStr">
         <is>
-          <t>Improving climate and weather models for Africa</t>
+          <t>Fighting disinformation and effectively communicating on climate change</t>
         </is>
       </c>
       <c r="C258" s="22" t="n"/>
@@ -9963,7 +10015,7 @@
       </c>
       <c r="B259" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-07-D1-05</t>
+          <t>HORIZON-CL5-2026-07-D1-04</t>
         </is>
       </c>
       <c r="C259" s="22" t="n"/>
@@ -10075,7 +10127,7 @@
       </c>
       <c r="B266" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved quality and performance of weather and climate models over Africa, tailored to the continent’s needs, enabling more effective adaptation actions and disaster risk response strategies, and informing the implementation of the international dimension of the EU Adaptation and Preparedness Union Strategies, the Sendai Framework for Disaster Risk Reduction, the Nairobi Declaration and the Team Europe Initiative on Adaptation and Resilience in Africa[1];Enhanced provision of weather predicti</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Advanced knowledge and understanding on the dynamics of disinformation affecting climate policy and climate policy backlash from a communication perspective;Tools and products are developed for public authorities, media and civil society to detect and combat the influence and spread of climate change-related disinformation at scale;Tailored, innovative and effective communication techniques, tools and materials are developed, tested and disseminated, to better communicate with and engage citiz</t>
         </is>
       </c>
       <c r="C266" s="22" t="n"/>
@@ -10119,7 +10171,7 @@
       </c>
       <c r="B269" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-07-D1-05</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-07-D1-04</t>
         </is>
       </c>
       <c r="C269" s="22" t="n"/>
@@ -12970,7 +13022,7 @@
     <row r="466" ht="30" customHeight="1">
       <c r="A466" s="18" t="inlineStr">
         <is>
-          <t>FICHA 32: HORIZON-CL5-2027-01-D1-13</t>
+          <t>FICHA 32: HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="B466" s="19" t="n"/>
@@ -13003,7 +13055,7 @@
       </c>
       <c r="B468" s="21" t="inlineStr">
         <is>
-          <t>Next generation scenarios for informing climate and sustainability transitions</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="C468" s="22" t="n"/>
@@ -13019,7 +13071,7 @@
       </c>
       <c r="B469" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-13</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C469" s="22" t="n"/>
@@ -13131,7 +13183,7 @@
       </c>
       <c r="B476" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to some of the following expected outcomes:Strengthened collaboration and integration across research communities, better capturing interactions and trade-offs between various climate domains as well as between climate and non-climate objectives, such as biodiversity or pollution related. This will support more comprehensive and consistent evaluations, benefiting key global assessments (IPCC, IPBES) and improving their impact on European and global policies (European Green Deal, UNFCCC, CBD);More relevant, robust and actionable scenar</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorporation into main EU repositories, such as Climate-ADAPT or the portal of the EU Mission on Adaptation to Climate Change;The risk and adaptation assessment frameworks are improved by better integrating the maladaptation dimension;Guidelines and tools for maladaptation prevention and correction strategies are made available to adaptation stakeholders at relevant scales and inform the design and impl</t>
         </is>
       </c>
       <c r="C476" s="22" t="n"/>
@@ -13175,7 +13227,7 @@
       </c>
       <c r="B479" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-13</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C479" s="22" t="n"/>
@@ -13186,7 +13238,7 @@
     <row r="481" ht="30" customHeight="1">
       <c r="A481" s="18" t="inlineStr">
         <is>
-          <t>FICHA 33: HORIZON-CL5-2027-01-D1-11</t>
+          <t>FICHA 33: HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="B481" s="19" t="n"/>
@@ -13211,7 +13263,7 @@
       <c r="E482" s="22" t="n"/>
       <c r="F482" s="22" t="n"/>
     </row>
-    <row r="483" ht="20" customHeight="1">
+    <row r="483" ht="45" customHeight="1">
       <c r="A483" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -13219,7 +13271,7 @@
       </c>
       <c r="B483" s="21" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
         </is>
       </c>
       <c r="C483" s="22" t="n"/>
@@ -13235,7 +13287,7 @@
       </c>
       <c r="B484" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C484" s="22" t="n"/>
@@ -13315,7 +13367,7 @@
       </c>
       <c r="B489" s="21" t="inlineStr">
         <is>
-          <t>Programme Cofund Actions</t>
+          <t xml:space="preserve"> Research and Innovation Actions</t>
         </is>
       </c>
       <c r="C489" s="22" t="n"/>
@@ -13347,7 +13399,7 @@
       </c>
       <c r="B491" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is established through development and implementation of the Climate Action pillar of the EU-AU Research and Innovation Partnership on Climate Change and Sustainable Energy (CCSE),[1] in co-design between African and European partners;Reduced fragmentation by aligning the EU, national and multilateral R&amp;amp;I efforts with increased leverage and impact of funding;African scientific, policy and practice com</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Europe and globally, as well as the interaction between different hazards, their cumulative and/or cascading effects.Enhanced seamless prediction and projection modelling and attribution capabilities for extreme events and their likelihood to support preparedness, response and resilience to climate change by EU and national and regional actors. The EU Union Preparedness Strategy, the EU Adaptation Str</t>
         </is>
       </c>
       <c r="C491" s="22" t="n"/>
@@ -13391,7 +13443,7 @@
       </c>
       <c r="B494" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-11</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C494" s="22" t="n"/>
@@ -13402,7 +13454,7 @@
     <row r="496" ht="30" customHeight="1">
       <c r="A496" s="18" t="inlineStr">
         <is>
-          <t>FICHA 34: HORIZON-CL5-2027-01-D1-10</t>
+          <t>FICHA 34: HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="B496" s="19" t="n"/>
@@ -13427,7 +13479,7 @@
       <c r="E497" s="22" t="n"/>
       <c r="F497" s="22" t="n"/>
     </row>
-    <row r="498" ht="20" customHeight="1">
+    <row r="498" ht="45" customHeight="1">
       <c r="A498" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -13435,7 +13487,7 @@
       </c>
       <c r="B498" s="21" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
         </is>
       </c>
       <c r="C498" s="22" t="n"/>
@@ -13451,7 +13503,7 @@
       </c>
       <c r="B499" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C499" s="22" t="n"/>
@@ -13563,7 +13615,7 @@
       </c>
       <c r="B506" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorporation into main EU repositories, such as Climate-ADAPT or the portal of the EU Mission on Adaptation to Climate Change;The risk and adaptation assessment frameworks are improved by better integrating the maladaptation dimension;Guidelines and tools for maladaptation prevention and correction strategies are made available to adaptation stakeholders at relevant scales and inform the design and impl</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to inform mitigation action and policy improvements, ensuring a fair transition and social acceptability;Methodologies are developed and improved for ex-ante assessment and ex-post evaluation of greenhouse gas emission reductions from climate policies and measures;Strengthened collaboration and established networks between researchers, policy experts and government officials involved in designing and eva</t>
         </is>
       </c>
       <c r="C506" s="22" t="n"/>
@@ -13607,7 +13659,7 @@
       </c>
       <c r="B509" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-10</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C509" s="22" t="n"/>
@@ -13618,7 +13670,7 @@
     <row r="511" ht="30" customHeight="1">
       <c r="A511" s="18" t="inlineStr">
         <is>
-          <t>FICHA 35: HORIZON-CL5-2027-01-D1-07</t>
+          <t>FICHA 35: HORIZON-CL5-2027-01-D1-13</t>
         </is>
       </c>
       <c r="B511" s="19" t="n"/>
@@ -13643,7 +13695,7 @@
       <c r="E512" s="22" t="n"/>
       <c r="F512" s="22" t="n"/>
     </row>
-    <row r="513" ht="45" customHeight="1">
+    <row r="513" ht="20" customHeight="1">
       <c r="A513" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -13651,7 +13703,7 @@
       </c>
       <c r="B513" s="21" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
+          <t>Next generation scenarios for informing climate and sustainability transitions</t>
         </is>
       </c>
       <c r="C513" s="22" t="n"/>
@@ -13667,7 +13719,7 @@
       </c>
       <c r="B514" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-13</t>
         </is>
       </c>
       <c r="C514" s="22" t="n"/>
@@ -13779,7 +13831,7 @@
       </c>
       <c r="B521" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Europe and globally, as well as the interaction between different hazards, their cumulative and/or cascading effects.Enhanced seamless prediction and projection modelling and attribution capabilities for extreme events and their likelihood to support preparedness, response and resilience to climate change by EU and national and regional actors. The EU Union Preparedness Strategy, the EU Adaptation Str</t>
+          <t>Expected Outcome:Project results are expected to contribute to some of the following expected outcomes:Strengthened collaboration and integration across research communities, better capturing interactions and trade-offs between various climate domains as well as between climate and non-climate objectives, such as biodiversity or pollution related. This will support more comprehensive and consistent evaluations, benefiting key global assessments (IPCC, IPBES) and improving their impact on European and global policies (European Green Deal, UNFCCC, CBD);More relevant, robust and actionable scenar</t>
         </is>
       </c>
       <c r="C521" s="22" t="n"/>
@@ -13823,7 +13875,7 @@
       </c>
       <c r="B524" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-07</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-13</t>
         </is>
       </c>
       <c r="C524" s="22" t="n"/>
@@ -13834,7 +13886,7 @@
     <row r="526" ht="30" customHeight="1">
       <c r="A526" s="18" t="inlineStr">
         <is>
-          <t>FICHA 36: HORIZON-CL5-2027-01-D1-09</t>
+          <t>FICHA 36: HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="B526" s="19" t="n"/>
@@ -13859,7 +13911,7 @@
       <c r="E527" s="22" t="n"/>
       <c r="F527" s="22" t="n"/>
     </row>
-    <row r="528" ht="45" customHeight="1">
+    <row r="528" ht="20" customHeight="1">
       <c r="A528" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -13867,7 +13919,7 @@
       </c>
       <c r="B528" s="21" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="C528" s="22" t="n"/>
@@ -13883,7 +13935,7 @@
       </c>
       <c r="B529" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C529" s="22" t="n"/>
@@ -13963,7 +14015,7 @@
       </c>
       <c r="B534" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Research and Innovation Actions</t>
+          <t>Programme Cofund Actions</t>
         </is>
       </c>
       <c r="C534" s="22" t="n"/>
@@ -13995,7 +14047,7 @@
       </c>
       <c r="B536" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to inform mitigation action and policy improvements, ensuring a fair transition and social acceptability;Methodologies are developed and improved for ex-ante assessment and ex-post evaluation of greenhouse gas emission reductions from climate policies and measures;Strengthened collaboration and established networks between researchers, policy experts and government officials involved in designing and eva</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is established through development and implementation of the Climate Action pillar of the EU-AU Research and Innovation Partnership on Climate Change and Sustainable Energy (CCSE),[1] in co-design between African and European partners;Reduced fragmentation by aligning the EU, national and multilateral R&amp;amp;I efforts with increased leverage and impact of funding;African scientific, policy and practice com</t>
         </is>
       </c>
       <c r="C536" s="22" t="n"/>
@@ -14039,7 +14091,7 @@
       </c>
       <c r="B539" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-09</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C539" s="22" t="n"/>
@@ -20038,7 +20090,7 @@
     <row r="961" ht="30" customHeight="1">
       <c r="A961" s="18" t="inlineStr">
         <is>
-          <t>FICHA 65: dc0033a0-cb94-44ed-8102-0fd0a386989e-EXA</t>
+          <t>FICHA 65: 4b45d249-5739-4bf7-9595-a4715b73c2f6-EXA</t>
         </is>
       </c>
       <c r="B961" s="19" t="n"/>
@@ -20087,7 +20139,7 @@
       </c>
       <c r="B964" s="21" t="inlineStr">
         <is>
-          <t>dc0033a0-cb94-44ed-8102-0fd0a386989e-EXA</t>
+          <t>4b45d249-5739-4bf7-9595-a4715b73c2f6-EXA</t>
         </is>
       </c>
       <c r="C964" s="22" t="n"/>
@@ -20175,7 +20227,7 @@
       </c>
       <c r="B970" s="21" t="inlineStr">
         <is>
-          <t>EC-REGIO/2025/MVP/0023-EXA</t>
+          <t>EC-REGIO/2025/MVP/0036-EXA</t>
         </is>
       </c>
       <c r="C970" s="22" t="n"/>
@@ -20235,7 +20287,7 @@
       </c>
       <c r="B974" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/dc0033a0-cb94-44ed-8102-0fd0a386989e-EXA</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/4b45d249-5739-4bf7-9595-a4715b73c2f6-EXA</t>
         </is>
       </c>
       <c r="C974" s="22" t="n"/>
@@ -20246,7 +20298,7 @@
     <row r="976" ht="30" customHeight="1">
       <c r="A976" s="18" t="inlineStr">
         <is>
-          <t>FICHA 66: 4b45d249-5739-4bf7-9595-a4715b73c2f6-EXA</t>
+          <t>FICHA 66: dc0033a0-cb94-44ed-8102-0fd0a386989e-EXA</t>
         </is>
       </c>
       <c r="B976" s="19" t="n"/>
@@ -20295,7 +20347,7 @@
       </c>
       <c r="B979" s="21" t="inlineStr">
         <is>
-          <t>4b45d249-5739-4bf7-9595-a4715b73c2f6-EXA</t>
+          <t>dc0033a0-cb94-44ed-8102-0fd0a386989e-EXA</t>
         </is>
       </c>
       <c r="C979" s="22" t="n"/>
@@ -20383,7 +20435,7 @@
       </c>
       <c r="B985" s="21" t="inlineStr">
         <is>
-          <t>EC-REGIO/2025/MVP/0036-EXA</t>
+          <t>EC-REGIO/2025/MVP/0023-EXA</t>
         </is>
       </c>
       <c r="C985" s="22" t="n"/>
@@ -20443,7 +20495,7 @@
       </c>
       <c r="B989" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/4b45d249-5739-4bf7-9595-a4715b73c2f6-EXA</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/dc0033a0-cb94-44ed-8102-0fd0a386989e-EXA</t>
         </is>
       </c>
       <c r="C989" s="22" t="n"/>
@@ -20878,7 +20930,7 @@
     <row r="1021" ht="30" customHeight="1">
       <c r="A1021" s="18" t="inlineStr">
         <is>
-          <t>FICHA 69: EUS-74373</t>
+          <t>FICHA 69: EUS-74952</t>
         </is>
       </c>
       <c r="B1021" s="19" t="n"/>
@@ -20911,7 +20963,7 @@
       </c>
       <c r="B1023" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a proyectos al amparo de la estrategia de desarrollo local participativo (EDLP), aprobada al grupo de acción local del sector pesquero (GALP) para el desarrollo sostenible de las zonas de pesca</t>
+          <t>Servicio de transporte y reparto de comida desde las cocinas de elaboración a domicilios del municipio de Vitoria-Gasteiz y comedores del Departamento de Políticas Sociales</t>
         </is>
       </c>
       <c r="C1023" s="22" t="n"/>
@@ -20927,7 +20979,7 @@
       </c>
       <c r="B1024" s="21" t="inlineStr">
         <is>
-          <t>EUS-74373</t>
+          <t>EUS-74952</t>
         </is>
       </c>
       <c r="C1024" s="22" t="n"/>
@@ -21003,7 +21055,7 @@
       </c>
       <c r="B1029" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C1029" s="22" t="n"/>
@@ -21061,9 +21113,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B1033" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ALTA — </t>
+      <c r="B1033" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MUY ALTA — </t>
         </is>
       </c>
       <c r="C1033" s="22" t="n"/>
@@ -21079,7 +21131,7 @@
       </c>
       <c r="B1034" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/ayudas-al-amparo-de-la-estrategia-de-desarrollo-local-participativo-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-transporte-y-reparto-comida-cocinas-elaboracion-domicilios-del-municipio-vitoria-gasteiz-y-comedores-del-departamento-politicas-sociales/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1034" s="22" t="n"/>
@@ -21090,7 +21142,7 @@
     <row r="1036" ht="30" customHeight="1">
       <c r="A1036" s="18" t="inlineStr">
         <is>
-          <t>FICHA 70: EUS-13151</t>
+          <t>FICHA 70: EUS-31018</t>
         </is>
       </c>
       <c r="B1036" s="19" t="n"/>
@@ -21123,7 +21175,7 @@
       </c>
       <c r="B1038" s="21" t="inlineStr">
         <is>
-          <t>ReSourceEU y materias primas críticas: la UE sigue tramitando convocatorias para favorecer proyectos otorgándoles carácter estratégico, de la mano del Banco Europeo de Inversiones, de cara a ámbitos c</t>
+          <t>Ayudas a proyectos al amparo de la estrategia de desarrollo local participativo (EDLP), aprobada al grupo de acción local del sector pesquero (GALP) para el desarrollo sostenible de las zonas de pesca</t>
         </is>
       </c>
       <c r="C1038" s="22" t="n"/>
@@ -21139,7 +21191,7 @@
       </c>
       <c r="B1039" s="21" t="inlineStr">
         <is>
-          <t>EUS-13151</t>
+          <t>EUS-31018</t>
         </is>
       </c>
       <c r="C1039" s="22" t="n"/>
@@ -21291,7 +21343,7 @@
       </c>
       <c r="B1049" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260119resourceeumateriaes/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/ayudas-al-amparo-de-la-estrategia-de-desarrollo-local-participativo-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1049" s="22" t="n"/>
@@ -21302,7 +21354,7 @@
     <row r="1051" ht="30" customHeight="1">
       <c r="A1051" s="18" t="inlineStr">
         <is>
-          <t>FICHA 71: EUS-33319</t>
+          <t>FICHA 71: EUS-53900</t>
         </is>
       </c>
       <c r="B1051" s="19" t="n"/>
@@ -21335,7 +21387,7 @@
       </c>
       <c r="B1053" s="21" t="inlineStr">
         <is>
-          <t>Ciudades sostenibles: los Premios Capital Verde Europea y Hoja Verde de 2028 abren su convocatoria hasta el 01.04.26 para ciudades de más de 100.000 y de más de 20.000 habitantes, climáticamente resil</t>
+          <t>ReSourceEU y materias primas críticas: la UE sigue tramitando convocatorias para favorecer proyectos otorgándoles carácter estratégico, de la mano del Banco Europeo de Inversiones, de cara a ámbitos c</t>
         </is>
       </c>
       <c r="C1053" s="22" t="n"/>
@@ -21351,7 +21403,7 @@
       </c>
       <c r="B1054" s="21" t="inlineStr">
         <is>
-          <t>EUS-33319</t>
+          <t>EUS-53900</t>
         </is>
       </c>
       <c r="C1054" s="22" t="n"/>
@@ -21503,7 +21555,7 @@
       </c>
       <c r="B1064" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/hiriburutahostoberdea2826/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260119resourceeumateriaes/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1064" s="22" t="n"/>
@@ -21514,7 +21566,7 @@
     <row r="1066" ht="30" customHeight="1">
       <c r="A1066" s="18" t="inlineStr">
         <is>
-          <t>FICHA 72: EUS-06487</t>
+          <t>FICHA 72: EUS-66315</t>
         </is>
       </c>
       <c r="B1066" s="19" t="n"/>
@@ -21547,7 +21599,7 @@
       </c>
       <c r="B1068" s="21" t="inlineStr">
         <is>
-          <t>Presolicitud para programa de ayudas a empresas que realicen inversiones productivas que permitan diversificar líneas de negocio, productos, servicios y mercados, con un enfoque en el crecimiento sost</t>
+          <t>Ciudades sostenibles: los Premios Capital Verde Europea y Hoja Verde de 2028 abren su convocatoria hasta el 01.04.26 para ciudades de más de 100.000 y de más de 20.000 habitantes, climáticamente resil</t>
         </is>
       </c>
       <c r="C1068" s="22" t="n"/>
@@ -21563,7 +21615,7 @@
       </c>
       <c r="B1069" s="21" t="inlineStr">
         <is>
-          <t>EUS-06487</t>
+          <t>EUS-66315</t>
         </is>
       </c>
       <c r="C1069" s="22" t="n"/>
@@ -21715,7 +21767,7 @@
       </c>
       <c r="B1079" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2025/presolicitud-dibertsifika-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/hiriburutahostoberdea2826/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1079" s="22" t="n"/>
@@ -21726,7 +21778,7 @@
     <row r="1081" ht="30" customHeight="1">
       <c r="A1081" s="18" t="inlineStr">
         <is>
-          <t>FICHA 73: EUS-05566</t>
+          <t>FICHA 73: EUS-81441</t>
         </is>
       </c>
       <c r="B1081" s="19" t="n"/>
@@ -21759,7 +21811,7 @@
       </c>
       <c r="B1083" s="21" t="inlineStr">
         <is>
-          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de aceleración de proyectos, a localidades de menos de 20.000 habitantes son objeto de convocatoria abierta hasta el 17.03.26. Transformacione</t>
+          <t>Presolicitud para programa de ayudas a empresas que realicen inversiones productivas que permitan diversificar líneas de negocio, productos, servicios y mercados, con un enfoque en el crecimiento sost</t>
         </is>
       </c>
       <c r="C1083" s="22" t="n"/>
@@ -21775,7 +21827,7 @@
       </c>
       <c r="B1084" s="21" t="inlineStr">
         <is>
-          <t>EUS-05566</t>
+          <t>EUS-81441</t>
         </is>
       </c>
       <c r="C1084" s="22" t="n"/>
@@ -21909,9 +21961,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B1093" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
+      <c r="B1093" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALTA — </t>
         </is>
       </c>
       <c r="C1093" s="22" t="n"/>
@@ -21927,7 +21979,7 @@
       </c>
       <c r="B1094" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260317neboostasariak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2025/presolicitud-dibertsifika-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1094" s="22" t="n"/>
@@ -21938,7 +21990,7 @@
     <row r="1096" ht="30" customHeight="1">
       <c r="A1096" s="18" t="inlineStr">
         <is>
-          <t>FICHA 74: EUS-49036</t>
+          <t>FICHA 74: EUS-88586</t>
         </is>
       </c>
       <c r="B1096" s="19" t="n"/>
@@ -21971,7 +22023,7 @@
       </c>
       <c r="B1098" s="21" t="inlineStr">
         <is>
-          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinancia convocatorias de ayudas de las Diputaciones a explotaciones con limitaciones o desfavorecidas, y a compromisos medioambientales, climátic</t>
+          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de aceleración de proyectos, a localidades de menos de 20.000 habitantes son objeto de convocatoria abierta hasta el 17.03.26. Transformacione</t>
         </is>
       </c>
       <c r="C1098" s="22" t="n"/>
@@ -21987,7 +22039,7 @@
       </c>
       <c r="B1099" s="21" t="inlineStr">
         <is>
-          <t>EUS-49036</t>
+          <t>EUS-88586</t>
         </is>
       </c>
       <c r="C1099" s="22" t="n"/>
@@ -22139,7 +22191,7 @@
       </c>
       <c r="B1109" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/lgenfnpbgfa260218/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260317neboostasariak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1109" s="22" t="n"/>
@@ -22150,7 +22202,7 @@
     <row r="1111" ht="30" customHeight="1">
       <c r="A1111" s="18" t="inlineStr">
         <is>
-          <t>FICHA 75: EUS-84033</t>
+          <t>FICHA 75: EUS-91314</t>
         </is>
       </c>
       <c r="B1111" s="19" t="n"/>
@@ -22183,7 +22235,7 @@
       </c>
       <c r="B1113" s="21" t="inlineStr">
         <is>
-          <t>Digital Europe, Horizon (programas de la UE). Apoyos para consorcios interestatales de I+D+i. IA, robótica, cuántica, computación, ciberseguridad, electrónica, fotónica, TICs e internet avanzadas, esp</t>
+          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinancia convocatorias de ayudas de las Diputaciones a explotaciones con limitaciones o desfavorecidas, y a compromisos medioambientales, climátic</t>
         </is>
       </c>
       <c r="C1113" s="22" t="n"/>
@@ -22199,7 +22251,7 @@
       </c>
       <c r="B1114" s="21" t="inlineStr">
         <is>
-          <t>EUS-84033</t>
+          <t>EUS-91314</t>
         </is>
       </c>
       <c r="C1114" s="22" t="n"/>
@@ -22351,7 +22403,7 @@
       </c>
       <c r="B1124" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260304digitalhorizoneen/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/lgenfnpbgfa260218/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1124" s="22" t="n"/>
@@ -22362,7 +22414,7 @@
     <row r="1126" ht="30" customHeight="1">
       <c r="A1126" s="18" t="inlineStr">
         <is>
-          <t>FICHA 76: EUS-55512</t>
+          <t>FICHA 76: EUS-84020</t>
         </is>
       </c>
       <c r="B1126" s="19" t="n"/>
@@ -22395,7 +22447,7 @@
       </c>
       <c r="B1128" s="21" t="inlineStr">
         <is>
-          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para consorcios internacionales de I+D+i. Jornada del Gobierno Vasco y con Enterprise Europe Network y otros socios. Digitalización, dispositivos,</t>
+          <t>Digital Europe, Horizon (programas de la UE). Apoyos para consorcios interestatales de I+D+i. IA, robótica, cuántica, computación, ciberseguridad, electrónica, fotónica, TICs e internet avanzadas, esp</t>
         </is>
       </c>
       <c r="C1128" s="22" t="n"/>
@@ -22411,7 +22463,7 @@
       </c>
       <c r="B1129" s="21" t="inlineStr">
         <is>
-          <t>EUS-55512</t>
+          <t>EUS-84020</t>
         </is>
       </c>
       <c r="C1129" s="22" t="n"/>
@@ -22563,7 +22615,7 @@
       </c>
       <c r="B1139" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260303eicihihorizon/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260304digitalhorizoneen/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1139" s="22" t="n"/>
@@ -22574,7 +22626,7 @@
     <row r="1141" ht="30" customHeight="1">
       <c r="A1141" s="18" t="inlineStr">
         <is>
-          <t>FICHA 77: EUS-90444</t>
+          <t>FICHA 77: EUS-18785</t>
         </is>
       </c>
       <c r="B1141" s="19" t="n"/>
@@ -22607,7 +22659,7 @@
       </c>
       <c r="B1143" s="21" t="inlineStr">
         <is>
-          <t>Política Agraria Común de la UE de 2026, y sus ayudas abiertas hasta el 30.4.26: el pilar 1, con el Fondo Europeo Agrícola de Garantía Agraria FEAGA, aborda sostenibilidad de renta, ayuda redistributi</t>
+          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para consorcios internacionales de I+D+i. Jornada del Gobierno Vasco y con Enterprise Europe Network y otros socios. Digitalización, dispositivos,</t>
         </is>
       </c>
       <c r="C1143" s="22" t="n"/>
@@ -22623,7 +22675,7 @@
       </c>
       <c r="B1144" s="21" t="inlineStr">
         <is>
-          <t>EUS-90444</t>
+          <t>EUS-18785</t>
         </is>
       </c>
       <c r="C1144" s="22" t="n"/>
@@ -22775,7 +22827,7 @@
       </c>
       <c r="B1154" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260216npblaguntzairekiak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260303eicihihorizon/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1154" s="22" t="n"/>
@@ -22786,7 +22838,7 @@
     <row r="1156" ht="30" customHeight="1">
       <c r="A1156" s="18" t="inlineStr">
         <is>
-          <t>FICHA 78: EUS-25327</t>
+          <t>FICHA 78: EUS-44870</t>
         </is>
       </c>
       <c r="B1156" s="19" t="n"/>
@@ -22819,7 +22871,7 @@
       </c>
       <c r="B1158" s="21" t="inlineStr">
         <is>
-          <t>Programa de impulso a las ciudades y territorios inteligentes para el fomento del desarrollo económico y productivo, que podrá ser cofinanciado por el Programa Plurirregional 2021-2027 del Fondo Europ</t>
+          <t>Política Agraria Común de la UE de 2026, y sus ayudas abiertas hasta el 30.4.26: el pilar 1, con el Fondo Europeo Agrícola de Garantía Agraria FEAGA, aborda sostenibilidad de renta, ayuda redistributi</t>
         </is>
       </c>
       <c r="C1158" s="22" t="n"/>
@@ -22835,7 +22887,7 @@
       </c>
       <c r="B1159" s="21" t="inlineStr">
         <is>
-          <t>EUS-25327</t>
+          <t>EUS-44870</t>
         </is>
       </c>
       <c r="C1159" s="22" t="n"/>
@@ -22987,7 +23039,7 @@
       </c>
       <c r="B1169" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260204smartcities/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260216npblaguntzairekiak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1169" s="22" t="n"/>
@@ -22998,7 +23050,7 @@
     <row r="1171" ht="30" customHeight="1">
       <c r="A1171" s="18" t="inlineStr">
         <is>
-          <t>FICHA 79: EUS-73767</t>
+          <t>FICHA 79: EUS-29143</t>
         </is>
       </c>
       <c r="B1171" s="19" t="n"/>
@@ -23031,7 +23083,7 @@
       </c>
       <c r="B1173" s="21" t="inlineStr">
         <is>
-          <t>Formación digital para empleabilidad turística: los fondos Next de la UE apoyan una convocatoria de Lanbide y el Gobierno Vasco, de cursos en línea para mejorar las competencias del sector y de sus py</t>
+          <t>Programa de impulso a las ciudades y territorios inteligentes para el fomento del desarrollo económico y productivo, que podrá ser cofinanciado por el Programa Plurirregional 2021-2027 del Fondo Europ</t>
         </is>
       </c>
       <c r="C1173" s="22" t="n"/>
@@ -23047,7 +23099,7 @@
       </c>
       <c r="B1174" s="21" t="inlineStr">
         <is>
-          <t>EUS-73767</t>
+          <t>EUS-29143</t>
         </is>
       </c>
       <c r="C1174" s="22" t="n"/>
@@ -23199,7 +23251,7 @@
       </c>
       <c r="B1184" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260119nextlanbidedigital/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260204smartcities/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1184" s="22" t="n"/>
@@ -23210,7 +23262,7 @@
     <row r="1186" ht="30" customHeight="1">
       <c r="A1186" s="18" t="inlineStr">
         <is>
-          <t>FICHA 80: EUS-54415</t>
+          <t>FICHA 80: EUS-05166</t>
         </is>
       </c>
       <c r="B1186" s="19" t="n"/>
@@ -23243,7 +23295,7 @@
       </c>
       <c r="B1188" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Horizon Europe. Clúster digital, industrial y espacial. Apoyos a proyectos para tecnologías de inteligencia artificial, internet, mundos virtuales, robótica, cuántica, fotónica, materias primas, bajo </t>
+          <t>Formación digital para empleabilidad turística: los fondos Next de la UE apoyan una convocatoria de Lanbide y el Gobierno Vasco, de cursos en línea para mejorar las competencias del sector y de sus py</t>
         </is>
       </c>
       <c r="C1188" s="22" t="n"/>
@@ -23259,7 +23311,7 @@
       </c>
       <c r="B1189" s="21" t="inlineStr">
         <is>
-          <t>EUS-54415</t>
+          <t>EUS-05166</t>
         </is>
       </c>
       <c r="C1189" s="22" t="n"/>
@@ -23411,7 +23463,7 @@
       </c>
       <c r="B1199" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/250119horizondiginduspaceklust/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260119nextlanbidedigital/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1199" s="22" t="n"/>
@@ -23422,7 +23474,7 @@
     <row r="1201" ht="30" customHeight="1">
       <c r="A1201" s="18" t="inlineStr">
         <is>
-          <t>FICHA 81: EUS-27582</t>
+          <t>FICHA 81: EUS-07020</t>
         </is>
       </c>
       <c r="B1201" s="19" t="n"/>
@@ -23455,7 +23507,7 @@
       </c>
       <c r="B1203" s="21" t="inlineStr">
         <is>
-          <t>Horizon Europe: ayudas de la línea de energía del clúster 5 y de la Misión Ciudades. Jornada informativa sobre estas y otras iniciativas en colaboración transestatal para la doble transición ecológica</t>
+          <t xml:space="preserve">Horizon Europe. Clúster digital, industrial y espacial. Apoyos a proyectos para tecnologías de inteligencia artificial, internet, mundos virtuales, robótica, cuántica, fotónica, materias primas, bajo </t>
         </is>
       </c>
       <c r="C1203" s="22" t="n"/>
@@ -23471,7 +23523,7 @@
       </c>
       <c r="B1204" s="21" t="inlineStr">
         <is>
-          <t>EUS-27582</t>
+          <t>EUS-07020</t>
         </is>
       </c>
       <c r="C1204" s="22" t="n"/>
@@ -23623,7 +23675,7 @@
       </c>
       <c r="B1214" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/horizonkluster5hirimisioa/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/250119horizondiginduspaceklust/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1214" s="22" t="n"/>
@@ -23634,7 +23686,7 @@
     <row r="1216" ht="30" customHeight="1">
       <c r="A1216" s="18" t="inlineStr">
         <is>
-          <t>FICHA 82: EUS-96937</t>
+          <t>FICHA 82: EUS-58974</t>
         </is>
       </c>
       <c r="B1216" s="19" t="n"/>
@@ -23667,7 +23719,7 @@
       </c>
       <c r="B1218" s="21" t="inlineStr">
         <is>
-          <t>Azpitek 2026: Programa de Ayudas para la Adquisición, Instalación, Renovación y Actualización de Infraestructuras de Investigación</t>
+          <t>Horizon Europe: ayudas de la línea de energía del clúster 5 y de la Misión Ciudades. Jornada informativa sobre estas y otras iniciativas en colaboración transestatal para la doble transición ecológica</t>
         </is>
       </c>
       <c r="C1218" s="22" t="n"/>
@@ -23683,7 +23735,7 @@
       </c>
       <c r="B1219" s="21" t="inlineStr">
         <is>
-          <t>EUS-96937</t>
+          <t>EUS-58974</t>
         </is>
       </c>
       <c r="C1219" s="22" t="n"/>
@@ -23835,7 +23887,7 @@
       </c>
       <c r="B1229" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2025/azpitek-2026-programa-de-ayudas/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/horizonkluster5hirimisioa/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1229" s="22" t="n"/>
@@ -23846,7 +23898,7 @@
     <row r="1231" ht="30" customHeight="1">
       <c r="A1231" s="18" t="inlineStr">
         <is>
-          <t>FICHA 83: EUS-68824</t>
+          <t>FICHA 83: EUS-81341</t>
         </is>
       </c>
       <c r="B1231" s="19" t="n"/>
@@ -23871,7 +23923,7 @@
       <c r="E1232" s="22" t="n"/>
       <c r="F1232" s="22" t="n"/>
     </row>
-    <row r="1233" ht="20" customHeight="1">
+    <row r="1233" ht="45" customHeight="1">
       <c r="A1233" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -23879,7 +23931,7 @@
       </c>
       <c r="B1233" s="21" t="inlineStr">
         <is>
-          <t>Subvenciones para innovación en economía circular 2026</t>
+          <t>Azpitek 2026: Programa de Ayudas para la Adquisición, Instalación, Renovación y Actualización de Infraestructuras de Investigación</t>
         </is>
       </c>
       <c r="C1233" s="22" t="n"/>
@@ -23895,7 +23947,7 @@
       </c>
       <c r="B1234" s="21" t="inlineStr">
         <is>
-          <t>EUS-68824</t>
+          <t>EUS-81341</t>
         </is>
       </c>
       <c r="C1234" s="22" t="n"/>
@@ -24047,7 +24099,7 @@
       </c>
       <c r="B1244" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2025/subvenciones-para-innovacion-en-economia-circular-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2025/azpitek-2026-programa-de-ayudas/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1244" s="22" t="n"/>
@@ -24058,7 +24110,7 @@
     <row r="1246" ht="30" customHeight="1">
       <c r="A1246" s="18" t="inlineStr">
         <is>
-          <t>FICHA 84: EUS-21415</t>
+          <t>FICHA 84: EUS-61815</t>
         </is>
       </c>
       <c r="B1246" s="19" t="n"/>
@@ -24083,7 +24135,7 @@
       <c r="E1247" s="22" t="n"/>
       <c r="F1247" s="22" t="n"/>
     </row>
-    <row r="1248" ht="45" customHeight="1">
+    <row r="1248" ht="20" customHeight="1">
       <c r="A1248" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -24091,7 +24143,7 @@
       </c>
       <c r="B1248" s="21" t="inlineStr">
         <is>
-          <t>Horizon Europe 2026-27: convocatorias ligadas a misiones ambientales de la UE, partenariados de economía circular, azul o bio, o a la división alimentaria EIT Food del Instituto Europeo de Tecnología,</t>
+          <t>Subvenciones para innovación en economía circular 2026</t>
         </is>
       </c>
       <c r="C1248" s="22" t="n"/>
@@ -24107,7 +24159,7 @@
       </c>
       <c r="B1249" s="21" t="inlineStr">
         <is>
-          <t>EUS-21415</t>
+          <t>EUS-61815</t>
         </is>
       </c>
       <c r="C1249" s="22" t="n"/>
@@ -24259,7 +24311,7 @@
       </c>
       <c r="B1259" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2025/251222horizon2627sprieeni/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2025/subvenciones-para-innovacion-en-economia-circular-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1259" s="22" t="n"/>
@@ -24270,7 +24322,7 @@
     <row r="1261" ht="30" customHeight="1">
       <c r="A1261" s="18" t="inlineStr">
         <is>
-          <t>FICHA 85: EUS-12091</t>
+          <t>FICHA 85: EUS-61141</t>
         </is>
       </c>
       <c r="B1261" s="19" t="n"/>
@@ -24303,7 +24355,7 @@
       </c>
       <c r="B1263" s="21" t="inlineStr">
         <is>
-          <t>Escudo Europeo de la Democracia: ayudas a proyectos de alfabetización mediática y fomento del diálogo y la comprensión en torno a la desinformación digital</t>
+          <t>Horizon Europe 2026-27: convocatorias ligadas a misiones ambientales de la UE, partenariados de economía circular, azul o bio, o a la división alimentaria EIT Food del Instituto Europeo de Tecnología,</t>
         </is>
       </c>
       <c r="C1263" s="22" t="n"/>
@@ -24319,7 +24371,7 @@
       </c>
       <c r="B1264" s="21" t="inlineStr">
         <is>
-          <t>EUS-12091</t>
+          <t>EUS-61141</t>
         </is>
       </c>
       <c r="C1264" s="22" t="n"/>
@@ -24471,7 +24523,7 @@
       </c>
       <c r="B1274" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2025/demokraziaezkutua251218/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2025/251222horizon2627sprieeni/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1274" s="22" t="n"/>
@@ -24482,7 +24534,7 @@
     <row r="1276" ht="30" customHeight="1">
       <c r="A1276" s="18" t="inlineStr">
         <is>
-          <t>FICHA 86: EUS-29046</t>
+          <t>FICHA 86: EUS-33047</t>
         </is>
       </c>
       <c r="B1276" s="19" t="n"/>
@@ -24515,7 +24567,7 @@
       </c>
       <c r="B1278" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">KSI Berritzaile Plus: ayudas del Gobierno Vasco a las Industrias Culturales y Creativas para proyectos innovadores en la triple transición tecnológico-digital, energético-climática y socio-sanitaria, </t>
+          <t>Escudo Europeo de la Democracia: ayudas a proyectos de alfabetización mediática y fomento del diálogo y la comprensión en torno a la desinformación digital</t>
         </is>
       </c>
       <c r="C1278" s="22" t="n"/>
@@ -24531,7 +24583,7 @@
       </c>
       <c r="B1279" s="21" t="inlineStr">
         <is>
-          <t>EUS-29046</t>
+          <t>EUS-33047</t>
         </is>
       </c>
       <c r="C1279" s="22" t="n"/>
@@ -24683,7 +24735,7 @@
       </c>
       <c r="B1289" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2025/ksiberritzalieplus251218/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2025/demokraziaezkutua251218/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1289" s="22" t="n"/>
@@ -24694,7 +24746,7 @@
     <row r="1291" ht="30" customHeight="1">
       <c r="A1291" s="18" t="inlineStr">
         <is>
-          <t>FICHA 87: EUS-78377</t>
+          <t>FICHA 87: EUS-49824</t>
         </is>
       </c>
       <c r="B1291" s="19" t="n"/>
@@ -24727,7 +24779,7 @@
       </c>
       <c r="B1293" s="21" t="inlineStr">
         <is>
-          <t>Desmontaje de dos depósitos de agua en local del polideportivo ipurua y tuberías que lo alimentan.</t>
+          <t xml:space="preserve">KSI Berritzaile Plus: ayudas del Gobierno Vasco a las Industrias Culturales y Creativas para proyectos innovadores en la triple transición tecnológico-digital, energético-climática y socio-sanitaria, </t>
         </is>
       </c>
       <c r="C1293" s="22" t="n"/>
@@ -24743,7 +24795,7 @@
       </c>
       <c r="B1294" s="21" t="inlineStr">
         <is>
-          <t>EUS-78377</t>
+          <t>EUS-49824</t>
         </is>
       </c>
       <c r="C1294" s="22" t="n"/>
@@ -24819,7 +24871,7 @@
       </c>
       <c r="B1299" s="21" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C1299" s="22" t="n"/>
@@ -24895,7 +24947,7 @@
       </c>
       <c r="B1304" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/desmontaje-dos-depositos-agua-local-del-polideportivo-ipurua-y-tuberias-que-alimentan/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2025/ksiberritzalieplus251218/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1304" s="22" t="n"/>
@@ -24906,7 +24958,7 @@
     <row r="1306" ht="30" customHeight="1">
       <c r="A1306" s="18" t="inlineStr">
         <is>
-          <t>FICHA 88: EUS-16975</t>
+          <t>FICHA 88: EUS-83207</t>
         </is>
       </c>
       <c r="B1306" s="19" t="n"/>
@@ -24931,7 +24983,7 @@
       <c r="E1307" s="22" t="n"/>
       <c r="F1307" s="22" t="n"/>
     </row>
-    <row r="1308" ht="20" customHeight="1">
+    <row r="1308" ht="45" customHeight="1">
       <c r="A1308" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -24939,7 +24991,7 @@
       </c>
       <c r="B1308" s="21" t="inlineStr">
         <is>
-          <t>Reparación del ascensor exterior de urki polonia tras entrada agua en cuadro</t>
+          <t>Desmontaje de dos depósitos de agua en local del polideportivo ipurua y tuberías que lo alimentan.</t>
         </is>
       </c>
       <c r="C1308" s="22" t="n"/>
@@ -24955,7 +25007,7 @@
       </c>
       <c r="B1309" s="21" t="inlineStr">
         <is>
-          <t>EUS-16975</t>
+          <t>EUS-83207</t>
         </is>
       </c>
       <c r="C1309" s="22" t="n"/>
@@ -25107,7 +25159,7 @@
       </c>
       <c r="B1319" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/reparacion-del-ascensor-exterior-urki-polonia-entrada-agua-cuadro/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/desmontaje-dos-depositos-agua-local-del-polideportivo-ipurua-y-tuberias-que-alimentan/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1319" s="22" t="n"/>
@@ -25118,7 +25170,7 @@
     <row r="1321" ht="30" customHeight="1">
       <c r="A1321" s="18" t="inlineStr">
         <is>
-          <t>FICHA 89: EUS-54763</t>
+          <t>FICHA 89: EUS-43218</t>
         </is>
       </c>
       <c r="B1321" s="19" t="n"/>
@@ -25151,7 +25203,7 @@
       </c>
       <c r="B1323" s="21" t="inlineStr">
         <is>
-          <t>Desatasco tanto de la red de pluviales como de la de fecales de errebal plazia</t>
+          <t>Reparación del ascensor exterior de urki polonia tras entrada agua en cuadro</t>
         </is>
       </c>
       <c r="C1323" s="22" t="n"/>
@@ -25167,7 +25219,7 @@
       </c>
       <c r="B1324" s="21" t="inlineStr">
         <is>
-          <t>EUS-54763</t>
+          <t>EUS-43218</t>
         </is>
       </c>
       <c r="C1324" s="22" t="n"/>
@@ -25319,7 +25371,7 @@
       </c>
       <c r="B1334" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/desatasco-tanto-red-pluviales-como-de-fecales-errebal-plazia/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/reparacion-del-ascensor-exterior-urki-polonia-entrada-agua-cuadro/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1334" s="22" t="n"/>
@@ -25330,7 +25382,7 @@
     <row r="1336" ht="30" customHeight="1">
       <c r="A1336" s="18" t="inlineStr">
         <is>
-          <t>FICHA 90: EUS-00010</t>
+          <t>FICHA 90: EUS-03214</t>
         </is>
       </c>
       <c r="B1336" s="19" t="n"/>
@@ -25355,7 +25407,7 @@
       <c r="E1337" s="22" t="n"/>
       <c r="F1337" s="22" t="n"/>
     </row>
-    <row r="1338" ht="45" customHeight="1">
+    <row r="1338" ht="20" customHeight="1">
       <c r="A1338" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -25363,7 +25415,7 @@
       </c>
       <c r="B1338" s="21" t="inlineStr">
         <is>
-          <t>Contratación de la actuación de unos bertsolaris el 8 y 14 de septiembre en el marco de las fiestas de ntra. sra. de arrate</t>
+          <t>Desatasco tanto de la red de pluviales como de la de fecales de errebal plazia</t>
         </is>
       </c>
       <c r="C1338" s="22" t="n"/>
@@ -25379,7 +25431,7 @@
       </c>
       <c r="B1339" s="21" t="inlineStr">
         <is>
-          <t>EUS-00010</t>
+          <t>EUS-03214</t>
         </is>
       </c>
       <c r="C1339" s="22" t="n"/>
@@ -25531,7 +25583,7 @@
       </c>
       <c r="B1349" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/contratacion-actuacion-bertsolaris-8-y-14-septiembre-marco-fiestas-ntra-sra-arrate/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/desatasco-tanto-red-pluviales-como-de-fecales-errebal-plazia/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1349" s="22" t="n"/>
@@ -25542,7 +25594,7 @@
     <row r="1351" ht="30" customHeight="1">
       <c r="A1351" s="18" t="inlineStr">
         <is>
-          <t>FICHA 91: EUS-50530</t>
+          <t>FICHA 91: EUS-68824</t>
         </is>
       </c>
       <c r="B1351" s="19" t="n"/>
@@ -25575,7 +25627,7 @@
       </c>
       <c r="B1353" s="21" t="inlineStr">
         <is>
-          <t>Suministro de botellines de agua mineral para atender a los grupos que actúan en el teatro coliseo</t>
+          <t>Contratación de la actuación de unos bertsolaris el 8 y 14 de septiembre en el marco de las fiestas de ntra. sra. de arrate</t>
         </is>
       </c>
       <c r="C1353" s="22" t="n"/>
@@ -25591,7 +25643,7 @@
       </c>
       <c r="B1354" s="21" t="inlineStr">
         <is>
-          <t>EUS-50530</t>
+          <t>EUS-68824</t>
         </is>
       </c>
       <c r="C1354" s="22" t="n"/>
@@ -25743,7 +25795,7 @@
       </c>
       <c r="B1364" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-botellines-agua-mineral-atender-grupos-que-actuan-teatro-coliseo/expgeeibar19188/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/contratacion-actuacion-bertsolaris-8-y-14-septiembre-marco-fiestas-ntra-sra-arrate/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1364" s="22" t="n"/>
@@ -25754,7 +25806,7 @@
     <row r="1366" ht="30" customHeight="1">
       <c r="A1366" s="18" t="inlineStr">
         <is>
-          <t>FICHA 92: EUS-28619</t>
+          <t>FICHA 92: EUS-26937</t>
         </is>
       </c>
       <c r="B1366" s="19" t="n"/>
@@ -25787,7 +25839,7 @@
       </c>
       <c r="B1368" s="21" t="inlineStr">
         <is>
-          <t>Servicio de organización de la sesión de bertsolaris de arrate del 7 de septiembre.</t>
+          <t>Suministro de botellines de agua mineral para atender a los grupos que actúan en el teatro coliseo</t>
         </is>
       </c>
       <c r="C1368" s="22" t="n"/>
@@ -25803,7 +25855,7 @@
       </c>
       <c r="B1369" s="21" t="inlineStr">
         <is>
-          <t>EUS-28619</t>
+          <t>EUS-26937</t>
         </is>
       </c>
       <c r="C1369" s="22" t="n"/>
@@ -25955,7 +26007,7 @@
       </c>
       <c r="B1379" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-organizacion-sesion-bertsolaris-arrate-del-7-septiembre/expgeeibar19095/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-botellines-agua-mineral-atender-grupos-que-actuan-teatro-coliseo/expgeeibar19188/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1379" s="22" t="n"/>
@@ -25963,8 +26015,220 @@
       <c r="E1379" s="22" t="n"/>
       <c r="F1379" s="22" t="n"/>
     </row>
+    <row r="1381" ht="30" customHeight="1">
+      <c r="A1381" s="18" t="inlineStr">
+        <is>
+          <t>FICHA 93: EUS-27498</t>
+        </is>
+      </c>
+      <c r="B1381" s="19" t="n"/>
+      <c r="C1381" s="19" t="n"/>
+      <c r="D1381" s="19" t="n"/>
+      <c r="E1381" s="19" t="n"/>
+      <c r="F1381" s="19" t="n"/>
+    </row>
+    <row r="1382" ht="20" customHeight="1">
+      <c r="A1382" s="20" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1382" s="21" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1382" s="22" t="n"/>
+      <c r="D1382" s="22" t="n"/>
+      <c r="E1382" s="22" t="n"/>
+      <c r="F1382" s="22" t="n"/>
+    </row>
+    <row r="1383" ht="45" customHeight="1">
+      <c r="A1383" s="20" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1383" s="21" t="inlineStr">
+        <is>
+          <t>Servicio de organización de la sesión de bertsolaris de arrate del 7 de septiembre.</t>
+        </is>
+      </c>
+      <c r="C1383" s="22" t="n"/>
+      <c r="D1383" s="22" t="n"/>
+      <c r="E1383" s="22" t="n"/>
+      <c r="F1383" s="22" t="n"/>
+    </row>
+    <row r="1384" ht="20" customHeight="1">
+      <c r="A1384" s="20" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1384" s="21" t="inlineStr">
+        <is>
+          <t>EUS-27498</t>
+        </is>
+      </c>
+      <c r="C1384" s="22" t="n"/>
+      <c r="D1384" s="22" t="n"/>
+      <c r="E1384" s="22" t="n"/>
+      <c r="F1384" s="22" t="n"/>
+    </row>
+    <row r="1385" ht="20" customHeight="1">
+      <c r="A1385" s="20" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1385" s="21" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1385" s="22" t="n"/>
+      <c r="D1385" s="22" t="n"/>
+      <c r="E1385" s="22" t="n"/>
+      <c r="F1385" s="22" t="n"/>
+    </row>
+    <row r="1386" ht="20" customHeight="1">
+      <c r="A1386" s="20" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1386" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1386" s="22" t="n"/>
+      <c r="D1386" s="22" t="n"/>
+      <c r="E1386" s="22" t="n"/>
+      <c r="F1386" s="22" t="n"/>
+    </row>
+    <row r="1387" ht="20" customHeight="1">
+      <c r="A1387" s="20" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1387" s="21" t="inlineStr"/>
+      <c r="C1387" s="22" t="n"/>
+      <c r="D1387" s="22" t="n"/>
+      <c r="E1387" s="22" t="n"/>
+      <c r="F1387" s="22" t="n"/>
+    </row>
+    <row r="1388" ht="20" customHeight="1">
+      <c r="A1388" s="20" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1388" s="21" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1388" s="22" t="n"/>
+      <c r="D1388" s="22" t="n"/>
+      <c r="E1388" s="22" t="n"/>
+      <c r="F1388" s="22" t="n"/>
+    </row>
+    <row r="1389" ht="20" customHeight="1">
+      <c r="A1389" s="20" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1389" s="21" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1389" s="22" t="n"/>
+      <c r="D1389" s="22" t="n"/>
+      <c r="E1389" s="22" t="n"/>
+      <c r="F1389" s="22" t="n"/>
+    </row>
+    <row r="1390" ht="20" customHeight="1">
+      <c r="A1390" s="20" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1390" s="21" t="inlineStr"/>
+      <c r="C1390" s="22" t="n"/>
+      <c r="D1390" s="22" t="n"/>
+      <c r="E1390" s="22" t="n"/>
+      <c r="F1390" s="22" t="n"/>
+    </row>
+    <row r="1391" ht="20" customHeight="1">
+      <c r="A1391" s="20" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1391" s="21" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1391" s="22" t="n"/>
+      <c r="D1391" s="22" t="n"/>
+      <c r="E1391" s="22" t="n"/>
+      <c r="F1391" s="22" t="n"/>
+    </row>
+    <row r="1392" ht="20" customHeight="1">
+      <c r="A1392" s="20" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1392" s="21" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1392" s="22" t="n"/>
+      <c r="D1392" s="22" t="n"/>
+      <c r="E1392" s="22" t="n"/>
+      <c r="F1392" s="22" t="n"/>
+    </row>
+    <row r="1393" ht="20" customHeight="1">
+      <c r="A1393" s="20" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1393" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1393" s="22" t="n"/>
+      <c r="D1393" s="22" t="n"/>
+      <c r="E1393" s="22" t="n"/>
+      <c r="F1393" s="22" t="n"/>
+    </row>
+    <row r="1394" ht="45" customHeight="1">
+      <c r="A1394" s="20" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1394" s="24" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-organizacion-sesion-bertsolaris-arrate-del-7-septiembre/expgeeibar19095/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1394" s="22" t="n"/>
+      <c r="D1394" s="22" t="n"/>
+      <c r="E1394" s="22" t="n"/>
+      <c r="F1394" s="22" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="1288">
+  <mergeCells count="1302">
     <mergeCell ref="B679:F679"/>
     <mergeCell ref="B1010:F1010"/>
     <mergeCell ref="B276:F276"/>
@@ -26171,6 +26435,7 @@
     <mergeCell ref="B321:F321"/>
     <mergeCell ref="B1040:F1040"/>
     <mergeCell ref="B323:F323"/>
+    <mergeCell ref="B1382:F1382"/>
     <mergeCell ref="A76:F76"/>
     <mergeCell ref="B621:F621"/>
     <mergeCell ref="B613:F613"/>
@@ -26225,17 +26490,20 @@
     <mergeCell ref="B1057:F1057"/>
     <mergeCell ref="B1093:F1093"/>
     <mergeCell ref="B1364:F1364"/>
+    <mergeCell ref="B1391:F1391"/>
     <mergeCell ref="B332:F332"/>
     <mergeCell ref="B937:F937"/>
     <mergeCell ref="B1059:F1059"/>
     <mergeCell ref="B1086:F1086"/>
     <mergeCell ref="B1357:F1357"/>
+    <mergeCell ref="B1393:F1393"/>
     <mergeCell ref="B632:F632"/>
     <mergeCell ref="B175:F175"/>
     <mergeCell ref="B790:F790"/>
     <mergeCell ref="B1088:F1088"/>
     <mergeCell ref="B1359:F1359"/>
     <mergeCell ref="A1291:F1291"/>
+    <mergeCell ref="B1388:F1388"/>
     <mergeCell ref="B806:F806"/>
     <mergeCell ref="B1077:F1077"/>
     <mergeCell ref="B343:F343"/>
@@ -26416,11 +26684,13 @@
     <mergeCell ref="B789:F789"/>
     <mergeCell ref="B248:F248"/>
     <mergeCell ref="A1216:F1216"/>
+    <mergeCell ref="B1394:F1394"/>
     <mergeCell ref="B362:F362"/>
     <mergeCell ref="B1334:F1334"/>
     <mergeCell ref="B579:F579"/>
     <mergeCell ref="B1089:F1089"/>
     <mergeCell ref="B877:F877"/>
+    <mergeCell ref="B1387:F1387"/>
     <mergeCell ref="B1300:F1300"/>
     <mergeCell ref="B205:F205"/>
     <mergeCell ref="B879:F879"/>
@@ -26505,6 +26775,7 @@
     <mergeCell ref="A511:F511"/>
     <mergeCell ref="B1056:F1056"/>
     <mergeCell ref="B24:F24"/>
+    <mergeCell ref="B1390:F1390"/>
     <mergeCell ref="B453:F453"/>
     <mergeCell ref="B629:F629"/>
     <mergeCell ref="B787:F787"/>
@@ -26516,6 +26787,7 @@
     <mergeCell ref="B482:F482"/>
     <mergeCell ref="B753:F753"/>
     <mergeCell ref="B1087:F1087"/>
+    <mergeCell ref="B1385:F1385"/>
     <mergeCell ref="B782:F782"/>
     <mergeCell ref="B27:F27"/>
     <mergeCell ref="B42:F42"/>
@@ -26676,6 +26948,7 @@
     <mergeCell ref="B626:F626"/>
     <mergeCell ref="B933:F933"/>
     <mergeCell ref="B172:F172"/>
+    <mergeCell ref="B1389:F1389"/>
     <mergeCell ref="B1345:F1345"/>
     <mergeCell ref="B506:F506"/>
     <mergeCell ref="B628:F628"/>
@@ -26727,6 +27000,7 @@
     <mergeCell ref="B713:F713"/>
     <mergeCell ref="B1011:F1011"/>
     <mergeCell ref="B110:F110"/>
+    <mergeCell ref="A1381:F1381"/>
     <mergeCell ref="B924:F924"/>
     <mergeCell ref="B584:F584"/>
     <mergeCell ref="B715:F715"/>
@@ -26989,6 +27263,7 @@
     <mergeCell ref="B1052:F1052"/>
     <mergeCell ref="B1044:F1044"/>
     <mergeCell ref="B327:F327"/>
+    <mergeCell ref="B1386:F1386"/>
     <mergeCell ref="B625:F625"/>
     <mergeCell ref="B923:F923"/>
     <mergeCell ref="B1054:F1054"/>
@@ -26996,6 +27271,7 @@
     <mergeCell ref="B1352:F1352"/>
     <mergeCell ref="B320:F320"/>
     <mergeCell ref="B1083:F1083"/>
+    <mergeCell ref="B1383:F1383"/>
     <mergeCell ref="B38:F38"/>
     <mergeCell ref="B467:F467"/>
     <mergeCell ref="B40:F40"/>
@@ -27033,6 +27309,7 @@
     <mergeCell ref="B710:F710"/>
     <mergeCell ref="B1348:F1348"/>
     <mergeCell ref="B868:F868"/>
+    <mergeCell ref="B1384:F1384"/>
     <mergeCell ref="B107:F107"/>
     <mergeCell ref="B1160:F1160"/>
     <mergeCell ref="B1377:F1377"/>
@@ -27056,6 +27333,7 @@
     <mergeCell ref="B39:F39"/>
     <mergeCell ref="B1092:F1092"/>
     <mergeCell ref="A961:F961"/>
+    <mergeCell ref="B1392:F1392"/>
     <mergeCell ref="B178:F178"/>
     <mergeCell ref="B476:F476"/>
     <mergeCell ref="B818:F818"/>
@@ -27347,6 +27625,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1349" r:id="rId90"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1364" r:id="rId91"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1379" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1394" r:id="rId93"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -27358,7 +27637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J93"/>
+  <dimension ref="A1:J94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -27980,12 +28259,12 @@
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-07-D1-01</t>
+          <t>HORIZON-CL5-2026-08-Two-Stage-D1-06</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Next generation climate monitoring and related capabilities</t>
+          <t>Closing knowledge gaps on Earth system science in support of</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -28020,12 +28299,12 @@
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-08-Two-Stage-D1-06</t>
+          <t>HORIZON-CL5-2026-07-D1-01</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Closing knowledge gaps on Earth system science in support of</t>
+          <t>Next generation climate monitoring and related capabilities</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -28060,12 +28339,12 @@
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-07-D1-04</t>
+          <t>HORIZON-CL5-2026-07-D1-05</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Fighting disinformation and effectively communicating on cli</t>
+          <t>Improving climate and weather models for Africa</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -28100,12 +28379,12 @@
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-07-D1-05</t>
+          <t>HORIZON-CL5-2026-07-D1-04</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Improving climate and weather models for Africa</t>
+          <t>Fighting disinformation and effectively communicating on cli</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -28656,12 +28935,12 @@
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-13</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>Next generation scenarios for informing climate and sustaina</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -28696,12 +28975,12 @@
     <row r="34" ht="28" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Advancing understanding, modelling and prediction of extreme</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
@@ -28736,12 +29015,12 @@
     <row r="35" ht="28" customHeight="1">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Assessing the performance of policy instruments to inform cl</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -28776,12 +29055,12 @@
     <row r="36" ht="28" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-13</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme</t>
+          <t>Next generation scenarios for informing climate and sustaina</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -28816,12 +29095,12 @@
     <row r="37" ht="28" customHeight="1">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform cl</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
@@ -29880,7 +30159,7 @@
     <row r="66" ht="28" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>dc0033a0-cb94-44ed-8102-0fd0a386989e-EXA</t>
+          <t>4b45d249-5739-4bf7-9595-a4715b73c2f6-EXA</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
@@ -29912,7 +30191,7 @@
     <row r="67" ht="28" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>4b45d249-5739-4bf7-9595-a4715b73c2f6-EXA</t>
+          <t>dc0033a0-cb94-44ed-8102-0fd0a386989e-EXA</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
@@ -30016,12 +30295,12 @@
     <row r="70" ht="28" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>EUS-74373</t>
+          <t>EUS-74952</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ayudas a proyectos al amparo de la estrategia de desarrollo </t>
+          <t>Servicio de transporte y reparto de comida desde las cocinas</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -30037,7 +30316,7 @@
       <c r="E70" s="6" t="inlineStr"/>
       <c r="F70" s="27" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>MUY ALTA</t>
         </is>
       </c>
       <c r="G70" s="6" t="inlineStr"/>
@@ -30052,12 +30331,12 @@
     <row r="71" ht="28" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>EUS-13151</t>
+          <t>EUS-31018</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>ReSourceEU y materias primas críticas: la UE sigue tramitand</t>
+          <t xml:space="preserve">Ayudas a proyectos al amparo de la estrategia de desarrollo </t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -30088,12 +30367,12 @@
     <row r="72" ht="28" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>EUS-33319</t>
+          <t>EUS-53900</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>Ciudades sostenibles: los Premios Capital Verde Europea y Ho</t>
+          <t>ReSourceEU y materias primas críticas: la UE sigue tramitand</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -30124,12 +30403,12 @@
     <row r="73" ht="28" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>EUS-06487</t>
+          <t>EUS-66315</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>Presolicitud para programa de ayudas a empresas que realicen</t>
+          <t>Ciudades sostenibles: los Premios Capital Verde Europea y Ho</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -30160,12 +30439,12 @@
     <row r="74" ht="28" customHeight="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>EUS-05566</t>
+          <t>EUS-81441</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de</t>
+          <t>Presolicitud para programa de ayudas a empresas que realicen</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
@@ -30181,7 +30460,7 @@
       <c r="E74" s="6" t="inlineStr"/>
       <c r="F74" s="27" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="G74" s="6" t="inlineStr"/>
@@ -30196,12 +30475,12 @@
     <row r="75" ht="28" customHeight="1">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>EUS-49036</t>
+          <t>EUS-88586</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinanc</t>
+          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
@@ -30232,12 +30511,12 @@
     <row r="76" ht="28" customHeight="1">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>EUS-84033</t>
+          <t>EUS-91314</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>Digital Europe, Horizon (programas de la UE). Apoyos para co</t>
+          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinanc</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
@@ -30268,12 +30547,12 @@
     <row r="77" ht="28" customHeight="1">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>EUS-55512</t>
+          <t>EUS-84020</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para c</t>
+          <t>Digital Europe, Horizon (programas de la UE). Apoyos para co</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
@@ -30304,12 +30583,12 @@
     <row r="78" ht="28" customHeight="1">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>EUS-90444</t>
+          <t>EUS-18785</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>Política Agraria Común de la UE de 2026, y sus ayudas abiert</t>
+          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para c</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
@@ -30340,12 +30619,12 @@
     <row r="79" ht="28" customHeight="1">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>EUS-25327</t>
+          <t>EUS-44870</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>Programa de impulso a las ciudades y territorios inteligente</t>
+          <t>Política Agraria Común de la UE de 2026, y sus ayudas abiert</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
@@ -30376,12 +30655,12 @@
     <row r="80" ht="28" customHeight="1">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>EUS-73767</t>
+          <t>EUS-29143</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>Formación digital para empleabilidad turística: los fondos N</t>
+          <t>Programa de impulso a las ciudades y territorios inteligente</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
@@ -30412,12 +30691,12 @@
     <row r="81" ht="28" customHeight="1">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>EUS-54415</t>
+          <t>EUS-05166</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>Horizon Europe. Clúster digital, industrial y espacial. Apoy</t>
+          <t>Formación digital para empleabilidad turística: los fondos N</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
@@ -30448,12 +30727,12 @@
     <row r="82" ht="28" customHeight="1">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>EUS-27582</t>
+          <t>EUS-07020</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Horizon Europe: ayudas de la línea de energía del clúster 5 </t>
+          <t>Horizon Europe. Clúster digital, industrial y espacial. Apoy</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
@@ -30484,12 +30763,12 @@
     <row r="83" ht="28" customHeight="1">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>EUS-96937</t>
+          <t>EUS-58974</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>Azpitek 2026: Programa de Ayudas para la Adquisición, Instal</t>
+          <t xml:space="preserve">Horizon Europe: ayudas de la línea de energía del clúster 5 </t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
@@ -30520,12 +30799,12 @@
     <row r="84" ht="28" customHeight="1">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>EUS-68824</t>
+          <t>EUS-81341</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>Subvenciones para innovación en economía circular 2026</t>
+          <t>Azpitek 2026: Programa de Ayudas para la Adquisición, Instal</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
@@ -30556,12 +30835,12 @@
     <row r="85" ht="28" customHeight="1">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>EUS-21415</t>
+          <t>EUS-61815</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>Horizon Europe 2026-27: convocatorias ligadas a misiones amb</t>
+          <t>Subvenciones para innovación en economía circular 2026</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
@@ -30592,12 +30871,12 @@
     <row r="86" ht="28" customHeight="1">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>EUS-12091</t>
+          <t>EUS-61141</t>
         </is>
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>Escudo Europeo de la Democracia: ayudas a proyectos de alfab</t>
+          <t>Horizon Europe 2026-27: convocatorias ligadas a misiones amb</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
@@ -30628,12 +30907,12 @@
     <row r="87" ht="28" customHeight="1">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>EUS-29046</t>
+          <t>EUS-33047</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>KSI Berritzaile Plus: ayudas del Gobierno Vasco a las Indust</t>
+          <t>Escudo Europeo de la Democracia: ayudas a proyectos de alfab</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
@@ -30664,12 +30943,12 @@
     <row r="88" ht="28" customHeight="1">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>EUS-78377</t>
+          <t>EUS-49824</t>
         </is>
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>Desmontaje de dos depósitos de agua en local del polideporti</t>
+          <t>KSI Berritzaile Plus: ayudas del Gobierno Vasco a las Indust</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
@@ -30700,12 +30979,12 @@
     <row r="89" ht="28" customHeight="1">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>EUS-16975</t>
+          <t>EUS-83207</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>Reparación del ascensor exterior de urki polonia tras entrad</t>
+          <t>Desmontaje de dos depósitos de agua en local del polideporti</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
@@ -30736,12 +31015,12 @@
     <row r="90" ht="28" customHeight="1">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>EUS-54763</t>
+          <t>EUS-43218</t>
         </is>
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>Desatasco tanto de la red de pluviales como de la de fecales</t>
+          <t>Reparación del ascensor exterior de urki polonia tras entrad</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
@@ -30772,12 +31051,12 @@
     <row r="91" ht="28" customHeight="1">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>EUS-00010</t>
+          <t>EUS-03214</t>
         </is>
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>Contratación de la actuación de unos bertsolaris el 8 y 14 d</t>
+          <t>Desatasco tanto de la red de pluviales como de la de fecales</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
@@ -30808,12 +31087,12 @@
     <row r="92" ht="28" customHeight="1">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>EUS-50530</t>
+          <t>EUS-68824</t>
         </is>
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Suministro de botellines de agua mineral para atender a los </t>
+          <t>Contratación de la actuación de unos bertsolaris el 8 y 14 d</t>
         </is>
       </c>
       <c r="C92" s="6" t="inlineStr">
@@ -30844,12 +31123,12 @@
     <row r="93" ht="28" customHeight="1">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>EUS-28619</t>
+          <t>EUS-26937</t>
         </is>
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>Servicio de organización de la sesión de bertsolaris de arra</t>
+          <t xml:space="preserve">Suministro de botellines de agua mineral para atender a los </t>
         </is>
       </c>
       <c r="C93" s="6" t="inlineStr">
@@ -30877,8 +31156,44 @@
       <c r="I93" s="6" t="inlineStr"/>
       <c r="J93" s="6" t="inlineStr"/>
     </row>
+    <row r="94" ht="28" customHeight="1">
+      <c r="A94" s="6" t="inlineStr">
+        <is>
+          <t>EUS-27498</t>
+        </is>
+      </c>
+      <c r="B94" s="6" t="inlineStr">
+        <is>
+          <t>Servicio de organización de la sesión de bertsolaris de arra</t>
+        </is>
+      </c>
+      <c r="C94" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D94" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E94" s="6" t="inlineStr"/>
+      <c r="F94" s="27" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G94" s="6" t="inlineStr"/>
+      <c r="H94" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I94" s="6" t="inlineStr"/>
+      <c r="J94" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J93"/>
+  <autoFilter ref="A1:J94"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update funding data 2026-03-02
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Recursos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$100</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$95</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -679,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M100"/>
+  <dimension ref="A1:M101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -707,7 +707,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 01/03/2026 07:52 - 93 convocatorias - 24 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 02/03/2026 08:04 - 94 convocatorias - 26 nuevas</t>
         </is>
       </c>
     </row>
@@ -1214,12 +1214,12 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>INNOVFUND-2025-NZT-GENERAL-SSP</t>
+          <t>INNOVFUND-2025-NZT-GENERAL-MSP</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Small-Scale Projects</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Medium-Scale Projects</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -1255,7 +1255,7 @@
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Small-Scale Projects</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Medium-Scale Projects</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr"/>
@@ -1273,12 +1273,12 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>INNOVFUND-2025-NZT-GENERAL-LSP</t>
+          <t>INNOVFUND-2025-NZT-GENERAL-SSP</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Large-Scale Projects</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Small-Scale Projects</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Large-Scale Projects</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Small-Scale Projects</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr"/>
@@ -1332,12 +1332,12 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>INNOVFUND-2025-NZT-GENERAL-MSP</t>
+          <t>INNOVFUND-2025-NZT-GENERAL-LSP</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Medium-Scale Projects</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Large-Scale Projects</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -1373,7 +1373,7 @@
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Medium-Scale Projects</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Large-Scale Projects</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr"/>
@@ -1627,12 +1627,12 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-08-Two-Stage-D1-06</t>
+          <t>HORIZON-CL5-2026-07-D1-01</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Closing knowledge gaps on Earth system science in support of global and regional assessments and climate policy</t>
+          <t>Next generation climate monitoring and related capabilities</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -1652,7 +1652,7 @@
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>5,000,000 - 9,000,000</t>
+          <t>4,000,000</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
@@ -1672,7 +1672,7 @@
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to some of the following expected outcomes:Improved quality and reduced uncertainty of global and regional climate change projections;Critic</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Climate data are improved both spatially and temporally, physically more consistent and better exp</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr"/>
@@ -1690,12 +1690,12 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-07-D1-01</t>
+          <t>HORIZON-CL5-2026-08-Two-Stage-D1-06</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Next generation climate monitoring and related capabilities</t>
+          <t>Closing knowledge gaps on Earth system science in support of global and regional assessments and climate policy</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>4,000,000</t>
+          <t>5,000,000 - 9,000,000</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="K21" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Climate data are improved both spatially and temporally, physically more consistent and better exp</t>
+          <t>Expected Outcome:Project results are expected to contribute to some of the following expected outcomes:Improved quality and reduced uncertainty of global and regional climate change projections;Critic</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr"/>
@@ -1753,12 +1753,12 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-07-D1-05</t>
+          <t>HORIZON-CL5-2026-07-D1-04</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Improving climate and weather models for Africa</t>
+          <t>Fighting disinformation and effectively communicating on climate change</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved quality and performance of weather and climate models over Africa, tailored to the contin</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Advanced knowledge and understanding on the dynamics of disinformation affecting climate policy an</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr"/>
@@ -1816,12 +1816,12 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-07-D1-04</t>
+          <t>HORIZON-CL5-2026-07-D1-05</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Fighting disinformation and effectively communicating on climate change</t>
+          <t>Improving climate and weather models for Africa</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="K23" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Advanced knowledge and understanding on the dynamics of disinformation affecting climate policy an</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved quality and performance of weather and climate models over Africa, tailored to the contin</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr"/>
@@ -2686,12 +2686,12 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-13</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Next generation scenarios for informing climate and sustainability transitions</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="K37" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorpo</t>
+          <t>Expected Outcome:Project results are expected to contribute to some of the following expected outcomes:Strengthened collaboration and integration across research communities, better capturing interact</t>
         </is>
       </c>
       <c r="L37" s="6" t="inlineStr"/>
@@ -2749,12 +2749,12 @@
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -2779,7 +2779,7 @@
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Research and Innovation Actions</t>
+          <t>Programme Cofund Actions</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="K38" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Euro</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is estab</t>
         </is>
       </c>
       <c r="L38" s="6" t="inlineStr"/>
@@ -2812,12 +2812,12 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -2857,7 +2857,7 @@
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to info</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorpo</t>
         </is>
       </c>
       <c r="L39" s="6" t="inlineStr"/>
@@ -2875,12 +2875,12 @@
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-13</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Next generation scenarios for informing climate and sustainability transitions</t>
+          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -2920,7 +2920,7 @@
       </c>
       <c r="K40" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to some of the following expected outcomes:Strengthened collaboration and integration across research communities, better capturing interact</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Euro</t>
         </is>
       </c>
       <c r="L40" s="6" t="inlineStr"/>
@@ -2938,12 +2938,12 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -2968,7 +2968,7 @@
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>Programme Cofund Actions</t>
+          <t xml:space="preserve"> Research and Innovation Actions</t>
         </is>
       </c>
       <c r="I41" s="11" t="inlineStr">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="K41" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is estab</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to info</t>
         </is>
       </c>
       <c r="L41" s="6" t="inlineStr"/>
@@ -4779,7 +4779,7 @@
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>EUS-74952</t>
+          <t>EUS-80078</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
@@ -4834,7 +4834,7 @@
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>EUS-31018</t>
+          <t>EUS-96450</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
@@ -4889,7 +4889,7 @@
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>EUS-53900</t>
+          <t>EUS-17669</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>EUS-66315</t>
+          <t>EUS-02163</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
@@ -4999,7 +4999,7 @@
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>EUS-81441</t>
+          <t>EUS-45408</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
@@ -5054,12 +5054,12 @@
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>EUS-88586</t>
+          <t>EUS-49463</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de aceleración de proyectos, a localidades de menos de 20.000 habitantes son objeto de convocatoria abierta hasta el 17.03.26. Transformacione</t>
+          <t>Suministro de contenedores para la recogida de residuos municipales mezclados correspondiente a la fracción resto, suministro de cerraduras electrónicas y su instalación en los contenedores, suministr</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
@@ -5076,12 +5076,12 @@
       <c r="G81" s="6" t="inlineStr"/>
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
-        </is>
-      </c>
-      <c r="I81" s="10" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I81" s="8" t="inlineStr">
+        <is>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="J81" s="6" t="inlineStr"/>
@@ -5109,12 +5109,12 @@
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>EUS-91314</t>
+          <t>EUS-95091</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinancia convocatorias de ayudas de las Diputaciones a explotaciones con limitaciones o desfavorecidas, y a compromisos medioambientales, climátic</t>
+          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de aceleración de proyectos, a localidades de menos de 20.000 habitantes son objeto de convocatoria abierta hasta el 17.03.26. Transformacione</t>
         </is>
       </c>
       <c r="D82" s="6" t="inlineStr">
@@ -5164,12 +5164,12 @@
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>EUS-84020</t>
+          <t>EUS-77783</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>Digital Europe, Horizon (programas de la UE). Apoyos para consorcios interestatales de I+D+i. IA, robótica, cuántica, computación, ciberseguridad, electrónica, fotónica, TICs e internet avanzadas, esp</t>
+          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinancia convocatorias de ayudas de las Diputaciones a explotaciones con limitaciones o desfavorecidas, y a compromisos medioambientales, climátic</t>
         </is>
       </c>
       <c r="D83" s="6" t="inlineStr">
@@ -5219,12 +5219,12 @@
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>EUS-18785</t>
+          <t>EUS-01590</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para consorcios internacionales de I+D+i. Jornada del Gobierno Vasco y con Enterprise Europe Network y otros socios. Digitalización, dispositivos,</t>
+          <t>Digital Europe, Horizon (programas de la UE). Apoyos para consorcios interestatales de I+D+i. IA, robótica, cuántica, computación, ciberseguridad, electrónica, fotónica, TICs e internet avanzadas, esp</t>
         </is>
       </c>
       <c r="D84" s="6" t="inlineStr">
@@ -5274,12 +5274,12 @@
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>EUS-44870</t>
+          <t>EUS-07292</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>Política Agraria Común de la UE de 2026, y sus ayudas abiertas hasta el 30.4.26: el pilar 1, con el Fondo Europeo Agrícola de Garantía Agraria FEAGA, aborda sostenibilidad de renta, ayuda redistributi</t>
+          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para consorcios internacionales de I+D+i. Jornada del Gobierno Vasco y con Enterprise Europe Network y otros socios. Digitalización, dispositivos,</t>
         </is>
       </c>
       <c r="D85" s="6" t="inlineStr">
@@ -5329,12 +5329,12 @@
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>EUS-29143</t>
+          <t>EUS-75051</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>Programa de impulso a las ciudades y territorios inteligentes para el fomento del desarrollo económico y productivo, que podrá ser cofinanciado por el Programa Plurirregional 2021-2027 del Fondo Europ</t>
+          <t>Política Agraria Común de la UE de 2026, y sus ayudas abiertas hasta el 30.4.26: el pilar 1, con el Fondo Europeo Agrícola de Garantía Agraria FEAGA, aborda sostenibilidad de renta, ayuda redistributi</t>
         </is>
       </c>
       <c r="D86" s="6" t="inlineStr">
@@ -5384,12 +5384,12 @@
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>EUS-05166</t>
+          <t>EUS-61906</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>Formación digital para empleabilidad turística: los fondos Next de la UE apoyan una convocatoria de Lanbide y el Gobierno Vasco, de cursos en línea para mejorar las competencias del sector y de sus py</t>
+          <t>Programa de impulso a las ciudades y territorios inteligentes para el fomento del desarrollo económico y productivo, que podrá ser cofinanciado por el Programa Plurirregional 2021-2027 del Fondo Europ</t>
         </is>
       </c>
       <c r="D87" s="6" t="inlineStr">
@@ -5439,12 +5439,12 @@
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>EUS-07020</t>
+          <t>EUS-41118</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Horizon Europe. Clúster digital, industrial y espacial. Apoyos a proyectos para tecnologías de inteligencia artificial, internet, mundos virtuales, robótica, cuántica, fotónica, materias primas, bajo </t>
+          <t>Formación digital para empleabilidad turística: los fondos Next de la UE apoyan una convocatoria de Lanbide y el Gobierno Vasco, de cursos en línea para mejorar las competencias del sector y de sus py</t>
         </is>
       </c>
       <c r="D88" s="6" t="inlineStr">
@@ -5494,12 +5494,12 @@
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>EUS-58974</t>
+          <t>EUS-29727</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>Horizon Europe: ayudas de la línea de energía del clúster 5 y de la Misión Ciudades. Jornada informativa sobre estas y otras iniciativas en colaboración transestatal para la doble transición ecológica</t>
+          <t xml:space="preserve">Horizon Europe. Clúster digital, industrial y espacial. Apoyos a proyectos para tecnologías de inteligencia artificial, internet, mundos virtuales, robótica, cuántica, fotónica, materias primas, bajo </t>
         </is>
       </c>
       <c r="D89" s="6" t="inlineStr">
@@ -5549,12 +5549,12 @@
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>EUS-81341</t>
+          <t>EUS-72731</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>Azpitek 2026: Programa de Ayudas para la Adquisición, Instalación, Renovación y Actualización de Infraestructuras de Investigación</t>
+          <t>Horizon Europe: ayudas de la línea de energía del clúster 5 y de la Misión Ciudades. Jornada informativa sobre estas y otras iniciativas en colaboración transestatal para la doble transición ecológica</t>
         </is>
       </c>
       <c r="D90" s="6" t="inlineStr">
@@ -5604,12 +5604,12 @@
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>EUS-61815</t>
+          <t>EUS-03084</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>Subvenciones para innovación en economía circular 2026</t>
+          <t>Azpitek 2026: Programa de Ayudas para la Adquisición, Instalación, Renovación y Actualización de Infraestructuras de Investigación</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr">
@@ -5659,12 +5659,12 @@
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>EUS-61141</t>
+          <t>EUS-78189</t>
         </is>
       </c>
       <c r="C92" s="6" t="inlineStr">
         <is>
-          <t>Horizon Europe 2026-27: convocatorias ligadas a misiones ambientales de la UE, partenariados de economía circular, azul o bio, o a la división alimentaria EIT Food del Instituto Europeo de Tecnología,</t>
+          <t>Subvenciones para innovación en economía circular 2026</t>
         </is>
       </c>
       <c r="D92" s="6" t="inlineStr">
@@ -5714,12 +5714,12 @@
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>EUS-33047</t>
+          <t>EUS-96006</t>
         </is>
       </c>
       <c r="C93" s="6" t="inlineStr">
         <is>
-          <t>Escudo Europeo de la Democracia: ayudas a proyectos de alfabetización mediática y fomento del diálogo y la comprensión en torno a la desinformación digital</t>
+          <t>Horizon Europe 2026-27: convocatorias ligadas a misiones ambientales de la UE, partenariados de economía circular, azul o bio, o a la división alimentaria EIT Food del Instituto Europeo de Tecnología,</t>
         </is>
       </c>
       <c r="D93" s="6" t="inlineStr">
@@ -5769,12 +5769,12 @@
       </c>
       <c r="B94" s="6" t="inlineStr">
         <is>
-          <t>EUS-49824</t>
+          <t>EUS-37801</t>
         </is>
       </c>
       <c r="C94" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">KSI Berritzaile Plus: ayudas del Gobierno Vasco a las Industrias Culturales y Creativas para proyectos innovadores en la triple transición tecnológico-digital, energético-climática y socio-sanitaria, </t>
+          <t>Escudo Europeo de la Democracia: ayudas a proyectos de alfabetización mediática y fomento del diálogo y la comprensión en torno a la desinformación digital</t>
         </is>
       </c>
       <c r="D94" s="6" t="inlineStr">
@@ -5824,12 +5824,12 @@
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>EUS-83207</t>
+          <t>EUS-98075</t>
         </is>
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>Desmontaje de dos depósitos de agua en local del polideportivo ipurua y tuberías que lo alimentan.</t>
+          <t xml:space="preserve">KSI Berritzaile Plus: ayudas del Gobierno Vasco a las Industrias Culturales y Creativas para proyectos innovadores en la triple transición tecnológico-digital, energético-climática y socio-sanitaria, </t>
         </is>
       </c>
       <c r="D95" s="6" t="inlineStr">
@@ -5846,7 +5846,7 @@
       <c r="G95" s="6" t="inlineStr"/>
       <c r="H95" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="I95" s="10" t="inlineStr">
@@ -5879,12 +5879,12 @@
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>EUS-43218</t>
+          <t>EUS-37368</t>
         </is>
       </c>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>Reparación del ascensor exterior de urki polonia tras entrada agua en cuadro</t>
+          <t>Mantenimiento de los servidores instalados en el edificio Onkologikoa (OSI Donostialdea)</t>
         </is>
       </c>
       <c r="D96" s="6" t="inlineStr">
@@ -5934,12 +5934,12 @@
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>EUS-03214</t>
+          <t>EUS-78987</t>
         </is>
       </c>
       <c r="C97" s="6" t="inlineStr">
         <is>
-          <t>Desatasco tanto de la red de pluviales como de la de fecales de errebal plazia</t>
+          <t>Gestión del servicio público de transporte colectivo urbano de Tolosa</t>
         </is>
       </c>
       <c r="D97" s="6" t="inlineStr">
@@ -5989,12 +5989,12 @@
       </c>
       <c r="B98" s="6" t="inlineStr">
         <is>
-          <t>EUS-68824</t>
+          <t>EUS-25969</t>
         </is>
       </c>
       <c r="C98" s="6" t="inlineStr">
         <is>
-          <t>Contratación de la actuación de unos bertsolaris el 8 y 14 de septiembre en el marco de las fiestas de ntra. sra. de arrate</t>
+          <t>Desmontaje de dos depósitos de agua en local del polideportivo ipurua y tuberías que lo alimentan.</t>
         </is>
       </c>
       <c r="D98" s="6" t="inlineStr">
@@ -6025,7 +6025,11 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L98" s="6" t="inlineStr"/>
+      <c r="L98" s="17" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
       <c r="M98" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
@@ -6040,12 +6044,12 @@
       </c>
       <c r="B99" s="6" t="inlineStr">
         <is>
-          <t>EUS-26937</t>
+          <t>EUS-14012</t>
         </is>
       </c>
       <c r="C99" s="6" t="inlineStr">
         <is>
-          <t>Suministro de botellines de agua mineral para atender a los grupos que actúan en el teatro coliseo</t>
+          <t>Reparación del ascensor exterior de urki polonia tras entrada agua en cuadro</t>
         </is>
       </c>
       <c r="D99" s="6" t="inlineStr">
@@ -6095,12 +6099,12 @@
       </c>
       <c r="B100" s="6" t="inlineStr">
         <is>
-          <t>EUS-27498</t>
+          <t>EUS-79105</t>
         </is>
       </c>
       <c r="C100" s="6" t="inlineStr">
         <is>
-          <t>Servicio de organización de la sesión de bertsolaris de arrate del 7 de septiembre.</t>
+          <t>Desatasco tanto de la red de pluviales como de la de fecales de errebal plazia</t>
         </is>
       </c>
       <c r="D100" s="6" t="inlineStr">
@@ -6142,8 +6146,63 @@
         </is>
       </c>
     </row>
+    <row r="101" ht="40" customHeight="1">
+      <c r="A101" s="16" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B101" s="6" t="inlineStr">
+        <is>
+          <t>EUS-32322</t>
+        </is>
+      </c>
+      <c r="C101" s="6" t="inlineStr">
+        <is>
+          <t>Contratación de la actuación de unos bertsolaris el 8 y 14 de septiembre en el marco de las fiestas de ntra. sra. de arrate</t>
+        </is>
+      </c>
+      <c r="D101" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E101" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F101" s="6" t="inlineStr"/>
+      <c r="G101" s="6" t="inlineStr"/>
+      <c r="H101" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I101" s="10" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J101" s="6" t="inlineStr"/>
+      <c r="K101" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L101" s="17" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M101" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:M100"/>
+  <autoFilter ref="A4:M101"/>
   <mergeCells count="5">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A75:M75"/>
@@ -6245,6 +6304,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M98" r:id="rId91"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M99" r:id="rId92"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M100" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M101" r:id="rId94"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6256,7 +6316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1394"/>
+  <dimension ref="A1:F1409"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7794,7 +7854,7 @@
     <row r="106" ht="30" customHeight="1">
       <c r="A106" s="18" t="inlineStr">
         <is>
-          <t>FICHA 8: INNOVFUND-2025-NZT-GENERAL-SSP</t>
+          <t>FICHA 8: INNOVFUND-2025-NZT-GENERAL-MSP</t>
         </is>
       </c>
       <c r="B106" s="19" t="n"/>
@@ -7827,7 +7887,7 @@
       </c>
       <c r="B108" s="21" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Small-Scale Projects</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Medium-Scale Projects</t>
         </is>
       </c>
       <c r="C108" s="22" t="n"/>
@@ -7843,7 +7903,7 @@
       </c>
       <c r="B109" s="21" t="inlineStr">
         <is>
-          <t>INNOVFUND-2025-NZT-GENERAL-SSP</t>
+          <t>INNOVFUND-2025-NZT-GENERAL-MSP</t>
         </is>
       </c>
       <c r="C109" s="22" t="n"/>
@@ -7955,7 +8015,7 @@
       </c>
       <c r="B116" s="21" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Small-Scale Projects</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Medium-Scale Projects</t>
         </is>
       </c>
       <c r="C116" s="22" t="n"/>
@@ -8003,7 +8063,7 @@
       </c>
       <c r="B119" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/INNOVFUND-2025-NZT-GENERAL-SSP</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/INNOVFUND-2025-NZT-GENERAL-MSP</t>
         </is>
       </c>
       <c r="C119" s="22" t="n"/>
@@ -8014,7 +8074,7 @@
     <row r="121" ht="30" customHeight="1">
       <c r="A121" s="18" t="inlineStr">
         <is>
-          <t>FICHA 9: INNOVFUND-2025-NZT-GENERAL-LSP</t>
+          <t>FICHA 9: INNOVFUND-2025-NZT-GENERAL-SSP</t>
         </is>
       </c>
       <c r="B121" s="19" t="n"/>
@@ -8047,7 +8107,7 @@
       </c>
       <c r="B123" s="21" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Large-Scale Projects</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Small-Scale Projects</t>
         </is>
       </c>
       <c r="C123" s="22" t="n"/>
@@ -8063,7 +8123,7 @@
       </c>
       <c r="B124" s="21" t="inlineStr">
         <is>
-          <t>INNOVFUND-2025-NZT-GENERAL-LSP</t>
+          <t>INNOVFUND-2025-NZT-GENERAL-SSP</t>
         </is>
       </c>
       <c r="C124" s="22" t="n"/>
@@ -8175,7 +8235,7 @@
       </c>
       <c r="B131" s="21" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Large-Scale Projects</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Small-Scale Projects</t>
         </is>
       </c>
       <c r="C131" s="22" t="n"/>
@@ -8223,7 +8283,7 @@
       </c>
       <c r="B134" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/INNOVFUND-2025-NZT-GENERAL-LSP</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/INNOVFUND-2025-NZT-GENERAL-SSP</t>
         </is>
       </c>
       <c r="C134" s="22" t="n"/>
@@ -8234,7 +8294,7 @@
     <row r="136" ht="30" customHeight="1">
       <c r="A136" s="18" t="inlineStr">
         <is>
-          <t>FICHA 10: INNOVFUND-2025-NZT-GENERAL-MSP</t>
+          <t>FICHA 10: INNOVFUND-2025-NZT-GENERAL-LSP</t>
         </is>
       </c>
       <c r="B136" s="19" t="n"/>
@@ -8267,7 +8327,7 @@
       </c>
       <c r="B138" s="21" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Medium-Scale Projects</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Large-Scale Projects</t>
         </is>
       </c>
       <c r="C138" s="22" t="n"/>
@@ -8283,7 +8343,7 @@
       </c>
       <c r="B139" s="21" t="inlineStr">
         <is>
-          <t>INNOVFUND-2025-NZT-GENERAL-MSP</t>
+          <t>INNOVFUND-2025-NZT-GENERAL-LSP</t>
         </is>
       </c>
       <c r="C139" s="22" t="n"/>
@@ -8395,7 +8455,7 @@
       </c>
       <c r="B146" s="21" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Medium-Scale Projects</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Large-Scale Projects</t>
         </is>
       </c>
       <c r="C146" s="22" t="n"/>
@@ -8443,7 +8503,7 @@
       </c>
       <c r="B149" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/INNOVFUND-2025-NZT-GENERAL-MSP</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/INNOVFUND-2025-NZT-GENERAL-LSP</t>
         </is>
       </c>
       <c r="C149" s="22" t="n"/>
@@ -9318,7 +9378,7 @@
     <row r="211" ht="30" customHeight="1">
       <c r="A211" s="18" t="inlineStr">
         <is>
-          <t>FICHA 15: HORIZON-CL5-2026-08-Two-Stage-D1-06</t>
+          <t>FICHA 15: HORIZON-CL5-2026-07-D1-01</t>
         </is>
       </c>
       <c r="B211" s="19" t="n"/>
@@ -9343,7 +9403,7 @@
       <c r="E212" s="22" t="n"/>
       <c r="F212" s="22" t="n"/>
     </row>
-    <row r="213" ht="45" customHeight="1">
+    <row r="213" ht="20" customHeight="1">
       <c r="A213" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -9351,7 +9411,7 @@
       </c>
       <c r="B213" s="21" t="inlineStr">
         <is>
-          <t>Closing knowledge gaps on Earth system science in support of global and regional assessments and climate policy</t>
+          <t>Next generation climate monitoring and related capabilities</t>
         </is>
       </c>
       <c r="C213" s="22" t="n"/>
@@ -9367,7 +9427,7 @@
       </c>
       <c r="B214" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-08-Two-Stage-D1-06</t>
+          <t>HORIZON-CL5-2026-07-D1-01</t>
         </is>
       </c>
       <c r="C214" s="22" t="n"/>
@@ -9431,7 +9491,7 @@
       </c>
       <c r="B218" s="21" t="inlineStr">
         <is>
-          <t>5,000,000 - 9,000,000</t>
+          <t>4,000,000</t>
         </is>
       </c>
       <c r="C218" s="22" t="n"/>
@@ -9463,7 +9523,7 @@
       </c>
       <c r="B220" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-08-Two-Stage</t>
+          <t>HORIZON-CL5-2026-07</t>
         </is>
       </c>
       <c r="C220" s="22" t="n"/>
@@ -9479,7 +9539,7 @@
       </c>
       <c r="B221" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to some of the following expected outcomes:Improved quality and reduced uncertainty of global and regional climate change projections;Critical knowledge and data gaps in Earth system science as identified in the IPCC Sixth Assessment Report (AR6) and other authoritative sources, are addressed, ensuring that future climate assessments are grounded in the most comprehensive and up-to-date scientific evidence;New climate science evidence is generated that is relevant for policy needs and for informing climate action. Scope:The global com</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Climate data are improved both spatially and temporally, physically more consistent and better exploited across a wide range of users, stakeholders and regions;The EU climate data sovereignty is strengthened, with enhanced EU contribution to climate monitoring and climate change assessments;Climate information distillation is facilitated by innovative methods to provide useful information to policy making in a more efficient way. Scope:Climate monitoring of Essential Climate Variables[1] at gl</t>
         </is>
       </c>
       <c r="C221" s="22" t="n"/>
@@ -9523,7 +9583,7 @@
       </c>
       <c r="B224" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-08-Two-Stage-D1-06</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-07-D1-01</t>
         </is>
       </c>
       <c r="C224" s="22" t="n"/>
@@ -9534,7 +9594,7 @@
     <row r="226" ht="30" customHeight="1">
       <c r="A226" s="18" t="inlineStr">
         <is>
-          <t>FICHA 16: HORIZON-CL5-2026-07-D1-01</t>
+          <t>FICHA 16: HORIZON-CL5-2026-08-Two-Stage-D1-06</t>
         </is>
       </c>
       <c r="B226" s="19" t="n"/>
@@ -9559,7 +9619,7 @@
       <c r="E227" s="22" t="n"/>
       <c r="F227" s="22" t="n"/>
     </row>
-    <row r="228" ht="20" customHeight="1">
+    <row r="228" ht="45" customHeight="1">
       <c r="A228" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -9567,7 +9627,7 @@
       </c>
       <c r="B228" s="21" t="inlineStr">
         <is>
-          <t>Next generation climate monitoring and related capabilities</t>
+          <t>Closing knowledge gaps on Earth system science in support of global and regional assessments and climate policy</t>
         </is>
       </c>
       <c r="C228" s="22" t="n"/>
@@ -9583,7 +9643,7 @@
       </c>
       <c r="B229" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-07-D1-01</t>
+          <t>HORIZON-CL5-2026-08-Two-Stage-D1-06</t>
         </is>
       </c>
       <c r="C229" s="22" t="n"/>
@@ -9647,7 +9707,7 @@
       </c>
       <c r="B233" s="21" t="inlineStr">
         <is>
-          <t>4,000,000</t>
+          <t>5,000,000 - 9,000,000</t>
         </is>
       </c>
       <c r="C233" s="22" t="n"/>
@@ -9679,7 +9739,7 @@
       </c>
       <c r="B235" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-07</t>
+          <t>HORIZON-CL5-2026-08-Two-Stage</t>
         </is>
       </c>
       <c r="C235" s="22" t="n"/>
@@ -9695,7 +9755,7 @@
       </c>
       <c r="B236" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Climate data are improved both spatially and temporally, physically more consistent and better exploited across a wide range of users, stakeholders and regions;The EU climate data sovereignty is strengthened, with enhanced EU contribution to climate monitoring and climate change assessments;Climate information distillation is facilitated by innovative methods to provide useful information to policy making in a more efficient way. Scope:Climate monitoring of Essential Climate Variables[1] at gl</t>
+          <t>Expected Outcome:Project results are expected to contribute to some of the following expected outcomes:Improved quality and reduced uncertainty of global and regional climate change projections;Critical knowledge and data gaps in Earth system science as identified in the IPCC Sixth Assessment Report (AR6) and other authoritative sources, are addressed, ensuring that future climate assessments are grounded in the most comprehensive and up-to-date scientific evidence;New climate science evidence is generated that is relevant for policy needs and for informing climate action. Scope:The global com</t>
         </is>
       </c>
       <c r="C236" s="22" t="n"/>
@@ -9739,7 +9799,7 @@
       </c>
       <c r="B239" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-07-D1-01</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-08-Two-Stage-D1-06</t>
         </is>
       </c>
       <c r="C239" s="22" t="n"/>
@@ -9750,7 +9810,7 @@
     <row r="241" ht="30" customHeight="1">
       <c r="A241" s="18" t="inlineStr">
         <is>
-          <t>FICHA 17: HORIZON-CL5-2026-07-D1-05</t>
+          <t>FICHA 17: HORIZON-CL5-2026-07-D1-04</t>
         </is>
       </c>
       <c r="B241" s="19" t="n"/>
@@ -9783,7 +9843,7 @@
       </c>
       <c r="B243" s="21" t="inlineStr">
         <is>
-          <t>Improving climate and weather models for Africa</t>
+          <t>Fighting disinformation and effectively communicating on climate change</t>
         </is>
       </c>
       <c r="C243" s="22" t="n"/>
@@ -9799,7 +9859,7 @@
       </c>
       <c r="B244" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-07-D1-05</t>
+          <t>HORIZON-CL5-2026-07-D1-04</t>
         </is>
       </c>
       <c r="C244" s="22" t="n"/>
@@ -9911,7 +9971,7 @@
       </c>
       <c r="B251" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved quality and performance of weather and climate models over Africa, tailored to the continent’s needs, enabling more effective adaptation actions and disaster risk response strategies, and informing the implementation of the international dimension of the EU Adaptation and Preparedness Union Strategies, the Sendai Framework for Disaster Risk Reduction, the Nairobi Declaration and the Team Europe Initiative on Adaptation and Resilience in Africa[1];Enhanced provision of weather predicti</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Advanced knowledge and understanding on the dynamics of disinformation affecting climate policy and climate policy backlash from a communication perspective;Tools and products are developed for public authorities, media and civil society to detect and combat the influence and spread of climate change-related disinformation at scale;Tailored, innovative and effective communication techniques, tools and materials are developed, tested and disseminated, to better communicate with and engage citiz</t>
         </is>
       </c>
       <c r="C251" s="22" t="n"/>
@@ -9955,7 +10015,7 @@
       </c>
       <c r="B254" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-07-D1-05</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-07-D1-04</t>
         </is>
       </c>
       <c r="C254" s="22" t="n"/>
@@ -9966,7 +10026,7 @@
     <row r="256" ht="30" customHeight="1">
       <c r="A256" s="18" t="inlineStr">
         <is>
-          <t>FICHA 18: HORIZON-CL5-2026-07-D1-04</t>
+          <t>FICHA 18: HORIZON-CL5-2026-07-D1-05</t>
         </is>
       </c>
       <c r="B256" s="19" t="n"/>
@@ -9999,7 +10059,7 @@
       </c>
       <c r="B258" s="21" t="inlineStr">
         <is>
-          <t>Fighting disinformation and effectively communicating on climate change</t>
+          <t>Improving climate and weather models for Africa</t>
         </is>
       </c>
       <c r="C258" s="22" t="n"/>
@@ -10015,7 +10075,7 @@
       </c>
       <c r="B259" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-07-D1-04</t>
+          <t>HORIZON-CL5-2026-07-D1-05</t>
         </is>
       </c>
       <c r="C259" s="22" t="n"/>
@@ -10127,7 +10187,7 @@
       </c>
       <c r="B266" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Advanced knowledge and understanding on the dynamics of disinformation affecting climate policy and climate policy backlash from a communication perspective;Tools and products are developed for public authorities, media and civil society to detect and combat the influence and spread of climate change-related disinformation at scale;Tailored, innovative and effective communication techniques, tools and materials are developed, tested and disseminated, to better communicate with and engage citiz</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved quality and performance of weather and climate models over Africa, tailored to the continent’s needs, enabling more effective adaptation actions and disaster risk response strategies, and informing the implementation of the international dimension of the EU Adaptation and Preparedness Union Strategies, the Sendai Framework for Disaster Risk Reduction, the Nairobi Declaration and the Team Europe Initiative on Adaptation and Resilience in Africa[1];Enhanced provision of weather predicti</t>
         </is>
       </c>
       <c r="C266" s="22" t="n"/>
@@ -10171,7 +10231,7 @@
       </c>
       <c r="B269" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-07-D1-04</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-07-D1-05</t>
         </is>
       </c>
       <c r="C269" s="22" t="n"/>
@@ -13022,7 +13082,7 @@
     <row r="466" ht="30" customHeight="1">
       <c r="A466" s="18" t="inlineStr">
         <is>
-          <t>FICHA 32: HORIZON-CL5-2027-01-D1-10</t>
+          <t>FICHA 32: HORIZON-CL5-2027-01-D1-13</t>
         </is>
       </c>
       <c r="B466" s="19" t="n"/>
@@ -13055,7 +13115,7 @@
       </c>
       <c r="B468" s="21" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Next generation scenarios for informing climate and sustainability transitions</t>
         </is>
       </c>
       <c r="C468" s="22" t="n"/>
@@ -13071,7 +13131,7 @@
       </c>
       <c r="B469" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-13</t>
         </is>
       </c>
       <c r="C469" s="22" t="n"/>
@@ -13183,7 +13243,7 @@
       </c>
       <c r="B476" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorporation into main EU repositories, such as Climate-ADAPT or the portal of the EU Mission on Adaptation to Climate Change;The risk and adaptation assessment frameworks are improved by better integrating the maladaptation dimension;Guidelines and tools for maladaptation prevention and correction strategies are made available to adaptation stakeholders at relevant scales and inform the design and impl</t>
+          <t>Expected Outcome:Project results are expected to contribute to some of the following expected outcomes:Strengthened collaboration and integration across research communities, better capturing interactions and trade-offs between various climate domains as well as between climate and non-climate objectives, such as biodiversity or pollution related. This will support more comprehensive and consistent evaluations, benefiting key global assessments (IPCC, IPBES) and improving their impact on European and global policies (European Green Deal, UNFCCC, CBD);More relevant, robust and actionable scenar</t>
         </is>
       </c>
       <c r="C476" s="22" t="n"/>
@@ -13227,7 +13287,7 @@
       </c>
       <c r="B479" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-10</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-13</t>
         </is>
       </c>
       <c r="C479" s="22" t="n"/>
@@ -13238,7 +13298,7 @@
     <row r="481" ht="30" customHeight="1">
       <c r="A481" s="18" t="inlineStr">
         <is>
-          <t>FICHA 33: HORIZON-CL5-2027-01-D1-07</t>
+          <t>FICHA 33: HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="B481" s="19" t="n"/>
@@ -13263,7 +13323,7 @@
       <c r="E482" s="22" t="n"/>
       <c r="F482" s="22" t="n"/>
     </row>
-    <row r="483" ht="45" customHeight="1">
+    <row r="483" ht="20" customHeight="1">
       <c r="A483" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -13271,7 +13331,7 @@
       </c>
       <c r="B483" s="21" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="C483" s="22" t="n"/>
@@ -13287,7 +13347,7 @@
       </c>
       <c r="B484" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C484" s="22" t="n"/>
@@ -13367,7 +13427,7 @@
       </c>
       <c r="B489" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Research and Innovation Actions</t>
+          <t>Programme Cofund Actions</t>
         </is>
       </c>
       <c r="C489" s="22" t="n"/>
@@ -13399,7 +13459,7 @@
       </c>
       <c r="B491" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Europe and globally, as well as the interaction between different hazards, their cumulative and/or cascading effects.Enhanced seamless prediction and projection modelling and attribution capabilities for extreme events and their likelihood to support preparedness, response and resilience to climate change by EU and national and regional actors. The EU Union Preparedness Strategy, the EU Adaptation Str</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is established through development and implementation of the Climate Action pillar of the EU-AU Research and Innovation Partnership on Climate Change and Sustainable Energy (CCSE),[1] in co-design between African and European partners;Reduced fragmentation by aligning the EU, national and multilateral R&amp;amp;I efforts with increased leverage and impact of funding;African scientific, policy and practice com</t>
         </is>
       </c>
       <c r="C491" s="22" t="n"/>
@@ -13443,7 +13503,7 @@
       </c>
       <c r="B494" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-07</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C494" s="22" t="n"/>
@@ -13454,7 +13514,7 @@
     <row r="496" ht="30" customHeight="1">
       <c r="A496" s="18" t="inlineStr">
         <is>
-          <t>FICHA 34: HORIZON-CL5-2027-01-D1-09</t>
+          <t>FICHA 34: HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="B496" s="19" t="n"/>
@@ -13479,7 +13539,7 @@
       <c r="E497" s="22" t="n"/>
       <c r="F497" s="22" t="n"/>
     </row>
-    <row r="498" ht="45" customHeight="1">
+    <row r="498" ht="20" customHeight="1">
       <c r="A498" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -13487,7 +13547,7 @@
       </c>
       <c r="B498" s="21" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="C498" s="22" t="n"/>
@@ -13503,7 +13563,7 @@
       </c>
       <c r="B499" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C499" s="22" t="n"/>
@@ -13615,7 +13675,7 @@
       </c>
       <c r="B506" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to inform mitigation action and policy improvements, ensuring a fair transition and social acceptability;Methodologies are developed and improved for ex-ante assessment and ex-post evaluation of greenhouse gas emission reductions from climate policies and measures;Strengthened collaboration and established networks between researchers, policy experts and government officials involved in designing and eva</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorporation into main EU repositories, such as Climate-ADAPT or the portal of the EU Mission on Adaptation to Climate Change;The risk and adaptation assessment frameworks are improved by better integrating the maladaptation dimension;Guidelines and tools for maladaptation prevention and correction strategies are made available to adaptation stakeholders at relevant scales and inform the design and impl</t>
         </is>
       </c>
       <c r="C506" s="22" t="n"/>
@@ -13659,7 +13719,7 @@
       </c>
       <c r="B509" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-09</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C509" s="22" t="n"/>
@@ -13670,7 +13730,7 @@
     <row r="511" ht="30" customHeight="1">
       <c r="A511" s="18" t="inlineStr">
         <is>
-          <t>FICHA 35: HORIZON-CL5-2027-01-D1-13</t>
+          <t>FICHA 35: HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="B511" s="19" t="n"/>
@@ -13695,7 +13755,7 @@
       <c r="E512" s="22" t="n"/>
       <c r="F512" s="22" t="n"/>
     </row>
-    <row r="513" ht="20" customHeight="1">
+    <row r="513" ht="45" customHeight="1">
       <c r="A513" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -13703,7 +13763,7 @@
       </c>
       <c r="B513" s="21" t="inlineStr">
         <is>
-          <t>Next generation scenarios for informing climate and sustainability transitions</t>
+          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
         </is>
       </c>
       <c r="C513" s="22" t="n"/>
@@ -13719,7 +13779,7 @@
       </c>
       <c r="B514" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-13</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C514" s="22" t="n"/>
@@ -13831,7 +13891,7 @@
       </c>
       <c r="B521" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to some of the following expected outcomes:Strengthened collaboration and integration across research communities, better capturing interactions and trade-offs between various climate domains as well as between climate and non-climate objectives, such as biodiversity or pollution related. This will support more comprehensive and consistent evaluations, benefiting key global assessments (IPCC, IPBES) and improving their impact on European and global policies (European Green Deal, UNFCCC, CBD);More relevant, robust and actionable scenar</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Europe and globally, as well as the interaction between different hazards, their cumulative and/or cascading effects.Enhanced seamless prediction and projection modelling and attribution capabilities for extreme events and their likelihood to support preparedness, response and resilience to climate change by EU and national and regional actors. The EU Union Preparedness Strategy, the EU Adaptation Str</t>
         </is>
       </c>
       <c r="C521" s="22" t="n"/>
@@ -13875,7 +13935,7 @@
       </c>
       <c r="B524" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-13</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C524" s="22" t="n"/>
@@ -13886,7 +13946,7 @@
     <row r="526" ht="30" customHeight="1">
       <c r="A526" s="18" t="inlineStr">
         <is>
-          <t>FICHA 36: HORIZON-CL5-2027-01-D1-11</t>
+          <t>FICHA 36: HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="B526" s="19" t="n"/>
@@ -13911,7 +13971,7 @@
       <c r="E527" s="22" t="n"/>
       <c r="F527" s="22" t="n"/>
     </row>
-    <row r="528" ht="20" customHeight="1">
+    <row r="528" ht="45" customHeight="1">
       <c r="A528" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -13919,7 +13979,7 @@
       </c>
       <c r="B528" s="21" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
         </is>
       </c>
       <c r="C528" s="22" t="n"/>
@@ -13935,7 +13995,7 @@
       </c>
       <c r="B529" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C529" s="22" t="n"/>
@@ -14015,7 +14075,7 @@
       </c>
       <c r="B534" s="21" t="inlineStr">
         <is>
-          <t>Programme Cofund Actions</t>
+          <t xml:space="preserve"> Research and Innovation Actions</t>
         </is>
       </c>
       <c r="C534" s="22" t="n"/>
@@ -14047,7 +14107,7 @@
       </c>
       <c r="B536" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is established through development and implementation of the Climate Action pillar of the EU-AU Research and Innovation Partnership on Climate Change and Sustainable Energy (CCSE),[1] in co-design between African and European partners;Reduced fragmentation by aligning the EU, national and multilateral R&amp;amp;I efforts with increased leverage and impact of funding;African scientific, policy and practice com</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to inform mitigation action and policy improvements, ensuring a fair transition and social acceptability;Methodologies are developed and improved for ex-ante assessment and ex-post evaluation of greenhouse gas emission reductions from climate policies and measures;Strengthened collaboration and established networks between researchers, policy experts and government officials involved in designing and eva</t>
         </is>
       </c>
       <c r="C536" s="22" t="n"/>
@@ -14091,7 +14151,7 @@
       </c>
       <c r="B539" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-11</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C539" s="22" t="n"/>
@@ -20930,7 +20990,7 @@
     <row r="1021" ht="30" customHeight="1">
       <c r="A1021" s="18" t="inlineStr">
         <is>
-          <t>FICHA 69: EUS-74952</t>
+          <t>FICHA 69: EUS-80078</t>
         </is>
       </c>
       <c r="B1021" s="19" t="n"/>
@@ -20979,7 +21039,7 @@
       </c>
       <c r="B1024" s="21" t="inlineStr">
         <is>
-          <t>EUS-74952</t>
+          <t>EUS-80078</t>
         </is>
       </c>
       <c r="C1024" s="22" t="n"/>
@@ -21142,7 +21202,7 @@
     <row r="1036" ht="30" customHeight="1">
       <c r="A1036" s="18" t="inlineStr">
         <is>
-          <t>FICHA 70: EUS-31018</t>
+          <t>FICHA 70: EUS-96450</t>
         </is>
       </c>
       <c r="B1036" s="19" t="n"/>
@@ -21191,7 +21251,7 @@
       </c>
       <c r="B1039" s="21" t="inlineStr">
         <is>
-          <t>EUS-31018</t>
+          <t>EUS-96450</t>
         </is>
       </c>
       <c r="C1039" s="22" t="n"/>
@@ -21354,7 +21414,7 @@
     <row r="1051" ht="30" customHeight="1">
       <c r="A1051" s="18" t="inlineStr">
         <is>
-          <t>FICHA 71: EUS-53900</t>
+          <t>FICHA 71: EUS-17669</t>
         </is>
       </c>
       <c r="B1051" s="19" t="n"/>
@@ -21403,7 +21463,7 @@
       </c>
       <c r="B1054" s="21" t="inlineStr">
         <is>
-          <t>EUS-53900</t>
+          <t>EUS-17669</t>
         </is>
       </c>
       <c r="C1054" s="22" t="n"/>
@@ -21566,7 +21626,7 @@
     <row r="1066" ht="30" customHeight="1">
       <c r="A1066" s="18" t="inlineStr">
         <is>
-          <t>FICHA 72: EUS-66315</t>
+          <t>FICHA 72: EUS-02163</t>
         </is>
       </c>
       <c r="B1066" s="19" t="n"/>
@@ -21615,7 +21675,7 @@
       </c>
       <c r="B1069" s="21" t="inlineStr">
         <is>
-          <t>EUS-66315</t>
+          <t>EUS-02163</t>
         </is>
       </c>
       <c r="C1069" s="22" t="n"/>
@@ -21778,7 +21838,7 @@
     <row r="1081" ht="30" customHeight="1">
       <c r="A1081" s="18" t="inlineStr">
         <is>
-          <t>FICHA 73: EUS-81441</t>
+          <t>FICHA 73: EUS-45408</t>
         </is>
       </c>
       <c r="B1081" s="19" t="n"/>
@@ -21827,7 +21887,7 @@
       </c>
       <c r="B1084" s="21" t="inlineStr">
         <is>
-          <t>EUS-81441</t>
+          <t>EUS-45408</t>
         </is>
       </c>
       <c r="C1084" s="22" t="n"/>
@@ -21990,7 +22050,7 @@
     <row r="1096" ht="30" customHeight="1">
       <c r="A1096" s="18" t="inlineStr">
         <is>
-          <t>FICHA 74: EUS-88586</t>
+          <t>FICHA 74: EUS-49463</t>
         </is>
       </c>
       <c r="B1096" s="19" t="n"/>
@@ -22023,7 +22083,7 @@
       </c>
       <c r="B1098" s="21" t="inlineStr">
         <is>
-          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de aceleración de proyectos, a localidades de menos de 20.000 habitantes son objeto de convocatoria abierta hasta el 17.03.26. Transformacione</t>
+          <t>Suministro de contenedores para la recogida de residuos municipales mezclados correspondiente a la fracción resto, suministro de cerraduras electrónicas y su instalación en los contenedores, suministr</t>
         </is>
       </c>
       <c r="C1098" s="22" t="n"/>
@@ -22039,7 +22099,7 @@
       </c>
       <c r="B1099" s="21" t="inlineStr">
         <is>
-          <t>EUS-88586</t>
+          <t>EUS-49463</t>
         </is>
       </c>
       <c r="C1099" s="22" t="n"/>
@@ -22115,7 +22175,7 @@
       </c>
       <c r="B1104" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C1104" s="22" t="n"/>
@@ -22173,9 +22233,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B1108" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
+      <c r="B1108" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALTA — </t>
         </is>
       </c>
       <c r="C1108" s="22" t="n"/>
@@ -22191,7 +22251,7 @@
       </c>
       <c r="B1109" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260317neboostasariak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-contenedores-recogida-residuos-municipales-mezclados-correspondiente-fraccion-resto-suministro-cerraduras-electronicas-y-su-instalacion-contenedores-suministro-tarjetas-apertura-cerraduras-electronicas-grabadoras-tarjetas-y-software-gestion-da/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1109" s="22" t="n"/>
@@ -22202,7 +22262,7 @@
     <row r="1111" ht="30" customHeight="1">
       <c r="A1111" s="18" t="inlineStr">
         <is>
-          <t>FICHA 75: EUS-91314</t>
+          <t>FICHA 75: EUS-95091</t>
         </is>
       </c>
       <c r="B1111" s="19" t="n"/>
@@ -22235,7 +22295,7 @@
       </c>
       <c r="B1113" s="21" t="inlineStr">
         <is>
-          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinancia convocatorias de ayudas de las Diputaciones a explotaciones con limitaciones o desfavorecidas, y a compromisos medioambientales, climátic</t>
+          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de aceleración de proyectos, a localidades de menos de 20.000 habitantes son objeto de convocatoria abierta hasta el 17.03.26. Transformacione</t>
         </is>
       </c>
       <c r="C1113" s="22" t="n"/>
@@ -22251,7 +22311,7 @@
       </c>
       <c r="B1114" s="21" t="inlineStr">
         <is>
-          <t>EUS-91314</t>
+          <t>EUS-95091</t>
         </is>
       </c>
       <c r="C1114" s="22" t="n"/>
@@ -22403,7 +22463,7 @@
       </c>
       <c r="B1124" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/lgenfnpbgfa260218/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260317neboostasariak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1124" s="22" t="n"/>
@@ -22414,7 +22474,7 @@
     <row r="1126" ht="30" customHeight="1">
       <c r="A1126" s="18" t="inlineStr">
         <is>
-          <t>FICHA 76: EUS-84020</t>
+          <t>FICHA 76: EUS-77783</t>
         </is>
       </c>
       <c r="B1126" s="19" t="n"/>
@@ -22447,7 +22507,7 @@
       </c>
       <c r="B1128" s="21" t="inlineStr">
         <is>
-          <t>Digital Europe, Horizon (programas de la UE). Apoyos para consorcios interestatales de I+D+i. IA, robótica, cuántica, computación, ciberseguridad, electrónica, fotónica, TICs e internet avanzadas, esp</t>
+          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinancia convocatorias de ayudas de las Diputaciones a explotaciones con limitaciones o desfavorecidas, y a compromisos medioambientales, climátic</t>
         </is>
       </c>
       <c r="C1128" s="22" t="n"/>
@@ -22463,7 +22523,7 @@
       </c>
       <c r="B1129" s="21" t="inlineStr">
         <is>
-          <t>EUS-84020</t>
+          <t>EUS-77783</t>
         </is>
       </c>
       <c r="C1129" s="22" t="n"/>
@@ -22615,7 +22675,7 @@
       </c>
       <c r="B1139" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260304digitalhorizoneen/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/lgenfnpbgfa260218/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1139" s="22" t="n"/>
@@ -22626,7 +22686,7 @@
     <row r="1141" ht="30" customHeight="1">
       <c r="A1141" s="18" t="inlineStr">
         <is>
-          <t>FICHA 77: EUS-18785</t>
+          <t>FICHA 77: EUS-01590</t>
         </is>
       </c>
       <c r="B1141" s="19" t="n"/>
@@ -22659,7 +22719,7 @@
       </c>
       <c r="B1143" s="21" t="inlineStr">
         <is>
-          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para consorcios internacionales de I+D+i. Jornada del Gobierno Vasco y con Enterprise Europe Network y otros socios. Digitalización, dispositivos,</t>
+          <t>Digital Europe, Horizon (programas de la UE). Apoyos para consorcios interestatales de I+D+i. IA, robótica, cuántica, computación, ciberseguridad, electrónica, fotónica, TICs e internet avanzadas, esp</t>
         </is>
       </c>
       <c r="C1143" s="22" t="n"/>
@@ -22675,7 +22735,7 @@
       </c>
       <c r="B1144" s="21" t="inlineStr">
         <is>
-          <t>EUS-18785</t>
+          <t>EUS-01590</t>
         </is>
       </c>
       <c r="C1144" s="22" t="n"/>
@@ -22827,7 +22887,7 @@
       </c>
       <c r="B1154" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260303eicihihorizon/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260304digitalhorizoneen/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1154" s="22" t="n"/>
@@ -22838,7 +22898,7 @@
     <row r="1156" ht="30" customHeight="1">
       <c r="A1156" s="18" t="inlineStr">
         <is>
-          <t>FICHA 78: EUS-44870</t>
+          <t>FICHA 78: EUS-07292</t>
         </is>
       </c>
       <c r="B1156" s="19" t="n"/>
@@ -22871,7 +22931,7 @@
       </c>
       <c r="B1158" s="21" t="inlineStr">
         <is>
-          <t>Política Agraria Común de la UE de 2026, y sus ayudas abiertas hasta el 30.4.26: el pilar 1, con el Fondo Europeo Agrícola de Garantía Agraria FEAGA, aborda sostenibilidad de renta, ayuda redistributi</t>
+          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para consorcios internacionales de I+D+i. Jornada del Gobierno Vasco y con Enterprise Europe Network y otros socios. Digitalización, dispositivos,</t>
         </is>
       </c>
       <c r="C1158" s="22" t="n"/>
@@ -22887,7 +22947,7 @@
       </c>
       <c r="B1159" s="21" t="inlineStr">
         <is>
-          <t>EUS-44870</t>
+          <t>EUS-07292</t>
         </is>
       </c>
       <c r="C1159" s="22" t="n"/>
@@ -23039,7 +23099,7 @@
       </c>
       <c r="B1169" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260216npblaguntzairekiak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260303eicihihorizon/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1169" s="22" t="n"/>
@@ -23050,7 +23110,7 @@
     <row r="1171" ht="30" customHeight="1">
       <c r="A1171" s="18" t="inlineStr">
         <is>
-          <t>FICHA 79: EUS-29143</t>
+          <t>FICHA 79: EUS-75051</t>
         </is>
       </c>
       <c r="B1171" s="19" t="n"/>
@@ -23083,7 +23143,7 @@
       </c>
       <c r="B1173" s="21" t="inlineStr">
         <is>
-          <t>Programa de impulso a las ciudades y territorios inteligentes para el fomento del desarrollo económico y productivo, que podrá ser cofinanciado por el Programa Plurirregional 2021-2027 del Fondo Europ</t>
+          <t>Política Agraria Común de la UE de 2026, y sus ayudas abiertas hasta el 30.4.26: el pilar 1, con el Fondo Europeo Agrícola de Garantía Agraria FEAGA, aborda sostenibilidad de renta, ayuda redistributi</t>
         </is>
       </c>
       <c r="C1173" s="22" t="n"/>
@@ -23099,7 +23159,7 @@
       </c>
       <c r="B1174" s="21" t="inlineStr">
         <is>
-          <t>EUS-29143</t>
+          <t>EUS-75051</t>
         </is>
       </c>
       <c r="C1174" s="22" t="n"/>
@@ -23251,7 +23311,7 @@
       </c>
       <c r="B1184" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260204smartcities/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260216npblaguntzairekiak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1184" s="22" t="n"/>
@@ -23262,7 +23322,7 @@
     <row r="1186" ht="30" customHeight="1">
       <c r="A1186" s="18" t="inlineStr">
         <is>
-          <t>FICHA 80: EUS-05166</t>
+          <t>FICHA 80: EUS-61906</t>
         </is>
       </c>
       <c r="B1186" s="19" t="n"/>
@@ -23295,7 +23355,7 @@
       </c>
       <c r="B1188" s="21" t="inlineStr">
         <is>
-          <t>Formación digital para empleabilidad turística: los fondos Next de la UE apoyan una convocatoria de Lanbide y el Gobierno Vasco, de cursos en línea para mejorar las competencias del sector y de sus py</t>
+          <t>Programa de impulso a las ciudades y territorios inteligentes para el fomento del desarrollo económico y productivo, que podrá ser cofinanciado por el Programa Plurirregional 2021-2027 del Fondo Europ</t>
         </is>
       </c>
       <c r="C1188" s="22" t="n"/>
@@ -23311,7 +23371,7 @@
       </c>
       <c r="B1189" s="21" t="inlineStr">
         <is>
-          <t>EUS-05166</t>
+          <t>EUS-61906</t>
         </is>
       </c>
       <c r="C1189" s="22" t="n"/>
@@ -23463,7 +23523,7 @@
       </c>
       <c r="B1199" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260119nextlanbidedigital/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260204smartcities/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1199" s="22" t="n"/>
@@ -23474,7 +23534,7 @@
     <row r="1201" ht="30" customHeight="1">
       <c r="A1201" s="18" t="inlineStr">
         <is>
-          <t>FICHA 81: EUS-07020</t>
+          <t>FICHA 81: EUS-41118</t>
         </is>
       </c>
       <c r="B1201" s="19" t="n"/>
@@ -23507,7 +23567,7 @@
       </c>
       <c r="B1203" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Horizon Europe. Clúster digital, industrial y espacial. Apoyos a proyectos para tecnologías de inteligencia artificial, internet, mundos virtuales, robótica, cuántica, fotónica, materias primas, bajo </t>
+          <t>Formación digital para empleabilidad turística: los fondos Next de la UE apoyan una convocatoria de Lanbide y el Gobierno Vasco, de cursos en línea para mejorar las competencias del sector y de sus py</t>
         </is>
       </c>
       <c r="C1203" s="22" t="n"/>
@@ -23523,7 +23583,7 @@
       </c>
       <c r="B1204" s="21" t="inlineStr">
         <is>
-          <t>EUS-07020</t>
+          <t>EUS-41118</t>
         </is>
       </c>
       <c r="C1204" s="22" t="n"/>
@@ -23675,7 +23735,7 @@
       </c>
       <c r="B1214" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/250119horizondiginduspaceklust/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260119nextlanbidedigital/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1214" s="22" t="n"/>
@@ -23686,7 +23746,7 @@
     <row r="1216" ht="30" customHeight="1">
       <c r="A1216" s="18" t="inlineStr">
         <is>
-          <t>FICHA 82: EUS-58974</t>
+          <t>FICHA 82: EUS-29727</t>
         </is>
       </c>
       <c r="B1216" s="19" t="n"/>
@@ -23719,7 +23779,7 @@
       </c>
       <c r="B1218" s="21" t="inlineStr">
         <is>
-          <t>Horizon Europe: ayudas de la línea de energía del clúster 5 y de la Misión Ciudades. Jornada informativa sobre estas y otras iniciativas en colaboración transestatal para la doble transición ecológica</t>
+          <t xml:space="preserve">Horizon Europe. Clúster digital, industrial y espacial. Apoyos a proyectos para tecnologías de inteligencia artificial, internet, mundos virtuales, robótica, cuántica, fotónica, materias primas, bajo </t>
         </is>
       </c>
       <c r="C1218" s="22" t="n"/>
@@ -23735,7 +23795,7 @@
       </c>
       <c r="B1219" s="21" t="inlineStr">
         <is>
-          <t>EUS-58974</t>
+          <t>EUS-29727</t>
         </is>
       </c>
       <c r="C1219" s="22" t="n"/>
@@ -23887,7 +23947,7 @@
       </c>
       <c r="B1229" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/horizonkluster5hirimisioa/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/250119horizondiginduspaceklust/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1229" s="22" t="n"/>
@@ -23898,7 +23958,7 @@
     <row r="1231" ht="30" customHeight="1">
       <c r="A1231" s="18" t="inlineStr">
         <is>
-          <t>FICHA 83: EUS-81341</t>
+          <t>FICHA 83: EUS-72731</t>
         </is>
       </c>
       <c r="B1231" s="19" t="n"/>
@@ -23931,7 +23991,7 @@
       </c>
       <c r="B1233" s="21" t="inlineStr">
         <is>
-          <t>Azpitek 2026: Programa de Ayudas para la Adquisición, Instalación, Renovación y Actualización de Infraestructuras de Investigación</t>
+          <t>Horizon Europe: ayudas de la línea de energía del clúster 5 y de la Misión Ciudades. Jornada informativa sobre estas y otras iniciativas en colaboración transestatal para la doble transición ecológica</t>
         </is>
       </c>
       <c r="C1233" s="22" t="n"/>
@@ -23947,7 +24007,7 @@
       </c>
       <c r="B1234" s="21" t="inlineStr">
         <is>
-          <t>EUS-81341</t>
+          <t>EUS-72731</t>
         </is>
       </c>
       <c r="C1234" s="22" t="n"/>
@@ -24099,7 +24159,7 @@
       </c>
       <c r="B1244" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2025/azpitek-2026-programa-de-ayudas/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/horizonkluster5hirimisioa/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1244" s="22" t="n"/>
@@ -24110,7 +24170,7 @@
     <row r="1246" ht="30" customHeight="1">
       <c r="A1246" s="18" t="inlineStr">
         <is>
-          <t>FICHA 84: EUS-61815</t>
+          <t>FICHA 84: EUS-03084</t>
         </is>
       </c>
       <c r="B1246" s="19" t="n"/>
@@ -24135,7 +24195,7 @@
       <c r="E1247" s="22" t="n"/>
       <c r="F1247" s="22" t="n"/>
     </row>
-    <row r="1248" ht="20" customHeight="1">
+    <row r="1248" ht="45" customHeight="1">
       <c r="A1248" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -24143,7 +24203,7 @@
       </c>
       <c r="B1248" s="21" t="inlineStr">
         <is>
-          <t>Subvenciones para innovación en economía circular 2026</t>
+          <t>Azpitek 2026: Programa de Ayudas para la Adquisición, Instalación, Renovación y Actualización de Infraestructuras de Investigación</t>
         </is>
       </c>
       <c r="C1248" s="22" t="n"/>
@@ -24159,7 +24219,7 @@
       </c>
       <c r="B1249" s="21" t="inlineStr">
         <is>
-          <t>EUS-61815</t>
+          <t>EUS-03084</t>
         </is>
       </c>
       <c r="C1249" s="22" t="n"/>
@@ -24311,7 +24371,7 @@
       </c>
       <c r="B1259" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2025/subvenciones-para-innovacion-en-economia-circular-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2025/azpitek-2026-programa-de-ayudas/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1259" s="22" t="n"/>
@@ -24322,7 +24382,7 @@
     <row r="1261" ht="30" customHeight="1">
       <c r="A1261" s="18" t="inlineStr">
         <is>
-          <t>FICHA 85: EUS-61141</t>
+          <t>FICHA 85: EUS-78189</t>
         </is>
       </c>
       <c r="B1261" s="19" t="n"/>
@@ -24347,7 +24407,7 @@
       <c r="E1262" s="22" t="n"/>
       <c r="F1262" s="22" t="n"/>
     </row>
-    <row r="1263" ht="45" customHeight="1">
+    <row r="1263" ht="20" customHeight="1">
       <c r="A1263" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -24355,7 +24415,7 @@
       </c>
       <c r="B1263" s="21" t="inlineStr">
         <is>
-          <t>Horizon Europe 2026-27: convocatorias ligadas a misiones ambientales de la UE, partenariados de economía circular, azul o bio, o a la división alimentaria EIT Food del Instituto Europeo de Tecnología,</t>
+          <t>Subvenciones para innovación en economía circular 2026</t>
         </is>
       </c>
       <c r="C1263" s="22" t="n"/>
@@ -24371,7 +24431,7 @@
       </c>
       <c r="B1264" s="21" t="inlineStr">
         <is>
-          <t>EUS-61141</t>
+          <t>EUS-78189</t>
         </is>
       </c>
       <c r="C1264" s="22" t="n"/>
@@ -24523,7 +24583,7 @@
       </c>
       <c r="B1274" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2025/251222horizon2627sprieeni/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2025/subvenciones-para-innovacion-en-economia-circular-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1274" s="22" t="n"/>
@@ -24534,7 +24594,7 @@
     <row r="1276" ht="30" customHeight="1">
       <c r="A1276" s="18" t="inlineStr">
         <is>
-          <t>FICHA 86: EUS-33047</t>
+          <t>FICHA 86: EUS-96006</t>
         </is>
       </c>
       <c r="B1276" s="19" t="n"/>
@@ -24567,7 +24627,7 @@
       </c>
       <c r="B1278" s="21" t="inlineStr">
         <is>
-          <t>Escudo Europeo de la Democracia: ayudas a proyectos de alfabetización mediática y fomento del diálogo y la comprensión en torno a la desinformación digital</t>
+          <t>Horizon Europe 2026-27: convocatorias ligadas a misiones ambientales de la UE, partenariados de economía circular, azul o bio, o a la división alimentaria EIT Food del Instituto Europeo de Tecnología,</t>
         </is>
       </c>
       <c r="C1278" s="22" t="n"/>
@@ -24583,7 +24643,7 @@
       </c>
       <c r="B1279" s="21" t="inlineStr">
         <is>
-          <t>EUS-33047</t>
+          <t>EUS-96006</t>
         </is>
       </c>
       <c r="C1279" s="22" t="n"/>
@@ -24735,7 +24795,7 @@
       </c>
       <c r="B1289" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2025/demokraziaezkutua251218/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2025/251222horizon2627sprieeni/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1289" s="22" t="n"/>
@@ -24746,7 +24806,7 @@
     <row r="1291" ht="30" customHeight="1">
       <c r="A1291" s="18" t="inlineStr">
         <is>
-          <t>FICHA 87: EUS-49824</t>
+          <t>FICHA 87: EUS-37801</t>
         </is>
       </c>
       <c r="B1291" s="19" t="n"/>
@@ -24779,7 +24839,7 @@
       </c>
       <c r="B1293" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">KSI Berritzaile Plus: ayudas del Gobierno Vasco a las Industrias Culturales y Creativas para proyectos innovadores en la triple transición tecnológico-digital, energético-climática y socio-sanitaria, </t>
+          <t>Escudo Europeo de la Democracia: ayudas a proyectos de alfabetización mediática y fomento del diálogo y la comprensión en torno a la desinformación digital</t>
         </is>
       </c>
       <c r="C1293" s="22" t="n"/>
@@ -24795,7 +24855,7 @@
       </c>
       <c r="B1294" s="21" t="inlineStr">
         <is>
-          <t>EUS-49824</t>
+          <t>EUS-37801</t>
         </is>
       </c>
       <c r="C1294" s="22" t="n"/>
@@ -24947,7 +25007,7 @@
       </c>
       <c r="B1304" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2025/ksiberritzalieplus251218/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2025/demokraziaezkutua251218/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1304" s="22" t="n"/>
@@ -24958,7 +25018,7 @@
     <row r="1306" ht="30" customHeight="1">
       <c r="A1306" s="18" t="inlineStr">
         <is>
-          <t>FICHA 88: EUS-83207</t>
+          <t>FICHA 88: EUS-98075</t>
         </is>
       </c>
       <c r="B1306" s="19" t="n"/>
@@ -24991,7 +25051,7 @@
       </c>
       <c r="B1308" s="21" t="inlineStr">
         <is>
-          <t>Desmontaje de dos depósitos de agua en local del polideportivo ipurua y tuberías que lo alimentan.</t>
+          <t xml:space="preserve">KSI Berritzaile Plus: ayudas del Gobierno Vasco a las Industrias Culturales y Creativas para proyectos innovadores en la triple transición tecnológico-digital, energético-climática y socio-sanitaria, </t>
         </is>
       </c>
       <c r="C1308" s="22" t="n"/>
@@ -25007,7 +25067,7 @@
       </c>
       <c r="B1309" s="21" t="inlineStr">
         <is>
-          <t>EUS-83207</t>
+          <t>EUS-98075</t>
         </is>
       </c>
       <c r="C1309" s="22" t="n"/>
@@ -25083,7 +25143,7 @@
       </c>
       <c r="B1314" s="21" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C1314" s="22" t="n"/>
@@ -25159,7 +25219,7 @@
       </c>
       <c r="B1319" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/desmontaje-dos-depositos-agua-local-del-polideportivo-ipurua-y-tuberias-que-alimentan/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2025/ksiberritzalieplus251218/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1319" s="22" t="n"/>
@@ -25170,7 +25230,7 @@
     <row r="1321" ht="30" customHeight="1">
       <c r="A1321" s="18" t="inlineStr">
         <is>
-          <t>FICHA 89: EUS-43218</t>
+          <t>FICHA 89: EUS-37368</t>
         </is>
       </c>
       <c r="B1321" s="19" t="n"/>
@@ -25195,7 +25255,7 @@
       <c r="E1322" s="22" t="n"/>
       <c r="F1322" s="22" t="n"/>
     </row>
-    <row r="1323" ht="20" customHeight="1">
+    <row r="1323" ht="45" customHeight="1">
       <c r="A1323" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -25203,7 +25263,7 @@
       </c>
       <c r="B1323" s="21" t="inlineStr">
         <is>
-          <t>Reparación del ascensor exterior de urki polonia tras entrada agua en cuadro</t>
+          <t>Mantenimiento de los servidores instalados en el edificio Onkologikoa (OSI Donostialdea)</t>
         </is>
       </c>
       <c r="C1323" s="22" t="n"/>
@@ -25219,7 +25279,7 @@
       </c>
       <c r="B1324" s="21" t="inlineStr">
         <is>
-          <t>EUS-43218</t>
+          <t>EUS-37368</t>
         </is>
       </c>
       <c r="C1324" s="22" t="n"/>
@@ -25371,7 +25431,7 @@
       </c>
       <c r="B1334" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/reparacion-del-ascensor-exterior-urki-polonia-entrada-agua-cuadro/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/mantenimiento-servidores-instalados-edificio-onkologikoa-osi-donostialdea/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1334" s="22" t="n"/>
@@ -25382,7 +25442,7 @@
     <row r="1336" ht="30" customHeight="1">
       <c r="A1336" s="18" t="inlineStr">
         <is>
-          <t>FICHA 90: EUS-03214</t>
+          <t>FICHA 90: EUS-78987</t>
         </is>
       </c>
       <c r="B1336" s="19" t="n"/>
@@ -25415,7 +25475,7 @@
       </c>
       <c r="B1338" s="21" t="inlineStr">
         <is>
-          <t>Desatasco tanto de la red de pluviales como de la de fecales de errebal plazia</t>
+          <t>Gestión del servicio público de transporte colectivo urbano de Tolosa</t>
         </is>
       </c>
       <c r="C1338" s="22" t="n"/>
@@ -25431,7 +25491,7 @@
       </c>
       <c r="B1339" s="21" t="inlineStr">
         <is>
-          <t>EUS-03214</t>
+          <t>EUS-78987</t>
         </is>
       </c>
       <c r="C1339" s="22" t="n"/>
@@ -25583,7 +25643,7 @@
       </c>
       <c r="B1349" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/desatasco-tanto-red-pluviales-como-de-fecales-errebal-plazia/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/gestion-del-servicio-publico-transporte-colectivo-urbano-tolosa/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1349" s="22" t="n"/>
@@ -25594,7 +25654,7 @@
     <row r="1351" ht="30" customHeight="1">
       <c r="A1351" s="18" t="inlineStr">
         <is>
-          <t>FICHA 91: EUS-68824</t>
+          <t>FICHA 91: EUS-25969</t>
         </is>
       </c>
       <c r="B1351" s="19" t="n"/>
@@ -25627,7 +25687,7 @@
       </c>
       <c r="B1353" s="21" t="inlineStr">
         <is>
-          <t>Contratación de la actuación de unos bertsolaris el 8 y 14 de septiembre en el marco de las fiestas de ntra. sra. de arrate</t>
+          <t>Desmontaje de dos depósitos de agua en local del polideportivo ipurua y tuberías que lo alimentan.</t>
         </is>
       </c>
       <c r="C1353" s="22" t="n"/>
@@ -25643,7 +25703,7 @@
       </c>
       <c r="B1354" s="21" t="inlineStr">
         <is>
-          <t>EUS-68824</t>
+          <t>EUS-25969</t>
         </is>
       </c>
       <c r="C1354" s="22" t="n"/>
@@ -25795,7 +25855,7 @@
       </c>
       <c r="B1364" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/contratacion-actuacion-bertsolaris-8-y-14-septiembre-marco-fiestas-ntra-sra-arrate/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/desmontaje-dos-depositos-agua-local-del-polideportivo-ipurua-y-tuberias-que-alimentan/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1364" s="22" t="n"/>
@@ -25806,7 +25866,7 @@
     <row r="1366" ht="30" customHeight="1">
       <c r="A1366" s="18" t="inlineStr">
         <is>
-          <t>FICHA 92: EUS-26937</t>
+          <t>FICHA 92: EUS-14012</t>
         </is>
       </c>
       <c r="B1366" s="19" t="n"/>
@@ -25831,7 +25891,7 @@
       <c r="E1367" s="22" t="n"/>
       <c r="F1367" s="22" t="n"/>
     </row>
-    <row r="1368" ht="45" customHeight="1">
+    <row r="1368" ht="20" customHeight="1">
       <c r="A1368" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -25839,7 +25899,7 @@
       </c>
       <c r="B1368" s="21" t="inlineStr">
         <is>
-          <t>Suministro de botellines de agua mineral para atender a los grupos que actúan en el teatro coliseo</t>
+          <t>Reparación del ascensor exterior de urki polonia tras entrada agua en cuadro</t>
         </is>
       </c>
       <c r="C1368" s="22" t="n"/>
@@ -25855,7 +25915,7 @@
       </c>
       <c r="B1369" s="21" t="inlineStr">
         <is>
-          <t>EUS-26937</t>
+          <t>EUS-14012</t>
         </is>
       </c>
       <c r="C1369" s="22" t="n"/>
@@ -26007,7 +26067,7 @@
       </c>
       <c r="B1379" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-botellines-agua-mineral-atender-grupos-que-actuan-teatro-coliseo/expgeeibar19188/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/reparacion-del-ascensor-exterior-urki-polonia-entrada-agua-cuadro/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1379" s="22" t="n"/>
@@ -26018,7 +26078,7 @@
     <row r="1381" ht="30" customHeight="1">
       <c r="A1381" s="18" t="inlineStr">
         <is>
-          <t>FICHA 93: EUS-27498</t>
+          <t>FICHA 93: EUS-79105</t>
         </is>
       </c>
       <c r="B1381" s="19" t="n"/>
@@ -26043,7 +26103,7 @@
       <c r="E1382" s="22" t="n"/>
       <c r="F1382" s="22" t="n"/>
     </row>
-    <row r="1383" ht="45" customHeight="1">
+    <row r="1383" ht="20" customHeight="1">
       <c r="A1383" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -26051,7 +26111,7 @@
       </c>
       <c r="B1383" s="21" t="inlineStr">
         <is>
-          <t>Servicio de organización de la sesión de bertsolaris de arrate del 7 de septiembre.</t>
+          <t>Desatasco tanto de la red de pluviales como de la de fecales de errebal plazia</t>
         </is>
       </c>
       <c r="C1383" s="22" t="n"/>
@@ -26067,7 +26127,7 @@
       </c>
       <c r="B1384" s="21" t="inlineStr">
         <is>
-          <t>EUS-27498</t>
+          <t>EUS-79105</t>
         </is>
       </c>
       <c r="C1384" s="22" t="n"/>
@@ -26219,7 +26279,7 @@
       </c>
       <c r="B1394" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-organizacion-sesion-bertsolaris-arrate-del-7-septiembre/expgeeibar19095/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/desatasco-tanto-red-pluviales-como-de-fecales-errebal-plazia/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1394" s="22" t="n"/>
@@ -26227,8 +26287,220 @@
       <c r="E1394" s="22" t="n"/>
       <c r="F1394" s="22" t="n"/>
     </row>
+    <row r="1396" ht="30" customHeight="1">
+      <c r="A1396" s="18" t="inlineStr">
+        <is>
+          <t>FICHA 94: EUS-32322</t>
+        </is>
+      </c>
+      <c r="B1396" s="19" t="n"/>
+      <c r="C1396" s="19" t="n"/>
+      <c r="D1396" s="19" t="n"/>
+      <c r="E1396" s="19" t="n"/>
+      <c r="F1396" s="19" t="n"/>
+    </row>
+    <row r="1397" ht="20" customHeight="1">
+      <c r="A1397" s="20" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1397" s="21" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1397" s="22" t="n"/>
+      <c r="D1397" s="22" t="n"/>
+      <c r="E1397" s="22" t="n"/>
+      <c r="F1397" s="22" t="n"/>
+    </row>
+    <row r="1398" ht="45" customHeight="1">
+      <c r="A1398" s="20" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1398" s="21" t="inlineStr">
+        <is>
+          <t>Contratación de la actuación de unos bertsolaris el 8 y 14 de septiembre en el marco de las fiestas de ntra. sra. de arrate</t>
+        </is>
+      </c>
+      <c r="C1398" s="22" t="n"/>
+      <c r="D1398" s="22" t="n"/>
+      <c r="E1398" s="22" t="n"/>
+      <c r="F1398" s="22" t="n"/>
+    </row>
+    <row r="1399" ht="20" customHeight="1">
+      <c r="A1399" s="20" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1399" s="21" t="inlineStr">
+        <is>
+          <t>EUS-32322</t>
+        </is>
+      </c>
+      <c r="C1399" s="22" t="n"/>
+      <c r="D1399" s="22" t="n"/>
+      <c r="E1399" s="22" t="n"/>
+      <c r="F1399" s="22" t="n"/>
+    </row>
+    <row r="1400" ht="20" customHeight="1">
+      <c r="A1400" s="20" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1400" s="21" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1400" s="22" t="n"/>
+      <c r="D1400" s="22" t="n"/>
+      <c r="E1400" s="22" t="n"/>
+      <c r="F1400" s="22" t="n"/>
+    </row>
+    <row r="1401" ht="20" customHeight="1">
+      <c r="A1401" s="20" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1401" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1401" s="22" t="n"/>
+      <c r="D1401" s="22" t="n"/>
+      <c r="E1401" s="22" t="n"/>
+      <c r="F1401" s="22" t="n"/>
+    </row>
+    <row r="1402" ht="20" customHeight="1">
+      <c r="A1402" s="20" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1402" s="21" t="inlineStr"/>
+      <c r="C1402" s="22" t="n"/>
+      <c r="D1402" s="22" t="n"/>
+      <c r="E1402" s="22" t="n"/>
+      <c r="F1402" s="22" t="n"/>
+    </row>
+    <row r="1403" ht="20" customHeight="1">
+      <c r="A1403" s="20" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1403" s="21" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1403" s="22" t="n"/>
+      <c r="D1403" s="22" t="n"/>
+      <c r="E1403" s="22" t="n"/>
+      <c r="F1403" s="22" t="n"/>
+    </row>
+    <row r="1404" ht="20" customHeight="1">
+      <c r="A1404" s="20" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1404" s="21" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1404" s="22" t="n"/>
+      <c r="D1404" s="22" t="n"/>
+      <c r="E1404" s="22" t="n"/>
+      <c r="F1404" s="22" t="n"/>
+    </row>
+    <row r="1405" ht="20" customHeight="1">
+      <c r="A1405" s="20" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1405" s="21" t="inlineStr"/>
+      <c r="C1405" s="22" t="n"/>
+      <c r="D1405" s="22" t="n"/>
+      <c r="E1405" s="22" t="n"/>
+      <c r="F1405" s="22" t="n"/>
+    </row>
+    <row r="1406" ht="20" customHeight="1">
+      <c r="A1406" s="20" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1406" s="21" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1406" s="22" t="n"/>
+      <c r="D1406" s="22" t="n"/>
+      <c r="E1406" s="22" t="n"/>
+      <c r="F1406" s="22" t="n"/>
+    </row>
+    <row r="1407" ht="20" customHeight="1">
+      <c r="A1407" s="20" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1407" s="21" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1407" s="22" t="n"/>
+      <c r="D1407" s="22" t="n"/>
+      <c r="E1407" s="22" t="n"/>
+      <c r="F1407" s="22" t="n"/>
+    </row>
+    <row r="1408" ht="20" customHeight="1">
+      <c r="A1408" s="20" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1408" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1408" s="22" t="n"/>
+      <c r="D1408" s="22" t="n"/>
+      <c r="E1408" s="22" t="n"/>
+      <c r="F1408" s="22" t="n"/>
+    </row>
+    <row r="1409" ht="45" customHeight="1">
+      <c r="A1409" s="20" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1409" s="24" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/contratacion-actuacion-bertsolaris-8-y-14-septiembre-marco-fiestas-ntra-sra-arrate/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1409" s="22" t="n"/>
+      <c r="D1409" s="22" t="n"/>
+      <c r="E1409" s="22" t="n"/>
+      <c r="F1409" s="22" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="1302">
+  <mergeCells count="1316">
     <mergeCell ref="B679:F679"/>
     <mergeCell ref="B1010:F1010"/>
     <mergeCell ref="B276:F276"/>
@@ -26268,8 +26540,10 @@
     <mergeCell ref="B448:F448"/>
     <mergeCell ref="B746:F746"/>
     <mergeCell ref="B1105:F1105"/>
+    <mergeCell ref="B1403:F1403"/>
     <mergeCell ref="B319:F319"/>
     <mergeCell ref="B1046:F1046"/>
+    <mergeCell ref="B1405:F1405"/>
     <mergeCell ref="A346:F346"/>
     <mergeCell ref="A136:F136"/>
     <mergeCell ref="B159:F159"/>
@@ -26518,6 +26792,7 @@
     <mergeCell ref="B1072:F1072"/>
     <mergeCell ref="A556:F556"/>
     <mergeCell ref="B1108:F1108"/>
+    <mergeCell ref="B1406:F1406"/>
     <mergeCell ref="B1289:F1289"/>
     <mergeCell ref="B48:F48"/>
     <mergeCell ref="B1101:F1101"/>
@@ -26724,6 +26999,7 @@
     <mergeCell ref="B1049:F1049"/>
     <mergeCell ref="B1347:F1347"/>
     <mergeCell ref="B1032:F1032"/>
+    <mergeCell ref="B1401:F1401"/>
     <mergeCell ref="B219:F219"/>
     <mergeCell ref="B460:F460"/>
     <mergeCell ref="B517:F517"/>
@@ -26778,6 +27054,7 @@
     <mergeCell ref="B1390:F1390"/>
     <mergeCell ref="B453:F453"/>
     <mergeCell ref="B629:F629"/>
+    <mergeCell ref="A1396:F1396"/>
     <mergeCell ref="B787:F787"/>
     <mergeCell ref="B32:F32"/>
     <mergeCell ref="B1058:F1058"/>
@@ -26971,7 +27248,9 @@
     <mergeCell ref="B639:F639"/>
     <mergeCell ref="B1068:F1068"/>
     <mergeCell ref="B1104:F1104"/>
+    <mergeCell ref="B1402:F1402"/>
     <mergeCell ref="B641:F641"/>
+    <mergeCell ref="B1404:F1404"/>
     <mergeCell ref="B1287:F1287"/>
     <mergeCell ref="B972:F972"/>
     <mergeCell ref="B359:F359"/>
@@ -27014,10 +27293,12 @@
     <mergeCell ref="B610:F610"/>
     <mergeCell ref="B1064:F1064"/>
     <mergeCell ref="B1100:F1100"/>
+    <mergeCell ref="B1398:F1398"/>
     <mergeCell ref="B339:F339"/>
     <mergeCell ref="B314:F314"/>
     <mergeCell ref="B643:F643"/>
     <mergeCell ref="B637:F637"/>
+    <mergeCell ref="B1400:F1400"/>
     <mergeCell ref="A1306:F1306"/>
     <mergeCell ref="B784:F784"/>
     <mergeCell ref="B1082:F1082"/>
@@ -27231,6 +27512,7 @@
     <mergeCell ref="B657:F657"/>
     <mergeCell ref="B672:F672"/>
     <mergeCell ref="B688:F688"/>
+    <mergeCell ref="B1399:F1399"/>
     <mergeCell ref="B682:F682"/>
     <mergeCell ref="B980:F980"/>
     <mergeCell ref="B217:F217"/>
@@ -27271,6 +27553,7 @@
     <mergeCell ref="B1352:F1352"/>
     <mergeCell ref="B320:F320"/>
     <mergeCell ref="B1083:F1083"/>
+    <mergeCell ref="B1408:F1408"/>
     <mergeCell ref="B1383:F1383"/>
     <mergeCell ref="B38:F38"/>
     <mergeCell ref="B467:F467"/>
@@ -27330,6 +27613,7 @@
     <mergeCell ref="B1090:F1090"/>
     <mergeCell ref="B1361:F1361"/>
     <mergeCell ref="B1221:F1221"/>
+    <mergeCell ref="B1397:F1397"/>
     <mergeCell ref="B39:F39"/>
     <mergeCell ref="B1092:F1092"/>
     <mergeCell ref="A961:F961"/>
@@ -27526,8 +27810,10 @@
     <mergeCell ref="B653:F653"/>
     <mergeCell ref="B1109:F1109"/>
     <mergeCell ref="B354:F354"/>
+    <mergeCell ref="B1407:F1407"/>
     <mergeCell ref="B348:F348"/>
     <mergeCell ref="B652:F652"/>
+    <mergeCell ref="B1409:F1409"/>
     <mergeCell ref="B1292:F1292"/>
     <mergeCell ref="B648:F648"/>
     <mergeCell ref="B51:F51"/>
@@ -27626,6 +27912,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1364" r:id="rId91"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1379" r:id="rId92"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1394" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1409" r:id="rId94"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -27637,7 +27924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J94"/>
+  <dimension ref="A1:J95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -27983,7 +28270,7 @@
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>INNOVFUND-2025-NZT-GENERAL-SSP</t>
+          <t>INNOVFUND-2025-NZT-GENERAL-MSP</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
@@ -28023,7 +28310,7 @@
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>INNOVFUND-2025-NZT-GENERAL-LSP</t>
+          <t>INNOVFUND-2025-NZT-GENERAL-SSP</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -28063,7 +28350,7 @@
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>INNOVFUND-2025-NZT-GENERAL-MSP</t>
+          <t>INNOVFUND-2025-NZT-GENERAL-LSP</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -28259,12 +28546,12 @@
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-08-Two-Stage-D1-06</t>
+          <t>HORIZON-CL5-2026-07-D1-01</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Closing knowledge gaps on Earth system science in support of</t>
+          <t>Next generation climate monitoring and related capabilities</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -28299,12 +28586,12 @@
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-07-D1-01</t>
+          <t>HORIZON-CL5-2026-08-Two-Stage-D1-06</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Next generation climate monitoring and related capabilities</t>
+          <t>Closing knowledge gaps on Earth system science in support of</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -28339,12 +28626,12 @@
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-07-D1-05</t>
+          <t>HORIZON-CL5-2026-07-D1-04</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Improving climate and weather models for Africa</t>
+          <t>Fighting disinformation and effectively communicating on cli</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -28379,12 +28666,12 @@
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-07-D1-04</t>
+          <t>HORIZON-CL5-2026-07-D1-05</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Fighting disinformation and effectively communicating on cli</t>
+          <t>Improving climate and weather models for Africa</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -28935,12 +29222,12 @@
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-13</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Next generation scenarios for informing climate and sustaina</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -28975,12 +29262,12 @@
     <row r="34" ht="28" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
@@ -29015,12 +29302,12 @@
     <row r="35" ht="28" customHeight="1">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform cl</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -29055,12 +29342,12 @@
     <row r="36" ht="28" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-13</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Next generation scenarios for informing climate and sustaina</t>
+          <t>Advancing understanding, modelling and prediction of extreme</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -29095,12 +29382,12 @@
     <row r="37" ht="28" customHeight="1">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Assessing the performance of policy instruments to inform cl</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
@@ -30295,7 +30582,7 @@
     <row r="70" ht="28" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>EUS-74952</t>
+          <t>EUS-80078</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
@@ -30331,7 +30618,7 @@
     <row r="71" ht="28" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>EUS-31018</t>
+          <t>EUS-96450</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
@@ -30367,7 +30654,7 @@
     <row r="72" ht="28" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>EUS-53900</t>
+          <t>EUS-17669</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
@@ -30403,7 +30690,7 @@
     <row r="73" ht="28" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>EUS-66315</t>
+          <t>EUS-02163</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
@@ -30439,7 +30726,7 @@
     <row r="74" ht="28" customHeight="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>EUS-81441</t>
+          <t>EUS-45408</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
@@ -30475,12 +30762,12 @@
     <row r="75" ht="28" customHeight="1">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>EUS-88586</t>
+          <t>EUS-49463</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de</t>
+          <t>Suministro de contenedores para la recogida de residuos muni</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
@@ -30496,7 +30783,7 @@
       <c r="E75" s="6" t="inlineStr"/>
       <c r="F75" s="27" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="G75" s="6" t="inlineStr"/>
@@ -30511,12 +30798,12 @@
     <row r="76" ht="28" customHeight="1">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>EUS-91314</t>
+          <t>EUS-95091</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinanc</t>
+          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
@@ -30547,12 +30834,12 @@
     <row r="77" ht="28" customHeight="1">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>EUS-84020</t>
+          <t>EUS-77783</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>Digital Europe, Horizon (programas de la UE). Apoyos para co</t>
+          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinanc</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
@@ -30583,12 +30870,12 @@
     <row r="78" ht="28" customHeight="1">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>EUS-18785</t>
+          <t>EUS-01590</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para c</t>
+          <t>Digital Europe, Horizon (programas de la UE). Apoyos para co</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
@@ -30619,12 +30906,12 @@
     <row r="79" ht="28" customHeight="1">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>EUS-44870</t>
+          <t>EUS-07292</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>Política Agraria Común de la UE de 2026, y sus ayudas abiert</t>
+          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para c</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
@@ -30655,12 +30942,12 @@
     <row r="80" ht="28" customHeight="1">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>EUS-29143</t>
+          <t>EUS-75051</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>Programa de impulso a las ciudades y territorios inteligente</t>
+          <t>Política Agraria Común de la UE de 2026, y sus ayudas abiert</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
@@ -30691,12 +30978,12 @@
     <row r="81" ht="28" customHeight="1">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>EUS-05166</t>
+          <t>EUS-61906</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>Formación digital para empleabilidad turística: los fondos N</t>
+          <t>Programa de impulso a las ciudades y territorios inteligente</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
@@ -30727,12 +31014,12 @@
     <row r="82" ht="28" customHeight="1">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>EUS-07020</t>
+          <t>EUS-41118</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>Horizon Europe. Clúster digital, industrial y espacial. Apoy</t>
+          <t>Formación digital para empleabilidad turística: los fondos N</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
@@ -30763,12 +31050,12 @@
     <row r="83" ht="28" customHeight="1">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>EUS-58974</t>
+          <t>EUS-29727</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Horizon Europe: ayudas de la línea de energía del clúster 5 </t>
+          <t>Horizon Europe. Clúster digital, industrial y espacial. Apoy</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
@@ -30799,12 +31086,12 @@
     <row r="84" ht="28" customHeight="1">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>EUS-81341</t>
+          <t>EUS-72731</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>Azpitek 2026: Programa de Ayudas para la Adquisición, Instal</t>
+          <t xml:space="preserve">Horizon Europe: ayudas de la línea de energía del clúster 5 </t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
@@ -30835,12 +31122,12 @@
     <row r="85" ht="28" customHeight="1">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>EUS-61815</t>
+          <t>EUS-03084</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>Subvenciones para innovación en economía circular 2026</t>
+          <t>Azpitek 2026: Programa de Ayudas para la Adquisición, Instal</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
@@ -30871,12 +31158,12 @@
     <row r="86" ht="28" customHeight="1">
       <c r="A86" s="6" t="inlineStr">
         <is>
-          <t>EUS-61141</t>
+          <t>EUS-78189</t>
         </is>
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>Horizon Europe 2026-27: convocatorias ligadas a misiones amb</t>
+          <t>Subvenciones para innovación en economía circular 2026</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
@@ -30907,12 +31194,12 @@
     <row r="87" ht="28" customHeight="1">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>EUS-33047</t>
+          <t>EUS-96006</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>Escudo Europeo de la Democracia: ayudas a proyectos de alfab</t>
+          <t>Horizon Europe 2026-27: convocatorias ligadas a misiones amb</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
@@ -30943,12 +31230,12 @@
     <row r="88" ht="28" customHeight="1">
       <c r="A88" s="6" t="inlineStr">
         <is>
-          <t>EUS-49824</t>
+          <t>EUS-37801</t>
         </is>
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>KSI Berritzaile Plus: ayudas del Gobierno Vasco a las Indust</t>
+          <t>Escudo Europeo de la Democracia: ayudas a proyectos de alfab</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
@@ -30979,12 +31266,12 @@
     <row r="89" ht="28" customHeight="1">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>EUS-83207</t>
+          <t>EUS-98075</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>Desmontaje de dos depósitos de agua en local del polideporti</t>
+          <t>KSI Berritzaile Plus: ayudas del Gobierno Vasco a las Indust</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
@@ -31015,12 +31302,12 @@
     <row r="90" ht="28" customHeight="1">
       <c r="A90" s="6" t="inlineStr">
         <is>
-          <t>EUS-43218</t>
+          <t>EUS-37368</t>
         </is>
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>Reparación del ascensor exterior de urki polonia tras entrad</t>
+          <t>Mantenimiento de los servidores instalados en el edificio On</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
@@ -31051,12 +31338,12 @@
     <row r="91" ht="28" customHeight="1">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>EUS-03214</t>
+          <t>EUS-78987</t>
         </is>
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>Desatasco tanto de la red de pluviales como de la de fecales</t>
+          <t xml:space="preserve">Gestión del servicio público de transporte colectivo urbano </t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
@@ -31087,12 +31374,12 @@
     <row r="92" ht="28" customHeight="1">
       <c r="A92" s="6" t="inlineStr">
         <is>
-          <t>EUS-68824</t>
+          <t>EUS-25969</t>
         </is>
       </c>
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>Contratación de la actuación de unos bertsolaris el 8 y 14 d</t>
+          <t>Desmontaje de dos depósitos de agua en local del polideporti</t>
         </is>
       </c>
       <c r="C92" s="6" t="inlineStr">
@@ -31123,12 +31410,12 @@
     <row r="93" ht="28" customHeight="1">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>EUS-26937</t>
+          <t>EUS-14012</t>
         </is>
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Suministro de botellines de agua mineral para atender a los </t>
+          <t>Reparación del ascensor exterior de urki polonia tras entrad</t>
         </is>
       </c>
       <c r="C93" s="6" t="inlineStr">
@@ -31159,12 +31446,12 @@
     <row r="94" ht="28" customHeight="1">
       <c r="A94" s="6" t="inlineStr">
         <is>
-          <t>EUS-27498</t>
+          <t>EUS-79105</t>
         </is>
       </c>
       <c r="B94" s="6" t="inlineStr">
         <is>
-          <t>Servicio de organización de la sesión de bertsolaris de arra</t>
+          <t>Desatasco tanto de la red de pluviales como de la de fecales</t>
         </is>
       </c>
       <c r="C94" s="6" t="inlineStr">
@@ -31192,8 +31479,44 @@
       <c r="I94" s="6" t="inlineStr"/>
       <c r="J94" s="6" t="inlineStr"/>
     </row>
+    <row r="95" ht="28" customHeight="1">
+      <c r="A95" s="6" t="inlineStr">
+        <is>
+          <t>EUS-32322</t>
+        </is>
+      </c>
+      <c r="B95" s="6" t="inlineStr">
+        <is>
+          <t>Contratación de la actuación de unos bertsolaris el 8 y 14 d</t>
+        </is>
+      </c>
+      <c r="C95" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D95" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E95" s="6" t="inlineStr"/>
+      <c r="F95" s="27" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G95" s="6" t="inlineStr"/>
+      <c r="H95" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I95" s="6" t="inlineStr"/>
+      <c r="J95" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J94"/>
+  <autoFilter ref="A1:J95"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update funding data 2026-03-20
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -685,7 +685,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 19/03/2026 06:48 - 83 convocatorias - 29 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 20/03/2026 06:43 - 83 convocatorias - 29 nuevas</t>
         </is>
       </c>
     </row>
@@ -3896,7 +3896,7 @@
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>EUS-97747</t>
+          <t>EUS-00787</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
@@ -3951,7 +3951,7 @@
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>EUS-74009</t>
+          <t>EUS-59163</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>EUS-43045</t>
+          <t>EUS-88500</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
@@ -4061,7 +4061,7 @@
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>EUS-40837</t>
+          <t>EUS-76639</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
@@ -4116,7 +4116,7 @@
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>EUS-53065</t>
+          <t>EUS-81169</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -4171,7 +4171,7 @@
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>EUS-39165</t>
+          <t>EUS-92514</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
@@ -4226,7 +4226,7 @@
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>EUS-99743</t>
+          <t>EUS-52924</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
@@ -4281,7 +4281,7 @@
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>EUS-42711</t>
+          <t>EUS-18113</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -4336,7 +4336,7 @@
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>EUS-60355</t>
+          <t>EUS-83079</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -4391,7 +4391,7 @@
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>EUS-80084</t>
+          <t>EUS-77148</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -4446,7 +4446,7 @@
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>EUS-45075</t>
+          <t>EUS-45619</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -4501,7 +4501,7 @@
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>EUS-41030</t>
+          <t>EUS-07148</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -4556,7 +4556,7 @@
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>EUS-01158</t>
+          <t>EUS-26860</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -4611,7 +4611,7 @@
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>EUS-04249</t>
+          <t>EUS-66169</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>EUS-68397</t>
+          <t>EUS-12972</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
@@ -4721,7 +4721,7 @@
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>EUS-64737</t>
+          <t>EUS-56698</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
@@ -4776,7 +4776,7 @@
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>EUS-00482</t>
+          <t>EUS-47190</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>EUS-93743</t>
+          <t>EUS-87522</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
@@ -4886,7 +4886,7 @@
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>EUS-84475</t>
+          <t>EUS-08113</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
@@ -4941,7 +4941,7 @@
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>EUS-73757</t>
+          <t>EUS-22613</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
@@ -4996,7 +4996,7 @@
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>EUS-68716</t>
+          <t>EUS-61987</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
@@ -5051,7 +5051,7 @@
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>EUS-70492</t>
+          <t>EUS-77717</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
@@ -5106,7 +5106,7 @@
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>EUS-27173</t>
+          <t>EUS-67496</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
@@ -5161,7 +5161,7 @@
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>EUS-84180</t>
+          <t>EUS-03052</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
@@ -5216,7 +5216,7 @@
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>EUS-49845</t>
+          <t>EUS-84012</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
@@ -5271,7 +5271,7 @@
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>EUS-27637</t>
+          <t>EUS-38815</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
@@ -5326,7 +5326,7 @@
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>EUS-33636</t>
+          <t>EUS-68967</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
@@ -5381,7 +5381,7 @@
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>EUS-76595</t>
+          <t>EUS-08547</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
@@ -5436,7 +5436,7 @@
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>EUS-63448</t>
+          <t>EUS-22249</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
@@ -17224,7 +17224,7 @@
     <row r="811" ht="30" customHeight="1">
       <c r="A811" s="16" t="inlineStr">
         <is>
-          <t>FICHA 55: EUS-97747</t>
+          <t>FICHA 55: EUS-00787</t>
         </is>
       </c>
       <c r="B811" s="17" t="n"/>
@@ -17273,7 +17273,7 @@
       </c>
       <c r="B814" s="19" t="inlineStr">
         <is>
-          <t>EUS-97747</t>
+          <t>EUS-00787</t>
         </is>
       </c>
       <c r="C814" s="20" t="n"/>
@@ -17436,7 +17436,7 @@
     <row r="826" ht="30" customHeight="1">
       <c r="A826" s="16" t="inlineStr">
         <is>
-          <t>FICHA 56: EUS-74009</t>
+          <t>FICHA 56: EUS-59163</t>
         </is>
       </c>
       <c r="B826" s="17" t="n"/>
@@ -17485,7 +17485,7 @@
       </c>
       <c r="B829" s="19" t="inlineStr">
         <is>
-          <t>EUS-74009</t>
+          <t>EUS-59163</t>
         </is>
       </c>
       <c r="C829" s="20" t="n"/>
@@ -17648,7 +17648,7 @@
     <row r="841" ht="30" customHeight="1">
       <c r="A841" s="16" t="inlineStr">
         <is>
-          <t>FICHA 57: EUS-43045</t>
+          <t>FICHA 57: EUS-88500</t>
         </is>
       </c>
       <c r="B841" s="17" t="n"/>
@@ -17697,7 +17697,7 @@
       </c>
       <c r="B844" s="19" t="inlineStr">
         <is>
-          <t>EUS-43045</t>
+          <t>EUS-88500</t>
         </is>
       </c>
       <c r="C844" s="20" t="n"/>
@@ -17860,7 +17860,7 @@
     <row r="856" ht="30" customHeight="1">
       <c r="A856" s="16" t="inlineStr">
         <is>
-          <t>FICHA 58: EUS-40837</t>
+          <t>FICHA 58: EUS-76639</t>
         </is>
       </c>
       <c r="B856" s="17" t="n"/>
@@ -17909,7 +17909,7 @@
       </c>
       <c r="B859" s="19" t="inlineStr">
         <is>
-          <t>EUS-40837</t>
+          <t>EUS-76639</t>
         </is>
       </c>
       <c r="C859" s="20" t="n"/>
@@ -18072,7 +18072,7 @@
     <row r="871" ht="30" customHeight="1">
       <c r="A871" s="16" t="inlineStr">
         <is>
-          <t>FICHA 59: EUS-53065</t>
+          <t>FICHA 59: EUS-81169</t>
         </is>
       </c>
       <c r="B871" s="17" t="n"/>
@@ -18121,7 +18121,7 @@
       </c>
       <c r="B874" s="19" t="inlineStr">
         <is>
-          <t>EUS-53065</t>
+          <t>EUS-81169</t>
         </is>
       </c>
       <c r="C874" s="20" t="n"/>
@@ -18284,7 +18284,7 @@
     <row r="886" ht="30" customHeight="1">
       <c r="A886" s="16" t="inlineStr">
         <is>
-          <t>FICHA 60: EUS-39165</t>
+          <t>FICHA 60: EUS-92514</t>
         </is>
       </c>
       <c r="B886" s="17" t="n"/>
@@ -18333,7 +18333,7 @@
       </c>
       <c r="B889" s="19" t="inlineStr">
         <is>
-          <t>EUS-39165</t>
+          <t>EUS-92514</t>
         </is>
       </c>
       <c r="C889" s="20" t="n"/>
@@ -18496,7 +18496,7 @@
     <row r="901" ht="30" customHeight="1">
       <c r="A901" s="16" t="inlineStr">
         <is>
-          <t>FICHA 61: EUS-99743</t>
+          <t>FICHA 61: EUS-52924</t>
         </is>
       </c>
       <c r="B901" s="17" t="n"/>
@@ -18545,7 +18545,7 @@
       </c>
       <c r="B904" s="19" t="inlineStr">
         <is>
-          <t>EUS-99743</t>
+          <t>EUS-52924</t>
         </is>
       </c>
       <c r="C904" s="20" t="n"/>
@@ -18708,7 +18708,7 @@
     <row r="916" ht="30" customHeight="1">
       <c r="A916" s="16" t="inlineStr">
         <is>
-          <t>FICHA 62: EUS-42711</t>
+          <t>FICHA 62: EUS-18113</t>
         </is>
       </c>
       <c r="B916" s="17" t="n"/>
@@ -18757,7 +18757,7 @@
       </c>
       <c r="B919" s="19" t="inlineStr">
         <is>
-          <t>EUS-42711</t>
+          <t>EUS-18113</t>
         </is>
       </c>
       <c r="C919" s="20" t="n"/>
@@ -18920,7 +18920,7 @@
     <row r="931" ht="30" customHeight="1">
       <c r="A931" s="16" t="inlineStr">
         <is>
-          <t>FICHA 63: EUS-60355</t>
+          <t>FICHA 63: EUS-83079</t>
         </is>
       </c>
       <c r="B931" s="17" t="n"/>
@@ -18969,7 +18969,7 @@
       </c>
       <c r="B934" s="19" t="inlineStr">
         <is>
-          <t>EUS-60355</t>
+          <t>EUS-83079</t>
         </is>
       </c>
       <c r="C934" s="20" t="n"/>
@@ -19132,7 +19132,7 @@
     <row r="946" ht="30" customHeight="1">
       <c r="A946" s="16" t="inlineStr">
         <is>
-          <t>FICHA 64: EUS-80084</t>
+          <t>FICHA 64: EUS-77148</t>
         </is>
       </c>
       <c r="B946" s="17" t="n"/>
@@ -19181,7 +19181,7 @@
       </c>
       <c r="B949" s="19" t="inlineStr">
         <is>
-          <t>EUS-80084</t>
+          <t>EUS-77148</t>
         </is>
       </c>
       <c r="C949" s="20" t="n"/>
@@ -19344,7 +19344,7 @@
     <row r="961" ht="30" customHeight="1">
       <c r="A961" s="16" t="inlineStr">
         <is>
-          <t>FICHA 65: EUS-45075</t>
+          <t>FICHA 65: EUS-45619</t>
         </is>
       </c>
       <c r="B961" s="17" t="n"/>
@@ -19393,7 +19393,7 @@
       </c>
       <c r="B964" s="19" t="inlineStr">
         <is>
-          <t>EUS-45075</t>
+          <t>EUS-45619</t>
         </is>
       </c>
       <c r="C964" s="20" t="n"/>
@@ -19556,7 +19556,7 @@
     <row r="976" ht="30" customHeight="1">
       <c r="A976" s="16" t="inlineStr">
         <is>
-          <t>FICHA 66: EUS-41030</t>
+          <t>FICHA 66: EUS-07148</t>
         </is>
       </c>
       <c r="B976" s="17" t="n"/>
@@ -19605,7 +19605,7 @@
       </c>
       <c r="B979" s="19" t="inlineStr">
         <is>
-          <t>EUS-41030</t>
+          <t>EUS-07148</t>
         </is>
       </c>
       <c r="C979" s="20" t="n"/>
@@ -19768,7 +19768,7 @@
     <row r="991" ht="30" customHeight="1">
       <c r="A991" s="16" t="inlineStr">
         <is>
-          <t>FICHA 67: EUS-01158</t>
+          <t>FICHA 67: EUS-26860</t>
         </is>
       </c>
       <c r="B991" s="17" t="n"/>
@@ -19817,7 +19817,7 @@
       </c>
       <c r="B994" s="19" t="inlineStr">
         <is>
-          <t>EUS-01158</t>
+          <t>EUS-26860</t>
         </is>
       </c>
       <c r="C994" s="20" t="n"/>
@@ -19980,7 +19980,7 @@
     <row r="1006" ht="30" customHeight="1">
       <c r="A1006" s="16" t="inlineStr">
         <is>
-          <t>FICHA 68: EUS-04249</t>
+          <t>FICHA 68: EUS-66169</t>
         </is>
       </c>
       <c r="B1006" s="17" t="n"/>
@@ -20029,7 +20029,7 @@
       </c>
       <c r="B1009" s="19" t="inlineStr">
         <is>
-          <t>EUS-04249</t>
+          <t>EUS-66169</t>
         </is>
       </c>
       <c r="C1009" s="20" t="n"/>
@@ -20192,7 +20192,7 @@
     <row r="1021" ht="30" customHeight="1">
       <c r="A1021" s="16" t="inlineStr">
         <is>
-          <t>FICHA 69: EUS-68397</t>
+          <t>FICHA 69: EUS-12972</t>
         </is>
       </c>
       <c r="B1021" s="17" t="n"/>
@@ -20241,7 +20241,7 @@
       </c>
       <c r="B1024" s="19" t="inlineStr">
         <is>
-          <t>EUS-68397</t>
+          <t>EUS-12972</t>
         </is>
       </c>
       <c r="C1024" s="20" t="n"/>
@@ -20404,7 +20404,7 @@
     <row r="1036" ht="30" customHeight="1">
       <c r="A1036" s="16" t="inlineStr">
         <is>
-          <t>FICHA 70: EUS-64737</t>
+          <t>FICHA 70: EUS-56698</t>
         </is>
       </c>
       <c r="B1036" s="17" t="n"/>
@@ -20453,7 +20453,7 @@
       </c>
       <c r="B1039" s="19" t="inlineStr">
         <is>
-          <t>EUS-64737</t>
+          <t>EUS-56698</t>
         </is>
       </c>
       <c r="C1039" s="20" t="n"/>
@@ -20616,7 +20616,7 @@
     <row r="1051" ht="30" customHeight="1">
       <c r="A1051" s="16" t="inlineStr">
         <is>
-          <t>FICHA 71: EUS-00482</t>
+          <t>FICHA 71: EUS-47190</t>
         </is>
       </c>
       <c r="B1051" s="17" t="n"/>
@@ -20665,7 +20665,7 @@
       </c>
       <c r="B1054" s="19" t="inlineStr">
         <is>
-          <t>EUS-00482</t>
+          <t>EUS-47190</t>
         </is>
       </c>
       <c r="C1054" s="20" t="n"/>
@@ -20828,7 +20828,7 @@
     <row r="1066" ht="30" customHeight="1">
       <c r="A1066" s="16" t="inlineStr">
         <is>
-          <t>FICHA 72: EUS-93743</t>
+          <t>FICHA 72: EUS-87522</t>
         </is>
       </c>
       <c r="B1066" s="17" t="n"/>
@@ -20877,7 +20877,7 @@
       </c>
       <c r="B1069" s="19" t="inlineStr">
         <is>
-          <t>EUS-93743</t>
+          <t>EUS-87522</t>
         </is>
       </c>
       <c r="C1069" s="20" t="n"/>
@@ -21040,7 +21040,7 @@
     <row r="1081" ht="30" customHeight="1">
       <c r="A1081" s="16" t="inlineStr">
         <is>
-          <t>FICHA 73: EUS-84475</t>
+          <t>FICHA 73: EUS-08113</t>
         </is>
       </c>
       <c r="B1081" s="17" t="n"/>
@@ -21089,7 +21089,7 @@
       </c>
       <c r="B1084" s="19" t="inlineStr">
         <is>
-          <t>EUS-84475</t>
+          <t>EUS-08113</t>
         </is>
       </c>
       <c r="C1084" s="20" t="n"/>
@@ -21252,7 +21252,7 @@
     <row r="1096" ht="30" customHeight="1">
       <c r="A1096" s="16" t="inlineStr">
         <is>
-          <t>FICHA 74: EUS-73757</t>
+          <t>FICHA 74: EUS-22613</t>
         </is>
       </c>
       <c r="B1096" s="17" t="n"/>
@@ -21301,7 +21301,7 @@
       </c>
       <c r="B1099" s="19" t="inlineStr">
         <is>
-          <t>EUS-73757</t>
+          <t>EUS-22613</t>
         </is>
       </c>
       <c r="C1099" s="20" t="n"/>
@@ -21464,7 +21464,7 @@
     <row r="1111" ht="30" customHeight="1">
       <c r="A1111" s="16" t="inlineStr">
         <is>
-          <t>FICHA 75: EUS-68716</t>
+          <t>FICHA 75: EUS-61987</t>
         </is>
       </c>
       <c r="B1111" s="17" t="n"/>
@@ -21513,7 +21513,7 @@
       </c>
       <c r="B1114" s="19" t="inlineStr">
         <is>
-          <t>EUS-68716</t>
+          <t>EUS-61987</t>
         </is>
       </c>
       <c r="C1114" s="20" t="n"/>
@@ -21676,7 +21676,7 @@
     <row r="1126" ht="30" customHeight="1">
       <c r="A1126" s="16" t="inlineStr">
         <is>
-          <t>FICHA 76: EUS-70492</t>
+          <t>FICHA 76: EUS-77717</t>
         </is>
       </c>
       <c r="B1126" s="17" t="n"/>
@@ -21725,7 +21725,7 @@
       </c>
       <c r="B1129" s="19" t="inlineStr">
         <is>
-          <t>EUS-70492</t>
+          <t>EUS-77717</t>
         </is>
       </c>
       <c r="C1129" s="20" t="n"/>
@@ -21888,7 +21888,7 @@
     <row r="1141" ht="30" customHeight="1">
       <c r="A1141" s="16" t="inlineStr">
         <is>
-          <t>FICHA 77: EUS-27173</t>
+          <t>FICHA 77: EUS-67496</t>
         </is>
       </c>
       <c r="B1141" s="17" t="n"/>
@@ -21937,7 +21937,7 @@
       </c>
       <c r="B1144" s="19" t="inlineStr">
         <is>
-          <t>EUS-27173</t>
+          <t>EUS-67496</t>
         </is>
       </c>
       <c r="C1144" s="20" t="n"/>
@@ -22100,7 +22100,7 @@
     <row r="1156" ht="30" customHeight="1">
       <c r="A1156" s="16" t="inlineStr">
         <is>
-          <t>FICHA 78: EUS-84180</t>
+          <t>FICHA 78: EUS-03052</t>
         </is>
       </c>
       <c r="B1156" s="17" t="n"/>
@@ -22149,7 +22149,7 @@
       </c>
       <c r="B1159" s="19" t="inlineStr">
         <is>
-          <t>EUS-84180</t>
+          <t>EUS-03052</t>
         </is>
       </c>
       <c r="C1159" s="20" t="n"/>
@@ -22312,7 +22312,7 @@
     <row r="1171" ht="30" customHeight="1">
       <c r="A1171" s="16" t="inlineStr">
         <is>
-          <t>FICHA 79: EUS-49845</t>
+          <t>FICHA 79: EUS-84012</t>
         </is>
       </c>
       <c r="B1171" s="17" t="n"/>
@@ -22361,7 +22361,7 @@
       </c>
       <c r="B1174" s="19" t="inlineStr">
         <is>
-          <t>EUS-49845</t>
+          <t>EUS-84012</t>
         </is>
       </c>
       <c r="C1174" s="20" t="n"/>
@@ -22524,7 +22524,7 @@
     <row r="1186" ht="30" customHeight="1">
       <c r="A1186" s="16" t="inlineStr">
         <is>
-          <t>FICHA 80: EUS-27637</t>
+          <t>FICHA 80: EUS-38815</t>
         </is>
       </c>
       <c r="B1186" s="17" t="n"/>
@@ -22573,7 +22573,7 @@
       </c>
       <c r="B1189" s="19" t="inlineStr">
         <is>
-          <t>EUS-27637</t>
+          <t>EUS-38815</t>
         </is>
       </c>
       <c r="C1189" s="20" t="n"/>
@@ -22736,7 +22736,7 @@
     <row r="1201" ht="30" customHeight="1">
       <c r="A1201" s="16" t="inlineStr">
         <is>
-          <t>FICHA 81: EUS-33636</t>
+          <t>FICHA 81: EUS-68967</t>
         </is>
       </c>
       <c r="B1201" s="17" t="n"/>
@@ -22785,7 +22785,7 @@
       </c>
       <c r="B1204" s="19" t="inlineStr">
         <is>
-          <t>EUS-33636</t>
+          <t>EUS-68967</t>
         </is>
       </c>
       <c r="C1204" s="20" t="n"/>
@@ -22948,7 +22948,7 @@
     <row r="1216" ht="30" customHeight="1">
       <c r="A1216" s="16" t="inlineStr">
         <is>
-          <t>FICHA 82: EUS-76595</t>
+          <t>FICHA 82: EUS-08547</t>
         </is>
       </c>
       <c r="B1216" s="17" t="n"/>
@@ -22997,7 +22997,7 @@
       </c>
       <c r="B1219" s="19" t="inlineStr">
         <is>
-          <t>EUS-76595</t>
+          <t>EUS-08547</t>
         </is>
       </c>
       <c r="C1219" s="20" t="n"/>
@@ -23160,7 +23160,7 @@
     <row r="1231" ht="30" customHeight="1">
       <c r="A1231" s="16" t="inlineStr">
         <is>
-          <t>FICHA 83: EUS-63448</t>
+          <t>FICHA 83: EUS-22249</t>
         </is>
       </c>
       <c r="B1231" s="17" t="n"/>
@@ -23209,7 +23209,7 @@
       </c>
       <c r="B1234" s="19" t="inlineStr">
         <is>
-          <t>EUS-63448</t>
+          <t>EUS-22249</t>
         </is>
       </c>
       <c r="C1234" s="20" t="n"/>
@@ -26735,7 +26735,7 @@
     <row r="56" ht="28" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>EUS-97747</t>
+          <t>EUS-00787</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
@@ -26771,7 +26771,7 @@
     <row r="57" ht="28" customHeight="1">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>EUS-74009</t>
+          <t>EUS-59163</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
@@ -26807,7 +26807,7 @@
     <row r="58" ht="28" customHeight="1">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>EUS-43045</t>
+          <t>EUS-88500</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
@@ -26843,7 +26843,7 @@
     <row r="59" ht="28" customHeight="1">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>EUS-40837</t>
+          <t>EUS-76639</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
@@ -26879,7 +26879,7 @@
     <row r="60" ht="28" customHeight="1">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>EUS-53065</t>
+          <t>EUS-81169</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
@@ -26915,7 +26915,7 @@
     <row r="61" ht="28" customHeight="1">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>EUS-39165</t>
+          <t>EUS-92514</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
@@ -26951,7 +26951,7 @@
     <row r="62" ht="28" customHeight="1">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>EUS-99743</t>
+          <t>EUS-52924</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
@@ -26987,7 +26987,7 @@
     <row r="63" ht="28" customHeight="1">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>EUS-42711</t>
+          <t>EUS-18113</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
@@ -27023,7 +27023,7 @@
     <row r="64" ht="28" customHeight="1">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>EUS-60355</t>
+          <t>EUS-83079</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
@@ -27059,7 +27059,7 @@
     <row r="65" ht="28" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>EUS-80084</t>
+          <t>EUS-77148</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
@@ -27095,7 +27095,7 @@
     <row r="66" ht="28" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>EUS-45075</t>
+          <t>EUS-45619</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
@@ -27131,7 +27131,7 @@
     <row r="67" ht="28" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>EUS-41030</t>
+          <t>EUS-07148</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
@@ -27167,7 +27167,7 @@
     <row r="68" ht="28" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>EUS-01158</t>
+          <t>EUS-26860</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
@@ -27203,7 +27203,7 @@
     <row r="69" ht="28" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>EUS-04249</t>
+          <t>EUS-66169</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
@@ -27239,7 +27239,7 @@
     <row r="70" ht="28" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>EUS-68397</t>
+          <t>EUS-12972</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
@@ -27275,7 +27275,7 @@
     <row r="71" ht="28" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>EUS-64737</t>
+          <t>EUS-56698</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
@@ -27311,7 +27311,7 @@
     <row r="72" ht="28" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>EUS-00482</t>
+          <t>EUS-47190</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
@@ -27347,7 +27347,7 @@
     <row r="73" ht="28" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>EUS-93743</t>
+          <t>EUS-87522</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
@@ -27383,7 +27383,7 @@
     <row r="74" ht="28" customHeight="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>EUS-84475</t>
+          <t>EUS-08113</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
@@ -27419,7 +27419,7 @@
     <row r="75" ht="28" customHeight="1">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>EUS-73757</t>
+          <t>EUS-22613</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
@@ -27455,7 +27455,7 @@
     <row r="76" ht="28" customHeight="1">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>EUS-68716</t>
+          <t>EUS-61987</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
@@ -27491,7 +27491,7 @@
     <row r="77" ht="28" customHeight="1">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>EUS-70492</t>
+          <t>EUS-77717</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
@@ -27527,7 +27527,7 @@
     <row r="78" ht="28" customHeight="1">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>EUS-27173</t>
+          <t>EUS-67496</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
@@ -27563,7 +27563,7 @@
     <row r="79" ht="28" customHeight="1">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>EUS-84180</t>
+          <t>EUS-03052</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
@@ -27599,7 +27599,7 @@
     <row r="80" ht="28" customHeight="1">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>EUS-49845</t>
+          <t>EUS-84012</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
@@ -27635,7 +27635,7 @@
     <row r="81" ht="28" customHeight="1">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>EUS-27637</t>
+          <t>EUS-38815</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
@@ -27671,7 +27671,7 @@
     <row r="82" ht="28" customHeight="1">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>EUS-33636</t>
+          <t>EUS-68967</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
@@ -27707,7 +27707,7 @@
     <row r="83" ht="28" customHeight="1">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>EUS-76595</t>
+          <t>EUS-08547</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
@@ -27743,7 +27743,7 @@
     <row r="84" ht="28" customHeight="1">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>EUS-63448</t>
+          <t>EUS-22249</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Update funding data 2026-03-22
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -685,7 +685,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 21/03/2026 06:33 - 73 convocatorias - 20 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 22/03/2026 06:38 - 73 convocatorias - 20 nuevas</t>
         </is>
       </c>
     </row>
@@ -3849,7 +3849,7 @@
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>EUS-04804</t>
+          <t>EUS-54537</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>EUS-40390</t>
+          <t>EUS-50343</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
@@ -3959,7 +3959,7 @@
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>EUS-81412</t>
+          <t>EUS-52804</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
@@ -4014,7 +4014,7 @@
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>EUS-79656</t>
+          <t>EUS-42482</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
@@ -4069,7 +4069,7 @@
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>EUS-17505</t>
+          <t>EUS-32296</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
@@ -4124,7 +4124,7 @@
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>EUS-83702</t>
+          <t>EUS-21142</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -4179,7 +4179,7 @@
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>EUS-22522</t>
+          <t>EUS-77157</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
@@ -4234,7 +4234,7 @@
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>EUS-99695</t>
+          <t>EUS-47217</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
@@ -4289,7 +4289,7 @@
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>EUS-65161</t>
+          <t>EUS-17090</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -4344,7 +4344,7 @@
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>EUS-54622</t>
+          <t>EUS-54644</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -4399,7 +4399,7 @@
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>EUS-03111</t>
+          <t>EUS-08071</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -4454,7 +4454,7 @@
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>EUS-29680</t>
+          <t>EUS-53374</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -4509,7 +4509,7 @@
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>EUS-06937</t>
+          <t>EUS-08180</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -4564,7 +4564,7 @@
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>EUS-47446</t>
+          <t>EUS-15428</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -4619,7 +4619,7 @@
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>EUS-75016</t>
+          <t>EUS-70478</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
@@ -4674,7 +4674,7 @@
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>EUS-08635</t>
+          <t>EUS-60414</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
@@ -4729,7 +4729,7 @@
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>EUS-67943</t>
+          <t>EUS-77936</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
@@ -4784,7 +4784,7 @@
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>EUS-97486</t>
+          <t>EUS-52649</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
@@ -4839,7 +4839,7 @@
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>EUS-36297</t>
+          <t>EUS-26111</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
@@ -4894,7 +4894,7 @@
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>EUS-41456</t>
+          <t>EUS-52906</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
@@ -16464,7 +16464,7 @@
     <row r="796" ht="30" customHeight="1">
       <c r="A796" s="16" t="inlineStr">
         <is>
-          <t>FICHA 54: EUS-04804</t>
+          <t>FICHA 54: EUS-54537</t>
         </is>
       </c>
       <c r="B796" s="17" t="n"/>
@@ -16513,7 +16513,7 @@
       </c>
       <c r="B799" s="19" t="inlineStr">
         <is>
-          <t>EUS-04804</t>
+          <t>EUS-54537</t>
         </is>
       </c>
       <c r="C799" s="20" t="n"/>
@@ -16676,7 +16676,7 @@
     <row r="811" ht="30" customHeight="1">
       <c r="A811" s="16" t="inlineStr">
         <is>
-          <t>FICHA 55: EUS-40390</t>
+          <t>FICHA 55: EUS-50343</t>
         </is>
       </c>
       <c r="B811" s="17" t="n"/>
@@ -16725,7 +16725,7 @@
       </c>
       <c r="B814" s="19" t="inlineStr">
         <is>
-          <t>EUS-40390</t>
+          <t>EUS-50343</t>
         </is>
       </c>
       <c r="C814" s="20" t="n"/>
@@ -16888,7 +16888,7 @@
     <row r="826" ht="30" customHeight="1">
       <c r="A826" s="16" t="inlineStr">
         <is>
-          <t>FICHA 56: EUS-81412</t>
+          <t>FICHA 56: EUS-52804</t>
         </is>
       </c>
       <c r="B826" s="17" t="n"/>
@@ -16937,7 +16937,7 @@
       </c>
       <c r="B829" s="19" t="inlineStr">
         <is>
-          <t>EUS-81412</t>
+          <t>EUS-52804</t>
         </is>
       </c>
       <c r="C829" s="20" t="n"/>
@@ -17100,7 +17100,7 @@
     <row r="841" ht="30" customHeight="1">
       <c r="A841" s="16" t="inlineStr">
         <is>
-          <t>FICHA 57: EUS-79656</t>
+          <t>FICHA 57: EUS-42482</t>
         </is>
       </c>
       <c r="B841" s="17" t="n"/>
@@ -17149,7 +17149,7 @@
       </c>
       <c r="B844" s="19" t="inlineStr">
         <is>
-          <t>EUS-79656</t>
+          <t>EUS-42482</t>
         </is>
       </c>
       <c r="C844" s="20" t="n"/>
@@ -17312,7 +17312,7 @@
     <row r="856" ht="30" customHeight="1">
       <c r="A856" s="16" t="inlineStr">
         <is>
-          <t>FICHA 58: EUS-17505</t>
+          <t>FICHA 58: EUS-32296</t>
         </is>
       </c>
       <c r="B856" s="17" t="n"/>
@@ -17361,7 +17361,7 @@
       </c>
       <c r="B859" s="19" t="inlineStr">
         <is>
-          <t>EUS-17505</t>
+          <t>EUS-32296</t>
         </is>
       </c>
       <c r="C859" s="20" t="n"/>
@@ -17524,7 +17524,7 @@
     <row r="871" ht="30" customHeight="1">
       <c r="A871" s="16" t="inlineStr">
         <is>
-          <t>FICHA 59: EUS-83702</t>
+          <t>FICHA 59: EUS-21142</t>
         </is>
       </c>
       <c r="B871" s="17" t="n"/>
@@ -17573,7 +17573,7 @@
       </c>
       <c r="B874" s="19" t="inlineStr">
         <is>
-          <t>EUS-83702</t>
+          <t>EUS-21142</t>
         </is>
       </c>
       <c r="C874" s="20" t="n"/>
@@ -17736,7 +17736,7 @@
     <row r="886" ht="30" customHeight="1">
       <c r="A886" s="16" t="inlineStr">
         <is>
-          <t>FICHA 60: EUS-22522</t>
+          <t>FICHA 60: EUS-77157</t>
         </is>
       </c>
       <c r="B886" s="17" t="n"/>
@@ -17785,7 +17785,7 @@
       </c>
       <c r="B889" s="19" t="inlineStr">
         <is>
-          <t>EUS-22522</t>
+          <t>EUS-77157</t>
         </is>
       </c>
       <c r="C889" s="20" t="n"/>
@@ -17948,7 +17948,7 @@
     <row r="901" ht="30" customHeight="1">
       <c r="A901" s="16" t="inlineStr">
         <is>
-          <t>FICHA 61: EUS-99695</t>
+          <t>FICHA 61: EUS-47217</t>
         </is>
       </c>
       <c r="B901" s="17" t="n"/>
@@ -17997,7 +17997,7 @@
       </c>
       <c r="B904" s="19" t="inlineStr">
         <is>
-          <t>EUS-99695</t>
+          <t>EUS-47217</t>
         </is>
       </c>
       <c r="C904" s="20" t="n"/>
@@ -18160,7 +18160,7 @@
     <row r="916" ht="30" customHeight="1">
       <c r="A916" s="16" t="inlineStr">
         <is>
-          <t>FICHA 62: EUS-65161</t>
+          <t>FICHA 62: EUS-17090</t>
         </is>
       </c>
       <c r="B916" s="17" t="n"/>
@@ -18209,7 +18209,7 @@
       </c>
       <c r="B919" s="19" t="inlineStr">
         <is>
-          <t>EUS-65161</t>
+          <t>EUS-17090</t>
         </is>
       </c>
       <c r="C919" s="20" t="n"/>
@@ -18372,7 +18372,7 @@
     <row r="931" ht="30" customHeight="1">
       <c r="A931" s="16" t="inlineStr">
         <is>
-          <t>FICHA 63: EUS-54622</t>
+          <t>FICHA 63: EUS-54644</t>
         </is>
       </c>
       <c r="B931" s="17" t="n"/>
@@ -18421,7 +18421,7 @@
       </c>
       <c r="B934" s="19" t="inlineStr">
         <is>
-          <t>EUS-54622</t>
+          <t>EUS-54644</t>
         </is>
       </c>
       <c r="C934" s="20" t="n"/>
@@ -18584,7 +18584,7 @@
     <row r="946" ht="30" customHeight="1">
       <c r="A946" s="16" t="inlineStr">
         <is>
-          <t>FICHA 64: EUS-03111</t>
+          <t>FICHA 64: EUS-08071</t>
         </is>
       </c>
       <c r="B946" s="17" t="n"/>
@@ -18633,7 +18633,7 @@
       </c>
       <c r="B949" s="19" t="inlineStr">
         <is>
-          <t>EUS-03111</t>
+          <t>EUS-08071</t>
         </is>
       </c>
       <c r="C949" s="20" t="n"/>
@@ -18796,7 +18796,7 @@
     <row r="961" ht="30" customHeight="1">
       <c r="A961" s="16" t="inlineStr">
         <is>
-          <t>FICHA 65: EUS-29680</t>
+          <t>FICHA 65: EUS-53374</t>
         </is>
       </c>
       <c r="B961" s="17" t="n"/>
@@ -18845,7 +18845,7 @@
       </c>
       <c r="B964" s="19" t="inlineStr">
         <is>
-          <t>EUS-29680</t>
+          <t>EUS-53374</t>
         </is>
       </c>
       <c r="C964" s="20" t="n"/>
@@ -19008,7 +19008,7 @@
     <row r="976" ht="30" customHeight="1">
       <c r="A976" s="16" t="inlineStr">
         <is>
-          <t>FICHA 66: EUS-06937</t>
+          <t>FICHA 66: EUS-08180</t>
         </is>
       </c>
       <c r="B976" s="17" t="n"/>
@@ -19057,7 +19057,7 @@
       </c>
       <c r="B979" s="19" t="inlineStr">
         <is>
-          <t>EUS-06937</t>
+          <t>EUS-08180</t>
         </is>
       </c>
       <c r="C979" s="20" t="n"/>
@@ -19220,7 +19220,7 @@
     <row r="991" ht="30" customHeight="1">
       <c r="A991" s="16" t="inlineStr">
         <is>
-          <t>FICHA 67: EUS-47446</t>
+          <t>FICHA 67: EUS-15428</t>
         </is>
       </c>
       <c r="B991" s="17" t="n"/>
@@ -19269,7 +19269,7 @@
       </c>
       <c r="B994" s="19" t="inlineStr">
         <is>
-          <t>EUS-47446</t>
+          <t>EUS-15428</t>
         </is>
       </c>
       <c r="C994" s="20" t="n"/>
@@ -19432,7 +19432,7 @@
     <row r="1006" ht="30" customHeight="1">
       <c r="A1006" s="16" t="inlineStr">
         <is>
-          <t>FICHA 68: EUS-75016</t>
+          <t>FICHA 68: EUS-70478</t>
         </is>
       </c>
       <c r="B1006" s="17" t="n"/>
@@ -19481,7 +19481,7 @@
       </c>
       <c r="B1009" s="19" t="inlineStr">
         <is>
-          <t>EUS-75016</t>
+          <t>EUS-70478</t>
         </is>
       </c>
       <c r="C1009" s="20" t="n"/>
@@ -19644,7 +19644,7 @@
     <row r="1021" ht="30" customHeight="1">
       <c r="A1021" s="16" t="inlineStr">
         <is>
-          <t>FICHA 69: EUS-08635</t>
+          <t>FICHA 69: EUS-60414</t>
         </is>
       </c>
       <c r="B1021" s="17" t="n"/>
@@ -19693,7 +19693,7 @@
       </c>
       <c r="B1024" s="19" t="inlineStr">
         <is>
-          <t>EUS-08635</t>
+          <t>EUS-60414</t>
         </is>
       </c>
       <c r="C1024" s="20" t="n"/>
@@ -19856,7 +19856,7 @@
     <row r="1036" ht="30" customHeight="1">
       <c r="A1036" s="16" t="inlineStr">
         <is>
-          <t>FICHA 70: EUS-67943</t>
+          <t>FICHA 70: EUS-77936</t>
         </is>
       </c>
       <c r="B1036" s="17" t="n"/>
@@ -19905,7 +19905,7 @@
       </c>
       <c r="B1039" s="19" t="inlineStr">
         <is>
-          <t>EUS-67943</t>
+          <t>EUS-77936</t>
         </is>
       </c>
       <c r="C1039" s="20" t="n"/>
@@ -20068,7 +20068,7 @@
     <row r="1051" ht="30" customHeight="1">
       <c r="A1051" s="16" t="inlineStr">
         <is>
-          <t>FICHA 71: EUS-97486</t>
+          <t>FICHA 71: EUS-52649</t>
         </is>
       </c>
       <c r="B1051" s="17" t="n"/>
@@ -20117,7 +20117,7 @@
       </c>
       <c r="B1054" s="19" t="inlineStr">
         <is>
-          <t>EUS-97486</t>
+          <t>EUS-52649</t>
         </is>
       </c>
       <c r="C1054" s="20" t="n"/>
@@ -20280,7 +20280,7 @@
     <row r="1066" ht="30" customHeight="1">
       <c r="A1066" s="16" t="inlineStr">
         <is>
-          <t>FICHA 72: EUS-36297</t>
+          <t>FICHA 72: EUS-26111</t>
         </is>
       </c>
       <c r="B1066" s="17" t="n"/>
@@ -20329,7 +20329,7 @@
       </c>
       <c r="B1069" s="19" t="inlineStr">
         <is>
-          <t>EUS-36297</t>
+          <t>EUS-26111</t>
         </is>
       </c>
       <c r="C1069" s="20" t="n"/>
@@ -20492,7 +20492,7 @@
     <row r="1081" ht="30" customHeight="1">
       <c r="A1081" s="16" t="inlineStr">
         <is>
-          <t>FICHA 73: EUS-41456</t>
+          <t>FICHA 73: EUS-52906</t>
         </is>
       </c>
       <c r="B1081" s="17" t="n"/>
@@ -20541,7 +20541,7 @@
       </c>
       <c r="B1084" s="19" t="inlineStr">
         <is>
-          <t>EUS-41456</t>
+          <t>EUS-52906</t>
         </is>
       </c>
       <c r="C1084" s="20" t="n"/>
@@ -23885,7 +23885,7 @@
     <row r="55" ht="28" customHeight="1">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>EUS-04804</t>
+          <t>EUS-54537</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
@@ -23921,7 +23921,7 @@
     <row r="56" ht="28" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>EUS-40390</t>
+          <t>EUS-50343</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
@@ -23957,7 +23957,7 @@
     <row r="57" ht="28" customHeight="1">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>EUS-81412</t>
+          <t>EUS-52804</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
@@ -23993,7 +23993,7 @@
     <row r="58" ht="28" customHeight="1">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>EUS-79656</t>
+          <t>EUS-42482</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
@@ -24029,7 +24029,7 @@
     <row r="59" ht="28" customHeight="1">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>EUS-17505</t>
+          <t>EUS-32296</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
@@ -24065,7 +24065,7 @@
     <row r="60" ht="28" customHeight="1">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>EUS-83702</t>
+          <t>EUS-21142</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
@@ -24101,7 +24101,7 @@
     <row r="61" ht="28" customHeight="1">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>EUS-22522</t>
+          <t>EUS-77157</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
@@ -24137,7 +24137,7 @@
     <row r="62" ht="28" customHeight="1">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>EUS-99695</t>
+          <t>EUS-47217</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
@@ -24173,7 +24173,7 @@
     <row r="63" ht="28" customHeight="1">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>EUS-65161</t>
+          <t>EUS-17090</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
@@ -24209,7 +24209,7 @@
     <row r="64" ht="28" customHeight="1">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>EUS-54622</t>
+          <t>EUS-54644</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
@@ -24245,7 +24245,7 @@
     <row r="65" ht="28" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>EUS-03111</t>
+          <t>EUS-08071</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
@@ -24281,7 +24281,7 @@
     <row r="66" ht="28" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>EUS-29680</t>
+          <t>EUS-53374</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
@@ -24317,7 +24317,7 @@
     <row r="67" ht="28" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>EUS-06937</t>
+          <t>EUS-08180</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
@@ -24353,7 +24353,7 @@
     <row r="68" ht="28" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>EUS-47446</t>
+          <t>EUS-15428</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
@@ -24389,7 +24389,7 @@
     <row r="69" ht="28" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>EUS-75016</t>
+          <t>EUS-70478</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
@@ -24425,7 +24425,7 @@
     <row r="70" ht="28" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>EUS-08635</t>
+          <t>EUS-60414</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
@@ -24461,7 +24461,7 @@
     <row r="71" ht="28" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>EUS-67943</t>
+          <t>EUS-77936</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
@@ -24497,7 +24497,7 @@
     <row r="72" ht="28" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>EUS-97486</t>
+          <t>EUS-52649</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
@@ -24533,7 +24533,7 @@
     <row r="73" ht="28" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>EUS-36297</t>
+          <t>EUS-26111</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
@@ -24569,7 +24569,7 @@
     <row r="74" ht="28" customHeight="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>EUS-41456</t>
+          <t>EUS-52906</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Update funding data 2026-03-23
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -685,7 +685,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 22/03/2026 06:38 - 73 convocatorias - 20 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 23/03/2026 06:59 - 73 convocatorias - 18 nuevas</t>
         </is>
       </c>
     </row>
@@ -3849,7 +3849,7 @@
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>EUS-54537</t>
+          <t>EUS-52341</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>EUS-50343</t>
+          <t>EUS-38721</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
@@ -3959,7 +3959,7 @@
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>EUS-52804</t>
+          <t>EUS-40875</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
@@ -3995,11 +3995,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L62" s="15" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
+      <c r="L62" s="6" t="inlineStr"/>
       <c r="M62" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
@@ -4014,7 +4010,7 @@
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>EUS-42482</t>
+          <t>EUS-46334</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
@@ -4069,7 +4065,7 @@
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>EUS-32296</t>
+          <t>EUS-62067</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
@@ -4124,7 +4120,7 @@
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>EUS-21142</t>
+          <t>EUS-84073</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -4179,7 +4175,7 @@
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>EUS-77157</t>
+          <t>EUS-89931</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
@@ -4234,7 +4230,7 @@
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>EUS-47217</t>
+          <t>EUS-60483</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
@@ -4289,7 +4285,7 @@
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>EUS-17090</t>
+          <t>EUS-46455</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -4344,7 +4340,7 @@
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>EUS-54644</t>
+          <t>EUS-38314</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -4380,11 +4376,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L69" s="15" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
+      <c r="L69" s="6" t="inlineStr"/>
       <c r="M69" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
@@ -4399,7 +4391,7 @@
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>EUS-08071</t>
+          <t>EUS-56475</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -4454,7 +4446,7 @@
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>EUS-53374</t>
+          <t>EUS-05137</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -4509,7 +4501,7 @@
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>EUS-08180</t>
+          <t>EUS-12265</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -4564,12 +4556,12 @@
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>EUS-15428</t>
+          <t>EUS-58053</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>Suministro de driver 75w y lamparas de 360w para farolas (alumbrado publico).(pre:2049409)</t>
+          <t>Suministro, Implementación y Soporte de un Servicio Digital de Telefonía y Videollamadas para los Centros Penitenciarios de Euskadi.</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
@@ -4619,12 +4611,12 @@
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>EUS-70478</t>
+          <t>EUS-97072</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>Suministro de material eléctrico (driver 150w) para alumbrado publico. maquinaria, instalaciones y utillaje. mantenimiento.</t>
+          <t>Suministro de driver 75w y lamparas de 360w para farolas (alumbrado publico).(pre:2049409)</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr">
@@ -4674,12 +4666,12 @@
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>EUS-60414</t>
+          <t>EUS-77422</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>Reparacion de la bomba del circuito de recirculacion del agua del polideportivo de orbea</t>
+          <t>Suministro de material eléctrico (driver 150w) para alumbrado publico. maquinaria, instalaciones y utillaje. mantenimiento.</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
@@ -4729,12 +4721,12 @@
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>EUS-77936</t>
+          <t>EUS-95174</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>Limpieza de foso ascensor errebal</t>
+          <t>Reparacion de la bomba del circuito de recirculacion del agua del polideportivo de orbea</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr">
@@ -4784,12 +4776,12 @@
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>EUS-52649</t>
+          <t>EUS-49048</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>Digitalización de la imagen del cartel de las jornadas de teatro</t>
+          <t>Limpieza de foso ascensor errebal</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
@@ -4839,12 +4831,12 @@
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>EUS-26111</t>
+          <t>EUS-90362</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>Servicio técnico para realizar la sustitución del servidor integrado en el proyector de cine digital del coliseo</t>
+          <t>Digitalización de la imagen del cartel de las jornadas de teatro</t>
         </is>
       </c>
       <c r="D78" s="6" t="inlineStr">
@@ -4894,12 +4886,12 @@
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>EUS-52906</t>
+          <t>EUS-98149</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>Actuación del dj xaibor el24 de junio en el parque de zuloagas</t>
+          <t>Servicio técnico para realizar la sustitución del servidor integrado en el proyector de cine digital del coliseo</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
@@ -16464,7 +16456,7 @@
     <row r="796" ht="30" customHeight="1">
       <c r="A796" s="16" t="inlineStr">
         <is>
-          <t>FICHA 54: EUS-54537</t>
+          <t>FICHA 54: EUS-52341</t>
         </is>
       </c>
       <c r="B796" s="17" t="n"/>
@@ -16513,7 +16505,7 @@
       </c>
       <c r="B799" s="19" t="inlineStr">
         <is>
-          <t>EUS-54537</t>
+          <t>EUS-52341</t>
         </is>
       </c>
       <c r="C799" s="20" t="n"/>
@@ -16676,7 +16668,7 @@
     <row r="811" ht="30" customHeight="1">
       <c r="A811" s="16" t="inlineStr">
         <is>
-          <t>FICHA 55: EUS-50343</t>
+          <t>FICHA 55: EUS-38721</t>
         </is>
       </c>
       <c r="B811" s="17" t="n"/>
@@ -16725,7 +16717,7 @@
       </c>
       <c r="B814" s="19" t="inlineStr">
         <is>
-          <t>EUS-50343</t>
+          <t>EUS-38721</t>
         </is>
       </c>
       <c r="C814" s="20" t="n"/>
@@ -16888,7 +16880,7 @@
     <row r="826" ht="30" customHeight="1">
       <c r="A826" s="16" t="inlineStr">
         <is>
-          <t>FICHA 56: EUS-52804</t>
+          <t>FICHA 56: EUS-40875</t>
         </is>
       </c>
       <c r="B826" s="17" t="n"/>
@@ -16937,7 +16929,7 @@
       </c>
       <c r="B829" s="19" t="inlineStr">
         <is>
-          <t>EUS-52804</t>
+          <t>EUS-40875</t>
         </is>
       </c>
       <c r="C829" s="20" t="n"/>
@@ -17100,7 +17092,7 @@
     <row r="841" ht="30" customHeight="1">
       <c r="A841" s="16" t="inlineStr">
         <is>
-          <t>FICHA 57: EUS-42482</t>
+          <t>FICHA 57: EUS-46334</t>
         </is>
       </c>
       <c r="B841" s="17" t="n"/>
@@ -17149,7 +17141,7 @@
       </c>
       <c r="B844" s="19" t="inlineStr">
         <is>
-          <t>EUS-42482</t>
+          <t>EUS-46334</t>
         </is>
       </c>
       <c r="C844" s="20" t="n"/>
@@ -17312,7 +17304,7 @@
     <row r="856" ht="30" customHeight="1">
       <c r="A856" s="16" t="inlineStr">
         <is>
-          <t>FICHA 58: EUS-32296</t>
+          <t>FICHA 58: EUS-62067</t>
         </is>
       </c>
       <c r="B856" s="17" t="n"/>
@@ -17361,7 +17353,7 @@
       </c>
       <c r="B859" s="19" t="inlineStr">
         <is>
-          <t>EUS-32296</t>
+          <t>EUS-62067</t>
         </is>
       </c>
       <c r="C859" s="20" t="n"/>
@@ -17524,7 +17516,7 @@
     <row r="871" ht="30" customHeight="1">
       <c r="A871" s="16" t="inlineStr">
         <is>
-          <t>FICHA 59: EUS-21142</t>
+          <t>FICHA 59: EUS-84073</t>
         </is>
       </c>
       <c r="B871" s="17" t="n"/>
@@ -17573,7 +17565,7 @@
       </c>
       <c r="B874" s="19" t="inlineStr">
         <is>
-          <t>EUS-21142</t>
+          <t>EUS-84073</t>
         </is>
       </c>
       <c r="C874" s="20" t="n"/>
@@ -17736,7 +17728,7 @@
     <row r="886" ht="30" customHeight="1">
       <c r="A886" s="16" t="inlineStr">
         <is>
-          <t>FICHA 60: EUS-77157</t>
+          <t>FICHA 60: EUS-89931</t>
         </is>
       </c>
       <c r="B886" s="17" t="n"/>
@@ -17785,7 +17777,7 @@
       </c>
       <c r="B889" s="19" t="inlineStr">
         <is>
-          <t>EUS-77157</t>
+          <t>EUS-89931</t>
         </is>
       </c>
       <c r="C889" s="20" t="n"/>
@@ -17948,7 +17940,7 @@
     <row r="901" ht="30" customHeight="1">
       <c r="A901" s="16" t="inlineStr">
         <is>
-          <t>FICHA 61: EUS-47217</t>
+          <t>FICHA 61: EUS-60483</t>
         </is>
       </c>
       <c r="B901" s="17" t="n"/>
@@ -17997,7 +17989,7 @@
       </c>
       <c r="B904" s="19" t="inlineStr">
         <is>
-          <t>EUS-47217</t>
+          <t>EUS-60483</t>
         </is>
       </c>
       <c r="C904" s="20" t="n"/>
@@ -18160,7 +18152,7 @@
     <row r="916" ht="30" customHeight="1">
       <c r="A916" s="16" t="inlineStr">
         <is>
-          <t>FICHA 62: EUS-17090</t>
+          <t>FICHA 62: EUS-46455</t>
         </is>
       </c>
       <c r="B916" s="17" t="n"/>
@@ -18209,7 +18201,7 @@
       </c>
       <c r="B919" s="19" t="inlineStr">
         <is>
-          <t>EUS-17090</t>
+          <t>EUS-46455</t>
         </is>
       </c>
       <c r="C919" s="20" t="n"/>
@@ -18372,7 +18364,7 @@
     <row r="931" ht="30" customHeight="1">
       <c r="A931" s="16" t="inlineStr">
         <is>
-          <t>FICHA 63: EUS-54644</t>
+          <t>FICHA 63: EUS-38314</t>
         </is>
       </c>
       <c r="B931" s="17" t="n"/>
@@ -18421,7 +18413,7 @@
       </c>
       <c r="B934" s="19" t="inlineStr">
         <is>
-          <t>EUS-54644</t>
+          <t>EUS-38314</t>
         </is>
       </c>
       <c r="C934" s="20" t="n"/>
@@ -18584,7 +18576,7 @@
     <row r="946" ht="30" customHeight="1">
       <c r="A946" s="16" t="inlineStr">
         <is>
-          <t>FICHA 64: EUS-08071</t>
+          <t>FICHA 64: EUS-56475</t>
         </is>
       </c>
       <c r="B946" s="17" t="n"/>
@@ -18633,7 +18625,7 @@
       </c>
       <c r="B949" s="19" t="inlineStr">
         <is>
-          <t>EUS-08071</t>
+          <t>EUS-56475</t>
         </is>
       </c>
       <c r="C949" s="20" t="n"/>
@@ -18796,7 +18788,7 @@
     <row r="961" ht="30" customHeight="1">
       <c r="A961" s="16" t="inlineStr">
         <is>
-          <t>FICHA 65: EUS-53374</t>
+          <t>FICHA 65: EUS-05137</t>
         </is>
       </c>
       <c r="B961" s="17" t="n"/>
@@ -18845,7 +18837,7 @@
       </c>
       <c r="B964" s="19" t="inlineStr">
         <is>
-          <t>EUS-53374</t>
+          <t>EUS-05137</t>
         </is>
       </c>
       <c r="C964" s="20" t="n"/>
@@ -19008,7 +19000,7 @@
     <row r="976" ht="30" customHeight="1">
       <c r="A976" s="16" t="inlineStr">
         <is>
-          <t>FICHA 66: EUS-08180</t>
+          <t>FICHA 66: EUS-12265</t>
         </is>
       </c>
       <c r="B976" s="17" t="n"/>
@@ -19057,7 +19049,7 @@
       </c>
       <c r="B979" s="19" t="inlineStr">
         <is>
-          <t>EUS-08180</t>
+          <t>EUS-12265</t>
         </is>
       </c>
       <c r="C979" s="20" t="n"/>
@@ -19220,7 +19212,7 @@
     <row r="991" ht="30" customHeight="1">
       <c r="A991" s="16" t="inlineStr">
         <is>
-          <t>FICHA 67: EUS-15428</t>
+          <t>FICHA 67: EUS-58053</t>
         </is>
       </c>
       <c r="B991" s="17" t="n"/>
@@ -19253,7 +19245,7 @@
       </c>
       <c r="B993" s="19" t="inlineStr">
         <is>
-          <t>Suministro de driver 75w y lamparas de 360w para farolas (alumbrado publico).(pre:2049409)</t>
+          <t>Suministro, Implementación y Soporte de un Servicio Digital de Telefonía y Videollamadas para los Centros Penitenciarios de Euskadi.</t>
         </is>
       </c>
       <c r="C993" s="20" t="n"/>
@@ -19269,7 +19261,7 @@
       </c>
       <c r="B994" s="19" t="inlineStr">
         <is>
-          <t>EUS-15428</t>
+          <t>EUS-58053</t>
         </is>
       </c>
       <c r="C994" s="20" t="n"/>
@@ -19389,7 +19381,7 @@
       </c>
       <c r="B1002" s="19" t="inlineStr">
         <is>
-          <t>energia</t>
+          <t>alumbrado</t>
         </is>
       </c>
       <c r="C1002" s="20" t="n"/>
@@ -19421,7 +19413,7 @@
       </c>
       <c r="B1004" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-driver-75w-y-lamparas-360w-farolas-alumbrado-publico-pre-2049409/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-implementacion-y-soporte-servicio-digital-telefonia-y-videollamadas-centros-penitenciarios-euskadi/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1004" s="20" t="n"/>
@@ -19432,7 +19424,7 @@
     <row r="1006" ht="30" customHeight="1">
       <c r="A1006" s="16" t="inlineStr">
         <is>
-          <t>FICHA 68: EUS-70478</t>
+          <t>FICHA 68: EUS-97072</t>
         </is>
       </c>
       <c r="B1006" s="17" t="n"/>
@@ -19465,7 +19457,7 @@
       </c>
       <c r="B1008" s="19" t="inlineStr">
         <is>
-          <t>Suministro de material eléctrico (driver 150w) para alumbrado publico. maquinaria, instalaciones y utillaje. mantenimiento.</t>
+          <t>Suministro de driver 75w y lamparas de 360w para farolas (alumbrado publico).(pre:2049409)</t>
         </is>
       </c>
       <c r="C1008" s="20" t="n"/>
@@ -19481,7 +19473,7 @@
       </c>
       <c r="B1009" s="19" t="inlineStr">
         <is>
-          <t>EUS-70478</t>
+          <t>EUS-97072</t>
         </is>
       </c>
       <c r="C1009" s="20" t="n"/>
@@ -19601,7 +19593,7 @@
       </c>
       <c r="B1017" s="19" t="inlineStr">
         <is>
-          <t>energia</t>
+          <t>alumbrado</t>
         </is>
       </c>
       <c r="C1017" s="20" t="n"/>
@@ -19633,7 +19625,7 @@
       </c>
       <c r="B1019" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-material-electrico-driver-150w-alumbrado-publico-maquinaria-instalaciones-y-utillaje-mantenimiento/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-driver-75w-y-lamparas-360w-farolas-alumbrado-publico-pre-2049409/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1019" s="20" t="n"/>
@@ -19644,7 +19636,7 @@
     <row r="1021" ht="30" customHeight="1">
       <c r="A1021" s="16" t="inlineStr">
         <is>
-          <t>FICHA 69: EUS-60414</t>
+          <t>FICHA 69: EUS-77422</t>
         </is>
       </c>
       <c r="B1021" s="17" t="n"/>
@@ -19677,7 +19669,7 @@
       </c>
       <c r="B1023" s="19" t="inlineStr">
         <is>
-          <t>Reparacion de la bomba del circuito de recirculacion del agua del polideportivo de orbea</t>
+          <t>Suministro de material eléctrico (driver 150w) para alumbrado publico. maquinaria, instalaciones y utillaje. mantenimiento.</t>
         </is>
       </c>
       <c r="C1023" s="20" t="n"/>
@@ -19693,7 +19685,7 @@
       </c>
       <c r="B1024" s="19" t="inlineStr">
         <is>
-          <t>EUS-60414</t>
+          <t>EUS-77422</t>
         </is>
       </c>
       <c r="C1024" s="20" t="n"/>
@@ -19813,7 +19805,7 @@
       </c>
       <c r="B1032" s="19" t="inlineStr">
         <is>
-          <t>energia</t>
+          <t>alumbrado</t>
         </is>
       </c>
       <c r="C1032" s="20" t="n"/>
@@ -19845,7 +19837,7 @@
       </c>
       <c r="B1034" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/reparacion-bomba-del-circuito-recirculacion-del-agua-del-polideportivo-orbea/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-material-electrico-driver-150w-alumbrado-publico-maquinaria-instalaciones-y-utillaje-mantenimiento/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1034" s="20" t="n"/>
@@ -19856,7 +19848,7 @@
     <row r="1036" ht="30" customHeight="1">
       <c r="A1036" s="16" t="inlineStr">
         <is>
-          <t>FICHA 70: EUS-77936</t>
+          <t>FICHA 70: EUS-95174</t>
         </is>
       </c>
       <c r="B1036" s="17" t="n"/>
@@ -19881,7 +19873,7 @@
       <c r="E1037" s="20" t="n"/>
       <c r="F1037" s="20" t="n"/>
     </row>
-    <row r="1038" ht="20" customHeight="1">
+    <row r="1038" ht="45" customHeight="1">
       <c r="A1038" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -19889,7 +19881,7 @@
       </c>
       <c r="B1038" s="19" t="inlineStr">
         <is>
-          <t>Limpieza de foso ascensor errebal</t>
+          <t>Reparacion de la bomba del circuito de recirculacion del agua del polideportivo de orbea</t>
         </is>
       </c>
       <c r="C1038" s="20" t="n"/>
@@ -19905,7 +19897,7 @@
       </c>
       <c r="B1039" s="19" t="inlineStr">
         <is>
-          <t>EUS-77936</t>
+          <t>EUS-95174</t>
         </is>
       </c>
       <c r="C1039" s="20" t="n"/>
@@ -20025,7 +20017,7 @@
       </c>
       <c r="B1047" s="19" t="inlineStr">
         <is>
-          <t>energia</t>
+          <t>alumbrado</t>
         </is>
       </c>
       <c r="C1047" s="20" t="n"/>
@@ -20057,7 +20049,7 @@
       </c>
       <c r="B1049" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/limpieza-foso-ascensor-errebal/expgeeibar20830/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/reparacion-bomba-del-circuito-recirculacion-del-agua-del-polideportivo-orbea/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1049" s="20" t="n"/>
@@ -20068,7 +20060,7 @@
     <row r="1051" ht="30" customHeight="1">
       <c r="A1051" s="16" t="inlineStr">
         <is>
-          <t>FICHA 71: EUS-52649</t>
+          <t>FICHA 71: EUS-49048</t>
         </is>
       </c>
       <c r="B1051" s="17" t="n"/>
@@ -20101,7 +20093,7 @@
       </c>
       <c r="B1053" s="19" t="inlineStr">
         <is>
-          <t>Digitalización de la imagen del cartel de las jornadas de teatro</t>
+          <t>Limpieza de foso ascensor errebal</t>
         </is>
       </c>
       <c r="C1053" s="20" t="n"/>
@@ -20117,7 +20109,7 @@
       </c>
       <c r="B1054" s="19" t="inlineStr">
         <is>
-          <t>EUS-52649</t>
+          <t>EUS-49048</t>
         </is>
       </c>
       <c r="C1054" s="20" t="n"/>
@@ -20237,7 +20229,7 @@
       </c>
       <c r="B1062" s="19" t="inlineStr">
         <is>
-          <t>energia</t>
+          <t>alumbrado</t>
         </is>
       </c>
       <c r="C1062" s="20" t="n"/>
@@ -20269,7 +20261,7 @@
       </c>
       <c r="B1064" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/digitalizacion-imagen-del-cartel-jornadas-teatro/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/limpieza-foso-ascensor-errebal/expgeeibar20830/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1064" s="20" t="n"/>
@@ -20280,7 +20272,7 @@
     <row r="1066" ht="30" customHeight="1">
       <c r="A1066" s="16" t="inlineStr">
         <is>
-          <t>FICHA 72: EUS-26111</t>
+          <t>FICHA 72: EUS-90362</t>
         </is>
       </c>
       <c r="B1066" s="17" t="n"/>
@@ -20305,7 +20297,7 @@
       <c r="E1067" s="20" t="n"/>
       <c r="F1067" s="20" t="n"/>
     </row>
-    <row r="1068" ht="45" customHeight="1">
+    <row r="1068" ht="20" customHeight="1">
       <c r="A1068" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -20313,7 +20305,7 @@
       </c>
       <c r="B1068" s="19" t="inlineStr">
         <is>
-          <t>Servicio técnico para realizar la sustitución del servidor integrado en el proyector de cine digital del coliseo</t>
+          <t>Digitalización de la imagen del cartel de las jornadas de teatro</t>
         </is>
       </c>
       <c r="C1068" s="20" t="n"/>
@@ -20329,7 +20321,7 @@
       </c>
       <c r="B1069" s="19" t="inlineStr">
         <is>
-          <t>EUS-26111</t>
+          <t>EUS-90362</t>
         </is>
       </c>
       <c r="C1069" s="20" t="n"/>
@@ -20449,7 +20441,7 @@
       </c>
       <c r="B1077" s="19" t="inlineStr">
         <is>
-          <t>energia</t>
+          <t>alumbrado</t>
         </is>
       </c>
       <c r="C1077" s="20" t="n"/>
@@ -20481,7 +20473,7 @@
       </c>
       <c r="B1079" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-tecnico-realizar-sustitucion-del-servidor-integrado-proyector-cine-digital-del-coliseo/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/digitalizacion-imagen-del-cartel-jornadas-teatro/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1079" s="20" t="n"/>
@@ -20492,7 +20484,7 @@
     <row r="1081" ht="30" customHeight="1">
       <c r="A1081" s="16" t="inlineStr">
         <is>
-          <t>FICHA 73: EUS-52906</t>
+          <t>FICHA 73: EUS-98149</t>
         </is>
       </c>
       <c r="B1081" s="17" t="n"/>
@@ -20517,7 +20509,7 @@
       <c r="E1082" s="20" t="n"/>
       <c r="F1082" s="20" t="n"/>
     </row>
-    <row r="1083" ht="20" customHeight="1">
+    <row r="1083" ht="45" customHeight="1">
       <c r="A1083" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -20525,7 +20517,7 @@
       </c>
       <c r="B1083" s="19" t="inlineStr">
         <is>
-          <t>Actuación del dj xaibor el24 de junio en el parque de zuloagas</t>
+          <t>Servicio técnico para realizar la sustitución del servidor integrado en el proyector de cine digital del coliseo</t>
         </is>
       </c>
       <c r="C1083" s="20" t="n"/>
@@ -20541,7 +20533,7 @@
       </c>
       <c r="B1084" s="19" t="inlineStr">
         <is>
-          <t>EUS-52906</t>
+          <t>EUS-98149</t>
         </is>
       </c>
       <c r="C1084" s="20" t="n"/>
@@ -20661,7 +20653,7 @@
       </c>
       <c r="B1092" s="19" t="inlineStr">
         <is>
-          <t>energia</t>
+          <t>alumbrado</t>
         </is>
       </c>
       <c r="C1092" s="20" t="n"/>
@@ -20693,7 +20685,7 @@
       </c>
       <c r="B1094" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/actuacion-del-dj-xaibor-el24-junio-parque-zuloagas/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-tecnico-realizar-sustitucion-del-servidor-integrado-proyector-cine-digital-del-coliseo/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1094" s="20" t="n"/>
@@ -23885,7 +23877,7 @@
     <row r="55" ht="28" customHeight="1">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>EUS-54537</t>
+          <t>EUS-52341</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
@@ -23921,7 +23913,7 @@
     <row r="56" ht="28" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>EUS-50343</t>
+          <t>EUS-38721</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
@@ -23957,7 +23949,7 @@
     <row r="57" ht="28" customHeight="1">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>EUS-52804</t>
+          <t>EUS-40875</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
@@ -23993,7 +23985,7 @@
     <row r="58" ht="28" customHeight="1">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>EUS-42482</t>
+          <t>EUS-46334</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
@@ -24029,7 +24021,7 @@
     <row r="59" ht="28" customHeight="1">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>EUS-32296</t>
+          <t>EUS-62067</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
@@ -24065,7 +24057,7 @@
     <row r="60" ht="28" customHeight="1">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>EUS-21142</t>
+          <t>EUS-84073</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
@@ -24101,7 +24093,7 @@
     <row r="61" ht="28" customHeight="1">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>EUS-77157</t>
+          <t>EUS-89931</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
@@ -24137,7 +24129,7 @@
     <row r="62" ht="28" customHeight="1">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>EUS-47217</t>
+          <t>EUS-60483</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
@@ -24173,7 +24165,7 @@
     <row r="63" ht="28" customHeight="1">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>EUS-17090</t>
+          <t>EUS-46455</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
@@ -24209,7 +24201,7 @@
     <row r="64" ht="28" customHeight="1">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>EUS-54644</t>
+          <t>EUS-38314</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
@@ -24245,7 +24237,7 @@
     <row r="65" ht="28" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>EUS-08071</t>
+          <t>EUS-56475</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
@@ -24281,7 +24273,7 @@
     <row r="66" ht="28" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>EUS-53374</t>
+          <t>EUS-05137</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
@@ -24317,7 +24309,7 @@
     <row r="67" ht="28" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>EUS-08180</t>
+          <t>EUS-12265</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
@@ -24353,12 +24345,12 @@
     <row r="68" ht="28" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>EUS-15428</t>
+          <t>EUS-58053</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>Suministro de driver 75w y lamparas de 360w para farolas (al</t>
+          <t xml:space="preserve">Suministro, Implementación y Soporte de un Servicio Digital </t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -24389,12 +24381,12 @@
     <row r="69" ht="28" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>EUS-70478</t>
+          <t>EUS-97072</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>Suministro de material eléctrico (driver 150w) para alumbrad</t>
+          <t>Suministro de driver 75w y lamparas de 360w para farolas (al</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -24425,12 +24417,12 @@
     <row r="70" ht="28" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>EUS-60414</t>
+          <t>EUS-77422</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>Reparacion de la bomba del circuito de recirculacion del agu</t>
+          <t>Suministro de material eléctrico (driver 150w) para alumbrad</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -24461,12 +24453,12 @@
     <row r="71" ht="28" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>EUS-77936</t>
+          <t>EUS-95174</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>Limpieza de foso ascensor errebal</t>
+          <t>Reparacion de la bomba del circuito de recirculacion del agu</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -24497,12 +24489,12 @@
     <row r="72" ht="28" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>EUS-52649</t>
+          <t>EUS-49048</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>Digitalización de la imagen del cartel de las jornadas de te</t>
+          <t>Limpieza de foso ascensor errebal</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -24533,12 +24525,12 @@
     <row r="73" ht="28" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>EUS-26111</t>
+          <t>EUS-90362</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>Servicio técnico para realizar la sustitución del servidor i</t>
+          <t>Digitalización de la imagen del cartel de las jornadas de te</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -24569,12 +24561,12 @@
     <row r="74" ht="28" customHeight="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>EUS-52906</t>
+          <t>EUS-98149</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>Actuación del dj xaibor el24 de junio en el parque de zuloag</t>
+          <t>Servicio técnico para realizar la sustitución del servidor i</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Update funding data 2026-03-24
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Recursos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$79</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$77</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -657,7 +657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M79"/>
+  <dimension ref="A1:M82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -685,7 +685,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 23/03/2026 06:59 - 73 convocatorias - 18 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 24/03/2026 06:54 - 76 convocatorias - 22 nuevas</t>
         </is>
       </c>
     </row>
@@ -3795,12 +3795,12 @@
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>c427200b-e175-4101-b8d4-4ec219539e45-PIN</t>
+          <t>4b45d249-5739-4bf7-9595-a4715b73c2f6-EXA</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>Mission Implementation Platform for Mission "A Soil Deal for Europe"</t>
+          <t>Border regions Peer exchange on solving border obstacles</t>
         </is>
       </c>
       <c r="D58" s="6" t="inlineStr"/>
@@ -3824,7 +3824,7 @@
       </c>
       <c r="K58" s="6" t="inlineStr">
         <is>
-          <t>Mission Implementation Platform for Mission "A Soil Deal for Europe"</t>
+          <t>Border regions Peer exchange on solving border obstacles</t>
         </is>
       </c>
       <c r="L58" s="6" t="inlineStr"/>
@@ -3834,65 +3834,57 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="28" customHeight="1">
-      <c r="A59" s="13" t="inlineStr">
+    <row r="59" ht="40" customHeight="1">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>Europa</t>
+        </is>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>c427200b-e175-4101-b8d4-4ec219539e45-PIN</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>Mission Implementation Platform for Mission "A Soil Deal for Europe"</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr"/>
+      <c r="E59" s="11" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F59" s="6" t="inlineStr"/>
+      <c r="G59" s="6" t="inlineStr"/>
+      <c r="H59" s="6" t="inlineStr"/>
+      <c r="I59" s="11" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="J59" s="6" t="inlineStr">
+        <is>
+          <t>Revisar relevancia para el Ayuntamiento de Bilbao.</t>
+        </is>
+      </c>
+      <c r="K59" s="6" t="inlineStr">
+        <is>
+          <t>Mission Implementation Platform for Mission "A Soil Deal for Europe"</t>
+        </is>
+      </c>
+      <c r="L59" s="6" t="inlineStr"/>
+      <c r="M59" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="28" customHeight="1">
+      <c r="A60" s="13" t="inlineStr">
         <is>
           <t>🟢 Euskadi</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="40" customHeight="1">
-      <c r="A60" s="14" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="B60" s="6" t="inlineStr">
-        <is>
-          <t>EUS-52341</t>
-        </is>
-      </c>
-      <c r="C60" s="6" t="inlineStr">
-        <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
-        </is>
-      </c>
-      <c r="D60" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="E60" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F60" s="6" t="inlineStr"/>
-      <c r="G60" s="6" t="inlineStr"/>
-      <c r="H60" s="6" t="inlineStr">
-        <is>
-          <t>Ayuda/Subvencion Euskadi</t>
-        </is>
-      </c>
-      <c r="I60" s="8" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
-      <c r="J60" s="6" t="inlineStr"/>
-      <c r="K60" s="6" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="L60" s="15" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="M60" s="9" t="inlineStr">
-        <is>
-          <t>Ver</t>
         </is>
       </c>
     </row>
@@ -3904,12 +3896,12 @@
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>EUS-38721</t>
+          <t>EUS-64028</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la gestión sostenible de los recursos pesqueros 2026</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
@@ -3959,12 +3951,12 @@
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>EUS-40875</t>
+          <t>EUS-77748</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la recogida de residuos con la participación de los pescadores en el mar y las playas 2026</t>
+          <t>Ayudas a la gestión sostenible de los recursos pesqueros 2026</t>
         </is>
       </c>
       <c r="D62" s="6" t="inlineStr">
@@ -3995,7 +3987,11 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L62" s="6" t="inlineStr"/>
+      <c r="L62" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
       <c r="M62" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
@@ -4010,12 +4006,12 @@
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>EUS-46334</t>
+          <t>EUS-23804</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático sin incremento de capacidad 2026</t>
+          <t>Ayudas a la recogida de residuos con la participación de los pescadores en el mar y las playas 2026</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
@@ -4065,12 +4061,12 @@
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>EUS-62067</t>
+          <t>EUS-89133</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio climático sin incremento de capacidad 2026</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
@@ -4090,9 +4086,9 @@
           <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
-      <c r="I64" s="10" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
+      <c r="I64" s="8" t="inlineStr">
+        <is>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="J64" s="6" t="inlineStr"/>
@@ -4120,12 +4116,12 @@
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>EUS-84073</t>
+          <t>EUS-48991</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>Ayudas al valor añadido, economía circular y seguridad alimentaria 2026</t>
+          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
@@ -4175,12 +4171,12 @@
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>EUS-89931</t>
+          <t>EUS-06375</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>Vino: el Gobierno Vasco volverá a convocar este mes las ayudas al arranque o cosecha en verde del viñedo, que van a contemplar como estructurales tras reformar la UE jurídicamente su Intervención Sect</t>
+          <t>Ayudas al valor añadido, economía circular y seguridad alimentaria 2026</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
@@ -4230,12 +4226,12 @@
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>EUS-60483</t>
+          <t>EUS-79267</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de aceleración de proyectos, a localidades de menos de 20.000 habitantes son objeto de convocatoria abierta hasta el 17.03.26. Transformacione</t>
+          <t>Vino: el Gobierno Vasco volverá a convocar este mes las ayudas al arranque o cosecha en verde del viñedo, que van a contemplar como estructurales tras reformar la UE jurídicamente su Intervención Sect</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
@@ -4285,12 +4281,12 @@
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>EUS-46455</t>
+          <t>EUS-85579</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para consorcios internacionales de I+D+i. Jornada del Gobierno Vasco y con Enterprise Europe Network y otros socios. Digitalización, dispositivos,</t>
+          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de aceleración de proyectos, a localidades de menos de 20.000 habitantes son objeto de convocatoria abierta hasta el 17.03.26. Transformacione</t>
         </is>
       </c>
       <c r="D68" s="6" t="inlineStr">
@@ -4340,12 +4336,12 @@
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>EUS-38314</t>
+          <t>EUS-03347</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinancia convocatorias de ayudas de las Diputaciones a explotaciones con limitaciones o desfavorecidas, y a compromisos medioambientales, climátic</t>
+          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para consorcios internacionales de I+D+i. Jornada del Gobierno Vasco y con Enterprise Europe Network y otros socios. Digitalización, dispositivos,</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
@@ -4376,7 +4372,11 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L69" s="6" t="inlineStr"/>
+      <c r="L69" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
       <c r="M69" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
@@ -4391,12 +4391,12 @@
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>EUS-56475</t>
+          <t>EUS-87925</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>Digital Europe, Horizon (programas de la UE). Apoyos para consorcios interestatales de I+D+i. IA, robótica, cuántica, computación, ciberseguridad, electrónica, fotónica, TICs e internet avanzadas, esp</t>
+          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinancia convocatorias de ayudas de las Diputaciones a explotaciones con limitaciones o desfavorecidas, y a compromisos medioambientales, climátic</t>
         </is>
       </c>
       <c r="D70" s="6" t="inlineStr">
@@ -4446,12 +4446,12 @@
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>EUS-05137</t>
+          <t>EUS-21599</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>Política Agraria Común de la UE de 2026, y sus ayudas abiertas hasta el 30.4.26: el pilar 1, con el Fondo Europeo Agrícola de Garantía Agraria FEAGA, aborda sostenibilidad de renta, ayuda redistributi</t>
+          <t>Digital Europe, Horizon (programas de la UE). Apoyos para consorcios interestatales de I+D+i. IA, robótica, cuántica, computación, ciberseguridad, electrónica, fotónica, TICs e internet avanzadas, esp</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
@@ -4501,12 +4501,12 @@
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>EUS-12265</t>
+          <t>EUS-91637</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>Programa de impulso a las ciudades y territorios inteligentes para el fomento del desarrollo económico y productivo, que podrá ser cofinanciado por el Programa Plurirregional 2021-2027 del Fondo Europ</t>
+          <t>Política Agraria Común de la UE de 2026, y sus ayudas abiertas hasta el 30.4.26: el pilar 1, con el Fondo Europeo Agrícola de Garantía Agraria FEAGA, aborda sostenibilidad de renta, ayuda redistributi</t>
         </is>
       </c>
       <c r="D72" s="6" t="inlineStr">
@@ -4556,12 +4556,12 @@
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>EUS-58053</t>
+          <t>EUS-38365</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>Suministro, Implementación y Soporte de un Servicio Digital de Telefonía y Videollamadas para los Centros Penitenciarios de Euskadi.</t>
+          <t>Programa de impulso a las ciudades y territorios inteligentes para el fomento del desarrollo económico y productivo, que podrá ser cofinanciado por el Programa Plurirregional 2021-2027 del Fondo Europ</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
@@ -4578,7 +4578,7 @@
       <c r="G73" s="6" t="inlineStr"/>
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="I73" s="10" t="inlineStr">
@@ -4611,12 +4611,12 @@
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>EUS-97072</t>
+          <t>EUS-84600</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>Suministro de driver 75w y lamparas de 360w para farolas (alumbrado publico).(pre:2049409)</t>
+          <t>Servicio de Punto Verde Móvil en el Territorio Histórico de Álava</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr">
@@ -4666,12 +4666,12 @@
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>EUS-77422</t>
+          <t>EUS-18669</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>Suministro de material eléctrico (driver 150w) para alumbrado publico. maquinaria, instalaciones y utillaje. mantenimiento.</t>
+          <t>Servicio de agencia de viajes para el Departamento de Hacienda y Finanzas con cláusulas ambientales.</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
@@ -4721,12 +4721,12 @@
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>EUS-95174</t>
+          <t>EUS-29543</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>Reparacion de la bomba del circuito de recirculacion del agua del polideportivo de orbea</t>
+          <t>Conferencia sobre "la bicicleta, un máquina móvil, veloz y bella"</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr">
@@ -4776,12 +4776,12 @@
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>EUS-49048</t>
+          <t>EUS-17370</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>Limpieza de foso ascensor errebal</t>
+          <t>Organización parque infantil de Navidad</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
@@ -4831,12 +4831,12 @@
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>EUS-90362</t>
+          <t>EUS-46342</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>Digitalización de la imagen del cartel de las jornadas de teatro</t>
+          <t>Alumbrado publico pasos peatonales en La Calzada</t>
         </is>
       </c>
       <c r="D78" s="6" t="inlineStr">
@@ -4886,12 +4886,12 @@
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>EUS-98149</t>
+          <t>EUS-02378</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>Servicio técnico para realizar la sustitución del servidor integrado en el proyector de cine digital del coliseo</t>
+          <t>Reparación faldón cubierta Museo Santa Clara</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
@@ -4933,10 +4933,175 @@
         </is>
       </c>
     </row>
+    <row r="80" ht="40" customHeight="1">
+      <c r="A80" s="14" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>EUS-69611</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>Limpieza y desescombro desatasco colector de saneamiento</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F80" s="6" t="inlineStr"/>
+      <c r="G80" s="6" t="inlineStr"/>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I80" s="10" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J80" s="6" t="inlineStr"/>
+      <c r="K80" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L80" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M80" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="40" customHeight="1">
+      <c r="A81" s="14" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>EUS-00349</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>Reparación instalación fotovoltaica refugio del Kolitza</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F81" s="6" t="inlineStr"/>
+      <c r="G81" s="6" t="inlineStr"/>
+      <c r="H81" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I81" s="10" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J81" s="6" t="inlineStr"/>
+      <c r="K81" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L81" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M81" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="40" customHeight="1">
+      <c r="A82" s="14" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>EUS-93515</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>Formación en jardineria forestal</t>
+        </is>
+      </c>
+      <c r="D82" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F82" s="6" t="inlineStr"/>
+      <c r="G82" s="6" t="inlineStr"/>
+      <c r="H82" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I82" s="10" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J82" s="6" t="inlineStr"/>
+      <c r="K82" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L82" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M82" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:M79"/>
+  <autoFilter ref="A4:M82"/>
   <mergeCells count="4">
-    <mergeCell ref="A59:M59"/>
+    <mergeCell ref="A60:M60"/>
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A5:M5"/>
@@ -4995,7 +5160,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M56" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M57" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M58" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M60" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M59" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M61" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M62" r:id="rId56"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M63" r:id="rId57"/>
@@ -5015,6 +5180,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M77" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M78" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M79" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M80" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M81" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M82" r:id="rId76"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5026,7 +5194,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1094"/>
+  <dimension ref="A1:F1139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -16248,7 +16416,7 @@
     <row r="781" ht="30" customHeight="1">
       <c r="A781" s="16" t="inlineStr">
         <is>
-          <t>FICHA 53: c427200b-e175-4101-b8d4-4ec219539e45-PIN</t>
+          <t>FICHA 53: 4b45d249-5739-4bf7-9595-a4715b73c2f6-EXA</t>
         </is>
       </c>
       <c r="B781" s="17" t="n"/>
@@ -16281,7 +16449,7 @@
       </c>
       <c r="B783" s="19" t="inlineStr">
         <is>
-          <t>Mission Implementation Platform for Mission "A Soil Deal for Europe"</t>
+          <t>Border regions Peer exchange on solving border obstacles</t>
         </is>
       </c>
       <c r="C783" s="20" t="n"/>
@@ -16297,7 +16465,7 @@
       </c>
       <c r="B784" s="19" t="inlineStr">
         <is>
-          <t>c427200b-e175-4101-b8d4-4ec219539e45-PIN</t>
+          <t>4b45d249-5739-4bf7-9595-a4715b73c2f6-EXA</t>
         </is>
       </c>
       <c r="C784" s="20" t="n"/>
@@ -16385,7 +16553,7 @@
       </c>
       <c r="B790" s="19" t="inlineStr">
         <is>
-          <t>REA/2025/OP/0009-PIN</t>
+          <t>EC-REGIO/2025/MVP/0036-EXA</t>
         </is>
       </c>
       <c r="C790" s="20" t="n"/>
@@ -16401,7 +16569,7 @@
       </c>
       <c r="B791" s="19" t="inlineStr">
         <is>
-          <t>Mission Implementation Platform for Mission "A Soil Deal for Europe"</t>
+          <t>Border regions Peer exchange on solving border obstacles</t>
         </is>
       </c>
       <c r="C791" s="20" t="n"/>
@@ -16445,7 +16613,7 @@
       </c>
       <c r="B794" s="22" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/c427200b-e175-4101-b8d4-4ec219539e45-PIN</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/4b45d249-5739-4bf7-9595-a4715b73c2f6-EXA</t>
         </is>
       </c>
       <c r="C794" s="20" t="n"/>
@@ -16456,7 +16624,7 @@
     <row r="796" ht="30" customHeight="1">
       <c r="A796" s="16" t="inlineStr">
         <is>
-          <t>FICHA 54: EUS-52341</t>
+          <t>FICHA 54: c427200b-e175-4101-b8d4-4ec219539e45-PIN</t>
         </is>
       </c>
       <c r="B796" s="17" t="n"/>
@@ -16473,7 +16641,7 @@
       </c>
       <c r="B797" s="19" t="inlineStr">
         <is>
-          <t>🟢 Euskadi</t>
+          <t>🇪🇺 Europa</t>
         </is>
       </c>
       <c r="C797" s="20" t="n"/>
@@ -16481,7 +16649,7 @@
       <c r="E797" s="20" t="n"/>
       <c r="F797" s="20" t="n"/>
     </row>
-    <row r="798" ht="45" customHeight="1">
+    <row r="798" ht="20" customHeight="1">
       <c r="A798" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -16489,7 +16657,7 @@
       </c>
       <c r="B798" s="19" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
+          <t>Mission Implementation Platform for Mission "A Soil Deal for Europe"</t>
         </is>
       </c>
       <c r="C798" s="20" t="n"/>
@@ -16505,7 +16673,7 @@
       </c>
       <c r="B799" s="19" t="inlineStr">
         <is>
-          <t>EUS-52341</t>
+          <t>c427200b-e175-4101-b8d4-4ec219539e45-PIN</t>
         </is>
       </c>
       <c r="C799" s="20" t="n"/>
@@ -16519,11 +16687,7 @@
           <t>Programa</t>
         </is>
       </c>
-      <c r="B800" s="19" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
+      <c r="B800" s="19" t="inlineStr"/>
       <c r="C800" s="20" t="n"/>
       <c r="D800" s="20" t="n"/>
       <c r="E800" s="20" t="n"/>
@@ -16537,7 +16701,7 @@
       </c>
       <c r="B801" s="19" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C801" s="20" t="n"/>
@@ -16581,7 +16745,7 @@
       </c>
       <c r="B804" s="19" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>No disponible</t>
         </is>
       </c>
       <c r="C804" s="20" t="n"/>
@@ -16595,7 +16759,11 @@
           <t>Call ID</t>
         </is>
       </c>
-      <c r="B805" s="19" t="inlineStr"/>
+      <c r="B805" s="19" t="inlineStr">
+        <is>
+          <t>REA/2025/OP/0009-PIN</t>
+        </is>
+      </c>
       <c r="C805" s="20" t="n"/>
       <c r="D805" s="20" t="n"/>
       <c r="E805" s="20" t="n"/>
@@ -16609,7 +16777,7 @@
       </c>
       <c r="B806" s="19" t="inlineStr">
         <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+          <t>Mission Implementation Platform for Mission "A Soil Deal for Europe"</t>
         </is>
       </c>
       <c r="C806" s="20" t="n"/>
@@ -16623,11 +16791,7 @@
           <t>Tags</t>
         </is>
       </c>
-      <c r="B807" s="19" t="inlineStr">
-        <is>
-          <t>energia</t>
-        </is>
-      </c>
+      <c r="B807" s="19" t="inlineStr"/>
       <c r="C807" s="20" t="n"/>
       <c r="D807" s="20" t="n"/>
       <c r="E807" s="20" t="n"/>
@@ -16639,9 +16803,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B808" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ALTA — </t>
+      <c r="B808" s="19" t="inlineStr">
+        <is>
+          <t>INFO — Revisar relevancia para el Ayuntamiento de Bilbao.</t>
         </is>
       </c>
       <c r="C808" s="20" t="n"/>
@@ -16657,7 +16821,7 @@
       </c>
       <c r="B809" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-con-incremento-de-capacidad-2026/web01-tramite/es/</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/c427200b-e175-4101-b8d4-4ec219539e45-PIN</t>
         </is>
       </c>
       <c r="C809" s="20" t="n"/>
@@ -16668,7 +16832,7 @@
     <row r="811" ht="30" customHeight="1">
       <c r="A811" s="16" t="inlineStr">
         <is>
-          <t>FICHA 55: EUS-38721</t>
+          <t>FICHA 55: EUS-64028</t>
         </is>
       </c>
       <c r="B811" s="17" t="n"/>
@@ -16693,7 +16857,7 @@
       <c r="E812" s="20" t="n"/>
       <c r="F812" s="20" t="n"/>
     </row>
-    <row r="813" ht="20" customHeight="1">
+    <row r="813" ht="45" customHeight="1">
       <c r="A813" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -16701,7 +16865,7 @@
       </c>
       <c r="B813" s="19" t="inlineStr">
         <is>
-          <t>Ayudas a la gestión sostenible de los recursos pesqueros 2026</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
         </is>
       </c>
       <c r="C813" s="20" t="n"/>
@@ -16717,7 +16881,7 @@
       </c>
       <c r="B814" s="19" t="inlineStr">
         <is>
-          <t>EUS-38721</t>
+          <t>EUS-64028</t>
         </is>
       </c>
       <c r="C814" s="20" t="n"/>
@@ -16869,7 +17033,7 @@
       </c>
       <c r="B824" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-gestion-sostenible-de-los-recursos-pesqueros-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-con-incremento-de-capacidad-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C824" s="20" t="n"/>
@@ -16880,7 +17044,7 @@
     <row r="826" ht="30" customHeight="1">
       <c r="A826" s="16" t="inlineStr">
         <is>
-          <t>FICHA 56: EUS-40875</t>
+          <t>FICHA 56: EUS-77748</t>
         </is>
       </c>
       <c r="B826" s="17" t="n"/>
@@ -16905,7 +17069,7 @@
       <c r="E827" s="20" t="n"/>
       <c r="F827" s="20" t="n"/>
     </row>
-    <row r="828" ht="45" customHeight="1">
+    <row r="828" ht="20" customHeight="1">
       <c r="A828" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -16913,7 +17077,7 @@
       </c>
       <c r="B828" s="19" t="inlineStr">
         <is>
-          <t>Ayudas a la recogida de residuos con la participación de los pescadores en el mar y las playas 2026</t>
+          <t>Ayudas a la gestión sostenible de los recursos pesqueros 2026</t>
         </is>
       </c>
       <c r="C828" s="20" t="n"/>
@@ -16929,7 +17093,7 @@
       </c>
       <c r="B829" s="19" t="inlineStr">
         <is>
-          <t>EUS-40875</t>
+          <t>EUS-77748</t>
         </is>
       </c>
       <c r="C829" s="20" t="n"/>
@@ -17073,7 +17237,7 @@
       <c r="E838" s="20" t="n"/>
       <c r="F838" s="20" t="n"/>
     </row>
-    <row r="839" ht="20" customHeight="1">
+    <row r="839" ht="45" customHeight="1">
       <c r="A839" s="18" t="inlineStr">
         <is>
           <t>Enlace al portal</t>
@@ -17081,7 +17245,7 @@
       </c>
       <c r="B839" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/fempa-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-gestion-sostenible-de-los-recursos-pesqueros-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C839" s="20" t="n"/>
@@ -17092,7 +17256,7 @@
     <row r="841" ht="30" customHeight="1">
       <c r="A841" s="16" t="inlineStr">
         <is>
-          <t>FICHA 57: EUS-46334</t>
+          <t>FICHA 57: EUS-23804</t>
         </is>
       </c>
       <c r="B841" s="17" t="n"/>
@@ -17125,7 +17289,7 @@
       </c>
       <c r="B843" s="19" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático sin incremento de capacidad 2026</t>
+          <t>Ayudas a la recogida de residuos con la participación de los pescadores en el mar y las playas 2026</t>
         </is>
       </c>
       <c r="C843" s="20" t="n"/>
@@ -17141,7 +17305,7 @@
       </c>
       <c r="B844" s="19" t="inlineStr">
         <is>
-          <t>EUS-46334</t>
+          <t>EUS-23804</t>
         </is>
       </c>
       <c r="C844" s="20" t="n"/>
@@ -17285,7 +17449,7 @@
       <c r="E853" s="20" t="n"/>
       <c r="F853" s="20" t="n"/>
     </row>
-    <row r="854" ht="45" customHeight="1">
+    <row r="854" ht="20" customHeight="1">
       <c r="A854" s="18" t="inlineStr">
         <is>
           <t>Enlace al portal</t>
@@ -17293,7 +17457,7 @@
       </c>
       <c r="B854" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-sin-incremento-de-capacidad-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/fempa-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C854" s="20" t="n"/>
@@ -17304,7 +17468,7 @@
     <row r="856" ht="30" customHeight="1">
       <c r="A856" s="16" t="inlineStr">
         <is>
-          <t>FICHA 58: EUS-62067</t>
+          <t>FICHA 58: EUS-89133</t>
         </is>
       </c>
       <c r="B856" s="17" t="n"/>
@@ -17337,7 +17501,7 @@
       </c>
       <c r="B858" s="19" t="inlineStr">
         <is>
-          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio climático sin incremento de capacidad 2026</t>
         </is>
       </c>
       <c r="C858" s="20" t="n"/>
@@ -17353,7 +17517,7 @@
       </c>
       <c r="B859" s="19" t="inlineStr">
         <is>
-          <t>EUS-62067</t>
+          <t>EUS-89133</t>
         </is>
       </c>
       <c r="C859" s="20" t="n"/>
@@ -17487,9 +17651,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B868" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
+      <c r="B868" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALTA — </t>
         </is>
       </c>
       <c r="C868" s="20" t="n"/>
@@ -17505,7 +17669,7 @@
       </c>
       <c r="B869" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-contribucion-de-la-acuicultura-al-buen-estado-ambiental-y-prestacion-de-servicios-ambientales-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-sin-incremento-de-capacidad-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C869" s="20" t="n"/>
@@ -17516,7 +17680,7 @@
     <row r="871" ht="30" customHeight="1">
       <c r="A871" s="16" t="inlineStr">
         <is>
-          <t>FICHA 59: EUS-84073</t>
+          <t>FICHA 59: EUS-48991</t>
         </is>
       </c>
       <c r="B871" s="17" t="n"/>
@@ -17541,7 +17705,7 @@
       <c r="E872" s="20" t="n"/>
       <c r="F872" s="20" t="n"/>
     </row>
-    <row r="873" ht="20" customHeight="1">
+    <row r="873" ht="45" customHeight="1">
       <c r="A873" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -17549,7 +17713,7 @@
       </c>
       <c r="B873" s="19" t="inlineStr">
         <is>
-          <t>Ayudas al valor añadido, economía circular y seguridad alimentaria 2026</t>
+          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
         </is>
       </c>
       <c r="C873" s="20" t="n"/>
@@ -17565,7 +17729,7 @@
       </c>
       <c r="B874" s="19" t="inlineStr">
         <is>
-          <t>EUS-84073</t>
+          <t>EUS-48991</t>
         </is>
       </c>
       <c r="C874" s="20" t="n"/>
@@ -17717,7 +17881,7 @@
       </c>
       <c r="B884" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-valor-anadido-economia-circular-y-seguridad-alimentaria-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-contribucion-de-la-acuicultura-al-buen-estado-ambiental-y-prestacion-de-servicios-ambientales-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C884" s="20" t="n"/>
@@ -17728,7 +17892,7 @@
     <row r="886" ht="30" customHeight="1">
       <c r="A886" s="16" t="inlineStr">
         <is>
-          <t>FICHA 60: EUS-89931</t>
+          <t>FICHA 60: EUS-06375</t>
         </is>
       </c>
       <c r="B886" s="17" t="n"/>
@@ -17753,7 +17917,7 @@
       <c r="E887" s="20" t="n"/>
       <c r="F887" s="20" t="n"/>
     </row>
-    <row r="888" ht="45" customHeight="1">
+    <row r="888" ht="20" customHeight="1">
       <c r="A888" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -17761,7 +17925,7 @@
       </c>
       <c r="B888" s="19" t="inlineStr">
         <is>
-          <t>Vino: el Gobierno Vasco volverá a convocar este mes las ayudas al arranque o cosecha en verde del viñedo, que van a contemplar como estructurales tras reformar la UE jurídicamente su Intervención Sect</t>
+          <t>Ayudas al valor añadido, economía circular y seguridad alimentaria 2026</t>
         </is>
       </c>
       <c r="C888" s="20" t="n"/>
@@ -17777,7 +17941,7 @@
       </c>
       <c r="B889" s="19" t="inlineStr">
         <is>
-          <t>EUS-89931</t>
+          <t>EUS-06375</t>
         </is>
       </c>
       <c r="C889" s="20" t="n"/>
@@ -17929,7 +18093,7 @@
       </c>
       <c r="B899" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260302berdezerauztekoak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-valor-anadido-economia-circular-y-seguridad-alimentaria-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C899" s="20" t="n"/>
@@ -17940,7 +18104,7 @@
     <row r="901" ht="30" customHeight="1">
       <c r="A901" s="16" t="inlineStr">
         <is>
-          <t>FICHA 61: EUS-60483</t>
+          <t>FICHA 61: EUS-79267</t>
         </is>
       </c>
       <c r="B901" s="17" t="n"/>
@@ -17973,7 +18137,7 @@
       </c>
       <c r="B903" s="19" t="inlineStr">
         <is>
-          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de aceleración de proyectos, a localidades de menos de 20.000 habitantes son objeto de convocatoria abierta hasta el 17.03.26. Transformacione</t>
+          <t>Vino: el Gobierno Vasco volverá a convocar este mes las ayudas al arranque o cosecha en verde del viñedo, que van a contemplar como estructurales tras reformar la UE jurídicamente su Intervención Sect</t>
         </is>
       </c>
       <c r="C903" s="20" t="n"/>
@@ -17989,7 +18153,7 @@
       </c>
       <c r="B904" s="19" t="inlineStr">
         <is>
-          <t>EUS-60483</t>
+          <t>EUS-79267</t>
         </is>
       </c>
       <c r="C904" s="20" t="n"/>
@@ -18141,7 +18305,7 @@
       </c>
       <c r="B914" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260317neboostasariak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260302berdezerauztekoak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C914" s="20" t="n"/>
@@ -18152,7 +18316,7 @@
     <row r="916" ht="30" customHeight="1">
       <c r="A916" s="16" t="inlineStr">
         <is>
-          <t>FICHA 62: EUS-46455</t>
+          <t>FICHA 62: EUS-85579</t>
         </is>
       </c>
       <c r="B916" s="17" t="n"/>
@@ -18185,7 +18349,7 @@
       </c>
       <c r="B918" s="19" t="inlineStr">
         <is>
-          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para consorcios internacionales de I+D+i. Jornada del Gobierno Vasco y con Enterprise Europe Network y otros socios. Digitalización, dispositivos,</t>
+          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de aceleración de proyectos, a localidades de menos de 20.000 habitantes son objeto de convocatoria abierta hasta el 17.03.26. Transformacione</t>
         </is>
       </c>
       <c r="C918" s="20" t="n"/>
@@ -18201,7 +18365,7 @@
       </c>
       <c r="B919" s="19" t="inlineStr">
         <is>
-          <t>EUS-46455</t>
+          <t>EUS-85579</t>
         </is>
       </c>
       <c r="C919" s="20" t="n"/>
@@ -18353,7 +18517,7 @@
       </c>
       <c r="B929" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260303eicihihorizon/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260317neboostasariak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C929" s="20" t="n"/>
@@ -18364,7 +18528,7 @@
     <row r="931" ht="30" customHeight="1">
       <c r="A931" s="16" t="inlineStr">
         <is>
-          <t>FICHA 63: EUS-38314</t>
+          <t>FICHA 63: EUS-03347</t>
         </is>
       </c>
       <c r="B931" s="17" t="n"/>
@@ -18397,7 +18561,7 @@
       </c>
       <c r="B933" s="19" t="inlineStr">
         <is>
-          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinancia convocatorias de ayudas de las Diputaciones a explotaciones con limitaciones o desfavorecidas, y a compromisos medioambientales, climátic</t>
+          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para consorcios internacionales de I+D+i. Jornada del Gobierno Vasco y con Enterprise Europe Network y otros socios. Digitalización, dispositivos,</t>
         </is>
       </c>
       <c r="C933" s="20" t="n"/>
@@ -18413,7 +18577,7 @@
       </c>
       <c r="B934" s="19" t="inlineStr">
         <is>
-          <t>EUS-38314</t>
+          <t>EUS-03347</t>
         </is>
       </c>
       <c r="C934" s="20" t="n"/>
@@ -18565,7 +18729,7 @@
       </c>
       <c r="B944" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/lgenfnpbgfa260218/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260303eicihihorizon/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C944" s="20" t="n"/>
@@ -18576,7 +18740,7 @@
     <row r="946" ht="30" customHeight="1">
       <c r="A946" s="16" t="inlineStr">
         <is>
-          <t>FICHA 64: EUS-56475</t>
+          <t>FICHA 64: EUS-87925</t>
         </is>
       </c>
       <c r="B946" s="17" t="n"/>
@@ -18609,7 +18773,7 @@
       </c>
       <c r="B948" s="19" t="inlineStr">
         <is>
-          <t>Digital Europe, Horizon (programas de la UE). Apoyos para consorcios interestatales de I+D+i. IA, robótica, cuántica, computación, ciberseguridad, electrónica, fotónica, TICs e internet avanzadas, esp</t>
+          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinancia convocatorias de ayudas de las Diputaciones a explotaciones con limitaciones o desfavorecidas, y a compromisos medioambientales, climátic</t>
         </is>
       </c>
       <c r="C948" s="20" t="n"/>
@@ -18625,7 +18789,7 @@
       </c>
       <c r="B949" s="19" t="inlineStr">
         <is>
-          <t>EUS-56475</t>
+          <t>EUS-87925</t>
         </is>
       </c>
       <c r="C949" s="20" t="n"/>
@@ -18777,7 +18941,7 @@
       </c>
       <c r="B959" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260304digitalhorizoneen/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/lgenfnpbgfa260218/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C959" s="20" t="n"/>
@@ -18788,7 +18952,7 @@
     <row r="961" ht="30" customHeight="1">
       <c r="A961" s="16" t="inlineStr">
         <is>
-          <t>FICHA 65: EUS-05137</t>
+          <t>FICHA 65: EUS-21599</t>
         </is>
       </c>
       <c r="B961" s="17" t="n"/>
@@ -18821,7 +18985,7 @@
       </c>
       <c r="B963" s="19" t="inlineStr">
         <is>
-          <t>Política Agraria Común de la UE de 2026, y sus ayudas abiertas hasta el 30.4.26: el pilar 1, con el Fondo Europeo Agrícola de Garantía Agraria FEAGA, aborda sostenibilidad de renta, ayuda redistributi</t>
+          <t>Digital Europe, Horizon (programas de la UE). Apoyos para consorcios interestatales de I+D+i. IA, robótica, cuántica, computación, ciberseguridad, electrónica, fotónica, TICs e internet avanzadas, esp</t>
         </is>
       </c>
       <c r="C963" s="20" t="n"/>
@@ -18837,7 +19001,7 @@
       </c>
       <c r="B964" s="19" t="inlineStr">
         <is>
-          <t>EUS-05137</t>
+          <t>EUS-21599</t>
         </is>
       </c>
       <c r="C964" s="20" t="n"/>
@@ -18989,7 +19153,7 @@
       </c>
       <c r="B974" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260216npblaguntzairekiak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260304digitalhorizoneen/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C974" s="20" t="n"/>
@@ -19000,7 +19164,7 @@
     <row r="976" ht="30" customHeight="1">
       <c r="A976" s="16" t="inlineStr">
         <is>
-          <t>FICHA 66: EUS-12265</t>
+          <t>FICHA 66: EUS-91637</t>
         </is>
       </c>
       <c r="B976" s="17" t="n"/>
@@ -19033,7 +19197,7 @@
       </c>
       <c r="B978" s="19" t="inlineStr">
         <is>
-          <t>Programa de impulso a las ciudades y territorios inteligentes para el fomento del desarrollo económico y productivo, que podrá ser cofinanciado por el Programa Plurirregional 2021-2027 del Fondo Europ</t>
+          <t>Política Agraria Común de la UE de 2026, y sus ayudas abiertas hasta el 30.4.26: el pilar 1, con el Fondo Europeo Agrícola de Garantía Agraria FEAGA, aborda sostenibilidad de renta, ayuda redistributi</t>
         </is>
       </c>
       <c r="C978" s="20" t="n"/>
@@ -19049,7 +19213,7 @@
       </c>
       <c r="B979" s="19" t="inlineStr">
         <is>
-          <t>EUS-12265</t>
+          <t>EUS-91637</t>
         </is>
       </c>
       <c r="C979" s="20" t="n"/>
@@ -19201,7 +19365,7 @@
       </c>
       <c r="B989" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260204smartcities/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260216npblaguntzairekiak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C989" s="20" t="n"/>
@@ -19212,7 +19376,7 @@
     <row r="991" ht="30" customHeight="1">
       <c r="A991" s="16" t="inlineStr">
         <is>
-          <t>FICHA 67: EUS-58053</t>
+          <t>FICHA 67: EUS-38365</t>
         </is>
       </c>
       <c r="B991" s="17" t="n"/>
@@ -19245,7 +19409,7 @@
       </c>
       <c r="B993" s="19" t="inlineStr">
         <is>
-          <t>Suministro, Implementación y Soporte de un Servicio Digital de Telefonía y Videollamadas para los Centros Penitenciarios de Euskadi.</t>
+          <t>Programa de impulso a las ciudades y territorios inteligentes para el fomento del desarrollo económico y productivo, que podrá ser cofinanciado por el Programa Plurirregional 2021-2027 del Fondo Europ</t>
         </is>
       </c>
       <c r="C993" s="20" t="n"/>
@@ -19261,7 +19425,7 @@
       </c>
       <c r="B994" s="19" t="inlineStr">
         <is>
-          <t>EUS-58053</t>
+          <t>EUS-38365</t>
         </is>
       </c>
       <c r="C994" s="20" t="n"/>
@@ -19337,7 +19501,7 @@
       </c>
       <c r="B999" s="19" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C999" s="20" t="n"/>
@@ -19381,7 +19545,7 @@
       </c>
       <c r="B1002" s="19" t="inlineStr">
         <is>
-          <t>alumbrado</t>
+          <t>energia</t>
         </is>
       </c>
       <c r="C1002" s="20" t="n"/>
@@ -19413,7 +19577,7 @@
       </c>
       <c r="B1004" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-implementacion-y-soporte-servicio-digital-telefonia-y-videollamadas-centros-penitenciarios-euskadi/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260204smartcities/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1004" s="20" t="n"/>
@@ -19424,7 +19588,7 @@
     <row r="1006" ht="30" customHeight="1">
       <c r="A1006" s="16" t="inlineStr">
         <is>
-          <t>FICHA 68: EUS-97072</t>
+          <t>FICHA 68: EUS-84600</t>
         </is>
       </c>
       <c r="B1006" s="17" t="n"/>
@@ -19449,7 +19613,7 @@
       <c r="E1007" s="20" t="n"/>
       <c r="F1007" s="20" t="n"/>
     </row>
-    <row r="1008" ht="45" customHeight="1">
+    <row r="1008" ht="20" customHeight="1">
       <c r="A1008" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -19457,7 +19621,7 @@
       </c>
       <c r="B1008" s="19" t="inlineStr">
         <is>
-          <t>Suministro de driver 75w y lamparas de 360w para farolas (alumbrado publico).(pre:2049409)</t>
+          <t>Servicio de Punto Verde Móvil en el Territorio Histórico de Álava</t>
         </is>
       </c>
       <c r="C1008" s="20" t="n"/>
@@ -19473,7 +19637,7 @@
       </c>
       <c r="B1009" s="19" t="inlineStr">
         <is>
-          <t>EUS-97072</t>
+          <t>EUS-84600</t>
         </is>
       </c>
       <c r="C1009" s="20" t="n"/>
@@ -19593,7 +19757,7 @@
       </c>
       <c r="B1017" s="19" t="inlineStr">
         <is>
-          <t>alumbrado</t>
+          <t>energia</t>
         </is>
       </c>
       <c r="C1017" s="20" t="n"/>
@@ -19625,7 +19789,7 @@
       </c>
       <c r="B1019" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-driver-75w-y-lamparas-360w-farolas-alumbrado-publico-pre-2049409/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-punto-verde-movil-territorio-historico-alava/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1019" s="20" t="n"/>
@@ -19636,7 +19800,7 @@
     <row r="1021" ht="30" customHeight="1">
       <c r="A1021" s="16" t="inlineStr">
         <is>
-          <t>FICHA 69: EUS-77422</t>
+          <t>FICHA 69: EUS-18669</t>
         </is>
       </c>
       <c r="B1021" s="17" t="n"/>
@@ -19669,7 +19833,7 @@
       </c>
       <c r="B1023" s="19" t="inlineStr">
         <is>
-          <t>Suministro de material eléctrico (driver 150w) para alumbrado publico. maquinaria, instalaciones y utillaje. mantenimiento.</t>
+          <t>Servicio de agencia de viajes para el Departamento de Hacienda y Finanzas con cláusulas ambientales.</t>
         </is>
       </c>
       <c r="C1023" s="20" t="n"/>
@@ -19685,7 +19849,7 @@
       </c>
       <c r="B1024" s="19" t="inlineStr">
         <is>
-          <t>EUS-77422</t>
+          <t>EUS-18669</t>
         </is>
       </c>
       <c r="C1024" s="20" t="n"/>
@@ -19805,7 +19969,7 @@
       </c>
       <c r="B1032" s="19" t="inlineStr">
         <is>
-          <t>alumbrado</t>
+          <t>energia</t>
         </is>
       </c>
       <c r="C1032" s="20" t="n"/>
@@ -19837,7 +20001,7 @@
       </c>
       <c r="B1034" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-material-electrico-driver-150w-alumbrado-publico-maquinaria-instalaciones-y-utillaje-mantenimiento/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-agencia-viajes-departamento-hacienda-y-finanzas-clausulas-ambientales/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1034" s="20" t="n"/>
@@ -19848,7 +20012,7 @@
     <row r="1036" ht="30" customHeight="1">
       <c r="A1036" s="16" t="inlineStr">
         <is>
-          <t>FICHA 70: EUS-95174</t>
+          <t>FICHA 70: EUS-29543</t>
         </is>
       </c>
       <c r="B1036" s="17" t="n"/>
@@ -19873,7 +20037,7 @@
       <c r="E1037" s="20" t="n"/>
       <c r="F1037" s="20" t="n"/>
     </row>
-    <row r="1038" ht="45" customHeight="1">
+    <row r="1038" ht="20" customHeight="1">
       <c r="A1038" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -19881,7 +20045,7 @@
       </c>
       <c r="B1038" s="19" t="inlineStr">
         <is>
-          <t>Reparacion de la bomba del circuito de recirculacion del agua del polideportivo de orbea</t>
+          <t>Conferencia sobre "la bicicleta, un máquina móvil, veloz y bella"</t>
         </is>
       </c>
       <c r="C1038" s="20" t="n"/>
@@ -19897,7 +20061,7 @@
       </c>
       <c r="B1039" s="19" t="inlineStr">
         <is>
-          <t>EUS-95174</t>
+          <t>EUS-29543</t>
         </is>
       </c>
       <c r="C1039" s="20" t="n"/>
@@ -20017,7 +20181,7 @@
       </c>
       <c r="B1047" s="19" t="inlineStr">
         <is>
-          <t>alumbrado</t>
+          <t>energia</t>
         </is>
       </c>
       <c r="C1047" s="20" t="n"/>
@@ -20049,7 +20213,7 @@
       </c>
       <c r="B1049" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/reparacion-bomba-del-circuito-recirculacion-del-agua-del-polideportivo-orbea/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/conferencia-bicicleta-maquina-movil-veloz-y-bella/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1049" s="20" t="n"/>
@@ -20060,7 +20224,7 @@
     <row r="1051" ht="30" customHeight="1">
       <c r="A1051" s="16" t="inlineStr">
         <is>
-          <t>FICHA 71: EUS-49048</t>
+          <t>FICHA 71: EUS-17370</t>
         </is>
       </c>
       <c r="B1051" s="17" t="n"/>
@@ -20093,7 +20257,7 @@
       </c>
       <c r="B1053" s="19" t="inlineStr">
         <is>
-          <t>Limpieza de foso ascensor errebal</t>
+          <t>Organización parque infantil de Navidad</t>
         </is>
       </c>
       <c r="C1053" s="20" t="n"/>
@@ -20109,7 +20273,7 @@
       </c>
       <c r="B1054" s="19" t="inlineStr">
         <is>
-          <t>EUS-49048</t>
+          <t>EUS-17370</t>
         </is>
       </c>
       <c r="C1054" s="20" t="n"/>
@@ -20229,7 +20393,7 @@
       </c>
       <c r="B1062" s="19" t="inlineStr">
         <is>
-          <t>alumbrado</t>
+          <t>energia</t>
         </is>
       </c>
       <c r="C1062" s="20" t="n"/>
@@ -20261,7 +20425,7 @@
       </c>
       <c r="B1064" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/limpieza-foso-ascensor-errebal/expgeeibar20830/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/organizacion-parque-infantil-navidad/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1064" s="20" t="n"/>
@@ -20272,7 +20436,7 @@
     <row r="1066" ht="30" customHeight="1">
       <c r="A1066" s="16" t="inlineStr">
         <is>
-          <t>FICHA 72: EUS-90362</t>
+          <t>FICHA 72: EUS-46342</t>
         </is>
       </c>
       <c r="B1066" s="17" t="n"/>
@@ -20305,7 +20469,7 @@
       </c>
       <c r="B1068" s="19" t="inlineStr">
         <is>
-          <t>Digitalización de la imagen del cartel de las jornadas de teatro</t>
+          <t>Alumbrado publico pasos peatonales en La Calzada</t>
         </is>
       </c>
       <c r="C1068" s="20" t="n"/>
@@ -20321,7 +20485,7 @@
       </c>
       <c r="B1069" s="19" t="inlineStr">
         <is>
-          <t>EUS-90362</t>
+          <t>EUS-46342</t>
         </is>
       </c>
       <c r="C1069" s="20" t="n"/>
@@ -20441,7 +20605,7 @@
       </c>
       <c r="B1077" s="19" t="inlineStr">
         <is>
-          <t>alumbrado</t>
+          <t>energia</t>
         </is>
       </c>
       <c r="C1077" s="20" t="n"/>
@@ -20473,7 +20637,7 @@
       </c>
       <c r="B1079" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/digitalizacion-imagen-del-cartel-jornadas-teatro/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/alumbrado-publico-pasos-peatonales-calzada/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1079" s="20" t="n"/>
@@ -20484,7 +20648,7 @@
     <row r="1081" ht="30" customHeight="1">
       <c r="A1081" s="16" t="inlineStr">
         <is>
-          <t>FICHA 73: EUS-98149</t>
+          <t>FICHA 73: EUS-02378</t>
         </is>
       </c>
       <c r="B1081" s="17" t="n"/>
@@ -20509,7 +20673,7 @@
       <c r="E1082" s="20" t="n"/>
       <c r="F1082" s="20" t="n"/>
     </row>
-    <row r="1083" ht="45" customHeight="1">
+    <row r="1083" ht="20" customHeight="1">
       <c r="A1083" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -20517,7 +20681,7 @@
       </c>
       <c r="B1083" s="19" t="inlineStr">
         <is>
-          <t>Servicio técnico para realizar la sustitución del servidor integrado en el proyector de cine digital del coliseo</t>
+          <t>Reparación faldón cubierta Museo Santa Clara</t>
         </is>
       </c>
       <c r="C1083" s="20" t="n"/>
@@ -20533,7 +20697,7 @@
       </c>
       <c r="B1084" s="19" t="inlineStr">
         <is>
-          <t>EUS-98149</t>
+          <t>EUS-02378</t>
         </is>
       </c>
       <c r="C1084" s="20" t="n"/>
@@ -20653,7 +20817,7 @@
       </c>
       <c r="B1092" s="19" t="inlineStr">
         <is>
-          <t>alumbrado</t>
+          <t>energia</t>
         </is>
       </c>
       <c r="C1092" s="20" t="n"/>
@@ -20685,7 +20849,7 @@
       </c>
       <c r="B1094" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-tecnico-realizar-sustitucion-del-servidor-integrado-proyector-cine-digital-del-coliseo/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/reparacion-faldon-cubierta-museo-santa-clara/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1094" s="20" t="n"/>
@@ -20693,8 +20857,644 @@
       <c r="E1094" s="20" t="n"/>
       <c r="F1094" s="20" t="n"/>
     </row>
+    <row r="1096" ht="30" customHeight="1">
+      <c r="A1096" s="16" t="inlineStr">
+        <is>
+          <t>FICHA 74: EUS-69611</t>
+        </is>
+      </c>
+      <c r="B1096" s="17" t="n"/>
+      <c r="C1096" s="17" t="n"/>
+      <c r="D1096" s="17" t="n"/>
+      <c r="E1096" s="17" t="n"/>
+      <c r="F1096" s="17" t="n"/>
+    </row>
+    <row r="1097" ht="20" customHeight="1">
+      <c r="A1097" s="18" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1097" s="19" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1097" s="20" t="n"/>
+      <c r="D1097" s="20" t="n"/>
+      <c r="E1097" s="20" t="n"/>
+      <c r="F1097" s="20" t="n"/>
+    </row>
+    <row r="1098" ht="20" customHeight="1">
+      <c r="A1098" s="18" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1098" s="19" t="inlineStr">
+        <is>
+          <t>Limpieza y desescombro desatasco colector de saneamiento</t>
+        </is>
+      </c>
+      <c r="C1098" s="20" t="n"/>
+      <c r="D1098" s="20" t="n"/>
+      <c r="E1098" s="20" t="n"/>
+      <c r="F1098" s="20" t="n"/>
+    </row>
+    <row r="1099" ht="20" customHeight="1">
+      <c r="A1099" s="18" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1099" s="19" t="inlineStr">
+        <is>
+          <t>EUS-69611</t>
+        </is>
+      </c>
+      <c r="C1099" s="20" t="n"/>
+      <c r="D1099" s="20" t="n"/>
+      <c r="E1099" s="20" t="n"/>
+      <c r="F1099" s="20" t="n"/>
+    </row>
+    <row r="1100" ht="20" customHeight="1">
+      <c r="A1100" s="18" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1100" s="19" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1100" s="20" t="n"/>
+      <c r="D1100" s="20" t="n"/>
+      <c r="E1100" s="20" t="n"/>
+      <c r="F1100" s="20" t="n"/>
+    </row>
+    <row r="1101" ht="20" customHeight="1">
+      <c r="A1101" s="18" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1101" s="19" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1101" s="20" t="n"/>
+      <c r="D1101" s="20" t="n"/>
+      <c r="E1101" s="20" t="n"/>
+      <c r="F1101" s="20" t="n"/>
+    </row>
+    <row r="1102" ht="20" customHeight="1">
+      <c r="A1102" s="18" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1102" s="19" t="inlineStr"/>
+      <c r="C1102" s="20" t="n"/>
+      <c r="D1102" s="20" t="n"/>
+      <c r="E1102" s="20" t="n"/>
+      <c r="F1102" s="20" t="n"/>
+    </row>
+    <row r="1103" ht="20" customHeight="1">
+      <c r="A1103" s="18" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1103" s="19" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1103" s="20" t="n"/>
+      <c r="D1103" s="20" t="n"/>
+      <c r="E1103" s="20" t="n"/>
+      <c r="F1103" s="20" t="n"/>
+    </row>
+    <row r="1104" ht="20" customHeight="1">
+      <c r="A1104" s="18" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1104" s="19" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1104" s="20" t="n"/>
+      <c r="D1104" s="20" t="n"/>
+      <c r="E1104" s="20" t="n"/>
+      <c r="F1104" s="20" t="n"/>
+    </row>
+    <row r="1105" ht="20" customHeight="1">
+      <c r="A1105" s="18" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1105" s="19" t="inlineStr"/>
+      <c r="C1105" s="20" t="n"/>
+      <c r="D1105" s="20" t="n"/>
+      <c r="E1105" s="20" t="n"/>
+      <c r="F1105" s="20" t="n"/>
+    </row>
+    <row r="1106" ht="20" customHeight="1">
+      <c r="A1106" s="18" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1106" s="19" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1106" s="20" t="n"/>
+      <c r="D1106" s="20" t="n"/>
+      <c r="E1106" s="20" t="n"/>
+      <c r="F1106" s="20" t="n"/>
+    </row>
+    <row r="1107" ht="20" customHeight="1">
+      <c r="A1107" s="18" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1107" s="19" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1107" s="20" t="n"/>
+      <c r="D1107" s="20" t="n"/>
+      <c r="E1107" s="20" t="n"/>
+      <c r="F1107" s="20" t="n"/>
+    </row>
+    <row r="1108" ht="20" customHeight="1">
+      <c r="A1108" s="18" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1108" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1108" s="20" t="n"/>
+      <c r="D1108" s="20" t="n"/>
+      <c r="E1108" s="20" t="n"/>
+      <c r="F1108" s="20" t="n"/>
+    </row>
+    <row r="1109" ht="45" customHeight="1">
+      <c r="A1109" s="18" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1109" s="22" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/limpieza-y-desescombro-desatasco-colector-saneamiento/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1109" s="20" t="n"/>
+      <c r="D1109" s="20" t="n"/>
+      <c r="E1109" s="20" t="n"/>
+      <c r="F1109" s="20" t="n"/>
+    </row>
+    <row r="1111" ht="30" customHeight="1">
+      <c r="A1111" s="16" t="inlineStr">
+        <is>
+          <t>FICHA 75: EUS-00349</t>
+        </is>
+      </c>
+      <c r="B1111" s="17" t="n"/>
+      <c r="C1111" s="17" t="n"/>
+      <c r="D1111" s="17" t="n"/>
+      <c r="E1111" s="17" t="n"/>
+      <c r="F1111" s="17" t="n"/>
+    </row>
+    <row r="1112" ht="20" customHeight="1">
+      <c r="A1112" s="18" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1112" s="19" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1112" s="20" t="n"/>
+      <c r="D1112" s="20" t="n"/>
+      <c r="E1112" s="20" t="n"/>
+      <c r="F1112" s="20" t="n"/>
+    </row>
+    <row r="1113" ht="20" customHeight="1">
+      <c r="A1113" s="18" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1113" s="19" t="inlineStr">
+        <is>
+          <t>Reparación instalación fotovoltaica refugio del Kolitza</t>
+        </is>
+      </c>
+      <c r="C1113" s="20" t="n"/>
+      <c r="D1113" s="20" t="n"/>
+      <c r="E1113" s="20" t="n"/>
+      <c r="F1113" s="20" t="n"/>
+    </row>
+    <row r="1114" ht="20" customHeight="1">
+      <c r="A1114" s="18" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1114" s="19" t="inlineStr">
+        <is>
+          <t>EUS-00349</t>
+        </is>
+      </c>
+      <c r="C1114" s="20" t="n"/>
+      <c r="D1114" s="20" t="n"/>
+      <c r="E1114" s="20" t="n"/>
+      <c r="F1114" s="20" t="n"/>
+    </row>
+    <row r="1115" ht="20" customHeight="1">
+      <c r="A1115" s="18" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1115" s="19" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1115" s="20" t="n"/>
+      <c r="D1115" s="20" t="n"/>
+      <c r="E1115" s="20" t="n"/>
+      <c r="F1115" s="20" t="n"/>
+    </row>
+    <row r="1116" ht="20" customHeight="1">
+      <c r="A1116" s="18" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1116" s="19" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1116" s="20" t="n"/>
+      <c r="D1116" s="20" t="n"/>
+      <c r="E1116" s="20" t="n"/>
+      <c r="F1116" s="20" t="n"/>
+    </row>
+    <row r="1117" ht="20" customHeight="1">
+      <c r="A1117" s="18" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1117" s="19" t="inlineStr"/>
+      <c r="C1117" s="20" t="n"/>
+      <c r="D1117" s="20" t="n"/>
+      <c r="E1117" s="20" t="n"/>
+      <c r="F1117" s="20" t="n"/>
+    </row>
+    <row r="1118" ht="20" customHeight="1">
+      <c r="A1118" s="18" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1118" s="19" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1118" s="20" t="n"/>
+      <c r="D1118" s="20" t="n"/>
+      <c r="E1118" s="20" t="n"/>
+      <c r="F1118" s="20" t="n"/>
+    </row>
+    <row r="1119" ht="20" customHeight="1">
+      <c r="A1119" s="18" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1119" s="19" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1119" s="20" t="n"/>
+      <c r="D1119" s="20" t="n"/>
+      <c r="E1119" s="20" t="n"/>
+      <c r="F1119" s="20" t="n"/>
+    </row>
+    <row r="1120" ht="20" customHeight="1">
+      <c r="A1120" s="18" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1120" s="19" t="inlineStr"/>
+      <c r="C1120" s="20" t="n"/>
+      <c r="D1120" s="20" t="n"/>
+      <c r="E1120" s="20" t="n"/>
+      <c r="F1120" s="20" t="n"/>
+    </row>
+    <row r="1121" ht="20" customHeight="1">
+      <c r="A1121" s="18" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1121" s="19" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1121" s="20" t="n"/>
+      <c r="D1121" s="20" t="n"/>
+      <c r="E1121" s="20" t="n"/>
+      <c r="F1121" s="20" t="n"/>
+    </row>
+    <row r="1122" ht="20" customHeight="1">
+      <c r="A1122" s="18" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1122" s="19" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1122" s="20" t="n"/>
+      <c r="D1122" s="20" t="n"/>
+      <c r="E1122" s="20" t="n"/>
+      <c r="F1122" s="20" t="n"/>
+    </row>
+    <row r="1123" ht="20" customHeight="1">
+      <c r="A1123" s="18" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1123" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1123" s="20" t="n"/>
+      <c r="D1123" s="20" t="n"/>
+      <c r="E1123" s="20" t="n"/>
+      <c r="F1123" s="20" t="n"/>
+    </row>
+    <row r="1124" ht="45" customHeight="1">
+      <c r="A1124" s="18" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1124" s="22" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/reparacion-instalacion-fotovoltaica-refugio-del-kolitza/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1124" s="20" t="n"/>
+      <c r="D1124" s="20" t="n"/>
+      <c r="E1124" s="20" t="n"/>
+      <c r="F1124" s="20" t="n"/>
+    </row>
+    <row r="1126" ht="30" customHeight="1">
+      <c r="A1126" s="16" t="inlineStr">
+        <is>
+          <t>FICHA 76: EUS-93515</t>
+        </is>
+      </c>
+      <c r="B1126" s="17" t="n"/>
+      <c r="C1126" s="17" t="n"/>
+      <c r="D1126" s="17" t="n"/>
+      <c r="E1126" s="17" t="n"/>
+      <c r="F1126" s="17" t="n"/>
+    </row>
+    <row r="1127" ht="20" customHeight="1">
+      <c r="A1127" s="18" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1127" s="19" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1127" s="20" t="n"/>
+      <c r="D1127" s="20" t="n"/>
+      <c r="E1127" s="20" t="n"/>
+      <c r="F1127" s="20" t="n"/>
+    </row>
+    <row r="1128" ht="20" customHeight="1">
+      <c r="A1128" s="18" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1128" s="19" t="inlineStr">
+        <is>
+          <t>Formación en jardineria forestal</t>
+        </is>
+      </c>
+      <c r="C1128" s="20" t="n"/>
+      <c r="D1128" s="20" t="n"/>
+      <c r="E1128" s="20" t="n"/>
+      <c r="F1128" s="20" t="n"/>
+    </row>
+    <row r="1129" ht="20" customHeight="1">
+      <c r="A1129" s="18" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1129" s="19" t="inlineStr">
+        <is>
+          <t>EUS-93515</t>
+        </is>
+      </c>
+      <c r="C1129" s="20" t="n"/>
+      <c r="D1129" s="20" t="n"/>
+      <c r="E1129" s="20" t="n"/>
+      <c r="F1129" s="20" t="n"/>
+    </row>
+    <row r="1130" ht="20" customHeight="1">
+      <c r="A1130" s="18" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1130" s="19" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1130" s="20" t="n"/>
+      <c r="D1130" s="20" t="n"/>
+      <c r="E1130" s="20" t="n"/>
+      <c r="F1130" s="20" t="n"/>
+    </row>
+    <row r="1131" ht="20" customHeight="1">
+      <c r="A1131" s="18" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1131" s="19" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1131" s="20" t="n"/>
+      <c r="D1131" s="20" t="n"/>
+      <c r="E1131" s="20" t="n"/>
+      <c r="F1131" s="20" t="n"/>
+    </row>
+    <row r="1132" ht="20" customHeight="1">
+      <c r="A1132" s="18" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1132" s="19" t="inlineStr"/>
+      <c r="C1132" s="20" t="n"/>
+      <c r="D1132" s="20" t="n"/>
+      <c r="E1132" s="20" t="n"/>
+      <c r="F1132" s="20" t="n"/>
+    </row>
+    <row r="1133" ht="20" customHeight="1">
+      <c r="A1133" s="18" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1133" s="19" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1133" s="20" t="n"/>
+      <c r="D1133" s="20" t="n"/>
+      <c r="E1133" s="20" t="n"/>
+      <c r="F1133" s="20" t="n"/>
+    </row>
+    <row r="1134" ht="20" customHeight="1">
+      <c r="A1134" s="18" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1134" s="19" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1134" s="20" t="n"/>
+      <c r="D1134" s="20" t="n"/>
+      <c r="E1134" s="20" t="n"/>
+      <c r="F1134" s="20" t="n"/>
+    </row>
+    <row r="1135" ht="20" customHeight="1">
+      <c r="A1135" s="18" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1135" s="19" t="inlineStr"/>
+      <c r="C1135" s="20" t="n"/>
+      <c r="D1135" s="20" t="n"/>
+      <c r="E1135" s="20" t="n"/>
+      <c r="F1135" s="20" t="n"/>
+    </row>
+    <row r="1136" ht="20" customHeight="1">
+      <c r="A1136" s="18" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1136" s="19" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1136" s="20" t="n"/>
+      <c r="D1136" s="20" t="n"/>
+      <c r="E1136" s="20" t="n"/>
+      <c r="F1136" s="20" t="n"/>
+    </row>
+    <row r="1137" ht="20" customHeight="1">
+      <c r="A1137" s="18" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1137" s="19" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1137" s="20" t="n"/>
+      <c r="D1137" s="20" t="n"/>
+      <c r="E1137" s="20" t="n"/>
+      <c r="F1137" s="20" t="n"/>
+    </row>
+    <row r="1138" ht="20" customHeight="1">
+      <c r="A1138" s="18" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1138" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1138" s="20" t="n"/>
+      <c r="D1138" s="20" t="n"/>
+      <c r="E1138" s="20" t="n"/>
+      <c r="F1138" s="20" t="n"/>
+    </row>
+    <row r="1139" ht="45" customHeight="1">
+      <c r="A1139" s="18" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1139" s="22" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/formacion-jardineria-forestal/expcm498199/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1139" s="20" t="n"/>
+      <c r="D1139" s="20" t="n"/>
+      <c r="E1139" s="20" t="n"/>
+      <c r="F1139" s="20" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="1022">
+  <mergeCells count="1064">
     <mergeCell ref="B679:F679"/>
     <mergeCell ref="B666:F666"/>
     <mergeCell ref="B964:F964"/>
@@ -20738,7 +21538,9 @@
     <mergeCell ref="B342:F342"/>
     <mergeCell ref="B578:F578"/>
     <mergeCell ref="A541:F541"/>
+    <mergeCell ref="B1099:F1099"/>
     <mergeCell ref="B515:F515"/>
+    <mergeCell ref="B1128:F1128"/>
     <mergeCell ref="A841:F841"/>
     <mergeCell ref="B158:F158"/>
     <mergeCell ref="B1094:F1094"/>
@@ -20747,6 +21549,7 @@
     <mergeCell ref="B894:F894"/>
     <mergeCell ref="B133:F133"/>
     <mergeCell ref="B959:F959"/>
+    <mergeCell ref="B1130:F1130"/>
     <mergeCell ref="B369:F369"/>
     <mergeCell ref="B667:F667"/>
     <mergeCell ref="B418:F418"/>
@@ -20773,11 +21576,13 @@
     <mergeCell ref="B662:F662"/>
     <mergeCell ref="B718:F718"/>
     <mergeCell ref="B889:F889"/>
+    <mergeCell ref="B1131:F1131"/>
     <mergeCell ref="B72:F72"/>
     <mergeCell ref="B954:F954"/>
     <mergeCell ref="B199:F199"/>
     <mergeCell ref="B370:F370"/>
     <mergeCell ref="B1025:F1025"/>
+    <mergeCell ref="B1112:F1112"/>
     <mergeCell ref="B291:F291"/>
     <mergeCell ref="B655:F655"/>
     <mergeCell ref="B974:F974"/>
@@ -20819,6 +21624,7 @@
     <mergeCell ref="B83:F83"/>
     <mergeCell ref="B254:F254"/>
     <mergeCell ref="B909:F909"/>
+    <mergeCell ref="B1105:F1105"/>
     <mergeCell ref="B319:F319"/>
     <mergeCell ref="B490:F490"/>
     <mergeCell ref="B604:F604"/>
@@ -20850,6 +21656,7 @@
     <mergeCell ref="B530:F530"/>
     <mergeCell ref="B726:F726"/>
     <mergeCell ref="B962:F962"/>
+    <mergeCell ref="B1133:F1133"/>
     <mergeCell ref="A886:F886"/>
     <mergeCell ref="B505:F505"/>
     <mergeCell ref="B1060:F1060"/>
@@ -20885,6 +21692,7 @@
     <mergeCell ref="B752:F752"/>
     <mergeCell ref="B1070:F1070"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B1115:F1115"/>
     <mergeCell ref="B325:F325"/>
     <mergeCell ref="B154:F154"/>
     <mergeCell ref="A271:F271"/>
@@ -20918,6 +21726,8 @@
     <mergeCell ref="B518:F518"/>
     <mergeCell ref="B562:F562"/>
     <mergeCell ref="B689:F689"/>
+    <mergeCell ref="B1121:F1121"/>
+    <mergeCell ref="B1123:F1123"/>
     <mergeCell ref="B86:F86"/>
     <mergeCell ref="B912:F912"/>
     <mergeCell ref="B1083:F1083"/>
@@ -20969,6 +21779,7 @@
     <mergeCell ref="B979:F979"/>
     <mergeCell ref="B381:F381"/>
     <mergeCell ref="B552:F552"/>
+    <mergeCell ref="A1111:F1111"/>
     <mergeCell ref="B1084:F1084"/>
     <mergeCell ref="A976:F976"/>
     <mergeCell ref="B170:F170"/>
@@ -21002,6 +21813,7 @@
     <mergeCell ref="B92:F92"/>
     <mergeCell ref="B984:F984"/>
     <mergeCell ref="A226:F226"/>
+    <mergeCell ref="B1124:F1124"/>
     <mergeCell ref="B394:F394"/>
     <mergeCell ref="B692:F692"/>
     <mergeCell ref="A931:F931"/>
@@ -21032,6 +21844,7 @@
     <mergeCell ref="B817:F817"/>
     <mergeCell ref="B944:F944"/>
     <mergeCell ref="B56:F56"/>
+    <mergeCell ref="B1102:F1102"/>
     <mergeCell ref="B43:F43"/>
     <mergeCell ref="B176:F176"/>
     <mergeCell ref="B347:F347"/>
@@ -21047,7 +21860,9 @@
     <mergeCell ref="B881:F881"/>
     <mergeCell ref="B1068:F1068"/>
     <mergeCell ref="B868:F868"/>
+    <mergeCell ref="B1117:F1117"/>
     <mergeCell ref="B107:F107"/>
+    <mergeCell ref="B1104:F1104"/>
     <mergeCell ref="B641:F641"/>
     <mergeCell ref="B57:F57"/>
     <mergeCell ref="B883:F883"/>
@@ -21073,6 +21888,7 @@
     <mergeCell ref="B999:F999"/>
     <mergeCell ref="B1061:F1061"/>
     <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B1097:F1097"/>
     <mergeCell ref="A46:F46"/>
     <mergeCell ref="B507:F507"/>
     <mergeCell ref="B62:F62"/>
@@ -21120,6 +21936,7 @@
     <mergeCell ref="B1018:F1018"/>
     <mergeCell ref="B624:F624"/>
     <mergeCell ref="B428:F428"/>
+    <mergeCell ref="B1118:F1118"/>
     <mergeCell ref="B284:F284"/>
     <mergeCell ref="B222:F222"/>
     <mergeCell ref="B344:F344"/>
@@ -21131,6 +21948,7 @@
     <mergeCell ref="B123:F123"/>
     <mergeCell ref="B949:F949"/>
     <mergeCell ref="B1011:F1011"/>
+    <mergeCell ref="B1120:F1120"/>
     <mergeCell ref="B50:F50"/>
     <mergeCell ref="B221:F221"/>
     <mergeCell ref="B110:F110"/>
@@ -21147,6 +21965,7 @@
     <mergeCell ref="B802:F802"/>
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B789:F789"/>
+    <mergeCell ref="B1136:F1136"/>
     <mergeCell ref="B248:F248"/>
     <mergeCell ref="B297:F297"/>
     <mergeCell ref="B813:F813"/>
@@ -21166,9 +21985,11 @@
     <mergeCell ref="B815:F815"/>
     <mergeCell ref="B597:F597"/>
     <mergeCell ref="B1064:F1064"/>
+    <mergeCell ref="B1113:F1113"/>
     <mergeCell ref="B103:F103"/>
     <mergeCell ref="B78:F78"/>
     <mergeCell ref="B833:F833"/>
+    <mergeCell ref="B1100:F1100"/>
     <mergeCell ref="B205:F205"/>
     <mergeCell ref="B339:F339"/>
     <mergeCell ref="B314:F314"/>
@@ -21264,6 +22085,7 @@
     <mergeCell ref="B305:F305"/>
     <mergeCell ref="B816:F816"/>
     <mergeCell ref="B918:F918"/>
+    <mergeCell ref="B1114:F1114"/>
     <mergeCell ref="B607:F607"/>
     <mergeCell ref="B663:F663"/>
     <mergeCell ref="B1049:F1049"/>
@@ -21274,6 +22096,7 @@
     <mergeCell ref="B442:F442"/>
     <mergeCell ref="B242:F242"/>
     <mergeCell ref="B880:F880"/>
+    <mergeCell ref="B1116:F1116"/>
     <mergeCell ref="B671:F671"/>
     <mergeCell ref="B969:F969"/>
     <mergeCell ref="B907:F907"/>
@@ -21291,12 +22114,15 @@
     <mergeCell ref="B760:F760"/>
     <mergeCell ref="B437:F437"/>
     <mergeCell ref="B852:F852"/>
+    <mergeCell ref="B1119:F1119"/>
     <mergeCell ref="B333:F333"/>
+    <mergeCell ref="B1098:F1098"/>
     <mergeCell ref="B898:F898"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="B520:F520"/>
     <mergeCell ref="B958:F958"/>
     <mergeCell ref="B308:F308"/>
+    <mergeCell ref="B1134:F1134"/>
     <mergeCell ref="B854:F854"/>
     <mergeCell ref="B99:F99"/>
     <mergeCell ref="B737:F737"/>
@@ -21315,12 +22141,14 @@
     <mergeCell ref="B372:F372"/>
     <mergeCell ref="B1071:F1071"/>
     <mergeCell ref="B608:F608"/>
+    <mergeCell ref="B1127:F1127"/>
     <mergeCell ref="B595:F595"/>
     <mergeCell ref="B1037:F1037"/>
     <mergeCell ref="B722:F722"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="A856:F856"/>
     <mergeCell ref="B893:F893"/>
+    <mergeCell ref="B1129:F1129"/>
     <mergeCell ref="B374:F374"/>
     <mergeCell ref="B659:F659"/>
     <mergeCell ref="B830:F830"/>
@@ -21389,6 +22217,7 @@
     <mergeCell ref="B309:F309"/>
     <mergeCell ref="A316:F316"/>
     <mergeCell ref="B380:F380"/>
+    <mergeCell ref="B1135:F1135"/>
     <mergeCell ref="A1081:F1081"/>
     <mergeCell ref="B100:F100"/>
     <mergeCell ref="B336:F336"/>
@@ -21398,10 +22227,12 @@
     <mergeCell ref="B140:F140"/>
     <mergeCell ref="B115:F115"/>
     <mergeCell ref="B382:F382"/>
+    <mergeCell ref="A1096:F1096"/>
     <mergeCell ref="B680:F680"/>
     <mergeCell ref="A376:F376"/>
     <mergeCell ref="B102:F102"/>
     <mergeCell ref="B674:F674"/>
+    <mergeCell ref="B1137:F1137"/>
     <mergeCell ref="B400:F400"/>
     <mergeCell ref="B698:F698"/>
     <mergeCell ref="B832:F832"/>
@@ -21414,6 +22245,7 @@
     <mergeCell ref="B598:F598"/>
     <mergeCell ref="B402:F402"/>
     <mergeCell ref="B669:F669"/>
+    <mergeCell ref="B1138:F1138"/>
     <mergeCell ref="B377:F377"/>
     <mergeCell ref="A451:F451"/>
     <mergeCell ref="B29:F29"/>
@@ -21620,11 +22452,14 @@
     <mergeCell ref="B409:F409"/>
     <mergeCell ref="B580:F580"/>
     <mergeCell ref="B920:F920"/>
+    <mergeCell ref="B1108:F1108"/>
     <mergeCell ref="B711:F711"/>
     <mergeCell ref="B1009:F1009"/>
     <mergeCell ref="B48:F48"/>
+    <mergeCell ref="B1101:F1101"/>
     <mergeCell ref="B582:F582"/>
     <mergeCell ref="B849:F849"/>
+    <mergeCell ref="B1132:F1132"/>
     <mergeCell ref="B73:F73"/>
     <mergeCell ref="B371:F371"/>
     <mergeCell ref="B638:F638"/>
@@ -21637,6 +22472,7 @@
     <mergeCell ref="A676:F676"/>
     <mergeCell ref="B137:F137"/>
     <mergeCell ref="B379:F379"/>
+    <mergeCell ref="B1106:F1106"/>
     <mergeCell ref="B702:F702"/>
     <mergeCell ref="B677:F677"/>
     <mergeCell ref="B640:F640"/>
@@ -21667,6 +22503,7 @@
     <mergeCell ref="B66:F66"/>
     <mergeCell ref="B326:F326"/>
     <mergeCell ref="B793:F793"/>
+    <mergeCell ref="B1103:F1103"/>
     <mergeCell ref="A406:F406"/>
     <mergeCell ref="B951:F951"/>
     <mergeCell ref="B130:F130"/>
@@ -21685,6 +22522,7 @@
     <mergeCell ref="B132:F132"/>
     <mergeCell ref="B425:F425"/>
     <mergeCell ref="B430:F430"/>
+    <mergeCell ref="B1107:F1107"/>
     <mergeCell ref="B1045:F1045"/>
     <mergeCell ref="B119:F119"/>
     <mergeCell ref="B290:F290"/>
@@ -21695,10 +22533,13 @@
     <mergeCell ref="B824:F824"/>
     <mergeCell ref="B1017:F1017"/>
     <mergeCell ref="B367:F367"/>
+    <mergeCell ref="B1122:F1122"/>
     <mergeCell ref="B427:F427"/>
+    <mergeCell ref="B1139:F1139"/>
     <mergeCell ref="B112:F112"/>
     <mergeCell ref="B283:F283"/>
     <mergeCell ref="B354:F354"/>
+    <mergeCell ref="B1109:F1109"/>
     <mergeCell ref="B348:F348"/>
     <mergeCell ref="B519:F519"/>
     <mergeCell ref="B419:F419"/>
@@ -21714,6 +22555,7 @@
     <mergeCell ref="B648:F648"/>
     <mergeCell ref="B64:F64"/>
     <mergeCell ref="B51:F51"/>
+    <mergeCell ref="A1126:F1126"/>
     <mergeCell ref="B443:F443"/>
     <mergeCell ref="A196:F196"/>
     <mergeCell ref="B237:F237"/>
@@ -21792,6 +22634,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1064" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1079" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1094" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1109" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1124" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1139" r:id="rId76"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -21803,7 +22648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J74"/>
+  <dimension ref="A1:J77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -23845,12 +24690,12 @@
     <row r="54" ht="28" customHeight="1">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>c427200b-e175-4101-b8d4-4ec219539e45-PIN</t>
+          <t>4b45d249-5739-4bf7-9595-a4715b73c2f6-EXA</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>Mission Implementation Platform for Mission "A Soil Deal for</t>
+          <t>Border regions Peer exchange on solving border obstacles</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr"/>
@@ -23877,28 +24722,24 @@
     <row r="55" ht="28" customHeight="1">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>EUS-52341</t>
+          <t>c427200b-e175-4101-b8d4-4ec219539e45-PIN</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
-        </is>
-      </c>
-      <c r="C55" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
+          <t>Mission Implementation Platform for Mission "A Soil Deal for</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr"/>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="E55" s="6" t="inlineStr"/>
       <c r="F55" s="25" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="G55" s="6" t="inlineStr"/>
@@ -23913,12 +24754,12 @@
     <row r="56" ht="28" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>EUS-38721</t>
+          <t>EUS-64028</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la gestión sostenible de los recursos pesqueros 202</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
@@ -23949,12 +24790,12 @@
     <row r="57" ht="28" customHeight="1">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>EUS-40875</t>
+          <t>EUS-77748</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la recogida de residuos con la participación de los</t>
+          <t>Ayudas a la gestión sostenible de los recursos pesqueros 202</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
@@ -23985,12 +24826,12 @@
     <row r="58" ht="28" customHeight="1">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>EUS-46334</t>
+          <t>EUS-23804</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
+          <t>Ayudas a la recogida de residuos con la participación de los</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
@@ -24021,12 +24862,12 @@
     <row r="59" ht="28" customHeight="1">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>EUS-62067</t>
+          <t>EUS-89133</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la contribución de la acuicultura al buen estado am</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
@@ -24042,7 +24883,7 @@
       <c r="E59" s="6" t="inlineStr"/>
       <c r="F59" s="25" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="G59" s="6" t="inlineStr"/>
@@ -24057,12 +24898,12 @@
     <row r="60" ht="28" customHeight="1">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>EUS-84073</t>
+          <t>EUS-48991</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>Ayudas al valor añadido, economía circular y seguridad alime</t>
+          <t>Ayudas a la contribución de la acuicultura al buen estado am</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -24093,12 +24934,12 @@
     <row r="61" ht="28" customHeight="1">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>EUS-89931</t>
+          <t>EUS-06375</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>Vino: el Gobierno Vasco volverá a convocar este mes las ayud</t>
+          <t>Ayudas al valor añadido, economía circular y seguridad alime</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
@@ -24129,12 +24970,12 @@
     <row r="62" ht="28" customHeight="1">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>EUS-60483</t>
+          <t>EUS-79267</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de</t>
+          <t>Vino: el Gobierno Vasco volverá a convocar este mes las ayud</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
@@ -24165,12 +25006,12 @@
     <row r="63" ht="28" customHeight="1">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>EUS-46455</t>
+          <t>EUS-85579</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para c</t>
+          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
@@ -24201,12 +25042,12 @@
     <row r="64" ht="28" customHeight="1">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>EUS-38314</t>
+          <t>EUS-03347</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinanc</t>
+          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para c</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
@@ -24237,12 +25078,12 @@
     <row r="65" ht="28" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>EUS-56475</t>
+          <t>EUS-87925</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>Digital Europe, Horizon (programas de la UE). Apoyos para co</t>
+          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinanc</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -24273,12 +25114,12 @@
     <row r="66" ht="28" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>EUS-05137</t>
+          <t>EUS-21599</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>Política Agraria Común de la UE de 2026, y sus ayudas abiert</t>
+          <t>Digital Europe, Horizon (programas de la UE). Apoyos para co</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
@@ -24309,12 +25150,12 @@
     <row r="67" ht="28" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>EUS-12265</t>
+          <t>EUS-91637</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>Programa de impulso a las ciudades y territorios inteligente</t>
+          <t>Política Agraria Común de la UE de 2026, y sus ayudas abiert</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
@@ -24345,12 +25186,12 @@
     <row r="68" ht="28" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>EUS-58053</t>
+          <t>EUS-38365</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Suministro, Implementación y Soporte de un Servicio Digital </t>
+          <t>Programa de impulso a las ciudades y territorios inteligente</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -24381,12 +25222,12 @@
     <row r="69" ht="28" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>EUS-97072</t>
+          <t>EUS-84600</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>Suministro de driver 75w y lamparas de 360w para farolas (al</t>
+          <t xml:space="preserve">Servicio de Punto Verde Móvil en el Territorio Histórico de </t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -24417,12 +25258,12 @@
     <row r="70" ht="28" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>EUS-77422</t>
+          <t>EUS-18669</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>Suministro de material eléctrico (driver 150w) para alumbrad</t>
+          <t>Servicio de agencia de viajes para el Departamento de Hacien</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -24453,12 +25294,12 @@
     <row r="71" ht="28" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>EUS-95174</t>
+          <t>EUS-29543</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>Reparacion de la bomba del circuito de recirculacion del agu</t>
+          <t>Conferencia sobre "la bicicleta, un máquina móvil, veloz y b</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -24489,12 +25330,12 @@
     <row r="72" ht="28" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>EUS-49048</t>
+          <t>EUS-17370</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>Limpieza de foso ascensor errebal</t>
+          <t>Organización parque infantil de Navidad</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -24525,12 +25366,12 @@
     <row r="73" ht="28" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>EUS-90362</t>
+          <t>EUS-46342</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>Digitalización de la imagen del cartel de las jornadas de te</t>
+          <t>Alumbrado publico pasos peatonales en La Calzada</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -24561,12 +25402,12 @@
     <row r="74" ht="28" customHeight="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>EUS-98149</t>
+          <t>EUS-02378</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>Servicio técnico para realizar la sustitución del servidor i</t>
+          <t>Reparación faldón cubierta Museo Santa Clara</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
@@ -24594,8 +25435,116 @@
       <c r="I74" s="6" t="inlineStr"/>
       <c r="J74" s="6" t="inlineStr"/>
     </row>
+    <row r="75" ht="28" customHeight="1">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>EUS-69611</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>Limpieza y desescombro desatasco colector de saneamiento</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D75" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E75" s="6" t="inlineStr"/>
+      <c r="F75" s="25" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G75" s="6" t="inlineStr"/>
+      <c r="H75" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I75" s="6" t="inlineStr"/>
+      <c r="J75" s="6" t="inlineStr"/>
+    </row>
+    <row r="76" ht="28" customHeight="1">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>EUS-00349</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>Reparación instalación fotovoltaica refugio del Kolitza</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E76" s="6" t="inlineStr"/>
+      <c r="F76" s="25" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G76" s="6" t="inlineStr"/>
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I76" s="6" t="inlineStr"/>
+      <c r="J76" s="6" t="inlineStr"/>
+    </row>
+    <row r="77" ht="28" customHeight="1">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>EUS-93515</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>Formación en jardineria forestal</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="inlineStr"/>
+      <c r="F77" s="25" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G77" s="6" t="inlineStr"/>
+      <c r="H77" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I77" s="6" t="inlineStr"/>
+      <c r="J77" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J74"/>
+  <autoFilter ref="A1:J77"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update funding data 2026-03-26
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Recursos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$84</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$74</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -84,13 +84,13 @@
     <font>
       <name val="Leelawadee UI"/>
       <b val="1"/>
-      <color rgb="00DC2626"/>
+      <color rgb="00065F46"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Leelawadee UI"/>
       <b val="1"/>
-      <color rgb="00065F46"/>
+      <color rgb="00DC2626"/>
       <sz val="10"/>
     </font>
     <font>
@@ -166,17 +166,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00065F46"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -268,11 +268,11 @@
     <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -312,8 +312,8 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -679,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M84"/>
+  <dimension ref="A1:M80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -707,7 +707,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 25/03/2026 06:50 - 77 convocatorias - 24 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 26/03/2026 07:03 - 73 convocatorias - 19 nuevas</t>
         </is>
       </c>
     </row>
@@ -919,19 +919,15 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>INNOVFUND-2025-NZT-GENERAL-MSP</t>
+          <t>02ea5f5c-3122-4e73-a32a-dfb5ff0f395c-CN</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Medium-Scale Projects</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>Innovation Fund</t>
-        </is>
-      </c>
+          <t>Analysis of target setting for a selection of common indicators used under the European Regional Development Fund, Cohesion Fund and Just Transition Fund in 2021-2027</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr"/>
       <c r="E8" s="7" t="inlineStr">
         <is>
           <t>Open</t>
@@ -939,15 +935,11 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr"/>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>INNOVFUND Lump Sum Grants</t>
-        </is>
-      </c>
+      <c r="H8" s="6" t="inlineStr"/>
       <c r="I8" s="10" t="inlineStr">
         <is>
           <t>MEDIA</t>
@@ -955,12 +947,12 @@
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>Aplicable a Petronor/Repsol (Muskiz) y Puerto de Bilbao.</t>
+          <t>Margen izquierda con pasado industrial. Potencial reconversión.</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Medium-Scale Projects</t>
+          <t>Analysis of target setting for a selection of common indicators used under the European Regional Development Fund, Cohesion Fund and Just Transition Fund in 2021-2027</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr"/>
@@ -978,12 +970,12 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>INNOVFUND-2025-NZT-GENERAL-SSP</t>
+          <t>INNOVFUND-2025-NZT-GENERAL-MSP</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Small-Scale Projects</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Medium-Scale Projects</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -1019,7 +1011,7 @@
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Small-Scale Projects</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Medium-Scale Projects</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr"/>
@@ -1037,12 +1029,12 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>INNOVFUND-2025-NZT-GENERAL-LSP</t>
+          <t>INNOVFUND-2025-NZT-GENERAL-SSP</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Large-Scale Projects</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Small-Scale Projects</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -1078,7 +1070,7 @@
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Large-Scale Projects</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Small-Scale Projects</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr"/>
@@ -1096,17 +1088,17 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-2-PRIZE</t>
+          <t>INNOVFUND-2025-NZT-GENERAL-LSP</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Renewable energy technology (RET) solutions in energy communities</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Large-Scale Projects</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Horizon Europe</t>
+          <t>Innovation Fund</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -1116,13 +1108,13 @@
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>25/06/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr"/>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>Recognition Prize</t>
+          <t>INNOVFUND Lump Sum Grants</t>
         </is>
       </c>
       <c r="I11" s="10" t="inlineStr">
@@ -1132,12 +1124,12 @@
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>Margen izquierda con pasado industrial. Potencial reconversión.</t>
+          <t>Aplicable a Petronor/Repsol (Muskiz) y Puerto de Bilbao.</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>Specific Challenge:Individual energy communities encounter different challenges, such as developing a successful governance structure that is sufficiently inclusive and involves different types of act</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Large-Scale Projects</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr"/>
@@ -1155,15 +1147,19 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>02ea5f5c-3122-4e73-a32a-dfb5ff0f395c-CN</t>
+          <t>HORIZON-CL5-2026-2-PRIZE</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Analysis of target setting for a selection of common indicators used under the European Regional Development Fund, Cohesion Fund and Just Transition Fund in 2021-2027</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr"/>
+          <t>Renewable energy technology (RET) solutions in energy communities</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Horizon Europe</t>
+        </is>
+      </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
           <t>Open</t>
@@ -1171,11 +1167,15 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>30/03/2026</t>
+          <t>25/06/2026</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr"/>
-      <c r="H12" s="6" t="inlineStr"/>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Recognition Prize</t>
+        </is>
+      </c>
       <c r="I12" s="10" t="inlineStr">
         <is>
           <t>MEDIA</t>
@@ -1188,7 +1188,7 @@
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>Analysis of target setting for a selection of common indicators used under the European Regional Development Fund, Cohesion Fund and Just Transition Fund in 2021-2027</t>
+          <t>Specific Challenge:Individual energy communities encounter different challenges, such as developing a successful governance structure that is sufficiently inclusive and involves different types of act</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr"/>
@@ -3911,11 +3911,7 @@
           <t>PYME Y PERSONAS FÍSICAS QUE DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
         </is>
       </c>
-      <c r="L60" s="15" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
+      <c r="L60" s="6" t="inlineStr"/>
       <c r="M60" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
@@ -3923,26 +3919,26 @@
       </c>
     </row>
     <row r="61" ht="28" customHeight="1">
-      <c r="A61" s="16" t="inlineStr">
+      <c r="A61" s="15" t="inlineStr">
         <is>
           <t>🟢 Euskadi</t>
         </is>
       </c>
     </row>
     <row r="62" ht="40" customHeight="1">
-      <c r="A62" s="17" t="inlineStr">
+      <c r="A62" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>EUS-97765</t>
+          <t>EUS-47030</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
+          <t>Servicios de transporte y manipulación de obras de arte para una exposición en el Museo de Bellas Artes de Bilbao</t>
         </is>
       </c>
       <c r="D62" s="6" t="inlineStr">
@@ -3959,12 +3955,12 @@
       <c r="G62" s="6" t="inlineStr"/>
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
-        </is>
-      </c>
-      <c r="I62" s="8" t="inlineStr">
-        <is>
-          <t>ALTA</t>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I62" s="12" t="inlineStr">
+        <is>
+          <t>MUY ALTA</t>
         </is>
       </c>
       <c r="J62" s="6" t="inlineStr"/>
@@ -3973,7 +3969,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L62" s="15" t="inlineStr">
+      <c r="L62" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -3985,19 +3981,19 @@
       </c>
     </row>
     <row r="63" ht="40" customHeight="1">
-      <c r="A63" s="17" t="inlineStr">
+      <c r="A63" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>EUS-23570</t>
+          <t>EUS-15017</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la gestión sostenible de los recursos pesqueros 2026</t>
+          <t>Mantenimiento de las instalaciones de climatización de la oficina de Bilbao</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
@@ -4014,12 +4010,12 @@
       <c r="G63" s="6" t="inlineStr"/>
       <c r="H63" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
-        </is>
-      </c>
-      <c r="I63" s="8" t="inlineStr">
-        <is>
-          <t>ALTA</t>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I63" s="12" t="inlineStr">
+        <is>
+          <t>MUY ALTA</t>
         </is>
       </c>
       <c r="J63" s="6" t="inlineStr"/>
@@ -4028,7 +4024,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L63" s="15" t="inlineStr">
+      <c r="L63" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4040,19 +4036,19 @@
       </c>
     </row>
     <row r="64" ht="40" customHeight="1">
-      <c r="A64" s="17" t="inlineStr">
+      <c r="A64" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>EUS-92691</t>
+          <t>EUS-25647</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la recogida de residuos con la participación de los pescadores en el mar y las playas 2026</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
@@ -4083,7 +4079,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L64" s="15" t="inlineStr">
+      <c r="L64" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4095,19 +4091,19 @@
       </c>
     </row>
     <row r="65" ht="40" customHeight="1">
-      <c r="A65" s="17" t="inlineStr">
+      <c r="A65" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>EUS-34245</t>
+          <t>EUS-39134</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático sin incremento de capacidad 2026</t>
+          <t>Ayudas a la gestión sostenible de los recursos pesqueros 2026</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
@@ -4138,7 +4134,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L65" s="15" t="inlineStr">
+      <c r="L65" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4150,19 +4146,19 @@
       </c>
     </row>
     <row r="66" ht="40" customHeight="1">
-      <c r="A66" s="17" t="inlineStr">
+      <c r="A66" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>EUS-17774</t>
+          <t>EUS-85153</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>Servicio de oficina técnica para la mejora del sistema de prevención y gestión de residuos de competencia local de Bizkaia</t>
+          <t>Ayudas a la recogida de residuos con la participación de los pescadores en el mar y las playas 2026</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
@@ -4179,7 +4175,7 @@
       <c r="G66" s="6" t="inlineStr"/>
       <c r="H66" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="I66" s="8" t="inlineStr">
@@ -4193,7 +4189,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L66" s="15" t="inlineStr">
+      <c r="L66" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4205,19 +4201,19 @@
       </c>
     </row>
     <row r="67" ht="40" customHeight="1">
-      <c r="A67" s="17" t="inlineStr">
+      <c r="A67" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>EUS-22731</t>
+          <t>EUS-21937</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>Redacción de un Plan de prevención y gestión de residuos</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio climático sin incremento de capacidad 2026</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
@@ -4234,7 +4230,7 @@
       <c r="G67" s="6" t="inlineStr"/>
       <c r="H67" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="I67" s="8" t="inlineStr">
@@ -4248,7 +4244,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L67" s="15" t="inlineStr">
+      <c r="L67" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4260,19 +4256,19 @@
       </c>
     </row>
     <row r="68" ht="40" customHeight="1">
-      <c r="A68" s="17" t="inlineStr">
+      <c r="A68" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>EUS-32199</t>
+          <t>EUS-02512</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
+          <t>Servicio de transporte y gestión de los residuos procedentes de corte de orilla de playas</t>
         </is>
       </c>
       <c r="D68" s="6" t="inlineStr">
@@ -4289,12 +4285,12 @@
       <c r="G68" s="6" t="inlineStr"/>
       <c r="H68" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
-        </is>
-      </c>
-      <c r="I68" s="10" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I68" s="8" t="inlineStr">
+        <is>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="J68" s="6" t="inlineStr"/>
@@ -4303,7 +4299,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L68" s="15" t="inlineStr">
+      <c r="L68" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4315,19 +4311,19 @@
       </c>
     </row>
     <row r="69" ht="40" customHeight="1">
-      <c r="A69" s="17" t="inlineStr">
+      <c r="A69" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>EUS-89864</t>
+          <t>EUS-91129</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>Ayudas al valor añadido, economía circular y seguridad alimentaria 2026</t>
+          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
@@ -4358,7 +4354,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L69" s="15" t="inlineStr">
+      <c r="L69" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4370,19 +4366,19 @@
       </c>
     </row>
     <row r="70" ht="40" customHeight="1">
-      <c r="A70" s="17" t="inlineStr">
+      <c r="A70" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>EUS-92385</t>
+          <t>EUS-46360</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>Vino: el Gobierno Vasco volverá a convocar este mes las ayudas al arranque o cosecha en verde del viñedo, que van a contemplar como estructurales tras reformar la UE jurídicamente su Intervención Sect</t>
+          <t>Ayudas al valor añadido, economía circular y seguridad alimentaria 2026</t>
         </is>
       </c>
       <c r="D70" s="6" t="inlineStr">
@@ -4413,7 +4409,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L70" s="15" t="inlineStr">
+      <c r="L70" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4425,19 +4421,19 @@
       </c>
     </row>
     <row r="71" ht="40" customHeight="1">
-      <c r="A71" s="17" t="inlineStr">
+      <c r="A71" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>EUS-45123</t>
+          <t>EUS-14446</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de aceleración de proyectos, a localidades de menos de 20.000 habitantes son objeto de convocatoria abierta hasta el 17.03.26. Transformacione</t>
+          <t>Vino: el Gobierno Vasco volverá a convocar este mes las ayudas al arranque o cosecha en verde del viñedo, que van a contemplar como estructurales tras reformar la UE jurídicamente su Intervención Sect</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
@@ -4468,7 +4464,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L71" s="15" t="inlineStr">
+      <c r="L71" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4480,19 +4476,19 @@
       </c>
     </row>
     <row r="72" ht="40" customHeight="1">
-      <c r="A72" s="17" t="inlineStr">
+      <c r="A72" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>EUS-63814</t>
+          <t>EUS-75188</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para consorcios internacionales de I+D+i. Jornada del Gobierno Vasco y con Enterprise Europe Network y otros socios. Digitalización, dispositivos,</t>
+          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de aceleración de proyectos, a localidades de menos de 20.000 habitantes son objeto de convocatoria abierta hasta el 17.03.26. Transformacione</t>
         </is>
       </c>
       <c r="D72" s="6" t="inlineStr">
@@ -4523,7 +4519,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L72" s="15" t="inlineStr">
+      <c r="L72" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4535,19 +4531,19 @@
       </c>
     </row>
     <row r="73" ht="40" customHeight="1">
-      <c r="A73" s="17" t="inlineStr">
+      <c r="A73" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>EUS-82158</t>
+          <t>EUS-45072</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinancia convocatorias de ayudas de las Diputaciones a explotaciones con limitaciones o desfavorecidas, y a compromisos medioambientales, climátic</t>
+          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para consorcios internacionales de I+D+i. Jornada del Gobierno Vasco y con Enterprise Europe Network y otros socios. Digitalización, dispositivos,</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
@@ -4578,7 +4574,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L73" s="15" t="inlineStr">
+      <c r="L73" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4590,19 +4586,19 @@
       </c>
     </row>
     <row r="74" ht="40" customHeight="1">
-      <c r="A74" s="17" t="inlineStr">
+      <c r="A74" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>EUS-92414</t>
+          <t>EUS-36943</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>Digital Europe, Horizon (programas de la UE). Apoyos para consorcios interestatales de I+D+i. IA, robótica, cuántica, computación, ciberseguridad, electrónica, fotónica, TICs e internet avanzadas, esp</t>
+          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinancia convocatorias de ayudas de las Diputaciones a explotaciones con limitaciones o desfavorecidas, y a compromisos medioambientales, climátic</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr">
@@ -4633,7 +4629,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L74" s="15" t="inlineStr">
+      <c r="L74" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4645,19 +4641,19 @@
       </c>
     </row>
     <row r="75" ht="40" customHeight="1">
-      <c r="A75" s="17" t="inlineStr">
+      <c r="A75" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>EUS-62683</t>
+          <t>EUS-80876</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>Política Agraria Común de la UE de 2026, y sus ayudas abiertas hasta el 30.4.26: el pilar 1, con el Fondo Europeo Agrícola de Garantía Agraria FEAGA, aborda sostenibilidad de renta, ayuda redistributi</t>
+          <t>Digital Europe, Horizon (programas de la UE). Apoyos para consorcios interestatales de I+D+i. IA, robótica, cuántica, computación, ciberseguridad, electrónica, fotónica, TICs e internet avanzadas, esp</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
@@ -4688,7 +4684,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L75" s="15" t="inlineStr">
+      <c r="L75" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4700,19 +4696,19 @@
       </c>
     </row>
     <row r="76" ht="40" customHeight="1">
-      <c r="A76" s="17" t="inlineStr">
+      <c r="A76" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>EUS-33389</t>
+          <t>EUS-03523</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>Programa de impulso a las ciudades y territorios inteligentes para el fomento del desarrollo económico y productivo, que podrá ser cofinanciado por el Programa Plurirregional 2021-2027 del Fondo Europ</t>
+          <t>Política Agraria Común de la UE de 2026, y sus ayudas abiertas hasta el 30.4.26: el pilar 1, con el Fondo Europeo Agrícola de Garantía Agraria FEAGA, aborda sostenibilidad de renta, ayuda redistributi</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr">
@@ -4743,7 +4739,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L76" s="15" t="inlineStr">
+      <c r="L76" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4755,19 +4751,19 @@
       </c>
     </row>
     <row r="77" ht="40" customHeight="1">
-      <c r="A77" s="17" t="inlineStr">
+      <c r="A77" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>EUS-40042</t>
+          <t>EUS-44113</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>Suministros y Servicios para la instalación de una red XGS-PON y electrónica de red en la nueva Sede de EITB Gasteiz y renovación de la infraestructura WLAN de EITB.</t>
+          <t>Programa de impulso a las ciudades y territorios inteligentes para el fomento del desarrollo económico y productivo, que podrá ser cofinanciado por el Programa Plurirregional 2021-2027 del Fondo Europ</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
@@ -4784,7 +4780,7 @@
       <c r="G77" s="6" t="inlineStr"/>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="I77" s="10" t="inlineStr">
@@ -4798,7 +4794,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L77" s="15" t="inlineStr">
+      <c r="L77" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4810,19 +4806,19 @@
       </c>
     </row>
     <row r="78" ht="40" customHeight="1">
-      <c r="A78" s="17" t="inlineStr">
+      <c r="A78" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>EUS-25076</t>
+          <t>EUS-71405</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>Realización del vuelo fotogramétrico digital multivista, escenas 3D y ortofotos verdaderas de 5cm de las localidades con más de 15.000 habitantes del País Vasco (2026)</t>
+          <t>Dirección facultativa de obra (dirección de obra, dirección de ejecución y coordinación de seguridad y salud) y ejecución del proyecto de la nueva cubierta exterior de Izarraizpe Ikastola</t>
         </is>
       </c>
       <c r="D78" s="6" t="inlineStr">
@@ -4853,7 +4849,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L78" s="15" t="inlineStr">
+      <c r="L78" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4865,19 +4861,19 @@
       </c>
     </row>
     <row r="79" ht="40" customHeight="1">
-      <c r="A79" s="17" t="inlineStr">
+      <c r="A79" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>EUS-13379</t>
+          <t>EUS-85319</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>Suministro para la ampliación de la infraestructura de los repositorios de Copias de Seguridad de EJIE</t>
+          <t>Licitación de la obra ?Adecuación del espacio público y ejecución de nuevas redes de pluviales y acometida de agua? en Mendiola (Álava).</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
@@ -4908,7 +4904,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L79" s="15" t="inlineStr">
+      <c r="L79" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4920,19 +4916,19 @@
       </c>
     </row>
     <row r="80" ht="40" customHeight="1">
-      <c r="A80" s="17" t="inlineStr">
+      <c r="A80" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>EUS-89192</t>
+          <t>EUS-57006</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>Suministro e instalación de fuente de agua fría para consumo de usuarios en zona de spa del polideportivo orbea</t>
+          <t>Suministro de un sistema de Seguridad e Información Turística en el edificio Cocheras de la Finca Munoa en el marco del Plan Europeo de Recuperación, Transformación y Resiliencia, financiado por la Un</t>
         </is>
       </c>
       <c r="D80" s="6" t="inlineStr">
@@ -4963,7 +4959,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L80" s="15" t="inlineStr">
+      <c r="L80" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4974,228 +4970,8 @@
         </is>
       </c>
     </row>
-    <row r="81" ht="40" customHeight="1">
-      <c r="A81" s="17" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="B81" s="6" t="inlineStr">
-        <is>
-          <t>EUS-06858</t>
-        </is>
-      </c>
-      <c r="C81" s="6" t="inlineStr">
-        <is>
-          <t>Equipamiento de muebles en vivienda municipal</t>
-        </is>
-      </c>
-      <c r="D81" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="E81" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F81" s="6" t="inlineStr"/>
-      <c r="G81" s="6" t="inlineStr"/>
-      <c r="H81" s="6" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I81" s="10" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="J81" s="6" t="inlineStr"/>
-      <c r="K81" s="6" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="L81" s="15" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="M81" s="9" t="inlineStr">
-        <is>
-          <t>Ver</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="40" customHeight="1">
-      <c r="A82" s="17" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="B82" s="6" t="inlineStr">
-        <is>
-          <t>EUS-68952</t>
-        </is>
-      </c>
-      <c r="C82" s="6" t="inlineStr">
-        <is>
-          <t>Servicio de limpieza, DDD y legionella de edificios municipales respetuosos con entorno de Muskiz</t>
-        </is>
-      </c>
-      <c r="D82" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="E82" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F82" s="6" t="inlineStr"/>
-      <c r="G82" s="6" t="inlineStr"/>
-      <c r="H82" s="6" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I82" s="10" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="J82" s="6" t="inlineStr"/>
-      <c r="K82" s="6" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="L82" s="15" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="M82" s="9" t="inlineStr">
-        <is>
-          <t>Ver</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="40" customHeight="1">
-      <c r="A83" s="17" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="B83" s="6" t="inlineStr">
-        <is>
-          <t>EUS-87256</t>
-        </is>
-      </c>
-      <c r="C83" s="6" t="inlineStr">
-        <is>
-          <t>Mantenimiento caldera y prevencion legionela</t>
-        </is>
-      </c>
-      <c r="D83" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="E83" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F83" s="6" t="inlineStr"/>
-      <c r="G83" s="6" t="inlineStr"/>
-      <c r="H83" s="6" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I83" s="10" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="J83" s="6" t="inlineStr"/>
-      <c r="K83" s="6" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="L83" s="15" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="M83" s="9" t="inlineStr">
-        <is>
-          <t>Ver</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="40" customHeight="1">
-      <c r="A84" s="17" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="B84" s="6" t="inlineStr">
-        <is>
-          <t>EUS-21550</t>
-        </is>
-      </c>
-      <c r="C84" s="6" t="inlineStr">
-        <is>
-          <t>Mantenimiento anual y servicio de limpieza de tubos de ozono</t>
-        </is>
-      </c>
-      <c r="D84" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="E84" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F84" s="6" t="inlineStr"/>
-      <c r="G84" s="6" t="inlineStr"/>
-      <c r="H84" s="6" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I84" s="10" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="J84" s="6" t="inlineStr"/>
-      <c r="K84" s="6" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="L84" s="15" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="M84" s="9" t="inlineStr">
-        <is>
-          <t>Ver</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:M84"/>
+  <autoFilter ref="A4:M80"/>
   <mergeCells count="5">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A5:M5"/>
@@ -5277,10 +5053,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M78" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M79" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M80" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M81" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M82" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M83" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M84" r:id="rId77"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5292,7 +5064,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1154"/>
+  <dimension ref="A1:F1094"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5738,7 +5510,7 @@
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="18" t="inlineStr">
         <is>
-          <t>FICHA 3: INNOVFUND-2025-NZT-GENERAL-MSP</t>
+          <t>FICHA 3: 02ea5f5c-3122-4e73-a32a-dfb5ff0f395c-CN</t>
         </is>
       </c>
       <c r="B31" s="19" t="n"/>
@@ -5771,7 +5543,7 @@
       </c>
       <c r="B33" s="21" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Medium-Scale Projects</t>
+          <t>Analysis of target setting for a selection of common indicators used under the European Regional Development Fund, Cohesion Fund and Just Transition Fund in 2021-2027</t>
         </is>
       </c>
       <c r="C33" s="22" t="n"/>
@@ -5787,7 +5559,7 @@
       </c>
       <c r="B34" s="21" t="inlineStr">
         <is>
-          <t>INNOVFUND-2025-NZT-GENERAL-MSP</t>
+          <t>02ea5f5c-3122-4e73-a32a-dfb5ff0f395c-CN</t>
         </is>
       </c>
       <c r="C34" s="22" t="n"/>
@@ -5801,11 +5573,7 @@
           <t>Programa</t>
         </is>
       </c>
-      <c r="B35" s="21" t="inlineStr">
-        <is>
-          <t>Innovation Fund</t>
-        </is>
-      </c>
+      <c r="B35" s="21" t="inlineStr"/>
       <c r="C35" s="22" t="n"/>
       <c r="D35" s="22" t="n"/>
       <c r="E35" s="22" t="n"/>
@@ -5835,7 +5603,7 @@
       </c>
       <c r="B37" s="21" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="C37" s="22" t="n"/>
@@ -5867,7 +5635,7 @@
       </c>
       <c r="B39" s="21" t="inlineStr">
         <is>
-          <t>INNOVFUND Lump Sum Grants</t>
+          <t>No disponible</t>
         </is>
       </c>
       <c r="C39" s="22" t="n"/>
@@ -5883,7 +5651,7 @@
       </c>
       <c r="B40" s="21" t="inlineStr">
         <is>
-          <t>INNOVFUND-2025-NZT</t>
+          <t>EC-REGIO/2026/OP/0013</t>
         </is>
       </c>
       <c r="C40" s="22" t="n"/>
@@ -5899,7 +5667,7 @@
       </c>
       <c r="B41" s="21" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Medium-Scale Projects</t>
+          <t>Analysis of target setting for a selection of common indicators used under the European Regional Development Fund, Cohesion Fund and Just Transition Fund in 2021-2027</t>
         </is>
       </c>
       <c r="C41" s="22" t="n"/>
@@ -5907,17 +5675,13 @@
       <c r="E41" s="22" t="n"/>
       <c r="F41" s="22" t="n"/>
     </row>
-    <row r="42" ht="45" customHeight="1">
+    <row r="42" ht="20" customHeight="1">
       <c r="A42" s="20" t="inlineStr">
         <is>
           <t>Tags</t>
         </is>
       </c>
-      <c r="B42" s="21" t="inlineStr">
-        <is>
-          <t>Aviation, Bioenergy, Buildings, CCS, CCU, CINEA, CLIMA, CO2, Carbon intensive, Circularity, ETS, ETS installation, Electrification, Emissions Trading System, GHG, Green Deal, Green Industry, Green hydrogen, H2, Hydrogen, Innovation Fund, Low Carbon Hydrogen, Maritime, Net-zero, Recycling, Road transport, carbon capture and storage, carbon capture and utilisation, carbon neutral, clean energy, clean tech, clean technologies, climate change, demonstration, emission avoidance, emission savings, energy intensive industry, energy storage, energy transition, greenhouse gas, heavy industry, industry, low-carbon technologies, renewable energy, STEP-Cleantech</t>
-        </is>
-      </c>
+      <c r="B42" s="21" t="inlineStr"/>
       <c r="C42" s="22" t="n"/>
       <c r="D42" s="22" t="n"/>
       <c r="E42" s="22" t="n"/>
@@ -5931,7 +5695,7 @@
       </c>
       <c r="B43" s="21" t="inlineStr">
         <is>
-          <t>MEDIA — Aplicable a Petronor/Repsol (Muskiz) y Puerto de Bilbao.</t>
+          <t>MEDIA — Margen izquierda con pasado industrial. Potencial reconversión.</t>
         </is>
       </c>
       <c r="C43" s="22" t="n"/>
@@ -5947,7 +5711,7 @@
       </c>
       <c r="B44" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/INNOVFUND-2025-NZT-GENERAL-MSP</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/02ea5f5c-3122-4e73-a32a-dfb5ff0f395c-CN</t>
         </is>
       </c>
       <c r="C44" s="22" t="n"/>
@@ -5958,7 +5722,7 @@
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="18" t="inlineStr">
         <is>
-          <t>FICHA 4: INNOVFUND-2025-NZT-GENERAL-SSP</t>
+          <t>FICHA 4: INNOVFUND-2025-NZT-GENERAL-MSP</t>
         </is>
       </c>
       <c r="B46" s="19" t="n"/>
@@ -5991,7 +5755,7 @@
       </c>
       <c r="B48" s="21" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Small-Scale Projects</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Medium-Scale Projects</t>
         </is>
       </c>
       <c r="C48" s="22" t="n"/>
@@ -6007,7 +5771,7 @@
       </c>
       <c r="B49" s="21" t="inlineStr">
         <is>
-          <t>INNOVFUND-2025-NZT-GENERAL-SSP</t>
+          <t>INNOVFUND-2025-NZT-GENERAL-MSP</t>
         </is>
       </c>
       <c r="C49" s="22" t="n"/>
@@ -6119,7 +5883,7 @@
       </c>
       <c r="B56" s="21" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Small-Scale Projects</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Medium-Scale Projects</t>
         </is>
       </c>
       <c r="C56" s="22" t="n"/>
@@ -6167,7 +5931,7 @@
       </c>
       <c r="B59" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/INNOVFUND-2025-NZT-GENERAL-SSP</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/INNOVFUND-2025-NZT-GENERAL-MSP</t>
         </is>
       </c>
       <c r="C59" s="22" t="n"/>
@@ -6178,7 +5942,7 @@
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="18" t="inlineStr">
         <is>
-          <t>FICHA 5: INNOVFUND-2025-NZT-GENERAL-LSP</t>
+          <t>FICHA 5: INNOVFUND-2025-NZT-GENERAL-SSP</t>
         </is>
       </c>
       <c r="B61" s="19" t="n"/>
@@ -6211,7 +5975,7 @@
       </c>
       <c r="B63" s="21" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Large-Scale Projects</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Small-Scale Projects</t>
         </is>
       </c>
       <c r="C63" s="22" t="n"/>
@@ -6227,7 +5991,7 @@
       </c>
       <c r="B64" s="21" t="inlineStr">
         <is>
-          <t>INNOVFUND-2025-NZT-GENERAL-LSP</t>
+          <t>INNOVFUND-2025-NZT-GENERAL-SSP</t>
         </is>
       </c>
       <c r="C64" s="22" t="n"/>
@@ -6339,7 +6103,7 @@
       </c>
       <c r="B71" s="21" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Large-Scale Projects</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Small-Scale Projects</t>
         </is>
       </c>
       <c r="C71" s="22" t="n"/>
@@ -6387,7 +6151,7 @@
       </c>
       <c r="B74" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/INNOVFUND-2025-NZT-GENERAL-LSP</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/INNOVFUND-2025-NZT-GENERAL-SSP</t>
         </is>
       </c>
       <c r="C74" s="22" t="n"/>
@@ -6398,7 +6162,7 @@
     <row r="76" ht="30" customHeight="1">
       <c r="A76" s="18" t="inlineStr">
         <is>
-          <t>FICHA 6: HORIZON-CL5-2026-2-PRIZE</t>
+          <t>FICHA 6: INNOVFUND-2025-NZT-GENERAL-LSP</t>
         </is>
       </c>
       <c r="B76" s="19" t="n"/>
@@ -6423,7 +6187,7 @@
       <c r="E77" s="22" t="n"/>
       <c r="F77" s="22" t="n"/>
     </row>
-    <row r="78" ht="20" customHeight="1">
+    <row r="78" ht="45" customHeight="1">
       <c r="A78" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -6431,7 +6195,7 @@
       </c>
       <c r="B78" s="21" t="inlineStr">
         <is>
-          <t>Renewable energy technology (RET) solutions in energy communities</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Large-Scale Projects</t>
         </is>
       </c>
       <c r="C78" s="22" t="n"/>
@@ -6447,7 +6211,7 @@
       </c>
       <c r="B79" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-2-PRIZE</t>
+          <t>INNOVFUND-2025-NZT-GENERAL-LSP</t>
         </is>
       </c>
       <c r="C79" s="22" t="n"/>
@@ -6463,7 +6227,7 @@
       </c>
       <c r="B80" s="21" t="inlineStr">
         <is>
-          <t>Horizon Europe</t>
+          <t>Innovation Fund</t>
         </is>
       </c>
       <c r="C80" s="22" t="n"/>
@@ -6495,7 +6259,7 @@
       </c>
       <c r="B82" s="21" t="inlineStr">
         <is>
-          <t>25/06/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="C82" s="22" t="n"/>
@@ -6527,7 +6291,7 @@
       </c>
       <c r="B84" s="21" t="inlineStr">
         <is>
-          <t>Recognition Prize</t>
+          <t>INNOVFUND Lump Sum Grants</t>
         </is>
       </c>
       <c r="C84" s="22" t="n"/>
@@ -6543,7 +6307,7 @@
       </c>
       <c r="B85" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-2-PRIZE</t>
+          <t>INNOVFUND-2025-NZT</t>
         </is>
       </c>
       <c r="C85" s="22" t="n"/>
@@ -6559,7 +6323,7 @@
       </c>
       <c r="B86" s="21" t="inlineStr">
         <is>
-          <t>Specific Challenge:Individual energy communities encounter different challenges, such as developing a successful governance structure that is sufficiently inclusive and involves different types of actors, carrying out an effective business model and embedding activities within the structure and management of the European Commission to territorial regional and/or local plans (e.g., Just Transition Plans, Climate City Contracts, etc.). By rewarding Energy Communities’ innovative governance structure and management of a RET, the prize aims to inspire other Energy Communities to improve their oper</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbonisation - Large-Scale Projects</t>
         </is>
       </c>
       <c r="C86" s="22" t="n"/>
@@ -6567,13 +6331,17 @@
       <c r="E86" s="22" t="n"/>
       <c r="F86" s="22" t="n"/>
     </row>
-    <row r="87" ht="20" customHeight="1">
+    <row r="87" ht="45" customHeight="1">
       <c r="A87" s="20" t="inlineStr">
         <is>
           <t>Tags</t>
         </is>
       </c>
-      <c r="B87" s="21" t="inlineStr"/>
+      <c r="B87" s="21" t="inlineStr">
+        <is>
+          <t>Aviation, Bioenergy, Buildings, CCS, CCU, CINEA, CLIMA, CO2, Carbon intensive, Circularity, ETS, ETS installation, Electrification, Emissions Trading System, GHG, Green Deal, Green Industry, Green hydrogen, H2, Hydrogen, Innovation Fund, Low Carbon Hydrogen, Maritime, Net-zero, Recycling, Road transport, carbon capture and storage, carbon capture and utilisation, carbon neutral, clean energy, clean tech, clean technologies, climate change, demonstration, emission avoidance, emission savings, energy intensive industry, energy storage, energy transition, greenhouse gas, heavy industry, industry, low-carbon technologies, renewable energy, STEP-Cleantech</t>
+        </is>
+      </c>
       <c r="C87" s="22" t="n"/>
       <c r="D87" s="22" t="n"/>
       <c r="E87" s="22" t="n"/>
@@ -6587,7 +6355,7 @@
       </c>
       <c r="B88" s="21" t="inlineStr">
         <is>
-          <t>MEDIA — Margen izquierda con pasado industrial. Potencial reconversión.</t>
+          <t>MEDIA — Aplicable a Petronor/Repsol (Muskiz) y Puerto de Bilbao.</t>
         </is>
       </c>
       <c r="C88" s="22" t="n"/>
@@ -6603,7 +6371,7 @@
       </c>
       <c r="B89" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-2-PRIZE</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/INNOVFUND-2025-NZT-GENERAL-LSP</t>
         </is>
       </c>
       <c r="C89" s="22" t="n"/>
@@ -6614,7 +6382,7 @@
     <row r="91" ht="30" customHeight="1">
       <c r="A91" s="18" t="inlineStr">
         <is>
-          <t>FICHA 7: 02ea5f5c-3122-4e73-a32a-dfb5ff0f395c-CN</t>
+          <t>FICHA 7: HORIZON-CL5-2026-2-PRIZE</t>
         </is>
       </c>
       <c r="B91" s="19" t="n"/>
@@ -6639,7 +6407,7 @@
       <c r="E92" s="22" t="n"/>
       <c r="F92" s="22" t="n"/>
     </row>
-    <row r="93" ht="45" customHeight="1">
+    <row r="93" ht="20" customHeight="1">
       <c r="A93" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -6647,7 +6415,7 @@
       </c>
       <c r="B93" s="21" t="inlineStr">
         <is>
-          <t>Analysis of target setting for a selection of common indicators used under the European Regional Development Fund, Cohesion Fund and Just Transition Fund in 2021-2027</t>
+          <t>Renewable energy technology (RET) solutions in energy communities</t>
         </is>
       </c>
       <c r="C93" s="22" t="n"/>
@@ -6663,7 +6431,7 @@
       </c>
       <c r="B94" s="21" t="inlineStr">
         <is>
-          <t>02ea5f5c-3122-4e73-a32a-dfb5ff0f395c-CN</t>
+          <t>HORIZON-CL5-2026-2-PRIZE</t>
         </is>
       </c>
       <c r="C94" s="22" t="n"/>
@@ -6677,7 +6445,11 @@
           <t>Programa</t>
         </is>
       </c>
-      <c r="B95" s="21" t="inlineStr"/>
+      <c r="B95" s="21" t="inlineStr">
+        <is>
+          <t>Horizon Europe</t>
+        </is>
+      </c>
       <c r="C95" s="22" t="n"/>
       <c r="D95" s="22" t="n"/>
       <c r="E95" s="22" t="n"/>
@@ -6707,7 +6479,7 @@
       </c>
       <c r="B97" s="21" t="inlineStr">
         <is>
-          <t>30/03/2026</t>
+          <t>25/06/2026</t>
         </is>
       </c>
       <c r="C97" s="22" t="n"/>
@@ -6739,7 +6511,7 @@
       </c>
       <c r="B99" s="21" t="inlineStr">
         <is>
-          <t>No disponible</t>
+          <t>Recognition Prize</t>
         </is>
       </c>
       <c r="C99" s="22" t="n"/>
@@ -6755,7 +6527,7 @@
       </c>
       <c r="B100" s="21" t="inlineStr">
         <is>
-          <t>EC-REGIO/2026/OP/0013</t>
+          <t>HORIZON-CL5-2026-2-PRIZE</t>
         </is>
       </c>
       <c r="C100" s="22" t="n"/>
@@ -6771,7 +6543,7 @@
       </c>
       <c r="B101" s="21" t="inlineStr">
         <is>
-          <t>Analysis of target setting for a selection of common indicators used under the European Regional Development Fund, Cohesion Fund and Just Transition Fund in 2021-2027</t>
+          <t>Specific Challenge:Individual energy communities encounter different challenges, such as developing a successful governance structure that is sufficiently inclusive and involves different types of actors, carrying out an effective business model and embedding activities within the structure and management of the European Commission to territorial regional and/or local plans (e.g., Just Transition Plans, Climate City Contracts, etc.). By rewarding Energy Communities’ innovative governance structure and management of a RET, the prize aims to inspire other Energy Communities to improve their oper</t>
         </is>
       </c>
       <c r="C101" s="22" t="n"/>
@@ -6815,7 +6587,7 @@
       </c>
       <c r="B104" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/02ea5f5c-3122-4e73-a32a-dfb5ff0f395c-CN</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-2-PRIZE</t>
         </is>
       </c>
       <c r="C104" s="22" t="n"/>
@@ -16938,7 +16710,7 @@
     <row r="811" ht="30" customHeight="1">
       <c r="A811" s="18" t="inlineStr">
         <is>
-          <t>FICHA 55: EUS-97765</t>
+          <t>FICHA 55: EUS-47030</t>
         </is>
       </c>
       <c r="B811" s="19" t="n"/>
@@ -16971,7 +16743,7 @@
       </c>
       <c r="B813" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
+          <t>Servicios de transporte y manipulación de obras de arte para una exposición en el Museo de Bellas Artes de Bilbao</t>
         </is>
       </c>
       <c r="C813" s="22" t="n"/>
@@ -16987,7 +16759,7 @@
       </c>
       <c r="B814" s="21" t="inlineStr">
         <is>
-          <t>EUS-97765</t>
+          <t>EUS-47030</t>
         </is>
       </c>
       <c r="C814" s="22" t="n"/>
@@ -17063,7 +16835,7 @@
       </c>
       <c r="B819" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C819" s="22" t="n"/>
@@ -17121,9 +16893,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B823" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ALTA — </t>
+      <c r="B823" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MUY ALTA — </t>
         </is>
       </c>
       <c r="C823" s="22" t="n"/>
@@ -17139,7 +16911,7 @@
       </c>
       <c r="B824" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-con-incremento-de-capacidad-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicios-transporte-y-manipulacion-obras-arte-exposicion-museo-bellas-artes-bilbao/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C824" s="22" t="n"/>
@@ -17150,7 +16922,7 @@
     <row r="826" ht="30" customHeight="1">
       <c r="A826" s="18" t="inlineStr">
         <is>
-          <t>FICHA 56: EUS-23570</t>
+          <t>FICHA 56: EUS-15017</t>
         </is>
       </c>
       <c r="B826" s="19" t="n"/>
@@ -17183,7 +16955,7 @@
       </c>
       <c r="B828" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a la gestión sostenible de los recursos pesqueros 2026</t>
+          <t>Mantenimiento de las instalaciones de climatización de la oficina de Bilbao</t>
         </is>
       </c>
       <c r="C828" s="22" t="n"/>
@@ -17199,7 +16971,7 @@
       </c>
       <c r="B829" s="21" t="inlineStr">
         <is>
-          <t>EUS-23570</t>
+          <t>EUS-15017</t>
         </is>
       </c>
       <c r="C829" s="22" t="n"/>
@@ -17275,7 +17047,7 @@
       </c>
       <c r="B834" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C834" s="22" t="n"/>
@@ -17333,9 +17105,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B838" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ALTA — </t>
+      <c r="B838" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MUY ALTA — </t>
         </is>
       </c>
       <c r="C838" s="22" t="n"/>
@@ -17351,7 +17123,7 @@
       </c>
       <c r="B839" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-gestion-sostenible-de-los-recursos-pesqueros-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/mantenimiento-instalaciones-climatizacion-oficina-bilbao/expjaso698301/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C839" s="22" t="n"/>
@@ -17362,7 +17134,7 @@
     <row r="841" ht="30" customHeight="1">
       <c r="A841" s="18" t="inlineStr">
         <is>
-          <t>FICHA 57: EUS-92691</t>
+          <t>FICHA 57: EUS-25647</t>
         </is>
       </c>
       <c r="B841" s="19" t="n"/>
@@ -17395,7 +17167,7 @@
       </c>
       <c r="B843" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a la recogida de residuos con la participación de los pescadores en el mar y las playas 2026</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
         </is>
       </c>
       <c r="C843" s="22" t="n"/>
@@ -17411,7 +17183,7 @@
       </c>
       <c r="B844" s="21" t="inlineStr">
         <is>
-          <t>EUS-92691</t>
+          <t>EUS-25647</t>
         </is>
       </c>
       <c r="C844" s="22" t="n"/>
@@ -17555,7 +17327,7 @@
       <c r="E853" s="22" t="n"/>
       <c r="F853" s="22" t="n"/>
     </row>
-    <row r="854" ht="20" customHeight="1">
+    <row r="854" ht="45" customHeight="1">
       <c r="A854" s="20" t="inlineStr">
         <is>
           <t>Enlace al portal</t>
@@ -17563,7 +17335,7 @@
       </c>
       <c r="B854" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/fempa-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-con-incremento-de-capacidad-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C854" s="22" t="n"/>
@@ -17574,7 +17346,7 @@
     <row r="856" ht="30" customHeight="1">
       <c r="A856" s="18" t="inlineStr">
         <is>
-          <t>FICHA 58: EUS-34245</t>
+          <t>FICHA 58: EUS-39134</t>
         </is>
       </c>
       <c r="B856" s="19" t="n"/>
@@ -17599,7 +17371,7 @@
       <c r="E857" s="22" t="n"/>
       <c r="F857" s="22" t="n"/>
     </row>
-    <row r="858" ht="45" customHeight="1">
+    <row r="858" ht="20" customHeight="1">
       <c r="A858" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -17607,7 +17379,7 @@
       </c>
       <c r="B858" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático sin incremento de capacidad 2026</t>
+          <t>Ayudas a la gestión sostenible de los recursos pesqueros 2026</t>
         </is>
       </c>
       <c r="C858" s="22" t="n"/>
@@ -17623,7 +17395,7 @@
       </c>
       <c r="B859" s="21" t="inlineStr">
         <is>
-          <t>EUS-34245</t>
+          <t>EUS-39134</t>
         </is>
       </c>
       <c r="C859" s="22" t="n"/>
@@ -17775,7 +17547,7 @@
       </c>
       <c r="B869" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-sin-incremento-de-capacidad-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-gestion-sostenible-de-los-recursos-pesqueros-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C869" s="22" t="n"/>
@@ -17786,7 +17558,7 @@
     <row r="871" ht="30" customHeight="1">
       <c r="A871" s="18" t="inlineStr">
         <is>
-          <t>FICHA 59: EUS-17774</t>
+          <t>FICHA 59: EUS-85153</t>
         </is>
       </c>
       <c r="B871" s="19" t="n"/>
@@ -17819,7 +17591,7 @@
       </c>
       <c r="B873" s="21" t="inlineStr">
         <is>
-          <t>Servicio de oficina técnica para la mejora del sistema de prevención y gestión de residuos de competencia local de Bizkaia</t>
+          <t>Ayudas a la recogida de residuos con la participación de los pescadores en el mar y las playas 2026</t>
         </is>
       </c>
       <c r="C873" s="22" t="n"/>
@@ -17835,7 +17607,7 @@
       </c>
       <c r="B874" s="21" t="inlineStr">
         <is>
-          <t>EUS-17774</t>
+          <t>EUS-85153</t>
         </is>
       </c>
       <c r="C874" s="22" t="n"/>
@@ -17911,7 +17683,7 @@
       </c>
       <c r="B879" s="21" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C879" s="22" t="n"/>
@@ -17979,7 +17751,7 @@
       <c r="E883" s="22" t="n"/>
       <c r="F883" s="22" t="n"/>
     </row>
-    <row r="884" ht="45" customHeight="1">
+    <row r="884" ht="20" customHeight="1">
       <c r="A884" s="20" t="inlineStr">
         <is>
           <t>Enlace al portal</t>
@@ -17987,7 +17759,7 @@
       </c>
       <c r="B884" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-oficina-tecnica-mejora-del-sistema-prevencion-y-gestion-residuos-competencia-local-bizkaia/expgebizkaia3387395/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/fempa-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C884" s="22" t="n"/>
@@ -17998,7 +17770,7 @@
     <row r="886" ht="30" customHeight="1">
       <c r="A886" s="18" t="inlineStr">
         <is>
-          <t>FICHA 60: EUS-22731</t>
+          <t>FICHA 60: EUS-21937</t>
         </is>
       </c>
       <c r="B886" s="19" t="n"/>
@@ -18023,7 +17795,7 @@
       <c r="E887" s="22" t="n"/>
       <c r="F887" s="22" t="n"/>
     </row>
-    <row r="888" ht="20" customHeight="1">
+    <row r="888" ht="45" customHeight="1">
       <c r="A888" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -18031,7 +17803,7 @@
       </c>
       <c r="B888" s="21" t="inlineStr">
         <is>
-          <t>Redacción de un Plan de prevención y gestión de residuos</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio climático sin incremento de capacidad 2026</t>
         </is>
       </c>
       <c r="C888" s="22" t="n"/>
@@ -18047,7 +17819,7 @@
       </c>
       <c r="B889" s="21" t="inlineStr">
         <is>
-          <t>EUS-22731</t>
+          <t>EUS-21937</t>
         </is>
       </c>
       <c r="C889" s="22" t="n"/>
@@ -18123,7 +17895,7 @@
       </c>
       <c r="B894" s="21" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C894" s="22" t="n"/>
@@ -18199,7 +17971,7 @@
       </c>
       <c r="B899" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/redaccion-plan-prevencion-y-gestion-residuos/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-sin-incremento-de-capacidad-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C899" s="22" t="n"/>
@@ -18210,7 +17982,7 @@
     <row r="901" ht="30" customHeight="1">
       <c r="A901" s="18" t="inlineStr">
         <is>
-          <t>FICHA 61: EUS-32199</t>
+          <t>FICHA 61: EUS-02512</t>
         </is>
       </c>
       <c r="B901" s="19" t="n"/>
@@ -18243,7 +18015,7 @@
       </c>
       <c r="B903" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
+          <t>Servicio de transporte y gestión de los residuos procedentes de corte de orilla de playas</t>
         </is>
       </c>
       <c r="C903" s="22" t="n"/>
@@ -18259,7 +18031,7 @@
       </c>
       <c r="B904" s="21" t="inlineStr">
         <is>
-          <t>EUS-32199</t>
+          <t>EUS-02512</t>
         </is>
       </c>
       <c r="C904" s="22" t="n"/>
@@ -18335,7 +18107,7 @@
       </c>
       <c r="B909" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C909" s="22" t="n"/>
@@ -18393,9 +18165,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B913" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
+      <c r="B913" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALTA — </t>
         </is>
       </c>
       <c r="C913" s="22" t="n"/>
@@ -18411,7 +18183,7 @@
       </c>
       <c r="B914" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-contribucion-de-la-acuicultura-al-buen-estado-ambiental-y-prestacion-de-servicios-ambientales-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-transporte-y-gestion-residuos-procedentes-corte-orilla-playas/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C914" s="22" t="n"/>
@@ -18422,7 +18194,7 @@
     <row r="916" ht="30" customHeight="1">
       <c r="A916" s="18" t="inlineStr">
         <is>
-          <t>FICHA 62: EUS-89864</t>
+          <t>FICHA 62: EUS-91129</t>
         </is>
       </c>
       <c r="B916" s="19" t="n"/>
@@ -18447,7 +18219,7 @@
       <c r="E917" s="22" t="n"/>
       <c r="F917" s="22" t="n"/>
     </row>
-    <row r="918" ht="20" customHeight="1">
+    <row r="918" ht="45" customHeight="1">
       <c r="A918" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -18455,7 +18227,7 @@
       </c>
       <c r="B918" s="21" t="inlineStr">
         <is>
-          <t>Ayudas al valor añadido, economía circular y seguridad alimentaria 2026</t>
+          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
         </is>
       </c>
       <c r="C918" s="22" t="n"/>
@@ -18471,7 +18243,7 @@
       </c>
       <c r="B919" s="21" t="inlineStr">
         <is>
-          <t>EUS-89864</t>
+          <t>EUS-91129</t>
         </is>
       </c>
       <c r="C919" s="22" t="n"/>
@@ -18623,7 +18395,7 @@
       </c>
       <c r="B929" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-valor-anadido-economia-circular-y-seguridad-alimentaria-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-contribucion-de-la-acuicultura-al-buen-estado-ambiental-y-prestacion-de-servicios-ambientales-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C929" s="22" t="n"/>
@@ -18634,7 +18406,7 @@
     <row r="931" ht="30" customHeight="1">
       <c r="A931" s="18" t="inlineStr">
         <is>
-          <t>FICHA 63: EUS-92385</t>
+          <t>FICHA 63: EUS-46360</t>
         </is>
       </c>
       <c r="B931" s="19" t="n"/>
@@ -18659,7 +18431,7 @@
       <c r="E932" s="22" t="n"/>
       <c r="F932" s="22" t="n"/>
     </row>
-    <row r="933" ht="45" customHeight="1">
+    <row r="933" ht="20" customHeight="1">
       <c r="A933" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -18667,7 +18439,7 @@
       </c>
       <c r="B933" s="21" t="inlineStr">
         <is>
-          <t>Vino: el Gobierno Vasco volverá a convocar este mes las ayudas al arranque o cosecha en verde del viñedo, que van a contemplar como estructurales tras reformar la UE jurídicamente su Intervención Sect</t>
+          <t>Ayudas al valor añadido, economía circular y seguridad alimentaria 2026</t>
         </is>
       </c>
       <c r="C933" s="22" t="n"/>
@@ -18683,7 +18455,7 @@
       </c>
       <c r="B934" s="21" t="inlineStr">
         <is>
-          <t>EUS-92385</t>
+          <t>EUS-46360</t>
         </is>
       </c>
       <c r="C934" s="22" t="n"/>
@@ -18835,7 +18607,7 @@
       </c>
       <c r="B944" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260302berdezerauztekoak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-valor-anadido-economia-circular-y-seguridad-alimentaria-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C944" s="22" t="n"/>
@@ -18846,7 +18618,7 @@
     <row r="946" ht="30" customHeight="1">
       <c r="A946" s="18" t="inlineStr">
         <is>
-          <t>FICHA 64: EUS-45123</t>
+          <t>FICHA 64: EUS-14446</t>
         </is>
       </c>
       <c r="B946" s="19" t="n"/>
@@ -18879,7 +18651,7 @@
       </c>
       <c r="B948" s="21" t="inlineStr">
         <is>
-          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de aceleración de proyectos, a localidades de menos de 20.000 habitantes son objeto de convocatoria abierta hasta el 17.03.26. Transformacione</t>
+          <t>Vino: el Gobierno Vasco volverá a convocar este mes las ayudas al arranque o cosecha en verde del viñedo, que van a contemplar como estructurales tras reformar la UE jurídicamente su Intervención Sect</t>
         </is>
       </c>
       <c r="C948" s="22" t="n"/>
@@ -18895,7 +18667,7 @@
       </c>
       <c r="B949" s="21" t="inlineStr">
         <is>
-          <t>EUS-45123</t>
+          <t>EUS-14446</t>
         </is>
       </c>
       <c r="C949" s="22" t="n"/>
@@ -19047,7 +18819,7 @@
       </c>
       <c r="B959" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260317neboostasariak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260302berdezerauztekoak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C959" s="22" t="n"/>
@@ -19058,7 +18830,7 @@
     <row r="961" ht="30" customHeight="1">
       <c r="A961" s="18" t="inlineStr">
         <is>
-          <t>FICHA 65: EUS-63814</t>
+          <t>FICHA 65: EUS-75188</t>
         </is>
       </c>
       <c r="B961" s="19" t="n"/>
@@ -19091,7 +18863,7 @@
       </c>
       <c r="B963" s="21" t="inlineStr">
         <is>
-          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para consorcios internacionales de I+D+i. Jornada del Gobierno Vasco y con Enterprise Europe Network y otros socios. Digitalización, dispositivos,</t>
+          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de aceleración de proyectos, a localidades de menos de 20.000 habitantes son objeto de convocatoria abierta hasta el 17.03.26. Transformacione</t>
         </is>
       </c>
       <c r="C963" s="22" t="n"/>
@@ -19107,7 +18879,7 @@
       </c>
       <c r="B964" s="21" t="inlineStr">
         <is>
-          <t>EUS-63814</t>
+          <t>EUS-75188</t>
         </is>
       </c>
       <c r="C964" s="22" t="n"/>
@@ -19259,7 +19031,7 @@
       </c>
       <c r="B974" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260303eicihihorizon/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260317neboostasariak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C974" s="22" t="n"/>
@@ -19270,7 +19042,7 @@
     <row r="976" ht="30" customHeight="1">
       <c r="A976" s="18" t="inlineStr">
         <is>
-          <t>FICHA 66: EUS-82158</t>
+          <t>FICHA 66: EUS-45072</t>
         </is>
       </c>
       <c r="B976" s="19" t="n"/>
@@ -19303,7 +19075,7 @@
       </c>
       <c r="B978" s="21" t="inlineStr">
         <is>
-          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinancia convocatorias de ayudas de las Diputaciones a explotaciones con limitaciones o desfavorecidas, y a compromisos medioambientales, climátic</t>
+          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para consorcios internacionales de I+D+i. Jornada del Gobierno Vasco y con Enterprise Europe Network y otros socios. Digitalización, dispositivos,</t>
         </is>
       </c>
       <c r="C978" s="22" t="n"/>
@@ -19319,7 +19091,7 @@
       </c>
       <c r="B979" s="21" t="inlineStr">
         <is>
-          <t>EUS-82158</t>
+          <t>EUS-45072</t>
         </is>
       </c>
       <c r="C979" s="22" t="n"/>
@@ -19471,7 +19243,7 @@
       </c>
       <c r="B989" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/lgenfnpbgfa260218/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260303eicihihorizon/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C989" s="22" t="n"/>
@@ -19482,7 +19254,7 @@
     <row r="991" ht="30" customHeight="1">
       <c r="A991" s="18" t="inlineStr">
         <is>
-          <t>FICHA 67: EUS-92414</t>
+          <t>FICHA 67: EUS-36943</t>
         </is>
       </c>
       <c r="B991" s="19" t="n"/>
@@ -19515,7 +19287,7 @@
       </c>
       <c r="B993" s="21" t="inlineStr">
         <is>
-          <t>Digital Europe, Horizon (programas de la UE). Apoyos para consorcios interestatales de I+D+i. IA, robótica, cuántica, computación, ciberseguridad, electrónica, fotónica, TICs e internet avanzadas, esp</t>
+          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinancia convocatorias de ayudas de las Diputaciones a explotaciones con limitaciones o desfavorecidas, y a compromisos medioambientales, climátic</t>
         </is>
       </c>
       <c r="C993" s="22" t="n"/>
@@ -19531,7 +19303,7 @@
       </c>
       <c r="B994" s="21" t="inlineStr">
         <is>
-          <t>EUS-92414</t>
+          <t>EUS-36943</t>
         </is>
       </c>
       <c r="C994" s="22" t="n"/>
@@ -19683,7 +19455,7 @@
       </c>
       <c r="B1004" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260304digitalhorizoneen/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/lgenfnpbgfa260218/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1004" s="22" t="n"/>
@@ -19694,7 +19466,7 @@
     <row r="1006" ht="30" customHeight="1">
       <c r="A1006" s="18" t="inlineStr">
         <is>
-          <t>FICHA 68: EUS-62683</t>
+          <t>FICHA 68: EUS-80876</t>
         </is>
       </c>
       <c r="B1006" s="19" t="n"/>
@@ -19727,7 +19499,7 @@
       </c>
       <c r="B1008" s="21" t="inlineStr">
         <is>
-          <t>Política Agraria Común de la UE de 2026, y sus ayudas abiertas hasta el 30.4.26: el pilar 1, con el Fondo Europeo Agrícola de Garantía Agraria FEAGA, aborda sostenibilidad de renta, ayuda redistributi</t>
+          <t>Digital Europe, Horizon (programas de la UE). Apoyos para consorcios interestatales de I+D+i. IA, robótica, cuántica, computación, ciberseguridad, electrónica, fotónica, TICs e internet avanzadas, esp</t>
         </is>
       </c>
       <c r="C1008" s="22" t="n"/>
@@ -19743,7 +19515,7 @@
       </c>
       <c r="B1009" s="21" t="inlineStr">
         <is>
-          <t>EUS-62683</t>
+          <t>EUS-80876</t>
         </is>
       </c>
       <c r="C1009" s="22" t="n"/>
@@ -19895,7 +19667,7 @@
       </c>
       <c r="B1019" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260216npblaguntzairekiak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260304digitalhorizoneen/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1019" s="22" t="n"/>
@@ -19906,7 +19678,7 @@
     <row r="1021" ht="30" customHeight="1">
       <c r="A1021" s="18" t="inlineStr">
         <is>
-          <t>FICHA 69: EUS-33389</t>
+          <t>FICHA 69: EUS-03523</t>
         </is>
       </c>
       <c r="B1021" s="19" t="n"/>
@@ -19939,7 +19711,7 @@
       </c>
       <c r="B1023" s="21" t="inlineStr">
         <is>
-          <t>Programa de impulso a las ciudades y territorios inteligentes para el fomento del desarrollo económico y productivo, que podrá ser cofinanciado por el Programa Plurirregional 2021-2027 del Fondo Europ</t>
+          <t>Política Agraria Común de la UE de 2026, y sus ayudas abiertas hasta el 30.4.26: el pilar 1, con el Fondo Europeo Agrícola de Garantía Agraria FEAGA, aborda sostenibilidad de renta, ayuda redistributi</t>
         </is>
       </c>
       <c r="C1023" s="22" t="n"/>
@@ -19955,7 +19727,7 @@
       </c>
       <c r="B1024" s="21" t="inlineStr">
         <is>
-          <t>EUS-33389</t>
+          <t>EUS-03523</t>
         </is>
       </c>
       <c r="C1024" s="22" t="n"/>
@@ -20107,7 +19879,7 @@
       </c>
       <c r="B1034" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260204smartcities/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260216npblaguntzairekiak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1034" s="22" t="n"/>
@@ -20118,7 +19890,7 @@
     <row r="1036" ht="30" customHeight="1">
       <c r="A1036" s="18" t="inlineStr">
         <is>
-          <t>FICHA 70: EUS-40042</t>
+          <t>FICHA 70: EUS-44113</t>
         </is>
       </c>
       <c r="B1036" s="19" t="n"/>
@@ -20151,7 +19923,7 @@
       </c>
       <c r="B1038" s="21" t="inlineStr">
         <is>
-          <t>Suministros y Servicios para la instalación de una red XGS-PON y electrónica de red en la nueva Sede de EITB Gasteiz y renovación de la infraestructura WLAN de EITB.</t>
+          <t>Programa de impulso a las ciudades y territorios inteligentes para el fomento del desarrollo económico y productivo, que podrá ser cofinanciado por el Programa Plurirregional 2021-2027 del Fondo Europ</t>
         </is>
       </c>
       <c r="C1038" s="22" t="n"/>
@@ -20167,7 +19939,7 @@
       </c>
       <c r="B1039" s="21" t="inlineStr">
         <is>
-          <t>EUS-40042</t>
+          <t>EUS-44113</t>
         </is>
       </c>
       <c r="C1039" s="22" t="n"/>
@@ -20243,7 +20015,7 @@
       </c>
       <c r="B1044" s="21" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C1044" s="22" t="n"/>
@@ -20319,7 +20091,7 @@
       </c>
       <c r="B1049" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministros-y-servicios-instalacion-red-xgs-pon-y-electronica-red-nueva-sede-eitb-gasteiz-y-renovacion-infraestructura-wlan-eitb/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260204smartcities/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1049" s="22" t="n"/>
@@ -20330,7 +20102,7 @@
     <row r="1051" ht="30" customHeight="1">
       <c r="A1051" s="18" t="inlineStr">
         <is>
-          <t>FICHA 71: EUS-25076</t>
+          <t>FICHA 71: EUS-71405</t>
         </is>
       </c>
       <c r="B1051" s="19" t="n"/>
@@ -20363,7 +20135,7 @@
       </c>
       <c r="B1053" s="21" t="inlineStr">
         <is>
-          <t>Realización del vuelo fotogramétrico digital multivista, escenas 3D y ortofotos verdaderas de 5cm de las localidades con más de 15.000 habitantes del País Vasco (2026)</t>
+          <t>Dirección facultativa de obra (dirección de obra, dirección de ejecución y coordinación de seguridad y salud) y ejecución del proyecto de la nueva cubierta exterior de Izarraizpe Ikastola</t>
         </is>
       </c>
       <c r="C1053" s="22" t="n"/>
@@ -20379,7 +20151,7 @@
       </c>
       <c r="B1054" s="21" t="inlineStr">
         <is>
-          <t>EUS-25076</t>
+          <t>EUS-71405</t>
         </is>
       </c>
       <c r="C1054" s="22" t="n"/>
@@ -20531,7 +20303,7 @@
       </c>
       <c r="B1064" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/realizacion-del-vuelo-fotogrametrico-digital-multivista-escenas-3d-y-ortofotos-verdaderas-5cm-localidades-mas-15-000-habitantes-del-pais-vasco-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/direccion-facultativa-obra-direccion-obra-direccion-ejecucion-y-coordinacion-seguridad-y-salud-y-ejecucion-del-proyecto-nueva-cubierta-exterior-izarraizpe-ikastola/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1064" s="22" t="n"/>
@@ -20542,7 +20314,7 @@
     <row r="1066" ht="30" customHeight="1">
       <c r="A1066" s="18" t="inlineStr">
         <is>
-          <t>FICHA 72: EUS-13379</t>
+          <t>FICHA 72: EUS-85319</t>
         </is>
       </c>
       <c r="B1066" s="19" t="n"/>
@@ -20575,7 +20347,7 @@
       </c>
       <c r="B1068" s="21" t="inlineStr">
         <is>
-          <t>Suministro para la ampliación de la infraestructura de los repositorios de Copias de Seguridad de EJIE</t>
+          <t>Licitación de la obra ?Adecuación del espacio público y ejecución de nuevas redes de pluviales y acometida de agua? en Mendiola (Álava).</t>
         </is>
       </c>
       <c r="C1068" s="22" t="n"/>
@@ -20591,7 +20363,7 @@
       </c>
       <c r="B1069" s="21" t="inlineStr">
         <is>
-          <t>EUS-13379</t>
+          <t>EUS-85319</t>
         </is>
       </c>
       <c r="C1069" s="22" t="n"/>
@@ -20743,7 +20515,7 @@
       </c>
       <c r="B1079" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-ampliacion-infraestructura-repositorios-copias-seguridad-ejie/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/licitacion-obra-adecuacion-del-espacio-publico-y-ejecucion-nuevas-redes-pluviales-y-acometida-agua-mendiola-alava/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1079" s="22" t="n"/>
@@ -20754,7 +20526,7 @@
     <row r="1081" ht="30" customHeight="1">
       <c r="A1081" s="18" t="inlineStr">
         <is>
-          <t>FICHA 73: EUS-89192</t>
+          <t>FICHA 73: EUS-57006</t>
         </is>
       </c>
       <c r="B1081" s="19" t="n"/>
@@ -20787,7 +20559,7 @@
       </c>
       <c r="B1083" s="21" t="inlineStr">
         <is>
-          <t>Suministro e instalación de fuente de agua fría para consumo de usuarios en zona de spa del polideportivo orbea</t>
+          <t>Suministro de un sistema de Seguridad e Información Turística en el edificio Cocheras de la Finca Munoa en el marco del Plan Europeo de Recuperación, Transformación y Resiliencia, financiado por la Un</t>
         </is>
       </c>
       <c r="C1083" s="22" t="n"/>
@@ -20803,7 +20575,7 @@
       </c>
       <c r="B1084" s="21" t="inlineStr">
         <is>
-          <t>EUS-89192</t>
+          <t>EUS-57006</t>
         </is>
       </c>
       <c r="C1084" s="22" t="n"/>
@@ -20955,7 +20727,7 @@
       </c>
       <c r="B1094" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-e-instalacion-fuente-agua-fria-consumo-usuarios-zona-spa-del-polideportivo-orbea/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-sistema-seguridad-e-informacion-turistica-edificio-cocheras-finca-munoa-marco-del-plan-europeo-recuperacion-transformacion-y-resiliencia-financiado-union-europea-next-generation-eu/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1094" s="22" t="n"/>
@@ -20963,856 +20735,8 @@
       <c r="E1094" s="22" t="n"/>
       <c r="F1094" s="22" t="n"/>
     </row>
-    <row r="1096" ht="30" customHeight="1">
-      <c r="A1096" s="18" t="inlineStr">
-        <is>
-          <t>FICHA 74: EUS-06858</t>
-        </is>
-      </c>
-      <c r="B1096" s="19" t="n"/>
-      <c r="C1096" s="19" t="n"/>
-      <c r="D1096" s="19" t="n"/>
-      <c r="E1096" s="19" t="n"/>
-      <c r="F1096" s="19" t="n"/>
-    </row>
-    <row r="1097" ht="20" customHeight="1">
-      <c r="A1097" s="20" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-      <c r="B1097" s="21" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
-        </is>
-      </c>
-      <c r="C1097" s="22" t="n"/>
-      <c r="D1097" s="22" t="n"/>
-      <c r="E1097" s="22" t="n"/>
-      <c r="F1097" s="22" t="n"/>
-    </row>
-    <row r="1098" ht="20" customHeight="1">
-      <c r="A1098" s="20" t="inlineStr">
-        <is>
-          <t>Titulo</t>
-        </is>
-      </c>
-      <c r="B1098" s="21" t="inlineStr">
-        <is>
-          <t>Equipamiento de muebles en vivienda municipal</t>
-        </is>
-      </c>
-      <c r="C1098" s="22" t="n"/>
-      <c r="D1098" s="22" t="n"/>
-      <c r="E1098" s="22" t="n"/>
-      <c r="F1098" s="22" t="n"/>
-    </row>
-    <row r="1099" ht="20" customHeight="1">
-      <c r="A1099" s="20" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1099" s="21" t="inlineStr">
-        <is>
-          <t>EUS-06858</t>
-        </is>
-      </c>
-      <c r="C1099" s="22" t="n"/>
-      <c r="D1099" s="22" t="n"/>
-      <c r="E1099" s="22" t="n"/>
-      <c r="F1099" s="22" t="n"/>
-    </row>
-    <row r="1100" ht="20" customHeight="1">
-      <c r="A1100" s="20" t="inlineStr">
-        <is>
-          <t>Programa</t>
-        </is>
-      </c>
-      <c r="B1100" s="21" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="C1100" s="22" t="n"/>
-      <c r="D1100" s="22" t="n"/>
-      <c r="E1100" s="22" t="n"/>
-      <c r="F1100" s="22" t="n"/>
-    </row>
-    <row r="1101" ht="20" customHeight="1">
-      <c r="A1101" s="20" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="B1101" s="21" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C1101" s="22" t="n"/>
-      <c r="D1101" s="22" t="n"/>
-      <c r="E1101" s="22" t="n"/>
-      <c r="F1101" s="22" t="n"/>
-    </row>
-    <row r="1102" ht="20" customHeight="1">
-      <c r="A1102" s="20" t="inlineStr">
-        <is>
-          <t>Deadline</t>
-        </is>
-      </c>
-      <c r="B1102" s="21" t="inlineStr"/>
-      <c r="C1102" s="22" t="n"/>
-      <c r="D1102" s="22" t="n"/>
-      <c r="E1102" s="22" t="n"/>
-      <c r="F1102" s="22" t="n"/>
-    </row>
-    <row r="1103" ht="20" customHeight="1">
-      <c r="A1103" s="20" t="inlineStr">
-        <is>
-          <t>Presupuesto (EUR)</t>
-        </is>
-      </c>
-      <c r="B1103" s="21" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="C1103" s="22" t="n"/>
-      <c r="D1103" s="22" t="n"/>
-      <c r="E1103" s="22" t="n"/>
-      <c r="F1103" s="22" t="n"/>
-    </row>
-    <row r="1104" ht="20" customHeight="1">
-      <c r="A1104" s="20" t="inlineStr">
-        <is>
-          <t>Tipo de Accion</t>
-        </is>
-      </c>
-      <c r="B1104" s="21" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="C1104" s="22" t="n"/>
-      <c r="D1104" s="22" t="n"/>
-      <c r="E1104" s="22" t="n"/>
-      <c r="F1104" s="22" t="n"/>
-    </row>
-    <row r="1105" ht="20" customHeight="1">
-      <c r="A1105" s="20" t="inlineStr">
-        <is>
-          <t>Call ID</t>
-        </is>
-      </c>
-      <c r="B1105" s="21" t="inlineStr"/>
-      <c r="C1105" s="22" t="n"/>
-      <c r="D1105" s="22" t="n"/>
-      <c r="E1105" s="22" t="n"/>
-      <c r="F1105" s="22" t="n"/>
-    </row>
-    <row r="1106" ht="20" customHeight="1">
-      <c r="A1106" s="20" t="inlineStr">
-        <is>
-          <t>Descripcion</t>
-        </is>
-      </c>
-      <c r="B1106" s="21" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="C1106" s="22" t="n"/>
-      <c r="D1106" s="22" t="n"/>
-      <c r="E1106" s="22" t="n"/>
-      <c r="F1106" s="22" t="n"/>
-    </row>
-    <row r="1107" ht="20" customHeight="1">
-      <c r="A1107" s="20" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-      <c r="B1107" s="21" t="inlineStr">
-        <is>
-          <t>energia</t>
-        </is>
-      </c>
-      <c r="C1107" s="22" t="n"/>
-      <c r="D1107" s="22" t="n"/>
-      <c r="E1107" s="22" t="n"/>
-      <c r="F1107" s="22" t="n"/>
-    </row>
-    <row r="1108" ht="20" customHeight="1">
-      <c r="A1108" s="20" t="inlineStr">
-        <is>
-          <t>Relevancia Bilbao</t>
-        </is>
-      </c>
-      <c r="B1108" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
-        </is>
-      </c>
-      <c r="C1108" s="22" t="n"/>
-      <c r="D1108" s="22" t="n"/>
-      <c r="E1108" s="22" t="n"/>
-      <c r="F1108" s="22" t="n"/>
-    </row>
-    <row r="1109" ht="45" customHeight="1">
-      <c r="A1109" s="20" t="inlineStr">
-        <is>
-          <t>Enlace al portal</t>
-        </is>
-      </c>
-      <c r="B1109" s="24" t="inlineStr">
-        <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/equipamiento-muebles-vivienda-municipal/expamorebieta202603244516/web01-tramite/es/</t>
-        </is>
-      </c>
-      <c r="C1109" s="22" t="n"/>
-      <c r="D1109" s="22" t="n"/>
-      <c r="E1109" s="22" t="n"/>
-      <c r="F1109" s="22" t="n"/>
-    </row>
-    <row r="1111" ht="30" customHeight="1">
-      <c r="A1111" s="18" t="inlineStr">
-        <is>
-          <t>FICHA 75: EUS-68952</t>
-        </is>
-      </c>
-      <c r="B1111" s="19" t="n"/>
-      <c r="C1111" s="19" t="n"/>
-      <c r="D1111" s="19" t="n"/>
-      <c r="E1111" s="19" t="n"/>
-      <c r="F1111" s="19" t="n"/>
-    </row>
-    <row r="1112" ht="20" customHeight="1">
-      <c r="A1112" s="20" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-      <c r="B1112" s="21" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
-        </is>
-      </c>
-      <c r="C1112" s="22" t="n"/>
-      <c r="D1112" s="22" t="n"/>
-      <c r="E1112" s="22" t="n"/>
-      <c r="F1112" s="22" t="n"/>
-    </row>
-    <row r="1113" ht="45" customHeight="1">
-      <c r="A1113" s="20" t="inlineStr">
-        <is>
-          <t>Titulo</t>
-        </is>
-      </c>
-      <c r="B1113" s="21" t="inlineStr">
-        <is>
-          <t>Servicio de limpieza, DDD y legionella de edificios municipales respetuosos con entorno de Muskiz</t>
-        </is>
-      </c>
-      <c r="C1113" s="22" t="n"/>
-      <c r="D1113" s="22" t="n"/>
-      <c r="E1113" s="22" t="n"/>
-      <c r="F1113" s="22" t="n"/>
-    </row>
-    <row r="1114" ht="20" customHeight="1">
-      <c r="A1114" s="20" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1114" s="21" t="inlineStr">
-        <is>
-          <t>EUS-68952</t>
-        </is>
-      </c>
-      <c r="C1114" s="22" t="n"/>
-      <c r="D1114" s="22" t="n"/>
-      <c r="E1114" s="22" t="n"/>
-      <c r="F1114" s="22" t="n"/>
-    </row>
-    <row r="1115" ht="20" customHeight="1">
-      <c r="A1115" s="20" t="inlineStr">
-        <is>
-          <t>Programa</t>
-        </is>
-      </c>
-      <c r="B1115" s="21" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="C1115" s="22" t="n"/>
-      <c r="D1115" s="22" t="n"/>
-      <c r="E1115" s="22" t="n"/>
-      <c r="F1115" s="22" t="n"/>
-    </row>
-    <row r="1116" ht="20" customHeight="1">
-      <c r="A1116" s="20" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="B1116" s="21" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C1116" s="22" t="n"/>
-      <c r="D1116" s="22" t="n"/>
-      <c r="E1116" s="22" t="n"/>
-      <c r="F1116" s="22" t="n"/>
-    </row>
-    <row r="1117" ht="20" customHeight="1">
-      <c r="A1117" s="20" t="inlineStr">
-        <is>
-          <t>Deadline</t>
-        </is>
-      </c>
-      <c r="B1117" s="21" t="inlineStr"/>
-      <c r="C1117" s="22" t="n"/>
-      <c r="D1117" s="22" t="n"/>
-      <c r="E1117" s="22" t="n"/>
-      <c r="F1117" s="22" t="n"/>
-    </row>
-    <row r="1118" ht="20" customHeight="1">
-      <c r="A1118" s="20" t="inlineStr">
-        <is>
-          <t>Presupuesto (EUR)</t>
-        </is>
-      </c>
-      <c r="B1118" s="21" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="C1118" s="22" t="n"/>
-      <c r="D1118" s="22" t="n"/>
-      <c r="E1118" s="22" t="n"/>
-      <c r="F1118" s="22" t="n"/>
-    </row>
-    <row r="1119" ht="20" customHeight="1">
-      <c r="A1119" s="20" t="inlineStr">
-        <is>
-          <t>Tipo de Accion</t>
-        </is>
-      </c>
-      <c r="B1119" s="21" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="C1119" s="22" t="n"/>
-      <c r="D1119" s="22" t="n"/>
-      <c r="E1119" s="22" t="n"/>
-      <c r="F1119" s="22" t="n"/>
-    </row>
-    <row r="1120" ht="20" customHeight="1">
-      <c r="A1120" s="20" t="inlineStr">
-        <is>
-          <t>Call ID</t>
-        </is>
-      </c>
-      <c r="B1120" s="21" t="inlineStr"/>
-      <c r="C1120" s="22" t="n"/>
-      <c r="D1120" s="22" t="n"/>
-      <c r="E1120" s="22" t="n"/>
-      <c r="F1120" s="22" t="n"/>
-    </row>
-    <row r="1121" ht="20" customHeight="1">
-      <c r="A1121" s="20" t="inlineStr">
-        <is>
-          <t>Descripcion</t>
-        </is>
-      </c>
-      <c r="B1121" s="21" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="C1121" s="22" t="n"/>
-      <c r="D1121" s="22" t="n"/>
-      <c r="E1121" s="22" t="n"/>
-      <c r="F1121" s="22" t="n"/>
-    </row>
-    <row r="1122" ht="20" customHeight="1">
-      <c r="A1122" s="20" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-      <c r="B1122" s="21" t="inlineStr">
-        <is>
-          <t>energia</t>
-        </is>
-      </c>
-      <c r="C1122" s="22" t="n"/>
-      <c r="D1122" s="22" t="n"/>
-      <c r="E1122" s="22" t="n"/>
-      <c r="F1122" s="22" t="n"/>
-    </row>
-    <row r="1123" ht="20" customHeight="1">
-      <c r="A1123" s="20" t="inlineStr">
-        <is>
-          <t>Relevancia Bilbao</t>
-        </is>
-      </c>
-      <c r="B1123" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
-        </is>
-      </c>
-      <c r="C1123" s="22" t="n"/>
-      <c r="D1123" s="22" t="n"/>
-      <c r="E1123" s="22" t="n"/>
-      <c r="F1123" s="22" t="n"/>
-    </row>
-    <row r="1124" ht="45" customHeight="1">
-      <c r="A1124" s="20" t="inlineStr">
-        <is>
-          <t>Enlace al portal</t>
-        </is>
-      </c>
-      <c r="B1124" s="24" t="inlineStr">
-        <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-limpieza-ddd-y-legionella-edificios-municipales-respetuosos-entorno-muskiz/web01-tramite/es/</t>
-        </is>
-      </c>
-      <c r="C1124" s="22" t="n"/>
-      <c r="D1124" s="22" t="n"/>
-      <c r="E1124" s="22" t="n"/>
-      <c r="F1124" s="22" t="n"/>
-    </row>
-    <row r="1126" ht="30" customHeight="1">
-      <c r="A1126" s="18" t="inlineStr">
-        <is>
-          <t>FICHA 76: EUS-87256</t>
-        </is>
-      </c>
-      <c r="B1126" s="19" t="n"/>
-      <c r="C1126" s="19" t="n"/>
-      <c r="D1126" s="19" t="n"/>
-      <c r="E1126" s="19" t="n"/>
-      <c r="F1126" s="19" t="n"/>
-    </row>
-    <row r="1127" ht="20" customHeight="1">
-      <c r="A1127" s="20" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-      <c r="B1127" s="21" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
-        </is>
-      </c>
-      <c r="C1127" s="22" t="n"/>
-      <c r="D1127" s="22" t="n"/>
-      <c r="E1127" s="22" t="n"/>
-      <c r="F1127" s="22" t="n"/>
-    </row>
-    <row r="1128" ht="20" customHeight="1">
-      <c r="A1128" s="20" t="inlineStr">
-        <is>
-          <t>Titulo</t>
-        </is>
-      </c>
-      <c r="B1128" s="21" t="inlineStr">
-        <is>
-          <t>Mantenimiento caldera y prevencion legionela</t>
-        </is>
-      </c>
-      <c r="C1128" s="22" t="n"/>
-      <c r="D1128" s="22" t="n"/>
-      <c r="E1128" s="22" t="n"/>
-      <c r="F1128" s="22" t="n"/>
-    </row>
-    <row r="1129" ht="20" customHeight="1">
-      <c r="A1129" s="20" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1129" s="21" t="inlineStr">
-        <is>
-          <t>EUS-87256</t>
-        </is>
-      </c>
-      <c r="C1129" s="22" t="n"/>
-      <c r="D1129" s="22" t="n"/>
-      <c r="E1129" s="22" t="n"/>
-      <c r="F1129" s="22" t="n"/>
-    </row>
-    <row r="1130" ht="20" customHeight="1">
-      <c r="A1130" s="20" t="inlineStr">
-        <is>
-          <t>Programa</t>
-        </is>
-      </c>
-      <c r="B1130" s="21" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="C1130" s="22" t="n"/>
-      <c r="D1130" s="22" t="n"/>
-      <c r="E1130" s="22" t="n"/>
-      <c r="F1130" s="22" t="n"/>
-    </row>
-    <row r="1131" ht="20" customHeight="1">
-      <c r="A1131" s="20" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="B1131" s="21" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C1131" s="22" t="n"/>
-      <c r="D1131" s="22" t="n"/>
-      <c r="E1131" s="22" t="n"/>
-      <c r="F1131" s="22" t="n"/>
-    </row>
-    <row r="1132" ht="20" customHeight="1">
-      <c r="A1132" s="20" t="inlineStr">
-        <is>
-          <t>Deadline</t>
-        </is>
-      </c>
-      <c r="B1132" s="21" t="inlineStr"/>
-      <c r="C1132" s="22" t="n"/>
-      <c r="D1132" s="22" t="n"/>
-      <c r="E1132" s="22" t="n"/>
-      <c r="F1132" s="22" t="n"/>
-    </row>
-    <row r="1133" ht="20" customHeight="1">
-      <c r="A1133" s="20" t="inlineStr">
-        <is>
-          <t>Presupuesto (EUR)</t>
-        </is>
-      </c>
-      <c r="B1133" s="21" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="C1133" s="22" t="n"/>
-      <c r="D1133" s="22" t="n"/>
-      <c r="E1133" s="22" t="n"/>
-      <c r="F1133" s="22" t="n"/>
-    </row>
-    <row r="1134" ht="20" customHeight="1">
-      <c r="A1134" s="20" t="inlineStr">
-        <is>
-          <t>Tipo de Accion</t>
-        </is>
-      </c>
-      <c r="B1134" s="21" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="C1134" s="22" t="n"/>
-      <c r="D1134" s="22" t="n"/>
-      <c r="E1134" s="22" t="n"/>
-      <c r="F1134" s="22" t="n"/>
-    </row>
-    <row r="1135" ht="20" customHeight="1">
-      <c r="A1135" s="20" t="inlineStr">
-        <is>
-          <t>Call ID</t>
-        </is>
-      </c>
-      <c r="B1135" s="21" t="inlineStr"/>
-      <c r="C1135" s="22" t="n"/>
-      <c r="D1135" s="22" t="n"/>
-      <c r="E1135" s="22" t="n"/>
-      <c r="F1135" s="22" t="n"/>
-    </row>
-    <row r="1136" ht="20" customHeight="1">
-      <c r="A1136" s="20" t="inlineStr">
-        <is>
-          <t>Descripcion</t>
-        </is>
-      </c>
-      <c r="B1136" s="21" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="C1136" s="22" t="n"/>
-      <c r="D1136" s="22" t="n"/>
-      <c r="E1136" s="22" t="n"/>
-      <c r="F1136" s="22" t="n"/>
-    </row>
-    <row r="1137" ht="20" customHeight="1">
-      <c r="A1137" s="20" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-      <c r="B1137" s="21" t="inlineStr">
-        <is>
-          <t>energia</t>
-        </is>
-      </c>
-      <c r="C1137" s="22" t="n"/>
-      <c r="D1137" s="22" t="n"/>
-      <c r="E1137" s="22" t="n"/>
-      <c r="F1137" s="22" t="n"/>
-    </row>
-    <row r="1138" ht="20" customHeight="1">
-      <c r="A1138" s="20" t="inlineStr">
-        <is>
-          <t>Relevancia Bilbao</t>
-        </is>
-      </c>
-      <c r="B1138" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
-        </is>
-      </c>
-      <c r="C1138" s="22" t="n"/>
-      <c r="D1138" s="22" t="n"/>
-      <c r="E1138" s="22" t="n"/>
-      <c r="F1138" s="22" t="n"/>
-    </row>
-    <row r="1139" ht="45" customHeight="1">
-      <c r="A1139" s="20" t="inlineStr">
-        <is>
-          <t>Enlace al portal</t>
-        </is>
-      </c>
-      <c r="B1139" s="24" t="inlineStr">
-        <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/mantenimiento-caldera-y-prevencion-legionela/expcm498235/web01-tramite/es/</t>
-        </is>
-      </c>
-      <c r="C1139" s="22" t="n"/>
-      <c r="D1139" s="22" t="n"/>
-      <c r="E1139" s="22" t="n"/>
-      <c r="F1139" s="22" t="n"/>
-    </row>
-    <row r="1141" ht="30" customHeight="1">
-      <c r="A1141" s="18" t="inlineStr">
-        <is>
-          <t>FICHA 77: EUS-21550</t>
-        </is>
-      </c>
-      <c r="B1141" s="19" t="n"/>
-      <c r="C1141" s="19" t="n"/>
-      <c r="D1141" s="19" t="n"/>
-      <c r="E1141" s="19" t="n"/>
-      <c r="F1141" s="19" t="n"/>
-    </row>
-    <row r="1142" ht="20" customHeight="1">
-      <c r="A1142" s="20" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-      <c r="B1142" s="21" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
-        </is>
-      </c>
-      <c r="C1142" s="22" t="n"/>
-      <c r="D1142" s="22" t="n"/>
-      <c r="E1142" s="22" t="n"/>
-      <c r="F1142" s="22" t="n"/>
-    </row>
-    <row r="1143" ht="20" customHeight="1">
-      <c r="A1143" s="20" t="inlineStr">
-        <is>
-          <t>Titulo</t>
-        </is>
-      </c>
-      <c r="B1143" s="21" t="inlineStr">
-        <is>
-          <t>Mantenimiento anual y servicio de limpieza de tubos de ozono</t>
-        </is>
-      </c>
-      <c r="C1143" s="22" t="n"/>
-      <c r="D1143" s="22" t="n"/>
-      <c r="E1143" s="22" t="n"/>
-      <c r="F1143" s="22" t="n"/>
-    </row>
-    <row r="1144" ht="20" customHeight="1">
-      <c r="A1144" s="20" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1144" s="21" t="inlineStr">
-        <is>
-          <t>EUS-21550</t>
-        </is>
-      </c>
-      <c r="C1144" s="22" t="n"/>
-      <c r="D1144" s="22" t="n"/>
-      <c r="E1144" s="22" t="n"/>
-      <c r="F1144" s="22" t="n"/>
-    </row>
-    <row r="1145" ht="20" customHeight="1">
-      <c r="A1145" s="20" t="inlineStr">
-        <is>
-          <t>Programa</t>
-        </is>
-      </c>
-      <c r="B1145" s="21" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="C1145" s="22" t="n"/>
-      <c r="D1145" s="22" t="n"/>
-      <c r="E1145" s="22" t="n"/>
-      <c r="F1145" s="22" t="n"/>
-    </row>
-    <row r="1146" ht="20" customHeight="1">
-      <c r="A1146" s="20" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="B1146" s="21" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C1146" s="22" t="n"/>
-      <c r="D1146" s="22" t="n"/>
-      <c r="E1146" s="22" t="n"/>
-      <c r="F1146" s="22" t="n"/>
-    </row>
-    <row r="1147" ht="20" customHeight="1">
-      <c r="A1147" s="20" t="inlineStr">
-        <is>
-          <t>Deadline</t>
-        </is>
-      </c>
-      <c r="B1147" s="21" t="inlineStr"/>
-      <c r="C1147" s="22" t="n"/>
-      <c r="D1147" s="22" t="n"/>
-      <c r="E1147" s="22" t="n"/>
-      <c r="F1147" s="22" t="n"/>
-    </row>
-    <row r="1148" ht="20" customHeight="1">
-      <c r="A1148" s="20" t="inlineStr">
-        <is>
-          <t>Presupuesto (EUR)</t>
-        </is>
-      </c>
-      <c r="B1148" s="21" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="C1148" s="22" t="n"/>
-      <c r="D1148" s="22" t="n"/>
-      <c r="E1148" s="22" t="n"/>
-      <c r="F1148" s="22" t="n"/>
-    </row>
-    <row r="1149" ht="20" customHeight="1">
-      <c r="A1149" s="20" t="inlineStr">
-        <is>
-          <t>Tipo de Accion</t>
-        </is>
-      </c>
-      <c r="B1149" s="21" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="C1149" s="22" t="n"/>
-      <c r="D1149" s="22" t="n"/>
-      <c r="E1149" s="22" t="n"/>
-      <c r="F1149" s="22" t="n"/>
-    </row>
-    <row r="1150" ht="20" customHeight="1">
-      <c r="A1150" s="20" t="inlineStr">
-        <is>
-          <t>Call ID</t>
-        </is>
-      </c>
-      <c r="B1150" s="21" t="inlineStr"/>
-      <c r="C1150" s="22" t="n"/>
-      <c r="D1150" s="22" t="n"/>
-      <c r="E1150" s="22" t="n"/>
-      <c r="F1150" s="22" t="n"/>
-    </row>
-    <row r="1151" ht="20" customHeight="1">
-      <c r="A1151" s="20" t="inlineStr">
-        <is>
-          <t>Descripcion</t>
-        </is>
-      </c>
-      <c r="B1151" s="21" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="C1151" s="22" t="n"/>
-      <c r="D1151" s="22" t="n"/>
-      <c r="E1151" s="22" t="n"/>
-      <c r="F1151" s="22" t="n"/>
-    </row>
-    <row r="1152" ht="20" customHeight="1">
-      <c r="A1152" s="20" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-      <c r="B1152" s="21" t="inlineStr">
-        <is>
-          <t>energia</t>
-        </is>
-      </c>
-      <c r="C1152" s="22" t="n"/>
-      <c r="D1152" s="22" t="n"/>
-      <c r="E1152" s="22" t="n"/>
-      <c r="F1152" s="22" t="n"/>
-    </row>
-    <row r="1153" ht="20" customHeight="1">
-      <c r="A1153" s="20" t="inlineStr">
-        <is>
-          <t>Relevancia Bilbao</t>
-        </is>
-      </c>
-      <c r="B1153" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
-        </is>
-      </c>
-      <c r="C1153" s="22" t="n"/>
-      <c r="D1153" s="22" t="n"/>
-      <c r="E1153" s="22" t="n"/>
-      <c r="F1153" s="22" t="n"/>
-    </row>
-    <row r="1154" ht="45" customHeight="1">
-      <c r="A1154" s="20" t="inlineStr">
-        <is>
-          <t>Enlace al portal</t>
-        </is>
-      </c>
-      <c r="B1154" s="24" t="inlineStr">
-        <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/mantenimiento-anual-y-servicio-limpieza-tubos-ozono/web01-tramite/es/</t>
-        </is>
-      </c>
-      <c r="C1154" s="22" t="n"/>
-      <c r="D1154" s="22" t="n"/>
-      <c r="E1154" s="22" t="n"/>
-      <c r="F1154" s="22" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="1078">
+  <mergeCells count="1022">
     <mergeCell ref="B679:F679"/>
     <mergeCell ref="B666:F666"/>
     <mergeCell ref="B964:F964"/>
@@ -21856,10 +20780,7 @@
     <mergeCell ref="B342:F342"/>
     <mergeCell ref="B578:F578"/>
     <mergeCell ref="A541:F541"/>
-    <mergeCell ref="B1148:F1148"/>
-    <mergeCell ref="B1099:F1099"/>
     <mergeCell ref="B515:F515"/>
-    <mergeCell ref="B1128:F1128"/>
     <mergeCell ref="A841:F841"/>
     <mergeCell ref="B158:F158"/>
     <mergeCell ref="B1094:F1094"/>
@@ -21868,11 +20789,9 @@
     <mergeCell ref="B894:F894"/>
     <mergeCell ref="B133:F133"/>
     <mergeCell ref="B959:F959"/>
-    <mergeCell ref="B1130:F1130"/>
     <mergeCell ref="B369:F369"/>
     <mergeCell ref="B667:F667"/>
     <mergeCell ref="B418:F418"/>
-    <mergeCell ref="B1142:F1142"/>
     <mergeCell ref="B356:F356"/>
     <mergeCell ref="B160:F160"/>
     <mergeCell ref="B489:F489"/>
@@ -21896,13 +20815,11 @@
     <mergeCell ref="B662:F662"/>
     <mergeCell ref="B718:F718"/>
     <mergeCell ref="B889:F889"/>
-    <mergeCell ref="B1131:F1131"/>
     <mergeCell ref="B72:F72"/>
     <mergeCell ref="B954:F954"/>
     <mergeCell ref="B199:F199"/>
     <mergeCell ref="B370:F370"/>
     <mergeCell ref="B1025:F1025"/>
-    <mergeCell ref="B1112:F1112"/>
     <mergeCell ref="B291:F291"/>
     <mergeCell ref="B655:F655"/>
     <mergeCell ref="B974:F974"/>
@@ -21944,7 +20861,6 @@
     <mergeCell ref="B83:F83"/>
     <mergeCell ref="B254:F254"/>
     <mergeCell ref="B909:F909"/>
-    <mergeCell ref="B1105:F1105"/>
     <mergeCell ref="B319:F319"/>
     <mergeCell ref="B490:F490"/>
     <mergeCell ref="B604:F604"/>
@@ -21956,7 +20872,6 @@
     <mergeCell ref="A346:F346"/>
     <mergeCell ref="B904:F904"/>
     <mergeCell ref="B635:F635"/>
-    <mergeCell ref="A1141:F1141"/>
     <mergeCell ref="B141:F141"/>
     <mergeCell ref="B439:F439"/>
     <mergeCell ref="A136:F136"/>
@@ -21977,7 +20892,6 @@
     <mergeCell ref="B530:F530"/>
     <mergeCell ref="B726:F726"/>
     <mergeCell ref="B962:F962"/>
-    <mergeCell ref="B1133:F1133"/>
     <mergeCell ref="A886:F886"/>
     <mergeCell ref="B505:F505"/>
     <mergeCell ref="B1060:F1060"/>
@@ -22009,12 +20923,10 @@
     <mergeCell ref="B1055:F1055"/>
     <mergeCell ref="B536:F536"/>
     <mergeCell ref="B834:F834"/>
-    <mergeCell ref="B1143:F1143"/>
     <mergeCell ref="B899:F899"/>
     <mergeCell ref="B752:F752"/>
     <mergeCell ref="B1070:F1070"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B1115:F1115"/>
     <mergeCell ref="B325:F325"/>
     <mergeCell ref="B154:F154"/>
     <mergeCell ref="A271:F271"/>
@@ -22029,7 +20941,6 @@
     <mergeCell ref="B1044:F1044"/>
     <mergeCell ref="B156:F156"/>
     <mergeCell ref="B327:F327"/>
-    <mergeCell ref="B1144:F1144"/>
     <mergeCell ref="B454:F454"/>
     <mergeCell ref="B625:F625"/>
     <mergeCell ref="B923:F923"/>
@@ -22049,9 +20960,6 @@
     <mergeCell ref="B518:F518"/>
     <mergeCell ref="B562:F562"/>
     <mergeCell ref="B689:F689"/>
-    <mergeCell ref="B1121:F1121"/>
-    <mergeCell ref="B1146:F1146"/>
-    <mergeCell ref="B1123:F1123"/>
     <mergeCell ref="B86:F86"/>
     <mergeCell ref="B912:F912"/>
     <mergeCell ref="B1083:F1083"/>
@@ -22103,7 +21011,6 @@
     <mergeCell ref="B979:F979"/>
     <mergeCell ref="B381:F381"/>
     <mergeCell ref="B552:F552"/>
-    <mergeCell ref="A1111:F1111"/>
     <mergeCell ref="B1084:F1084"/>
     <mergeCell ref="A976:F976"/>
     <mergeCell ref="B170:F170"/>
@@ -22137,7 +21044,6 @@
     <mergeCell ref="B92:F92"/>
     <mergeCell ref="B984:F984"/>
     <mergeCell ref="A226:F226"/>
-    <mergeCell ref="B1124:F1124"/>
     <mergeCell ref="B394:F394"/>
     <mergeCell ref="B692:F692"/>
     <mergeCell ref="A931:F931"/>
@@ -22168,7 +21074,6 @@
     <mergeCell ref="B817:F817"/>
     <mergeCell ref="B944:F944"/>
     <mergeCell ref="B56:F56"/>
-    <mergeCell ref="B1102:F1102"/>
     <mergeCell ref="B43:F43"/>
     <mergeCell ref="B176:F176"/>
     <mergeCell ref="B347:F347"/>
@@ -22184,9 +21089,7 @@
     <mergeCell ref="B881:F881"/>
     <mergeCell ref="B1068:F1068"/>
     <mergeCell ref="B868:F868"/>
-    <mergeCell ref="B1117:F1117"/>
     <mergeCell ref="B107:F107"/>
-    <mergeCell ref="B1104:F1104"/>
     <mergeCell ref="B641:F641"/>
     <mergeCell ref="B57:F57"/>
     <mergeCell ref="B883:F883"/>
@@ -22198,7 +21101,6 @@
     <mergeCell ref="B9:F9"/>
     <mergeCell ref="B463:F463"/>
     <mergeCell ref="B438:F438"/>
-    <mergeCell ref="B1145:F1145"/>
     <mergeCell ref="B359:F359"/>
     <mergeCell ref="B207:F207"/>
     <mergeCell ref="B788:F788"/>
@@ -22213,8 +21115,6 @@
     <mergeCell ref="B999:F999"/>
     <mergeCell ref="B1061:F1061"/>
     <mergeCell ref="B4:F4"/>
-    <mergeCell ref="B1097:F1097"/>
-    <mergeCell ref="B1153:F1153"/>
     <mergeCell ref="A46:F46"/>
     <mergeCell ref="B507:F507"/>
     <mergeCell ref="B62:F62"/>
@@ -22262,7 +21162,6 @@
     <mergeCell ref="B1018:F1018"/>
     <mergeCell ref="B624:F624"/>
     <mergeCell ref="B428:F428"/>
-    <mergeCell ref="B1118:F1118"/>
     <mergeCell ref="B284:F284"/>
     <mergeCell ref="B222:F222"/>
     <mergeCell ref="B344:F344"/>
@@ -22274,7 +21173,6 @@
     <mergeCell ref="B123:F123"/>
     <mergeCell ref="B949:F949"/>
     <mergeCell ref="B1011:F1011"/>
-    <mergeCell ref="B1120:F1120"/>
     <mergeCell ref="B50:F50"/>
     <mergeCell ref="B221:F221"/>
     <mergeCell ref="B110:F110"/>
@@ -22291,7 +21189,6 @@
     <mergeCell ref="B802:F802"/>
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B789:F789"/>
-    <mergeCell ref="B1136:F1136"/>
     <mergeCell ref="B248:F248"/>
     <mergeCell ref="B297:F297"/>
     <mergeCell ref="B813:F813"/>
@@ -22311,11 +21208,9 @@
     <mergeCell ref="B815:F815"/>
     <mergeCell ref="B597:F597"/>
     <mergeCell ref="B1064:F1064"/>
-    <mergeCell ref="B1113:F1113"/>
     <mergeCell ref="B103:F103"/>
     <mergeCell ref="B78:F78"/>
     <mergeCell ref="B833:F833"/>
-    <mergeCell ref="B1100:F1100"/>
     <mergeCell ref="B205:F205"/>
     <mergeCell ref="B339:F339"/>
     <mergeCell ref="B314:F314"/>
@@ -22388,7 +21283,6 @@
     <mergeCell ref="A721:F721"/>
     <mergeCell ref="A31:F31"/>
     <mergeCell ref="B747:F747"/>
-    <mergeCell ref="B1152:F1152"/>
     <mergeCell ref="B668:F668"/>
     <mergeCell ref="B84:F84"/>
     <mergeCell ref="A736:F736"/>
@@ -22412,7 +21306,6 @@
     <mergeCell ref="B305:F305"/>
     <mergeCell ref="B816:F816"/>
     <mergeCell ref="B918:F918"/>
-    <mergeCell ref="B1114:F1114"/>
     <mergeCell ref="B607:F607"/>
     <mergeCell ref="B663:F663"/>
     <mergeCell ref="B1049:F1049"/>
@@ -22423,7 +21316,6 @@
     <mergeCell ref="B442:F442"/>
     <mergeCell ref="B242:F242"/>
     <mergeCell ref="B880:F880"/>
-    <mergeCell ref="B1116:F1116"/>
     <mergeCell ref="B671:F671"/>
     <mergeCell ref="B969:F969"/>
     <mergeCell ref="B907:F907"/>
@@ -22441,15 +21333,12 @@
     <mergeCell ref="B760:F760"/>
     <mergeCell ref="B437:F437"/>
     <mergeCell ref="B852:F852"/>
-    <mergeCell ref="B1119:F1119"/>
     <mergeCell ref="B333:F333"/>
-    <mergeCell ref="B1098:F1098"/>
     <mergeCell ref="B898:F898"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="B520:F520"/>
     <mergeCell ref="B958:F958"/>
     <mergeCell ref="B308:F308"/>
-    <mergeCell ref="B1134:F1134"/>
     <mergeCell ref="B854:F854"/>
     <mergeCell ref="B99:F99"/>
     <mergeCell ref="B737:F737"/>
@@ -22468,14 +21357,12 @@
     <mergeCell ref="B372:F372"/>
     <mergeCell ref="B1071:F1071"/>
     <mergeCell ref="B608:F608"/>
-    <mergeCell ref="B1127:F1127"/>
     <mergeCell ref="B595:F595"/>
     <mergeCell ref="B1037:F1037"/>
     <mergeCell ref="B722:F722"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="A856:F856"/>
     <mergeCell ref="B893:F893"/>
-    <mergeCell ref="B1129:F1129"/>
     <mergeCell ref="B374:F374"/>
     <mergeCell ref="B659:F659"/>
     <mergeCell ref="B830:F830"/>
@@ -22544,7 +21431,6 @@
     <mergeCell ref="B309:F309"/>
     <mergeCell ref="A316:F316"/>
     <mergeCell ref="B380:F380"/>
-    <mergeCell ref="B1135:F1135"/>
     <mergeCell ref="A1081:F1081"/>
     <mergeCell ref="B100:F100"/>
     <mergeCell ref="B336:F336"/>
@@ -22554,12 +21440,10 @@
     <mergeCell ref="B140:F140"/>
     <mergeCell ref="B115:F115"/>
     <mergeCell ref="B382:F382"/>
-    <mergeCell ref="A1096:F1096"/>
     <mergeCell ref="B680:F680"/>
     <mergeCell ref="A376:F376"/>
     <mergeCell ref="B102:F102"/>
     <mergeCell ref="B674:F674"/>
-    <mergeCell ref="B1137:F1137"/>
     <mergeCell ref="B400:F400"/>
     <mergeCell ref="B698:F698"/>
     <mergeCell ref="B832:F832"/>
@@ -22572,7 +21456,6 @@
     <mergeCell ref="B598:F598"/>
     <mergeCell ref="B402:F402"/>
     <mergeCell ref="B669:F669"/>
-    <mergeCell ref="B1138:F1138"/>
     <mergeCell ref="B377:F377"/>
     <mergeCell ref="A451:F451"/>
     <mergeCell ref="B29:F29"/>
@@ -22582,7 +21465,6 @@
     <mergeCell ref="B756:F756"/>
     <mergeCell ref="B992:F992"/>
     <mergeCell ref="A811:F811"/>
-    <mergeCell ref="B1150:F1150"/>
     <mergeCell ref="B329:F329"/>
     <mergeCell ref="B627:F627"/>
     <mergeCell ref="B49:F49"/>
@@ -22630,7 +21512,6 @@
     <mergeCell ref="B845:F845"/>
     <mergeCell ref="B261:F261"/>
     <mergeCell ref="B1087:F1087"/>
-    <mergeCell ref="B1149:F1149"/>
     <mergeCell ref="B184:F184"/>
     <mergeCell ref="B1062:F1062"/>
     <mergeCell ref="A301:F301"/>
@@ -22717,7 +21598,6 @@
     <mergeCell ref="B1024:F1024"/>
     <mergeCell ref="B396:F396"/>
     <mergeCell ref="B567:F567"/>
-    <mergeCell ref="B1151:F1151"/>
     <mergeCell ref="B632:F632"/>
     <mergeCell ref="B803:F803"/>
     <mergeCell ref="B996:F996"/>
@@ -22737,7 +21617,6 @@
     <mergeCell ref="B269:F269"/>
     <mergeCell ref="B187:F187"/>
     <mergeCell ref="B485:F485"/>
-    <mergeCell ref="B1154:F1154"/>
     <mergeCell ref="B124:F124"/>
     <mergeCell ref="B251:F251"/>
     <mergeCell ref="B806:F806"/>
@@ -22783,15 +21662,11 @@
     <mergeCell ref="B409:F409"/>
     <mergeCell ref="B580:F580"/>
     <mergeCell ref="B920:F920"/>
-    <mergeCell ref="B1108:F1108"/>
     <mergeCell ref="B711:F711"/>
     <mergeCell ref="B1009:F1009"/>
     <mergeCell ref="B48:F48"/>
-    <mergeCell ref="B1101:F1101"/>
     <mergeCell ref="B582:F582"/>
     <mergeCell ref="B849:F849"/>
-    <mergeCell ref="B1147:F1147"/>
-    <mergeCell ref="B1132:F1132"/>
     <mergeCell ref="B73:F73"/>
     <mergeCell ref="B371:F371"/>
     <mergeCell ref="B638:F638"/>
@@ -22804,7 +21679,6 @@
     <mergeCell ref="A676:F676"/>
     <mergeCell ref="B137:F137"/>
     <mergeCell ref="B379:F379"/>
-    <mergeCell ref="B1106:F1106"/>
     <mergeCell ref="B702:F702"/>
     <mergeCell ref="B677:F677"/>
     <mergeCell ref="B640:F640"/>
@@ -22835,7 +21709,6 @@
     <mergeCell ref="B66:F66"/>
     <mergeCell ref="B326:F326"/>
     <mergeCell ref="B793:F793"/>
-    <mergeCell ref="B1103:F1103"/>
     <mergeCell ref="A406:F406"/>
     <mergeCell ref="B951:F951"/>
     <mergeCell ref="B130:F130"/>
@@ -22854,7 +21727,6 @@
     <mergeCell ref="B132:F132"/>
     <mergeCell ref="B425:F425"/>
     <mergeCell ref="B430:F430"/>
-    <mergeCell ref="B1107:F1107"/>
     <mergeCell ref="B1045:F1045"/>
     <mergeCell ref="B119:F119"/>
     <mergeCell ref="B290:F290"/>
@@ -22865,13 +21737,10 @@
     <mergeCell ref="B824:F824"/>
     <mergeCell ref="B1017:F1017"/>
     <mergeCell ref="B367:F367"/>
-    <mergeCell ref="B1122:F1122"/>
     <mergeCell ref="B427:F427"/>
-    <mergeCell ref="B1139:F1139"/>
     <mergeCell ref="B112:F112"/>
     <mergeCell ref="B283:F283"/>
     <mergeCell ref="B354:F354"/>
-    <mergeCell ref="B1109:F1109"/>
     <mergeCell ref="B348:F348"/>
     <mergeCell ref="B519:F519"/>
     <mergeCell ref="B419:F419"/>
@@ -22887,7 +21756,6 @@
     <mergeCell ref="B648:F648"/>
     <mergeCell ref="B64:F64"/>
     <mergeCell ref="B51:F51"/>
-    <mergeCell ref="A1126:F1126"/>
     <mergeCell ref="B443:F443"/>
     <mergeCell ref="A196:F196"/>
     <mergeCell ref="B237:F237"/>
@@ -22966,10 +21834,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1064" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1079" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1094" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1109" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1124" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1139" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1154" r:id="rId77"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -22981,7 +21845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J78"/>
+  <dimension ref="A1:J74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -23131,19 +21995,15 @@
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>INNOVFUND-2025-NZT-GENERAL-MSP</t>
+          <t>02ea5f5c-3122-4e73-a32a-dfb5ff0f395c-CN</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Innovation Fund 2025 Net Zero Technologies - General decarbo</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Innovation Fund</t>
-        </is>
-      </c>
+          <t>Analysis of target setting for a selection of common indicat</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr"/>
       <c r="D4" s="6" t="inlineStr">
         <is>
           <t>Open</t>
@@ -23151,7 +22011,7 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="F4" s="27" t="inlineStr">
@@ -23171,7 +22031,7 @@
     <row r="5" ht="28" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>INNOVFUND-2025-NZT-GENERAL-SSP</t>
+          <t>INNOVFUND-2025-NZT-GENERAL-MSP</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -23211,7 +22071,7 @@
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>INNOVFUND-2025-NZT-GENERAL-LSP</t>
+          <t>INNOVFUND-2025-NZT-GENERAL-SSP</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -23251,17 +22111,17 @@
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-2-PRIZE</t>
+          <t>INNOVFUND-2025-NZT-GENERAL-LSP</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Renewable energy technology (RET) solutions in energy commun</t>
+          <t>Innovation Fund 2025 Net Zero Technologies - General decarbo</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Horizon Europe</t>
+          <t>Innovation Fund</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -23271,7 +22131,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>25/06/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="F7" s="27" t="inlineStr">
@@ -23291,15 +22151,19 @@
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>02ea5f5c-3122-4e73-a32a-dfb5ff0f395c-CN</t>
+          <t>HORIZON-CL5-2026-2-PRIZE</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Analysis of target setting for a selection of common indicat</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr"/>
+          <t>Renewable energy technology (RET) solutions in energy commun</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Horizon Europe</t>
+        </is>
+      </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Open</t>
@@ -23307,7 +22171,7 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>30/03/2026</t>
+          <t>25/06/2026</t>
         </is>
       </c>
       <c r="F8" s="27" t="inlineStr">
@@ -25091,12 +23955,12 @@
     <row r="56" ht="28" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>EUS-97765</t>
+          <t>EUS-47030</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
+          <t>Servicios de transporte y manipulación de obras de arte para</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
@@ -25112,7 +23976,7 @@
       <c r="E56" s="6" t="inlineStr"/>
       <c r="F56" s="27" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>MUY ALTA</t>
         </is>
       </c>
       <c r="G56" s="6" t="inlineStr"/>
@@ -25127,12 +23991,12 @@
     <row r="57" ht="28" customHeight="1">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>EUS-23570</t>
+          <t>EUS-15017</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la gestión sostenible de los recursos pesqueros 202</t>
+          <t>Mantenimiento de las instalaciones de climatización de la of</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
@@ -25148,7 +24012,7 @@
       <c r="E57" s="6" t="inlineStr"/>
       <c r="F57" s="27" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>MUY ALTA</t>
         </is>
       </c>
       <c r="G57" s="6" t="inlineStr"/>
@@ -25163,12 +24027,12 @@
     <row r="58" ht="28" customHeight="1">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>EUS-92691</t>
+          <t>EUS-25647</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la recogida de residuos con la participación de los</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
@@ -25199,12 +24063,12 @@
     <row r="59" ht="28" customHeight="1">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>EUS-34245</t>
+          <t>EUS-39134</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
+          <t>Ayudas a la gestión sostenible de los recursos pesqueros 202</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
@@ -25235,12 +24099,12 @@
     <row r="60" ht="28" customHeight="1">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>EUS-17774</t>
+          <t>EUS-85153</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>Servicio de oficina técnica para la mejora del sistema de pr</t>
+          <t>Ayudas a la recogida de residuos con la participación de los</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -25271,12 +24135,12 @@
     <row r="61" ht="28" customHeight="1">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>EUS-22731</t>
+          <t>EUS-21937</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>Redacción de un Plan de prevención y gestión de residuos</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
@@ -25307,12 +24171,12 @@
     <row r="62" ht="28" customHeight="1">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>EUS-32199</t>
+          <t>EUS-02512</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la contribución de la acuicultura al buen estado am</t>
+          <t>Servicio de transporte y gestión de los residuos procedentes</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
@@ -25328,7 +24192,7 @@
       <c r="E62" s="6" t="inlineStr"/>
       <c r="F62" s="27" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="G62" s="6" t="inlineStr"/>
@@ -25343,12 +24207,12 @@
     <row r="63" ht="28" customHeight="1">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>EUS-89864</t>
+          <t>EUS-91129</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>Ayudas al valor añadido, economía circular y seguridad alime</t>
+          <t>Ayudas a la contribución de la acuicultura al buen estado am</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
@@ -25379,12 +24243,12 @@
     <row r="64" ht="28" customHeight="1">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>EUS-92385</t>
+          <t>EUS-46360</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>Vino: el Gobierno Vasco volverá a convocar este mes las ayud</t>
+          <t>Ayudas al valor añadido, economía circular y seguridad alime</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
@@ -25415,12 +24279,12 @@
     <row r="65" ht="28" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>EUS-45123</t>
+          <t>EUS-14446</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de</t>
+          <t>Vino: el Gobierno Vasco volverá a convocar este mes las ayud</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -25451,12 +24315,12 @@
     <row r="66" ht="28" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>EUS-63814</t>
+          <t>EUS-75188</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para c</t>
+          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
@@ -25487,12 +24351,12 @@
     <row r="67" ht="28" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>EUS-82158</t>
+          <t>EUS-45072</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinanc</t>
+          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para c</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
@@ -25523,12 +24387,12 @@
     <row r="68" ht="28" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>EUS-92414</t>
+          <t>EUS-36943</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>Digital Europe, Horizon (programas de la UE). Apoyos para co</t>
+          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinanc</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -25559,12 +24423,12 @@
     <row r="69" ht="28" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>EUS-62683</t>
+          <t>EUS-80876</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>Política Agraria Común de la UE de 2026, y sus ayudas abiert</t>
+          <t>Digital Europe, Horizon (programas de la UE). Apoyos para co</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -25595,12 +24459,12 @@
     <row r="70" ht="28" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>EUS-33389</t>
+          <t>EUS-03523</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>Programa de impulso a las ciudades y territorios inteligente</t>
+          <t>Política Agraria Común de la UE de 2026, y sus ayudas abiert</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -25631,12 +24495,12 @@
     <row r="71" ht="28" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>EUS-40042</t>
+          <t>EUS-44113</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>Suministros y Servicios para la instalación de una red XGS-P</t>
+          <t>Programa de impulso a las ciudades y territorios inteligente</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -25667,12 +24531,12 @@
     <row r="72" ht="28" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>EUS-25076</t>
+          <t>EUS-71405</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>Realización del vuelo fotogramétrico digital multivista, esc</t>
+          <t xml:space="preserve">Dirección facultativa de obra (dirección de obra, dirección </t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -25703,12 +24567,12 @@
     <row r="73" ht="28" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>EUS-13379</t>
+          <t>EUS-85319</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>Suministro para la ampliación de la infraestructura de los r</t>
+          <t>Licitación de la obra ?Adecuación del espacio público y ejec</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -25739,12 +24603,12 @@
     <row r="74" ht="28" customHeight="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>EUS-89192</t>
+          <t>EUS-57006</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>Suministro e instalación de fuente de agua fría para consumo</t>
+          <t>Suministro de un sistema de Seguridad e Información Turístic</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
@@ -25772,152 +24636,8 @@
       <c r="I74" s="6" t="inlineStr"/>
       <c r="J74" s="6" t="inlineStr"/>
     </row>
-    <row r="75" ht="28" customHeight="1">
-      <c r="A75" s="6" t="inlineStr">
-        <is>
-          <t>EUS-06858</t>
-        </is>
-      </c>
-      <c r="B75" s="6" t="inlineStr">
-        <is>
-          <t>Equipamiento de muebles en vivienda municipal</t>
-        </is>
-      </c>
-      <c r="C75" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="D75" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E75" s="6" t="inlineStr"/>
-      <c r="F75" s="27" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="G75" s="6" t="inlineStr"/>
-      <c r="H75" s="6" t="inlineStr">
-        <is>
-          <t>Por revisar</t>
-        </is>
-      </c>
-      <c r="I75" s="6" t="inlineStr"/>
-      <c r="J75" s="6" t="inlineStr"/>
-    </row>
-    <row r="76" ht="28" customHeight="1">
-      <c r="A76" s="6" t="inlineStr">
-        <is>
-          <t>EUS-68952</t>
-        </is>
-      </c>
-      <c r="B76" s="6" t="inlineStr">
-        <is>
-          <t>Servicio de limpieza, DDD y legionella de edificios municipa</t>
-        </is>
-      </c>
-      <c r="C76" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="D76" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E76" s="6" t="inlineStr"/>
-      <c r="F76" s="27" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="G76" s="6" t="inlineStr"/>
-      <c r="H76" s="6" t="inlineStr">
-        <is>
-          <t>Por revisar</t>
-        </is>
-      </c>
-      <c r="I76" s="6" t="inlineStr"/>
-      <c r="J76" s="6" t="inlineStr"/>
-    </row>
-    <row r="77" ht="28" customHeight="1">
-      <c r="A77" s="6" t="inlineStr">
-        <is>
-          <t>EUS-87256</t>
-        </is>
-      </c>
-      <c r="B77" s="6" t="inlineStr">
-        <is>
-          <t>Mantenimiento caldera y prevencion legionela</t>
-        </is>
-      </c>
-      <c r="C77" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="D77" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E77" s="6" t="inlineStr"/>
-      <c r="F77" s="27" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="G77" s="6" t="inlineStr"/>
-      <c r="H77" s="6" t="inlineStr">
-        <is>
-          <t>Por revisar</t>
-        </is>
-      </c>
-      <c r="I77" s="6" t="inlineStr"/>
-      <c r="J77" s="6" t="inlineStr"/>
-    </row>
-    <row r="78" ht="28" customHeight="1">
-      <c r="A78" s="6" t="inlineStr">
-        <is>
-          <t>EUS-21550</t>
-        </is>
-      </c>
-      <c r="B78" s="6" t="inlineStr">
-        <is>
-          <t>Mantenimiento anual y servicio de limpieza de tubos de ozono</t>
-        </is>
-      </c>
-      <c r="C78" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="D78" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E78" s="6" t="inlineStr"/>
-      <c r="F78" s="27" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="G78" s="6" t="inlineStr"/>
-      <c r="H78" s="6" t="inlineStr">
-        <is>
-          <t>Por revisar</t>
-        </is>
-      </c>
-      <c r="I78" s="6" t="inlineStr"/>
-      <c r="J78" s="6" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J78"/>
+  <autoFilter ref="A1:J74"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update funding data 2026-03-30
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Recursos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$77</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$73</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -679,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M77"/>
+  <dimension ref="A1:M79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -707,7 +707,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 29/03/2026 06:53 - 70 convocatorias - 18 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 30/03/2026 07:16 - 72 convocatorias - 20 nuevas</t>
         </is>
       </c>
     </row>
@@ -3811,12 +3811,12 @@
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>EUS-04481</t>
+          <t>EUS-48814</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>Mantenimiento de Infraestructuras y Jardinería en el Tramo Común, Línea 1 y Línea 2 de Metro Bilbao.</t>
+          <t>Suministro de once (11) relojes de pulsera (analogicos o inteligentes) para el Ayuntamiento de Basauri.</t>
         </is>
       </c>
       <c r="D60" s="6" t="inlineStr">
@@ -3866,12 +3866,12 @@
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>EUS-27303</t>
+          <t>EUS-07430</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
+          <t>Servicio para el desarrollo de campañas de sensibilización sobre la gestión selectiva de residuos, y en especial, para el fomento de la recogida separada de la fracción orgánica, dirigidas a la ciudad</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
@@ -3888,12 +3888,12 @@
       <c r="G61" s="6" t="inlineStr"/>
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
-        </is>
-      </c>
-      <c r="I61" s="8" t="inlineStr">
-        <is>
-          <t>ALTA</t>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I61" s="12" t="inlineStr">
+        <is>
+          <t>MUY ALTA</t>
         </is>
       </c>
       <c r="J61" s="6" t="inlineStr"/>
@@ -3921,12 +3921,12 @@
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>EUS-38413</t>
+          <t>EUS-94512</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la gestión sostenible de los recursos pesqueros 2026</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
         </is>
       </c>
       <c r="D62" s="6" t="inlineStr">
@@ -3976,12 +3976,12 @@
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>EUS-09490</t>
+          <t>EUS-52245</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la recogida de residuos con la participación de los pescadores en el mar y las playas 2026</t>
+          <t>Ayudas a la gestión sostenible de los recursos pesqueros 2026</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
@@ -4031,12 +4031,12 @@
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>EUS-09919</t>
+          <t>EUS-93243</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático sin incremento de capacidad 2026</t>
+          <t>Ayudas a la recogida de residuos con la participación de los pescadores en el mar y las playas 2026</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
@@ -4086,12 +4086,12 @@
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>EUS-33827</t>
+          <t>EUS-27478</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio climático sin incremento de capacidad 2026</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
@@ -4111,9 +4111,9 @@
           <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
-      <c r="I65" s="10" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
+      <c r="I65" s="8" t="inlineStr">
+        <is>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="J65" s="6" t="inlineStr"/>
@@ -4141,12 +4141,12 @@
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>EUS-47315</t>
+          <t>EUS-36149</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>Ayudas al valor añadido, economía circular y seguridad alimentaria 2026</t>
+          <t>Elaboracion de un Plan de Comunicación y Promocion en medios digitales del Plan de Movilidad (NEXT)</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
@@ -4163,12 +4163,12 @@
       <c r="G66" s="6" t="inlineStr"/>
       <c r="H66" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
-        </is>
-      </c>
-      <c r="I66" s="10" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I66" s="8" t="inlineStr">
+        <is>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="J66" s="6" t="inlineStr"/>
@@ -4196,12 +4196,12 @@
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>EUS-97811</t>
+          <t>EUS-33038</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>Vino: el Gobierno Vasco volverá a convocar este mes las ayudas al arranque o cosecha en verde del viñedo, que van a contemplar como estructurales tras reformar la UE jurídicamente su Intervención Sect</t>
+          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
@@ -4251,12 +4251,12 @@
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>EUS-56533</t>
+          <t>EUS-46453</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de aceleración de proyectos, a localidades de menos de 20.000 habitantes son objeto de convocatoria abierta hasta el 17.03.26. Transformacione</t>
+          <t>Ayudas al valor añadido, economía circular y seguridad alimentaria 2026</t>
         </is>
       </c>
       <c r="D68" s="6" t="inlineStr">
@@ -4306,12 +4306,12 @@
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>EUS-02669</t>
+          <t>EUS-86136</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para consorcios internacionales de I+D+i. Jornada del Gobierno Vasco y con Enterprise Europe Network y otros socios. Digitalización, dispositivos,</t>
+          <t>Vino: el Gobierno Vasco volverá a convocar este mes las ayudas al arranque o cosecha en verde del viñedo, que van a contemplar como estructurales tras reformar la UE jurídicamente su Intervención Sect</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
@@ -4361,12 +4361,12 @@
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>EUS-15404</t>
+          <t>EUS-37235</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinancia convocatorias de ayudas de las Diputaciones a explotaciones con limitaciones o desfavorecidas, y a compromisos medioambientales, climátic</t>
+          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de aceleración de proyectos, a localidades de menos de 20.000 habitantes son objeto de convocatoria abierta hasta el 17.03.26. Transformacione</t>
         </is>
       </c>
       <c r="D70" s="6" t="inlineStr">
@@ -4416,12 +4416,12 @@
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>EUS-08599</t>
+          <t>EUS-41490</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>Digital Europe, Horizon (programas de la UE). Apoyos para consorcios interestatales de I+D+i. IA, robótica, cuántica, computación, ciberseguridad, electrónica, fotónica, TICs e internet avanzadas, esp</t>
+          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para consorcios internacionales de I+D+i. Jornada del Gobierno Vasco y con Enterprise Europe Network y otros socios. Digitalización, dispositivos,</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
@@ -4471,12 +4471,12 @@
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>EUS-58604</t>
+          <t>EUS-03701</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>EPIS Ropa Impermeable Jardinería</t>
+          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinancia convocatorias de ayudas de las Diputaciones a explotaciones con limitaciones o desfavorecidas, y a compromisos medioambientales, climátic</t>
         </is>
       </c>
       <c r="D72" s="6" t="inlineStr">
@@ -4493,7 +4493,7 @@
       <c r="G72" s="6" t="inlineStr"/>
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="I72" s="10" t="inlineStr">
@@ -4526,12 +4526,12 @@
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>EUS-85654</t>
+          <t>EUS-52104</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>Ropa Laboral Tecnica Jardinería</t>
+          <t>Digital Europe, Horizon (programas de la UE). Apoyos para consorcios interestatales de I+D+i. IA, robótica, cuántica, computación, ciberseguridad, electrónica, fotónica, TICs e internet avanzadas, esp</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
@@ -4548,7 +4548,7 @@
       <c r="G73" s="6" t="inlineStr"/>
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="I73" s="10" t="inlineStr">
@@ -4581,15 +4581,12 @@
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>EUS-72988</t>
+          <t>EUS-06210</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>Proyecto Técnico para
-la legalización de la instalación eléctrica en baja
-tensión del edificio LARREKOETXE de IES
-ORIARTE de Lasarte-Oria (Gipuzkoa)</t>
+          <t>Obras definidas en el Proyecto de Ejecución de reforma de la cubierta del comedor en el Colegio Santo Angel</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr">
@@ -4639,16 +4636,12 @@
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>EUS-53698</t>
+          <t>EUS-35472</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>Coordinación de
-seguridad y salud en las obras de sustitución y
-reparción de ventanas y reparaciòn de filtraciones
-de agua y alicatados en ARTAZUGOIKO IRALE de
-Bilbo (Bizkaia)</t>
+          <t>Ejecución de la obras contempladas en el proyecto de reforma para mejora de la accesibilidad en el edificio Urigain Etxea (rampa exterior y ascensor interior).</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
@@ -4698,15 +4691,12 @@
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>EUS-23560</t>
+          <t>EUS-55008</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>Proyecto Técnico para
-la legalización de la instalación eléctrica en baja
-tensión del edificio LANDABERRI de IES ORIARTE
-de Lasarte-Oria (Gipuzkoa)</t>
+          <t>Servicio de reparación de chapa y pintura de vehículos del Parque Móvil de Gobierno Vasco.</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr">
@@ -4756,12 +4746,12 @@
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>EUS-11351</t>
+          <t>EUS-40257</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>Redacción de proyecto de rehabilitación y dirección de las obras de los edificios de forja, materias primas, laminación en frío, y tren de chapa de la parcela b.10.35.5 del ámbito A.U. 35 Bellota - GS</t>
+          <t>Contrato Menor para la fabricación e instalación de una tubería para transporte de helio líquido para la Fundación Donostia International Physics Center</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
@@ -4803,8 +4793,118 @@
         </is>
       </c>
     </row>
+    <row r="78" ht="40" customHeight="1">
+      <c r="A78" s="16" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>EUS-07597</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>Contrato Menor para el servicio de una póliza de seguro para el muevo edificio de la Fundación Donostia International Physics Center</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F78" s="6" t="inlineStr"/>
+      <c r="G78" s="6" t="inlineStr"/>
+      <c r="H78" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I78" s="10" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J78" s="6" t="inlineStr"/>
+      <c r="K78" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L78" s="17" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M78" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="40" customHeight="1">
+      <c r="A79" s="16" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>EUS-57375</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>Obras de construccion de un aparcamiento de 30 bicicletas electricas (NEXT)</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F79" s="6" t="inlineStr"/>
+      <c r="G79" s="6" t="inlineStr"/>
+      <c r="H79" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I79" s="10" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J79" s="6" t="inlineStr"/>
+      <c r="K79" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L79" s="17" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M79" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:M77"/>
+  <autoFilter ref="A4:M79"/>
   <mergeCells count="5">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A5:M5"/>
@@ -4883,6 +4983,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M75" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M76" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M77" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M78" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M79" r:id="rId72"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4894,7 +4996,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1049"/>
+  <dimension ref="A1:F1079"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -16104,7 +16206,7 @@
     <row r="781" ht="30" customHeight="1">
       <c r="A781" s="18" t="inlineStr">
         <is>
-          <t>FICHA 53: EUS-04481</t>
+          <t>FICHA 53: EUS-48814</t>
         </is>
       </c>
       <c r="B781" s="19" t="n"/>
@@ -16137,7 +16239,7 @@
       </c>
       <c r="B783" s="21" t="inlineStr">
         <is>
-          <t>Mantenimiento de Infraestructuras y Jardinería en el Tramo Común, Línea 1 y Línea 2 de Metro Bilbao.</t>
+          <t>Suministro de once (11) relojes de pulsera (analogicos o inteligentes) para el Ayuntamiento de Basauri.</t>
         </is>
       </c>
       <c r="C783" s="22" t="n"/>
@@ -16153,7 +16255,7 @@
       </c>
       <c r="B784" s="21" t="inlineStr">
         <is>
-          <t>EUS-04481</t>
+          <t>EUS-48814</t>
         </is>
       </c>
       <c r="C784" s="22" t="n"/>
@@ -16305,7 +16407,7 @@
       </c>
       <c r="B794" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/mantenimiento-infraestructuras-y-jardineria-tramo-comun-linea-1-y-linea-2-metro-bilbao/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-once-11-relojes-pulsera-analogicos-o-inteligentes-ayuntamiento-basauri/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C794" s="22" t="n"/>
@@ -16316,7 +16418,7 @@
     <row r="796" ht="30" customHeight="1">
       <c r="A796" s="18" t="inlineStr">
         <is>
-          <t>FICHA 54: EUS-27303</t>
+          <t>FICHA 54: EUS-07430</t>
         </is>
       </c>
       <c r="B796" s="19" t="n"/>
@@ -16349,7 +16451,7 @@
       </c>
       <c r="B798" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
+          <t>Servicio para el desarrollo de campañas de sensibilización sobre la gestión selectiva de residuos, y en especial, para el fomento de la recogida separada de la fracción orgánica, dirigidas a la ciudad</t>
         </is>
       </c>
       <c r="C798" s="22" t="n"/>
@@ -16365,7 +16467,7 @@
       </c>
       <c r="B799" s="21" t="inlineStr">
         <is>
-          <t>EUS-27303</t>
+          <t>EUS-07430</t>
         </is>
       </c>
       <c r="C799" s="22" t="n"/>
@@ -16441,7 +16543,7 @@
       </c>
       <c r="B804" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C804" s="22" t="n"/>
@@ -16499,9 +16601,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B808" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ALTA — </t>
+      <c r="B808" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MUY ALTA — </t>
         </is>
       </c>
       <c r="C808" s="22" t="n"/>
@@ -16517,7 +16619,7 @@
       </c>
       <c r="B809" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-con-incremento-de-capacidad-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-desarrollo-campanas-sensibilizacion-gestion-selectiva-residuos-y-especial-fomento-recogida-separada-fraccion-organica-dirigidas-ciudadania-y-al-pequeno-comercio-y-hosteleria-del-municipio-basauri/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C809" s="22" t="n"/>
@@ -16528,7 +16630,7 @@
     <row r="811" ht="30" customHeight="1">
       <c r="A811" s="18" t="inlineStr">
         <is>
-          <t>FICHA 55: EUS-38413</t>
+          <t>FICHA 55: EUS-94512</t>
         </is>
       </c>
       <c r="B811" s="19" t="n"/>
@@ -16553,7 +16655,7 @@
       <c r="E812" s="22" t="n"/>
       <c r="F812" s="22" t="n"/>
     </row>
-    <row r="813" ht="20" customHeight="1">
+    <row r="813" ht="45" customHeight="1">
       <c r="A813" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -16561,7 +16663,7 @@
       </c>
       <c r="B813" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a la gestión sostenible de los recursos pesqueros 2026</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
         </is>
       </c>
       <c r="C813" s="22" t="n"/>
@@ -16577,7 +16679,7 @@
       </c>
       <c r="B814" s="21" t="inlineStr">
         <is>
-          <t>EUS-38413</t>
+          <t>EUS-94512</t>
         </is>
       </c>
       <c r="C814" s="22" t="n"/>
@@ -16729,7 +16831,7 @@
       </c>
       <c r="B824" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-gestion-sostenible-de-los-recursos-pesqueros-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-con-incremento-de-capacidad-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C824" s="22" t="n"/>
@@ -16740,7 +16842,7 @@
     <row r="826" ht="30" customHeight="1">
       <c r="A826" s="18" t="inlineStr">
         <is>
-          <t>FICHA 56: EUS-09490</t>
+          <t>FICHA 56: EUS-52245</t>
         </is>
       </c>
       <c r="B826" s="19" t="n"/>
@@ -16765,7 +16867,7 @@
       <c r="E827" s="22" t="n"/>
       <c r="F827" s="22" t="n"/>
     </row>
-    <row r="828" ht="45" customHeight="1">
+    <row r="828" ht="20" customHeight="1">
       <c r="A828" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -16773,7 +16875,7 @@
       </c>
       <c r="B828" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a la recogida de residuos con la participación de los pescadores en el mar y las playas 2026</t>
+          <t>Ayudas a la gestión sostenible de los recursos pesqueros 2026</t>
         </is>
       </c>
       <c r="C828" s="22" t="n"/>
@@ -16789,7 +16891,7 @@
       </c>
       <c r="B829" s="21" t="inlineStr">
         <is>
-          <t>EUS-09490</t>
+          <t>EUS-52245</t>
         </is>
       </c>
       <c r="C829" s="22" t="n"/>
@@ -16933,7 +17035,7 @@
       <c r="E838" s="22" t="n"/>
       <c r="F838" s="22" t="n"/>
     </row>
-    <row r="839" ht="20" customHeight="1">
+    <row r="839" ht="45" customHeight="1">
       <c r="A839" s="20" t="inlineStr">
         <is>
           <t>Enlace al portal</t>
@@ -16941,7 +17043,7 @@
       </c>
       <c r="B839" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/fempa-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-gestion-sostenible-de-los-recursos-pesqueros-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C839" s="22" t="n"/>
@@ -16952,7 +17054,7 @@
     <row r="841" ht="30" customHeight="1">
       <c r="A841" s="18" t="inlineStr">
         <is>
-          <t>FICHA 57: EUS-09919</t>
+          <t>FICHA 57: EUS-93243</t>
         </is>
       </c>
       <c r="B841" s="19" t="n"/>
@@ -16985,7 +17087,7 @@
       </c>
       <c r="B843" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático sin incremento de capacidad 2026</t>
+          <t>Ayudas a la recogida de residuos con la participación de los pescadores en el mar y las playas 2026</t>
         </is>
       </c>
       <c r="C843" s="22" t="n"/>
@@ -17001,7 +17103,7 @@
       </c>
       <c r="B844" s="21" t="inlineStr">
         <is>
-          <t>EUS-09919</t>
+          <t>EUS-93243</t>
         </is>
       </c>
       <c r="C844" s="22" t="n"/>
@@ -17145,7 +17247,7 @@
       <c r="E853" s="22" t="n"/>
       <c r="F853" s="22" t="n"/>
     </row>
-    <row r="854" ht="45" customHeight="1">
+    <row r="854" ht="20" customHeight="1">
       <c r="A854" s="20" t="inlineStr">
         <is>
           <t>Enlace al portal</t>
@@ -17153,7 +17255,7 @@
       </c>
       <c r="B854" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-sin-incremento-de-capacidad-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/fempa-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C854" s="22" t="n"/>
@@ -17164,7 +17266,7 @@
     <row r="856" ht="30" customHeight="1">
       <c r="A856" s="18" t="inlineStr">
         <is>
-          <t>FICHA 58: EUS-33827</t>
+          <t>FICHA 58: EUS-27478</t>
         </is>
       </c>
       <c r="B856" s="19" t="n"/>
@@ -17197,7 +17299,7 @@
       </c>
       <c r="B858" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio climático sin incremento de capacidad 2026</t>
         </is>
       </c>
       <c r="C858" s="22" t="n"/>
@@ -17213,7 +17315,7 @@
       </c>
       <c r="B859" s="21" t="inlineStr">
         <is>
-          <t>EUS-33827</t>
+          <t>EUS-27478</t>
         </is>
       </c>
       <c r="C859" s="22" t="n"/>
@@ -17347,9 +17449,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B868" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
+      <c r="B868" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALTA — </t>
         </is>
       </c>
       <c r="C868" s="22" t="n"/>
@@ -17365,7 +17467,7 @@
       </c>
       <c r="B869" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-contribucion-de-la-acuicultura-al-buen-estado-ambiental-y-prestacion-de-servicios-ambientales-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-sin-incremento-de-capacidad-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C869" s="22" t="n"/>
@@ -17376,7 +17478,7 @@
     <row r="871" ht="30" customHeight="1">
       <c r="A871" s="18" t="inlineStr">
         <is>
-          <t>FICHA 59: EUS-47315</t>
+          <t>FICHA 59: EUS-36149</t>
         </is>
       </c>
       <c r="B871" s="19" t="n"/>
@@ -17401,7 +17503,7 @@
       <c r="E872" s="22" t="n"/>
       <c r="F872" s="22" t="n"/>
     </row>
-    <row r="873" ht="20" customHeight="1">
+    <row r="873" ht="45" customHeight="1">
       <c r="A873" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -17409,7 +17511,7 @@
       </c>
       <c r="B873" s="21" t="inlineStr">
         <is>
-          <t>Ayudas al valor añadido, economía circular y seguridad alimentaria 2026</t>
+          <t>Elaboracion de un Plan de Comunicación y Promocion en medios digitales del Plan de Movilidad (NEXT)</t>
         </is>
       </c>
       <c r="C873" s="22" t="n"/>
@@ -17425,7 +17527,7 @@
       </c>
       <c r="B874" s="21" t="inlineStr">
         <is>
-          <t>EUS-47315</t>
+          <t>EUS-36149</t>
         </is>
       </c>
       <c r="C874" s="22" t="n"/>
@@ -17501,7 +17603,7 @@
       </c>
       <c r="B879" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C879" s="22" t="n"/>
@@ -17559,9 +17661,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B883" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
+      <c r="B883" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALTA — </t>
         </is>
       </c>
       <c r="C883" s="22" t="n"/>
@@ -17577,7 +17679,7 @@
       </c>
       <c r="B884" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-valor-anadido-economia-circular-y-seguridad-alimentaria-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/elaboracion-plan-comunicacion-y-promocion-medios-digitales-del-plan-movilidad-next/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C884" s="22" t="n"/>
@@ -17588,7 +17690,7 @@
     <row r="886" ht="30" customHeight="1">
       <c r="A886" s="18" t="inlineStr">
         <is>
-          <t>FICHA 60: EUS-97811</t>
+          <t>FICHA 60: EUS-33038</t>
         </is>
       </c>
       <c r="B886" s="19" t="n"/>
@@ -17621,7 +17723,7 @@
       </c>
       <c r="B888" s="21" t="inlineStr">
         <is>
-          <t>Vino: el Gobierno Vasco volverá a convocar este mes las ayudas al arranque o cosecha en verde del viñedo, que van a contemplar como estructurales tras reformar la UE jurídicamente su Intervención Sect</t>
+          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
         </is>
       </c>
       <c r="C888" s="22" t="n"/>
@@ -17637,7 +17739,7 @@
       </c>
       <c r="B889" s="21" t="inlineStr">
         <is>
-          <t>EUS-97811</t>
+          <t>EUS-33038</t>
         </is>
       </c>
       <c r="C889" s="22" t="n"/>
@@ -17789,7 +17891,7 @@
       </c>
       <c r="B899" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260302berdezerauztekoak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-contribucion-de-la-acuicultura-al-buen-estado-ambiental-y-prestacion-de-servicios-ambientales-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C899" s="22" t="n"/>
@@ -17800,7 +17902,7 @@
     <row r="901" ht="30" customHeight="1">
       <c r="A901" s="18" t="inlineStr">
         <is>
-          <t>FICHA 61: EUS-56533</t>
+          <t>FICHA 61: EUS-46453</t>
         </is>
       </c>
       <c r="B901" s="19" t="n"/>
@@ -17825,7 +17927,7 @@
       <c r="E902" s="22" t="n"/>
       <c r="F902" s="22" t="n"/>
     </row>
-    <row r="903" ht="45" customHeight="1">
+    <row r="903" ht="20" customHeight="1">
       <c r="A903" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -17833,7 +17935,7 @@
       </c>
       <c r="B903" s="21" t="inlineStr">
         <is>
-          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de aceleración de proyectos, a localidades de menos de 20.000 habitantes son objeto de convocatoria abierta hasta el 17.03.26. Transformacione</t>
+          <t>Ayudas al valor añadido, economía circular y seguridad alimentaria 2026</t>
         </is>
       </c>
       <c r="C903" s="22" t="n"/>
@@ -17849,7 +17951,7 @@
       </c>
       <c r="B904" s="21" t="inlineStr">
         <is>
-          <t>EUS-56533</t>
+          <t>EUS-46453</t>
         </is>
       </c>
       <c r="C904" s="22" t="n"/>
@@ -18001,7 +18103,7 @@
       </c>
       <c r="B914" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260317neboostasariak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-valor-anadido-economia-circular-y-seguridad-alimentaria-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C914" s="22" t="n"/>
@@ -18012,7 +18114,7 @@
     <row r="916" ht="30" customHeight="1">
       <c r="A916" s="18" t="inlineStr">
         <is>
-          <t>FICHA 62: EUS-02669</t>
+          <t>FICHA 62: EUS-86136</t>
         </is>
       </c>
       <c r="B916" s="19" t="n"/>
@@ -18045,7 +18147,7 @@
       </c>
       <c r="B918" s="21" t="inlineStr">
         <is>
-          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para consorcios internacionales de I+D+i. Jornada del Gobierno Vasco y con Enterprise Europe Network y otros socios. Digitalización, dispositivos,</t>
+          <t>Vino: el Gobierno Vasco volverá a convocar este mes las ayudas al arranque o cosecha en verde del viñedo, que van a contemplar como estructurales tras reformar la UE jurídicamente su Intervención Sect</t>
         </is>
       </c>
       <c r="C918" s="22" t="n"/>
@@ -18061,7 +18163,7 @@
       </c>
       <c r="B919" s="21" t="inlineStr">
         <is>
-          <t>EUS-02669</t>
+          <t>EUS-86136</t>
         </is>
       </c>
       <c r="C919" s="22" t="n"/>
@@ -18213,7 +18315,7 @@
       </c>
       <c r="B929" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260303eicihihorizon/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260302berdezerauztekoak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C929" s="22" t="n"/>
@@ -18224,7 +18326,7 @@
     <row r="931" ht="30" customHeight="1">
       <c r="A931" s="18" t="inlineStr">
         <is>
-          <t>FICHA 63: EUS-15404</t>
+          <t>FICHA 63: EUS-37235</t>
         </is>
       </c>
       <c r="B931" s="19" t="n"/>
@@ -18257,7 +18359,7 @@
       </c>
       <c r="B933" s="21" t="inlineStr">
         <is>
-          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinancia convocatorias de ayudas de las Diputaciones a explotaciones con limitaciones o desfavorecidas, y a compromisos medioambientales, climátic</t>
+          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de aceleración de proyectos, a localidades de menos de 20.000 habitantes son objeto de convocatoria abierta hasta el 17.03.26. Transformacione</t>
         </is>
       </c>
       <c r="C933" s="22" t="n"/>
@@ -18273,7 +18375,7 @@
       </c>
       <c r="B934" s="21" t="inlineStr">
         <is>
-          <t>EUS-15404</t>
+          <t>EUS-37235</t>
         </is>
       </c>
       <c r="C934" s="22" t="n"/>
@@ -18425,7 +18527,7 @@
       </c>
       <c r="B944" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/lgenfnpbgfa260218/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260317neboostasariak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C944" s="22" t="n"/>
@@ -18436,7 +18538,7 @@
     <row r="946" ht="30" customHeight="1">
       <c r="A946" s="18" t="inlineStr">
         <is>
-          <t>FICHA 64: EUS-08599</t>
+          <t>FICHA 64: EUS-41490</t>
         </is>
       </c>
       <c r="B946" s="19" t="n"/>
@@ -18469,7 +18571,7 @@
       </c>
       <c r="B948" s="21" t="inlineStr">
         <is>
-          <t>Digital Europe, Horizon (programas de la UE). Apoyos para consorcios interestatales de I+D+i. IA, robótica, cuántica, computación, ciberseguridad, electrónica, fotónica, TICs e internet avanzadas, esp</t>
+          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para consorcios internacionales de I+D+i. Jornada del Gobierno Vasco y con Enterprise Europe Network y otros socios. Digitalización, dispositivos,</t>
         </is>
       </c>
       <c r="C948" s="22" t="n"/>
@@ -18485,7 +18587,7 @@
       </c>
       <c r="B949" s="21" t="inlineStr">
         <is>
-          <t>EUS-08599</t>
+          <t>EUS-41490</t>
         </is>
       </c>
       <c r="C949" s="22" t="n"/>
@@ -18637,7 +18739,7 @@
       </c>
       <c r="B959" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260304digitalhorizoneen/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260303eicihihorizon/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C959" s="22" t="n"/>
@@ -18648,7 +18750,7 @@
     <row r="961" ht="30" customHeight="1">
       <c r="A961" s="18" t="inlineStr">
         <is>
-          <t>FICHA 65: EUS-58604</t>
+          <t>FICHA 65: EUS-03701</t>
         </is>
       </c>
       <c r="B961" s="19" t="n"/>
@@ -18673,7 +18775,7 @@
       <c r="E962" s="22" t="n"/>
       <c r="F962" s="22" t="n"/>
     </row>
-    <row r="963" ht="20" customHeight="1">
+    <row r="963" ht="45" customHeight="1">
       <c r="A963" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -18681,7 +18783,7 @@
       </c>
       <c r="B963" s="21" t="inlineStr">
         <is>
-          <t>EPIS Ropa Impermeable Jardinería</t>
+          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinancia convocatorias de ayudas de las Diputaciones a explotaciones con limitaciones o desfavorecidas, y a compromisos medioambientales, climátic</t>
         </is>
       </c>
       <c r="C963" s="22" t="n"/>
@@ -18697,7 +18799,7 @@
       </c>
       <c r="B964" s="21" t="inlineStr">
         <is>
-          <t>EUS-58604</t>
+          <t>EUS-03701</t>
         </is>
       </c>
       <c r="C964" s="22" t="n"/>
@@ -18773,7 +18875,7 @@
       </c>
       <c r="B969" s="21" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C969" s="22" t="n"/>
@@ -18849,7 +18951,7 @@
       </c>
       <c r="B974" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/epis-ropa-impermeable-jardineria/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/lgenfnpbgfa260218/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C974" s="22" t="n"/>
@@ -18860,7 +18962,7 @@
     <row r="976" ht="30" customHeight="1">
       <c r="A976" s="18" t="inlineStr">
         <is>
-          <t>FICHA 66: EUS-85654</t>
+          <t>FICHA 66: EUS-52104</t>
         </is>
       </c>
       <c r="B976" s="19" t="n"/>
@@ -18885,7 +18987,7 @@
       <c r="E977" s="22" t="n"/>
       <c r="F977" s="22" t="n"/>
     </row>
-    <row r="978" ht="20" customHeight="1">
+    <row r="978" ht="45" customHeight="1">
       <c r="A978" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -18893,7 +18995,7 @@
       </c>
       <c r="B978" s="21" t="inlineStr">
         <is>
-          <t>Ropa Laboral Tecnica Jardinería</t>
+          <t>Digital Europe, Horizon (programas de la UE). Apoyos para consorcios interestatales de I+D+i. IA, robótica, cuántica, computación, ciberseguridad, electrónica, fotónica, TICs e internet avanzadas, esp</t>
         </is>
       </c>
       <c r="C978" s="22" t="n"/>
@@ -18909,7 +19011,7 @@
       </c>
       <c r="B979" s="21" t="inlineStr">
         <is>
-          <t>EUS-85654</t>
+          <t>EUS-52104</t>
         </is>
       </c>
       <c r="C979" s="22" t="n"/>
@@ -18985,7 +19087,7 @@
       </c>
       <c r="B984" s="21" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C984" s="22" t="n"/>
@@ -19061,7 +19163,7 @@
       </c>
       <c r="B989" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/ropa-laboral-tecnica-jardineria/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260304digitalhorizoneen/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C989" s="22" t="n"/>
@@ -19072,7 +19174,7 @@
     <row r="991" ht="30" customHeight="1">
       <c r="A991" s="18" t="inlineStr">
         <is>
-          <t>FICHA 67: EUS-72988</t>
+          <t>FICHA 67: EUS-06210</t>
         </is>
       </c>
       <c r="B991" s="19" t="n"/>
@@ -19105,10 +19207,7 @@
       </c>
       <c r="B993" s="21" t="inlineStr">
         <is>
-          <t>Proyecto Técnico para
-la legalización de la instalación eléctrica en baja
-tensión del edificio LARREKOETXE de IES
-ORIARTE de Lasarte-Oria (Gipuzkoa)</t>
+          <t>Obras definidas en el Proyecto de Ejecución de reforma de la cubierta del comedor en el Colegio Santo Angel</t>
         </is>
       </c>
       <c r="C993" s="22" t="n"/>
@@ -19124,7 +19223,7 @@
       </c>
       <c r="B994" s="21" t="inlineStr">
         <is>
-          <t>EUS-72988</t>
+          <t>EUS-06210</t>
         </is>
       </c>
       <c r="C994" s="22" t="n"/>
@@ -19276,7 +19375,7 @@
       </c>
       <c r="B1004" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/proyecto-tecnico-legalizacion-instalacion-electrica-baja-tension-del-edificio-larrekoetxe-ies-oriarte-lasarte-oria-gipuzkoa/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/obras-definidas-proyecto-ejecucion-reforma-cubierta-del-comedor-colegio-santo-angel/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1004" s="22" t="n"/>
@@ -19287,7 +19386,7 @@
     <row r="1006" ht="30" customHeight="1">
       <c r="A1006" s="18" t="inlineStr">
         <is>
-          <t>FICHA 68: EUS-53698</t>
+          <t>FICHA 68: EUS-35472</t>
         </is>
       </c>
       <c r="B1006" s="19" t="n"/>
@@ -19320,11 +19419,7 @@
       </c>
       <c r="B1008" s="21" t="inlineStr">
         <is>
-          <t>Coordinación de
-seguridad y salud en las obras de sustitución y
-reparción de ventanas y reparaciòn de filtraciones
-de agua y alicatados en ARTAZUGOIKO IRALE de
-Bilbo (Bizkaia)</t>
+          <t>Ejecución de la obras contempladas en el proyecto de reforma para mejora de la accesibilidad en el edificio Urigain Etxea (rampa exterior y ascensor interior).</t>
         </is>
       </c>
       <c r="C1008" s="22" t="n"/>
@@ -19340,7 +19435,7 @@
       </c>
       <c r="B1009" s="21" t="inlineStr">
         <is>
-          <t>EUS-53698</t>
+          <t>EUS-35472</t>
         </is>
       </c>
       <c r="C1009" s="22" t="n"/>
@@ -19492,7 +19587,7 @@
       </c>
       <c r="B1019" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/coordinacion-seguridad-y-salud-obras-sustitucion-y-reparcion-ventanas-y-reparacion-filtraciones-agua-y-alicatados-artazugoiko-irale-bilbo-bizkaia/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/ejecucion-obras-contempladas-proyecto-reforma-mejora-accesibilidad-edificio-urigain-etxea-rampa-exterior-y-ascensor-interior/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1019" s="22" t="n"/>
@@ -19503,7 +19598,7 @@
     <row r="1021" ht="30" customHeight="1">
       <c r="A1021" s="18" t="inlineStr">
         <is>
-          <t>FICHA 69: EUS-23560</t>
+          <t>FICHA 69: EUS-55008</t>
         </is>
       </c>
       <c r="B1021" s="19" t="n"/>
@@ -19536,10 +19631,7 @@
       </c>
       <c r="B1023" s="21" t="inlineStr">
         <is>
-          <t>Proyecto Técnico para
-la legalización de la instalación eléctrica en baja
-tensión del edificio LANDABERRI de IES ORIARTE
-de Lasarte-Oria (Gipuzkoa)</t>
+          <t>Servicio de reparación de chapa y pintura de vehículos del Parque Móvil de Gobierno Vasco.</t>
         </is>
       </c>
       <c r="C1023" s="22" t="n"/>
@@ -19555,7 +19647,7 @@
       </c>
       <c r="B1024" s="21" t="inlineStr">
         <is>
-          <t>EUS-23560</t>
+          <t>EUS-55008</t>
         </is>
       </c>
       <c r="C1024" s="22" t="n"/>
@@ -19707,7 +19799,7 @@
       </c>
       <c r="B1034" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/proyecto-tecnico-legalizacion-instalacion-electrica-baja-tension-del-edificio-landaberri-ies-oriarte-lasarte-oria-gipuzkoa/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-reparacion-chapa-y-pintura-vehiculos-del-parque-movil-gobierno-vasco/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1034" s="22" t="n"/>
@@ -19718,7 +19810,7 @@
     <row r="1036" ht="30" customHeight="1">
       <c r="A1036" s="18" t="inlineStr">
         <is>
-          <t>FICHA 70: EUS-11351</t>
+          <t>FICHA 70: EUS-40257</t>
         </is>
       </c>
       <c r="B1036" s="19" t="n"/>
@@ -19751,7 +19843,7 @@
       </c>
       <c r="B1038" s="21" t="inlineStr">
         <is>
-          <t>Redacción de proyecto de rehabilitación y dirección de las obras de los edificios de forja, materias primas, laminación en frío, y tren de chapa de la parcela b.10.35.5 del ámbito A.U. 35 Bellota - GS</t>
+          <t>Contrato Menor para la fabricación e instalación de una tubería para transporte de helio líquido para la Fundación Donostia International Physics Center</t>
         </is>
       </c>
       <c r="C1038" s="22" t="n"/>
@@ -19767,7 +19859,7 @@
       </c>
       <c r="B1039" s="21" t="inlineStr">
         <is>
-          <t>EUS-11351</t>
+          <t>EUS-40257</t>
         </is>
       </c>
       <c r="C1039" s="22" t="n"/>
@@ -19919,7 +20011,7 @@
       </c>
       <c r="B1049" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/redaccion-proyecto-rehabilitacion-y-direccion-obras-edificios-forja-materias-primas-laminacion-frio-y-tren-chapa-parcela-b-10-35-5-del-ambito-u-35-bellota-gsb-legazpi/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/contrato-menor-fabricacion-e-instalacion-tuberia-transporte-helio-liquido-fundacion-donostia-international-physics-center/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1049" s="22" t="n"/>
@@ -19927,8 +20019,432 @@
       <c r="E1049" s="22" t="n"/>
       <c r="F1049" s="22" t="n"/>
     </row>
+    <row r="1051" ht="30" customHeight="1">
+      <c r="A1051" s="18" t="inlineStr">
+        <is>
+          <t>FICHA 71: EUS-07597</t>
+        </is>
+      </c>
+      <c r="B1051" s="19" t="n"/>
+      <c r="C1051" s="19" t="n"/>
+      <c r="D1051" s="19" t="n"/>
+      <c r="E1051" s="19" t="n"/>
+      <c r="F1051" s="19" t="n"/>
+    </row>
+    <row r="1052" ht="20" customHeight="1">
+      <c r="A1052" s="20" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1052" s="21" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1052" s="22" t="n"/>
+      <c r="D1052" s="22" t="n"/>
+      <c r="E1052" s="22" t="n"/>
+      <c r="F1052" s="22" t="n"/>
+    </row>
+    <row r="1053" ht="45" customHeight="1">
+      <c r="A1053" s="20" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1053" s="21" t="inlineStr">
+        <is>
+          <t>Contrato Menor para el servicio de una póliza de seguro para el muevo edificio de la Fundación Donostia International Physics Center</t>
+        </is>
+      </c>
+      <c r="C1053" s="22" t="n"/>
+      <c r="D1053" s="22" t="n"/>
+      <c r="E1053" s="22" t="n"/>
+      <c r="F1053" s="22" t="n"/>
+    </row>
+    <row r="1054" ht="20" customHeight="1">
+      <c r="A1054" s="20" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1054" s="21" t="inlineStr">
+        <is>
+          <t>EUS-07597</t>
+        </is>
+      </c>
+      <c r="C1054" s="22" t="n"/>
+      <c r="D1054" s="22" t="n"/>
+      <c r="E1054" s="22" t="n"/>
+      <c r="F1054" s="22" t="n"/>
+    </row>
+    <row r="1055" ht="20" customHeight="1">
+      <c r="A1055" s="20" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1055" s="21" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1055" s="22" t="n"/>
+      <c r="D1055" s="22" t="n"/>
+      <c r="E1055" s="22" t="n"/>
+      <c r="F1055" s="22" t="n"/>
+    </row>
+    <row r="1056" ht="20" customHeight="1">
+      <c r="A1056" s="20" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1056" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1056" s="22" t="n"/>
+      <c r="D1056" s="22" t="n"/>
+      <c r="E1056" s="22" t="n"/>
+      <c r="F1056" s="22" t="n"/>
+    </row>
+    <row r="1057" ht="20" customHeight="1">
+      <c r="A1057" s="20" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1057" s="21" t="inlineStr"/>
+      <c r="C1057" s="22" t="n"/>
+      <c r="D1057" s="22" t="n"/>
+      <c r="E1057" s="22" t="n"/>
+      <c r="F1057" s="22" t="n"/>
+    </row>
+    <row r="1058" ht="20" customHeight="1">
+      <c r="A1058" s="20" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1058" s="21" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1058" s="22" t="n"/>
+      <c r="D1058" s="22" t="n"/>
+      <c r="E1058" s="22" t="n"/>
+      <c r="F1058" s="22" t="n"/>
+    </row>
+    <row r="1059" ht="20" customHeight="1">
+      <c r="A1059" s="20" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1059" s="21" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1059" s="22" t="n"/>
+      <c r="D1059" s="22" t="n"/>
+      <c r="E1059" s="22" t="n"/>
+      <c r="F1059" s="22" t="n"/>
+    </row>
+    <row r="1060" ht="20" customHeight="1">
+      <c r="A1060" s="20" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1060" s="21" t="inlineStr"/>
+      <c r="C1060" s="22" t="n"/>
+      <c r="D1060" s="22" t="n"/>
+      <c r="E1060" s="22" t="n"/>
+      <c r="F1060" s="22" t="n"/>
+    </row>
+    <row r="1061" ht="20" customHeight="1">
+      <c r="A1061" s="20" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1061" s="21" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1061" s="22" t="n"/>
+      <c r="D1061" s="22" t="n"/>
+      <c r="E1061" s="22" t="n"/>
+      <c r="F1061" s="22" t="n"/>
+    </row>
+    <row r="1062" ht="20" customHeight="1">
+      <c r="A1062" s="20" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1062" s="21" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1062" s="22" t="n"/>
+      <c r="D1062" s="22" t="n"/>
+      <c r="E1062" s="22" t="n"/>
+      <c r="F1062" s="22" t="n"/>
+    </row>
+    <row r="1063" ht="20" customHeight="1">
+      <c r="A1063" s="20" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1063" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1063" s="22" t="n"/>
+      <c r="D1063" s="22" t="n"/>
+      <c r="E1063" s="22" t="n"/>
+      <c r="F1063" s="22" t="n"/>
+    </row>
+    <row r="1064" ht="45" customHeight="1">
+      <c r="A1064" s="20" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1064" s="24" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/contrato-menor-servicio-poliza-seguro-muevo-edificio-fundacion-donostia-international-physics-center/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1064" s="22" t="n"/>
+      <c r="D1064" s="22" t="n"/>
+      <c r="E1064" s="22" t="n"/>
+      <c r="F1064" s="22" t="n"/>
+    </row>
+    <row r="1066" ht="30" customHeight="1">
+      <c r="A1066" s="18" t="inlineStr">
+        <is>
+          <t>FICHA 72: EUS-57375</t>
+        </is>
+      </c>
+      <c r="B1066" s="19" t="n"/>
+      <c r="C1066" s="19" t="n"/>
+      <c r="D1066" s="19" t="n"/>
+      <c r="E1066" s="19" t="n"/>
+      <c r="F1066" s="19" t="n"/>
+    </row>
+    <row r="1067" ht="20" customHeight="1">
+      <c r="A1067" s="20" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1067" s="21" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1067" s="22" t="n"/>
+      <c r="D1067" s="22" t="n"/>
+      <c r="E1067" s="22" t="n"/>
+      <c r="F1067" s="22" t="n"/>
+    </row>
+    <row r="1068" ht="20" customHeight="1">
+      <c r="A1068" s="20" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1068" s="21" t="inlineStr">
+        <is>
+          <t>Obras de construccion de un aparcamiento de 30 bicicletas electricas (NEXT)</t>
+        </is>
+      </c>
+      <c r="C1068" s="22" t="n"/>
+      <c r="D1068" s="22" t="n"/>
+      <c r="E1068" s="22" t="n"/>
+      <c r="F1068" s="22" t="n"/>
+    </row>
+    <row r="1069" ht="20" customHeight="1">
+      <c r="A1069" s="20" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1069" s="21" t="inlineStr">
+        <is>
+          <t>EUS-57375</t>
+        </is>
+      </c>
+      <c r="C1069" s="22" t="n"/>
+      <c r="D1069" s="22" t="n"/>
+      <c r="E1069" s="22" t="n"/>
+      <c r="F1069" s="22" t="n"/>
+    </row>
+    <row r="1070" ht="20" customHeight="1">
+      <c r="A1070" s="20" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1070" s="21" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1070" s="22" t="n"/>
+      <c r="D1070" s="22" t="n"/>
+      <c r="E1070" s="22" t="n"/>
+      <c r="F1070" s="22" t="n"/>
+    </row>
+    <row r="1071" ht="20" customHeight="1">
+      <c r="A1071" s="20" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1071" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1071" s="22" t="n"/>
+      <c r="D1071" s="22" t="n"/>
+      <c r="E1071" s="22" t="n"/>
+      <c r="F1071" s="22" t="n"/>
+    </row>
+    <row r="1072" ht="20" customHeight="1">
+      <c r="A1072" s="20" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1072" s="21" t="inlineStr"/>
+      <c r="C1072" s="22" t="n"/>
+      <c r="D1072" s="22" t="n"/>
+      <c r="E1072" s="22" t="n"/>
+      <c r="F1072" s="22" t="n"/>
+    </row>
+    <row r="1073" ht="20" customHeight="1">
+      <c r="A1073" s="20" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1073" s="21" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1073" s="22" t="n"/>
+      <c r="D1073" s="22" t="n"/>
+      <c r="E1073" s="22" t="n"/>
+      <c r="F1073" s="22" t="n"/>
+    </row>
+    <row r="1074" ht="20" customHeight="1">
+      <c r="A1074" s="20" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1074" s="21" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1074" s="22" t="n"/>
+      <c r="D1074" s="22" t="n"/>
+      <c r="E1074" s="22" t="n"/>
+      <c r="F1074" s="22" t="n"/>
+    </row>
+    <row r="1075" ht="20" customHeight="1">
+      <c r="A1075" s="20" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1075" s="21" t="inlineStr"/>
+      <c r="C1075" s="22" t="n"/>
+      <c r="D1075" s="22" t="n"/>
+      <c r="E1075" s="22" t="n"/>
+      <c r="F1075" s="22" t="n"/>
+    </row>
+    <row r="1076" ht="20" customHeight="1">
+      <c r="A1076" s="20" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1076" s="21" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1076" s="22" t="n"/>
+      <c r="D1076" s="22" t="n"/>
+      <c r="E1076" s="22" t="n"/>
+      <c r="F1076" s="22" t="n"/>
+    </row>
+    <row r="1077" ht="20" customHeight="1">
+      <c r="A1077" s="20" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1077" s="21" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1077" s="22" t="n"/>
+      <c r="D1077" s="22" t="n"/>
+      <c r="E1077" s="22" t="n"/>
+      <c r="F1077" s="22" t="n"/>
+    </row>
+    <row r="1078" ht="20" customHeight="1">
+      <c r="A1078" s="20" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1078" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1078" s="22" t="n"/>
+      <c r="D1078" s="22" t="n"/>
+      <c r="E1078" s="22" t="n"/>
+      <c r="F1078" s="22" t="n"/>
+    </row>
+    <row r="1079" ht="45" customHeight="1">
+      <c r="A1079" s="20" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1079" s="24" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/obras-construccion-aparcamiento-30-bicicletas-electricas-next/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1079" s="22" t="n"/>
+      <c r="D1079" s="22" t="n"/>
+      <c r="E1079" s="22" t="n"/>
+      <c r="F1079" s="22" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="980">
+  <mergeCells count="1008">
     <mergeCell ref="B679:F679"/>
     <mergeCell ref="B666:F666"/>
     <mergeCell ref="B964:F964"/>
@@ -19997,6 +20513,7 @@
     <mergeCell ref="B1023:F1023"/>
     <mergeCell ref="B433:F433"/>
     <mergeCell ref="B233:F233"/>
+    <mergeCell ref="B1067:F1067"/>
     <mergeCell ref="B227:F227"/>
     <mergeCell ref="B531:F531"/>
     <mergeCell ref="B591:F591"/>
@@ -20013,6 +20530,7 @@
     <mergeCell ref="B655:F655"/>
     <mergeCell ref="B974:F974"/>
     <mergeCell ref="B891:F891"/>
+    <mergeCell ref="B1072:F1072"/>
     <mergeCell ref="B70:F70"/>
     <mergeCell ref="B228:F228"/>
     <mergeCell ref="B293:F293"/>
@@ -20082,6 +20600,7 @@
     <mergeCell ref="B962:F962"/>
     <mergeCell ref="A886:F886"/>
     <mergeCell ref="B505:F505"/>
+    <mergeCell ref="B1060:F1060"/>
     <mergeCell ref="B499:F499"/>
     <mergeCell ref="B299:F299"/>
     <mergeCell ref="B274:F274"/>
@@ -20097,6 +20616,7 @@
     <mergeCell ref="B559:F559"/>
     <mergeCell ref="B243:F243"/>
     <mergeCell ref="B1026:F1026"/>
+    <mergeCell ref="B1075:F1075"/>
     <mergeCell ref="B678:F678"/>
     <mergeCell ref="B363:F363"/>
     <mergeCell ref="B534:F534"/>
@@ -20106,10 +20626,12 @@
     <mergeCell ref="B957:F957"/>
     <mergeCell ref="B373:F373"/>
     <mergeCell ref="B1028:F1028"/>
+    <mergeCell ref="B1055:F1055"/>
     <mergeCell ref="B536:F536"/>
     <mergeCell ref="B834:F834"/>
     <mergeCell ref="B899:F899"/>
     <mergeCell ref="B752:F752"/>
+    <mergeCell ref="B1070:F1070"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B325:F325"/>
     <mergeCell ref="B154:F154"/>
@@ -20117,6 +20639,7 @@
     <mergeCell ref="B561:F561"/>
     <mergeCell ref="B754:F754"/>
     <mergeCell ref="B859:F859"/>
+    <mergeCell ref="B1052:F1052"/>
     <mergeCell ref="B981:F981"/>
     <mergeCell ref="B846:F846"/>
     <mergeCell ref="B973:F973"/>
@@ -20129,6 +20652,7 @@
     <mergeCell ref="B923:F923"/>
     <mergeCell ref="A571:F571"/>
     <mergeCell ref="B612:F612"/>
+    <mergeCell ref="B1054:F1054"/>
     <mergeCell ref="B910:F910"/>
     <mergeCell ref="B22:F22"/>
     <mergeCell ref="B155:F155"/>
@@ -20173,6 +20697,7 @@
     <mergeCell ref="B778:F778"/>
     <mergeCell ref="B978:F978"/>
     <mergeCell ref="B79:F79"/>
+    <mergeCell ref="B1076:F1076"/>
     <mergeCell ref="B41:F41"/>
     <mergeCell ref="B35:F35"/>
     <mergeCell ref="B302:F302"/>
@@ -20241,6 +20766,7 @@
     <mergeCell ref="B54:F54"/>
     <mergeCell ref="A286:F286"/>
     <mergeCell ref="B125:F125"/>
+    <mergeCell ref="B1073:F1073"/>
     <mergeCell ref="B185:F185"/>
     <mergeCell ref="A826:F826"/>
     <mergeCell ref="B483:F483"/>
@@ -20264,6 +20790,7 @@
     <mergeCell ref="B639:F639"/>
     <mergeCell ref="B710:F710"/>
     <mergeCell ref="B881:F881"/>
+    <mergeCell ref="B1068:F1068"/>
     <mergeCell ref="B868:F868"/>
     <mergeCell ref="B107:F107"/>
     <mergeCell ref="B641:F641"/>
@@ -20289,6 +20816,7 @@
     <mergeCell ref="B934:F934"/>
     <mergeCell ref="B173:F173"/>
     <mergeCell ref="B999:F999"/>
+    <mergeCell ref="B1061:F1061"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="A46:F46"/>
     <mergeCell ref="B507:F507"/>
@@ -20303,6 +20831,7 @@
     <mergeCell ref="B473:F473"/>
     <mergeCell ref="B273:F273"/>
     <mergeCell ref="B857:F857"/>
+    <mergeCell ref="B1063:F1063"/>
     <mergeCell ref="B807:F807"/>
     <mergeCell ref="B1000:F1000"/>
     <mergeCell ref="B39:F39"/>
@@ -20378,6 +20907,7 @@
     <mergeCell ref="B877:F877"/>
     <mergeCell ref="B815:F815"/>
     <mergeCell ref="B597:F597"/>
+    <mergeCell ref="B1064:F1064"/>
     <mergeCell ref="B103:F103"/>
     <mergeCell ref="B78:F78"/>
     <mergeCell ref="B833:F833"/>
@@ -20446,6 +20976,7 @@
     <mergeCell ref="B892:F892"/>
     <mergeCell ref="B53:F53"/>
     <mergeCell ref="A436:F436"/>
+    <mergeCell ref="B1079:F1079"/>
     <mergeCell ref="A121:F121"/>
     <mergeCell ref="B289:F289"/>
     <mergeCell ref="A721:F721"/>
@@ -20523,6 +21054,7 @@
     <mergeCell ref="B239:F239"/>
     <mergeCell ref="B310:F310"/>
     <mergeCell ref="B372:F372"/>
+    <mergeCell ref="B1071:F1071"/>
     <mergeCell ref="B608:F608"/>
     <mergeCell ref="B595:F595"/>
     <mergeCell ref="B1037:F1037"/>
@@ -20541,6 +21073,7 @@
     <mergeCell ref="B513:F513"/>
     <mergeCell ref="B684:F684"/>
     <mergeCell ref="B982:F982"/>
+    <mergeCell ref="B1053:F1053"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="B847:F847"/>
     <mergeCell ref="B263:F263"/>
@@ -20615,6 +21148,7 @@
     <mergeCell ref="B77:F77"/>
     <mergeCell ref="B903:F903"/>
     <mergeCell ref="B965:F965"/>
+    <mergeCell ref="B1074:F1074"/>
     <mergeCell ref="B440:F440"/>
     <mergeCell ref="B611:F611"/>
     <mergeCell ref="B598:F598"/>
@@ -20638,6 +21172,7 @@
     <mergeCell ref="B614:F614"/>
     <mergeCell ref="A511:F511"/>
     <mergeCell ref="B785:F785"/>
+    <mergeCell ref="B1056:F1056"/>
     <mergeCell ref="B24:F24"/>
     <mergeCell ref="B850:F850"/>
     <mergeCell ref="B95:F95"/>
@@ -20656,6 +21191,7 @@
     <mergeCell ref="B987:F987"/>
     <mergeCell ref="B787:F787"/>
     <mergeCell ref="B32:F32"/>
+    <mergeCell ref="B1058:F1058"/>
     <mergeCell ref="B914:F914"/>
     <mergeCell ref="B197:F197"/>
     <mergeCell ref="B26:F26"/>
@@ -20674,10 +21210,12 @@
     <mergeCell ref="B845:F845"/>
     <mergeCell ref="B261:F261"/>
     <mergeCell ref="B184:F184"/>
+    <mergeCell ref="B1062:F1062"/>
     <mergeCell ref="A301:F301"/>
     <mergeCell ref="B27:F27"/>
     <mergeCell ref="B782:F782"/>
     <mergeCell ref="A331:F331"/>
+    <mergeCell ref="B1069:F1069"/>
     <mergeCell ref="B548:F548"/>
     <mergeCell ref="B42:F42"/>
     <mergeCell ref="A616:F616"/>
@@ -20726,12 +21264,14 @@
     <mergeCell ref="B497:F497"/>
     <mergeCell ref="B1033:F1033"/>
     <mergeCell ref="B983:F983"/>
+    <mergeCell ref="A1051:F1051"/>
     <mergeCell ref="B970:F970"/>
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="B355:F355"/>
     <mergeCell ref="B134:F134"/>
     <mergeCell ref="B572:F572"/>
     <mergeCell ref="B759:F759"/>
+    <mergeCell ref="B1057:F1057"/>
     <mergeCell ref="B357:F357"/>
     <mergeCell ref="B995:F995"/>
     <mergeCell ref="B96:F96"/>
@@ -20746,6 +21286,7 @@
     <mergeCell ref="B111:F111"/>
     <mergeCell ref="B617:F617"/>
     <mergeCell ref="B937:F937"/>
+    <mergeCell ref="B1059:F1059"/>
     <mergeCell ref="B853:F853"/>
     <mergeCell ref="B98:F98"/>
     <mergeCell ref="B986:F986"/>
@@ -20766,6 +21307,7 @@
     <mergeCell ref="A466:F466"/>
     <mergeCell ref="B696:F696"/>
     <mergeCell ref="B867:F867"/>
+    <mergeCell ref="A1066:F1066"/>
     <mergeCell ref="B269:F269"/>
     <mergeCell ref="B187:F187"/>
     <mergeCell ref="B485:F485"/>
@@ -20776,6 +21318,7 @@
     <mergeCell ref="B493:F493"/>
     <mergeCell ref="B216:F216"/>
     <mergeCell ref="B487:F487"/>
+    <mergeCell ref="B1077:F1077"/>
     <mergeCell ref="B343:F343"/>
     <mergeCell ref="B414:F414"/>
     <mergeCell ref="B474:F474"/>
@@ -20863,6 +21406,7 @@
     <mergeCell ref="A406:F406"/>
     <mergeCell ref="B951:F951"/>
     <mergeCell ref="B130:F130"/>
+    <mergeCell ref="B1078:F1078"/>
     <mergeCell ref="A946:F946"/>
     <mergeCell ref="A631:F631"/>
     <mergeCell ref="B117:F117"/>
@@ -20981,6 +21525,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1019" r:id="rId68"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1034" r:id="rId69"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1049" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1064" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1079" r:id="rId72"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -20992,7 +21538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J71"/>
+  <dimension ref="A1:J73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -23026,12 +23572,12 @@
     <row r="54" ht="28" customHeight="1">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>EUS-04481</t>
+          <t>EUS-48814</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>Mantenimiento de Infraestructuras y Jardinería en el Tramo C</t>
+          <t>Suministro de once (11) relojes de pulsera (analogicos o int</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
@@ -23062,12 +23608,12 @@
     <row r="55" ht="28" customHeight="1">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>EUS-27303</t>
+          <t>EUS-07430</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
+          <t>Servicio para el desarrollo de campañas de sensibilización s</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
@@ -23083,7 +23629,7 @@
       <c r="E55" s="6" t="inlineStr"/>
       <c r="F55" s="27" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>MUY ALTA</t>
         </is>
       </c>
       <c r="G55" s="6" t="inlineStr"/>
@@ -23098,12 +23644,12 @@
     <row r="56" ht="28" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>EUS-38413</t>
+          <t>EUS-94512</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la gestión sostenible de los recursos pesqueros 202</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
@@ -23134,12 +23680,12 @@
     <row r="57" ht="28" customHeight="1">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>EUS-09490</t>
+          <t>EUS-52245</t>
         </is>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la recogida de residuos con la participación de los</t>
+          <t>Ayudas a la gestión sostenible de los recursos pesqueros 202</t>
         </is>
       </c>
       <c r="C57" s="6" t="inlineStr">
@@ -23170,12 +23716,12 @@
     <row r="58" ht="28" customHeight="1">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>EUS-09919</t>
+          <t>EUS-93243</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
+          <t>Ayudas a la recogida de residuos con la participación de los</t>
         </is>
       </c>
       <c r="C58" s="6" t="inlineStr">
@@ -23206,12 +23752,12 @@
     <row r="59" ht="28" customHeight="1">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>EUS-33827</t>
+          <t>EUS-27478</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la contribución de la acuicultura al buen estado am</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
@@ -23227,7 +23773,7 @@
       <c r="E59" s="6" t="inlineStr"/>
       <c r="F59" s="27" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="G59" s="6" t="inlineStr"/>
@@ -23242,12 +23788,12 @@
     <row r="60" ht="28" customHeight="1">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>EUS-47315</t>
+          <t>EUS-36149</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>Ayudas al valor añadido, economía circular y seguridad alime</t>
+          <t>Elaboracion de un Plan de Comunicación y Promocion en medios</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
@@ -23263,7 +23809,7 @@
       <c r="E60" s="6" t="inlineStr"/>
       <c r="F60" s="27" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="G60" s="6" t="inlineStr"/>
@@ -23278,12 +23824,12 @@
     <row r="61" ht="28" customHeight="1">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>EUS-97811</t>
+          <t>EUS-33038</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>Vino: el Gobierno Vasco volverá a convocar este mes las ayud</t>
+          <t>Ayudas a la contribución de la acuicultura al buen estado am</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
@@ -23314,12 +23860,12 @@
     <row r="62" ht="28" customHeight="1">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>EUS-56533</t>
+          <t>EUS-46453</t>
         </is>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de</t>
+          <t>Ayudas al valor añadido, economía circular y seguridad alime</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
@@ -23350,12 +23896,12 @@
     <row r="63" ht="28" customHeight="1">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>EUS-02669</t>
+          <t>EUS-86136</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para c</t>
+          <t>Vino: el Gobierno Vasco volverá a convocar este mes las ayud</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
@@ -23386,12 +23932,12 @@
     <row r="64" ht="28" customHeight="1">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>EUS-15404</t>
+          <t>EUS-37235</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinanc</t>
+          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
@@ -23422,12 +23968,12 @@
     <row r="65" ht="28" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>EUS-08599</t>
+          <t>EUS-41490</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>Digital Europe, Horizon (programas de la UE). Apoyos para co</t>
+          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para c</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -23458,12 +24004,12 @@
     <row r="66" ht="28" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>EUS-58604</t>
+          <t>EUS-03701</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>EPIS Ropa Impermeable Jardinería</t>
+          <t>FEADER, Fondo Europeo Agrícola de Desarrollo Rural, cofinanc</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
@@ -23494,12 +24040,12 @@
     <row r="67" ht="28" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>EUS-85654</t>
+          <t>EUS-52104</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>Ropa Laboral Tecnica Jardinería</t>
+          <t>Digital Europe, Horizon (programas de la UE). Apoyos para co</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
@@ -23530,13 +24076,12 @@
     <row r="68" ht="28" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>EUS-72988</t>
+          <t>EUS-06210</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>Proyecto Técnico para
-la legalización de la instalación eléc</t>
+          <t>Obras definidas en el Proyecto de Ejecución de reforma de la</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -23567,13 +24112,12 @@
     <row r="69" ht="28" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>EUS-53698</t>
+          <t>EUS-35472</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>Coordinación de
-seguridad y salud en las obras de sustitució</t>
+          <t>Ejecución de la obras contempladas en el proyecto de reforma</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -23604,13 +24148,12 @@
     <row r="70" ht="28" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>EUS-23560</t>
+          <t>EUS-55008</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>Proyecto Técnico para
-la legalización de la instalación eléc</t>
+          <t>Servicio de reparación de chapa y pintura de vehículos del P</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -23641,12 +24184,12 @@
     <row r="71" ht="28" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>EUS-11351</t>
+          <t>EUS-40257</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>Redacción de proyecto de rehabilitación y dirección de las o</t>
+          <t>Contrato Menor para la fabricación e instalación de una tube</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -23674,8 +24217,80 @@
       <c r="I71" s="6" t="inlineStr"/>
       <c r="J71" s="6" t="inlineStr"/>
     </row>
+    <row r="72" ht="28" customHeight="1">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>EUS-07597</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>Contrato Menor para el servicio de una póliza de seguro para</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D72" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E72" s="6" t="inlineStr"/>
+      <c r="F72" s="27" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G72" s="6" t="inlineStr"/>
+      <c r="H72" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I72" s="6" t="inlineStr"/>
+      <c r="J72" s="6" t="inlineStr"/>
+    </row>
+    <row r="73" ht="28" customHeight="1">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t>EUS-57375</t>
+        </is>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>Obras de construccion de un aparcamiento de 30 bicicletas el</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D73" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E73" s="6" t="inlineStr"/>
+      <c r="F73" s="27" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G73" s="6" t="inlineStr"/>
+      <c r="H73" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I73" s="6" t="inlineStr"/>
+      <c r="J73" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J71"/>
+  <autoFilter ref="A1:J73"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update funding data 2026-04-04
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -685,7 +685,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 03/04/2026 06:57 - 120 convocatorias - 19 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 04/04/2026 06:47 - 120 convocatorias - 19 nuevas</t>
         </is>
       </c>
     </row>
@@ -6901,7 +6901,7 @@
       </c>
       <c r="B108" s="6" t="inlineStr">
         <is>
-          <t>EUS-46178</t>
+          <t>EUS-77758</t>
         </is>
       </c>
       <c r="C108" s="6" t="inlineStr">
@@ -6956,7 +6956,7 @@
       </c>
       <c r="B109" s="6" t="inlineStr">
         <is>
-          <t>EUS-26244</t>
+          <t>EUS-52578</t>
         </is>
       </c>
       <c r="C109" s="6" t="inlineStr">
@@ -7011,7 +7011,7 @@
       </c>
       <c r="B110" s="6" t="inlineStr">
         <is>
-          <t>EUS-99399</t>
+          <t>EUS-40394</t>
         </is>
       </c>
       <c r="C110" s="6" t="inlineStr">
@@ -7066,7 +7066,7 @@
       </c>
       <c r="B111" s="6" t="inlineStr">
         <is>
-          <t>EUS-45301</t>
+          <t>EUS-24034</t>
         </is>
       </c>
       <c r="C111" s="6" t="inlineStr">
@@ -7121,7 +7121,7 @@
       </c>
       <c r="B112" s="6" t="inlineStr">
         <is>
-          <t>EUS-86016</t>
+          <t>EUS-61908</t>
         </is>
       </c>
       <c r="C112" s="6" t="inlineStr">
@@ -7176,7 +7176,7 @@
       </c>
       <c r="B113" s="6" t="inlineStr">
         <is>
-          <t>EUS-41191</t>
+          <t>EUS-51546</t>
         </is>
       </c>
       <c r="C113" s="6" t="inlineStr">
@@ -7231,7 +7231,7 @@
       </c>
       <c r="B114" s="6" t="inlineStr">
         <is>
-          <t>EUS-90152</t>
+          <t>EUS-21402</t>
         </is>
       </c>
       <c r="C114" s="6" t="inlineStr">
@@ -7286,7 +7286,7 @@
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>EUS-27615</t>
+          <t>EUS-98709</t>
         </is>
       </c>
       <c r="C115" s="6" t="inlineStr">
@@ -7341,7 +7341,7 @@
       </c>
       <c r="B116" s="6" t="inlineStr">
         <is>
-          <t>EUS-65967</t>
+          <t>EUS-70083</t>
         </is>
       </c>
       <c r="C116" s="6" t="inlineStr">
@@ -7396,7 +7396,7 @@
       </c>
       <c r="B117" s="6" t="inlineStr">
         <is>
-          <t>EUS-53340</t>
+          <t>EUS-45246</t>
         </is>
       </c>
       <c r="C117" s="6" t="inlineStr">
@@ -7451,7 +7451,7 @@
       </c>
       <c r="B118" s="6" t="inlineStr">
         <is>
-          <t>EUS-62231</t>
+          <t>EUS-05455</t>
         </is>
       </c>
       <c r="C118" s="6" t="inlineStr">
@@ -7506,7 +7506,7 @@
       </c>
       <c r="B119" s="6" t="inlineStr">
         <is>
-          <t>EUS-80144</t>
+          <t>EUS-26630</t>
         </is>
       </c>
       <c r="C119" s="6" t="inlineStr">
@@ -7561,7 +7561,7 @@
       </c>
       <c r="B120" s="6" t="inlineStr">
         <is>
-          <t>EUS-06334</t>
+          <t>EUS-49660</t>
         </is>
       </c>
       <c r="C120" s="6" t="inlineStr">
@@ -7616,7 +7616,7 @@
       </c>
       <c r="B121" s="6" t="inlineStr">
         <is>
-          <t>EUS-79115</t>
+          <t>EUS-28074</t>
         </is>
       </c>
       <c r="C121" s="6" t="inlineStr">
@@ -7671,7 +7671,7 @@
       </c>
       <c r="B122" s="6" t="inlineStr">
         <is>
-          <t>EUS-72311</t>
+          <t>EUS-29222</t>
         </is>
       </c>
       <c r="C122" s="6" t="inlineStr">
@@ -7726,7 +7726,7 @@
       </c>
       <c r="B123" s="6" t="inlineStr">
         <is>
-          <t>EUS-74211</t>
+          <t>EUS-24918</t>
         </is>
       </c>
       <c r="C123" s="6" t="inlineStr">
@@ -7781,7 +7781,7 @@
       </c>
       <c r="B124" s="6" t="inlineStr">
         <is>
-          <t>EUS-79764</t>
+          <t>EUS-03691</t>
         </is>
       </c>
       <c r="C124" s="6" t="inlineStr">
@@ -7836,7 +7836,7 @@
       </c>
       <c r="B125" s="6" t="inlineStr">
         <is>
-          <t>EUS-37095</t>
+          <t>EUS-47441</t>
         </is>
       </c>
       <c r="C125" s="6" t="inlineStr">
@@ -7891,7 +7891,7 @@
       </c>
       <c r="B126" s="6" t="inlineStr">
         <is>
-          <t>EUS-43093</t>
+          <t>EUS-64744</t>
         </is>
       </c>
       <c r="C126" s="6" t="inlineStr">
@@ -29972,7 +29972,7 @@
     <row r="1516" ht="30" customHeight="1">
       <c r="A1516" s="16" t="inlineStr">
         <is>
-          <t>FICHA 102: EUS-46178</t>
+          <t>FICHA 102: EUS-77758</t>
         </is>
       </c>
       <c r="B1516" s="17" t="n"/>
@@ -30021,7 +30021,7 @@
       </c>
       <c r="B1519" s="19" t="inlineStr">
         <is>
-          <t>EUS-46178</t>
+          <t>EUS-77758</t>
         </is>
       </c>
       <c r="C1519" s="20" t="n"/>
@@ -30184,7 +30184,7 @@
     <row r="1531" ht="30" customHeight="1">
       <c r="A1531" s="16" t="inlineStr">
         <is>
-          <t>FICHA 103: EUS-26244</t>
+          <t>FICHA 103: EUS-52578</t>
         </is>
       </c>
       <c r="B1531" s="17" t="n"/>
@@ -30233,7 +30233,7 @@
       </c>
       <c r="B1534" s="19" t="inlineStr">
         <is>
-          <t>EUS-26244</t>
+          <t>EUS-52578</t>
         </is>
       </c>
       <c r="C1534" s="20" t="n"/>
@@ -30396,7 +30396,7 @@
     <row r="1546" ht="30" customHeight="1">
       <c r="A1546" s="16" t="inlineStr">
         <is>
-          <t>FICHA 104: EUS-99399</t>
+          <t>FICHA 104: EUS-40394</t>
         </is>
       </c>
       <c r="B1546" s="17" t="n"/>
@@ -30445,7 +30445,7 @@
       </c>
       <c r="B1549" s="19" t="inlineStr">
         <is>
-          <t>EUS-99399</t>
+          <t>EUS-40394</t>
         </is>
       </c>
       <c r="C1549" s="20" t="n"/>
@@ -30608,7 +30608,7 @@
     <row r="1561" ht="30" customHeight="1">
       <c r="A1561" s="16" t="inlineStr">
         <is>
-          <t>FICHA 105: EUS-45301</t>
+          <t>FICHA 105: EUS-24034</t>
         </is>
       </c>
       <c r="B1561" s="17" t="n"/>
@@ -30657,7 +30657,7 @@
       </c>
       <c r="B1564" s="19" t="inlineStr">
         <is>
-          <t>EUS-45301</t>
+          <t>EUS-24034</t>
         </is>
       </c>
       <c r="C1564" s="20" t="n"/>
@@ -30820,7 +30820,7 @@
     <row r="1576" ht="30" customHeight="1">
       <c r="A1576" s="16" t="inlineStr">
         <is>
-          <t>FICHA 106: EUS-86016</t>
+          <t>FICHA 106: EUS-61908</t>
         </is>
       </c>
       <c r="B1576" s="17" t="n"/>
@@ -30869,7 +30869,7 @@
       </c>
       <c r="B1579" s="19" t="inlineStr">
         <is>
-          <t>EUS-86016</t>
+          <t>EUS-61908</t>
         </is>
       </c>
       <c r="C1579" s="20" t="n"/>
@@ -31032,7 +31032,7 @@
     <row r="1591" ht="30" customHeight="1">
       <c r="A1591" s="16" t="inlineStr">
         <is>
-          <t>FICHA 107: EUS-41191</t>
+          <t>FICHA 107: EUS-51546</t>
         </is>
       </c>
       <c r="B1591" s="17" t="n"/>
@@ -31081,7 +31081,7 @@
       </c>
       <c r="B1594" s="19" t="inlineStr">
         <is>
-          <t>EUS-41191</t>
+          <t>EUS-51546</t>
         </is>
       </c>
       <c r="C1594" s="20" t="n"/>
@@ -31244,7 +31244,7 @@
     <row r="1606" ht="30" customHeight="1">
       <c r="A1606" s="16" t="inlineStr">
         <is>
-          <t>FICHA 108: EUS-90152</t>
+          <t>FICHA 108: EUS-21402</t>
         </is>
       </c>
       <c r="B1606" s="17" t="n"/>
@@ -31293,7 +31293,7 @@
       </c>
       <c r="B1609" s="19" t="inlineStr">
         <is>
-          <t>EUS-90152</t>
+          <t>EUS-21402</t>
         </is>
       </c>
       <c r="C1609" s="20" t="n"/>
@@ -31456,7 +31456,7 @@
     <row r="1621" ht="30" customHeight="1">
       <c r="A1621" s="16" t="inlineStr">
         <is>
-          <t>FICHA 109: EUS-27615</t>
+          <t>FICHA 109: EUS-98709</t>
         </is>
       </c>
       <c r="B1621" s="17" t="n"/>
@@ -31505,7 +31505,7 @@
       </c>
       <c r="B1624" s="19" t="inlineStr">
         <is>
-          <t>EUS-27615</t>
+          <t>EUS-98709</t>
         </is>
       </c>
       <c r="C1624" s="20" t="n"/>
@@ -31668,7 +31668,7 @@
     <row r="1636" ht="30" customHeight="1">
       <c r="A1636" s="16" t="inlineStr">
         <is>
-          <t>FICHA 110: EUS-65967</t>
+          <t>FICHA 110: EUS-70083</t>
         </is>
       </c>
       <c r="B1636" s="17" t="n"/>
@@ -31717,7 +31717,7 @@
       </c>
       <c r="B1639" s="19" t="inlineStr">
         <is>
-          <t>EUS-65967</t>
+          <t>EUS-70083</t>
         </is>
       </c>
       <c r="C1639" s="20" t="n"/>
@@ -31880,7 +31880,7 @@
     <row r="1651" ht="30" customHeight="1">
       <c r="A1651" s="16" t="inlineStr">
         <is>
-          <t>FICHA 111: EUS-53340</t>
+          <t>FICHA 111: EUS-45246</t>
         </is>
       </c>
       <c r="B1651" s="17" t="n"/>
@@ -31929,7 +31929,7 @@
       </c>
       <c r="B1654" s="19" t="inlineStr">
         <is>
-          <t>EUS-53340</t>
+          <t>EUS-45246</t>
         </is>
       </c>
       <c r="C1654" s="20" t="n"/>
@@ -32092,7 +32092,7 @@
     <row r="1666" ht="30" customHeight="1">
       <c r="A1666" s="16" t="inlineStr">
         <is>
-          <t>FICHA 112: EUS-62231</t>
+          <t>FICHA 112: EUS-05455</t>
         </is>
       </c>
       <c r="B1666" s="17" t="n"/>
@@ -32141,7 +32141,7 @@
       </c>
       <c r="B1669" s="19" t="inlineStr">
         <is>
-          <t>EUS-62231</t>
+          <t>EUS-05455</t>
         </is>
       </c>
       <c r="C1669" s="20" t="n"/>
@@ -32304,7 +32304,7 @@
     <row r="1681" ht="30" customHeight="1">
       <c r="A1681" s="16" t="inlineStr">
         <is>
-          <t>FICHA 113: EUS-80144</t>
+          <t>FICHA 113: EUS-26630</t>
         </is>
       </c>
       <c r="B1681" s="17" t="n"/>
@@ -32353,7 +32353,7 @@
       </c>
       <c r="B1684" s="19" t="inlineStr">
         <is>
-          <t>EUS-80144</t>
+          <t>EUS-26630</t>
         </is>
       </c>
       <c r="C1684" s="20" t="n"/>
@@ -32516,7 +32516,7 @@
     <row r="1696" ht="30" customHeight="1">
       <c r="A1696" s="16" t="inlineStr">
         <is>
-          <t>FICHA 114: EUS-06334</t>
+          <t>FICHA 114: EUS-49660</t>
         </is>
       </c>
       <c r="B1696" s="17" t="n"/>
@@ -32565,7 +32565,7 @@
       </c>
       <c r="B1699" s="19" t="inlineStr">
         <is>
-          <t>EUS-06334</t>
+          <t>EUS-49660</t>
         </is>
       </c>
       <c r="C1699" s="20" t="n"/>
@@ -32728,7 +32728,7 @@
     <row r="1711" ht="30" customHeight="1">
       <c r="A1711" s="16" t="inlineStr">
         <is>
-          <t>FICHA 115: EUS-79115</t>
+          <t>FICHA 115: EUS-28074</t>
         </is>
       </c>
       <c r="B1711" s="17" t="n"/>
@@ -32777,7 +32777,7 @@
       </c>
       <c r="B1714" s="19" t="inlineStr">
         <is>
-          <t>EUS-79115</t>
+          <t>EUS-28074</t>
         </is>
       </c>
       <c r="C1714" s="20" t="n"/>
@@ -32940,7 +32940,7 @@
     <row r="1726" ht="30" customHeight="1">
       <c r="A1726" s="16" t="inlineStr">
         <is>
-          <t>FICHA 116: EUS-72311</t>
+          <t>FICHA 116: EUS-29222</t>
         </is>
       </c>
       <c r="B1726" s="17" t="n"/>
@@ -32989,7 +32989,7 @@
       </c>
       <c r="B1729" s="19" t="inlineStr">
         <is>
-          <t>EUS-72311</t>
+          <t>EUS-29222</t>
         </is>
       </c>
       <c r="C1729" s="20" t="n"/>
@@ -33152,7 +33152,7 @@
     <row r="1741" ht="30" customHeight="1">
       <c r="A1741" s="16" t="inlineStr">
         <is>
-          <t>FICHA 117: EUS-74211</t>
+          <t>FICHA 117: EUS-24918</t>
         </is>
       </c>
       <c r="B1741" s="17" t="n"/>
@@ -33201,7 +33201,7 @@
       </c>
       <c r="B1744" s="19" t="inlineStr">
         <is>
-          <t>EUS-74211</t>
+          <t>EUS-24918</t>
         </is>
       </c>
       <c r="C1744" s="20" t="n"/>
@@ -33364,7 +33364,7 @@
     <row r="1756" ht="30" customHeight="1">
       <c r="A1756" s="16" t="inlineStr">
         <is>
-          <t>FICHA 118: EUS-79764</t>
+          <t>FICHA 118: EUS-03691</t>
         </is>
       </c>
       <c r="B1756" s="17" t="n"/>
@@ -33413,7 +33413,7 @@
       </c>
       <c r="B1759" s="19" t="inlineStr">
         <is>
-          <t>EUS-79764</t>
+          <t>EUS-03691</t>
         </is>
       </c>
       <c r="C1759" s="20" t="n"/>
@@ -33576,7 +33576,7 @@
     <row r="1771" ht="30" customHeight="1">
       <c r="A1771" s="16" t="inlineStr">
         <is>
-          <t>FICHA 119: EUS-37095</t>
+          <t>FICHA 119: EUS-47441</t>
         </is>
       </c>
       <c r="B1771" s="17" t="n"/>
@@ -33625,7 +33625,7 @@
       </c>
       <c r="B1774" s="19" t="inlineStr">
         <is>
-          <t>EUS-37095</t>
+          <t>EUS-47441</t>
         </is>
       </c>
       <c r="C1774" s="20" t="n"/>
@@ -33788,7 +33788,7 @@
     <row r="1786" ht="30" customHeight="1">
       <c r="A1786" s="16" t="inlineStr">
         <is>
-          <t>FICHA 120: EUS-43093</t>
+          <t>FICHA 120: EUS-64744</t>
         </is>
       </c>
       <c r="B1786" s="17" t="n"/>
@@ -33837,7 +33837,7 @@
       </c>
       <c r="B1789" s="19" t="inlineStr">
         <is>
-          <t>EUS-43093</t>
+          <t>EUS-64744</t>
         </is>
       </c>
       <c r="C1789" s="20" t="n"/>
@@ -39818,7 +39818,7 @@
     <row r="103" ht="28" customHeight="1">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>EUS-46178</t>
+          <t>EUS-77758</t>
         </is>
       </c>
       <c r="B103" s="6" t="inlineStr">
@@ -39854,7 +39854,7 @@
     <row r="104" ht="28" customHeight="1">
       <c r="A104" s="6" t="inlineStr">
         <is>
-          <t>EUS-26244</t>
+          <t>EUS-52578</t>
         </is>
       </c>
       <c r="B104" s="6" t="inlineStr">
@@ -39890,7 +39890,7 @@
     <row r="105" ht="28" customHeight="1">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>EUS-99399</t>
+          <t>EUS-40394</t>
         </is>
       </c>
       <c r="B105" s="6" t="inlineStr">
@@ -39926,7 +39926,7 @@
     <row r="106" ht="28" customHeight="1">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>EUS-45301</t>
+          <t>EUS-24034</t>
         </is>
       </c>
       <c r="B106" s="6" t="inlineStr">
@@ -39962,7 +39962,7 @@
     <row r="107" ht="28" customHeight="1">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>EUS-86016</t>
+          <t>EUS-61908</t>
         </is>
       </c>
       <c r="B107" s="6" t="inlineStr">
@@ -39998,7 +39998,7 @@
     <row r="108" ht="28" customHeight="1">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>EUS-41191</t>
+          <t>EUS-51546</t>
         </is>
       </c>
       <c r="B108" s="6" t="inlineStr">
@@ -40034,7 +40034,7 @@
     <row r="109" ht="28" customHeight="1">
       <c r="A109" s="6" t="inlineStr">
         <is>
-          <t>EUS-90152</t>
+          <t>EUS-21402</t>
         </is>
       </c>
       <c r="B109" s="6" t="inlineStr">
@@ -40070,7 +40070,7 @@
     <row r="110" ht="28" customHeight="1">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>EUS-27615</t>
+          <t>EUS-98709</t>
         </is>
       </c>
       <c r="B110" s="6" t="inlineStr">
@@ -40106,7 +40106,7 @@
     <row r="111" ht="28" customHeight="1">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>EUS-65967</t>
+          <t>EUS-70083</t>
         </is>
       </c>
       <c r="B111" s="6" t="inlineStr">
@@ -40142,7 +40142,7 @@
     <row r="112" ht="28" customHeight="1">
       <c r="A112" s="6" t="inlineStr">
         <is>
-          <t>EUS-53340</t>
+          <t>EUS-45246</t>
         </is>
       </c>
       <c r="B112" s="6" t="inlineStr">
@@ -40178,7 +40178,7 @@
     <row r="113" ht="28" customHeight="1">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>EUS-62231</t>
+          <t>EUS-05455</t>
         </is>
       </c>
       <c r="B113" s="6" t="inlineStr">
@@ -40214,7 +40214,7 @@
     <row r="114" ht="28" customHeight="1">
       <c r="A114" s="6" t="inlineStr">
         <is>
-          <t>EUS-80144</t>
+          <t>EUS-26630</t>
         </is>
       </c>
       <c r="B114" s="6" t="inlineStr">
@@ -40250,7 +40250,7 @@
     <row r="115" ht="28" customHeight="1">
       <c r="A115" s="6" t="inlineStr">
         <is>
-          <t>EUS-06334</t>
+          <t>EUS-49660</t>
         </is>
       </c>
       <c r="B115" s="6" t="inlineStr">
@@ -40286,7 +40286,7 @@
     <row r="116" ht="28" customHeight="1">
       <c r="A116" s="6" t="inlineStr">
         <is>
-          <t>EUS-79115</t>
+          <t>EUS-28074</t>
         </is>
       </c>
       <c r="B116" s="6" t="inlineStr">
@@ -40322,7 +40322,7 @@
     <row r="117" ht="28" customHeight="1">
       <c r="A117" s="6" t="inlineStr">
         <is>
-          <t>EUS-72311</t>
+          <t>EUS-29222</t>
         </is>
       </c>
       <c r="B117" s="6" t="inlineStr">
@@ -40358,7 +40358,7 @@
     <row r="118" ht="28" customHeight="1">
       <c r="A118" s="6" t="inlineStr">
         <is>
-          <t>EUS-74211</t>
+          <t>EUS-24918</t>
         </is>
       </c>
       <c r="B118" s="6" t="inlineStr">
@@ -40394,7 +40394,7 @@
     <row r="119" ht="28" customHeight="1">
       <c r="A119" s="6" t="inlineStr">
         <is>
-          <t>EUS-79764</t>
+          <t>EUS-03691</t>
         </is>
       </c>
       <c r="B119" s="6" t="inlineStr">
@@ -40430,7 +40430,7 @@
     <row r="120" ht="28" customHeight="1">
       <c r="A120" s="6" t="inlineStr">
         <is>
-          <t>EUS-37095</t>
+          <t>EUS-47441</t>
         </is>
       </c>
       <c r="B120" s="6" t="inlineStr">
@@ -40466,7 +40466,7 @@
     <row r="121" ht="28" customHeight="1">
       <c r="A121" s="6" t="inlineStr">
         <is>
-          <t>EUS-43093</t>
+          <t>EUS-64744</t>
         </is>
       </c>
       <c r="B121" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Update funding data 2026-04-07
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Recursos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$127</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$122</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$131</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$126</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -657,7 +657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M127"/>
+  <dimension ref="A1:M131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -685,7 +685,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 06/04/2026 07:25 - 121 convocatorias - 20 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 07/04/2026 07:10 - 125 convocatorias - 23 nuevas</t>
         </is>
       </c>
     </row>
@@ -6901,12 +6901,12 @@
       </c>
       <c r="B108" s="6" t="inlineStr">
         <is>
-          <t>EUS-23520</t>
+          <t>EUS-78309</t>
         </is>
       </c>
       <c r="C108" s="6" t="inlineStr">
         <is>
-          <t>Contratación para el suministro, sustitución e instalación de la unidad exterior del sistema de climatización VRV existente en la Oficina Técnica del Ayuntamiento de Amorebieta-Etxano</t>
+          <t>Servicio de redacción del Plan de Clima y Energía (PCE) del municipio de Leioa.</t>
         </is>
       </c>
       <c r="D108" s="6" t="inlineStr">
@@ -6956,12 +6956,12 @@
       </c>
       <c r="B109" s="6" t="inlineStr">
         <is>
-          <t>EUS-31752</t>
+          <t>EUS-50766</t>
         </is>
       </c>
       <c r="C109" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
+          <t>Contratación para el suministro, sustitución e instalación de la unidad exterior del sistema de climatización VRV existente en la Oficina Técnica del Ayuntamiento de Amorebieta-Etxano</t>
         </is>
       </c>
       <c r="D109" s="6" t="inlineStr">
@@ -6978,12 +6978,12 @@
       <c r="G109" s="6" t="inlineStr"/>
       <c r="H109" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
-        </is>
-      </c>
-      <c r="I109" s="8" t="inlineStr">
-        <is>
-          <t>ALTA</t>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I109" s="12" t="inlineStr">
+        <is>
+          <t>MUY ALTA</t>
         </is>
       </c>
       <c r="J109" s="6" t="inlineStr"/>
@@ -7011,12 +7011,12 @@
       </c>
       <c r="B110" s="6" t="inlineStr">
         <is>
-          <t>EUS-23938</t>
+          <t>EUS-67043</t>
         </is>
       </c>
       <c r="C110" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la gestión sostenible de los recursos pesqueros 2026</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
         </is>
       </c>
       <c r="D110" s="6" t="inlineStr">
@@ -7066,12 +7066,12 @@
       </c>
       <c r="B111" s="6" t="inlineStr">
         <is>
-          <t>EUS-61297</t>
+          <t>EUS-58756</t>
         </is>
       </c>
       <c r="C111" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la recogida de residuos con la participación de los pescadores en el mar y las playas 2026</t>
+          <t>Ayudas a la gestión sostenible de los recursos pesqueros 2026</t>
         </is>
       </c>
       <c r="D111" s="6" t="inlineStr">
@@ -7121,12 +7121,12 @@
       </c>
       <c r="B112" s="6" t="inlineStr">
         <is>
-          <t>EUS-23417</t>
+          <t>EUS-12835</t>
         </is>
       </c>
       <c r="C112" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático sin incremento de capacidad 2026</t>
+          <t>Ayudas a la recogida de residuos con la participación de los pescadores en el mar y las playas 2026</t>
         </is>
       </c>
       <c r="D112" s="6" t="inlineStr">
@@ -7176,12 +7176,12 @@
       </c>
       <c r="B113" s="6" t="inlineStr">
         <is>
-          <t>EUS-56608</t>
+          <t>EUS-45037</t>
         </is>
       </c>
       <c r="C113" s="6" t="inlineStr">
         <is>
-          <t>servicio de recogida y transporte de residuos papel y cartón y destrucción documental de Alonsotegi y suministro de Contenedores.</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio climático sin incremento de capacidad 2026</t>
         </is>
       </c>
       <c r="D113" s="6" t="inlineStr">
@@ -7198,7 +7198,7 @@
       <c r="G113" s="6" t="inlineStr"/>
       <c r="H113" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="I113" s="8" t="inlineStr">
@@ -7231,12 +7231,12 @@
       </c>
       <c r="B114" s="6" t="inlineStr">
         <is>
-          <t>EUS-72014</t>
+          <t>EUS-02688</t>
         </is>
       </c>
       <c r="C114" s="6" t="inlineStr">
         <is>
-          <t>Estudio del estado de las instalaciones, prestación del servicio de operación y mantenimiento de los elementos que conforman el sistema operativo del sistema de recogida neumática de R.S.U. implantado</t>
+          <t>servicio de recogida y transporte de residuos papel y cartón y destrucción documental de Alonsotegi y suministro de Contenedores.</t>
         </is>
       </c>
       <c r="D114" s="6" t="inlineStr">
@@ -7286,12 +7286,12 @@
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>EUS-13924</t>
+          <t>EUS-22640</t>
         </is>
       </c>
       <c r="C115" s="6" t="inlineStr">
         <is>
-          <t>Trabajos de limpieza de residuos en los parques de Garaio, Landa y Mendixur, y en zonas de especial presión de visitantes del entorno de los embalses.</t>
+          <t>Estudio del estado de las instalaciones, prestación del servicio de operación y mantenimiento de los elementos que conforman el sistema operativo del sistema de recogida neumática de R.S.U. implantado</t>
         </is>
       </c>
       <c r="D115" s="6" t="inlineStr">
@@ -7341,12 +7341,12 @@
       </c>
       <c r="B116" s="6" t="inlineStr">
         <is>
-          <t>EUS-82252</t>
+          <t>EUS-99053</t>
         </is>
       </c>
       <c r="C116" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
+          <t>Trabajos de limpieza de residuos en los parques de Garaio, Landa y Mendixur, y en zonas de especial presión de visitantes del entorno de los embalses.</t>
         </is>
       </c>
       <c r="D116" s="6" t="inlineStr">
@@ -7363,12 +7363,12 @@
       <c r="G116" s="6" t="inlineStr"/>
       <c r="H116" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
-        </is>
-      </c>
-      <c r="I116" s="10" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I116" s="8" t="inlineStr">
+        <is>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="J116" s="6" t="inlineStr"/>
@@ -7377,11 +7377,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L116" s="15" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
+      <c r="L116" s="6" t="inlineStr"/>
       <c r="M116" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
@@ -7396,12 +7392,12 @@
       </c>
       <c r="B117" s="6" t="inlineStr">
         <is>
-          <t>EUS-41510</t>
+          <t>EUS-99424</t>
         </is>
       </c>
       <c r="C117" s="6" t="inlineStr">
         <is>
-          <t>Ayudas al valor añadido, economía circular y seguridad alimentaria 2026</t>
+          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
         </is>
       </c>
       <c r="D117" s="6" t="inlineStr">
@@ -7451,12 +7447,12 @@
       </c>
       <c r="B118" s="6" t="inlineStr">
         <is>
-          <t>EUS-19595</t>
+          <t>EUS-66735</t>
         </is>
       </c>
       <c r="C118" s="6" t="inlineStr">
         <is>
-          <t>Vino: el Gobierno Vasco volverá a convocar este mes las ayudas al arranque o cosecha en verde del viñedo, que van a contemplar como estructurales tras reformar la UE jurídicamente su Intervención Sect</t>
+          <t>Ayudas al valor añadido, economía circular y seguridad alimentaria 2026</t>
         </is>
       </c>
       <c r="D118" s="6" t="inlineStr">
@@ -7506,12 +7502,12 @@
       </c>
       <c r="B119" s="6" t="inlineStr">
         <is>
-          <t>EUS-04008</t>
+          <t>EUS-86673</t>
         </is>
       </c>
       <c r="C119" s="6" t="inlineStr">
         <is>
-          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de aceleración de proyectos, a localidades de menos de 20.000 habitantes son objeto de convocatoria abierta hasta el 17.03.26. Transformacione</t>
+          <t>Vino: el Gobierno Vasco volverá a convocar este mes las ayudas al arranque o cosecha en verde del viñedo, que van a contemplar como estructurales tras reformar la UE jurídicamente su Intervención Sect</t>
         </is>
       </c>
       <c r="D119" s="6" t="inlineStr">
@@ -7561,12 +7557,12 @@
       </c>
       <c r="B120" s="6" t="inlineStr">
         <is>
-          <t>EUS-33753</t>
+          <t>EUS-67797</t>
         </is>
       </c>
       <c r="C120" s="6" t="inlineStr">
         <is>
-          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para consorcios internacionales de I+D+i. Jornada del Gobierno Vasco y con Enterprise Europe Network y otros socios. Digitalización, dispositivos,</t>
+          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de aceleración de proyectos, a localidades de menos de 20.000 habitantes son objeto de convocatoria abierta hasta el 17.03.26. Transformacione</t>
         </is>
       </c>
       <c r="D120" s="6" t="inlineStr">
@@ -7616,12 +7612,12 @@
       </c>
       <c r="B121" s="6" t="inlineStr">
         <is>
-          <t>EUS-15589</t>
+          <t>EUS-19482</t>
         </is>
       </c>
       <c r="C121" s="6" t="inlineStr">
         <is>
-          <t>Servicio de limpieza integral del Complejo Deportivo Mendizorrotza</t>
+          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para consorcios internacionales de I+D+i. Jornada del Gobierno Vasco y con Enterprise Europe Network y otros socios. Digitalización, dispositivos,</t>
         </is>
       </c>
       <c r="D121" s="6" t="inlineStr">
@@ -7638,7 +7634,7 @@
       <c r="G121" s="6" t="inlineStr"/>
       <c r="H121" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="I121" s="10" t="inlineStr">
@@ -7671,12 +7667,12 @@
       </c>
       <c r="B122" s="6" t="inlineStr">
         <is>
-          <t>EUS-84889</t>
+          <t>EUS-20210</t>
         </is>
       </c>
       <c r="C122" s="6" t="inlineStr">
         <is>
-          <t>Servicios Profesionales en el ámbito de la Presencia Digital para el Proyecto IREKIA BERRIA</t>
+          <t>Redacción del proyecto de los trabajos de mejora de las redes de distribución de agua</t>
         </is>
       </c>
       <c r="D122" s="6" t="inlineStr">
@@ -7726,12 +7722,12 @@
       </c>
       <c r="B123" s="6" t="inlineStr">
         <is>
-          <t>EUS-16064</t>
+          <t>EUS-08817</t>
         </is>
       </c>
       <c r="C123" s="6" t="inlineStr">
         <is>
-          <t>Obras de distribución de la red de saneamiento y aguas pluviales del barrio Malats (1. fasea)</t>
+          <t>Servicio de recogida, custodia y protección de animales de compañía abandonados y perdidos/extraviados y control de colonias felinas en el término municipal de Leioa</t>
         </is>
       </c>
       <c r="D123" s="6" t="inlineStr">
@@ -7781,12 +7777,12 @@
       </c>
       <c r="B124" s="6" t="inlineStr">
         <is>
-          <t>EUS-36514</t>
+          <t>EUS-72869</t>
         </is>
       </c>
       <c r="C124" s="6" t="inlineStr">
         <is>
-          <t>Elaboración del diagnóstico de vivienda en el termino municipal de Orozko</t>
+          <t>Dirección de obra y reparación y sustitución de la cobertura de la cubierta en el edificio de enfermería en el Centro Penitenciario de Bizkaia</t>
         </is>
       </c>
       <c r="D124" s="6" t="inlineStr">
@@ -7836,12 +7832,12 @@
       </c>
       <c r="B125" s="6" t="inlineStr">
         <is>
-          <t>EUS-98928</t>
+          <t>EUS-40836</t>
         </is>
       </c>
       <c r="C125" s="6" t="inlineStr">
         <is>
-          <t>Instalación de nuevo alumbrado en el barrio de Andra Mari</t>
+          <t>Organización y ejecución de un programa de animación en parques de la ciudad.</t>
         </is>
       </c>
       <c r="D125" s="6" t="inlineStr">
@@ -7891,12 +7887,12 @@
       </c>
       <c r="B126" s="6" t="inlineStr">
         <is>
-          <t>EUS-29541</t>
+          <t>EUS-53028</t>
         </is>
       </c>
       <c r="C126" s="6" t="inlineStr">
         <is>
-          <t>Implementación en gis de la infraestructura municipal de limpieza de instalaciones mediante tecnología NFC</t>
+          <t>Servicio de limpieza integral del Complejo Deportivo Mendizorrotza</t>
         </is>
       </c>
       <c r="D126" s="6" t="inlineStr">
@@ -7946,12 +7942,12 @@
       </c>
       <c r="B127" s="6" t="inlineStr">
         <is>
-          <t>EUS-78417</t>
+          <t>EUS-78111</t>
         </is>
       </c>
       <c r="C127" s="6" t="inlineStr">
         <is>
-          <t>Recogida y adopción de perros</t>
+          <t>Servicios Profesionales en el ámbito de la Presencia Digital para el Proyecto IREKIA BERRIA</t>
         </is>
       </c>
       <c r="D127" s="6" t="inlineStr">
@@ -7993,8 +7989,228 @@
         </is>
       </c>
     </row>
+    <row r="128" ht="40" customHeight="1">
+      <c r="A128" s="14" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B128" s="6" t="inlineStr">
+        <is>
+          <t>EUS-36895</t>
+        </is>
+      </c>
+      <c r="C128" s="6" t="inlineStr">
+        <is>
+          <t>Obras de distribución de la red de saneamiento y aguas pluviales del barrio Malats (1. fasea)</t>
+        </is>
+      </c>
+      <c r="D128" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E128" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F128" s="6" t="inlineStr"/>
+      <c r="G128" s="6" t="inlineStr"/>
+      <c r="H128" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I128" s="10" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J128" s="6" t="inlineStr"/>
+      <c r="K128" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L128" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M128" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="40" customHeight="1">
+      <c r="A129" s="14" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B129" s="6" t="inlineStr">
+        <is>
+          <t>EUS-78769</t>
+        </is>
+      </c>
+      <c r="C129" s="6" t="inlineStr">
+        <is>
+          <t>Elaboración del diagnóstico de vivienda en el termino municipal de Orozko</t>
+        </is>
+      </c>
+      <c r="D129" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E129" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F129" s="6" t="inlineStr"/>
+      <c r="G129" s="6" t="inlineStr"/>
+      <c r="H129" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I129" s="10" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J129" s="6" t="inlineStr"/>
+      <c r="K129" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L129" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M129" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="40" customHeight="1">
+      <c r="A130" s="14" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B130" s="6" t="inlineStr">
+        <is>
+          <t>EUS-87188</t>
+        </is>
+      </c>
+      <c r="C130" s="6" t="inlineStr">
+        <is>
+          <t>Instalación de nuevo alumbrado en el barrio de Andra Mari</t>
+        </is>
+      </c>
+      <c r="D130" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E130" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F130" s="6" t="inlineStr"/>
+      <c r="G130" s="6" t="inlineStr"/>
+      <c r="H130" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I130" s="10" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J130" s="6" t="inlineStr"/>
+      <c r="K130" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L130" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M130" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="40" customHeight="1">
+      <c r="A131" s="14" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B131" s="6" t="inlineStr">
+        <is>
+          <t>EUS-87035</t>
+        </is>
+      </c>
+      <c r="C131" s="6" t="inlineStr">
+        <is>
+          <t>Implementación en gis de la infraestructura municipal de limpieza de instalaciones mediante tecnología NFC</t>
+        </is>
+      </c>
+      <c r="D131" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E131" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F131" s="6" t="inlineStr"/>
+      <c r="G131" s="6" t="inlineStr"/>
+      <c r="H131" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I131" s="10" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J131" s="6" t="inlineStr"/>
+      <c r="K131" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L131" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M131" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:M127"/>
+  <autoFilter ref="A4:M131"/>
   <mergeCells count="4">
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A107:M107"/>
@@ -8123,6 +8339,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M125" r:id="rId119"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M126" r:id="rId120"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M127" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M128" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M129" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M130" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M131" r:id="rId125"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8134,7 +8354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1814"/>
+  <dimension ref="A1:F1874"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -30028,7 +30248,7 @@
     <row r="1516" ht="30" customHeight="1">
       <c r="A1516" s="16" t="inlineStr">
         <is>
-          <t>FICHA 102: EUS-23520</t>
+          <t>FICHA 102: EUS-78309</t>
         </is>
       </c>
       <c r="B1516" s="17" t="n"/>
@@ -30053,7 +30273,7 @@
       <c r="E1517" s="20" t="n"/>
       <c r="F1517" s="20" t="n"/>
     </row>
-    <row r="1518" ht="45" customHeight="1">
+    <row r="1518" ht="20" customHeight="1">
       <c r="A1518" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -30061,7 +30281,7 @@
       </c>
       <c r="B1518" s="19" t="inlineStr">
         <is>
-          <t>Contratación para el suministro, sustitución e instalación de la unidad exterior del sistema de climatización VRV existente en la Oficina Técnica del Ayuntamiento de Amorebieta-Etxano</t>
+          <t>Servicio de redacción del Plan de Clima y Energía (PCE) del municipio de Leioa.</t>
         </is>
       </c>
       <c r="C1518" s="20" t="n"/>
@@ -30077,7 +30297,7 @@
       </c>
       <c r="B1519" s="19" t="inlineStr">
         <is>
-          <t>EUS-23520</t>
+          <t>EUS-78309</t>
         </is>
       </c>
       <c r="C1519" s="20" t="n"/>
@@ -30229,7 +30449,7 @@
       </c>
       <c r="B1529" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/contratacion-suministro-sustitucion-e-instalacion-unidad-exterior-del-sistema-climatizacion-vrv-existente-oficina-tecnica-del-ayuntamiento-amorebieta-etxano/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-redaccion-del-plan-clima-y-energia-pce-del-municipio-leioa/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1529" s="20" t="n"/>
@@ -30240,7 +30460,7 @@
     <row r="1531" ht="30" customHeight="1">
       <c r="A1531" s="16" t="inlineStr">
         <is>
-          <t>FICHA 103: EUS-31752</t>
+          <t>FICHA 103: EUS-50766</t>
         </is>
       </c>
       <c r="B1531" s="17" t="n"/>
@@ -30273,7 +30493,7 @@
       </c>
       <c r="B1533" s="19" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
+          <t>Contratación para el suministro, sustitución e instalación de la unidad exterior del sistema de climatización VRV existente en la Oficina Técnica del Ayuntamiento de Amorebieta-Etxano</t>
         </is>
       </c>
       <c r="C1533" s="20" t="n"/>
@@ -30289,7 +30509,7 @@
       </c>
       <c r="B1534" s="19" t="inlineStr">
         <is>
-          <t>EUS-31752</t>
+          <t>EUS-50766</t>
         </is>
       </c>
       <c r="C1534" s="20" t="n"/>
@@ -30365,7 +30585,7 @@
       </c>
       <c r="B1539" s="19" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C1539" s="20" t="n"/>
@@ -30423,9 +30643,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B1543" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ALTA — </t>
+      <c r="B1543" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MUY ALTA — </t>
         </is>
       </c>
       <c r="C1543" s="20" t="n"/>
@@ -30441,7 +30661,7 @@
       </c>
       <c r="B1544" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-con-incremento-de-capacidad-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/contratacion-suministro-sustitucion-e-instalacion-unidad-exterior-del-sistema-climatizacion-vrv-existente-oficina-tecnica-del-ayuntamiento-amorebieta-etxano/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1544" s="20" t="n"/>
@@ -30452,7 +30672,7 @@
     <row r="1546" ht="30" customHeight="1">
       <c r="A1546" s="16" t="inlineStr">
         <is>
-          <t>FICHA 104: EUS-23938</t>
+          <t>FICHA 104: EUS-67043</t>
         </is>
       </c>
       <c r="B1546" s="17" t="n"/>
@@ -30477,7 +30697,7 @@
       <c r="E1547" s="20" t="n"/>
       <c r="F1547" s="20" t="n"/>
     </row>
-    <row r="1548" ht="20" customHeight="1">
+    <row r="1548" ht="45" customHeight="1">
       <c r="A1548" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -30485,7 +30705,7 @@
       </c>
       <c r="B1548" s="19" t="inlineStr">
         <is>
-          <t>Ayudas a la gestión sostenible de los recursos pesqueros 2026</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
         </is>
       </c>
       <c r="C1548" s="20" t="n"/>
@@ -30501,7 +30721,7 @@
       </c>
       <c r="B1549" s="19" t="inlineStr">
         <is>
-          <t>EUS-23938</t>
+          <t>EUS-67043</t>
         </is>
       </c>
       <c r="C1549" s="20" t="n"/>
@@ -30653,7 +30873,7 @@
       </c>
       <c r="B1559" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-gestion-sostenible-de-los-recursos-pesqueros-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-con-incremento-de-capacidad-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1559" s="20" t="n"/>
@@ -30664,7 +30884,7 @@
     <row r="1561" ht="30" customHeight="1">
       <c r="A1561" s="16" t="inlineStr">
         <is>
-          <t>FICHA 105: EUS-61297</t>
+          <t>FICHA 105: EUS-58756</t>
         </is>
       </c>
       <c r="B1561" s="17" t="n"/>
@@ -30689,7 +30909,7 @@
       <c r="E1562" s="20" t="n"/>
       <c r="F1562" s="20" t="n"/>
     </row>
-    <row r="1563" ht="45" customHeight="1">
+    <row r="1563" ht="20" customHeight="1">
       <c r="A1563" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -30697,7 +30917,7 @@
       </c>
       <c r="B1563" s="19" t="inlineStr">
         <is>
-          <t>Ayudas a la recogida de residuos con la participación de los pescadores en el mar y las playas 2026</t>
+          <t>Ayudas a la gestión sostenible de los recursos pesqueros 2026</t>
         </is>
       </c>
       <c r="C1563" s="20" t="n"/>
@@ -30713,7 +30933,7 @@
       </c>
       <c r="B1564" s="19" t="inlineStr">
         <is>
-          <t>EUS-61297</t>
+          <t>EUS-58756</t>
         </is>
       </c>
       <c r="C1564" s="20" t="n"/>
@@ -30857,7 +31077,7 @@
       <c r="E1573" s="20" t="n"/>
       <c r="F1573" s="20" t="n"/>
     </row>
-    <row r="1574" ht="20" customHeight="1">
+    <row r="1574" ht="45" customHeight="1">
       <c r="A1574" s="18" t="inlineStr">
         <is>
           <t>Enlace al portal</t>
@@ -30865,7 +31085,7 @@
       </c>
       <c r="B1574" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/fempa-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-gestion-sostenible-de-los-recursos-pesqueros-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1574" s="20" t="n"/>
@@ -30876,7 +31096,7 @@
     <row r="1576" ht="30" customHeight="1">
       <c r="A1576" s="16" t="inlineStr">
         <is>
-          <t>FICHA 106: EUS-23417</t>
+          <t>FICHA 106: EUS-12835</t>
         </is>
       </c>
       <c r="B1576" s="17" t="n"/>
@@ -30909,7 +31129,7 @@
       </c>
       <c r="B1578" s="19" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático sin incremento de capacidad 2026</t>
+          <t>Ayudas a la recogida de residuos con la participación de los pescadores en el mar y las playas 2026</t>
         </is>
       </c>
       <c r="C1578" s="20" t="n"/>
@@ -30925,7 +31145,7 @@
       </c>
       <c r="B1579" s="19" t="inlineStr">
         <is>
-          <t>EUS-23417</t>
+          <t>EUS-12835</t>
         </is>
       </c>
       <c r="C1579" s="20" t="n"/>
@@ -31069,7 +31289,7 @@
       <c r="E1588" s="20" t="n"/>
       <c r="F1588" s="20" t="n"/>
     </row>
-    <row r="1589" ht="45" customHeight="1">
+    <row r="1589" ht="20" customHeight="1">
       <c r="A1589" s="18" t="inlineStr">
         <is>
           <t>Enlace al portal</t>
@@ -31077,7 +31297,7 @@
       </c>
       <c r="B1589" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-sin-incremento-de-capacidad-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/fempa-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1589" s="20" t="n"/>
@@ -31088,7 +31308,7 @@
     <row r="1591" ht="30" customHeight="1">
       <c r="A1591" s="16" t="inlineStr">
         <is>
-          <t>FICHA 107: EUS-56608</t>
+          <t>FICHA 107: EUS-45037</t>
         </is>
       </c>
       <c r="B1591" s="17" t="n"/>
@@ -31121,7 +31341,7 @@
       </c>
       <c r="B1593" s="19" t="inlineStr">
         <is>
-          <t>servicio de recogida y transporte de residuos papel y cartón y destrucción documental de Alonsotegi y suministro de Contenedores.</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio climático sin incremento de capacidad 2026</t>
         </is>
       </c>
       <c r="C1593" s="20" t="n"/>
@@ -31137,7 +31357,7 @@
       </c>
       <c r="B1594" s="19" t="inlineStr">
         <is>
-          <t>EUS-56608</t>
+          <t>EUS-45037</t>
         </is>
       </c>
       <c r="C1594" s="20" t="n"/>
@@ -31213,7 +31433,7 @@
       </c>
       <c r="B1599" s="19" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C1599" s="20" t="n"/>
@@ -31289,7 +31509,7 @@
       </c>
       <c r="B1604" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-recogida-y-transporte-residuos-papel-y-carton-y-destruccion-documental-alonsotegi-y-suministro-contenedores/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-sin-incremento-de-capacidad-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1604" s="20" t="n"/>
@@ -31300,7 +31520,7 @@
     <row r="1606" ht="30" customHeight="1">
       <c r="A1606" s="16" t="inlineStr">
         <is>
-          <t>FICHA 108: EUS-72014</t>
+          <t>FICHA 108: EUS-02688</t>
         </is>
       </c>
       <c r="B1606" s="17" t="n"/>
@@ -31333,7 +31553,7 @@
       </c>
       <c r="B1608" s="19" t="inlineStr">
         <is>
-          <t>Estudio del estado de las instalaciones, prestación del servicio de operación y mantenimiento de los elementos que conforman el sistema operativo del sistema de recogida neumática de R.S.U. implantado</t>
+          <t>servicio de recogida y transporte de residuos papel y cartón y destrucción documental de Alonsotegi y suministro de Contenedores.</t>
         </is>
       </c>
       <c r="C1608" s="20" t="n"/>
@@ -31349,7 +31569,7 @@
       </c>
       <c r="B1609" s="19" t="inlineStr">
         <is>
-          <t>EUS-72014</t>
+          <t>EUS-02688</t>
         </is>
       </c>
       <c r="C1609" s="20" t="n"/>
@@ -31501,7 +31721,7 @@
       </c>
       <c r="B1619" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/estudio-del-estado-instalaciones-prestacion-del-servicio-operacion-y-mantenimiento-elementos-que-conforman-sistema-operativo-del-sistema-recogida-neumatica-r-s-u-implantado-zona-noroeste-barakaldo-asi-como-traslado-residuos-recogidos-plantas-tratamiento/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-recogida-y-transporte-residuos-papel-y-carton-y-destruccion-documental-alonsotegi-y-suministro-contenedores/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1619" s="20" t="n"/>
@@ -31512,7 +31732,7 @@
     <row r="1621" ht="30" customHeight="1">
       <c r="A1621" s="16" t="inlineStr">
         <is>
-          <t>FICHA 109: EUS-13924</t>
+          <t>FICHA 109: EUS-22640</t>
         </is>
       </c>
       <c r="B1621" s="17" t="n"/>
@@ -31545,7 +31765,7 @@
       </c>
       <c r="B1623" s="19" t="inlineStr">
         <is>
-          <t>Trabajos de limpieza de residuos en los parques de Garaio, Landa y Mendixur, y en zonas de especial presión de visitantes del entorno de los embalses.</t>
+          <t>Estudio del estado de las instalaciones, prestación del servicio de operación y mantenimiento de los elementos que conforman el sistema operativo del sistema de recogida neumática de R.S.U. implantado</t>
         </is>
       </c>
       <c r="C1623" s="20" t="n"/>
@@ -31561,7 +31781,7 @@
       </c>
       <c r="B1624" s="19" t="inlineStr">
         <is>
-          <t>EUS-13924</t>
+          <t>EUS-22640</t>
         </is>
       </c>
       <c r="C1624" s="20" t="n"/>
@@ -31713,7 +31933,7 @@
       </c>
       <c r="B1634" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/trabajos-limpieza-residuos-parques-garaio-landa-y-mendixur-y-zonas-especial-presion-visitantes-del-entorno-embalses/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/estudio-del-estado-instalaciones-prestacion-del-servicio-operacion-y-mantenimiento-elementos-que-conforman-sistema-operativo-del-sistema-recogida-neumatica-r-s-u-implantado-zona-noroeste-barakaldo-asi-como-traslado-residuos-recogidos-plantas-tratamiento/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1634" s="20" t="n"/>
@@ -31724,7 +31944,7 @@
     <row r="1636" ht="30" customHeight="1">
       <c r="A1636" s="16" t="inlineStr">
         <is>
-          <t>FICHA 110: EUS-82252</t>
+          <t>FICHA 110: EUS-99053</t>
         </is>
       </c>
       <c r="B1636" s="17" t="n"/>
@@ -31757,7 +31977,7 @@
       </c>
       <c r="B1638" s="19" t="inlineStr">
         <is>
-          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
+          <t>Trabajos de limpieza de residuos en los parques de Garaio, Landa y Mendixur, y en zonas de especial presión de visitantes del entorno de los embalses.</t>
         </is>
       </c>
       <c r="C1638" s="20" t="n"/>
@@ -31773,7 +31993,7 @@
       </c>
       <c r="B1639" s="19" t="inlineStr">
         <is>
-          <t>EUS-82252</t>
+          <t>EUS-99053</t>
         </is>
       </c>
       <c r="C1639" s="20" t="n"/>
@@ -31849,7 +32069,7 @@
       </c>
       <c r="B1644" s="19" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C1644" s="20" t="n"/>
@@ -31907,9 +32127,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B1648" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
+      <c r="B1648" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALTA — </t>
         </is>
       </c>
       <c r="C1648" s="20" t="n"/>
@@ -31925,7 +32145,7 @@
       </c>
       <c r="B1649" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-contribucion-de-la-acuicultura-al-buen-estado-ambiental-y-prestacion-de-servicios-ambientales-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/trabajos-limpieza-residuos-parques-garaio-landa-y-mendixur-y-zonas-especial-presion-visitantes-del-entorno-embalses/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1649" s="20" t="n"/>
@@ -31936,7 +32156,7 @@
     <row r="1651" ht="30" customHeight="1">
       <c r="A1651" s="16" t="inlineStr">
         <is>
-          <t>FICHA 111: EUS-41510</t>
+          <t>FICHA 111: EUS-99424</t>
         </is>
       </c>
       <c r="B1651" s="17" t="n"/>
@@ -31961,7 +32181,7 @@
       <c r="E1652" s="20" t="n"/>
       <c r="F1652" s="20" t="n"/>
     </row>
-    <row r="1653" ht="20" customHeight="1">
+    <row r="1653" ht="45" customHeight="1">
       <c r="A1653" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -31969,7 +32189,7 @@
       </c>
       <c r="B1653" s="19" t="inlineStr">
         <is>
-          <t>Ayudas al valor añadido, economía circular y seguridad alimentaria 2026</t>
+          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
         </is>
       </c>
       <c r="C1653" s="20" t="n"/>
@@ -31985,7 +32205,7 @@
       </c>
       <c r="B1654" s="19" t="inlineStr">
         <is>
-          <t>EUS-41510</t>
+          <t>EUS-99424</t>
         </is>
       </c>
       <c r="C1654" s="20" t="n"/>
@@ -32137,7 +32357,7 @@
       </c>
       <c r="B1664" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-valor-anadido-economia-circular-y-seguridad-alimentaria-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-contribucion-de-la-acuicultura-al-buen-estado-ambiental-y-prestacion-de-servicios-ambientales-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1664" s="20" t="n"/>
@@ -32148,7 +32368,7 @@
     <row r="1666" ht="30" customHeight="1">
       <c r="A1666" s="16" t="inlineStr">
         <is>
-          <t>FICHA 112: EUS-19595</t>
+          <t>FICHA 112: EUS-66735</t>
         </is>
       </c>
       <c r="B1666" s="17" t="n"/>
@@ -32173,7 +32393,7 @@
       <c r="E1667" s="20" t="n"/>
       <c r="F1667" s="20" t="n"/>
     </row>
-    <row r="1668" ht="45" customHeight="1">
+    <row r="1668" ht="20" customHeight="1">
       <c r="A1668" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -32181,7 +32401,7 @@
       </c>
       <c r="B1668" s="19" t="inlineStr">
         <is>
-          <t>Vino: el Gobierno Vasco volverá a convocar este mes las ayudas al arranque o cosecha en verde del viñedo, que van a contemplar como estructurales tras reformar la UE jurídicamente su Intervención Sect</t>
+          <t>Ayudas al valor añadido, economía circular y seguridad alimentaria 2026</t>
         </is>
       </c>
       <c r="C1668" s="20" t="n"/>
@@ -32197,7 +32417,7 @@
       </c>
       <c r="B1669" s="19" t="inlineStr">
         <is>
-          <t>EUS-19595</t>
+          <t>EUS-66735</t>
         </is>
       </c>
       <c r="C1669" s="20" t="n"/>
@@ -32349,7 +32569,7 @@
       </c>
       <c r="B1679" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260302berdezerauztekoak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-valor-anadido-economia-circular-y-seguridad-alimentaria-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1679" s="20" t="n"/>
@@ -32360,7 +32580,7 @@
     <row r="1681" ht="30" customHeight="1">
       <c r="A1681" s="16" t="inlineStr">
         <is>
-          <t>FICHA 113: EUS-04008</t>
+          <t>FICHA 113: EUS-86673</t>
         </is>
       </c>
       <c r="B1681" s="17" t="n"/>
@@ -32393,7 +32613,7 @@
       </c>
       <c r="B1683" s="19" t="inlineStr">
         <is>
-          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de aceleración de proyectos, a localidades de menos de 20.000 habitantes son objeto de convocatoria abierta hasta el 17.03.26. Transformacione</t>
+          <t>Vino: el Gobierno Vasco volverá a convocar este mes las ayudas al arranque o cosecha en verde del viñedo, que van a contemplar como estructurales tras reformar la UE jurídicamente su Intervención Sect</t>
         </is>
       </c>
       <c r="C1683" s="20" t="n"/>
@@ -32409,7 +32629,7 @@
       </c>
       <c r="B1684" s="19" t="inlineStr">
         <is>
-          <t>EUS-04008</t>
+          <t>EUS-86673</t>
         </is>
       </c>
       <c r="C1684" s="20" t="n"/>
@@ -32561,7 +32781,7 @@
       </c>
       <c r="B1694" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260317neboostasariak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260302berdezerauztekoak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1694" s="20" t="n"/>
@@ -32572,7 +32792,7 @@
     <row r="1696" ht="30" customHeight="1">
       <c r="A1696" s="16" t="inlineStr">
         <is>
-          <t>FICHA 114: EUS-33753</t>
+          <t>FICHA 114: EUS-67797</t>
         </is>
       </c>
       <c r="B1696" s="17" t="n"/>
@@ -32605,7 +32825,7 @@
       </c>
       <c r="B1698" s="19" t="inlineStr">
         <is>
-          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para consorcios internacionales de I+D+i. Jornada del Gobierno Vasco y con Enterprise Europe Network y otros socios. Digitalización, dispositivos,</t>
+          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de aceleración de proyectos, a localidades de menos de 20.000 habitantes son objeto de convocatoria abierta hasta el 17.03.26. Transformacione</t>
         </is>
       </c>
       <c r="C1698" s="20" t="n"/>
@@ -32621,7 +32841,7 @@
       </c>
       <c r="B1699" s="19" t="inlineStr">
         <is>
-          <t>EUS-33753</t>
+          <t>EUS-67797</t>
         </is>
       </c>
       <c r="C1699" s="20" t="n"/>
@@ -32773,7 +32993,7 @@
       </c>
       <c r="B1709" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260303eicihihorizon/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260317neboostasariak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1709" s="20" t="n"/>
@@ -32784,7 +33004,7 @@
     <row r="1711" ht="30" customHeight="1">
       <c r="A1711" s="16" t="inlineStr">
         <is>
-          <t>FICHA 115: EUS-15589</t>
+          <t>FICHA 115: EUS-19482</t>
         </is>
       </c>
       <c r="B1711" s="17" t="n"/>
@@ -32809,7 +33029,7 @@
       <c r="E1712" s="20" t="n"/>
       <c r="F1712" s="20" t="n"/>
     </row>
-    <row r="1713" ht="20" customHeight="1">
+    <row r="1713" ht="45" customHeight="1">
       <c r="A1713" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -32817,7 +33037,7 @@
       </c>
       <c r="B1713" s="19" t="inlineStr">
         <is>
-          <t>Servicio de limpieza integral del Complejo Deportivo Mendizorrotza</t>
+          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para consorcios internacionales de I+D+i. Jornada del Gobierno Vasco y con Enterprise Europe Network y otros socios. Digitalización, dispositivos,</t>
         </is>
       </c>
       <c r="C1713" s="20" t="n"/>
@@ -32833,7 +33053,7 @@
       </c>
       <c r="B1714" s="19" t="inlineStr">
         <is>
-          <t>EUS-15589</t>
+          <t>EUS-19482</t>
         </is>
       </c>
       <c r="C1714" s="20" t="n"/>
@@ -32909,7 +33129,7 @@
       </c>
       <c r="B1719" s="19" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C1719" s="20" t="n"/>
@@ -32985,7 +33205,7 @@
       </c>
       <c r="B1724" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-limpieza-integral-del-complejo-deportivo-mendizorrotza/expjaso701010/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260303eicihihorizon/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1724" s="20" t="n"/>
@@ -32996,7 +33216,7 @@
     <row r="1726" ht="30" customHeight="1">
       <c r="A1726" s="16" t="inlineStr">
         <is>
-          <t>FICHA 116: EUS-84889</t>
+          <t>FICHA 116: EUS-20210</t>
         </is>
       </c>
       <c r="B1726" s="17" t="n"/>
@@ -33029,7 +33249,7 @@
       </c>
       <c r="B1728" s="19" t="inlineStr">
         <is>
-          <t>Servicios Profesionales en el ámbito de la Presencia Digital para el Proyecto IREKIA BERRIA</t>
+          <t>Redacción del proyecto de los trabajos de mejora de las redes de distribución de agua</t>
         </is>
       </c>
       <c r="C1728" s="20" t="n"/>
@@ -33045,7 +33265,7 @@
       </c>
       <c r="B1729" s="19" t="inlineStr">
         <is>
-          <t>EUS-84889</t>
+          <t>EUS-20210</t>
         </is>
       </c>
       <c r="C1729" s="20" t="n"/>
@@ -33197,7 +33417,7 @@
       </c>
       <c r="B1739" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/servicios-profesionales-ambito-presencia-digital-proyecto-irekia-berria/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/redaccion-del-proyecto-trabajos-mejora-redes-distribucion-agua/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1739" s="20" t="n"/>
@@ -33208,7 +33428,7 @@
     <row r="1741" ht="30" customHeight="1">
       <c r="A1741" s="16" t="inlineStr">
         <is>
-          <t>FICHA 117: EUS-16064</t>
+          <t>FICHA 117: EUS-08817</t>
         </is>
       </c>
       <c r="B1741" s="17" t="n"/>
@@ -33241,7 +33461,7 @@
       </c>
       <c r="B1743" s="19" t="inlineStr">
         <is>
-          <t>Obras de distribución de la red de saneamiento y aguas pluviales del barrio Malats (1. fasea)</t>
+          <t>Servicio de recogida, custodia y protección de animales de compañía abandonados y perdidos/extraviados y control de colonias felinas en el término municipal de Leioa</t>
         </is>
       </c>
       <c r="C1743" s="20" t="n"/>
@@ -33257,7 +33477,7 @@
       </c>
       <c r="B1744" s="19" t="inlineStr">
         <is>
-          <t>EUS-16064</t>
+          <t>EUS-08817</t>
         </is>
       </c>
       <c r="C1744" s="20" t="n"/>
@@ -33409,7 +33629,7 @@
       </c>
       <c r="B1754" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/obras-distribucion-red-saneamiento-y-aguas-pluviales-del-barrio-malats-1-fasea/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-recogida-custodia-y-proteccion-animales-compania-abandonados-y-perdidos-extraviados-y-control-colonias-felinas-termino-municipal-leioa/expjaso692925/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1754" s="20" t="n"/>
@@ -33420,7 +33640,7 @@
     <row r="1756" ht="30" customHeight="1">
       <c r="A1756" s="16" t="inlineStr">
         <is>
-          <t>FICHA 118: EUS-36514</t>
+          <t>FICHA 118: EUS-72869</t>
         </is>
       </c>
       <c r="B1756" s="17" t="n"/>
@@ -33445,7 +33665,7 @@
       <c r="E1757" s="20" t="n"/>
       <c r="F1757" s="20" t="n"/>
     </row>
-    <row r="1758" ht="20" customHeight="1">
+    <row r="1758" ht="45" customHeight="1">
       <c r="A1758" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -33453,7 +33673,7 @@
       </c>
       <c r="B1758" s="19" t="inlineStr">
         <is>
-          <t>Elaboración del diagnóstico de vivienda en el termino municipal de Orozko</t>
+          <t>Dirección de obra y reparación y sustitución de la cobertura de la cubierta en el edificio de enfermería en el Centro Penitenciario de Bizkaia</t>
         </is>
       </c>
       <c r="C1758" s="20" t="n"/>
@@ -33469,7 +33689,7 @@
       </c>
       <c r="B1759" s="19" t="inlineStr">
         <is>
-          <t>EUS-36514</t>
+          <t>EUS-72869</t>
         </is>
       </c>
       <c r="C1759" s="20" t="n"/>
@@ -33621,7 +33841,7 @@
       </c>
       <c r="B1769" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/elaboracion-del-diagnostico-vivienda-termino-municipal-orozko/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/direccion-obra-y-reparacion-y-sustitucion-cobertura-cubierta-edificio-enfermeria-centro-penitenciario-bizkaia/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1769" s="20" t="n"/>
@@ -33632,7 +33852,7 @@
     <row r="1771" ht="30" customHeight="1">
       <c r="A1771" s="16" t="inlineStr">
         <is>
-          <t>FICHA 119: EUS-98928</t>
+          <t>FICHA 119: EUS-40836</t>
         </is>
       </c>
       <c r="B1771" s="17" t="n"/>
@@ -33665,7 +33885,7 @@
       </c>
       <c r="B1773" s="19" t="inlineStr">
         <is>
-          <t>Instalación de nuevo alumbrado en el barrio de Andra Mari</t>
+          <t>Organización y ejecución de un programa de animación en parques de la ciudad.</t>
         </is>
       </c>
       <c r="C1773" s="20" t="n"/>
@@ -33681,7 +33901,7 @@
       </c>
       <c r="B1774" s="19" t="inlineStr">
         <is>
-          <t>EUS-98928</t>
+          <t>EUS-40836</t>
         </is>
       </c>
       <c r="C1774" s="20" t="n"/>
@@ -33833,7 +34053,7 @@
       </c>
       <c r="B1784" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/instalacion-nuevo-alumbrado-barrio-andra-mari/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/organizacion-y-ejecucion-programa-animacion-parques-ciudad/expjaso700427/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1784" s="20" t="n"/>
@@ -33844,7 +34064,7 @@
     <row r="1786" ht="30" customHeight="1">
       <c r="A1786" s="16" t="inlineStr">
         <is>
-          <t>FICHA 120: EUS-29541</t>
+          <t>FICHA 120: EUS-53028</t>
         </is>
       </c>
       <c r="B1786" s="17" t="n"/>
@@ -33869,7 +34089,7 @@
       <c r="E1787" s="20" t="n"/>
       <c r="F1787" s="20" t="n"/>
     </row>
-    <row r="1788" ht="45" customHeight="1">
+    <row r="1788" ht="20" customHeight="1">
       <c r="A1788" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -33877,7 +34097,7 @@
       </c>
       <c r="B1788" s="19" t="inlineStr">
         <is>
-          <t>Implementación en gis de la infraestructura municipal de limpieza de instalaciones mediante tecnología NFC</t>
+          <t>Servicio de limpieza integral del Complejo Deportivo Mendizorrotza</t>
         </is>
       </c>
       <c r="C1788" s="20" t="n"/>
@@ -33893,7 +34113,7 @@
       </c>
       <c r="B1789" s="19" t="inlineStr">
         <is>
-          <t>EUS-29541</t>
+          <t>EUS-53028</t>
         </is>
       </c>
       <c r="C1789" s="20" t="n"/>
@@ -34045,7 +34265,7 @@
       </c>
       <c r="B1799" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/implementacion-gis-infraestructura-municipal-limpieza-instalaciones-mediante-tecnologia-nfc/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-limpieza-integral-del-complejo-deportivo-mendizorrotza/expjaso701010/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1799" s="20" t="n"/>
@@ -34056,7 +34276,7 @@
     <row r="1801" ht="30" customHeight="1">
       <c r="A1801" s="16" t="inlineStr">
         <is>
-          <t>FICHA 121: EUS-78417</t>
+          <t>FICHA 121: EUS-78111</t>
         </is>
       </c>
       <c r="B1801" s="17" t="n"/>
@@ -34081,7 +34301,7 @@
       <c r="E1802" s="20" t="n"/>
       <c r="F1802" s="20" t="n"/>
     </row>
-    <row r="1803" ht="20" customHeight="1">
+    <row r="1803" ht="45" customHeight="1">
       <c r="A1803" s="18" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -34089,7 +34309,7 @@
       </c>
       <c r="B1803" s="19" t="inlineStr">
         <is>
-          <t>Recogida y adopción de perros</t>
+          <t>Servicios Profesionales en el ámbito de la Presencia Digital para el Proyecto IREKIA BERRIA</t>
         </is>
       </c>
       <c r="C1803" s="20" t="n"/>
@@ -34105,7 +34325,7 @@
       </c>
       <c r="B1804" s="19" t="inlineStr">
         <is>
-          <t>EUS-78417</t>
+          <t>EUS-78111</t>
         </is>
       </c>
       <c r="C1804" s="20" t="n"/>
@@ -34257,7 +34477,7 @@
       </c>
       <c r="B1814" s="22" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/recogida-y-adopcion-perros/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicios-profesionales-ambito-presencia-digital-proyecto-irekia-berria/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1814" s="20" t="n"/>
@@ -34265,8 +34485,856 @@
       <c r="E1814" s="20" t="n"/>
       <c r="F1814" s="20" t="n"/>
     </row>
+    <row r="1816" ht="30" customHeight="1">
+      <c r="A1816" s="16" t="inlineStr">
+        <is>
+          <t>FICHA 122: EUS-36895</t>
+        </is>
+      </c>
+      <c r="B1816" s="17" t="n"/>
+      <c r="C1816" s="17" t="n"/>
+      <c r="D1816" s="17" t="n"/>
+      <c r="E1816" s="17" t="n"/>
+      <c r="F1816" s="17" t="n"/>
+    </row>
+    <row r="1817" ht="20" customHeight="1">
+      <c r="A1817" s="18" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1817" s="19" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1817" s="20" t="n"/>
+      <c r="D1817" s="20" t="n"/>
+      <c r="E1817" s="20" t="n"/>
+      <c r="F1817" s="20" t="n"/>
+    </row>
+    <row r="1818" ht="45" customHeight="1">
+      <c r="A1818" s="18" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1818" s="19" t="inlineStr">
+        <is>
+          <t>Obras de distribución de la red de saneamiento y aguas pluviales del barrio Malats (1. fasea)</t>
+        </is>
+      </c>
+      <c r="C1818" s="20" t="n"/>
+      <c r="D1818" s="20" t="n"/>
+      <c r="E1818" s="20" t="n"/>
+      <c r="F1818" s="20" t="n"/>
+    </row>
+    <row r="1819" ht="20" customHeight="1">
+      <c r="A1819" s="18" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1819" s="19" t="inlineStr">
+        <is>
+          <t>EUS-36895</t>
+        </is>
+      </c>
+      <c r="C1819" s="20" t="n"/>
+      <c r="D1819" s="20" t="n"/>
+      <c r="E1819" s="20" t="n"/>
+      <c r="F1819" s="20" t="n"/>
+    </row>
+    <row r="1820" ht="20" customHeight="1">
+      <c r="A1820" s="18" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1820" s="19" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1820" s="20" t="n"/>
+      <c r="D1820" s="20" t="n"/>
+      <c r="E1820" s="20" t="n"/>
+      <c r="F1820" s="20" t="n"/>
+    </row>
+    <row r="1821" ht="20" customHeight="1">
+      <c r="A1821" s="18" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1821" s="19" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1821" s="20" t="n"/>
+      <c r="D1821" s="20" t="n"/>
+      <c r="E1821" s="20" t="n"/>
+      <c r="F1821" s="20" t="n"/>
+    </row>
+    <row r="1822" ht="20" customHeight="1">
+      <c r="A1822" s="18" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1822" s="19" t="inlineStr"/>
+      <c r="C1822" s="20" t="n"/>
+      <c r="D1822" s="20" t="n"/>
+      <c r="E1822" s="20" t="n"/>
+      <c r="F1822" s="20" t="n"/>
+    </row>
+    <row r="1823" ht="20" customHeight="1">
+      <c r="A1823" s="18" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1823" s="19" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1823" s="20" t="n"/>
+      <c r="D1823" s="20" t="n"/>
+      <c r="E1823" s="20" t="n"/>
+      <c r="F1823" s="20" t="n"/>
+    </row>
+    <row r="1824" ht="20" customHeight="1">
+      <c r="A1824" s="18" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1824" s="19" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1824" s="20" t="n"/>
+      <c r="D1824" s="20" t="n"/>
+      <c r="E1824" s="20" t="n"/>
+      <c r="F1824" s="20" t="n"/>
+    </row>
+    <row r="1825" ht="20" customHeight="1">
+      <c r="A1825" s="18" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1825" s="19" t="inlineStr"/>
+      <c r="C1825" s="20" t="n"/>
+      <c r="D1825" s="20" t="n"/>
+      <c r="E1825" s="20" t="n"/>
+      <c r="F1825" s="20" t="n"/>
+    </row>
+    <row r="1826" ht="20" customHeight="1">
+      <c r="A1826" s="18" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1826" s="19" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1826" s="20" t="n"/>
+      <c r="D1826" s="20" t="n"/>
+      <c r="E1826" s="20" t="n"/>
+      <c r="F1826" s="20" t="n"/>
+    </row>
+    <row r="1827" ht="20" customHeight="1">
+      <c r="A1827" s="18" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1827" s="19" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1827" s="20" t="n"/>
+      <c r="D1827" s="20" t="n"/>
+      <c r="E1827" s="20" t="n"/>
+      <c r="F1827" s="20" t="n"/>
+    </row>
+    <row r="1828" ht="20" customHeight="1">
+      <c r="A1828" s="18" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1828" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1828" s="20" t="n"/>
+      <c r="D1828" s="20" t="n"/>
+      <c r="E1828" s="20" t="n"/>
+      <c r="F1828" s="20" t="n"/>
+    </row>
+    <row r="1829" ht="45" customHeight="1">
+      <c r="A1829" s="18" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1829" s="22" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/obras-distribucion-red-saneamiento-y-aguas-pluviales-del-barrio-malats-1-fasea/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1829" s="20" t="n"/>
+      <c r="D1829" s="20" t="n"/>
+      <c r="E1829" s="20" t="n"/>
+      <c r="F1829" s="20" t="n"/>
+    </row>
+    <row r="1831" ht="30" customHeight="1">
+      <c r="A1831" s="16" t="inlineStr">
+        <is>
+          <t>FICHA 123: EUS-78769</t>
+        </is>
+      </c>
+      <c r="B1831" s="17" t="n"/>
+      <c r="C1831" s="17" t="n"/>
+      <c r="D1831" s="17" t="n"/>
+      <c r="E1831" s="17" t="n"/>
+      <c r="F1831" s="17" t="n"/>
+    </row>
+    <row r="1832" ht="20" customHeight="1">
+      <c r="A1832" s="18" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1832" s="19" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1832" s="20" t="n"/>
+      <c r="D1832" s="20" t="n"/>
+      <c r="E1832" s="20" t="n"/>
+      <c r="F1832" s="20" t="n"/>
+    </row>
+    <row r="1833" ht="20" customHeight="1">
+      <c r="A1833" s="18" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1833" s="19" t="inlineStr">
+        <is>
+          <t>Elaboración del diagnóstico de vivienda en el termino municipal de Orozko</t>
+        </is>
+      </c>
+      <c r="C1833" s="20" t="n"/>
+      <c r="D1833" s="20" t="n"/>
+      <c r="E1833" s="20" t="n"/>
+      <c r="F1833" s="20" t="n"/>
+    </row>
+    <row r="1834" ht="20" customHeight="1">
+      <c r="A1834" s="18" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1834" s="19" t="inlineStr">
+        <is>
+          <t>EUS-78769</t>
+        </is>
+      </c>
+      <c r="C1834" s="20" t="n"/>
+      <c r="D1834" s="20" t="n"/>
+      <c r="E1834" s="20" t="n"/>
+      <c r="F1834" s="20" t="n"/>
+    </row>
+    <row r="1835" ht="20" customHeight="1">
+      <c r="A1835" s="18" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1835" s="19" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1835" s="20" t="n"/>
+      <c r="D1835" s="20" t="n"/>
+      <c r="E1835" s="20" t="n"/>
+      <c r="F1835" s="20" t="n"/>
+    </row>
+    <row r="1836" ht="20" customHeight="1">
+      <c r="A1836" s="18" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1836" s="19" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1836" s="20" t="n"/>
+      <c r="D1836" s="20" t="n"/>
+      <c r="E1836" s="20" t="n"/>
+      <c r="F1836" s="20" t="n"/>
+    </row>
+    <row r="1837" ht="20" customHeight="1">
+      <c r="A1837" s="18" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1837" s="19" t="inlineStr"/>
+      <c r="C1837" s="20" t="n"/>
+      <c r="D1837" s="20" t="n"/>
+      <c r="E1837" s="20" t="n"/>
+      <c r="F1837" s="20" t="n"/>
+    </row>
+    <row r="1838" ht="20" customHeight="1">
+      <c r="A1838" s="18" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1838" s="19" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1838" s="20" t="n"/>
+      <c r="D1838" s="20" t="n"/>
+      <c r="E1838" s="20" t="n"/>
+      <c r="F1838" s="20" t="n"/>
+    </row>
+    <row r="1839" ht="20" customHeight="1">
+      <c r="A1839" s="18" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1839" s="19" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1839" s="20" t="n"/>
+      <c r="D1839" s="20" t="n"/>
+      <c r="E1839" s="20" t="n"/>
+      <c r="F1839" s="20" t="n"/>
+    </row>
+    <row r="1840" ht="20" customHeight="1">
+      <c r="A1840" s="18" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1840" s="19" t="inlineStr"/>
+      <c r="C1840" s="20" t="n"/>
+      <c r="D1840" s="20" t="n"/>
+      <c r="E1840" s="20" t="n"/>
+      <c r="F1840" s="20" t="n"/>
+    </row>
+    <row r="1841" ht="20" customHeight="1">
+      <c r="A1841" s="18" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1841" s="19" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1841" s="20" t="n"/>
+      <c r="D1841" s="20" t="n"/>
+      <c r="E1841" s="20" t="n"/>
+      <c r="F1841" s="20" t="n"/>
+    </row>
+    <row r="1842" ht="20" customHeight="1">
+      <c r="A1842" s="18" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1842" s="19" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1842" s="20" t="n"/>
+      <c r="D1842" s="20" t="n"/>
+      <c r="E1842" s="20" t="n"/>
+      <c r="F1842" s="20" t="n"/>
+    </row>
+    <row r="1843" ht="20" customHeight="1">
+      <c r="A1843" s="18" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1843" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1843" s="20" t="n"/>
+      <c r="D1843" s="20" t="n"/>
+      <c r="E1843" s="20" t="n"/>
+      <c r="F1843" s="20" t="n"/>
+    </row>
+    <row r="1844" ht="45" customHeight="1">
+      <c r="A1844" s="18" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1844" s="22" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/elaboracion-del-diagnostico-vivienda-termino-municipal-orozko/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1844" s="20" t="n"/>
+      <c r="D1844" s="20" t="n"/>
+      <c r="E1844" s="20" t="n"/>
+      <c r="F1844" s="20" t="n"/>
+    </row>
+    <row r="1846" ht="30" customHeight="1">
+      <c r="A1846" s="16" t="inlineStr">
+        <is>
+          <t>FICHA 124: EUS-87188</t>
+        </is>
+      </c>
+      <c r="B1846" s="17" t="n"/>
+      <c r="C1846" s="17" t="n"/>
+      <c r="D1846" s="17" t="n"/>
+      <c r="E1846" s="17" t="n"/>
+      <c r="F1846" s="17" t="n"/>
+    </row>
+    <row r="1847" ht="20" customHeight="1">
+      <c r="A1847" s="18" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1847" s="19" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1847" s="20" t="n"/>
+      <c r="D1847" s="20" t="n"/>
+      <c r="E1847" s="20" t="n"/>
+      <c r="F1847" s="20" t="n"/>
+    </row>
+    <row r="1848" ht="20" customHeight="1">
+      <c r="A1848" s="18" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1848" s="19" t="inlineStr">
+        <is>
+          <t>Instalación de nuevo alumbrado en el barrio de Andra Mari</t>
+        </is>
+      </c>
+      <c r="C1848" s="20" t="n"/>
+      <c r="D1848" s="20" t="n"/>
+      <c r="E1848" s="20" t="n"/>
+      <c r="F1848" s="20" t="n"/>
+    </row>
+    <row r="1849" ht="20" customHeight="1">
+      <c r="A1849" s="18" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1849" s="19" t="inlineStr">
+        <is>
+          <t>EUS-87188</t>
+        </is>
+      </c>
+      <c r="C1849" s="20" t="n"/>
+      <c r="D1849" s="20" t="n"/>
+      <c r="E1849" s="20" t="n"/>
+      <c r="F1849" s="20" t="n"/>
+    </row>
+    <row r="1850" ht="20" customHeight="1">
+      <c r="A1850" s="18" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1850" s="19" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1850" s="20" t="n"/>
+      <c r="D1850" s="20" t="n"/>
+      <c r="E1850" s="20" t="n"/>
+      <c r="F1850" s="20" t="n"/>
+    </row>
+    <row r="1851" ht="20" customHeight="1">
+      <c r="A1851" s="18" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1851" s="19" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1851" s="20" t="n"/>
+      <c r="D1851" s="20" t="n"/>
+      <c r="E1851" s="20" t="n"/>
+      <c r="F1851" s="20" t="n"/>
+    </row>
+    <row r="1852" ht="20" customHeight="1">
+      <c r="A1852" s="18" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1852" s="19" t="inlineStr"/>
+      <c r="C1852" s="20" t="n"/>
+      <c r="D1852" s="20" t="n"/>
+      <c r="E1852" s="20" t="n"/>
+      <c r="F1852" s="20" t="n"/>
+    </row>
+    <row r="1853" ht="20" customHeight="1">
+      <c r="A1853" s="18" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1853" s="19" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1853" s="20" t="n"/>
+      <c r="D1853" s="20" t="n"/>
+      <c r="E1853" s="20" t="n"/>
+      <c r="F1853" s="20" t="n"/>
+    </row>
+    <row r="1854" ht="20" customHeight="1">
+      <c r="A1854" s="18" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1854" s="19" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1854" s="20" t="n"/>
+      <c r="D1854" s="20" t="n"/>
+      <c r="E1854" s="20" t="n"/>
+      <c r="F1854" s="20" t="n"/>
+    </row>
+    <row r="1855" ht="20" customHeight="1">
+      <c r="A1855" s="18" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1855" s="19" t="inlineStr"/>
+      <c r="C1855" s="20" t="n"/>
+      <c r="D1855" s="20" t="n"/>
+      <c r="E1855" s="20" t="n"/>
+      <c r="F1855" s="20" t="n"/>
+    </row>
+    <row r="1856" ht="20" customHeight="1">
+      <c r="A1856" s="18" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1856" s="19" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1856" s="20" t="n"/>
+      <c r="D1856" s="20" t="n"/>
+      <c r="E1856" s="20" t="n"/>
+      <c r="F1856" s="20" t="n"/>
+    </row>
+    <row r="1857" ht="20" customHeight="1">
+      <c r="A1857" s="18" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1857" s="19" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1857" s="20" t="n"/>
+      <c r="D1857" s="20" t="n"/>
+      <c r="E1857" s="20" t="n"/>
+      <c r="F1857" s="20" t="n"/>
+    </row>
+    <row r="1858" ht="20" customHeight="1">
+      <c r="A1858" s="18" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1858" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1858" s="20" t="n"/>
+      <c r="D1858" s="20" t="n"/>
+      <c r="E1858" s="20" t="n"/>
+      <c r="F1858" s="20" t="n"/>
+    </row>
+    <row r="1859" ht="45" customHeight="1">
+      <c r="A1859" s="18" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1859" s="22" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/instalacion-nuevo-alumbrado-barrio-andra-mari/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1859" s="20" t="n"/>
+      <c r="D1859" s="20" t="n"/>
+      <c r="E1859" s="20" t="n"/>
+      <c r="F1859" s="20" t="n"/>
+    </row>
+    <row r="1861" ht="30" customHeight="1">
+      <c r="A1861" s="16" t="inlineStr">
+        <is>
+          <t>FICHA 125: EUS-87035</t>
+        </is>
+      </c>
+      <c r="B1861" s="17" t="n"/>
+      <c r="C1861" s="17" t="n"/>
+      <c r="D1861" s="17" t="n"/>
+      <c r="E1861" s="17" t="n"/>
+      <c r="F1861" s="17" t="n"/>
+    </row>
+    <row r="1862" ht="20" customHeight="1">
+      <c r="A1862" s="18" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1862" s="19" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1862" s="20" t="n"/>
+      <c r="D1862" s="20" t="n"/>
+      <c r="E1862" s="20" t="n"/>
+      <c r="F1862" s="20" t="n"/>
+    </row>
+    <row r="1863" ht="45" customHeight="1">
+      <c r="A1863" s="18" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1863" s="19" t="inlineStr">
+        <is>
+          <t>Implementación en gis de la infraestructura municipal de limpieza de instalaciones mediante tecnología NFC</t>
+        </is>
+      </c>
+      <c r="C1863" s="20" t="n"/>
+      <c r="D1863" s="20" t="n"/>
+      <c r="E1863" s="20" t="n"/>
+      <c r="F1863" s="20" t="n"/>
+    </row>
+    <row r="1864" ht="20" customHeight="1">
+      <c r="A1864" s="18" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1864" s="19" t="inlineStr">
+        <is>
+          <t>EUS-87035</t>
+        </is>
+      </c>
+      <c r="C1864" s="20" t="n"/>
+      <c r="D1864" s="20" t="n"/>
+      <c r="E1864" s="20" t="n"/>
+      <c r="F1864" s="20" t="n"/>
+    </row>
+    <row r="1865" ht="20" customHeight="1">
+      <c r="A1865" s="18" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1865" s="19" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1865" s="20" t="n"/>
+      <c r="D1865" s="20" t="n"/>
+      <c r="E1865" s="20" t="n"/>
+      <c r="F1865" s="20" t="n"/>
+    </row>
+    <row r="1866" ht="20" customHeight="1">
+      <c r="A1866" s="18" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1866" s="19" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1866" s="20" t="n"/>
+      <c r="D1866" s="20" t="n"/>
+      <c r="E1866" s="20" t="n"/>
+      <c r="F1866" s="20" t="n"/>
+    </row>
+    <row r="1867" ht="20" customHeight="1">
+      <c r="A1867" s="18" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1867" s="19" t="inlineStr"/>
+      <c r="C1867" s="20" t="n"/>
+      <c r="D1867" s="20" t="n"/>
+      <c r="E1867" s="20" t="n"/>
+      <c r="F1867" s="20" t="n"/>
+    </row>
+    <row r="1868" ht="20" customHeight="1">
+      <c r="A1868" s="18" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1868" s="19" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1868" s="20" t="n"/>
+      <c r="D1868" s="20" t="n"/>
+      <c r="E1868" s="20" t="n"/>
+      <c r="F1868" s="20" t="n"/>
+    </row>
+    <row r="1869" ht="20" customHeight="1">
+      <c r="A1869" s="18" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1869" s="19" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1869" s="20" t="n"/>
+      <c r="D1869" s="20" t="n"/>
+      <c r="E1869" s="20" t="n"/>
+      <c r="F1869" s="20" t="n"/>
+    </row>
+    <row r="1870" ht="20" customHeight="1">
+      <c r="A1870" s="18" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1870" s="19" t="inlineStr"/>
+      <c r="C1870" s="20" t="n"/>
+      <c r="D1870" s="20" t="n"/>
+      <c r="E1870" s="20" t="n"/>
+      <c r="F1870" s="20" t="n"/>
+    </row>
+    <row r="1871" ht="20" customHeight="1">
+      <c r="A1871" s="18" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1871" s="19" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1871" s="20" t="n"/>
+      <c r="D1871" s="20" t="n"/>
+      <c r="E1871" s="20" t="n"/>
+      <c r="F1871" s="20" t="n"/>
+    </row>
+    <row r="1872" ht="20" customHeight="1">
+      <c r="A1872" s="18" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1872" s="19" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1872" s="20" t="n"/>
+      <c r="D1872" s="20" t="n"/>
+      <c r="E1872" s="20" t="n"/>
+      <c r="F1872" s="20" t="n"/>
+    </row>
+    <row r="1873" ht="20" customHeight="1">
+      <c r="A1873" s="18" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1873" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1873" s="20" t="n"/>
+      <c r="D1873" s="20" t="n"/>
+      <c r="E1873" s="20" t="n"/>
+      <c r="F1873" s="20" t="n"/>
+    </row>
+    <row r="1874" ht="45" customHeight="1">
+      <c r="A1874" s="18" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1874" s="22" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/implementacion-gis-infraestructura-municipal-limpieza-instalaciones-mediante-tecnologia-nfc/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1874" s="20" t="n"/>
+      <c r="D1874" s="20" t="n"/>
+      <c r="E1874" s="20" t="n"/>
+      <c r="F1874" s="20" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="1694">
+  <mergeCells count="1750">
     <mergeCell ref="B679:F679"/>
     <mergeCell ref="B1765:F1765"/>
     <mergeCell ref="B1010:F1010"/>
@@ -34320,9 +35388,11 @@
     <mergeCell ref="B1105:F1105"/>
     <mergeCell ref="B1403:F1403"/>
     <mergeCell ref="B319:F319"/>
+    <mergeCell ref="B1832:F1832"/>
     <mergeCell ref="B1046:F1046"/>
     <mergeCell ref="B1405:F1405"/>
     <mergeCell ref="A346:F346"/>
+    <mergeCell ref="B1834:F1834"/>
     <mergeCell ref="B1705:F1705"/>
     <mergeCell ref="A136:F136"/>
     <mergeCell ref="B159:F159"/>
@@ -34330,7 +35400,9 @@
     <mergeCell ref="B764:F764"/>
     <mergeCell ref="B1736:F1736"/>
     <mergeCell ref="B161:F161"/>
+    <mergeCell ref="B1858:F1858"/>
     <mergeCell ref="B459:F459"/>
+    <mergeCell ref="B1850:F1850"/>
     <mergeCell ref="B1133:F1133"/>
     <mergeCell ref="A886:F886"/>
     <mergeCell ref="B1431:F1431"/>
@@ -34351,6 +35423,7 @@
     <mergeCell ref="B1144:F1144"/>
     <mergeCell ref="B389:F389"/>
     <mergeCell ref="B1573:F1573"/>
+    <mergeCell ref="B1871:F1871"/>
     <mergeCell ref="A571:F571"/>
     <mergeCell ref="B1152:F1152"/>
     <mergeCell ref="B93:F93"/>
@@ -34358,6 +35431,7 @@
     <mergeCell ref="B1444:F1444"/>
     <mergeCell ref="B385:F385"/>
     <mergeCell ref="B689:F689"/>
+    <mergeCell ref="B1873:F1873"/>
     <mergeCell ref="B86:F86"/>
     <mergeCell ref="B262:F262"/>
     <mergeCell ref="A1771:F1771"/>
@@ -34384,6 +35458,7 @@
     <mergeCell ref="B455:F455"/>
     <mergeCell ref="B491:F491"/>
     <mergeCell ref="B762:F762"/>
+    <mergeCell ref="B1821:F1821"/>
     <mergeCell ref="B34:F34"/>
     <mergeCell ref="B28:F28"/>
     <mergeCell ref="B1218:F1218"/>
@@ -34410,10 +35485,13 @@
     <mergeCell ref="B1569:F1569"/>
     <mergeCell ref="B176:F176"/>
     <mergeCell ref="B1544:F1544"/>
+    <mergeCell ref="B1867:F1867"/>
+    <mergeCell ref="B1842:F1842"/>
     <mergeCell ref="B783:F783"/>
     <mergeCell ref="B468:F468"/>
     <mergeCell ref="B1117:F1117"/>
     <mergeCell ref="B1571:F1571"/>
+    <mergeCell ref="B1869:F1869"/>
     <mergeCell ref="B1529:F1529"/>
     <mergeCell ref="B57:F57"/>
     <mergeCell ref="B171:F171"/>
@@ -34457,6 +35535,7 @@
     <mergeCell ref="B597:F597"/>
     <mergeCell ref="B1113:F1113"/>
     <mergeCell ref="B1542:F1542"/>
+    <mergeCell ref="B1840:F1840"/>
     <mergeCell ref="B808:F808"/>
     <mergeCell ref="B1237:F1237"/>
     <mergeCell ref="B897:F897"/>
@@ -34530,6 +35609,7 @@
     <mergeCell ref="B1656:F1656"/>
     <mergeCell ref="B895:F895"/>
     <mergeCell ref="B1622:F1622"/>
+    <mergeCell ref="A1861:F1861"/>
     <mergeCell ref="B321:F321"/>
     <mergeCell ref="B1040:F1040"/>
     <mergeCell ref="B323:F323"/>
@@ -34606,6 +35686,7 @@
     <mergeCell ref="B1391:F1391"/>
     <mergeCell ref="B332:F332"/>
     <mergeCell ref="B1662:F1662"/>
+    <mergeCell ref="B1820:F1820"/>
     <mergeCell ref="B937:F937"/>
     <mergeCell ref="B1059:F1059"/>
     <mergeCell ref="B1086:F1086"/>
@@ -34613,6 +35694,7 @@
     <mergeCell ref="B1393:F1393"/>
     <mergeCell ref="B1691:F1691"/>
     <mergeCell ref="B632:F632"/>
+    <mergeCell ref="B1822:F1822"/>
     <mergeCell ref="B175:F175"/>
     <mergeCell ref="B790:F790"/>
     <mergeCell ref="B1088:F1088"/>
@@ -34634,6 +35716,7 @@
     <mergeCell ref="B351:F351"/>
     <mergeCell ref="B1744:F1744"/>
     <mergeCell ref="B1535:F1535"/>
+    <mergeCell ref="B1833:F1833"/>
     <mergeCell ref="B774:F774"/>
     <mergeCell ref="B801:F801"/>
     <mergeCell ref="B1072:F1072"/>
@@ -34641,6 +35724,7 @@
     <mergeCell ref="B1108:F1108"/>
     <mergeCell ref="B1406:F1406"/>
     <mergeCell ref="B1289:F1289"/>
+    <mergeCell ref="B1835:F1835"/>
     <mergeCell ref="B48:F48"/>
     <mergeCell ref="B1101:F1101"/>
     <mergeCell ref="B1132:F1132"/>
@@ -34683,6 +35767,7 @@
     <mergeCell ref="A1711:F1711"/>
     <mergeCell ref="B18:F18"/>
     <mergeCell ref="B1506:F1506"/>
+    <mergeCell ref="B1829:F1829"/>
     <mergeCell ref="B1804:F1804"/>
     <mergeCell ref="B797:F797"/>
     <mergeCell ref="B11:F11"/>
@@ -34703,6 +35788,7 @@
     <mergeCell ref="B160:F160"/>
     <mergeCell ref="B527:F527"/>
     <mergeCell ref="B1219:F1219"/>
+    <mergeCell ref="B1857:F1857"/>
     <mergeCell ref="B1123:F1123"/>
     <mergeCell ref="B368:F368"/>
     <mergeCell ref="B1254:F1254"/>
@@ -34710,6 +35796,7 @@
     <mergeCell ref="B1552:F1552"/>
     <mergeCell ref="B1728:F1728"/>
     <mergeCell ref="B1588:F1588"/>
+    <mergeCell ref="B1859:F1859"/>
     <mergeCell ref="B1131:F1131"/>
     <mergeCell ref="B72:F72"/>
     <mergeCell ref="B370:F370"/>
@@ -34763,6 +35850,7 @@
     <mergeCell ref="B910:F910"/>
     <mergeCell ref="B155:F155"/>
     <mergeCell ref="B149:F149"/>
+    <mergeCell ref="B1855:F1855"/>
     <mergeCell ref="B1637:F1637"/>
     <mergeCell ref="B1121:F1121"/>
     <mergeCell ref="B1673:F1673"/>
@@ -34778,9 +35866,11 @@
     <mergeCell ref="B1541:F1541"/>
     <mergeCell ref="B177:F177"/>
     <mergeCell ref="B1568:F1568"/>
+    <mergeCell ref="B1866:F1866"/>
     <mergeCell ref="B79:F79"/>
     <mergeCell ref="B1263:F1263"/>
     <mergeCell ref="B842:F842"/>
+    <mergeCell ref="B1868:F1868"/>
     <mergeCell ref="B836:F836"/>
     <mergeCell ref="B81:F81"/>
     <mergeCell ref="B1563:F1563"/>
@@ -34927,17 +36017,20 @@
     <mergeCell ref="B664:F664"/>
     <mergeCell ref="B1717:F1717"/>
     <mergeCell ref="B658:F658"/>
+    <mergeCell ref="B1848:F1848"/>
     <mergeCell ref="B239:F239"/>
     <mergeCell ref="B1429:F1429"/>
     <mergeCell ref="B1727:F1727"/>
     <mergeCell ref="B1421:F1421"/>
     <mergeCell ref="B1719:F1719"/>
+    <mergeCell ref="B1841:F1841"/>
     <mergeCell ref="B659:F659"/>
     <mergeCell ref="A871:F871"/>
     <mergeCell ref="B232:F232"/>
     <mergeCell ref="B1445:F1445"/>
     <mergeCell ref="B684:F684"/>
     <mergeCell ref="B982:F982"/>
+    <mergeCell ref="B1874:F1874"/>
     <mergeCell ref="B263:F263"/>
     <mergeCell ref="B1447:F1447"/>
     <mergeCell ref="B1745:F1745"/>
@@ -34981,6 +36074,7 @@
     <mergeCell ref="B756:F756"/>
     <mergeCell ref="B329:F329"/>
     <mergeCell ref="B627:F627"/>
+    <mergeCell ref="B1817:F1817"/>
     <mergeCell ref="B758:F758"/>
     <mergeCell ref="B785:F785"/>
     <mergeCell ref="A511:F511"/>
@@ -35004,10 +36098,12 @@
     <mergeCell ref="B1812:F1812"/>
     <mergeCell ref="B1087:F1087"/>
     <mergeCell ref="B1385:F1385"/>
+    <mergeCell ref="B1839:F1839"/>
     <mergeCell ref="B1814:F1814"/>
     <mergeCell ref="B782:F782"/>
     <mergeCell ref="B27:F27"/>
     <mergeCell ref="B42:F42"/>
+    <mergeCell ref="B1870:F1870"/>
     <mergeCell ref="B471:F471"/>
     <mergeCell ref="B769:F769"/>
     <mergeCell ref="B927:F927"/>
@@ -35023,6 +36119,7 @@
     <mergeCell ref="B168:F168"/>
     <mergeCell ref="B472:F472"/>
     <mergeCell ref="B1743:F1743"/>
+    <mergeCell ref="B1865:F1865"/>
     <mergeCell ref="B1438:F1438"/>
     <mergeCell ref="B683:F683"/>
     <mergeCell ref="B1742:F1742"/>
@@ -35087,16 +36184,19 @@
     <mergeCell ref="B1523:F1523"/>
     <mergeCell ref="B66:F66"/>
     <mergeCell ref="B1525:F1525"/>
+    <mergeCell ref="B1823:F1823"/>
     <mergeCell ref="B793:F793"/>
     <mergeCell ref="A406:F406"/>
     <mergeCell ref="B951:F951"/>
     <mergeCell ref="B1249:F1249"/>
     <mergeCell ref="B524:F524"/>
+    <mergeCell ref="B1854:F1854"/>
     <mergeCell ref="B822:F822"/>
     <mergeCell ref="B67:F67"/>
     <mergeCell ref="B953:F953"/>
     <mergeCell ref="B1251:F1251"/>
     <mergeCell ref="B1549:F1549"/>
+    <mergeCell ref="B1856:F1856"/>
     <mergeCell ref="B824:F824"/>
     <mergeCell ref="B69:F69"/>
     <mergeCell ref="B1122:F1122"/>
@@ -35104,6 +36204,7 @@
     <mergeCell ref="B1551:F1551"/>
     <mergeCell ref="B519:F519"/>
     <mergeCell ref="B823:F823"/>
+    <mergeCell ref="B1849:F1849"/>
     <mergeCell ref="B64:F64"/>
     <mergeCell ref="B237:F237"/>
     <mergeCell ref="B666:F666"/>
@@ -35125,6 +36226,7 @@
     <mergeCell ref="B1193:F1193"/>
     <mergeCell ref="B894:F894"/>
     <mergeCell ref="B133:F133"/>
+    <mergeCell ref="A1831:F1831"/>
     <mergeCell ref="B896:F896"/>
     <mergeCell ref="B1194:F1194"/>
     <mergeCell ref="B1188:F1188"/>
@@ -35154,6 +36256,7 @@
     <mergeCell ref="B1338:F1338"/>
     <mergeCell ref="B604:F604"/>
     <mergeCell ref="A61:F61"/>
+    <mergeCell ref="B1847:F1847"/>
     <mergeCell ref="B904:F904"/>
     <mergeCell ref="B635:F635"/>
     <mergeCell ref="B935:F935"/>
@@ -35190,6 +36293,7 @@
     <mergeCell ref="B1007:F1007"/>
     <mergeCell ref="B1001:F1001"/>
     <mergeCell ref="B246:F246"/>
+    <mergeCell ref="A1846:F1846"/>
     <mergeCell ref="B1332:F1332"/>
     <mergeCell ref="B275:F275"/>
     <mergeCell ref="B302:F302"/>
@@ -35290,6 +36394,7 @@
     <mergeCell ref="B337:F337"/>
     <mergeCell ref="B312:F312"/>
     <mergeCell ref="B610:F610"/>
+    <mergeCell ref="B1825:F1825"/>
     <mergeCell ref="B1064:F1064"/>
     <mergeCell ref="B1100:F1100"/>
     <mergeCell ref="B1398:F1398"/>
@@ -35298,6 +36403,7 @@
     <mergeCell ref="B643:F643"/>
     <mergeCell ref="B637:F637"/>
     <mergeCell ref="B1669:F1669"/>
+    <mergeCell ref="B1827:F1827"/>
     <mergeCell ref="B1400:F1400"/>
     <mergeCell ref="B1698:F1698"/>
     <mergeCell ref="A1306:F1306"/>
@@ -35306,6 +36412,7 @@
     <mergeCell ref="B365:F365"/>
     <mergeCell ref="B25:F25"/>
     <mergeCell ref="B1240:F1240"/>
+    <mergeCell ref="B1853:F1853"/>
     <mergeCell ref="A1606:F1606"/>
     <mergeCell ref="B236:F236"/>
     <mergeCell ref="B1084:F1084"/>
@@ -35314,6 +36421,7 @@
     <mergeCell ref="B665:F665"/>
     <mergeCell ref="B350:F350"/>
     <mergeCell ref="B1540:F1540"/>
+    <mergeCell ref="B1838:F1838"/>
     <mergeCell ref="B779:F779"/>
     <mergeCell ref="B358:F358"/>
     <mergeCell ref="B53:F53"/>
@@ -35371,6 +36479,7 @@
     <mergeCell ref="B906:F906"/>
     <mergeCell ref="B23:F23"/>
     <mergeCell ref="B145:F145"/>
+    <mergeCell ref="B1851:F1851"/>
     <mergeCell ref="B1511:F1511"/>
     <mergeCell ref="B452:F452"/>
     <mergeCell ref="A661:F661"/>
@@ -35385,6 +36494,7 @@
     <mergeCell ref="B1433:F1433"/>
     <mergeCell ref="B1564:F1564"/>
     <mergeCell ref="B1224:F1224"/>
+    <mergeCell ref="B1862:F1862"/>
     <mergeCell ref="B1137:F1137"/>
     <mergeCell ref="B382:F382"/>
     <mergeCell ref="B1435:F1435"/>
@@ -35393,6 +36503,7 @@
     <mergeCell ref="B1733:F1733"/>
     <mergeCell ref="B674:F674"/>
     <mergeCell ref="B1226:F1226"/>
+    <mergeCell ref="B1864:F1864"/>
     <mergeCell ref="B832:F832"/>
     <mergeCell ref="B77:F77"/>
     <mergeCell ref="B1138:F1138"/>
@@ -35543,6 +36654,7 @@
     <mergeCell ref="A1141:F1141"/>
     <mergeCell ref="B654:F654"/>
     <mergeCell ref="B952:F952"/>
+    <mergeCell ref="B1844:F1844"/>
     <mergeCell ref="B233:F233"/>
     <mergeCell ref="B1259:F1259"/>
     <mergeCell ref="B227:F227"/>
@@ -35631,6 +36743,7 @@
     <mergeCell ref="B1739:F1739"/>
     <mergeCell ref="B340:F340"/>
     <mergeCell ref="B978:F978"/>
+    <mergeCell ref="B1828:F1828"/>
     <mergeCell ref="B1434:F1434"/>
     <mergeCell ref="B41:F41"/>
     <mergeCell ref="B35:F35"/>
@@ -35691,16 +36804,20 @@
     <mergeCell ref="B1061:F1061"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="B1097:F1097"/>
+    <mergeCell ref="B1824:F1824"/>
     <mergeCell ref="B792:F792"/>
     <mergeCell ref="B1063:F1063"/>
+    <mergeCell ref="B1818:F1818"/>
     <mergeCell ref="B1090:F1090"/>
     <mergeCell ref="B1361:F1361"/>
     <mergeCell ref="B1221:F1221"/>
     <mergeCell ref="B1397:F1397"/>
     <mergeCell ref="B1519:F1519"/>
+    <mergeCell ref="B1826:F1826"/>
     <mergeCell ref="B39:F39"/>
     <mergeCell ref="B1092:F1092"/>
     <mergeCell ref="B1521:F1521"/>
+    <mergeCell ref="B1819:F1819"/>
     <mergeCell ref="A961:F961"/>
     <mergeCell ref="B1392:F1392"/>
     <mergeCell ref="B178:F178"/>
@@ -35708,15 +36825,18 @@
     <mergeCell ref="B818:F818"/>
     <mergeCell ref="B1423:F1423"/>
     <mergeCell ref="B364:F364"/>
+    <mergeCell ref="B1852:F1852"/>
     <mergeCell ref="B1537:F1537"/>
     <mergeCell ref="B478:F478"/>
     <mergeCell ref="B65:F65"/>
     <mergeCell ref="B820:F820"/>
     <mergeCell ref="B776:F776"/>
     <mergeCell ref="B1118:F1118"/>
+    <mergeCell ref="B1837:F1837"/>
     <mergeCell ref="B1120:F1120"/>
     <mergeCell ref="B50:F50"/>
     <mergeCell ref="B1418:F1418"/>
+    <mergeCell ref="B1872:F1872"/>
     <mergeCell ref="B479:F479"/>
     <mergeCell ref="B777:F777"/>
     <mergeCell ref="B1749:F1749"/>
@@ -35726,6 +36846,7 @@
     <mergeCell ref="B235:F235"/>
     <mergeCell ref="B1565:F1565"/>
     <mergeCell ref="B533:F533"/>
+    <mergeCell ref="B1863:F1863"/>
     <mergeCell ref="B831:F831"/>
     <mergeCell ref="B1592:F1592"/>
     <mergeCell ref="B103:F103"/>
@@ -35776,6 +36897,7 @@
     <mergeCell ref="B1414:F1414"/>
     <mergeCell ref="B907:F907"/>
     <mergeCell ref="B1205:F1205"/>
+    <mergeCell ref="B1843:F1843"/>
     <mergeCell ref="B1503:F1503"/>
     <mergeCell ref="A1441:F1441"/>
     <mergeCell ref="B318:F318"/>
@@ -35826,6 +36948,7 @@
     <mergeCell ref="B1488:F1488"/>
     <mergeCell ref="B456:F456"/>
     <mergeCell ref="B545:F545"/>
+    <mergeCell ref="A1816:F1816"/>
     <mergeCell ref="B576:F576"/>
     <mergeCell ref="B138:F138"/>
     <mergeCell ref="B113:F113"/>
@@ -35955,6 +37078,7 @@
     <mergeCell ref="B652:F652"/>
     <mergeCell ref="B1538:F1538"/>
     <mergeCell ref="B1714:F1714"/>
+    <mergeCell ref="B1836:F1836"/>
     <mergeCell ref="B1409:F1409"/>
     <mergeCell ref="B1292:F1292"/>
     <mergeCell ref="B1707:F1707"/>
@@ -36084,6 +37208,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1784" r:id="rId119"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1799" r:id="rId120"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1814" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1829" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1844" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1859" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1874" r:id="rId125"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -36095,7 +37223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J122"/>
+  <dimension ref="A1:J126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -40101,12 +41229,12 @@
     <row r="103" ht="28" customHeight="1">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>EUS-23520</t>
+          <t>EUS-78309</t>
         </is>
       </c>
       <c r="B103" s="6" t="inlineStr">
         <is>
-          <t>Contratación para el suministro, sustitución e instalación d</t>
+          <t xml:space="preserve">Servicio de redacción del Plan de Clima y Energía (PCE) del </t>
         </is>
       </c>
       <c r="C103" s="6" t="inlineStr">
@@ -40137,12 +41265,12 @@
     <row r="104" ht="28" customHeight="1">
       <c r="A104" s="6" t="inlineStr">
         <is>
-          <t>EUS-31752</t>
+          <t>EUS-50766</t>
         </is>
       </c>
       <c r="B104" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
+          <t>Contratación para el suministro, sustitución e instalación d</t>
         </is>
       </c>
       <c r="C104" s="6" t="inlineStr">
@@ -40158,7 +41286,7 @@
       <c r="E104" s="6" t="inlineStr"/>
       <c r="F104" s="25" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>MUY ALTA</t>
         </is>
       </c>
       <c r="G104" s="6" t="inlineStr"/>
@@ -40173,12 +41301,12 @@
     <row r="105" ht="28" customHeight="1">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>EUS-23938</t>
+          <t>EUS-67043</t>
         </is>
       </c>
       <c r="B105" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la gestión sostenible de los recursos pesqueros 202</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
         </is>
       </c>
       <c r="C105" s="6" t="inlineStr">
@@ -40209,12 +41337,12 @@
     <row r="106" ht="28" customHeight="1">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>EUS-61297</t>
+          <t>EUS-58756</t>
         </is>
       </c>
       <c r="B106" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la recogida de residuos con la participación de los</t>
+          <t>Ayudas a la gestión sostenible de los recursos pesqueros 202</t>
         </is>
       </c>
       <c r="C106" s="6" t="inlineStr">
@@ -40245,12 +41373,12 @@
     <row r="107" ht="28" customHeight="1">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>EUS-23417</t>
+          <t>EUS-12835</t>
         </is>
       </c>
       <c r="B107" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
+          <t>Ayudas a la recogida de residuos con la participación de los</t>
         </is>
       </c>
       <c r="C107" s="6" t="inlineStr">
@@ -40281,12 +41409,12 @@
     <row r="108" ht="28" customHeight="1">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>EUS-56608</t>
+          <t>EUS-45037</t>
         </is>
       </c>
       <c r="B108" s="6" t="inlineStr">
         <is>
-          <t>servicio de recogida y transporte de residuos papel y cartón</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
         </is>
       </c>
       <c r="C108" s="6" t="inlineStr">
@@ -40317,12 +41445,12 @@
     <row r="109" ht="28" customHeight="1">
       <c r="A109" s="6" t="inlineStr">
         <is>
-          <t>EUS-72014</t>
+          <t>EUS-02688</t>
         </is>
       </c>
       <c r="B109" s="6" t="inlineStr">
         <is>
-          <t>Estudio del estado de las instalaciones, prestación del serv</t>
+          <t>servicio de recogida y transporte de residuos papel y cartón</t>
         </is>
       </c>
       <c r="C109" s="6" t="inlineStr">
@@ -40353,12 +41481,12 @@
     <row r="110" ht="28" customHeight="1">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>EUS-13924</t>
+          <t>EUS-22640</t>
         </is>
       </c>
       <c r="B110" s="6" t="inlineStr">
         <is>
-          <t>Trabajos de limpieza de residuos en los parques de Garaio, L</t>
+          <t>Estudio del estado de las instalaciones, prestación del serv</t>
         </is>
       </c>
       <c r="C110" s="6" t="inlineStr">
@@ -40389,12 +41517,12 @@
     <row r="111" ht="28" customHeight="1">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>EUS-82252</t>
+          <t>EUS-99053</t>
         </is>
       </c>
       <c r="B111" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la contribución de la acuicultura al buen estado am</t>
+          <t>Trabajos de limpieza de residuos en los parques de Garaio, L</t>
         </is>
       </c>
       <c r="C111" s="6" t="inlineStr">
@@ -40410,7 +41538,7 @@
       <c r="E111" s="6" t="inlineStr"/>
       <c r="F111" s="25" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="G111" s="6" t="inlineStr"/>
@@ -40425,12 +41553,12 @@
     <row r="112" ht="28" customHeight="1">
       <c r="A112" s="6" t="inlineStr">
         <is>
-          <t>EUS-41510</t>
+          <t>EUS-99424</t>
         </is>
       </c>
       <c r="B112" s="6" t="inlineStr">
         <is>
-          <t>Ayudas al valor añadido, economía circular y seguridad alime</t>
+          <t>Ayudas a la contribución de la acuicultura al buen estado am</t>
         </is>
       </c>
       <c r="C112" s="6" t="inlineStr">
@@ -40461,12 +41589,12 @@
     <row r="113" ht="28" customHeight="1">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>EUS-19595</t>
+          <t>EUS-66735</t>
         </is>
       </c>
       <c r="B113" s="6" t="inlineStr">
         <is>
-          <t>Vino: el Gobierno Vasco volverá a convocar este mes las ayud</t>
+          <t>Ayudas al valor añadido, economía circular y seguridad alime</t>
         </is>
       </c>
       <c r="C113" s="6" t="inlineStr">
@@ -40497,12 +41625,12 @@
     <row r="114" ht="28" customHeight="1">
       <c r="A114" s="6" t="inlineStr">
         <is>
-          <t>EUS-04008</t>
+          <t>EUS-86673</t>
         </is>
       </c>
       <c r="B114" s="6" t="inlineStr">
         <is>
-          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de</t>
+          <t>Vino: el Gobierno Vasco volverá a convocar este mes las ayud</t>
         </is>
       </c>
       <c r="C114" s="6" t="inlineStr">
@@ -40533,12 +41661,12 @@
     <row r="115" ht="28" customHeight="1">
       <c r="A115" s="6" t="inlineStr">
         <is>
-          <t>EUS-33753</t>
+          <t>EUS-67797</t>
         </is>
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para c</t>
+          <t>Nueva Bauhaus Europea y NEB Boost: 13 premios y 20 ayudas de</t>
         </is>
       </c>
       <c r="C115" s="6" t="inlineStr">
@@ -40569,12 +41697,12 @@
     <row r="116" ht="28" customHeight="1">
       <c r="A116" s="6" t="inlineStr">
         <is>
-          <t>EUS-15589</t>
+          <t>EUS-19482</t>
         </is>
       </c>
       <c r="B116" s="6" t="inlineStr">
         <is>
-          <t>Servicio de limpieza integral del Complejo Deportivo Mendizo</t>
+          <t>Salud, cáncer. Programas de Horizon, EIC, IHI. Apoyos para c</t>
         </is>
       </c>
       <c r="C116" s="6" t="inlineStr">
@@ -40605,12 +41733,12 @@
     <row r="117" ht="28" customHeight="1">
       <c r="A117" s="6" t="inlineStr">
         <is>
-          <t>EUS-84889</t>
+          <t>EUS-20210</t>
         </is>
       </c>
       <c r="B117" s="6" t="inlineStr">
         <is>
-          <t>Servicios Profesionales en el ámbito de la Presencia Digital</t>
+          <t>Redacción del proyecto de los trabajos de mejora de las rede</t>
         </is>
       </c>
       <c r="C117" s="6" t="inlineStr">
@@ -40641,12 +41769,12 @@
     <row r="118" ht="28" customHeight="1">
       <c r="A118" s="6" t="inlineStr">
         <is>
-          <t>EUS-16064</t>
+          <t>EUS-08817</t>
         </is>
       </c>
       <c r="B118" s="6" t="inlineStr">
         <is>
-          <t>Obras de distribución de la red de saneamiento y aguas pluvi</t>
+          <t>Servicio de recogida, custodia y protección de animales de c</t>
         </is>
       </c>
       <c r="C118" s="6" t="inlineStr">
@@ -40677,12 +41805,12 @@
     <row r="119" ht="28" customHeight="1">
       <c r="A119" s="6" t="inlineStr">
         <is>
-          <t>EUS-36514</t>
+          <t>EUS-72869</t>
         </is>
       </c>
       <c r="B119" s="6" t="inlineStr">
         <is>
-          <t>Elaboración del diagnóstico de vivienda en el termino munici</t>
+          <t>Dirección de obra y reparación y sustitución de la cobertura</t>
         </is>
       </c>
       <c r="C119" s="6" t="inlineStr">
@@ -40713,12 +41841,12 @@
     <row r="120" ht="28" customHeight="1">
       <c r="A120" s="6" t="inlineStr">
         <is>
-          <t>EUS-98928</t>
+          <t>EUS-40836</t>
         </is>
       </c>
       <c r="B120" s="6" t="inlineStr">
         <is>
-          <t>Instalación de nuevo alumbrado en el barrio de Andra Mari</t>
+          <t>Organización y ejecución de un programa de animación en parq</t>
         </is>
       </c>
       <c r="C120" s="6" t="inlineStr">
@@ -40749,12 +41877,12 @@
     <row r="121" ht="28" customHeight="1">
       <c r="A121" s="6" t="inlineStr">
         <is>
-          <t>EUS-29541</t>
+          <t>EUS-53028</t>
         </is>
       </c>
       <c r="B121" s="6" t="inlineStr">
         <is>
-          <t>Implementación en gis de la infraestructura municipal de lim</t>
+          <t>Servicio de limpieza integral del Complejo Deportivo Mendizo</t>
         </is>
       </c>
       <c r="C121" s="6" t="inlineStr">
@@ -40785,12 +41913,12 @@
     <row r="122" ht="28" customHeight="1">
       <c r="A122" s="6" t="inlineStr">
         <is>
-          <t>EUS-78417</t>
+          <t>EUS-78111</t>
         </is>
       </c>
       <c r="B122" s="6" t="inlineStr">
         <is>
-          <t>Recogida y adopción de perros</t>
+          <t>Servicios Profesionales en el ámbito de la Presencia Digital</t>
         </is>
       </c>
       <c r="C122" s="6" t="inlineStr">
@@ -40818,8 +41946,152 @@
       <c r="I122" s="6" t="inlineStr"/>
       <c r="J122" s="6" t="inlineStr"/>
     </row>
+    <row r="123" ht="28" customHeight="1">
+      <c r="A123" s="6" t="inlineStr">
+        <is>
+          <t>EUS-36895</t>
+        </is>
+      </c>
+      <c r="B123" s="6" t="inlineStr">
+        <is>
+          <t>Obras de distribución de la red de saneamiento y aguas pluvi</t>
+        </is>
+      </c>
+      <c r="C123" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D123" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E123" s="6" t="inlineStr"/>
+      <c r="F123" s="25" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G123" s="6" t="inlineStr"/>
+      <c r="H123" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I123" s="6" t="inlineStr"/>
+      <c r="J123" s="6" t="inlineStr"/>
+    </row>
+    <row r="124" ht="28" customHeight="1">
+      <c r="A124" s="6" t="inlineStr">
+        <is>
+          <t>EUS-78769</t>
+        </is>
+      </c>
+      <c r="B124" s="6" t="inlineStr">
+        <is>
+          <t>Elaboración del diagnóstico de vivienda en el termino munici</t>
+        </is>
+      </c>
+      <c r="C124" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D124" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E124" s="6" t="inlineStr"/>
+      <c r="F124" s="25" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G124" s="6" t="inlineStr"/>
+      <c r="H124" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I124" s="6" t="inlineStr"/>
+      <c r="J124" s="6" t="inlineStr"/>
+    </row>
+    <row r="125" ht="28" customHeight="1">
+      <c r="A125" s="6" t="inlineStr">
+        <is>
+          <t>EUS-87188</t>
+        </is>
+      </c>
+      <c r="B125" s="6" t="inlineStr">
+        <is>
+          <t>Instalación de nuevo alumbrado en el barrio de Andra Mari</t>
+        </is>
+      </c>
+      <c r="C125" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D125" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E125" s="6" t="inlineStr"/>
+      <c r="F125" s="25" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G125" s="6" t="inlineStr"/>
+      <c r="H125" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I125" s="6" t="inlineStr"/>
+      <c r="J125" s="6" t="inlineStr"/>
+    </row>
+    <row r="126" ht="28" customHeight="1">
+      <c r="A126" s="6" t="inlineStr">
+        <is>
+          <t>EUS-87035</t>
+        </is>
+      </c>
+      <c r="B126" s="6" t="inlineStr">
+        <is>
+          <t>Implementación en gis de la infraestructura municipal de lim</t>
+        </is>
+      </c>
+      <c r="C126" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D126" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E126" s="6" t="inlineStr"/>
+      <c r="F126" s="25" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G126" s="6" t="inlineStr"/>
+      <c r="H126" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I126" s="6" t="inlineStr"/>
+      <c r="J126" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J122"/>
+  <autoFilter ref="A1:J126"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update funding data 2026-04-10
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Recursos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$126</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$120</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$121</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$115</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -78,12 +78,6 @@
     <font>
       <name val="Leelawadee UI"/>
       <b val="1"/>
-      <color rgb="00DC2626"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Leelawadee UI"/>
-      <b val="1"/>
       <color rgb="0092400E"/>
       <sz val="10"/>
     </font>
@@ -91,6 +85,12 @@
       <name val="Leelawadee UI"/>
       <b val="1"/>
       <color rgb="00065F46"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Leelawadee UI"/>
+      <b val="1"/>
+      <color rgb="00DC2626"/>
       <sz val="10"/>
     </font>
     <font>
@@ -156,11 +156,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00B45309"/>
       </patternFill>
     </fill>
@@ -177,6 +172,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -262,17 +262,17 @@
     <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -312,8 +312,8 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -679,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M126"/>
+  <dimension ref="A1:M121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -707,7 +707,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 09/04/2026 07:12 - 119 convocatorias - 19 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 10/04/2026 07:16 - 114 convocatorias - 11 nuevas</t>
         </is>
       </c>
     </row>
@@ -6850,11 +6850,7 @@
           <t>Services to Communities to support the achievement of the objectives of the Mission Ocean and Waters</t>
         </is>
       </c>
-      <c r="L105" s="13" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
+      <c r="L105" s="6" t="inlineStr"/>
       <c r="M105" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
@@ -6909,14 +6905,14 @@
       </c>
     </row>
     <row r="107" ht="28" customHeight="1">
-      <c r="A107" s="14" t="inlineStr">
+      <c r="A107" s="13" t="inlineStr">
         <is>
           <t>🇪🇸 España</t>
         </is>
       </c>
     </row>
     <row r="108" ht="40" customHeight="1">
-      <c r="A108" s="15" t="inlineStr">
+      <c r="A108" s="14" t="inlineStr">
         <is>
           <t>España</t>
         </is>
@@ -6967,11 +6963,7 @@
           <t>PERSONAS JURÍDICAS QUE NO DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
         </is>
       </c>
-      <c r="L108" s="13" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
+      <c r="L108" s="6" t="inlineStr"/>
       <c r="M108" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
@@ -6979,24 +6971,24 @@
       </c>
     </row>
     <row r="109" ht="40" customHeight="1">
-      <c r="A109" s="15" t="inlineStr">
+      <c r="A109" s="14" t="inlineStr">
         <is>
           <t>España</t>
         </is>
       </c>
       <c r="B109" s="6" t="inlineStr">
         <is>
-          <t>BDNS-897355</t>
+          <t>BDNS-897535</t>
         </is>
       </c>
       <c r="C109" s="6" t="inlineStr">
         <is>
-          <t>Programa de ayudas digitalización cadena alim. y madera 2025</t>
+          <t>Ayudas a la implantación, modernización y transformación digital de las pequeñas empresas de comercio, servicios personales y hostelería de Vitoria-Gasteiz 2026</t>
         </is>
       </c>
       <c r="D109" s="6" t="inlineStr">
         <is>
-          <t>PAÍS VASCO</t>
+          <t>VITORIA-GASTEIZ</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr">
@@ -7006,12 +6998,12 @@
       </c>
       <c r="F109" s="6" t="inlineStr">
         <is>
-          <t>31/12/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="G109" s="6" t="inlineStr">
         <is>
-          <t>734,022.67 EUR</t>
+          <t>490,000.00 EUR</t>
         </is>
       </c>
       <c r="H109" s="6" t="inlineStr">
@@ -7019,144 +7011,76 @@
           <t>Subvencion Nacional</t>
         </is>
       </c>
-      <c r="I109" s="12" t="inlineStr">
-        <is>
-          <t>MUY ALTA</t>
+      <c r="I109" s="10" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
         </is>
       </c>
       <c r="J109" s="6" t="inlineStr"/>
       <c r="K109" s="6" t="inlineStr">
         <is>
-          <t>PYME Y PERSONAS FÍSICAS QUE DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES21 - PAIS VASCO</t>
-        </is>
-      </c>
-      <c r="L109" s="13" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
+          <t>PYME Y PERSONAS FÍSICAS QUE DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
+        </is>
+      </c>
+      <c r="L109" s="6" t="inlineStr"/>
       <c r="M109" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
         </is>
       </c>
     </row>
-    <row r="110" ht="40" customHeight="1">
+    <row r="110" ht="28" customHeight="1">
       <c r="A110" s="15" t="inlineStr">
         <is>
-          <t>España</t>
-        </is>
-      </c>
-      <c r="B110" s="6" t="inlineStr">
-        <is>
-          <t>BDNS-897535</t>
-        </is>
-      </c>
-      <c r="C110" s="6" t="inlineStr">
-        <is>
-          <t>Ayudas a la implantación, modernización y transformación digital de las pequeñas empresas de comercio, servicios personales y hostelería de Vitoria-Gasteiz 2026</t>
-        </is>
-      </c>
-      <c r="D110" s="6" t="inlineStr">
-        <is>
-          <t>VITORIA-GASTEIZ</t>
-        </is>
-      </c>
-      <c r="E110" s="7" t="inlineStr">
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="40" customHeight="1">
+      <c r="A111" s="16" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B111" s="6" t="inlineStr">
+        <is>
+          <t>EUS-18545</t>
+        </is>
+      </c>
+      <c r="C111" s="6" t="inlineStr">
+        <is>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
+        </is>
+      </c>
+      <c r="D111" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E111" s="7" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F110" s="6" t="inlineStr">
-        <is>
-          <t>05/05/2026</t>
-        </is>
-      </c>
-      <c r="G110" s="6" t="inlineStr">
-        <is>
-          <t>490,000.00 EUR</t>
-        </is>
-      </c>
-      <c r="H110" s="6" t="inlineStr">
-        <is>
-          <t>Subvencion Nacional</t>
-        </is>
-      </c>
-      <c r="I110" s="10" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="J110" s="6" t="inlineStr"/>
-      <c r="K110" s="6" t="inlineStr">
-        <is>
-          <t>PYME Y PERSONAS FÍSICAS QUE DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
-        </is>
-      </c>
-      <c r="L110" s="13" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="M110" s="9" t="inlineStr">
-        <is>
-          <t>Ver</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" ht="40" customHeight="1">
-      <c r="A111" s="15" t="inlineStr">
-        <is>
-          <t>España</t>
-        </is>
-      </c>
-      <c r="B111" s="6" t="inlineStr">
-        <is>
-          <t>BDNS-897198</t>
-        </is>
-      </c>
-      <c r="C111" s="6" t="inlineStr">
-        <is>
-          <t>Ayudas para actividades educativas organizadas por asociaciones del ámbito de las necesidades educativas especiales, curso 2026-2027</t>
-        </is>
-      </c>
-      <c r="D111" s="6" t="inlineStr">
-        <is>
-          <t>VITORIA-GASTEIZ</t>
-        </is>
-      </c>
-      <c r="E111" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F111" s="6" t="inlineStr">
-        <is>
-          <t>29/05/2026</t>
-        </is>
-      </c>
-      <c r="G111" s="6" t="inlineStr">
-        <is>
-          <t>20,000.00 EUR</t>
-        </is>
-      </c>
+      <c r="F111" s="6" t="inlineStr"/>
+      <c r="G111" s="6" t="inlineStr"/>
       <c r="H111" s="6" t="inlineStr">
         <is>
-          <t>Subvencion Nacional</t>
-        </is>
-      </c>
-      <c r="I111" s="10" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
+          <t>Ayuda/Subvencion Euskadi</t>
+        </is>
+      </c>
+      <c r="I111" s="8" t="inlineStr">
+        <is>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="J111" s="6" t="inlineStr"/>
       <c r="K111" s="6" t="inlineStr">
         <is>
-          <t>PERSONAS JURÍDICAS QUE NO DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
-        </is>
-      </c>
-      <c r="L111" s="13" t="inlineStr">
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L111" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7167,27 +7091,75 @@
         </is>
       </c>
     </row>
-    <row r="112" ht="28" customHeight="1">
+    <row r="112" ht="40" customHeight="1">
       <c r="A112" s="16" t="inlineStr">
         <is>
-          <t>🟢 Euskadi</t>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B112" s="6" t="inlineStr">
+        <is>
+          <t>EUS-98881</t>
+        </is>
+      </c>
+      <c r="C112" s="6" t="inlineStr">
+        <is>
+          <t>Ayudas a la gestión sostenible de los recursos pesqueros 2026</t>
+        </is>
+      </c>
+      <c r="D112" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E112" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F112" s="6" t="inlineStr"/>
+      <c r="G112" s="6" t="inlineStr"/>
+      <c r="H112" s="6" t="inlineStr">
+        <is>
+          <t>Ayuda/Subvencion Euskadi</t>
+        </is>
+      </c>
+      <c r="I112" s="8" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J112" s="6" t="inlineStr"/>
+      <c r="K112" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L112" s="17" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M112" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
         </is>
       </c>
     </row>
     <row r="113" ht="40" customHeight="1">
-      <c r="A113" s="17" t="inlineStr">
+      <c r="A113" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B113" s="6" t="inlineStr">
         <is>
-          <t>EUS-25527</t>
+          <t>EUS-38210</t>
         </is>
       </c>
       <c r="C113" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
+          <t>Ayudas a la recogida de residuos con la participación de los pescadores en el mar y las playas 2026</t>
         </is>
       </c>
       <c r="D113" s="6" t="inlineStr">
@@ -7218,7 +7190,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L113" s="13" t="inlineStr">
+      <c r="L113" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7230,19 +7202,19 @@
       </c>
     </row>
     <row r="114" ht="40" customHeight="1">
-      <c r="A114" s="17" t="inlineStr">
+      <c r="A114" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B114" s="6" t="inlineStr">
         <is>
-          <t>EUS-67276</t>
+          <t>EUS-62379</t>
         </is>
       </c>
       <c r="C114" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la gestión sostenible de los recursos pesqueros 2026</t>
+          <t>Poli ipurua: conduccion aportacion aire exterior ?filtrado? para ?climatizador vestuarios piscinas?.</t>
         </is>
       </c>
       <c r="D114" s="6" t="inlineStr">
@@ -7259,7 +7231,7 @@
       <c r="G114" s="6" t="inlineStr"/>
       <c r="H114" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="I114" s="8" t="inlineStr">
@@ -7273,7 +7245,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L114" s="13" t="inlineStr">
+      <c r="L114" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7285,19 +7257,19 @@
       </c>
     </row>
     <row r="115" ht="40" customHeight="1">
-      <c r="A115" s="17" t="inlineStr">
+      <c r="A115" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>EUS-54829</t>
+          <t>EUS-68865</t>
         </is>
       </c>
       <c r="C115" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la recogida de residuos con la participación de los pescadores en el mar y las playas 2026</t>
+          <t>Poli orbea: conduccion aportacion aire exterior para ?climatizador sotano?</t>
         </is>
       </c>
       <c r="D115" s="6" t="inlineStr">
@@ -7314,7 +7286,7 @@
       <c r="G115" s="6" t="inlineStr"/>
       <c r="H115" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="I115" s="8" t="inlineStr">
@@ -7328,7 +7300,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L115" s="13" t="inlineStr">
+      <c r="L115" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7340,19 +7312,19 @@
       </c>
     </row>
     <row r="116" ht="40" customHeight="1">
-      <c r="A116" s="17" t="inlineStr">
+      <c r="A116" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B116" s="6" t="inlineStr">
         <is>
-          <t>EUS-45197</t>
+          <t>EUS-45735</t>
         </is>
       </c>
       <c r="C116" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático sin incremento de capacidad 2026</t>
+          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversidad, participación, principios de la UE. Eventos, difusiones e intercambios. Programa de Ciudadanos, Igualdad, Derechos y Valores de la UE (</t>
         </is>
       </c>
       <c r="D116" s="6" t="inlineStr">
@@ -7372,9 +7344,9 @@
           <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
-      <c r="I116" s="8" t="inlineStr">
-        <is>
-          <t>ALTA</t>
+      <c r="I116" s="10" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
         </is>
       </c>
       <c r="J116" s="6" t="inlineStr"/>
@@ -7383,7 +7355,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L116" s="13" t="inlineStr">
+      <c r="L116" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7395,19 +7367,19 @@
       </c>
     </row>
     <row r="117" ht="40" customHeight="1">
-      <c r="A117" s="17" t="inlineStr">
+      <c r="A117" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B117" s="6" t="inlineStr">
         <is>
-          <t>EUS-83922</t>
+          <t>EUS-28095</t>
         </is>
       </c>
       <c r="C117" s="6" t="inlineStr">
         <is>
-          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversidad, participación, principios de la UE. Eventos, difusiones e intercambios. Programa de Ciudadanos, Igualdad, Derechos y Valores de la UE (</t>
+          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el marco de la Intervención Sectorial Vitivinícola del Plan Estratégico (PEPAC) de la Política Agrícola Común de la UE 2023-2027</t>
         </is>
       </c>
       <c r="D117" s="6" t="inlineStr">
@@ -7438,7 +7410,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L117" s="13" t="inlineStr">
+      <c r="L117" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7450,19 +7422,19 @@
       </c>
     </row>
     <row r="118" ht="40" customHeight="1">
-      <c r="A118" s="17" t="inlineStr">
+      <c r="A118" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B118" s="6" t="inlineStr">
         <is>
-          <t>EUS-69965</t>
+          <t>EUS-41533</t>
         </is>
       </c>
       <c r="C118" s="6" t="inlineStr">
         <is>
-          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el marco de la Intervención Sectorial Vitivinícola del Plan Estratégico (PEPAC) de la Política Agrícola Común de la UE 2023-2027</t>
+          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
         </is>
       </c>
       <c r="D118" s="6" t="inlineStr">
@@ -7493,7 +7465,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L118" s="13" t="inlineStr">
+      <c r="L118" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7505,19 +7477,19 @@
       </c>
     </row>
     <row r="119" ht="40" customHeight="1">
-      <c r="A119" s="17" t="inlineStr">
+      <c r="A119" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B119" s="6" t="inlineStr">
         <is>
-          <t>EUS-97870</t>
+          <t>EUS-46847</t>
         </is>
       </c>
       <c r="C119" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
+          <t>Enajenación mediante procedimiento de subasta pública del local letra D del entresuelo del edificio ubicado en la Avenida de Navarra nº 16 de Pasaia</t>
         </is>
       </c>
       <c r="D119" s="6" t="inlineStr">
@@ -7534,7 +7506,7 @@
       <c r="G119" s="6" t="inlineStr"/>
       <c r="H119" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="I119" s="10" t="inlineStr">
@@ -7548,7 +7520,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L119" s="13" t="inlineStr">
+      <c r="L119" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7560,19 +7532,19 @@
       </c>
     </row>
     <row r="120" ht="40" customHeight="1">
-      <c r="A120" s="17" t="inlineStr">
+      <c r="A120" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B120" s="6" t="inlineStr">
         <is>
-          <t>EUS-63161</t>
+          <t>EUS-44891</t>
         </is>
       </c>
       <c r="C120" s="6" t="inlineStr">
         <is>
-          <t>Ayudas al valor añadido, economía circular y seguridad alimentaria 2026</t>
+          <t>Suministro de Equipamiento para ampliaciones de capacidad de la red de transporte de ITELAZPI S.A</t>
         </is>
       </c>
       <c r="D120" s="6" t="inlineStr">
@@ -7589,7 +7561,7 @@
       <c r="G120" s="6" t="inlineStr"/>
       <c r="H120" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="I120" s="10" t="inlineStr">
@@ -7603,7 +7575,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L120" s="13" t="inlineStr">
+      <c r="L120" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7615,19 +7587,19 @@
       </c>
     </row>
     <row r="121" ht="40" customHeight="1">
-      <c r="A121" s="17" t="inlineStr">
+      <c r="A121" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B121" s="6" t="inlineStr">
         <is>
-          <t>EUS-27678</t>
+          <t>EUS-95830</t>
         </is>
       </c>
       <c r="C121" s="6" t="inlineStr">
         <is>
-          <t>Reparación máquina M300 y M104 de limpieza de piezas de taller</t>
+          <t>Suministro de 4 mesas tipo picnic para zona verde en el Polígono Zubieta</t>
         </is>
       </c>
       <c r="D121" s="6" t="inlineStr">
@@ -7658,7 +7630,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L121" s="13" t="inlineStr">
+      <c r="L121" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7669,287 +7641,12 @@
         </is>
       </c>
     </row>
-    <row r="122" ht="40" customHeight="1">
-      <c r="A122" s="17" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="B122" s="6" t="inlineStr">
-        <is>
-          <t>EUS-78269</t>
-        </is>
-      </c>
-      <c r="C122" s="6" t="inlineStr">
-        <is>
-          <t>Reparación manguera de limpieza marquesinas</t>
-        </is>
-      </c>
-      <c r="D122" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="E122" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F122" s="6" t="inlineStr"/>
-      <c r="G122" s="6" t="inlineStr"/>
-      <c r="H122" s="6" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I122" s="10" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="J122" s="6" t="inlineStr"/>
-      <c r="K122" s="6" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="L122" s="13" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="M122" s="9" t="inlineStr">
-        <is>
-          <t>Ver</t>
-        </is>
-      </c>
-    </row>
-    <row r="123" ht="40" customHeight="1">
-      <c r="A123" s="17" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="B123" s="6" t="inlineStr">
-        <is>
-          <t>EUS-87993</t>
-        </is>
-      </c>
-      <c r="C123" s="6" t="inlineStr">
-        <is>
-          <t>Reparación manguera de limpieza marquesinas</t>
-        </is>
-      </c>
-      <c r="D123" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="E123" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F123" s="6" t="inlineStr"/>
-      <c r="G123" s="6" t="inlineStr"/>
-      <c r="H123" s="6" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I123" s="10" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="J123" s="6" t="inlineStr"/>
-      <c r="K123" s="6" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="L123" s="13" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="M123" s="9" t="inlineStr">
-        <is>
-          <t>Ver</t>
-        </is>
-      </c>
-    </row>
-    <row r="124" ht="40" customHeight="1">
-      <c r="A124" s="17" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="B124" s="6" t="inlineStr">
-        <is>
-          <t>EUS-99225</t>
-        </is>
-      </c>
-      <c r="C124" s="6" t="inlineStr">
-        <is>
-          <t>Reparación manguera de limpieza marquesinas</t>
-        </is>
-      </c>
-      <c r="D124" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="E124" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F124" s="6" t="inlineStr"/>
-      <c r="G124" s="6" t="inlineStr"/>
-      <c r="H124" s="6" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I124" s="10" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="J124" s="6" t="inlineStr"/>
-      <c r="K124" s="6" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="L124" s="13" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="M124" s="9" t="inlineStr">
-        <is>
-          <t>Ver</t>
-        </is>
-      </c>
-    </row>
-    <row r="125" ht="40" customHeight="1">
-      <c r="A125" s="17" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="B125" s="6" t="inlineStr">
-        <is>
-          <t>EUS-09085</t>
-        </is>
-      </c>
-      <c r="C125" s="6" t="inlineStr">
-        <is>
-          <t>Transporte Internacional de compra de recambios</t>
-        </is>
-      </c>
-      <c r="D125" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="E125" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F125" s="6" t="inlineStr"/>
-      <c r="G125" s="6" t="inlineStr"/>
-      <c r="H125" s="6" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I125" s="10" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="J125" s="6" t="inlineStr"/>
-      <c r="K125" s="6" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="L125" s="13" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="M125" s="9" t="inlineStr">
-        <is>
-          <t>Ver</t>
-        </is>
-      </c>
-    </row>
-    <row r="126" ht="40" customHeight="1">
-      <c r="A126" s="17" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="B126" s="6" t="inlineStr">
-        <is>
-          <t>EUS-46800</t>
-        </is>
-      </c>
-      <c r="C126" s="6" t="inlineStr">
-        <is>
-          <t>Reparación máquina M300 de limpieza de piezas de taller carrocería</t>
-        </is>
-      </c>
-      <c r="D126" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="E126" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F126" s="6" t="inlineStr"/>
-      <c r="G126" s="6" t="inlineStr"/>
-      <c r="H126" s="6" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I126" s="10" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="J126" s="6" t="inlineStr"/>
-      <c r="K126" s="6" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="L126" s="13" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="M126" s="9" t="inlineStr">
-        <is>
-          <t>Ver</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:M126"/>
+  <autoFilter ref="A4:M121"/>
   <mergeCells count="5">
-    <mergeCell ref="A112:M112"/>
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A5:M5"/>
+    <mergeCell ref="A110:M110"/>
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A107:M107"/>
   </mergeCells>
@@ -8057,8 +7754,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M106" r:id="rId101"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M108" r:id="rId102"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M109" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M110" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M111" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M111" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M112" r:id="rId105"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M113" r:id="rId106"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M114" r:id="rId107"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M115" r:id="rId108"/>
@@ -8068,11 +7765,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M119" r:id="rId112"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M120" r:id="rId113"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M121" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M122" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M123" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M124" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M125" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M126" r:id="rId119"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8084,7 +7776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1784"/>
+  <dimension ref="A1:F1709"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -30190,7 +29882,7 @@
     <row r="1531" ht="30" customHeight="1">
       <c r="A1531" s="18" t="inlineStr">
         <is>
-          <t>FICHA 103: BDNS-897355</t>
+          <t>FICHA 103: BDNS-897535</t>
         </is>
       </c>
       <c r="B1531" s="19" t="n"/>
@@ -30215,7 +29907,7 @@
       <c r="E1532" s="22" t="n"/>
       <c r="F1532" s="22" t="n"/>
     </row>
-    <row r="1533" ht="20" customHeight="1">
+    <row r="1533" ht="45" customHeight="1">
       <c r="A1533" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -30223,7 +29915,7 @@
       </c>
       <c r="B1533" s="21" t="inlineStr">
         <is>
-          <t>Programa de ayudas digitalización cadena alim. y madera 2025</t>
+          <t>Ayudas a la implantación, modernización y transformación digital de las pequeñas empresas de comercio, servicios personales y hostelería de Vitoria-Gasteiz 2026</t>
         </is>
       </c>
       <c r="C1533" s="22" t="n"/>
@@ -30239,7 +29931,7 @@
       </c>
       <c r="B1534" s="21" t="inlineStr">
         <is>
-          <t>BDNS-897355</t>
+          <t>BDNS-897535</t>
         </is>
       </c>
       <c r="C1534" s="22" t="n"/>
@@ -30255,7 +29947,7 @@
       </c>
       <c r="B1535" s="21" t="inlineStr">
         <is>
-          <t>PAÍS VASCO</t>
+          <t>VITORIA-GASTEIZ</t>
         </is>
       </c>
       <c r="C1535" s="22" t="n"/>
@@ -30287,7 +29979,7 @@
       </c>
       <c r="B1537" s="21" t="inlineStr">
         <is>
-          <t>31/12/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="C1537" s="22" t="n"/>
@@ -30303,7 +29995,7 @@
       </c>
       <c r="B1538" s="21" t="inlineStr">
         <is>
-          <t>734,022.67 EUR</t>
+          <t>490,000.00 EUR</t>
         </is>
       </c>
       <c r="C1538" s="22" t="n"/>
@@ -30335,7 +30027,7 @@
       </c>
       <c r="B1540" s="21" t="inlineStr">
         <is>
-          <t>BDNS 897355</t>
+          <t>BDNS 897535</t>
         </is>
       </c>
       <c r="C1540" s="22" t="n"/>
@@ -30351,7 +30043,7 @@
       </c>
       <c r="B1541" s="21" t="inlineStr">
         <is>
-          <t>PYME Y PERSONAS FÍSICAS QUE DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES21 - PAIS VASCO</t>
+          <t>PYME Y PERSONAS FÍSICAS QUE DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
         </is>
       </c>
       <c r="C1541" s="22" t="n"/>
@@ -30377,9 +30069,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B1543" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MUY ALTA — </t>
+      <c r="B1543" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
         </is>
       </c>
       <c r="C1543" s="22" t="n"/>
@@ -30395,7 +30087,7 @@
       </c>
       <c r="B1544" s="24" t="inlineStr">
         <is>
-          <t>https://www.infosubvenciones.es/bdnstrans/GE/es/convocatoria/897355</t>
+          <t>https://www.infosubvenciones.es/bdnstrans/GE/es/convocatoria/897535</t>
         </is>
       </c>
       <c r="C1544" s="22" t="n"/>
@@ -30406,7 +30098,7 @@
     <row r="1546" ht="30" customHeight="1">
       <c r="A1546" s="18" t="inlineStr">
         <is>
-          <t>FICHA 104: BDNS-897535</t>
+          <t>FICHA 104: EUS-18545</t>
         </is>
       </c>
       <c r="B1546" s="19" t="n"/>
@@ -30423,7 +30115,7 @@
       </c>
       <c r="B1547" s="21" t="inlineStr">
         <is>
-          <t>🇪🇸 España</t>
+          <t>🟢 Euskadi</t>
         </is>
       </c>
       <c r="C1547" s="22" t="n"/>
@@ -30439,7 +30131,7 @@
       </c>
       <c r="B1548" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a la implantación, modernización y transformación digital de las pequeñas empresas de comercio, servicios personales y hostelería de Vitoria-Gasteiz 2026</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
         </is>
       </c>
       <c r="C1548" s="22" t="n"/>
@@ -30455,7 +30147,7 @@
       </c>
       <c r="B1549" s="21" t="inlineStr">
         <is>
-          <t>BDNS-897535</t>
+          <t>EUS-18545</t>
         </is>
       </c>
       <c r="C1549" s="22" t="n"/>
@@ -30471,7 +30163,7 @@
       </c>
       <c r="B1550" s="21" t="inlineStr">
         <is>
-          <t>VITORIA-GASTEIZ</t>
+          <t>Euskadi</t>
         </is>
       </c>
       <c r="C1550" s="22" t="n"/>
@@ -30501,11 +30193,7 @@
           <t>Deadline</t>
         </is>
       </c>
-      <c r="B1552" s="21" t="inlineStr">
-        <is>
-          <t>05/05/2026</t>
-        </is>
-      </c>
+      <c r="B1552" s="21" t="inlineStr"/>
       <c r="C1552" s="22" t="n"/>
       <c r="D1552" s="22" t="n"/>
       <c r="E1552" s="22" t="n"/>
@@ -30519,7 +30207,7 @@
       </c>
       <c r="B1553" s="21" t="inlineStr">
         <is>
-          <t>490,000.00 EUR</t>
+          <t>No disponible</t>
         </is>
       </c>
       <c r="C1553" s="22" t="n"/>
@@ -30535,7 +30223,7 @@
       </c>
       <c r="B1554" s="21" t="inlineStr">
         <is>
-          <t>Subvencion Nacional</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C1554" s="22" t="n"/>
@@ -30549,17 +30237,13 @@
           <t>Call ID</t>
         </is>
       </c>
-      <c r="B1555" s="21" t="inlineStr">
-        <is>
-          <t>BDNS 897535</t>
-        </is>
-      </c>
+      <c r="B1555" s="21" t="inlineStr"/>
       <c r="C1555" s="22" t="n"/>
       <c r="D1555" s="22" t="n"/>
       <c r="E1555" s="22" t="n"/>
       <c r="F1555" s="22" t="n"/>
     </row>
-    <row r="1556" ht="45" customHeight="1">
+    <row r="1556" ht="20" customHeight="1">
       <c r="A1556" s="20" t="inlineStr">
         <is>
           <t>Descripcion</t>
@@ -30567,7 +30251,7 @@
       </c>
       <c r="B1556" s="21" t="inlineStr">
         <is>
-          <t>PYME Y PERSONAS FÍSICAS QUE DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
       <c r="C1556" s="22" t="n"/>
@@ -30581,7 +30265,11 @@
           <t>Tags</t>
         </is>
       </c>
-      <c r="B1557" s="21" t="inlineStr"/>
+      <c r="B1557" s="21" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
       <c r="C1557" s="22" t="n"/>
       <c r="D1557" s="22" t="n"/>
       <c r="E1557" s="22" t="n"/>
@@ -30593,9 +30281,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B1558" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
+      <c r="B1558" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALTA — </t>
         </is>
       </c>
       <c r="C1558" s="22" t="n"/>
@@ -30603,7 +30291,7 @@
       <c r="E1558" s="22" t="n"/>
       <c r="F1558" s="22" t="n"/>
     </row>
-    <row r="1559" ht="20" customHeight="1">
+    <row r="1559" ht="45" customHeight="1">
       <c r="A1559" s="20" t="inlineStr">
         <is>
           <t>Enlace al portal</t>
@@ -30611,7 +30299,7 @@
       </c>
       <c r="B1559" s="24" t="inlineStr">
         <is>
-          <t>https://www.infosubvenciones.es/bdnstrans/GE/es/convocatoria/897535</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-con-incremento-de-capacidad-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1559" s="22" t="n"/>
@@ -30622,7 +30310,7 @@
     <row r="1561" ht="30" customHeight="1">
       <c r="A1561" s="18" t="inlineStr">
         <is>
-          <t>FICHA 105: BDNS-897198</t>
+          <t>FICHA 105: EUS-98881</t>
         </is>
       </c>
       <c r="B1561" s="19" t="n"/>
@@ -30639,7 +30327,7 @@
       </c>
       <c r="B1562" s="21" t="inlineStr">
         <is>
-          <t>🇪🇸 España</t>
+          <t>🟢 Euskadi</t>
         </is>
       </c>
       <c r="C1562" s="22" t="n"/>
@@ -30647,7 +30335,7 @@
       <c r="E1562" s="22" t="n"/>
       <c r="F1562" s="22" t="n"/>
     </row>
-    <row r="1563" ht="45" customHeight="1">
+    <row r="1563" ht="20" customHeight="1">
       <c r="A1563" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -30655,7 +30343,7 @@
       </c>
       <c r="B1563" s="21" t="inlineStr">
         <is>
-          <t>Ayudas para actividades educativas organizadas por asociaciones del ámbito de las necesidades educativas especiales, curso 2026-2027</t>
+          <t>Ayudas a la gestión sostenible de los recursos pesqueros 2026</t>
         </is>
       </c>
       <c r="C1563" s="22" t="n"/>
@@ -30671,7 +30359,7 @@
       </c>
       <c r="B1564" s="21" t="inlineStr">
         <is>
-          <t>BDNS-897198</t>
+          <t>EUS-98881</t>
         </is>
       </c>
       <c r="C1564" s="22" t="n"/>
@@ -30687,7 +30375,7 @@
       </c>
       <c r="B1565" s="21" t="inlineStr">
         <is>
-          <t>VITORIA-GASTEIZ</t>
+          <t>Euskadi</t>
         </is>
       </c>
       <c r="C1565" s="22" t="n"/>
@@ -30717,11 +30405,7 @@
           <t>Deadline</t>
         </is>
       </c>
-      <c r="B1567" s="21" t="inlineStr">
-        <is>
-          <t>29/05/2026</t>
-        </is>
-      </c>
+      <c r="B1567" s="21" t="inlineStr"/>
       <c r="C1567" s="22" t="n"/>
       <c r="D1567" s="22" t="n"/>
       <c r="E1567" s="22" t="n"/>
@@ -30735,7 +30419,7 @@
       </c>
       <c r="B1568" s="21" t="inlineStr">
         <is>
-          <t>20,000.00 EUR</t>
+          <t>No disponible</t>
         </is>
       </c>
       <c r="C1568" s="22" t="n"/>
@@ -30751,7 +30435,7 @@
       </c>
       <c r="B1569" s="21" t="inlineStr">
         <is>
-          <t>Subvencion Nacional</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C1569" s="22" t="n"/>
@@ -30765,17 +30449,13 @@
           <t>Call ID</t>
         </is>
       </c>
-      <c r="B1570" s="21" t="inlineStr">
-        <is>
-          <t>BDNS 897198</t>
-        </is>
-      </c>
+      <c r="B1570" s="21" t="inlineStr"/>
       <c r="C1570" s="22" t="n"/>
       <c r="D1570" s="22" t="n"/>
       <c r="E1570" s="22" t="n"/>
       <c r="F1570" s="22" t="n"/>
     </row>
-    <row r="1571" ht="45" customHeight="1">
+    <row r="1571" ht="20" customHeight="1">
       <c r="A1571" s="20" t="inlineStr">
         <is>
           <t>Descripcion</t>
@@ -30783,7 +30463,7 @@
       </c>
       <c r="B1571" s="21" t="inlineStr">
         <is>
-          <t>PERSONAS JURÍDICAS QUE NO DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
       <c r="C1571" s="22" t="n"/>
@@ -30797,7 +30477,11 @@
           <t>Tags</t>
         </is>
       </c>
-      <c r="B1572" s="21" t="inlineStr"/>
+      <c r="B1572" s="21" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
       <c r="C1572" s="22" t="n"/>
       <c r="D1572" s="22" t="n"/>
       <c r="E1572" s="22" t="n"/>
@@ -30809,9 +30493,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B1573" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
+      <c r="B1573" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALTA — </t>
         </is>
       </c>
       <c r="C1573" s="22" t="n"/>
@@ -30819,7 +30503,7 @@
       <c r="E1573" s="22" t="n"/>
       <c r="F1573" s="22" t="n"/>
     </row>
-    <row r="1574" ht="20" customHeight="1">
+    <row r="1574" ht="45" customHeight="1">
       <c r="A1574" s="20" t="inlineStr">
         <is>
           <t>Enlace al portal</t>
@@ -30827,7 +30511,7 @@
       </c>
       <c r="B1574" s="24" t="inlineStr">
         <is>
-          <t>https://www.infosubvenciones.es/bdnstrans/GE/es/convocatoria/897198</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-gestion-sostenible-de-los-recursos-pesqueros-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1574" s="22" t="n"/>
@@ -30838,7 +30522,7 @@
     <row r="1576" ht="30" customHeight="1">
       <c r="A1576" s="18" t="inlineStr">
         <is>
-          <t>FICHA 106: EUS-25527</t>
+          <t>FICHA 106: EUS-38210</t>
         </is>
       </c>
       <c r="B1576" s="19" t="n"/>
@@ -30871,7 +30555,7 @@
       </c>
       <c r="B1578" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
+          <t>Ayudas a la recogida de residuos con la participación de los pescadores en el mar y las playas 2026</t>
         </is>
       </c>
       <c r="C1578" s="22" t="n"/>
@@ -30887,7 +30571,7 @@
       </c>
       <c r="B1579" s="21" t="inlineStr">
         <is>
-          <t>EUS-25527</t>
+          <t>EUS-38210</t>
         </is>
       </c>
       <c r="C1579" s="22" t="n"/>
@@ -31031,7 +30715,7 @@
       <c r="E1588" s="22" t="n"/>
       <c r="F1588" s="22" t="n"/>
     </row>
-    <row r="1589" ht="45" customHeight="1">
+    <row r="1589" ht="20" customHeight="1">
       <c r="A1589" s="20" t="inlineStr">
         <is>
           <t>Enlace al portal</t>
@@ -31039,7 +30723,7 @@
       </c>
       <c r="B1589" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-con-incremento-de-capacidad-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/fempa-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1589" s="22" t="n"/>
@@ -31050,7 +30734,7 @@
     <row r="1591" ht="30" customHeight="1">
       <c r="A1591" s="18" t="inlineStr">
         <is>
-          <t>FICHA 107: EUS-67276</t>
+          <t>FICHA 107: EUS-62379</t>
         </is>
       </c>
       <c r="B1591" s="19" t="n"/>
@@ -31075,7 +30759,7 @@
       <c r="E1592" s="22" t="n"/>
       <c r="F1592" s="22" t="n"/>
     </row>
-    <row r="1593" ht="20" customHeight="1">
+    <row r="1593" ht="45" customHeight="1">
       <c r="A1593" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -31083,7 +30767,7 @@
       </c>
       <c r="B1593" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a la gestión sostenible de los recursos pesqueros 2026</t>
+          <t>Poli ipurua: conduccion aportacion aire exterior ?filtrado? para ?climatizador vestuarios piscinas?.</t>
         </is>
       </c>
       <c r="C1593" s="22" t="n"/>
@@ -31099,7 +30783,7 @@
       </c>
       <c r="B1594" s="21" t="inlineStr">
         <is>
-          <t>EUS-67276</t>
+          <t>EUS-62379</t>
         </is>
       </c>
       <c r="C1594" s="22" t="n"/>
@@ -31175,7 +30859,7 @@
       </c>
       <c r="B1599" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C1599" s="22" t="n"/>
@@ -31251,7 +30935,7 @@
       </c>
       <c r="B1604" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-gestion-sostenible-de-los-recursos-pesqueros-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/poli-ipurua-conduccion-aportacion-aire-exterior-filtrado-climatizador-vestuarios-piscinas/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1604" s="22" t="n"/>
@@ -31262,7 +30946,7 @@
     <row r="1606" ht="30" customHeight="1">
       <c r="A1606" s="18" t="inlineStr">
         <is>
-          <t>FICHA 108: EUS-54829</t>
+          <t>FICHA 108: EUS-68865</t>
         </is>
       </c>
       <c r="B1606" s="19" t="n"/>
@@ -31287,7 +30971,7 @@
       <c r="E1607" s="22" t="n"/>
       <c r="F1607" s="22" t="n"/>
     </row>
-    <row r="1608" ht="45" customHeight="1">
+    <row r="1608" ht="20" customHeight="1">
       <c r="A1608" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -31295,7 +30979,7 @@
       </c>
       <c r="B1608" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a la recogida de residuos con la participación de los pescadores en el mar y las playas 2026</t>
+          <t>Poli orbea: conduccion aportacion aire exterior para ?climatizador sotano?</t>
         </is>
       </c>
       <c r="C1608" s="22" t="n"/>
@@ -31311,7 +30995,7 @@
       </c>
       <c r="B1609" s="21" t="inlineStr">
         <is>
-          <t>EUS-54829</t>
+          <t>EUS-68865</t>
         </is>
       </c>
       <c r="C1609" s="22" t="n"/>
@@ -31387,7 +31071,7 @@
       </c>
       <c r="B1614" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C1614" s="22" t="n"/>
@@ -31455,7 +31139,7 @@
       <c r="E1618" s="22" t="n"/>
       <c r="F1618" s="22" t="n"/>
     </row>
-    <row r="1619" ht="20" customHeight="1">
+    <row r="1619" ht="45" customHeight="1">
       <c r="A1619" s="20" t="inlineStr">
         <is>
           <t>Enlace al portal</t>
@@ -31463,7 +31147,7 @@
       </c>
       <c r="B1619" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/fempa-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/poli-orbea-conduccion-aportacion-aire-exterior-climatizador-sotano/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1619" s="22" t="n"/>
@@ -31474,7 +31158,7 @@
     <row r="1621" ht="30" customHeight="1">
       <c r="A1621" s="18" t="inlineStr">
         <is>
-          <t>FICHA 109: EUS-45197</t>
+          <t>FICHA 109: EUS-45735</t>
         </is>
       </c>
       <c r="B1621" s="19" t="n"/>
@@ -31507,7 +31191,7 @@
       </c>
       <c r="B1623" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático sin incremento de capacidad 2026</t>
+          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversidad, participación, principios de la UE. Eventos, difusiones e intercambios. Programa de Ciudadanos, Igualdad, Derechos y Valores de la UE (</t>
         </is>
       </c>
       <c r="C1623" s="22" t="n"/>
@@ -31523,7 +31207,7 @@
       </c>
       <c r="B1624" s="21" t="inlineStr">
         <is>
-          <t>EUS-45197</t>
+          <t>EUS-45735</t>
         </is>
       </c>
       <c r="C1624" s="22" t="n"/>
@@ -31657,9 +31341,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B1633" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ALTA — </t>
+      <c r="B1633" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
         </is>
       </c>
       <c r="C1633" s="22" t="n"/>
@@ -31675,7 +31359,7 @@
       </c>
       <c r="B1634" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-sin-incremento-de-capacidad-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260408cervhirisareak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1634" s="22" t="n"/>
@@ -31686,7 +31370,7 @@
     <row r="1636" ht="30" customHeight="1">
       <c r="A1636" s="18" t="inlineStr">
         <is>
-          <t>FICHA 110: EUS-83922</t>
+          <t>FICHA 110: EUS-28095</t>
         </is>
       </c>
       <c r="B1636" s="19" t="n"/>
@@ -31719,7 +31403,7 @@
       </c>
       <c r="B1638" s="21" t="inlineStr">
         <is>
-          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversidad, participación, principios de la UE. Eventos, difusiones e intercambios. Programa de Ciudadanos, Igualdad, Derechos y Valores de la UE (</t>
+          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el marco de la Intervención Sectorial Vitivinícola del Plan Estratégico (PEPAC) de la Política Agrícola Común de la UE 2023-2027</t>
         </is>
       </c>
       <c r="C1638" s="22" t="n"/>
@@ -31735,7 +31419,7 @@
       </c>
       <c r="B1639" s="21" t="inlineStr">
         <is>
-          <t>EUS-83922</t>
+          <t>EUS-28095</t>
         </is>
       </c>
       <c r="C1639" s="22" t="n"/>
@@ -31887,7 +31571,7 @@
       </c>
       <c r="B1649" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260408cervhirisareak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/20260407mahastiardogintza/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1649" s="22" t="n"/>
@@ -31898,7 +31582,7 @@
     <row r="1651" ht="30" customHeight="1">
       <c r="A1651" s="18" t="inlineStr">
         <is>
-          <t>FICHA 111: EUS-69965</t>
+          <t>FICHA 111: EUS-41533</t>
         </is>
       </c>
       <c r="B1651" s="19" t="n"/>
@@ -31931,7 +31615,7 @@
       </c>
       <c r="B1653" s="21" t="inlineStr">
         <is>
-          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el marco de la Intervención Sectorial Vitivinícola del Plan Estratégico (PEPAC) de la Política Agrícola Común de la UE 2023-2027</t>
+          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
         </is>
       </c>
       <c r="C1653" s="22" t="n"/>
@@ -31947,7 +31631,7 @@
       </c>
       <c r="B1654" s="21" t="inlineStr">
         <is>
-          <t>EUS-69965</t>
+          <t>EUS-41533</t>
         </is>
       </c>
       <c r="C1654" s="22" t="n"/>
@@ -32099,7 +31783,7 @@
       </c>
       <c r="B1664" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/20260407mahastiardogintza/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-contribucion-de-la-acuicultura-al-buen-estado-ambiental-y-prestacion-de-servicios-ambientales-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1664" s="22" t="n"/>
@@ -32110,7 +31794,7 @@
     <row r="1666" ht="30" customHeight="1">
       <c r="A1666" s="18" t="inlineStr">
         <is>
-          <t>FICHA 112: EUS-97870</t>
+          <t>FICHA 112: EUS-46847</t>
         </is>
       </c>
       <c r="B1666" s="19" t="n"/>
@@ -32143,7 +31827,7 @@
       </c>
       <c r="B1668" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
+          <t>Enajenación mediante procedimiento de subasta pública del local letra D del entresuelo del edificio ubicado en la Avenida de Navarra nº 16 de Pasaia</t>
         </is>
       </c>
       <c r="C1668" s="22" t="n"/>
@@ -32159,7 +31843,7 @@
       </c>
       <c r="B1669" s="21" t="inlineStr">
         <is>
-          <t>EUS-97870</t>
+          <t>EUS-46847</t>
         </is>
       </c>
       <c r="C1669" s="22" t="n"/>
@@ -32235,7 +31919,7 @@
       </c>
       <c r="B1674" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C1674" s="22" t="n"/>
@@ -32311,7 +31995,7 @@
       </c>
       <c r="B1679" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-contribucion-de-la-acuicultura-al-buen-estado-ambiental-y-prestacion-de-servicios-ambientales-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/enajenacion-mediante-procedimiento-subasta-publica-del-local-letra-d-del-entresuelo-del-edificio-ubicado-avenida-navarra-n-16-pasaia/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1679" s="22" t="n"/>
@@ -32322,7 +32006,7 @@
     <row r="1681" ht="30" customHeight="1">
       <c r="A1681" s="18" t="inlineStr">
         <is>
-          <t>FICHA 113: EUS-63161</t>
+          <t>FICHA 113: EUS-44891</t>
         </is>
       </c>
       <c r="B1681" s="19" t="n"/>
@@ -32347,7 +32031,7 @@
       <c r="E1682" s="22" t="n"/>
       <c r="F1682" s="22" t="n"/>
     </row>
-    <row r="1683" ht="20" customHeight="1">
+    <row r="1683" ht="45" customHeight="1">
       <c r="A1683" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -32355,7 +32039,7 @@
       </c>
       <c r="B1683" s="21" t="inlineStr">
         <is>
-          <t>Ayudas al valor añadido, economía circular y seguridad alimentaria 2026</t>
+          <t>Suministro de Equipamiento para ampliaciones de capacidad de la red de transporte de ITELAZPI S.A</t>
         </is>
       </c>
       <c r="C1683" s="22" t="n"/>
@@ -32371,7 +32055,7 @@
       </c>
       <c r="B1684" s="21" t="inlineStr">
         <is>
-          <t>EUS-63161</t>
+          <t>EUS-44891</t>
         </is>
       </c>
       <c r="C1684" s="22" t="n"/>
@@ -32447,7 +32131,7 @@
       </c>
       <c r="B1689" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C1689" s="22" t="n"/>
@@ -32523,7 +32207,7 @@
       </c>
       <c r="B1694" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-valor-anadido-economia-circular-y-seguridad-alimentaria-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-equipamiento-ampliaciones-capacidad-red-transporte-itelazpi-s-a/expapjaso692459/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1694" s="22" t="n"/>
@@ -32534,7 +32218,7 @@
     <row r="1696" ht="30" customHeight="1">
       <c r="A1696" s="18" t="inlineStr">
         <is>
-          <t>FICHA 114: EUS-27678</t>
+          <t>FICHA 114: EUS-95830</t>
         </is>
       </c>
       <c r="B1696" s="19" t="n"/>
@@ -32567,7 +32251,7 @@
       </c>
       <c r="B1698" s="21" t="inlineStr">
         <is>
-          <t>Reparación máquina M300 y M104 de limpieza de piezas de taller</t>
+          <t>Suministro de 4 mesas tipo picnic para zona verde en el Polígono Zubieta</t>
         </is>
       </c>
       <c r="C1698" s="22" t="n"/>
@@ -32583,7 +32267,7 @@
       </c>
       <c r="B1699" s="21" t="inlineStr">
         <is>
-          <t>EUS-27678</t>
+          <t>EUS-95830</t>
         </is>
       </c>
       <c r="C1699" s="22" t="n"/>
@@ -32735,7 +32419,7 @@
       </c>
       <c r="B1709" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/reparacion-maquina-m300-y-m104-limpieza-piezas-taller/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-4-mesas-tipo-picnic-zona-verde-poligono-zubieta/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1709" s="22" t="n"/>
@@ -32743,1070 +32427,9 @@
       <c r="E1709" s="22" t="n"/>
       <c r="F1709" s="22" t="n"/>
     </row>
-    <row r="1711" ht="30" customHeight="1">
-      <c r="A1711" s="18" t="inlineStr">
-        <is>
-          <t>FICHA 115: EUS-78269</t>
-        </is>
-      </c>
-      <c r="B1711" s="19" t="n"/>
-      <c r="C1711" s="19" t="n"/>
-      <c r="D1711" s="19" t="n"/>
-      <c r="E1711" s="19" t="n"/>
-      <c r="F1711" s="19" t="n"/>
-    </row>
-    <row r="1712" ht="20" customHeight="1">
-      <c r="A1712" s="20" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-      <c r="B1712" s="21" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
-        </is>
-      </c>
-      <c r="C1712" s="22" t="n"/>
-      <c r="D1712" s="22" t="n"/>
-      <c r="E1712" s="22" t="n"/>
-      <c r="F1712" s="22" t="n"/>
-    </row>
-    <row r="1713" ht="20" customHeight="1">
-      <c r="A1713" s="20" t="inlineStr">
-        <is>
-          <t>Titulo</t>
-        </is>
-      </c>
-      <c r="B1713" s="21" t="inlineStr">
-        <is>
-          <t>Reparación manguera de limpieza marquesinas</t>
-        </is>
-      </c>
-      <c r="C1713" s="22" t="n"/>
-      <c r="D1713" s="22" t="n"/>
-      <c r="E1713" s="22" t="n"/>
-      <c r="F1713" s="22" t="n"/>
-    </row>
-    <row r="1714" ht="20" customHeight="1">
-      <c r="A1714" s="20" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1714" s="21" t="inlineStr">
-        <is>
-          <t>EUS-78269</t>
-        </is>
-      </c>
-      <c r="C1714" s="22" t="n"/>
-      <c r="D1714" s="22" t="n"/>
-      <c r="E1714" s="22" t="n"/>
-      <c r="F1714" s="22" t="n"/>
-    </row>
-    <row r="1715" ht="20" customHeight="1">
-      <c r="A1715" s="20" t="inlineStr">
-        <is>
-          <t>Programa</t>
-        </is>
-      </c>
-      <c r="B1715" s="21" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="C1715" s="22" t="n"/>
-      <c r="D1715" s="22" t="n"/>
-      <c r="E1715" s="22" t="n"/>
-      <c r="F1715" s="22" t="n"/>
-    </row>
-    <row r="1716" ht="20" customHeight="1">
-      <c r="A1716" s="20" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="B1716" s="21" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C1716" s="22" t="n"/>
-      <c r="D1716" s="22" t="n"/>
-      <c r="E1716" s="22" t="n"/>
-      <c r="F1716" s="22" t="n"/>
-    </row>
-    <row r="1717" ht="20" customHeight="1">
-      <c r="A1717" s="20" t="inlineStr">
-        <is>
-          <t>Deadline</t>
-        </is>
-      </c>
-      <c r="B1717" s="21" t="inlineStr"/>
-      <c r="C1717" s="22" t="n"/>
-      <c r="D1717" s="22" t="n"/>
-      <c r="E1717" s="22" t="n"/>
-      <c r="F1717" s="22" t="n"/>
-    </row>
-    <row r="1718" ht="20" customHeight="1">
-      <c r="A1718" s="20" t="inlineStr">
-        <is>
-          <t>Presupuesto (EUR)</t>
-        </is>
-      </c>
-      <c r="B1718" s="21" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="C1718" s="22" t="n"/>
-      <c r="D1718" s="22" t="n"/>
-      <c r="E1718" s="22" t="n"/>
-      <c r="F1718" s="22" t="n"/>
-    </row>
-    <row r="1719" ht="20" customHeight="1">
-      <c r="A1719" s="20" t="inlineStr">
-        <is>
-          <t>Tipo de Accion</t>
-        </is>
-      </c>
-      <c r="B1719" s="21" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="C1719" s="22" t="n"/>
-      <c r="D1719" s="22" t="n"/>
-      <c r="E1719" s="22" t="n"/>
-      <c r="F1719" s="22" t="n"/>
-    </row>
-    <row r="1720" ht="20" customHeight="1">
-      <c r="A1720" s="20" t="inlineStr">
-        <is>
-          <t>Call ID</t>
-        </is>
-      </c>
-      <c r="B1720" s="21" t="inlineStr"/>
-      <c r="C1720" s="22" t="n"/>
-      <c r="D1720" s="22" t="n"/>
-      <c r="E1720" s="22" t="n"/>
-      <c r="F1720" s="22" t="n"/>
-    </row>
-    <row r="1721" ht="20" customHeight="1">
-      <c r="A1721" s="20" t="inlineStr">
-        <is>
-          <t>Descripcion</t>
-        </is>
-      </c>
-      <c r="B1721" s="21" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="C1721" s="22" t="n"/>
-      <c r="D1721" s="22" t="n"/>
-      <c r="E1721" s="22" t="n"/>
-      <c r="F1721" s="22" t="n"/>
-    </row>
-    <row r="1722" ht="20" customHeight="1">
-      <c r="A1722" s="20" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-      <c r="B1722" s="21" t="inlineStr">
-        <is>
-          <t>energia</t>
-        </is>
-      </c>
-      <c r="C1722" s="22" t="n"/>
-      <c r="D1722" s="22" t="n"/>
-      <c r="E1722" s="22" t="n"/>
-      <c r="F1722" s="22" t="n"/>
-    </row>
-    <row r="1723" ht="20" customHeight="1">
-      <c r="A1723" s="20" t="inlineStr">
-        <is>
-          <t>Relevancia Bilbao</t>
-        </is>
-      </c>
-      <c r="B1723" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
-        </is>
-      </c>
-      <c r="C1723" s="22" t="n"/>
-      <c r="D1723" s="22" t="n"/>
-      <c r="E1723" s="22" t="n"/>
-      <c r="F1723" s="22" t="n"/>
-    </row>
-    <row r="1724" ht="45" customHeight="1">
-      <c r="A1724" s="20" t="inlineStr">
-        <is>
-          <t>Enlace al portal</t>
-        </is>
-      </c>
-      <c r="B1724" s="24" t="inlineStr">
-        <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/reparacion-manguera-limpieza-marquesinas/expcm502145/web01-tramite/es/</t>
-        </is>
-      </c>
-      <c r="C1724" s="22" t="n"/>
-      <c r="D1724" s="22" t="n"/>
-      <c r="E1724" s="22" t="n"/>
-      <c r="F1724" s="22" t="n"/>
-    </row>
-    <row r="1726" ht="30" customHeight="1">
-      <c r="A1726" s="18" t="inlineStr">
-        <is>
-          <t>FICHA 116: EUS-87993</t>
-        </is>
-      </c>
-      <c r="B1726" s="19" t="n"/>
-      <c r="C1726" s="19" t="n"/>
-      <c r="D1726" s="19" t="n"/>
-      <c r="E1726" s="19" t="n"/>
-      <c r="F1726" s="19" t="n"/>
-    </row>
-    <row r="1727" ht="20" customHeight="1">
-      <c r="A1727" s="20" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-      <c r="B1727" s="21" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
-        </is>
-      </c>
-      <c r="C1727" s="22" t="n"/>
-      <c r="D1727" s="22" t="n"/>
-      <c r="E1727" s="22" t="n"/>
-      <c r="F1727" s="22" t="n"/>
-    </row>
-    <row r="1728" ht="20" customHeight="1">
-      <c r="A1728" s="20" t="inlineStr">
-        <is>
-          <t>Titulo</t>
-        </is>
-      </c>
-      <c r="B1728" s="21" t="inlineStr">
-        <is>
-          <t>Reparación manguera de limpieza marquesinas</t>
-        </is>
-      </c>
-      <c r="C1728" s="22" t="n"/>
-      <c r="D1728" s="22" t="n"/>
-      <c r="E1728" s="22" t="n"/>
-      <c r="F1728" s="22" t="n"/>
-    </row>
-    <row r="1729" ht="20" customHeight="1">
-      <c r="A1729" s="20" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1729" s="21" t="inlineStr">
-        <is>
-          <t>EUS-87993</t>
-        </is>
-      </c>
-      <c r="C1729" s="22" t="n"/>
-      <c r="D1729" s="22" t="n"/>
-      <c r="E1729" s="22" t="n"/>
-      <c r="F1729" s="22" t="n"/>
-    </row>
-    <row r="1730" ht="20" customHeight="1">
-      <c r="A1730" s="20" t="inlineStr">
-        <is>
-          <t>Programa</t>
-        </is>
-      </c>
-      <c r="B1730" s="21" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="C1730" s="22" t="n"/>
-      <c r="D1730" s="22" t="n"/>
-      <c r="E1730" s="22" t="n"/>
-      <c r="F1730" s="22" t="n"/>
-    </row>
-    <row r="1731" ht="20" customHeight="1">
-      <c r="A1731" s="20" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="B1731" s="21" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C1731" s="22" t="n"/>
-      <c r="D1731" s="22" t="n"/>
-      <c r="E1731" s="22" t="n"/>
-      <c r="F1731" s="22" t="n"/>
-    </row>
-    <row r="1732" ht="20" customHeight="1">
-      <c r="A1732" s="20" t="inlineStr">
-        <is>
-          <t>Deadline</t>
-        </is>
-      </c>
-      <c r="B1732" s="21" t="inlineStr"/>
-      <c r="C1732" s="22" t="n"/>
-      <c r="D1732" s="22" t="n"/>
-      <c r="E1732" s="22" t="n"/>
-      <c r="F1732" s="22" t="n"/>
-    </row>
-    <row r="1733" ht="20" customHeight="1">
-      <c r="A1733" s="20" t="inlineStr">
-        <is>
-          <t>Presupuesto (EUR)</t>
-        </is>
-      </c>
-      <c r="B1733" s="21" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="C1733" s="22" t="n"/>
-      <c r="D1733" s="22" t="n"/>
-      <c r="E1733" s="22" t="n"/>
-      <c r="F1733" s="22" t="n"/>
-    </row>
-    <row r="1734" ht="20" customHeight="1">
-      <c r="A1734" s="20" t="inlineStr">
-        <is>
-          <t>Tipo de Accion</t>
-        </is>
-      </c>
-      <c r="B1734" s="21" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="C1734" s="22" t="n"/>
-      <c r="D1734" s="22" t="n"/>
-      <c r="E1734" s="22" t="n"/>
-      <c r="F1734" s="22" t="n"/>
-    </row>
-    <row r="1735" ht="20" customHeight="1">
-      <c r="A1735" s="20" t="inlineStr">
-        <is>
-          <t>Call ID</t>
-        </is>
-      </c>
-      <c r="B1735" s="21" t="inlineStr"/>
-      <c r="C1735" s="22" t="n"/>
-      <c r="D1735" s="22" t="n"/>
-      <c r="E1735" s="22" t="n"/>
-      <c r="F1735" s="22" t="n"/>
-    </row>
-    <row r="1736" ht="20" customHeight="1">
-      <c r="A1736" s="20" t="inlineStr">
-        <is>
-          <t>Descripcion</t>
-        </is>
-      </c>
-      <c r="B1736" s="21" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="C1736" s="22" t="n"/>
-      <c r="D1736" s="22" t="n"/>
-      <c r="E1736" s="22" t="n"/>
-      <c r="F1736" s="22" t="n"/>
-    </row>
-    <row r="1737" ht="20" customHeight="1">
-      <c r="A1737" s="20" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-      <c r="B1737" s="21" t="inlineStr">
-        <is>
-          <t>energia</t>
-        </is>
-      </c>
-      <c r="C1737" s="22" t="n"/>
-      <c r="D1737" s="22" t="n"/>
-      <c r="E1737" s="22" t="n"/>
-      <c r="F1737" s="22" t="n"/>
-    </row>
-    <row r="1738" ht="20" customHeight="1">
-      <c r="A1738" s="20" t="inlineStr">
-        <is>
-          <t>Relevancia Bilbao</t>
-        </is>
-      </c>
-      <c r="B1738" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
-        </is>
-      </c>
-      <c r="C1738" s="22" t="n"/>
-      <c r="D1738" s="22" t="n"/>
-      <c r="E1738" s="22" t="n"/>
-      <c r="F1738" s="22" t="n"/>
-    </row>
-    <row r="1739" ht="45" customHeight="1">
-      <c r="A1739" s="20" t="inlineStr">
-        <is>
-          <t>Enlace al portal</t>
-        </is>
-      </c>
-      <c r="B1739" s="24" t="inlineStr">
-        <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/reparacion-manguera-limpieza-marquesinas/expcm502156/web01-tramite/es/</t>
-        </is>
-      </c>
-      <c r="C1739" s="22" t="n"/>
-      <c r="D1739" s="22" t="n"/>
-      <c r="E1739" s="22" t="n"/>
-      <c r="F1739" s="22" t="n"/>
-    </row>
-    <row r="1741" ht="30" customHeight="1">
-      <c r="A1741" s="18" t="inlineStr">
-        <is>
-          <t>FICHA 117: EUS-99225</t>
-        </is>
-      </c>
-      <c r="B1741" s="19" t="n"/>
-      <c r="C1741" s="19" t="n"/>
-      <c r="D1741" s="19" t="n"/>
-      <c r="E1741" s="19" t="n"/>
-      <c r="F1741" s="19" t="n"/>
-    </row>
-    <row r="1742" ht="20" customHeight="1">
-      <c r="A1742" s="20" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-      <c r="B1742" s="21" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
-        </is>
-      </c>
-      <c r="C1742" s="22" t="n"/>
-      <c r="D1742" s="22" t="n"/>
-      <c r="E1742" s="22" t="n"/>
-      <c r="F1742" s="22" t="n"/>
-    </row>
-    <row r="1743" ht="20" customHeight="1">
-      <c r="A1743" s="20" t="inlineStr">
-        <is>
-          <t>Titulo</t>
-        </is>
-      </c>
-      <c r="B1743" s="21" t="inlineStr">
-        <is>
-          <t>Reparación manguera de limpieza marquesinas</t>
-        </is>
-      </c>
-      <c r="C1743" s="22" t="n"/>
-      <c r="D1743" s="22" t="n"/>
-      <c r="E1743" s="22" t="n"/>
-      <c r="F1743" s="22" t="n"/>
-    </row>
-    <row r="1744" ht="20" customHeight="1">
-      <c r="A1744" s="20" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1744" s="21" t="inlineStr">
-        <is>
-          <t>EUS-99225</t>
-        </is>
-      </c>
-      <c r="C1744" s="22" t="n"/>
-      <c r="D1744" s="22" t="n"/>
-      <c r="E1744" s="22" t="n"/>
-      <c r="F1744" s="22" t="n"/>
-    </row>
-    <row r="1745" ht="20" customHeight="1">
-      <c r="A1745" s="20" t="inlineStr">
-        <is>
-          <t>Programa</t>
-        </is>
-      </c>
-      <c r="B1745" s="21" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="C1745" s="22" t="n"/>
-      <c r="D1745" s="22" t="n"/>
-      <c r="E1745" s="22" t="n"/>
-      <c r="F1745" s="22" t="n"/>
-    </row>
-    <row r="1746" ht="20" customHeight="1">
-      <c r="A1746" s="20" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="B1746" s="21" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C1746" s="22" t="n"/>
-      <c r="D1746" s="22" t="n"/>
-      <c r="E1746" s="22" t="n"/>
-      <c r="F1746" s="22" t="n"/>
-    </row>
-    <row r="1747" ht="20" customHeight="1">
-      <c r="A1747" s="20" t="inlineStr">
-        <is>
-          <t>Deadline</t>
-        </is>
-      </c>
-      <c r="B1747" s="21" t="inlineStr"/>
-      <c r="C1747" s="22" t="n"/>
-      <c r="D1747" s="22" t="n"/>
-      <c r="E1747" s="22" t="n"/>
-      <c r="F1747" s="22" t="n"/>
-    </row>
-    <row r="1748" ht="20" customHeight="1">
-      <c r="A1748" s="20" t="inlineStr">
-        <is>
-          <t>Presupuesto (EUR)</t>
-        </is>
-      </c>
-      <c r="B1748" s="21" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="C1748" s="22" t="n"/>
-      <c r="D1748" s="22" t="n"/>
-      <c r="E1748" s="22" t="n"/>
-      <c r="F1748" s="22" t="n"/>
-    </row>
-    <row r="1749" ht="20" customHeight="1">
-      <c r="A1749" s="20" t="inlineStr">
-        <is>
-          <t>Tipo de Accion</t>
-        </is>
-      </c>
-      <c r="B1749" s="21" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="C1749" s="22" t="n"/>
-      <c r="D1749" s="22" t="n"/>
-      <c r="E1749" s="22" t="n"/>
-      <c r="F1749" s="22" t="n"/>
-    </row>
-    <row r="1750" ht="20" customHeight="1">
-      <c r="A1750" s="20" t="inlineStr">
-        <is>
-          <t>Call ID</t>
-        </is>
-      </c>
-      <c r="B1750" s="21" t="inlineStr"/>
-      <c r="C1750" s="22" t="n"/>
-      <c r="D1750" s="22" t="n"/>
-      <c r="E1750" s="22" t="n"/>
-      <c r="F1750" s="22" t="n"/>
-    </row>
-    <row r="1751" ht="20" customHeight="1">
-      <c r="A1751" s="20" t="inlineStr">
-        <is>
-          <t>Descripcion</t>
-        </is>
-      </c>
-      <c r="B1751" s="21" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="C1751" s="22" t="n"/>
-      <c r="D1751" s="22" t="n"/>
-      <c r="E1751" s="22" t="n"/>
-      <c r="F1751" s="22" t="n"/>
-    </row>
-    <row r="1752" ht="20" customHeight="1">
-      <c r="A1752" s="20" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-      <c r="B1752" s="21" t="inlineStr">
-        <is>
-          <t>energia</t>
-        </is>
-      </c>
-      <c r="C1752" s="22" t="n"/>
-      <c r="D1752" s="22" t="n"/>
-      <c r="E1752" s="22" t="n"/>
-      <c r="F1752" s="22" t="n"/>
-    </row>
-    <row r="1753" ht="20" customHeight="1">
-      <c r="A1753" s="20" t="inlineStr">
-        <is>
-          <t>Relevancia Bilbao</t>
-        </is>
-      </c>
-      <c r="B1753" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
-        </is>
-      </c>
-      <c r="C1753" s="22" t="n"/>
-      <c r="D1753" s="22" t="n"/>
-      <c r="E1753" s="22" t="n"/>
-      <c r="F1753" s="22" t="n"/>
-    </row>
-    <row r="1754" ht="45" customHeight="1">
-      <c r="A1754" s="20" t="inlineStr">
-        <is>
-          <t>Enlace al portal</t>
-        </is>
-      </c>
-      <c r="B1754" s="24" t="inlineStr">
-        <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/reparacion-manguera-limpieza-marquesinas/expcm502144/web01-tramite/es/</t>
-        </is>
-      </c>
-      <c r="C1754" s="22" t="n"/>
-      <c r="D1754" s="22" t="n"/>
-      <c r="E1754" s="22" t="n"/>
-      <c r="F1754" s="22" t="n"/>
-    </row>
-    <row r="1756" ht="30" customHeight="1">
-      <c r="A1756" s="18" t="inlineStr">
-        <is>
-          <t>FICHA 118: EUS-09085</t>
-        </is>
-      </c>
-      <c r="B1756" s="19" t="n"/>
-      <c r="C1756" s="19" t="n"/>
-      <c r="D1756" s="19" t="n"/>
-      <c r="E1756" s="19" t="n"/>
-      <c r="F1756" s="19" t="n"/>
-    </row>
-    <row r="1757" ht="20" customHeight="1">
-      <c r="A1757" s="20" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-      <c r="B1757" s="21" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
-        </is>
-      </c>
-      <c r="C1757" s="22" t="n"/>
-      <c r="D1757" s="22" t="n"/>
-      <c r="E1757" s="22" t="n"/>
-      <c r="F1757" s="22" t="n"/>
-    </row>
-    <row r="1758" ht="20" customHeight="1">
-      <c r="A1758" s="20" t="inlineStr">
-        <is>
-          <t>Titulo</t>
-        </is>
-      </c>
-      <c r="B1758" s="21" t="inlineStr">
-        <is>
-          <t>Transporte Internacional de compra de recambios</t>
-        </is>
-      </c>
-      <c r="C1758" s="22" t="n"/>
-      <c r="D1758" s="22" t="n"/>
-      <c r="E1758" s="22" t="n"/>
-      <c r="F1758" s="22" t="n"/>
-    </row>
-    <row r="1759" ht="20" customHeight="1">
-      <c r="A1759" s="20" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1759" s="21" t="inlineStr">
-        <is>
-          <t>EUS-09085</t>
-        </is>
-      </c>
-      <c r="C1759" s="22" t="n"/>
-      <c r="D1759" s="22" t="n"/>
-      <c r="E1759" s="22" t="n"/>
-      <c r="F1759" s="22" t="n"/>
-    </row>
-    <row r="1760" ht="20" customHeight="1">
-      <c r="A1760" s="20" t="inlineStr">
-        <is>
-          <t>Programa</t>
-        </is>
-      </c>
-      <c r="B1760" s="21" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="C1760" s="22" t="n"/>
-      <c r="D1760" s="22" t="n"/>
-      <c r="E1760" s="22" t="n"/>
-      <c r="F1760" s="22" t="n"/>
-    </row>
-    <row r="1761" ht="20" customHeight="1">
-      <c r="A1761" s="20" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="B1761" s="21" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C1761" s="22" t="n"/>
-      <c r="D1761" s="22" t="n"/>
-      <c r="E1761" s="22" t="n"/>
-      <c r="F1761" s="22" t="n"/>
-    </row>
-    <row r="1762" ht="20" customHeight="1">
-      <c r="A1762" s="20" t="inlineStr">
-        <is>
-          <t>Deadline</t>
-        </is>
-      </c>
-      <c r="B1762" s="21" t="inlineStr"/>
-      <c r="C1762" s="22" t="n"/>
-      <c r="D1762" s="22" t="n"/>
-      <c r="E1762" s="22" t="n"/>
-      <c r="F1762" s="22" t="n"/>
-    </row>
-    <row r="1763" ht="20" customHeight="1">
-      <c r="A1763" s="20" t="inlineStr">
-        <is>
-          <t>Presupuesto (EUR)</t>
-        </is>
-      </c>
-      <c r="B1763" s="21" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="C1763" s="22" t="n"/>
-      <c r="D1763" s="22" t="n"/>
-      <c r="E1763" s="22" t="n"/>
-      <c r="F1763" s="22" t="n"/>
-    </row>
-    <row r="1764" ht="20" customHeight="1">
-      <c r="A1764" s="20" t="inlineStr">
-        <is>
-          <t>Tipo de Accion</t>
-        </is>
-      </c>
-      <c r="B1764" s="21" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="C1764" s="22" t="n"/>
-      <c r="D1764" s="22" t="n"/>
-      <c r="E1764" s="22" t="n"/>
-      <c r="F1764" s="22" t="n"/>
-    </row>
-    <row r="1765" ht="20" customHeight="1">
-      <c r="A1765" s="20" t="inlineStr">
-        <is>
-          <t>Call ID</t>
-        </is>
-      </c>
-      <c r="B1765" s="21" t="inlineStr"/>
-      <c r="C1765" s="22" t="n"/>
-      <c r="D1765" s="22" t="n"/>
-      <c r="E1765" s="22" t="n"/>
-      <c r="F1765" s="22" t="n"/>
-    </row>
-    <row r="1766" ht="20" customHeight="1">
-      <c r="A1766" s="20" t="inlineStr">
-        <is>
-          <t>Descripcion</t>
-        </is>
-      </c>
-      <c r="B1766" s="21" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="C1766" s="22" t="n"/>
-      <c r="D1766" s="22" t="n"/>
-      <c r="E1766" s="22" t="n"/>
-      <c r="F1766" s="22" t="n"/>
-    </row>
-    <row r="1767" ht="20" customHeight="1">
-      <c r="A1767" s="20" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-      <c r="B1767" s="21" t="inlineStr">
-        <is>
-          <t>energia</t>
-        </is>
-      </c>
-      <c r="C1767" s="22" t="n"/>
-      <c r="D1767" s="22" t="n"/>
-      <c r="E1767" s="22" t="n"/>
-      <c r="F1767" s="22" t="n"/>
-    </row>
-    <row r="1768" ht="20" customHeight="1">
-      <c r="A1768" s="20" t="inlineStr">
-        <is>
-          <t>Relevancia Bilbao</t>
-        </is>
-      </c>
-      <c r="B1768" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
-        </is>
-      </c>
-      <c r="C1768" s="22" t="n"/>
-      <c r="D1768" s="22" t="n"/>
-      <c r="E1768" s="22" t="n"/>
-      <c r="F1768" s="22" t="n"/>
-    </row>
-    <row r="1769" ht="45" customHeight="1">
-      <c r="A1769" s="20" t="inlineStr">
-        <is>
-          <t>Enlace al portal</t>
-        </is>
-      </c>
-      <c r="B1769" s="24" t="inlineStr">
-        <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/transporte-internacional-compra-recambios/web01-tramite/es/</t>
-        </is>
-      </c>
-      <c r="C1769" s="22" t="n"/>
-      <c r="D1769" s="22" t="n"/>
-      <c r="E1769" s="22" t="n"/>
-      <c r="F1769" s="22" t="n"/>
-    </row>
-    <row r="1771" ht="30" customHeight="1">
-      <c r="A1771" s="18" t="inlineStr">
-        <is>
-          <t>FICHA 119: EUS-46800</t>
-        </is>
-      </c>
-      <c r="B1771" s="19" t="n"/>
-      <c r="C1771" s="19" t="n"/>
-      <c r="D1771" s="19" t="n"/>
-      <c r="E1771" s="19" t="n"/>
-      <c r="F1771" s="19" t="n"/>
-    </row>
-    <row r="1772" ht="20" customHeight="1">
-      <c r="A1772" s="20" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-      <c r="B1772" s="21" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
-        </is>
-      </c>
-      <c r="C1772" s="22" t="n"/>
-      <c r="D1772" s="22" t="n"/>
-      <c r="E1772" s="22" t="n"/>
-      <c r="F1772" s="22" t="n"/>
-    </row>
-    <row r="1773" ht="20" customHeight="1">
-      <c r="A1773" s="20" t="inlineStr">
-        <is>
-          <t>Titulo</t>
-        </is>
-      </c>
-      <c r="B1773" s="21" t="inlineStr">
-        <is>
-          <t>Reparación máquina M300 de limpieza de piezas de taller carrocería</t>
-        </is>
-      </c>
-      <c r="C1773" s="22" t="n"/>
-      <c r="D1773" s="22" t="n"/>
-      <c r="E1773" s="22" t="n"/>
-      <c r="F1773" s="22" t="n"/>
-    </row>
-    <row r="1774" ht="20" customHeight="1">
-      <c r="A1774" s="20" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1774" s="21" t="inlineStr">
-        <is>
-          <t>EUS-46800</t>
-        </is>
-      </c>
-      <c r="C1774" s="22" t="n"/>
-      <c r="D1774" s="22" t="n"/>
-      <c r="E1774" s="22" t="n"/>
-      <c r="F1774" s="22" t="n"/>
-    </row>
-    <row r="1775" ht="20" customHeight="1">
-      <c r="A1775" s="20" t="inlineStr">
-        <is>
-          <t>Programa</t>
-        </is>
-      </c>
-      <c r="B1775" s="21" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="C1775" s="22" t="n"/>
-      <c r="D1775" s="22" t="n"/>
-      <c r="E1775" s="22" t="n"/>
-      <c r="F1775" s="22" t="n"/>
-    </row>
-    <row r="1776" ht="20" customHeight="1">
-      <c r="A1776" s="20" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="B1776" s="21" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C1776" s="22" t="n"/>
-      <c r="D1776" s="22" t="n"/>
-      <c r="E1776" s="22" t="n"/>
-      <c r="F1776" s="22" t="n"/>
-    </row>
-    <row r="1777" ht="20" customHeight="1">
-      <c r="A1777" s="20" t="inlineStr">
-        <is>
-          <t>Deadline</t>
-        </is>
-      </c>
-      <c r="B1777" s="21" t="inlineStr"/>
-      <c r="C1777" s="22" t="n"/>
-      <c r="D1777" s="22" t="n"/>
-      <c r="E1777" s="22" t="n"/>
-      <c r="F1777" s="22" t="n"/>
-    </row>
-    <row r="1778" ht="20" customHeight="1">
-      <c r="A1778" s="20" t="inlineStr">
-        <is>
-          <t>Presupuesto (EUR)</t>
-        </is>
-      </c>
-      <c r="B1778" s="21" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="C1778" s="22" t="n"/>
-      <c r="D1778" s="22" t="n"/>
-      <c r="E1778" s="22" t="n"/>
-      <c r="F1778" s="22" t="n"/>
-    </row>
-    <row r="1779" ht="20" customHeight="1">
-      <c r="A1779" s="20" t="inlineStr">
-        <is>
-          <t>Tipo de Accion</t>
-        </is>
-      </c>
-      <c r="B1779" s="21" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="C1779" s="22" t="n"/>
-      <c r="D1779" s="22" t="n"/>
-      <c r="E1779" s="22" t="n"/>
-      <c r="F1779" s="22" t="n"/>
-    </row>
-    <row r="1780" ht="20" customHeight="1">
-      <c r="A1780" s="20" t="inlineStr">
-        <is>
-          <t>Call ID</t>
-        </is>
-      </c>
-      <c r="B1780" s="21" t="inlineStr"/>
-      <c r="C1780" s="22" t="n"/>
-      <c r="D1780" s="22" t="n"/>
-      <c r="E1780" s="22" t="n"/>
-      <c r="F1780" s="22" t="n"/>
-    </row>
-    <row r="1781" ht="20" customHeight="1">
-      <c r="A1781" s="20" t="inlineStr">
-        <is>
-          <t>Descripcion</t>
-        </is>
-      </c>
-      <c r="B1781" s="21" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="C1781" s="22" t="n"/>
-      <c r="D1781" s="22" t="n"/>
-      <c r="E1781" s="22" t="n"/>
-      <c r="F1781" s="22" t="n"/>
-    </row>
-    <row r="1782" ht="20" customHeight="1">
-      <c r="A1782" s="20" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-      <c r="B1782" s="21" t="inlineStr">
-        <is>
-          <t>energia</t>
-        </is>
-      </c>
-      <c r="C1782" s="22" t="n"/>
-      <c r="D1782" s="22" t="n"/>
-      <c r="E1782" s="22" t="n"/>
-      <c r="F1782" s="22" t="n"/>
-    </row>
-    <row r="1783" ht="20" customHeight="1">
-      <c r="A1783" s="20" t="inlineStr">
-        <is>
-          <t>Relevancia Bilbao</t>
-        </is>
-      </c>
-      <c r="B1783" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
-        </is>
-      </c>
-      <c r="C1783" s="22" t="n"/>
-      <c r="D1783" s="22" t="n"/>
-      <c r="E1783" s="22" t="n"/>
-      <c r="F1783" s="22" t="n"/>
-    </row>
-    <row r="1784" ht="45" customHeight="1">
-      <c r="A1784" s="20" t="inlineStr">
-        <is>
-          <t>Enlace al portal</t>
-        </is>
-      </c>
-      <c r="B1784" s="24" t="inlineStr">
-        <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/reparacion-maquina-m300-limpieza-piezas-taller-carroceria/web01-tramite/es/</t>
-        </is>
-      </c>
-      <c r="C1784" s="22" t="n"/>
-      <c r="D1784" s="22" t="n"/>
-      <c r="E1784" s="22" t="n"/>
-      <c r="F1784" s="22" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="1666">
+  <mergeCells count="1596">
     <mergeCell ref="B679:F679"/>
-    <mergeCell ref="B1765:F1765"/>
     <mergeCell ref="B1010:F1010"/>
     <mergeCell ref="B276:F276"/>
     <mergeCell ref="B1012:F1012"/>
@@ -33816,11 +32439,9 @@
     <mergeCell ref="B253:F253"/>
     <mergeCell ref="B551:F551"/>
     <mergeCell ref="B707:F707"/>
-    <mergeCell ref="B1760:F1760"/>
     <mergeCell ref="B1041:F1041"/>
     <mergeCell ref="B1339:F1339"/>
     <mergeCell ref="B578:F578"/>
-    <mergeCell ref="B1768:F1768"/>
     <mergeCell ref="A1246:F1246"/>
     <mergeCell ref="B723:F723"/>
     <mergeCell ref="B6:F6"/>
@@ -33829,7 +32450,6 @@
     <mergeCell ref="B1664:F1664"/>
     <mergeCell ref="B725:F725"/>
     <mergeCell ref="B1067:F1067"/>
-    <mergeCell ref="B1778:F1778"/>
     <mergeCell ref="B719:F719"/>
     <mergeCell ref="B306:F306"/>
     <mergeCell ref="B1023:F1023"/>
@@ -33839,7 +32459,6 @@
     <mergeCell ref="B1323:F1323"/>
     <mergeCell ref="B291:F291"/>
     <mergeCell ref="B1481:F1481"/>
-    <mergeCell ref="B1779:F1779"/>
     <mergeCell ref="B1692:F1692"/>
     <mergeCell ref="B293:F293"/>
     <mergeCell ref="B322:F322"/>
@@ -33863,20 +32482,17 @@
     <mergeCell ref="B159:F159"/>
     <mergeCell ref="A586:F586"/>
     <mergeCell ref="B764:F764"/>
-    <mergeCell ref="B1736:F1736"/>
     <mergeCell ref="B161:F161"/>
     <mergeCell ref="B459:F459"/>
     <mergeCell ref="B1133:F1133"/>
     <mergeCell ref="A886:F886"/>
     <mergeCell ref="B1431:F1431"/>
-    <mergeCell ref="B1729:F1729"/>
     <mergeCell ref="B670:F670"/>
     <mergeCell ref="B461:F461"/>
     <mergeCell ref="B249:F249"/>
     <mergeCell ref="B243:F243"/>
     <mergeCell ref="B678:F678"/>
     <mergeCell ref="B363:F363"/>
-    <mergeCell ref="B1731:F1731"/>
     <mergeCell ref="B373:F373"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="B1115:F1115"/>
@@ -33895,7 +32511,6 @@
     <mergeCell ref="B689:F689"/>
     <mergeCell ref="B86:F86"/>
     <mergeCell ref="B262:F262"/>
-    <mergeCell ref="A1771:F1771"/>
     <mergeCell ref="B1286:F1286"/>
     <mergeCell ref="B865:F865"/>
     <mergeCell ref="B444:F444"/>
@@ -33979,7 +32594,6 @@
     <mergeCell ref="B1184:F1184"/>
     <mergeCell ref="B297:F297"/>
     <mergeCell ref="B813:F813"/>
-    <mergeCell ref="A1756:F1756"/>
     <mergeCell ref="B1242:F1242"/>
     <mergeCell ref="B902:F902"/>
     <mergeCell ref="B1331:F1331"/>
@@ -34018,7 +32632,6 @@
     <mergeCell ref="B529:F529"/>
     <mergeCell ref="B523:F523"/>
     <mergeCell ref="B827:F827"/>
-    <mergeCell ref="B1713:F1713"/>
     <mergeCell ref="A436:F436"/>
     <mergeCell ref="A121:F121"/>
     <mergeCell ref="B668:F668"/>
@@ -34033,7 +32646,6 @@
     <mergeCell ref="B880:F880"/>
     <mergeCell ref="B671:F671"/>
     <mergeCell ref="B1187:F1187"/>
-    <mergeCell ref="B1724:F1724"/>
     <mergeCell ref="B969:F969"/>
     <mergeCell ref="B1607:F1607"/>
     <mergeCell ref="B963:F963"/>
@@ -34078,16 +32690,13 @@
     <mergeCell ref="B36:F36"/>
     <mergeCell ref="A1486:F1486"/>
     <mergeCell ref="B334:F334"/>
-    <mergeCell ref="B1735:F1735"/>
     <mergeCell ref="B1368:F1368"/>
     <mergeCell ref="B1420:F1420"/>
     <mergeCell ref="B336:F336"/>
     <mergeCell ref="B634:F634"/>
     <mergeCell ref="B1422:F1422"/>
-    <mergeCell ref="B1720:F1720"/>
     <mergeCell ref="B965:F965"/>
     <mergeCell ref="B669:F669"/>
-    <mergeCell ref="B1722:F1722"/>
     <mergeCell ref="A451:F451"/>
     <mergeCell ref="A901:F901"/>
     <mergeCell ref="B563:F563"/>
@@ -34097,13 +32706,11 @@
     <mergeCell ref="A1201:F1201"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="B565:F565"/>
-    <mergeCell ref="B1746:F1746"/>
     <mergeCell ref="B266:F266"/>
     <mergeCell ref="B564:F564"/>
     <mergeCell ref="B558:F558"/>
     <mergeCell ref="B695:F695"/>
     <mergeCell ref="B1450:F1450"/>
-    <mergeCell ref="B1748:F1748"/>
     <mergeCell ref="B993:F993"/>
     <mergeCell ref="A1501:F1501"/>
     <mergeCell ref="B987:F987"/>
@@ -34163,7 +32770,6 @@
     <mergeCell ref="B1106:F1106"/>
     <mergeCell ref="B47:F47"/>
     <mergeCell ref="B351:F351"/>
-    <mergeCell ref="B1744:F1744"/>
     <mergeCell ref="B1535:F1535"/>
     <mergeCell ref="B774:F774"/>
     <mergeCell ref="B801:F801"/>
@@ -34183,17 +32789,14 @@
     <mergeCell ref="B1465:F1465"/>
     <mergeCell ref="B1459:F1459"/>
     <mergeCell ref="B704:F704"/>
-    <mergeCell ref="B1757:F1757"/>
     <mergeCell ref="B1002:F1002"/>
     <mergeCell ref="B399:F399"/>
-    <mergeCell ref="B1759:F1759"/>
     <mergeCell ref="B1004:F1004"/>
     <mergeCell ref="B1302:F1302"/>
     <mergeCell ref="B1460:F1460"/>
     <mergeCell ref="A946:F946"/>
     <mergeCell ref="A631:F631"/>
     <mergeCell ref="B117:F117"/>
-    <mergeCell ref="B1783:F1783"/>
     <mergeCell ref="B425:F425"/>
     <mergeCell ref="B1178:F1178"/>
     <mergeCell ref="B119:F119"/>
@@ -34211,7 +32814,6 @@
     <mergeCell ref="B1504:F1504"/>
     <mergeCell ref="B445:F445"/>
     <mergeCell ref="B743:F743"/>
-    <mergeCell ref="A1711:F1711"/>
     <mergeCell ref="B18:F18"/>
     <mergeCell ref="B1506:F1506"/>
     <mergeCell ref="B797:F797"/>
@@ -34238,7 +32840,6 @@
     <mergeCell ref="B1254:F1254"/>
     <mergeCell ref="B1430:F1430"/>
     <mergeCell ref="B1552:F1552"/>
-    <mergeCell ref="B1728:F1728"/>
     <mergeCell ref="B1588:F1588"/>
     <mergeCell ref="B1131:F1131"/>
     <mergeCell ref="B72:F72"/>
@@ -34261,7 +32862,6 @@
     <mergeCell ref="B85:F85"/>
     <mergeCell ref="B383:F383"/>
     <mergeCell ref="B1355:F1355"/>
-    <mergeCell ref="B1784:F1784"/>
     <mergeCell ref="B141:F141"/>
     <mergeCell ref="B439:F439"/>
     <mergeCell ref="B985:F985"/>
@@ -34395,8 +32995,6 @@
     <mergeCell ref="B1089:F1089"/>
     <mergeCell ref="B877:F877"/>
     <mergeCell ref="B1387:F1387"/>
-    <mergeCell ref="B1763:F1763"/>
-    <mergeCell ref="B1721:F1721"/>
     <mergeCell ref="B1300:F1300"/>
     <mergeCell ref="B1604:F1604"/>
     <mergeCell ref="B205:F205"/>
@@ -34411,22 +33009,18 @@
     <mergeCell ref="B1337:F1337"/>
     <mergeCell ref="B292:F292"/>
     <mergeCell ref="B1476:F1476"/>
-    <mergeCell ref="B1774:F1774"/>
     <mergeCell ref="B1019:F1019"/>
     <mergeCell ref="B294:F294"/>
     <mergeCell ref="B592:F592"/>
     <mergeCell ref="B714:F714"/>
     <mergeCell ref="B890:F890"/>
-    <mergeCell ref="B1776:F1776"/>
     <mergeCell ref="B1319:F1319"/>
     <mergeCell ref="B287:F287"/>
-    <mergeCell ref="B1775:F1775"/>
     <mergeCell ref="B594:F594"/>
     <mergeCell ref="B716:F716"/>
     <mergeCell ref="B892:F892"/>
     <mergeCell ref="B289:F289"/>
     <mergeCell ref="B1479:F1479"/>
-    <mergeCell ref="B1777:F1777"/>
     <mergeCell ref="A1261:F1261"/>
     <mergeCell ref="B747:F747"/>
     <mergeCell ref="B618:F618"/>
@@ -34450,16 +33044,12 @@
     <mergeCell ref="B1119:F1119"/>
     <mergeCell ref="B333:F333"/>
     <mergeCell ref="B1427:F1427"/>
-    <mergeCell ref="B1734:F1734"/>
     <mergeCell ref="B1419:F1419"/>
     <mergeCell ref="B664:F664"/>
-    <mergeCell ref="B1717:F1717"/>
     <mergeCell ref="B658:F658"/>
     <mergeCell ref="B239:F239"/>
     <mergeCell ref="B1429:F1429"/>
-    <mergeCell ref="B1727:F1727"/>
     <mergeCell ref="B1421:F1421"/>
-    <mergeCell ref="B1719:F1719"/>
     <mergeCell ref="B659:F659"/>
     <mergeCell ref="A871:F871"/>
     <mergeCell ref="B232:F232"/>
@@ -34468,13 +33058,11 @@
     <mergeCell ref="B982:F982"/>
     <mergeCell ref="B263:F263"/>
     <mergeCell ref="B1447:F1447"/>
-    <mergeCell ref="B1745:F1745"/>
     <mergeCell ref="B686:F686"/>
     <mergeCell ref="B229:F229"/>
     <mergeCell ref="B1142:F1142"/>
     <mergeCell ref="B387:F387"/>
     <mergeCell ref="B685:F685"/>
-    <mergeCell ref="B1747:F1747"/>
     <mergeCell ref="B258:F258"/>
     <mergeCell ref="B1442:F1442"/>
     <mergeCell ref="B687:F687"/>
@@ -34546,20 +33134,16 @@
     <mergeCell ref="B1227:F1227"/>
     <mergeCell ref="B168:F168"/>
     <mergeCell ref="B472:F472"/>
-    <mergeCell ref="B1743:F1743"/>
     <mergeCell ref="B1438:F1438"/>
     <mergeCell ref="B683:F683"/>
-    <mergeCell ref="B1742:F1742"/>
     <mergeCell ref="B1527:F1527"/>
     <mergeCell ref="A1036:F1036"/>
     <mergeCell ref="B497:F497"/>
-    <mergeCell ref="B1738:F1738"/>
     <mergeCell ref="B983:F983"/>
     <mergeCell ref="A1336:F1336"/>
     <mergeCell ref="A1636:F1636"/>
     <mergeCell ref="B96:F96"/>
     <mergeCell ref="B701:F701"/>
-    <mergeCell ref="B1754:F1754"/>
     <mergeCell ref="B1614:F1614"/>
     <mergeCell ref="B853:F853"/>
     <mergeCell ref="B98:F98"/>
@@ -34683,11 +33267,9 @@
     <mergeCell ref="B1558:F1558"/>
     <mergeCell ref="B499:F499"/>
     <mergeCell ref="A1171:F1171"/>
-    <mergeCell ref="B1716:F1716"/>
     <mergeCell ref="B1262:F1262"/>
     <mergeCell ref="B534:F534"/>
     <mergeCell ref="B805:F805"/>
-    <mergeCell ref="B1718:F1718"/>
     <mergeCell ref="B957:F957"/>
     <mergeCell ref="B536:F536"/>
     <mergeCell ref="B834:F834"/>
@@ -34706,7 +33288,6 @@
     <mergeCell ref="B862:F862"/>
     <mergeCell ref="B547:F547"/>
     <mergeCell ref="B101:F101"/>
-    <mergeCell ref="B1762:F1762"/>
     <mergeCell ref="B703:F703"/>
     <mergeCell ref="B1007:F1007"/>
     <mergeCell ref="B1001:F1001"/>
@@ -34762,7 +33343,6 @@
     <mergeCell ref="B1287:F1287"/>
     <mergeCell ref="B972:F972"/>
     <mergeCell ref="B1702:F1702"/>
-    <mergeCell ref="B1758:F1758"/>
     <mergeCell ref="B359:F359"/>
     <mergeCell ref="B788:F788"/>
     <mergeCell ref="B999:F999"/>
@@ -34770,10 +33350,8 @@
     <mergeCell ref="B1297:F1297"/>
     <mergeCell ref="B62:F62"/>
     <mergeCell ref="B700:F700"/>
-    <mergeCell ref="B1753:F1753"/>
     <mergeCell ref="B998:F998"/>
     <mergeCell ref="B273:F273"/>
-    <mergeCell ref="B1761:F1761"/>
     <mergeCell ref="B1000:F1000"/>
     <mergeCell ref="B1298:F1298"/>
     <mergeCell ref="B573:F573"/>
@@ -34783,7 +33361,6 @@
     <mergeCell ref="A166:F166"/>
     <mergeCell ref="B589:F589"/>
     <mergeCell ref="B1597:F1597"/>
-    <mergeCell ref="B1773:F1773"/>
     <mergeCell ref="B1018:F1018"/>
     <mergeCell ref="B624:F624"/>
     <mergeCell ref="B1316:F1316"/>
@@ -34793,7 +33370,6 @@
     <mergeCell ref="B415:F415"/>
     <mergeCell ref="B1468:F1468"/>
     <mergeCell ref="B713:F713"/>
-    <mergeCell ref="B1766:F1766"/>
     <mergeCell ref="B1011:F1011"/>
     <mergeCell ref="B1685:F1685"/>
     <mergeCell ref="B110:F110"/>
@@ -34852,7 +33428,6 @@
     <mergeCell ref="B1464:F1464"/>
     <mergeCell ref="B1439:F1439"/>
     <mergeCell ref="B1472:F1472"/>
-    <mergeCell ref="B1764:F1764"/>
     <mergeCell ref="B740:F740"/>
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="B1467:F1467"/>
@@ -34906,7 +33481,6 @@
     <mergeCell ref="B1435:F1435"/>
     <mergeCell ref="B680:F680"/>
     <mergeCell ref="A376:F376"/>
-    <mergeCell ref="B1733:F1733"/>
     <mergeCell ref="B674:F674"/>
     <mergeCell ref="B1226:F1226"/>
     <mergeCell ref="B832:F832"/>
@@ -35019,7 +33593,6 @@
     <mergeCell ref="B1045:F1045"/>
     <mergeCell ref="B290:F290"/>
     <mergeCell ref="B588:F588"/>
-    <mergeCell ref="B1772:F1772"/>
     <mergeCell ref="B1017:F1017"/>
     <mergeCell ref="B1315:F1315"/>
     <mergeCell ref="B283:F283"/>
@@ -35039,7 +33612,6 @@
     <mergeCell ref="B512:F512"/>
     <mergeCell ref="B303:F303"/>
     <mergeCell ref="B941:F941"/>
-    <mergeCell ref="A1726:F1726"/>
     <mergeCell ref="B1239:F1239"/>
     <mergeCell ref="B484:F484"/>
     <mergeCell ref="B732:F732"/>
@@ -35064,7 +33636,6 @@
     <mergeCell ref="B531:F531"/>
     <mergeCell ref="B1417:F1417"/>
     <mergeCell ref="B662:F662"/>
-    <mergeCell ref="B1715:F1715"/>
     <mergeCell ref="B954:F954"/>
     <mergeCell ref="B199:F199"/>
     <mergeCell ref="B1112:F1112"/>
@@ -35099,7 +33670,6 @@
     <mergeCell ref="B274:F274"/>
     <mergeCell ref="B1667:F1667"/>
     <mergeCell ref="B728:F728"/>
-    <mergeCell ref="B1781:F1781"/>
     <mergeCell ref="A481:F481"/>
     <mergeCell ref="B1026:F1026"/>
     <mergeCell ref="B1324:F1324"/>
@@ -35109,7 +33679,6 @@
     <mergeCell ref="B1055:F1055"/>
     <mergeCell ref="B1326:F1326"/>
     <mergeCell ref="B1668:F1668"/>
-    <mergeCell ref="B1782:F1782"/>
     <mergeCell ref="B899:F899"/>
     <mergeCell ref="B752:F752"/>
     <mergeCell ref="B325:F325"/>
@@ -35131,7 +33700,6 @@
     <mergeCell ref="B1383:F1383"/>
     <mergeCell ref="B38:F38"/>
     <mergeCell ref="B467:F467"/>
-    <mergeCell ref="B1737:F1737"/>
     <mergeCell ref="B40:F40"/>
     <mergeCell ref="B338:F338"/>
     <mergeCell ref="B1528:F1528"/>
@@ -35139,7 +33707,6 @@
     <mergeCell ref="A1621:F1621"/>
     <mergeCell ref="B767:F767"/>
     <mergeCell ref="B33:F33"/>
-    <mergeCell ref="B1739:F1739"/>
     <mergeCell ref="B340:F340"/>
     <mergeCell ref="B978:F978"/>
     <mergeCell ref="B1434:F1434"/>
@@ -35152,14 +33719,12 @@
     <mergeCell ref="B1581:F1581"/>
     <mergeCell ref="B1452:F1452"/>
     <mergeCell ref="B697:F697"/>
-    <mergeCell ref="B1750:F1750"/>
     <mergeCell ref="B989:F989"/>
     <mergeCell ref="B234:F234"/>
     <mergeCell ref="B392:F392"/>
     <mergeCell ref="B568:F568"/>
     <mergeCell ref="B1454:F1454"/>
     <mergeCell ref="B699:F699"/>
-    <mergeCell ref="B1752:F1752"/>
     <mergeCell ref="B997:F997"/>
     <mergeCell ref="B1295:F1295"/>
     <mergeCell ref="B1453:F1453"/>
@@ -35170,7 +33735,6 @@
     <mergeCell ref="B694:F694"/>
     <mergeCell ref="A1231:F1231"/>
     <mergeCell ref="A286:F286"/>
-    <mergeCell ref="B1780:F1780"/>
     <mergeCell ref="B1480:F1480"/>
     <mergeCell ref="B1165:F1165"/>
     <mergeCell ref="B1048:F1048"/>
@@ -35229,7 +33793,6 @@
     <mergeCell ref="B1418:F1418"/>
     <mergeCell ref="B479:F479"/>
     <mergeCell ref="B777:F777"/>
-    <mergeCell ref="B1749:F1749"/>
     <mergeCell ref="B504:F504"/>
     <mergeCell ref="B802:F802"/>
     <mergeCell ref="B1136:F1136"/>
@@ -35289,7 +33852,6 @@
     <mergeCell ref="B1503:F1503"/>
     <mergeCell ref="A1441:F1441"/>
     <mergeCell ref="B318:F318"/>
-    <mergeCell ref="A1741:F1741"/>
     <mergeCell ref="B1098:F1098"/>
     <mergeCell ref="B958:F958"/>
     <mergeCell ref="B1134:F1134"/>
@@ -35319,7 +33881,6 @@
     <mergeCell ref="B819:F819"/>
     <mergeCell ref="B1574:F1574"/>
     <mergeCell ref="B542:F542"/>
-    <mergeCell ref="B1732:F1732"/>
     <mergeCell ref="B673:F673"/>
     <mergeCell ref="B977:F977"/>
     <mergeCell ref="B971:F971"/>
@@ -35378,12 +33939,10 @@
     <mergeCell ref="B644:F644"/>
     <mergeCell ref="B967:F967"/>
     <mergeCell ref="B942:F942"/>
-    <mergeCell ref="B1730:F1730"/>
     <mergeCell ref="B1273:F1273"/>
     <mergeCell ref="B1267:F1267"/>
     <mergeCell ref="B1609:F1609"/>
     <mergeCell ref="A751:F751"/>
-    <mergeCell ref="B1723:F1723"/>
     <mergeCell ref="B1567:F1567"/>
     <mergeCell ref="A1051:F1051"/>
     <mergeCell ref="B970:F970"/>
@@ -35402,7 +33961,6 @@
     <mergeCell ref="B1024:F1024"/>
     <mergeCell ref="B567:F567"/>
     <mergeCell ref="B1593:F1593"/>
-    <mergeCell ref="B1751:F1751"/>
     <mergeCell ref="B996:F996"/>
     <mergeCell ref="B1330:F1330"/>
     <mergeCell ref="B569:F569"/>
@@ -35411,10 +33969,8 @@
     <mergeCell ref="B1296:F1296"/>
     <mergeCell ref="A1351:F1351"/>
     <mergeCell ref="B1469:F1469"/>
-    <mergeCell ref="B1767:F1767"/>
     <mergeCell ref="B251:F251"/>
     <mergeCell ref="A1651:F1651"/>
-    <mergeCell ref="B1769:F1769"/>
     <mergeCell ref="B1014:F1014"/>
     <mergeCell ref="B1008:F1008"/>
     <mergeCell ref="B280:F280"/>
@@ -35456,7 +34012,6 @@
     <mergeCell ref="B1107:F1107"/>
     <mergeCell ref="B1378:F1378"/>
     <mergeCell ref="B1536:F1536"/>
-    <mergeCell ref="B1712:F1712"/>
     <mergeCell ref="B653:F653"/>
     <mergeCell ref="B1109:F1109"/>
     <mergeCell ref="B354:F354"/>
@@ -35464,7 +34019,6 @@
     <mergeCell ref="B348:F348"/>
     <mergeCell ref="B652:F652"/>
     <mergeCell ref="B1538:F1538"/>
-    <mergeCell ref="B1714:F1714"/>
     <mergeCell ref="B1409:F1409"/>
     <mergeCell ref="B1292:F1292"/>
     <mergeCell ref="B1707:F1707"/>
@@ -35587,11 +34141,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1679" r:id="rId112"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1694" r:id="rId113"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1709" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1724" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1739" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1754" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1769" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1784" r:id="rId119"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -35603,7 +34152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J120"/>
+  <dimension ref="A1:J115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -39645,17 +38194,17 @@
     <row r="104" ht="28" customHeight="1">
       <c r="A104" s="6" t="inlineStr">
         <is>
-          <t>BDNS-897355</t>
+          <t>BDNS-897535</t>
         </is>
       </c>
       <c r="B104" s="6" t="inlineStr">
         <is>
-          <t>Programa de ayudas digitalización cadena alim. y madera 2025</t>
+          <t>Ayudas a la implantación, modernización y transformación dig</t>
         </is>
       </c>
       <c r="C104" s="6" t="inlineStr">
         <is>
-          <t>PAÍS VASCO</t>
+          <t>VITORIA-GASTEIZ</t>
         </is>
       </c>
       <c r="D104" s="6" t="inlineStr">
@@ -39665,12 +38214,12 @@
       </c>
       <c r="E104" s="6" t="inlineStr">
         <is>
-          <t>31/12/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="F104" s="27" t="inlineStr">
         <is>
-          <t>MUY ALTA</t>
+          <t>MEDIA</t>
         </is>
       </c>
       <c r="G104" s="6" t="inlineStr"/>
@@ -39685,17 +38234,17 @@
     <row r="105" ht="28" customHeight="1">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>BDNS-897535</t>
+          <t>EUS-18545</t>
         </is>
       </c>
       <c r="B105" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la implantación, modernización y transformación dig</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
         </is>
       </c>
       <c r="C105" s="6" t="inlineStr">
         <is>
-          <t>VITORIA-GASTEIZ</t>
+          <t>Euskadi</t>
         </is>
       </c>
       <c r="D105" s="6" t="inlineStr">
@@ -39703,14 +38252,10 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="E105" s="6" t="inlineStr">
-        <is>
-          <t>05/05/2026</t>
-        </is>
-      </c>
+      <c r="E105" s="6" t="inlineStr"/>
       <c r="F105" s="27" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="G105" s="6" t="inlineStr"/>
@@ -39725,17 +38270,17 @@
     <row r="106" ht="28" customHeight="1">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>BDNS-897198</t>
+          <t>EUS-98881</t>
         </is>
       </c>
       <c r="B106" s="6" t="inlineStr">
         <is>
-          <t>Ayudas para actividades educativas organizadas por asociacio</t>
+          <t>Ayudas a la gestión sostenible de los recursos pesqueros 202</t>
         </is>
       </c>
       <c r="C106" s="6" t="inlineStr">
         <is>
-          <t>VITORIA-GASTEIZ</t>
+          <t>Euskadi</t>
         </is>
       </c>
       <c r="D106" s="6" t="inlineStr">
@@ -39743,14 +38288,10 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="E106" s="6" t="inlineStr">
-        <is>
-          <t>29/05/2026</t>
-        </is>
-      </c>
+      <c r="E106" s="6" t="inlineStr"/>
       <c r="F106" s="27" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="G106" s="6" t="inlineStr"/>
@@ -39765,12 +38306,12 @@
     <row r="107" ht="28" customHeight="1">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>EUS-25527</t>
+          <t>EUS-38210</t>
         </is>
       </c>
       <c r="B107" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
+          <t>Ayudas a la recogida de residuos con la participación de los</t>
         </is>
       </c>
       <c r="C107" s="6" t="inlineStr">
@@ -39801,12 +38342,12 @@
     <row r="108" ht="28" customHeight="1">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>EUS-67276</t>
+          <t>EUS-62379</t>
         </is>
       </c>
       <c r="B108" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la gestión sostenible de los recursos pesqueros 202</t>
+          <t xml:space="preserve">Poli ipurua: conduccion aportacion aire exterior ?filtrado? </t>
         </is>
       </c>
       <c r="C108" s="6" t="inlineStr">
@@ -39837,12 +38378,12 @@
     <row r="109" ht="28" customHeight="1">
       <c r="A109" s="6" t="inlineStr">
         <is>
-          <t>EUS-54829</t>
+          <t>EUS-68865</t>
         </is>
       </c>
       <c r="B109" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la recogida de residuos con la participación de los</t>
+          <t>Poli orbea: conduccion aportacion aire exterior para ?climat</t>
         </is>
       </c>
       <c r="C109" s="6" t="inlineStr">
@@ -39873,12 +38414,12 @@
     <row r="110" ht="28" customHeight="1">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>EUS-45197</t>
+          <t>EUS-45735</t>
         </is>
       </c>
       <c r="B110" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
+          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversi</t>
         </is>
       </c>
       <c r="C110" s="6" t="inlineStr">
@@ -39894,7 +38435,7 @@
       <c r="E110" s="6" t="inlineStr"/>
       <c r="F110" s="27" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>MEDIA</t>
         </is>
       </c>
       <c r="G110" s="6" t="inlineStr"/>
@@ -39909,12 +38450,12 @@
     <row r="111" ht="28" customHeight="1">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>EUS-83922</t>
+          <t>EUS-28095</t>
         </is>
       </c>
       <c r="B111" s="6" t="inlineStr">
         <is>
-          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversi</t>
+          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el ma</t>
         </is>
       </c>
       <c r="C111" s="6" t="inlineStr">
@@ -39945,12 +38486,12 @@
     <row r="112" ht="28" customHeight="1">
       <c r="A112" s="6" t="inlineStr">
         <is>
-          <t>EUS-69965</t>
+          <t>EUS-41533</t>
         </is>
       </c>
       <c r="B112" s="6" t="inlineStr">
         <is>
-          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el ma</t>
+          <t>Ayudas a la contribución de la acuicultura al buen estado am</t>
         </is>
       </c>
       <c r="C112" s="6" t="inlineStr">
@@ -39981,12 +38522,12 @@
     <row r="113" ht="28" customHeight="1">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>EUS-97870</t>
+          <t>EUS-46847</t>
         </is>
       </c>
       <c r="B113" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la contribución de la acuicultura al buen estado am</t>
+          <t>Enajenación mediante procedimiento de subasta pública del lo</t>
         </is>
       </c>
       <c r="C113" s="6" t="inlineStr">
@@ -40017,12 +38558,12 @@
     <row r="114" ht="28" customHeight="1">
       <c r="A114" s="6" t="inlineStr">
         <is>
-          <t>EUS-63161</t>
+          <t>EUS-44891</t>
         </is>
       </c>
       <c r="B114" s="6" t="inlineStr">
         <is>
-          <t>Ayudas al valor añadido, economía circular y seguridad alime</t>
+          <t>Suministro de Equipamiento para ampliaciones de capacidad de</t>
         </is>
       </c>
       <c r="C114" s="6" t="inlineStr">
@@ -40053,12 +38594,12 @@
     <row r="115" ht="28" customHeight="1">
       <c r="A115" s="6" t="inlineStr">
         <is>
-          <t>EUS-27678</t>
+          <t>EUS-95830</t>
         </is>
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>Reparación máquina M300 y M104 de limpieza de piezas de tall</t>
+          <t>Suministro de 4 mesas tipo picnic para zona verde en el Polí</t>
         </is>
       </c>
       <c r="C115" s="6" t="inlineStr">
@@ -40086,188 +38627,8 @@
       <c r="I115" s="6" t="inlineStr"/>
       <c r="J115" s="6" t="inlineStr"/>
     </row>
-    <row r="116" ht="28" customHeight="1">
-      <c r="A116" s="6" t="inlineStr">
-        <is>
-          <t>EUS-78269</t>
-        </is>
-      </c>
-      <c r="B116" s="6" t="inlineStr">
-        <is>
-          <t>Reparación manguera de limpieza marquesinas</t>
-        </is>
-      </c>
-      <c r="C116" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="D116" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E116" s="6" t="inlineStr"/>
-      <c r="F116" s="27" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="G116" s="6" t="inlineStr"/>
-      <c r="H116" s="6" t="inlineStr">
-        <is>
-          <t>Por revisar</t>
-        </is>
-      </c>
-      <c r="I116" s="6" t="inlineStr"/>
-      <c r="J116" s="6" t="inlineStr"/>
-    </row>
-    <row r="117" ht="28" customHeight="1">
-      <c r="A117" s="6" t="inlineStr">
-        <is>
-          <t>EUS-87993</t>
-        </is>
-      </c>
-      <c r="B117" s="6" t="inlineStr">
-        <is>
-          <t>Reparación manguera de limpieza marquesinas</t>
-        </is>
-      </c>
-      <c r="C117" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="D117" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E117" s="6" t="inlineStr"/>
-      <c r="F117" s="27" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="G117" s="6" t="inlineStr"/>
-      <c r="H117" s="6" t="inlineStr">
-        <is>
-          <t>Por revisar</t>
-        </is>
-      </c>
-      <c r="I117" s="6" t="inlineStr"/>
-      <c r="J117" s="6" t="inlineStr"/>
-    </row>
-    <row r="118" ht="28" customHeight="1">
-      <c r="A118" s="6" t="inlineStr">
-        <is>
-          <t>EUS-99225</t>
-        </is>
-      </c>
-      <c r="B118" s="6" t="inlineStr">
-        <is>
-          <t>Reparación manguera de limpieza marquesinas</t>
-        </is>
-      </c>
-      <c r="C118" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="D118" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E118" s="6" t="inlineStr"/>
-      <c r="F118" s="27" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="G118" s="6" t="inlineStr"/>
-      <c r="H118" s="6" t="inlineStr">
-        <is>
-          <t>Por revisar</t>
-        </is>
-      </c>
-      <c r="I118" s="6" t="inlineStr"/>
-      <c r="J118" s="6" t="inlineStr"/>
-    </row>
-    <row r="119" ht="28" customHeight="1">
-      <c r="A119" s="6" t="inlineStr">
-        <is>
-          <t>EUS-09085</t>
-        </is>
-      </c>
-      <c r="B119" s="6" t="inlineStr">
-        <is>
-          <t>Transporte Internacional de compra de recambios</t>
-        </is>
-      </c>
-      <c r="C119" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="D119" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E119" s="6" t="inlineStr"/>
-      <c r="F119" s="27" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="G119" s="6" t="inlineStr"/>
-      <c r="H119" s="6" t="inlineStr">
-        <is>
-          <t>Por revisar</t>
-        </is>
-      </c>
-      <c r="I119" s="6" t="inlineStr"/>
-      <c r="J119" s="6" t="inlineStr"/>
-    </row>
-    <row r="120" ht="28" customHeight="1">
-      <c r="A120" s="6" t="inlineStr">
-        <is>
-          <t>EUS-46800</t>
-        </is>
-      </c>
-      <c r="B120" s="6" t="inlineStr">
-        <is>
-          <t>Reparación máquina M300 de limpieza de piezas de taller carr</t>
-        </is>
-      </c>
-      <c r="C120" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="D120" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E120" s="6" t="inlineStr"/>
-      <c r="F120" s="27" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="G120" s="6" t="inlineStr"/>
-      <c r="H120" s="6" t="inlineStr">
-        <is>
-          <t>Por revisar</t>
-        </is>
-      </c>
-      <c r="I120" s="6" t="inlineStr"/>
-      <c r="J120" s="6" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J120"/>
+  <autoFilter ref="A1:J115"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update funding data 2026-04-11
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Recursos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$121</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$115</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$122</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$116</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -84,13 +84,13 @@
     <font>
       <name val="Leelawadee UI"/>
       <b val="1"/>
-      <color rgb="00065F46"/>
+      <color rgb="00DC2626"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Leelawadee UI"/>
       <b val="1"/>
-      <color rgb="00DC2626"/>
+      <color rgb="00065F46"/>
       <sz val="10"/>
     </font>
     <font>
@@ -166,17 +166,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FEF2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00065F46"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D1FAE5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEF2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -268,11 +268,11 @@
     <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -312,8 +312,8 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -679,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M121"/>
+  <dimension ref="A1:M122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -707,7 +707,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 10/04/2026 07:16 - 114 convocatorias - 11 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 11/04/2026 06:48 - 115 convocatorias - 14 nuevas</t>
         </is>
       </c>
     </row>
@@ -6919,12 +6919,12 @@
       </c>
       <c r="B108" s="6" t="inlineStr">
         <is>
-          <t>BDNS-897488</t>
+          <t>BDNS-898162</t>
         </is>
       </c>
       <c r="C108" s="6" t="inlineStr">
         <is>
-          <t>CONVENIO DE SUBVENCIÓN NOMINATIVA ENTRE EL AYUNTAMIENTO DE VITORIA-GASTEIZ Y LA ASOCIACION DE PRODUCTORES AUDIOVISUALES   APIKA, PARA EL DESARROLLO DEL PROGRAMA APIKA AUDIOVISUAL PROJET LAB 2026</t>
+          <t>CONVENIO DE SUBVENCIÓN NOMINATIVA ENTRE EL AYUNTAMIENTO DE VITORIA-GASTEIZ, FUNDACIÓN VITAL, FUNDACIÓN ADSIS, FUNDACIÓN DIOCESANAS-JESÚS OBRERO FUNDAZIOA-EGIBIDE Y CÁRITAS DIOCESANA DE VITORIA, PARA O</t>
         </is>
       </c>
       <c r="D108" s="6" t="inlineStr">
@@ -6939,12 +6939,12 @@
       </c>
       <c r="F108" s="6" t="inlineStr">
         <is>
-          <t>31/12/2026</t>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="G108" s="6" t="inlineStr">
         <is>
-          <t>20,000.00 EUR</t>
+          <t>120,000.00 EUR</t>
         </is>
       </c>
       <c r="H108" s="6" t="inlineStr">
@@ -6963,93 +6963,93 @@
           <t>PERSONAS JURÍDICAS QUE NO DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
         </is>
       </c>
-      <c r="L108" s="6" t="inlineStr"/>
+      <c r="L108" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
       <c r="M108" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
         </is>
       </c>
     </row>
-    <row r="109" ht="40" customHeight="1">
-      <c r="A109" s="14" t="inlineStr">
-        <is>
-          <t>España</t>
-        </is>
-      </c>
-      <c r="B109" s="6" t="inlineStr">
-        <is>
-          <t>BDNS-897535</t>
-        </is>
-      </c>
-      <c r="C109" s="6" t="inlineStr">
-        <is>
-          <t>Ayudas a la implantación, modernización y transformación digital de las pequeñas empresas de comercio, servicios personales y hostelería de Vitoria-Gasteiz 2026</t>
-        </is>
-      </c>
-      <c r="D109" s="6" t="inlineStr">
-        <is>
-          <t>VITORIA-GASTEIZ</t>
-        </is>
-      </c>
-      <c r="E109" s="7" t="inlineStr">
+    <row r="109" ht="28" customHeight="1">
+      <c r="A109" s="16" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="40" customHeight="1">
+      <c r="A110" s="17" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B110" s="6" t="inlineStr">
+        <is>
+          <t>EUS-17340</t>
+        </is>
+      </c>
+      <c r="C110" s="6" t="inlineStr">
+        <is>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
+        </is>
+      </c>
+      <c r="D110" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E110" s="7" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F109" s="6" t="inlineStr">
-        <is>
-          <t>05/05/2026</t>
-        </is>
-      </c>
-      <c r="G109" s="6" t="inlineStr">
-        <is>
-          <t>490,000.00 EUR</t>
-        </is>
-      </c>
-      <c r="H109" s="6" t="inlineStr">
-        <is>
-          <t>Subvencion Nacional</t>
-        </is>
-      </c>
-      <c r="I109" s="10" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="J109" s="6" t="inlineStr"/>
-      <c r="K109" s="6" t="inlineStr">
-        <is>
-          <t>PYME Y PERSONAS FÍSICAS QUE DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
-        </is>
-      </c>
-      <c r="L109" s="6" t="inlineStr"/>
-      <c r="M109" s="9" t="inlineStr">
+      <c r="F110" s="6" t="inlineStr"/>
+      <c r="G110" s="6" t="inlineStr"/>
+      <c r="H110" s="6" t="inlineStr">
+        <is>
+          <t>Ayuda/Subvencion Euskadi</t>
+        </is>
+      </c>
+      <c r="I110" s="8" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J110" s="6" t="inlineStr"/>
+      <c r="K110" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L110" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M110" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
         </is>
       </c>
     </row>
-    <row r="110" ht="28" customHeight="1">
-      <c r="A110" s="15" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
-        </is>
-      </c>
-    </row>
     <row r="111" ht="40" customHeight="1">
-      <c r="A111" s="16" t="inlineStr">
+      <c r="A111" s="17" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B111" s="6" t="inlineStr">
         <is>
-          <t>EUS-18545</t>
+          <t>EUS-60249</t>
         </is>
       </c>
       <c r="C111" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
+          <t>Ayudas a la gestión sostenible de los recursos pesqueros 2026</t>
         </is>
       </c>
       <c r="D111" s="6" t="inlineStr">
@@ -7080,7 +7080,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L111" s="17" t="inlineStr">
+      <c r="L111" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7092,19 +7092,19 @@
       </c>
     </row>
     <row r="112" ht="40" customHeight="1">
-      <c r="A112" s="16" t="inlineStr">
+      <c r="A112" s="17" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B112" s="6" t="inlineStr">
         <is>
-          <t>EUS-98881</t>
+          <t>EUS-83408</t>
         </is>
       </c>
       <c r="C112" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la gestión sostenible de los recursos pesqueros 2026</t>
+          <t>Ayudas a la recogida de residuos con la participación de los pescadores en el mar y las playas 2026</t>
         </is>
       </c>
       <c r="D112" s="6" t="inlineStr">
@@ -7135,7 +7135,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L112" s="17" t="inlineStr">
+      <c r="L112" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7147,19 +7147,19 @@
       </c>
     </row>
     <row r="113" ht="40" customHeight="1">
-      <c r="A113" s="16" t="inlineStr">
+      <c r="A113" s="17" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B113" s="6" t="inlineStr">
         <is>
-          <t>EUS-38210</t>
+          <t>EUS-21722</t>
         </is>
       </c>
       <c r="C113" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la recogida de residuos con la participación de los pescadores en el mar y las playas 2026</t>
+          <t>Servicios de realización de una campaña de información y sensibilización en materia de residuos de AUM</t>
         </is>
       </c>
       <c r="D113" s="6" t="inlineStr">
@@ -7176,7 +7176,7 @@
       <c r="G113" s="6" t="inlineStr"/>
       <c r="H113" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="I113" s="8" t="inlineStr">
@@ -7190,7 +7190,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L113" s="17" t="inlineStr">
+      <c r="L113" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7202,19 +7202,19 @@
       </c>
     </row>
     <row r="114" ht="40" customHeight="1">
-      <c r="A114" s="16" t="inlineStr">
+      <c r="A114" s="17" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B114" s="6" t="inlineStr">
         <is>
-          <t>EUS-62379</t>
+          <t>EUS-74325</t>
         </is>
       </c>
       <c r="C114" s="6" t="inlineStr">
         <is>
-          <t>Poli ipurua: conduccion aportacion aire exterior ?filtrado? para ?climatizador vestuarios piscinas?.</t>
+          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversidad, participación, principios de la UE. Eventos, difusiones e intercambios. Programa de Ciudadanos, Igualdad, Derechos y Valores de la UE (</t>
         </is>
       </c>
       <c r="D114" s="6" t="inlineStr">
@@ -7231,12 +7231,12 @@
       <c r="G114" s="6" t="inlineStr"/>
       <c r="H114" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I114" s="8" t="inlineStr">
-        <is>
-          <t>ALTA</t>
+          <t>Ayuda/Subvencion Euskadi</t>
+        </is>
+      </c>
+      <c r="I114" s="10" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
         </is>
       </c>
       <c r="J114" s="6" t="inlineStr"/>
@@ -7245,7 +7245,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L114" s="17" t="inlineStr">
+      <c r="L114" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7257,19 +7257,19 @@
       </c>
     </row>
     <row r="115" ht="40" customHeight="1">
-      <c r="A115" s="16" t="inlineStr">
+      <c r="A115" s="17" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>EUS-68865</t>
+          <t>EUS-88845</t>
         </is>
       </c>
       <c r="C115" s="6" t="inlineStr">
         <is>
-          <t>Poli orbea: conduccion aportacion aire exterior para ?climatizador sotano?</t>
+          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el marco de la Intervención Sectorial Vitivinícola del Plan Estratégico (PEPAC) de la Política Agrícola Común de la UE 2023-2027</t>
         </is>
       </c>
       <c r="D115" s="6" t="inlineStr">
@@ -7286,12 +7286,12 @@
       <c r="G115" s="6" t="inlineStr"/>
       <c r="H115" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I115" s="8" t="inlineStr">
-        <is>
-          <t>ALTA</t>
+          <t>Ayuda/Subvencion Euskadi</t>
+        </is>
+      </c>
+      <c r="I115" s="10" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
         </is>
       </c>
       <c r="J115" s="6" t="inlineStr"/>
@@ -7300,7 +7300,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L115" s="17" t="inlineStr">
+      <c r="L115" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7312,19 +7312,19 @@
       </c>
     </row>
     <row r="116" ht="40" customHeight="1">
-      <c r="A116" s="16" t="inlineStr">
+      <c r="A116" s="17" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B116" s="6" t="inlineStr">
         <is>
-          <t>EUS-45735</t>
+          <t>EUS-38197</t>
         </is>
       </c>
       <c r="C116" s="6" t="inlineStr">
         <is>
-          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversidad, participación, principios de la UE. Eventos, difusiones e intercambios. Programa de Ciudadanos, Igualdad, Derechos y Valores de la UE (</t>
+          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
         </is>
       </c>
       <c r="D116" s="6" t="inlineStr">
@@ -7355,7 +7355,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L116" s="17" t="inlineStr">
+      <c r="L116" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7367,19 +7367,19 @@
       </c>
     </row>
     <row r="117" ht="40" customHeight="1">
-      <c r="A117" s="16" t="inlineStr">
+      <c r="A117" s="17" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B117" s="6" t="inlineStr">
         <is>
-          <t>EUS-28095</t>
+          <t>EUS-28551</t>
         </is>
       </c>
       <c r="C117" s="6" t="inlineStr">
         <is>
-          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el marco de la Intervención Sectorial Vitivinícola del Plan Estratégico (PEPAC) de la Política Agrícola Común de la UE 2023-2027</t>
+          <t>Coordinación de Seguridad y Salud en Fase de Ejecución de obra de Renovación de Infraestructuras Urbanas y Pavimentación de la Calle El Campillo-Segunda fase- y Norte de Leza</t>
         </is>
       </c>
       <c r="D117" s="6" t="inlineStr">
@@ -7396,7 +7396,7 @@
       <c r="G117" s="6" t="inlineStr"/>
       <c r="H117" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="I117" s="10" t="inlineStr">
@@ -7410,7 +7410,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L117" s="17" t="inlineStr">
+      <c r="L117" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7422,19 +7422,19 @@
       </c>
     </row>
     <row r="118" ht="40" customHeight="1">
-      <c r="A118" s="16" t="inlineStr">
+      <c r="A118" s="17" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B118" s="6" t="inlineStr">
         <is>
-          <t>EUS-41533</t>
+          <t>EUS-68422</t>
         </is>
       </c>
       <c r="C118" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
+          <t>Procedimiento abierto para la contratación de la limpieza de edificios municipales</t>
         </is>
       </c>
       <c r="D118" s="6" t="inlineStr">
@@ -7451,7 +7451,7 @@
       <c r="G118" s="6" t="inlineStr"/>
       <c r="H118" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="I118" s="10" t="inlineStr">
@@ -7465,7 +7465,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L118" s="17" t="inlineStr">
+      <c r="L118" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7477,19 +7477,19 @@
       </c>
     </row>
     <row r="119" ht="40" customHeight="1">
-      <c r="A119" s="16" t="inlineStr">
+      <c r="A119" s="17" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B119" s="6" t="inlineStr">
         <is>
-          <t>EUS-46847</t>
+          <t>EUS-20992</t>
         </is>
       </c>
       <c r="C119" s="6" t="inlineStr">
         <is>
-          <t>Enajenación mediante procedimiento de subasta pública del local letra D del entresuelo del edificio ubicado en la Avenida de Navarra nº 16 de Pasaia</t>
+          <t>Compra de una reja para el parque del polideportivo.</t>
         </is>
       </c>
       <c r="D119" s="6" t="inlineStr">
@@ -7520,7 +7520,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L119" s="17" t="inlineStr">
+      <c r="L119" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7532,19 +7532,19 @@
       </c>
     </row>
     <row r="120" ht="40" customHeight="1">
-      <c r="A120" s="16" t="inlineStr">
+      <c r="A120" s="17" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B120" s="6" t="inlineStr">
         <is>
-          <t>EUS-44891</t>
+          <t>EUS-44621</t>
         </is>
       </c>
       <c r="C120" s="6" t="inlineStr">
         <is>
-          <t>Suministro de Equipamiento para ampliaciones de capacidad de la red de transporte de ITELAZPI S.A</t>
+          <t>Realización de copias de llaves de la habitación del grupo de consumo y de las viviendas tuteladas</t>
         </is>
       </c>
       <c r="D120" s="6" t="inlineStr">
@@ -7575,7 +7575,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L120" s="17" t="inlineStr">
+      <c r="L120" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7587,19 +7587,19 @@
       </c>
     </row>
     <row r="121" ht="40" customHeight="1">
-      <c r="A121" s="16" t="inlineStr">
+      <c r="A121" s="17" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B121" s="6" t="inlineStr">
         <is>
-          <t>EUS-95830</t>
+          <t>EUS-49620</t>
         </is>
       </c>
       <c r="C121" s="6" t="inlineStr">
         <is>
-          <t>Suministro de 4 mesas tipo picnic para zona verde en el Polígono Zubieta</t>
+          <t>Contratación de un Organismo de Control Autorizado (OCA) para realizar la inspección reglamentaria de los ascensores de los edificios judiciales de la CAPV</t>
         </is>
       </c>
       <c r="D121" s="6" t="inlineStr">
@@ -7630,7 +7630,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L121" s="17" t="inlineStr">
+      <c r="L121" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7641,12 +7641,67 @@
         </is>
       </c>
     </row>
+    <row r="122" ht="40" customHeight="1">
+      <c r="A122" s="17" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B122" s="6" t="inlineStr">
+        <is>
+          <t>EUS-03622</t>
+        </is>
+      </c>
+      <c r="C122" s="6" t="inlineStr">
+        <is>
+          <t>Servicio de limpieza de vestuarios de Izki Golf</t>
+        </is>
+      </c>
+      <c r="D122" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E122" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F122" s="6" t="inlineStr"/>
+      <c r="G122" s="6" t="inlineStr"/>
+      <c r="H122" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I122" s="10" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J122" s="6" t="inlineStr"/>
+      <c r="K122" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L122" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M122" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:M121"/>
+  <autoFilter ref="A4:M122"/>
   <mergeCells count="5">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A5:M5"/>
-    <mergeCell ref="A110:M110"/>
+    <mergeCell ref="A109:M109"/>
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A107:M107"/>
   </mergeCells>
@@ -7753,7 +7808,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M105" r:id="rId100"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M106" r:id="rId101"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M108" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M109" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M110" r:id="rId103"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M111" r:id="rId104"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M112" r:id="rId105"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M113" r:id="rId106"/>
@@ -7765,6 +7820,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M119" r:id="rId112"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M120" r:id="rId113"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M121" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M122" r:id="rId115"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7776,7 +7832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1709"/>
+  <dimension ref="A1:F1724"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -29666,7 +29722,7 @@
     <row r="1516" ht="30" customHeight="1">
       <c r="A1516" s="18" t="inlineStr">
         <is>
-          <t>FICHA 102: BDNS-897488</t>
+          <t>FICHA 102: BDNS-898162</t>
         </is>
       </c>
       <c r="B1516" s="19" t="n"/>
@@ -29699,7 +29755,7 @@
       </c>
       <c r="B1518" s="21" t="inlineStr">
         <is>
-          <t>CONVENIO DE SUBVENCIÓN NOMINATIVA ENTRE EL AYUNTAMIENTO DE VITORIA-GASTEIZ Y LA ASOCIACION DE PRODUCTORES AUDIOVISUALES   APIKA, PARA EL DESARROLLO DEL PROGRAMA APIKA AUDIOVISUAL PROJET LAB 2026</t>
+          <t>CONVENIO DE SUBVENCIÓN NOMINATIVA ENTRE EL AYUNTAMIENTO DE VITORIA-GASTEIZ, FUNDACIÓN VITAL, FUNDACIÓN ADSIS, FUNDACIÓN DIOCESANAS-JESÚS OBRERO FUNDAZIOA-EGIBIDE Y CÁRITAS DIOCESANA DE VITORIA, PARA O</t>
         </is>
       </c>
       <c r="C1518" s="22" t="n"/>
@@ -29715,7 +29771,7 @@
       </c>
       <c r="B1519" s="21" t="inlineStr">
         <is>
-          <t>BDNS-897488</t>
+          <t>BDNS-898162</t>
         </is>
       </c>
       <c r="C1519" s="22" t="n"/>
@@ -29763,7 +29819,7 @@
       </c>
       <c r="B1522" s="21" t="inlineStr">
         <is>
-          <t>31/12/2026</t>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="C1522" s="22" t="n"/>
@@ -29779,7 +29835,7 @@
       </c>
       <c r="B1523" s="21" t="inlineStr">
         <is>
-          <t>20,000.00 EUR</t>
+          <t>120,000.00 EUR</t>
         </is>
       </c>
       <c r="C1523" s="22" t="n"/>
@@ -29811,7 +29867,7 @@
       </c>
       <c r="B1525" s="21" t="inlineStr">
         <is>
-          <t>BDNS 897488</t>
+          <t>BDNS 898162</t>
         </is>
       </c>
       <c r="C1525" s="22" t="n"/>
@@ -29871,7 +29927,7 @@
       </c>
       <c r="B1529" s="24" t="inlineStr">
         <is>
-          <t>https://www.infosubvenciones.es/bdnstrans/GE/es/convocatoria/897488</t>
+          <t>https://www.infosubvenciones.es/bdnstrans/GE/es/convocatoria/898162</t>
         </is>
       </c>
       <c r="C1529" s="22" t="n"/>
@@ -29882,7 +29938,7 @@
     <row r="1531" ht="30" customHeight="1">
       <c r="A1531" s="18" t="inlineStr">
         <is>
-          <t>FICHA 103: BDNS-897535</t>
+          <t>FICHA 103: EUS-17340</t>
         </is>
       </c>
       <c r="B1531" s="19" t="n"/>
@@ -29899,7 +29955,7 @@
       </c>
       <c r="B1532" s="21" t="inlineStr">
         <is>
-          <t>🇪🇸 España</t>
+          <t>🟢 Euskadi</t>
         </is>
       </c>
       <c r="C1532" s="22" t="n"/>
@@ -29915,7 +29971,7 @@
       </c>
       <c r="B1533" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a la implantación, modernización y transformación digital de las pequeñas empresas de comercio, servicios personales y hostelería de Vitoria-Gasteiz 2026</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
         </is>
       </c>
       <c r="C1533" s="22" t="n"/>
@@ -29931,7 +29987,7 @@
       </c>
       <c r="B1534" s="21" t="inlineStr">
         <is>
-          <t>BDNS-897535</t>
+          <t>EUS-17340</t>
         </is>
       </c>
       <c r="C1534" s="22" t="n"/>
@@ -29947,7 +30003,7 @@
       </c>
       <c r="B1535" s="21" t="inlineStr">
         <is>
-          <t>VITORIA-GASTEIZ</t>
+          <t>Euskadi</t>
         </is>
       </c>
       <c r="C1535" s="22" t="n"/>
@@ -29977,11 +30033,7 @@
           <t>Deadline</t>
         </is>
       </c>
-      <c r="B1537" s="21" t="inlineStr">
-        <is>
-          <t>05/05/2026</t>
-        </is>
-      </c>
+      <c r="B1537" s="21" t="inlineStr"/>
       <c r="C1537" s="22" t="n"/>
       <c r="D1537" s="22" t="n"/>
       <c r="E1537" s="22" t="n"/>
@@ -29995,7 +30047,7 @@
       </c>
       <c r="B1538" s="21" t="inlineStr">
         <is>
-          <t>490,000.00 EUR</t>
+          <t>No disponible</t>
         </is>
       </c>
       <c r="C1538" s="22" t="n"/>
@@ -30011,7 +30063,7 @@
       </c>
       <c r="B1539" s="21" t="inlineStr">
         <is>
-          <t>Subvencion Nacional</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C1539" s="22" t="n"/>
@@ -30025,17 +30077,13 @@
           <t>Call ID</t>
         </is>
       </c>
-      <c r="B1540" s="21" t="inlineStr">
-        <is>
-          <t>BDNS 897535</t>
-        </is>
-      </c>
+      <c r="B1540" s="21" t="inlineStr"/>
       <c r="C1540" s="22" t="n"/>
       <c r="D1540" s="22" t="n"/>
       <c r="E1540" s="22" t="n"/>
       <c r="F1540" s="22" t="n"/>
     </row>
-    <row r="1541" ht="45" customHeight="1">
+    <row r="1541" ht="20" customHeight="1">
       <c r="A1541" s="20" t="inlineStr">
         <is>
           <t>Descripcion</t>
@@ -30043,7 +30091,7 @@
       </c>
       <c r="B1541" s="21" t="inlineStr">
         <is>
-          <t>PYME Y PERSONAS FÍSICAS QUE DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
       <c r="C1541" s="22" t="n"/>
@@ -30057,7 +30105,11 @@
           <t>Tags</t>
         </is>
       </c>
-      <c r="B1542" s="21" t="inlineStr"/>
+      <c r="B1542" s="21" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
       <c r="C1542" s="22" t="n"/>
       <c r="D1542" s="22" t="n"/>
       <c r="E1542" s="22" t="n"/>
@@ -30069,9 +30121,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B1543" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
+      <c r="B1543" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALTA — </t>
         </is>
       </c>
       <c r="C1543" s="22" t="n"/>
@@ -30079,7 +30131,7 @@
       <c r="E1543" s="22" t="n"/>
       <c r="F1543" s="22" t="n"/>
     </row>
-    <row r="1544" ht="20" customHeight="1">
+    <row r="1544" ht="45" customHeight="1">
       <c r="A1544" s="20" t="inlineStr">
         <is>
           <t>Enlace al portal</t>
@@ -30087,7 +30139,7 @@
       </c>
       <c r="B1544" s="24" t="inlineStr">
         <is>
-          <t>https://www.infosubvenciones.es/bdnstrans/GE/es/convocatoria/897535</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-con-incremento-de-capacidad-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1544" s="22" t="n"/>
@@ -30098,7 +30150,7 @@
     <row r="1546" ht="30" customHeight="1">
       <c r="A1546" s="18" t="inlineStr">
         <is>
-          <t>FICHA 104: EUS-18545</t>
+          <t>FICHA 104: EUS-60249</t>
         </is>
       </c>
       <c r="B1546" s="19" t="n"/>
@@ -30123,7 +30175,7 @@
       <c r="E1547" s="22" t="n"/>
       <c r="F1547" s="22" t="n"/>
     </row>
-    <row r="1548" ht="45" customHeight="1">
+    <row r="1548" ht="20" customHeight="1">
       <c r="A1548" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -30131,7 +30183,7 @@
       </c>
       <c r="B1548" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
+          <t>Ayudas a la gestión sostenible de los recursos pesqueros 2026</t>
         </is>
       </c>
       <c r="C1548" s="22" t="n"/>
@@ -30147,7 +30199,7 @@
       </c>
       <c r="B1549" s="21" t="inlineStr">
         <is>
-          <t>EUS-18545</t>
+          <t>EUS-60249</t>
         </is>
       </c>
       <c r="C1549" s="22" t="n"/>
@@ -30299,7 +30351,7 @@
       </c>
       <c r="B1559" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-con-incremento-de-capacidad-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-gestion-sostenible-de-los-recursos-pesqueros-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1559" s="22" t="n"/>
@@ -30310,7 +30362,7 @@
     <row r="1561" ht="30" customHeight="1">
       <c r="A1561" s="18" t="inlineStr">
         <is>
-          <t>FICHA 105: EUS-98881</t>
+          <t>FICHA 105: EUS-83408</t>
         </is>
       </c>
       <c r="B1561" s="19" t="n"/>
@@ -30335,7 +30387,7 @@
       <c r="E1562" s="22" t="n"/>
       <c r="F1562" s="22" t="n"/>
     </row>
-    <row r="1563" ht="20" customHeight="1">
+    <row r="1563" ht="45" customHeight="1">
       <c r="A1563" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -30343,7 +30395,7 @@
       </c>
       <c r="B1563" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a la gestión sostenible de los recursos pesqueros 2026</t>
+          <t>Ayudas a la recogida de residuos con la participación de los pescadores en el mar y las playas 2026</t>
         </is>
       </c>
       <c r="C1563" s="22" t="n"/>
@@ -30359,7 +30411,7 @@
       </c>
       <c r="B1564" s="21" t="inlineStr">
         <is>
-          <t>EUS-98881</t>
+          <t>EUS-83408</t>
         </is>
       </c>
       <c r="C1564" s="22" t="n"/>
@@ -30503,7 +30555,7 @@
       <c r="E1573" s="22" t="n"/>
       <c r="F1573" s="22" t="n"/>
     </row>
-    <row r="1574" ht="45" customHeight="1">
+    <row r="1574" ht="20" customHeight="1">
       <c r="A1574" s="20" t="inlineStr">
         <is>
           <t>Enlace al portal</t>
@@ -30511,7 +30563,7 @@
       </c>
       <c r="B1574" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-gestion-sostenible-de-los-recursos-pesqueros-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/fempa-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1574" s="22" t="n"/>
@@ -30522,7 +30574,7 @@
     <row r="1576" ht="30" customHeight="1">
       <c r="A1576" s="18" t="inlineStr">
         <is>
-          <t>FICHA 106: EUS-38210</t>
+          <t>FICHA 106: EUS-21722</t>
         </is>
       </c>
       <c r="B1576" s="19" t="n"/>
@@ -30555,7 +30607,7 @@
       </c>
       <c r="B1578" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a la recogida de residuos con la participación de los pescadores en el mar y las playas 2026</t>
+          <t>Servicios de realización de una campaña de información y sensibilización en materia de residuos de AUM</t>
         </is>
       </c>
       <c r="C1578" s="22" t="n"/>
@@ -30571,7 +30623,7 @@
       </c>
       <c r="B1579" s="21" t="inlineStr">
         <is>
-          <t>EUS-38210</t>
+          <t>EUS-21722</t>
         </is>
       </c>
       <c r="C1579" s="22" t="n"/>
@@ -30647,7 +30699,7 @@
       </c>
       <c r="B1584" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C1584" s="22" t="n"/>
@@ -30715,7 +30767,7 @@
       <c r="E1588" s="22" t="n"/>
       <c r="F1588" s="22" t="n"/>
     </row>
-    <row r="1589" ht="20" customHeight="1">
+    <row r="1589" ht="45" customHeight="1">
       <c r="A1589" s="20" t="inlineStr">
         <is>
           <t>Enlace al portal</t>
@@ -30723,7 +30775,7 @@
       </c>
       <c r="B1589" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/fempa-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicios-realizacion-campana-informacion-y-sensibilizacion-materia-residuos-aum/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1589" s="22" t="n"/>
@@ -30734,7 +30786,7 @@
     <row r="1591" ht="30" customHeight="1">
       <c r="A1591" s="18" t="inlineStr">
         <is>
-          <t>FICHA 107: EUS-62379</t>
+          <t>FICHA 107: EUS-74325</t>
         </is>
       </c>
       <c r="B1591" s="19" t="n"/>
@@ -30767,7 +30819,7 @@
       </c>
       <c r="B1593" s="21" t="inlineStr">
         <is>
-          <t>Poli ipurua: conduccion aportacion aire exterior ?filtrado? para ?climatizador vestuarios piscinas?.</t>
+          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversidad, participación, principios de la UE. Eventos, difusiones e intercambios. Programa de Ciudadanos, Igualdad, Derechos y Valores de la UE (</t>
         </is>
       </c>
       <c r="C1593" s="22" t="n"/>
@@ -30783,7 +30835,7 @@
       </c>
       <c r="B1594" s="21" t="inlineStr">
         <is>
-          <t>EUS-62379</t>
+          <t>EUS-74325</t>
         </is>
       </c>
       <c r="C1594" s="22" t="n"/>
@@ -30859,7 +30911,7 @@
       </c>
       <c r="B1599" s="21" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C1599" s="22" t="n"/>
@@ -30917,9 +30969,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B1603" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ALTA — </t>
+      <c r="B1603" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
         </is>
       </c>
       <c r="C1603" s="22" t="n"/>
@@ -30935,7 +30987,7 @@
       </c>
       <c r="B1604" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/poli-ipurua-conduccion-aportacion-aire-exterior-filtrado-climatizador-vestuarios-piscinas/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260408cervhirisareak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1604" s="22" t="n"/>
@@ -30946,7 +30998,7 @@
     <row r="1606" ht="30" customHeight="1">
       <c r="A1606" s="18" t="inlineStr">
         <is>
-          <t>FICHA 108: EUS-68865</t>
+          <t>FICHA 108: EUS-88845</t>
         </is>
       </c>
       <c r="B1606" s="19" t="n"/>
@@ -30971,7 +31023,7 @@
       <c r="E1607" s="22" t="n"/>
       <c r="F1607" s="22" t="n"/>
     </row>
-    <row r="1608" ht="20" customHeight="1">
+    <row r="1608" ht="45" customHeight="1">
       <c r="A1608" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -30979,7 +31031,7 @@
       </c>
       <c r="B1608" s="21" t="inlineStr">
         <is>
-          <t>Poli orbea: conduccion aportacion aire exterior para ?climatizador sotano?</t>
+          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el marco de la Intervención Sectorial Vitivinícola del Plan Estratégico (PEPAC) de la Política Agrícola Común de la UE 2023-2027</t>
         </is>
       </c>
       <c r="C1608" s="22" t="n"/>
@@ -30995,7 +31047,7 @@
       </c>
       <c r="B1609" s="21" t="inlineStr">
         <is>
-          <t>EUS-68865</t>
+          <t>EUS-88845</t>
         </is>
       </c>
       <c r="C1609" s="22" t="n"/>
@@ -31071,7 +31123,7 @@
       </c>
       <c r="B1614" s="21" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C1614" s="22" t="n"/>
@@ -31129,9 +31181,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B1618" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ALTA — </t>
+      <c r="B1618" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
         </is>
       </c>
       <c r="C1618" s="22" t="n"/>
@@ -31147,7 +31199,7 @@
       </c>
       <c r="B1619" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/poli-orbea-conduccion-aportacion-aire-exterior-climatizador-sotano/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/20260407mahastiardogintza/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1619" s="22" t="n"/>
@@ -31158,7 +31210,7 @@
     <row r="1621" ht="30" customHeight="1">
       <c r="A1621" s="18" t="inlineStr">
         <is>
-          <t>FICHA 109: EUS-45735</t>
+          <t>FICHA 109: EUS-38197</t>
         </is>
       </c>
       <c r="B1621" s="19" t="n"/>
@@ -31191,7 +31243,7 @@
       </c>
       <c r="B1623" s="21" t="inlineStr">
         <is>
-          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversidad, participación, principios de la UE. Eventos, difusiones e intercambios. Programa de Ciudadanos, Igualdad, Derechos y Valores de la UE (</t>
+          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
         </is>
       </c>
       <c r="C1623" s="22" t="n"/>
@@ -31207,7 +31259,7 @@
       </c>
       <c r="B1624" s="21" t="inlineStr">
         <is>
-          <t>EUS-45735</t>
+          <t>EUS-38197</t>
         </is>
       </c>
       <c r="C1624" s="22" t="n"/>
@@ -31359,7 +31411,7 @@
       </c>
       <c r="B1634" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260408cervhirisareak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-contribucion-de-la-acuicultura-al-buen-estado-ambiental-y-prestacion-de-servicios-ambientales-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1634" s="22" t="n"/>
@@ -31370,7 +31422,7 @@
     <row r="1636" ht="30" customHeight="1">
       <c r="A1636" s="18" t="inlineStr">
         <is>
-          <t>FICHA 110: EUS-28095</t>
+          <t>FICHA 110: EUS-28551</t>
         </is>
       </c>
       <c r="B1636" s="19" t="n"/>
@@ -31403,7 +31455,7 @@
       </c>
       <c r="B1638" s="21" t="inlineStr">
         <is>
-          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el marco de la Intervención Sectorial Vitivinícola del Plan Estratégico (PEPAC) de la Política Agrícola Común de la UE 2023-2027</t>
+          <t>Coordinación de Seguridad y Salud en Fase de Ejecución de obra de Renovación de Infraestructuras Urbanas y Pavimentación de la Calle El Campillo-Segunda fase- y Norte de Leza</t>
         </is>
       </c>
       <c r="C1638" s="22" t="n"/>
@@ -31419,7 +31471,7 @@
       </c>
       <c r="B1639" s="21" t="inlineStr">
         <is>
-          <t>EUS-28095</t>
+          <t>EUS-28551</t>
         </is>
       </c>
       <c r="C1639" s="22" t="n"/>
@@ -31495,7 +31547,7 @@
       </c>
       <c r="B1644" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C1644" s="22" t="n"/>
@@ -31571,7 +31623,7 @@
       </c>
       <c r="B1649" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/20260407mahastiardogintza/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/coordinacion-seguridad-y-salud-fase-ejecucion-obra-renovacion-infraestructuras-urbanas-y-pavimentacion-calle-campillo-segunda-fase-y-norte-leza/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1649" s="22" t="n"/>
@@ -31582,7 +31634,7 @@
     <row r="1651" ht="30" customHeight="1">
       <c r="A1651" s="18" t="inlineStr">
         <is>
-          <t>FICHA 111: EUS-41533</t>
+          <t>FICHA 111: EUS-68422</t>
         </is>
       </c>
       <c r="B1651" s="19" t="n"/>
@@ -31615,7 +31667,7 @@
       </c>
       <c r="B1653" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
+          <t>Procedimiento abierto para la contratación de la limpieza de edificios municipales</t>
         </is>
       </c>
       <c r="C1653" s="22" t="n"/>
@@ -31631,7 +31683,7 @@
       </c>
       <c r="B1654" s="21" t="inlineStr">
         <is>
-          <t>EUS-41533</t>
+          <t>EUS-68422</t>
         </is>
       </c>
       <c r="C1654" s="22" t="n"/>
@@ -31707,7 +31759,7 @@
       </c>
       <c r="B1659" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C1659" s="22" t="n"/>
@@ -31783,7 +31835,7 @@
       </c>
       <c r="B1664" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-contribucion-de-la-acuicultura-al-buen-estado-ambiental-y-prestacion-de-servicios-ambientales-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/procedimiento-abierto-contratacion-limpieza-edificios-municipales/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1664" s="22" t="n"/>
@@ -31794,7 +31846,7 @@
     <row r="1666" ht="30" customHeight="1">
       <c r="A1666" s="18" t="inlineStr">
         <is>
-          <t>FICHA 112: EUS-46847</t>
+          <t>FICHA 112: EUS-20992</t>
         </is>
       </c>
       <c r="B1666" s="19" t="n"/>
@@ -31819,7 +31871,7 @@
       <c r="E1667" s="22" t="n"/>
       <c r="F1667" s="22" t="n"/>
     </row>
-    <row r="1668" ht="45" customHeight="1">
+    <row r="1668" ht="20" customHeight="1">
       <c r="A1668" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -31827,7 +31879,7 @@
       </c>
       <c r="B1668" s="21" t="inlineStr">
         <is>
-          <t>Enajenación mediante procedimiento de subasta pública del local letra D del entresuelo del edificio ubicado en la Avenida de Navarra nº 16 de Pasaia</t>
+          <t>Compra de una reja para el parque del polideportivo.</t>
         </is>
       </c>
       <c r="C1668" s="22" t="n"/>
@@ -31843,7 +31895,7 @@
       </c>
       <c r="B1669" s="21" t="inlineStr">
         <is>
-          <t>EUS-46847</t>
+          <t>EUS-20992</t>
         </is>
       </c>
       <c r="C1669" s="22" t="n"/>
@@ -31995,7 +32047,7 @@
       </c>
       <c r="B1679" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/enajenacion-mediante-procedimiento-subasta-publica-del-local-letra-d-del-entresuelo-del-edificio-ubicado-avenida-navarra-n-16-pasaia/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/compra-reja-parque-del-polideportivo/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1679" s="22" t="n"/>
@@ -32006,7 +32058,7 @@
     <row r="1681" ht="30" customHeight="1">
       <c r="A1681" s="18" t="inlineStr">
         <is>
-          <t>FICHA 113: EUS-44891</t>
+          <t>FICHA 113: EUS-44621</t>
         </is>
       </c>
       <c r="B1681" s="19" t="n"/>
@@ -32039,7 +32091,7 @@
       </c>
       <c r="B1683" s="21" t="inlineStr">
         <is>
-          <t>Suministro de Equipamiento para ampliaciones de capacidad de la red de transporte de ITELAZPI S.A</t>
+          <t>Realización de copias de llaves de la habitación del grupo de consumo y de las viviendas tuteladas</t>
         </is>
       </c>
       <c r="C1683" s="22" t="n"/>
@@ -32055,7 +32107,7 @@
       </c>
       <c r="B1684" s="21" t="inlineStr">
         <is>
-          <t>EUS-44891</t>
+          <t>EUS-44621</t>
         </is>
       </c>
       <c r="C1684" s="22" t="n"/>
@@ -32207,7 +32259,7 @@
       </c>
       <c r="B1694" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-equipamiento-ampliaciones-capacidad-red-transporte-itelazpi-s-a/expapjaso692459/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/realizacion-copias-llaves-habitacion-del-grupo-consumo-y-viviendas-tuteladas/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1694" s="22" t="n"/>
@@ -32218,7 +32270,7 @@
     <row r="1696" ht="30" customHeight="1">
       <c r="A1696" s="18" t="inlineStr">
         <is>
-          <t>FICHA 114: EUS-95830</t>
+          <t>FICHA 114: EUS-49620</t>
         </is>
       </c>
       <c r="B1696" s="19" t="n"/>
@@ -32243,7 +32295,7 @@
       <c r="E1697" s="22" t="n"/>
       <c r="F1697" s="22" t="n"/>
     </row>
-    <row r="1698" ht="20" customHeight="1">
+    <row r="1698" ht="45" customHeight="1">
       <c r="A1698" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -32251,7 +32303,7 @@
       </c>
       <c r="B1698" s="21" t="inlineStr">
         <is>
-          <t>Suministro de 4 mesas tipo picnic para zona verde en el Polígono Zubieta</t>
+          <t>Contratación de un Organismo de Control Autorizado (OCA) para realizar la inspección reglamentaria de los ascensores de los edificios judiciales de la CAPV</t>
         </is>
       </c>
       <c r="C1698" s="22" t="n"/>
@@ -32267,7 +32319,7 @@
       </c>
       <c r="B1699" s="21" t="inlineStr">
         <is>
-          <t>EUS-95830</t>
+          <t>EUS-49620</t>
         </is>
       </c>
       <c r="C1699" s="22" t="n"/>
@@ -32419,7 +32471,7 @@
       </c>
       <c r="B1709" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-4-mesas-tipo-picnic-zona-verde-poligono-zubieta/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/contratacion-organismo-control-autorizado-oca-realizar-inspeccion-reglamentaria-ascensores-edificios-judiciales-capv/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1709" s="22" t="n"/>
@@ -32427,8 +32479,220 @@
       <c r="E1709" s="22" t="n"/>
       <c r="F1709" s="22" t="n"/>
     </row>
+    <row r="1711" ht="30" customHeight="1">
+      <c r="A1711" s="18" t="inlineStr">
+        <is>
+          <t>FICHA 115: EUS-03622</t>
+        </is>
+      </c>
+      <c r="B1711" s="19" t="n"/>
+      <c r="C1711" s="19" t="n"/>
+      <c r="D1711" s="19" t="n"/>
+      <c r="E1711" s="19" t="n"/>
+      <c r="F1711" s="19" t="n"/>
+    </row>
+    <row r="1712" ht="20" customHeight="1">
+      <c r="A1712" s="20" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1712" s="21" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1712" s="22" t="n"/>
+      <c r="D1712" s="22" t="n"/>
+      <c r="E1712" s="22" t="n"/>
+      <c r="F1712" s="22" t="n"/>
+    </row>
+    <row r="1713" ht="20" customHeight="1">
+      <c r="A1713" s="20" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1713" s="21" t="inlineStr">
+        <is>
+          <t>Servicio de limpieza de vestuarios de Izki Golf</t>
+        </is>
+      </c>
+      <c r="C1713" s="22" t="n"/>
+      <c r="D1713" s="22" t="n"/>
+      <c r="E1713" s="22" t="n"/>
+      <c r="F1713" s="22" t="n"/>
+    </row>
+    <row r="1714" ht="20" customHeight="1">
+      <c r="A1714" s="20" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1714" s="21" t="inlineStr">
+        <is>
+          <t>EUS-03622</t>
+        </is>
+      </c>
+      <c r="C1714" s="22" t="n"/>
+      <c r="D1714" s="22" t="n"/>
+      <c r="E1714" s="22" t="n"/>
+      <c r="F1714" s="22" t="n"/>
+    </row>
+    <row r="1715" ht="20" customHeight="1">
+      <c r="A1715" s="20" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1715" s="21" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1715" s="22" t="n"/>
+      <c r="D1715" s="22" t="n"/>
+      <c r="E1715" s="22" t="n"/>
+      <c r="F1715" s="22" t="n"/>
+    </row>
+    <row r="1716" ht="20" customHeight="1">
+      <c r="A1716" s="20" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1716" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1716" s="22" t="n"/>
+      <c r="D1716" s="22" t="n"/>
+      <c r="E1716" s="22" t="n"/>
+      <c r="F1716" s="22" t="n"/>
+    </row>
+    <row r="1717" ht="20" customHeight="1">
+      <c r="A1717" s="20" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1717" s="21" t="inlineStr"/>
+      <c r="C1717" s="22" t="n"/>
+      <c r="D1717" s="22" t="n"/>
+      <c r="E1717" s="22" t="n"/>
+      <c r="F1717" s="22" t="n"/>
+    </row>
+    <row r="1718" ht="20" customHeight="1">
+      <c r="A1718" s="20" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1718" s="21" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1718" s="22" t="n"/>
+      <c r="D1718" s="22" t="n"/>
+      <c r="E1718" s="22" t="n"/>
+      <c r="F1718" s="22" t="n"/>
+    </row>
+    <row r="1719" ht="20" customHeight="1">
+      <c r="A1719" s="20" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1719" s="21" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1719" s="22" t="n"/>
+      <c r="D1719" s="22" t="n"/>
+      <c r="E1719" s="22" t="n"/>
+      <c r="F1719" s="22" t="n"/>
+    </row>
+    <row r="1720" ht="20" customHeight="1">
+      <c r="A1720" s="20" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1720" s="21" t="inlineStr"/>
+      <c r="C1720" s="22" t="n"/>
+      <c r="D1720" s="22" t="n"/>
+      <c r="E1720" s="22" t="n"/>
+      <c r="F1720" s="22" t="n"/>
+    </row>
+    <row r="1721" ht="20" customHeight="1">
+      <c r="A1721" s="20" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1721" s="21" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1721" s="22" t="n"/>
+      <c r="D1721" s="22" t="n"/>
+      <c r="E1721" s="22" t="n"/>
+      <c r="F1721" s="22" t="n"/>
+    </row>
+    <row r="1722" ht="20" customHeight="1">
+      <c r="A1722" s="20" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1722" s="21" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1722" s="22" t="n"/>
+      <c r="D1722" s="22" t="n"/>
+      <c r="E1722" s="22" t="n"/>
+      <c r="F1722" s="22" t="n"/>
+    </row>
+    <row r="1723" ht="20" customHeight="1">
+      <c r="A1723" s="20" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1723" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1723" s="22" t="n"/>
+      <c r="D1723" s="22" t="n"/>
+      <c r="E1723" s="22" t="n"/>
+      <c r="F1723" s="22" t="n"/>
+    </row>
+    <row r="1724" ht="45" customHeight="1">
+      <c r="A1724" s="20" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1724" s="24" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-limpieza-vestuarios-izki-golf/expcm502232/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1724" s="22" t="n"/>
+      <c r="D1724" s="22" t="n"/>
+      <c r="E1724" s="22" t="n"/>
+      <c r="F1724" s="22" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="1596">
+  <mergeCells count="1610">
     <mergeCell ref="B679:F679"/>
     <mergeCell ref="B1010:F1010"/>
     <mergeCell ref="B276:F276"/>
@@ -32632,6 +32896,7 @@
     <mergeCell ref="B529:F529"/>
     <mergeCell ref="B523:F523"/>
     <mergeCell ref="B827:F827"/>
+    <mergeCell ref="B1713:F1713"/>
     <mergeCell ref="A436:F436"/>
     <mergeCell ref="A121:F121"/>
     <mergeCell ref="B668:F668"/>
@@ -32646,6 +32911,7 @@
     <mergeCell ref="B880:F880"/>
     <mergeCell ref="B671:F671"/>
     <mergeCell ref="B1187:F1187"/>
+    <mergeCell ref="B1724:F1724"/>
     <mergeCell ref="B969:F969"/>
     <mergeCell ref="B1607:F1607"/>
     <mergeCell ref="B963:F963"/>
@@ -32695,8 +32961,10 @@
     <mergeCell ref="B336:F336"/>
     <mergeCell ref="B634:F634"/>
     <mergeCell ref="B1422:F1422"/>
+    <mergeCell ref="B1720:F1720"/>
     <mergeCell ref="B965:F965"/>
     <mergeCell ref="B669:F669"/>
+    <mergeCell ref="B1722:F1722"/>
     <mergeCell ref="A451:F451"/>
     <mergeCell ref="A901:F901"/>
     <mergeCell ref="B563:F563"/>
@@ -32814,6 +33082,7 @@
     <mergeCell ref="B1504:F1504"/>
     <mergeCell ref="B445:F445"/>
     <mergeCell ref="B743:F743"/>
+    <mergeCell ref="A1711:F1711"/>
     <mergeCell ref="B18:F18"/>
     <mergeCell ref="B1506:F1506"/>
     <mergeCell ref="B797:F797"/>
@@ -32995,6 +33264,7 @@
     <mergeCell ref="B1089:F1089"/>
     <mergeCell ref="B877:F877"/>
     <mergeCell ref="B1387:F1387"/>
+    <mergeCell ref="B1721:F1721"/>
     <mergeCell ref="B1300:F1300"/>
     <mergeCell ref="B1604:F1604"/>
     <mergeCell ref="B205:F205"/>
@@ -33046,10 +33316,12 @@
     <mergeCell ref="B1427:F1427"/>
     <mergeCell ref="B1419:F1419"/>
     <mergeCell ref="B664:F664"/>
+    <mergeCell ref="B1717:F1717"/>
     <mergeCell ref="B658:F658"/>
     <mergeCell ref="B239:F239"/>
     <mergeCell ref="B1429:F1429"/>
     <mergeCell ref="B1421:F1421"/>
+    <mergeCell ref="B1719:F1719"/>
     <mergeCell ref="B659:F659"/>
     <mergeCell ref="A871:F871"/>
     <mergeCell ref="B232:F232"/>
@@ -33267,9 +33539,11 @@
     <mergeCell ref="B1558:F1558"/>
     <mergeCell ref="B499:F499"/>
     <mergeCell ref="A1171:F1171"/>
+    <mergeCell ref="B1716:F1716"/>
     <mergeCell ref="B1262:F1262"/>
     <mergeCell ref="B534:F534"/>
     <mergeCell ref="B805:F805"/>
+    <mergeCell ref="B1718:F1718"/>
     <mergeCell ref="B957:F957"/>
     <mergeCell ref="B536:F536"/>
     <mergeCell ref="B834:F834"/>
@@ -33636,6 +33910,7 @@
     <mergeCell ref="B531:F531"/>
     <mergeCell ref="B1417:F1417"/>
     <mergeCell ref="B662:F662"/>
+    <mergeCell ref="B1715:F1715"/>
     <mergeCell ref="B954:F954"/>
     <mergeCell ref="B199:F199"/>
     <mergeCell ref="B1112:F1112"/>
@@ -33943,6 +34218,7 @@
     <mergeCell ref="B1267:F1267"/>
     <mergeCell ref="B1609:F1609"/>
     <mergeCell ref="A751:F751"/>
+    <mergeCell ref="B1723:F1723"/>
     <mergeCell ref="B1567:F1567"/>
     <mergeCell ref="A1051:F1051"/>
     <mergeCell ref="B970:F970"/>
@@ -34012,6 +34288,7 @@
     <mergeCell ref="B1107:F1107"/>
     <mergeCell ref="B1378:F1378"/>
     <mergeCell ref="B1536:F1536"/>
+    <mergeCell ref="B1712:F1712"/>
     <mergeCell ref="B653:F653"/>
     <mergeCell ref="B1109:F1109"/>
     <mergeCell ref="B354:F354"/>
@@ -34019,6 +34296,7 @@
     <mergeCell ref="B348:F348"/>
     <mergeCell ref="B652:F652"/>
     <mergeCell ref="B1538:F1538"/>
+    <mergeCell ref="B1714:F1714"/>
     <mergeCell ref="B1409:F1409"/>
     <mergeCell ref="B1292:F1292"/>
     <mergeCell ref="B1707:F1707"/>
@@ -34141,6 +34419,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1679" r:id="rId112"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1694" r:id="rId113"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1709" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1724" r:id="rId115"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -34152,7 +34431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J115"/>
+  <dimension ref="A1:J116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -38154,7 +38433,7 @@
     <row r="103" ht="28" customHeight="1">
       <c r="A103" s="6" t="inlineStr">
         <is>
-          <t>BDNS-897488</t>
+          <t>BDNS-898162</t>
         </is>
       </c>
       <c r="B103" s="6" t="inlineStr">
@@ -38174,7 +38453,7 @@
       </c>
       <c r="E103" s="6" t="inlineStr">
         <is>
-          <t>31/12/2026</t>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="F103" s="27" t="inlineStr">
@@ -38194,17 +38473,17 @@
     <row r="104" ht="28" customHeight="1">
       <c r="A104" s="6" t="inlineStr">
         <is>
-          <t>BDNS-897535</t>
+          <t>EUS-17340</t>
         </is>
       </c>
       <c r="B104" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la implantación, modernización y transformación dig</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
         </is>
       </c>
       <c r="C104" s="6" t="inlineStr">
         <is>
-          <t>VITORIA-GASTEIZ</t>
+          <t>Euskadi</t>
         </is>
       </c>
       <c r="D104" s="6" t="inlineStr">
@@ -38212,14 +38491,10 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="E104" s="6" t="inlineStr">
-        <is>
-          <t>05/05/2026</t>
-        </is>
-      </c>
+      <c r="E104" s="6" t="inlineStr"/>
       <c r="F104" s="27" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="G104" s="6" t="inlineStr"/>
@@ -38234,12 +38509,12 @@
     <row r="105" ht="28" customHeight="1">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>EUS-18545</t>
+          <t>EUS-60249</t>
         </is>
       </c>
       <c r="B105" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
+          <t>Ayudas a la gestión sostenible de los recursos pesqueros 202</t>
         </is>
       </c>
       <c r="C105" s="6" t="inlineStr">
@@ -38270,12 +38545,12 @@
     <row r="106" ht="28" customHeight="1">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>EUS-98881</t>
+          <t>EUS-83408</t>
         </is>
       </c>
       <c r="B106" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la gestión sostenible de los recursos pesqueros 202</t>
+          <t>Ayudas a la recogida de residuos con la participación de los</t>
         </is>
       </c>
       <c r="C106" s="6" t="inlineStr">
@@ -38306,12 +38581,12 @@
     <row r="107" ht="28" customHeight="1">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>EUS-38210</t>
+          <t>EUS-21722</t>
         </is>
       </c>
       <c r="B107" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la recogida de residuos con la participación de los</t>
+          <t>Servicios de realización de una campaña de información y sen</t>
         </is>
       </c>
       <c r="C107" s="6" t="inlineStr">
@@ -38342,12 +38617,12 @@
     <row r="108" ht="28" customHeight="1">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>EUS-62379</t>
+          <t>EUS-74325</t>
         </is>
       </c>
       <c r="B108" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Poli ipurua: conduccion aportacion aire exterior ?filtrado? </t>
+          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversi</t>
         </is>
       </c>
       <c r="C108" s="6" t="inlineStr">
@@ -38363,7 +38638,7 @@
       <c r="E108" s="6" t="inlineStr"/>
       <c r="F108" s="27" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>MEDIA</t>
         </is>
       </c>
       <c r="G108" s="6" t="inlineStr"/>
@@ -38378,12 +38653,12 @@
     <row r="109" ht="28" customHeight="1">
       <c r="A109" s="6" t="inlineStr">
         <is>
-          <t>EUS-68865</t>
+          <t>EUS-88845</t>
         </is>
       </c>
       <c r="B109" s="6" t="inlineStr">
         <is>
-          <t>Poli orbea: conduccion aportacion aire exterior para ?climat</t>
+          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el ma</t>
         </is>
       </c>
       <c r="C109" s="6" t="inlineStr">
@@ -38399,7 +38674,7 @@
       <c r="E109" s="6" t="inlineStr"/>
       <c r="F109" s="27" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>MEDIA</t>
         </is>
       </c>
       <c r="G109" s="6" t="inlineStr"/>
@@ -38414,12 +38689,12 @@
     <row r="110" ht="28" customHeight="1">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>EUS-45735</t>
+          <t>EUS-38197</t>
         </is>
       </c>
       <c r="B110" s="6" t="inlineStr">
         <is>
-          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversi</t>
+          <t>Ayudas a la contribución de la acuicultura al buen estado am</t>
         </is>
       </c>
       <c r="C110" s="6" t="inlineStr">
@@ -38450,12 +38725,12 @@
     <row r="111" ht="28" customHeight="1">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>EUS-28095</t>
+          <t>EUS-28551</t>
         </is>
       </c>
       <c r="B111" s="6" t="inlineStr">
         <is>
-          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el ma</t>
+          <t>Coordinación de Seguridad y Salud en Fase de Ejecución de ob</t>
         </is>
       </c>
       <c r="C111" s="6" t="inlineStr">
@@ -38486,12 +38761,12 @@
     <row r="112" ht="28" customHeight="1">
       <c r="A112" s="6" t="inlineStr">
         <is>
-          <t>EUS-41533</t>
+          <t>EUS-68422</t>
         </is>
       </c>
       <c r="B112" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la contribución de la acuicultura al buen estado am</t>
+          <t>Procedimiento abierto para la contratación de la limpieza de</t>
         </is>
       </c>
       <c r="C112" s="6" t="inlineStr">
@@ -38522,12 +38797,12 @@
     <row r="113" ht="28" customHeight="1">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>EUS-46847</t>
+          <t>EUS-20992</t>
         </is>
       </c>
       <c r="B113" s="6" t="inlineStr">
         <is>
-          <t>Enajenación mediante procedimiento de subasta pública del lo</t>
+          <t>Compra de una reja para el parque del polideportivo.</t>
         </is>
       </c>
       <c r="C113" s="6" t="inlineStr">
@@ -38558,12 +38833,12 @@
     <row r="114" ht="28" customHeight="1">
       <c r="A114" s="6" t="inlineStr">
         <is>
-          <t>EUS-44891</t>
+          <t>EUS-44621</t>
         </is>
       </c>
       <c r="B114" s="6" t="inlineStr">
         <is>
-          <t>Suministro de Equipamiento para ampliaciones de capacidad de</t>
+          <t>Realización de copias de llaves de la habitación del grupo d</t>
         </is>
       </c>
       <c r="C114" s="6" t="inlineStr">
@@ -38594,12 +38869,12 @@
     <row r="115" ht="28" customHeight="1">
       <c r="A115" s="6" t="inlineStr">
         <is>
-          <t>EUS-95830</t>
+          <t>EUS-49620</t>
         </is>
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>Suministro de 4 mesas tipo picnic para zona verde en el Polí</t>
+          <t>Contratación de un Organismo de Control Autorizado (OCA) par</t>
         </is>
       </c>
       <c r="C115" s="6" t="inlineStr">
@@ -38627,8 +38902,44 @@
       <c r="I115" s="6" t="inlineStr"/>
       <c r="J115" s="6" t="inlineStr"/>
     </row>
+    <row r="116" ht="28" customHeight="1">
+      <c r="A116" s="6" t="inlineStr">
+        <is>
+          <t>EUS-03622</t>
+        </is>
+      </c>
+      <c r="B116" s="6" t="inlineStr">
+        <is>
+          <t>Servicio de limpieza de vestuarios de Izki Golf</t>
+        </is>
+      </c>
+      <c r="C116" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D116" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E116" s="6" t="inlineStr"/>
+      <c r="F116" s="27" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G116" s="6" t="inlineStr"/>
+      <c r="H116" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I116" s="6" t="inlineStr"/>
+      <c r="J116" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J115"/>
+  <autoFilter ref="A1:J116"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update funding data 2026-04-12
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -84,13 +84,13 @@
     <font>
       <name val="Leelawadee UI"/>
       <b val="1"/>
-      <color rgb="00DC2626"/>
+      <color rgb="00065F46"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Leelawadee UI"/>
       <b val="1"/>
-      <color rgb="00065F46"/>
+      <color rgb="00DC2626"/>
       <sz val="10"/>
     </font>
     <font>
@@ -166,17 +166,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00065F46"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -268,11 +268,11 @@
     <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -312,8 +312,8 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -707,7 +707,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 11/04/2026 06:48 - 115 convocatorias - 14 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 12/04/2026 07:07 - 115 convocatorias - 13 nuevas</t>
         </is>
       </c>
     </row>
@@ -6963,11 +6963,7 @@
           <t>PERSONAS JURÍDICAS QUE NO DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
         </is>
       </c>
-      <c r="L108" s="15" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
+      <c r="L108" s="6" t="inlineStr"/>
       <c r="M108" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
@@ -6975,21 +6971,21 @@
       </c>
     </row>
     <row r="109" ht="28" customHeight="1">
-      <c r="A109" s="16" t="inlineStr">
+      <c r="A109" s="15" t="inlineStr">
         <is>
           <t>🟢 Euskadi</t>
         </is>
       </c>
     </row>
     <row r="110" ht="40" customHeight="1">
-      <c r="A110" s="17" t="inlineStr">
+      <c r="A110" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B110" s="6" t="inlineStr">
         <is>
-          <t>EUS-17340</t>
+          <t>EUS-04597</t>
         </is>
       </c>
       <c r="C110" s="6" t="inlineStr">
@@ -7025,7 +7021,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L110" s="15" t="inlineStr">
+      <c r="L110" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7037,14 +7033,14 @@
       </c>
     </row>
     <row r="111" ht="40" customHeight="1">
-      <c r="A111" s="17" t="inlineStr">
+      <c r="A111" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B111" s="6" t="inlineStr">
         <is>
-          <t>EUS-60249</t>
+          <t>EUS-61747</t>
         </is>
       </c>
       <c r="C111" s="6" t="inlineStr">
@@ -7080,7 +7076,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L111" s="15" t="inlineStr">
+      <c r="L111" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7092,14 +7088,14 @@
       </c>
     </row>
     <row r="112" ht="40" customHeight="1">
-      <c r="A112" s="17" t="inlineStr">
+      <c r="A112" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B112" s="6" t="inlineStr">
         <is>
-          <t>EUS-83408</t>
+          <t>EUS-57563</t>
         </is>
       </c>
       <c r="C112" s="6" t="inlineStr">
@@ -7135,7 +7131,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L112" s="15" t="inlineStr">
+      <c r="L112" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7147,14 +7143,14 @@
       </c>
     </row>
     <row r="113" ht="40" customHeight="1">
-      <c r="A113" s="17" t="inlineStr">
+      <c r="A113" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B113" s="6" t="inlineStr">
         <is>
-          <t>EUS-21722</t>
+          <t>EUS-46669</t>
         </is>
       </c>
       <c r="C113" s="6" t="inlineStr">
@@ -7190,7 +7186,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L113" s="15" t="inlineStr">
+      <c r="L113" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7202,14 +7198,14 @@
       </c>
     </row>
     <row r="114" ht="40" customHeight="1">
-      <c r="A114" s="17" t="inlineStr">
+      <c r="A114" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B114" s="6" t="inlineStr">
         <is>
-          <t>EUS-74325</t>
+          <t>EUS-93406</t>
         </is>
       </c>
       <c r="C114" s="6" t="inlineStr">
@@ -7245,7 +7241,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L114" s="15" t="inlineStr">
+      <c r="L114" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7257,14 +7253,14 @@
       </c>
     </row>
     <row r="115" ht="40" customHeight="1">
-      <c r="A115" s="17" t="inlineStr">
+      <c r="A115" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>EUS-88845</t>
+          <t>EUS-55744</t>
         </is>
       </c>
       <c r="C115" s="6" t="inlineStr">
@@ -7300,7 +7296,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L115" s="15" t="inlineStr">
+      <c r="L115" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7312,14 +7308,14 @@
       </c>
     </row>
     <row r="116" ht="40" customHeight="1">
-      <c r="A116" s="17" t="inlineStr">
+      <c r="A116" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B116" s="6" t="inlineStr">
         <is>
-          <t>EUS-38197</t>
+          <t>EUS-31585</t>
         </is>
       </c>
       <c r="C116" s="6" t="inlineStr">
@@ -7355,7 +7351,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L116" s="15" t="inlineStr">
+      <c r="L116" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7367,14 +7363,14 @@
       </c>
     </row>
     <row r="117" ht="40" customHeight="1">
-      <c r="A117" s="17" t="inlineStr">
+      <c r="A117" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B117" s="6" t="inlineStr">
         <is>
-          <t>EUS-28551</t>
+          <t>EUS-49777</t>
         </is>
       </c>
       <c r="C117" s="6" t="inlineStr">
@@ -7410,7 +7406,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L117" s="15" t="inlineStr">
+      <c r="L117" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7422,14 +7418,14 @@
       </c>
     </row>
     <row r="118" ht="40" customHeight="1">
-      <c r="A118" s="17" t="inlineStr">
+      <c r="A118" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B118" s="6" t="inlineStr">
         <is>
-          <t>EUS-68422</t>
+          <t>EUS-92482</t>
         </is>
       </c>
       <c r="C118" s="6" t="inlineStr">
@@ -7465,7 +7461,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L118" s="15" t="inlineStr">
+      <c r="L118" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7477,14 +7473,14 @@
       </c>
     </row>
     <row r="119" ht="40" customHeight="1">
-      <c r="A119" s="17" t="inlineStr">
+      <c r="A119" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B119" s="6" t="inlineStr">
         <is>
-          <t>EUS-20992</t>
+          <t>EUS-00835</t>
         </is>
       </c>
       <c r="C119" s="6" t="inlineStr">
@@ -7520,7 +7516,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L119" s="15" t="inlineStr">
+      <c r="L119" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7532,14 +7528,14 @@
       </c>
     </row>
     <row r="120" ht="40" customHeight="1">
-      <c r="A120" s="17" t="inlineStr">
+      <c r="A120" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B120" s="6" t="inlineStr">
         <is>
-          <t>EUS-44621</t>
+          <t>EUS-84505</t>
         </is>
       </c>
       <c r="C120" s="6" t="inlineStr">
@@ -7575,7 +7571,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L120" s="15" t="inlineStr">
+      <c r="L120" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7587,14 +7583,14 @@
       </c>
     </row>
     <row r="121" ht="40" customHeight="1">
-      <c r="A121" s="17" t="inlineStr">
+      <c r="A121" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B121" s="6" t="inlineStr">
         <is>
-          <t>EUS-49620</t>
+          <t>EUS-08803</t>
         </is>
       </c>
       <c r="C121" s="6" t="inlineStr">
@@ -7630,7 +7626,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L121" s="15" t="inlineStr">
+      <c r="L121" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -7642,14 +7638,14 @@
       </c>
     </row>
     <row r="122" ht="40" customHeight="1">
-      <c r="A122" s="17" t="inlineStr">
+      <c r="A122" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B122" s="6" t="inlineStr">
         <is>
-          <t>EUS-03622</t>
+          <t>EUS-81700</t>
         </is>
       </c>
       <c r="C122" s="6" t="inlineStr">
@@ -7685,7 +7681,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L122" s="15" t="inlineStr">
+      <c r="L122" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -29938,7 +29934,7 @@
     <row r="1531" ht="30" customHeight="1">
       <c r="A1531" s="18" t="inlineStr">
         <is>
-          <t>FICHA 103: EUS-17340</t>
+          <t>FICHA 103: EUS-04597</t>
         </is>
       </c>
       <c r="B1531" s="19" t="n"/>
@@ -29987,7 +29983,7 @@
       </c>
       <c r="B1534" s="21" t="inlineStr">
         <is>
-          <t>EUS-17340</t>
+          <t>EUS-04597</t>
         </is>
       </c>
       <c r="C1534" s="22" t="n"/>
@@ -30150,7 +30146,7 @@
     <row r="1546" ht="30" customHeight="1">
       <c r="A1546" s="18" t="inlineStr">
         <is>
-          <t>FICHA 104: EUS-60249</t>
+          <t>FICHA 104: EUS-61747</t>
         </is>
       </c>
       <c r="B1546" s="19" t="n"/>
@@ -30199,7 +30195,7 @@
       </c>
       <c r="B1549" s="21" t="inlineStr">
         <is>
-          <t>EUS-60249</t>
+          <t>EUS-61747</t>
         </is>
       </c>
       <c r="C1549" s="22" t="n"/>
@@ -30362,7 +30358,7 @@
     <row r="1561" ht="30" customHeight="1">
       <c r="A1561" s="18" t="inlineStr">
         <is>
-          <t>FICHA 105: EUS-83408</t>
+          <t>FICHA 105: EUS-57563</t>
         </is>
       </c>
       <c r="B1561" s="19" t="n"/>
@@ -30411,7 +30407,7 @@
       </c>
       <c r="B1564" s="21" t="inlineStr">
         <is>
-          <t>EUS-83408</t>
+          <t>EUS-57563</t>
         </is>
       </c>
       <c r="C1564" s="22" t="n"/>
@@ -30574,7 +30570,7 @@
     <row r="1576" ht="30" customHeight="1">
       <c r="A1576" s="18" t="inlineStr">
         <is>
-          <t>FICHA 106: EUS-21722</t>
+          <t>FICHA 106: EUS-46669</t>
         </is>
       </c>
       <c r="B1576" s="19" t="n"/>
@@ -30623,7 +30619,7 @@
       </c>
       <c r="B1579" s="21" t="inlineStr">
         <is>
-          <t>EUS-21722</t>
+          <t>EUS-46669</t>
         </is>
       </c>
       <c r="C1579" s="22" t="n"/>
@@ -30786,7 +30782,7 @@
     <row r="1591" ht="30" customHeight="1">
       <c r="A1591" s="18" t="inlineStr">
         <is>
-          <t>FICHA 107: EUS-74325</t>
+          <t>FICHA 107: EUS-93406</t>
         </is>
       </c>
       <c r="B1591" s="19" t="n"/>
@@ -30835,7 +30831,7 @@
       </c>
       <c r="B1594" s="21" t="inlineStr">
         <is>
-          <t>EUS-74325</t>
+          <t>EUS-93406</t>
         </is>
       </c>
       <c r="C1594" s="22" t="n"/>
@@ -30998,7 +30994,7 @@
     <row r="1606" ht="30" customHeight="1">
       <c r="A1606" s="18" t="inlineStr">
         <is>
-          <t>FICHA 108: EUS-88845</t>
+          <t>FICHA 108: EUS-55744</t>
         </is>
       </c>
       <c r="B1606" s="19" t="n"/>
@@ -31047,7 +31043,7 @@
       </c>
       <c r="B1609" s="21" t="inlineStr">
         <is>
-          <t>EUS-88845</t>
+          <t>EUS-55744</t>
         </is>
       </c>
       <c r="C1609" s="22" t="n"/>
@@ -31210,7 +31206,7 @@
     <row r="1621" ht="30" customHeight="1">
       <c r="A1621" s="18" t="inlineStr">
         <is>
-          <t>FICHA 109: EUS-38197</t>
+          <t>FICHA 109: EUS-31585</t>
         </is>
       </c>
       <c r="B1621" s="19" t="n"/>
@@ -31259,7 +31255,7 @@
       </c>
       <c r="B1624" s="21" t="inlineStr">
         <is>
-          <t>EUS-38197</t>
+          <t>EUS-31585</t>
         </is>
       </c>
       <c r="C1624" s="22" t="n"/>
@@ -31422,7 +31418,7 @@
     <row r="1636" ht="30" customHeight="1">
       <c r="A1636" s="18" t="inlineStr">
         <is>
-          <t>FICHA 110: EUS-28551</t>
+          <t>FICHA 110: EUS-49777</t>
         </is>
       </c>
       <c r="B1636" s="19" t="n"/>
@@ -31471,7 +31467,7 @@
       </c>
       <c r="B1639" s="21" t="inlineStr">
         <is>
-          <t>EUS-28551</t>
+          <t>EUS-49777</t>
         </is>
       </c>
       <c r="C1639" s="22" t="n"/>
@@ -31634,7 +31630,7 @@
     <row r="1651" ht="30" customHeight="1">
       <c r="A1651" s="18" t="inlineStr">
         <is>
-          <t>FICHA 111: EUS-68422</t>
+          <t>FICHA 111: EUS-92482</t>
         </is>
       </c>
       <c r="B1651" s="19" t="n"/>
@@ -31683,7 +31679,7 @@
       </c>
       <c r="B1654" s="21" t="inlineStr">
         <is>
-          <t>EUS-68422</t>
+          <t>EUS-92482</t>
         </is>
       </c>
       <c r="C1654" s="22" t="n"/>
@@ -31846,7 +31842,7 @@
     <row r="1666" ht="30" customHeight="1">
       <c r="A1666" s="18" t="inlineStr">
         <is>
-          <t>FICHA 112: EUS-20992</t>
+          <t>FICHA 112: EUS-00835</t>
         </is>
       </c>
       <c r="B1666" s="19" t="n"/>
@@ -31895,7 +31891,7 @@
       </c>
       <c r="B1669" s="21" t="inlineStr">
         <is>
-          <t>EUS-20992</t>
+          <t>EUS-00835</t>
         </is>
       </c>
       <c r="C1669" s="22" t="n"/>
@@ -32058,7 +32054,7 @@
     <row r="1681" ht="30" customHeight="1">
       <c r="A1681" s="18" t="inlineStr">
         <is>
-          <t>FICHA 113: EUS-44621</t>
+          <t>FICHA 113: EUS-84505</t>
         </is>
       </c>
       <c r="B1681" s="19" t="n"/>
@@ -32107,7 +32103,7 @@
       </c>
       <c r="B1684" s="21" t="inlineStr">
         <is>
-          <t>EUS-44621</t>
+          <t>EUS-84505</t>
         </is>
       </c>
       <c r="C1684" s="22" t="n"/>
@@ -32270,7 +32266,7 @@
     <row r="1696" ht="30" customHeight="1">
       <c r="A1696" s="18" t="inlineStr">
         <is>
-          <t>FICHA 114: EUS-49620</t>
+          <t>FICHA 114: EUS-08803</t>
         </is>
       </c>
       <c r="B1696" s="19" t="n"/>
@@ -32319,7 +32315,7 @@
       </c>
       <c r="B1699" s="21" t="inlineStr">
         <is>
-          <t>EUS-49620</t>
+          <t>EUS-08803</t>
         </is>
       </c>
       <c r="C1699" s="22" t="n"/>
@@ -32482,7 +32478,7 @@
     <row r="1711" ht="30" customHeight="1">
       <c r="A1711" s="18" t="inlineStr">
         <is>
-          <t>FICHA 115: EUS-03622</t>
+          <t>FICHA 115: EUS-81700</t>
         </is>
       </c>
       <c r="B1711" s="19" t="n"/>
@@ -32531,7 +32527,7 @@
       </c>
       <c r="B1714" s="21" t="inlineStr">
         <is>
-          <t>EUS-03622</t>
+          <t>EUS-81700</t>
         </is>
       </c>
       <c r="C1714" s="22" t="n"/>
@@ -38473,7 +38469,7 @@
     <row r="104" ht="28" customHeight="1">
       <c r="A104" s="6" t="inlineStr">
         <is>
-          <t>EUS-17340</t>
+          <t>EUS-04597</t>
         </is>
       </c>
       <c r="B104" s="6" t="inlineStr">
@@ -38509,7 +38505,7 @@
     <row r="105" ht="28" customHeight="1">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>EUS-60249</t>
+          <t>EUS-61747</t>
         </is>
       </c>
       <c r="B105" s="6" t="inlineStr">
@@ -38545,7 +38541,7 @@
     <row r="106" ht="28" customHeight="1">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>EUS-83408</t>
+          <t>EUS-57563</t>
         </is>
       </c>
       <c r="B106" s="6" t="inlineStr">
@@ -38581,7 +38577,7 @@
     <row r="107" ht="28" customHeight="1">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>EUS-21722</t>
+          <t>EUS-46669</t>
         </is>
       </c>
       <c r="B107" s="6" t="inlineStr">
@@ -38617,7 +38613,7 @@
     <row r="108" ht="28" customHeight="1">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>EUS-74325</t>
+          <t>EUS-93406</t>
         </is>
       </c>
       <c r="B108" s="6" t="inlineStr">
@@ -38653,7 +38649,7 @@
     <row r="109" ht="28" customHeight="1">
       <c r="A109" s="6" t="inlineStr">
         <is>
-          <t>EUS-88845</t>
+          <t>EUS-55744</t>
         </is>
       </c>
       <c r="B109" s="6" t="inlineStr">
@@ -38689,7 +38685,7 @@
     <row r="110" ht="28" customHeight="1">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>EUS-38197</t>
+          <t>EUS-31585</t>
         </is>
       </c>
       <c r="B110" s="6" t="inlineStr">
@@ -38725,7 +38721,7 @@
     <row r="111" ht="28" customHeight="1">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>EUS-28551</t>
+          <t>EUS-49777</t>
         </is>
       </c>
       <c r="B111" s="6" t="inlineStr">
@@ -38761,7 +38757,7 @@
     <row r="112" ht="28" customHeight="1">
       <c r="A112" s="6" t="inlineStr">
         <is>
-          <t>EUS-68422</t>
+          <t>EUS-92482</t>
         </is>
       </c>
       <c r="B112" s="6" t="inlineStr">
@@ -38797,7 +38793,7 @@
     <row r="113" ht="28" customHeight="1">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>EUS-20992</t>
+          <t>EUS-00835</t>
         </is>
       </c>
       <c r="B113" s="6" t="inlineStr">
@@ -38833,7 +38829,7 @@
     <row r="114" ht="28" customHeight="1">
       <c r="A114" s="6" t="inlineStr">
         <is>
-          <t>EUS-44621</t>
+          <t>EUS-84505</t>
         </is>
       </c>
       <c r="B114" s="6" t="inlineStr">
@@ -38869,7 +38865,7 @@
     <row r="115" ht="28" customHeight="1">
       <c r="A115" s="6" t="inlineStr">
         <is>
-          <t>EUS-49620</t>
+          <t>EUS-08803</t>
         </is>
       </c>
       <c r="B115" s="6" t="inlineStr">
@@ -38905,7 +38901,7 @@
     <row r="116" ht="28" customHeight="1">
       <c r="A116" s="6" t="inlineStr">
         <is>
-          <t>EUS-03622</t>
+          <t>EUS-81700</t>
         </is>
       </c>
       <c r="B116" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Update funding data 2026-04-13
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -707,7 +707,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 12/04/2026 07:07 - 115 convocatorias - 13 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 13/04/2026 07:36 - 115 convocatorias - 12 nuevas</t>
         </is>
       </c>
     </row>
@@ -6985,7 +6985,7 @@
       </c>
       <c r="B110" s="6" t="inlineStr">
         <is>
-          <t>EUS-04597</t>
+          <t>EUS-22153</t>
         </is>
       </c>
       <c r="C110" s="6" t="inlineStr">
@@ -7040,7 +7040,7 @@
       </c>
       <c r="B111" s="6" t="inlineStr">
         <is>
-          <t>EUS-61747</t>
+          <t>EUS-98702</t>
         </is>
       </c>
       <c r="C111" s="6" t="inlineStr">
@@ -7095,7 +7095,7 @@
       </c>
       <c r="B112" s="6" t="inlineStr">
         <is>
-          <t>EUS-57563</t>
+          <t>EUS-55703</t>
         </is>
       </c>
       <c r="C112" s="6" t="inlineStr">
@@ -7150,7 +7150,7 @@
       </c>
       <c r="B113" s="6" t="inlineStr">
         <is>
-          <t>EUS-46669</t>
+          <t>EUS-01426</t>
         </is>
       </c>
       <c r="C113" s="6" t="inlineStr">
@@ -7205,7 +7205,7 @@
       </c>
       <c r="B114" s="6" t="inlineStr">
         <is>
-          <t>EUS-93406</t>
+          <t>EUS-75953</t>
         </is>
       </c>
       <c r="C114" s="6" t="inlineStr">
@@ -7260,7 +7260,7 @@
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>EUS-55744</t>
+          <t>EUS-87968</t>
         </is>
       </c>
       <c r="C115" s="6" t="inlineStr">
@@ -7315,7 +7315,7 @@
       </c>
       <c r="B116" s="6" t="inlineStr">
         <is>
-          <t>EUS-31585</t>
+          <t>EUS-02362</t>
         </is>
       </c>
       <c r="C116" s="6" t="inlineStr">
@@ -7370,12 +7370,12 @@
       </c>
       <c r="B117" s="6" t="inlineStr">
         <is>
-          <t>EUS-49777</t>
+          <t>EUS-67124</t>
         </is>
       </c>
       <c r="C117" s="6" t="inlineStr">
         <is>
-          <t>Coordinación de Seguridad y Salud en Fase de Ejecución de obra de Renovación de Infraestructuras Urbanas y Pavimentación de la Calle El Campillo-Segunda fase- y Norte de Leza</t>
+          <t>Obras para la sustitución de cubierta y ventanas en Ermita San Marcial.</t>
         </is>
       </c>
       <c r="D117" s="6" t="inlineStr">
@@ -7425,12 +7425,12 @@
       </c>
       <c r="B118" s="6" t="inlineStr">
         <is>
-          <t>EUS-92482</t>
+          <t>EUS-98636</t>
         </is>
       </c>
       <c r="C118" s="6" t="inlineStr">
         <is>
-          <t>Procedimiento abierto para la contratación de la limpieza de edificios municipales</t>
+          <t>Coordinación de Seguridad y Salud en Fase de Ejecución de obra de Renovación de Infraestructuras Urbanas y Pavimentación de la Calle El Campillo-Segunda fase- y Norte de Leza</t>
         </is>
       </c>
       <c r="D118" s="6" t="inlineStr">
@@ -7461,11 +7461,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L118" s="17" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
+      <c r="L118" s="6" t="inlineStr"/>
       <c r="M118" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
@@ -7480,12 +7476,12 @@
       </c>
       <c r="B119" s="6" t="inlineStr">
         <is>
-          <t>EUS-00835</t>
+          <t>EUS-79655</t>
         </is>
       </c>
       <c r="C119" s="6" t="inlineStr">
         <is>
-          <t>Compra de una reja para el parque del polideportivo.</t>
+          <t>Procedimiento abierto para la contratación de la limpieza de edificios municipales</t>
         </is>
       </c>
       <c r="D119" s="6" t="inlineStr">
@@ -7535,12 +7531,12 @@
       </c>
       <c r="B120" s="6" t="inlineStr">
         <is>
-          <t>EUS-84505</t>
+          <t>EUS-82436</t>
         </is>
       </c>
       <c r="C120" s="6" t="inlineStr">
         <is>
-          <t>Realización de copias de llaves de la habitación del grupo de consumo y de las viviendas tuteladas</t>
+          <t>Compra de una reja para el parque del polideportivo.</t>
         </is>
       </c>
       <c r="D120" s="6" t="inlineStr">
@@ -7590,12 +7586,12 @@
       </c>
       <c r="B121" s="6" t="inlineStr">
         <is>
-          <t>EUS-08803</t>
+          <t>EUS-71968</t>
         </is>
       </c>
       <c r="C121" s="6" t="inlineStr">
         <is>
-          <t>Contratación de un Organismo de Control Autorizado (OCA) para realizar la inspección reglamentaria de los ascensores de los edificios judiciales de la CAPV</t>
+          <t>Realización de copias de llaves de la habitación del grupo de consumo y de las viviendas tuteladas</t>
         </is>
       </c>
       <c r="D121" s="6" t="inlineStr">
@@ -7645,12 +7641,12 @@
       </c>
       <c r="B122" s="6" t="inlineStr">
         <is>
-          <t>EUS-81700</t>
+          <t>EUS-48990</t>
         </is>
       </c>
       <c r="C122" s="6" t="inlineStr">
         <is>
-          <t>Servicio de limpieza de vestuarios de Izki Golf</t>
+          <t>Contratación de un Organismo de Control Autorizado (OCA) para realizar la inspección reglamentaria de los ascensores de los edificios judiciales de la CAPV</t>
         </is>
       </c>
       <c r="D122" s="6" t="inlineStr">
@@ -29934,7 +29930,7 @@
     <row r="1531" ht="30" customHeight="1">
       <c r="A1531" s="18" t="inlineStr">
         <is>
-          <t>FICHA 103: EUS-04597</t>
+          <t>FICHA 103: EUS-22153</t>
         </is>
       </c>
       <c r="B1531" s="19" t="n"/>
@@ -29983,7 +29979,7 @@
       </c>
       <c r="B1534" s="21" t="inlineStr">
         <is>
-          <t>EUS-04597</t>
+          <t>EUS-22153</t>
         </is>
       </c>
       <c r="C1534" s="22" t="n"/>
@@ -30146,7 +30142,7 @@
     <row r="1546" ht="30" customHeight="1">
       <c r="A1546" s="18" t="inlineStr">
         <is>
-          <t>FICHA 104: EUS-61747</t>
+          <t>FICHA 104: EUS-98702</t>
         </is>
       </c>
       <c r="B1546" s="19" t="n"/>
@@ -30195,7 +30191,7 @@
       </c>
       <c r="B1549" s="21" t="inlineStr">
         <is>
-          <t>EUS-61747</t>
+          <t>EUS-98702</t>
         </is>
       </c>
       <c r="C1549" s="22" t="n"/>
@@ -30358,7 +30354,7 @@
     <row r="1561" ht="30" customHeight="1">
       <c r="A1561" s="18" t="inlineStr">
         <is>
-          <t>FICHA 105: EUS-57563</t>
+          <t>FICHA 105: EUS-55703</t>
         </is>
       </c>
       <c r="B1561" s="19" t="n"/>
@@ -30407,7 +30403,7 @@
       </c>
       <c r="B1564" s="21" t="inlineStr">
         <is>
-          <t>EUS-57563</t>
+          <t>EUS-55703</t>
         </is>
       </c>
       <c r="C1564" s="22" t="n"/>
@@ -30570,7 +30566,7 @@
     <row r="1576" ht="30" customHeight="1">
       <c r="A1576" s="18" t="inlineStr">
         <is>
-          <t>FICHA 106: EUS-46669</t>
+          <t>FICHA 106: EUS-01426</t>
         </is>
       </c>
       <c r="B1576" s="19" t="n"/>
@@ -30619,7 +30615,7 @@
       </c>
       <c r="B1579" s="21" t="inlineStr">
         <is>
-          <t>EUS-46669</t>
+          <t>EUS-01426</t>
         </is>
       </c>
       <c r="C1579" s="22" t="n"/>
@@ -30782,7 +30778,7 @@
     <row r="1591" ht="30" customHeight="1">
       <c r="A1591" s="18" t="inlineStr">
         <is>
-          <t>FICHA 107: EUS-93406</t>
+          <t>FICHA 107: EUS-75953</t>
         </is>
       </c>
       <c r="B1591" s="19" t="n"/>
@@ -30831,7 +30827,7 @@
       </c>
       <c r="B1594" s="21" t="inlineStr">
         <is>
-          <t>EUS-93406</t>
+          <t>EUS-75953</t>
         </is>
       </c>
       <c r="C1594" s="22" t="n"/>
@@ -30994,7 +30990,7 @@
     <row r="1606" ht="30" customHeight="1">
       <c r="A1606" s="18" t="inlineStr">
         <is>
-          <t>FICHA 108: EUS-55744</t>
+          <t>FICHA 108: EUS-87968</t>
         </is>
       </c>
       <c r="B1606" s="19" t="n"/>
@@ -31043,7 +31039,7 @@
       </c>
       <c r="B1609" s="21" t="inlineStr">
         <is>
-          <t>EUS-55744</t>
+          <t>EUS-87968</t>
         </is>
       </c>
       <c r="C1609" s="22" t="n"/>
@@ -31206,7 +31202,7 @@
     <row r="1621" ht="30" customHeight="1">
       <c r="A1621" s="18" t="inlineStr">
         <is>
-          <t>FICHA 109: EUS-31585</t>
+          <t>FICHA 109: EUS-02362</t>
         </is>
       </c>
       <c r="B1621" s="19" t="n"/>
@@ -31255,7 +31251,7 @@
       </c>
       <c r="B1624" s="21" t="inlineStr">
         <is>
-          <t>EUS-31585</t>
+          <t>EUS-02362</t>
         </is>
       </c>
       <c r="C1624" s="22" t="n"/>
@@ -31418,7 +31414,7 @@
     <row r="1636" ht="30" customHeight="1">
       <c r="A1636" s="18" t="inlineStr">
         <is>
-          <t>FICHA 110: EUS-49777</t>
+          <t>FICHA 110: EUS-67124</t>
         </is>
       </c>
       <c r="B1636" s="19" t="n"/>
@@ -31443,7 +31439,7 @@
       <c r="E1637" s="22" t="n"/>
       <c r="F1637" s="22" t="n"/>
     </row>
-    <row r="1638" ht="45" customHeight="1">
+    <row r="1638" ht="20" customHeight="1">
       <c r="A1638" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -31451,7 +31447,7 @@
       </c>
       <c r="B1638" s="21" t="inlineStr">
         <is>
-          <t>Coordinación de Seguridad y Salud en Fase de Ejecución de obra de Renovación de Infraestructuras Urbanas y Pavimentación de la Calle El Campillo-Segunda fase- y Norte de Leza</t>
+          <t>Obras para la sustitución de cubierta y ventanas en Ermita San Marcial.</t>
         </is>
       </c>
       <c r="C1638" s="22" t="n"/>
@@ -31467,7 +31463,7 @@
       </c>
       <c r="B1639" s="21" t="inlineStr">
         <is>
-          <t>EUS-49777</t>
+          <t>EUS-67124</t>
         </is>
       </c>
       <c r="C1639" s="22" t="n"/>
@@ -31619,7 +31615,7 @@
       </c>
       <c r="B1649" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/coordinacion-seguridad-y-salud-fase-ejecucion-obra-renovacion-infraestructuras-urbanas-y-pavimentacion-calle-campillo-segunda-fase-y-norte-leza/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/obras-sustitucion-cubierta-y-ventanas-ermita-san-marcial/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1649" s="22" t="n"/>
@@ -31630,7 +31626,7 @@
     <row r="1651" ht="30" customHeight="1">
       <c r="A1651" s="18" t="inlineStr">
         <is>
-          <t>FICHA 111: EUS-92482</t>
+          <t>FICHA 111: EUS-98636</t>
         </is>
       </c>
       <c r="B1651" s="19" t="n"/>
@@ -31663,7 +31659,7 @@
       </c>
       <c r="B1653" s="21" t="inlineStr">
         <is>
-          <t>Procedimiento abierto para la contratación de la limpieza de edificios municipales</t>
+          <t>Coordinación de Seguridad y Salud en Fase de Ejecución de obra de Renovación de Infraestructuras Urbanas y Pavimentación de la Calle El Campillo-Segunda fase- y Norte de Leza</t>
         </is>
       </c>
       <c r="C1653" s="22" t="n"/>
@@ -31679,7 +31675,7 @@
       </c>
       <c r="B1654" s="21" t="inlineStr">
         <is>
-          <t>EUS-92482</t>
+          <t>EUS-98636</t>
         </is>
       </c>
       <c r="C1654" s="22" t="n"/>
@@ -31831,7 +31827,7 @@
       </c>
       <c r="B1664" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/procedimiento-abierto-contratacion-limpieza-edificios-municipales/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/coordinacion-seguridad-y-salud-fase-ejecucion-obra-renovacion-infraestructuras-urbanas-y-pavimentacion-calle-campillo-segunda-fase-y-norte-leza/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1664" s="22" t="n"/>
@@ -31842,7 +31838,7 @@
     <row r="1666" ht="30" customHeight="1">
       <c r="A1666" s="18" t="inlineStr">
         <is>
-          <t>FICHA 112: EUS-00835</t>
+          <t>FICHA 112: EUS-79655</t>
         </is>
       </c>
       <c r="B1666" s="19" t="n"/>
@@ -31867,7 +31863,7 @@
       <c r="E1667" s="22" t="n"/>
       <c r="F1667" s="22" t="n"/>
     </row>
-    <row r="1668" ht="20" customHeight="1">
+    <row r="1668" ht="45" customHeight="1">
       <c r="A1668" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -31875,7 +31871,7 @@
       </c>
       <c r="B1668" s="21" t="inlineStr">
         <is>
-          <t>Compra de una reja para el parque del polideportivo.</t>
+          <t>Procedimiento abierto para la contratación de la limpieza de edificios municipales</t>
         </is>
       </c>
       <c r="C1668" s="22" t="n"/>
@@ -31891,7 +31887,7 @@
       </c>
       <c r="B1669" s="21" t="inlineStr">
         <is>
-          <t>EUS-00835</t>
+          <t>EUS-79655</t>
         </is>
       </c>
       <c r="C1669" s="22" t="n"/>
@@ -32043,7 +32039,7 @@
       </c>
       <c r="B1679" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/compra-reja-parque-del-polideportivo/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/procedimiento-abierto-contratacion-limpieza-edificios-municipales/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1679" s="22" t="n"/>
@@ -32054,7 +32050,7 @@
     <row r="1681" ht="30" customHeight="1">
       <c r="A1681" s="18" t="inlineStr">
         <is>
-          <t>FICHA 113: EUS-84505</t>
+          <t>FICHA 113: EUS-82436</t>
         </is>
       </c>
       <c r="B1681" s="19" t="n"/>
@@ -32079,7 +32075,7 @@
       <c r="E1682" s="22" t="n"/>
       <c r="F1682" s="22" t="n"/>
     </row>
-    <row r="1683" ht="45" customHeight="1">
+    <row r="1683" ht="20" customHeight="1">
       <c r="A1683" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -32087,7 +32083,7 @@
       </c>
       <c r="B1683" s="21" t="inlineStr">
         <is>
-          <t>Realización de copias de llaves de la habitación del grupo de consumo y de las viviendas tuteladas</t>
+          <t>Compra de una reja para el parque del polideportivo.</t>
         </is>
       </c>
       <c r="C1683" s="22" t="n"/>
@@ -32103,7 +32099,7 @@
       </c>
       <c r="B1684" s="21" t="inlineStr">
         <is>
-          <t>EUS-84505</t>
+          <t>EUS-82436</t>
         </is>
       </c>
       <c r="C1684" s="22" t="n"/>
@@ -32255,7 +32251,7 @@
       </c>
       <c r="B1694" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/realizacion-copias-llaves-habitacion-del-grupo-consumo-y-viviendas-tuteladas/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/compra-reja-parque-del-polideportivo/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1694" s="22" t="n"/>
@@ -32266,7 +32262,7 @@
     <row r="1696" ht="30" customHeight="1">
       <c r="A1696" s="18" t="inlineStr">
         <is>
-          <t>FICHA 114: EUS-08803</t>
+          <t>FICHA 114: EUS-71968</t>
         </is>
       </c>
       <c r="B1696" s="19" t="n"/>
@@ -32299,7 +32295,7 @@
       </c>
       <c r="B1698" s="21" t="inlineStr">
         <is>
-          <t>Contratación de un Organismo de Control Autorizado (OCA) para realizar la inspección reglamentaria de los ascensores de los edificios judiciales de la CAPV</t>
+          <t>Realización de copias de llaves de la habitación del grupo de consumo y de las viviendas tuteladas</t>
         </is>
       </c>
       <c r="C1698" s="22" t="n"/>
@@ -32315,7 +32311,7 @@
       </c>
       <c r="B1699" s="21" t="inlineStr">
         <is>
-          <t>EUS-08803</t>
+          <t>EUS-71968</t>
         </is>
       </c>
       <c r="C1699" s="22" t="n"/>
@@ -32467,7 +32463,7 @@
       </c>
       <c r="B1709" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/contratacion-organismo-control-autorizado-oca-realizar-inspeccion-reglamentaria-ascensores-edificios-judiciales-capv/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/realizacion-copias-llaves-habitacion-del-grupo-consumo-y-viviendas-tuteladas/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1709" s="22" t="n"/>
@@ -32478,7 +32474,7 @@
     <row r="1711" ht="30" customHeight="1">
       <c r="A1711" s="18" t="inlineStr">
         <is>
-          <t>FICHA 115: EUS-81700</t>
+          <t>FICHA 115: EUS-48990</t>
         </is>
       </c>
       <c r="B1711" s="19" t="n"/>
@@ -32503,7 +32499,7 @@
       <c r="E1712" s="22" t="n"/>
       <c r="F1712" s="22" t="n"/>
     </row>
-    <row r="1713" ht="20" customHeight="1">
+    <row r="1713" ht="45" customHeight="1">
       <c r="A1713" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -32511,7 +32507,7 @@
       </c>
       <c r="B1713" s="21" t="inlineStr">
         <is>
-          <t>Servicio de limpieza de vestuarios de Izki Golf</t>
+          <t>Contratación de un Organismo de Control Autorizado (OCA) para realizar la inspección reglamentaria de los ascensores de los edificios judiciales de la CAPV</t>
         </is>
       </c>
       <c r="C1713" s="22" t="n"/>
@@ -32527,7 +32523,7 @@
       </c>
       <c r="B1714" s="21" t="inlineStr">
         <is>
-          <t>EUS-81700</t>
+          <t>EUS-48990</t>
         </is>
       </c>
       <c r="C1714" s="22" t="n"/>
@@ -32679,7 +32675,7 @@
       </c>
       <c r="B1724" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-limpieza-vestuarios-izki-golf/expcm502232/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/contratacion-organismo-control-autorizado-oca-realizar-inspeccion-reglamentaria-ascensores-edificios-judiciales-capv/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1724" s="22" t="n"/>
@@ -38469,7 +38465,7 @@
     <row r="104" ht="28" customHeight="1">
       <c r="A104" s="6" t="inlineStr">
         <is>
-          <t>EUS-04597</t>
+          <t>EUS-22153</t>
         </is>
       </c>
       <c r="B104" s="6" t="inlineStr">
@@ -38505,7 +38501,7 @@
     <row r="105" ht="28" customHeight="1">
       <c r="A105" s="6" t="inlineStr">
         <is>
-          <t>EUS-61747</t>
+          <t>EUS-98702</t>
         </is>
       </c>
       <c r="B105" s="6" t="inlineStr">
@@ -38541,7 +38537,7 @@
     <row r="106" ht="28" customHeight="1">
       <c r="A106" s="6" t="inlineStr">
         <is>
-          <t>EUS-57563</t>
+          <t>EUS-55703</t>
         </is>
       </c>
       <c r="B106" s="6" t="inlineStr">
@@ -38577,7 +38573,7 @@
     <row r="107" ht="28" customHeight="1">
       <c r="A107" s="6" t="inlineStr">
         <is>
-          <t>EUS-46669</t>
+          <t>EUS-01426</t>
         </is>
       </c>
       <c r="B107" s="6" t="inlineStr">
@@ -38613,7 +38609,7 @@
     <row r="108" ht="28" customHeight="1">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>EUS-93406</t>
+          <t>EUS-75953</t>
         </is>
       </c>
       <c r="B108" s="6" t="inlineStr">
@@ -38649,7 +38645,7 @@
     <row r="109" ht="28" customHeight="1">
       <c r="A109" s="6" t="inlineStr">
         <is>
-          <t>EUS-55744</t>
+          <t>EUS-87968</t>
         </is>
       </c>
       <c r="B109" s="6" t="inlineStr">
@@ -38685,7 +38681,7 @@
     <row r="110" ht="28" customHeight="1">
       <c r="A110" s="6" t="inlineStr">
         <is>
-          <t>EUS-31585</t>
+          <t>EUS-02362</t>
         </is>
       </c>
       <c r="B110" s="6" t="inlineStr">
@@ -38721,12 +38717,12 @@
     <row r="111" ht="28" customHeight="1">
       <c r="A111" s="6" t="inlineStr">
         <is>
-          <t>EUS-49777</t>
+          <t>EUS-67124</t>
         </is>
       </c>
       <c r="B111" s="6" t="inlineStr">
         <is>
-          <t>Coordinación de Seguridad y Salud en Fase de Ejecución de ob</t>
+          <t>Obras para la sustitución de cubierta y ventanas en Ermita S</t>
         </is>
       </c>
       <c r="C111" s="6" t="inlineStr">
@@ -38757,12 +38753,12 @@
     <row r="112" ht="28" customHeight="1">
       <c r="A112" s="6" t="inlineStr">
         <is>
-          <t>EUS-92482</t>
+          <t>EUS-98636</t>
         </is>
       </c>
       <c r="B112" s="6" t="inlineStr">
         <is>
-          <t>Procedimiento abierto para la contratación de la limpieza de</t>
+          <t>Coordinación de Seguridad y Salud en Fase de Ejecución de ob</t>
         </is>
       </c>
       <c r="C112" s="6" t="inlineStr">
@@ -38793,12 +38789,12 @@
     <row r="113" ht="28" customHeight="1">
       <c r="A113" s="6" t="inlineStr">
         <is>
-          <t>EUS-00835</t>
+          <t>EUS-79655</t>
         </is>
       </c>
       <c r="B113" s="6" t="inlineStr">
         <is>
-          <t>Compra de una reja para el parque del polideportivo.</t>
+          <t>Procedimiento abierto para la contratación de la limpieza de</t>
         </is>
       </c>
       <c r="C113" s="6" t="inlineStr">
@@ -38829,12 +38825,12 @@
     <row r="114" ht="28" customHeight="1">
       <c r="A114" s="6" t="inlineStr">
         <is>
-          <t>EUS-84505</t>
+          <t>EUS-82436</t>
         </is>
       </c>
       <c r="B114" s="6" t="inlineStr">
         <is>
-          <t>Realización de copias de llaves de la habitación del grupo d</t>
+          <t>Compra de una reja para el parque del polideportivo.</t>
         </is>
       </c>
       <c r="C114" s="6" t="inlineStr">
@@ -38865,12 +38861,12 @@
     <row r="115" ht="28" customHeight="1">
       <c r="A115" s="6" t="inlineStr">
         <is>
-          <t>EUS-08803</t>
+          <t>EUS-71968</t>
         </is>
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>Contratación de un Organismo de Control Autorizado (OCA) par</t>
+          <t>Realización de copias de llaves de la habitación del grupo d</t>
         </is>
       </c>
       <c r="C115" s="6" t="inlineStr">
@@ -38901,12 +38897,12 @@
     <row r="116" ht="28" customHeight="1">
       <c r="A116" s="6" t="inlineStr">
         <is>
-          <t>EUS-81700</t>
+          <t>EUS-48990</t>
         </is>
       </c>
       <c r="B116" s="6" t="inlineStr">
         <is>
-          <t>Servicio de limpieza de vestuarios de Izki Golf</t>
+          <t>Contratación de un Organismo de Control Autorizado (OCA) par</t>
         </is>
       </c>
       <c r="C116" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Update funding data 2026-04-19
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Recursos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$91</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$93</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$87</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -84,13 +84,13 @@
     <font>
       <name val="Leelawadee UI"/>
       <b val="1"/>
-      <color rgb="00DC2626"/>
+      <color rgb="00065F46"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Leelawadee UI"/>
       <b val="1"/>
-      <color rgb="00065F46"/>
+      <color rgb="00DC2626"/>
       <sz val="10"/>
     </font>
     <font>
@@ -166,17 +166,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00065F46"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -268,11 +268,11 @@
     <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -312,8 +312,8 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -679,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M91"/>
+  <dimension ref="A1:M93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -707,7 +707,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 18/04/2026 07:00 - 84 convocatorias - 12 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 19/04/2026 07:07 - 86 convocatorias - 10 nuevas</t>
         </is>
       </c>
     </row>
@@ -2529,12 +2529,12 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-08</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
+          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -2574,7 +2574,7 @@
       </c>
       <c r="K34" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and inter</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Euro</t>
         </is>
       </c>
       <c r="L34" s="6" t="inlineStr"/>
@@ -2718,12 +2718,12 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -2748,7 +2748,7 @@
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>Programme Cofund Actions</t>
+          <t xml:space="preserve"> Research and Innovation Actions</t>
         </is>
       </c>
       <c r="I37" s="11" t="inlineStr">
@@ -2763,7 +2763,7 @@
       </c>
       <c r="K37" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is estab</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to info</t>
         </is>
       </c>
       <c r="L37" s="6" t="inlineStr"/>
@@ -2781,12 +2781,12 @@
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -2826,7 +2826,7 @@
       </c>
       <c r="K38" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorpo</t>
+          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and inter</t>
         </is>
       </c>
       <c r="L38" s="6" t="inlineStr"/>
@@ -2844,12 +2844,12 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -2874,7 +2874,7 @@
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Research and Innovation Actions</t>
+          <t>Programme Cofund Actions</t>
         </is>
       </c>
       <c r="I39" s="11" t="inlineStr">
@@ -2889,7 +2889,7 @@
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to info</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is estab</t>
         </is>
       </c>
       <c r="L39" s="6" t="inlineStr"/>
@@ -2907,12 +2907,12 @@
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -2952,7 +2952,7 @@
       </c>
       <c r="K40" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Euro</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorpo</t>
         </is>
       </c>
       <c r="L40" s="6" t="inlineStr"/>
@@ -4998,11 +4998,7 @@
           <t>PYME Y PERSONAS FÍSICAS QUE DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES213 - Bizkaia</t>
         </is>
       </c>
-      <c r="L77" s="15" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
+      <c r="L77" s="6" t="inlineStr"/>
       <c r="M77" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
@@ -5120,11 +5116,7 @@
           <t>PYME Y PERSONAS FÍSICAS QUE DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES213 - Bizkaia</t>
         </is>
       </c>
-      <c r="L79" s="15" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
+      <c r="L79" s="6" t="inlineStr"/>
       <c r="M79" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
@@ -5183,11 +5175,7 @@
           <t>PERSONAS JURÍDICAS QUE NO DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES213 - Bizkaia</t>
         </is>
       </c>
-      <c r="L80" s="15" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
+      <c r="L80" s="6" t="inlineStr"/>
       <c r="M80" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
@@ -5246,11 +5234,7 @@
           <t>PYME Y PERSONAS FÍSICAS QUE DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES213 - Bizkaia</t>
         </is>
       </c>
-      <c r="L81" s="15" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
+      <c r="L81" s="6" t="inlineStr"/>
       <c r="M81" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
@@ -5317,26 +5301,26 @@
       </c>
     </row>
     <row r="83" ht="28" customHeight="1">
-      <c r="A83" s="16" t="inlineStr">
+      <c r="A83" s="15" t="inlineStr">
         <is>
           <t>🟢 Euskadi</t>
         </is>
       </c>
     </row>
     <row r="84" ht="40" customHeight="1">
-      <c r="A84" s="17" t="inlineStr">
+      <c r="A84" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>EUS-89440</t>
+          <t>EUS-19519</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
+          <t>Actualización  de servidores,  SAI y aislamiento acústico. Dravok. Escuela Ingeniería Bilbao.</t>
         </is>
       </c>
       <c r="D84" s="6" t="inlineStr">
@@ -5353,12 +5337,12 @@
       <c r="G84" s="6" t="inlineStr"/>
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
-        </is>
-      </c>
-      <c r="I84" s="8" t="inlineStr">
-        <is>
-          <t>ALTA</t>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I84" s="12" t="inlineStr">
+        <is>
+          <t>MUY ALTA</t>
         </is>
       </c>
       <c r="J84" s="6" t="inlineStr"/>
@@ -5367,7 +5351,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L84" s="15" t="inlineStr">
+      <c r="L84" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -5379,19 +5363,19 @@
       </c>
     </row>
     <row r="85" ht="40" customHeight="1">
-      <c r="A85" s="17" t="inlineStr">
+      <c r="A85" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>EUS-95275</t>
+          <t>EUS-37183</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversidad, participación, principios de la UE. Eventos, difusiones e intercambios. Programa de Ciudadanos, Igualdad, Derechos y Valores de la UE (</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
         </is>
       </c>
       <c r="D85" s="6" t="inlineStr">
@@ -5411,9 +5395,9 @@
           <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
-      <c r="I85" s="10" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
+      <c r="I85" s="8" t="inlineStr">
+        <is>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="J85" s="6" t="inlineStr"/>
@@ -5422,7 +5406,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L85" s="15" t="inlineStr">
+      <c r="L85" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -5434,19 +5418,19 @@
       </c>
     </row>
     <row r="86" ht="40" customHeight="1">
-      <c r="A86" s="17" t="inlineStr">
+      <c r="A86" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>EUS-02578</t>
+          <t>EUS-57324</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el marco de la Intervención Sectorial Vitivinícola del Plan Estratégico (PEPAC) de la Política Agrícola Común de la UE 2023-2027</t>
+          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversidad, participación, principios de la UE. Eventos, difusiones e intercambios. Programa de Ciudadanos, Igualdad, Derechos y Valores de la UE (</t>
         </is>
       </c>
       <c r="D86" s="6" t="inlineStr">
@@ -5477,7 +5461,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L86" s="15" t="inlineStr">
+      <c r="L86" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -5489,19 +5473,19 @@
       </c>
     </row>
     <row r="87" ht="40" customHeight="1">
-      <c r="A87" s="17" t="inlineStr">
+      <c r="A87" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>EUS-34975</t>
+          <t>EUS-46961</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
+          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el marco de la Intervención Sectorial Vitivinícola del Plan Estratégico (PEPAC) de la Política Agrícola Común de la UE 2023-2027</t>
         </is>
       </c>
       <c r="D87" s="6" t="inlineStr">
@@ -5532,7 +5516,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L87" s="15" t="inlineStr">
+      <c r="L87" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -5544,19 +5528,19 @@
       </c>
     </row>
     <row r="88" ht="40" customHeight="1">
-      <c r="A88" s="17" t="inlineStr">
+      <c r="A88" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>EUS-76587</t>
+          <t>EUS-97678</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>Reparacion averia por fallo electrico en imfpbe</t>
+          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
         </is>
       </c>
       <c r="D88" s="6" t="inlineStr">
@@ -5573,7 +5557,7 @@
       <c r="G88" s="6" t="inlineStr"/>
       <c r="H88" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="I88" s="10" t="inlineStr">
@@ -5587,7 +5571,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L88" s="15" t="inlineStr">
+      <c r="L88" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -5599,19 +5583,19 @@
       </c>
     </row>
     <row r="89" ht="40" customHeight="1">
-      <c r="A89" s="17" t="inlineStr">
+      <c r="A89" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>EUS-98771</t>
+          <t>EUS-08237</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>Transporte de las personas participantes en la campaña de verano Udalekuak 2026</t>
+          <t>PTO. Limpieza pintadas</t>
         </is>
       </c>
       <c r="D89" s="6" t="inlineStr">
@@ -5642,7 +5626,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L89" s="15" t="inlineStr">
+      <c r="L89" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -5654,19 +5638,19 @@
       </c>
     </row>
     <row r="90" ht="40" customHeight="1">
-      <c r="A90" s="17" t="inlineStr">
+      <c r="A90" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>EUS-50550</t>
+          <t>EUS-22282</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>Auditoría de las instalaciones existentes en los edificios que conforman el Campo de Golf de Bizkaia - Meaztegi Golf.</t>
+          <t>Garbiketa eta higienerako produktuak/Productos de limpieza y aseo</t>
         </is>
       </c>
       <c r="D90" s="6" t="inlineStr">
@@ -5697,7 +5681,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L90" s="15" t="inlineStr">
+      <c r="L90" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -5709,19 +5693,19 @@
       </c>
     </row>
     <row r="91" ht="40" customHeight="1">
-      <c r="A91" s="17" t="inlineStr">
+      <c r="A91" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>EUS-83048</t>
+          <t>EUS-52631</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>Contrato de servicio de limpieza y desbroce de caminos públicos de Artea</t>
+          <t>Transporte de las personas participantes en la campaña de verano Udalekuak 2026</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr">
@@ -5752,7 +5736,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L91" s="15" t="inlineStr">
+      <c r="L91" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -5763,8 +5747,118 @@
         </is>
       </c>
     </row>
+    <row r="92" ht="40" customHeight="1">
+      <c r="A92" s="16" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B92" s="6" t="inlineStr">
+        <is>
+          <t>EUS-08085</t>
+        </is>
+      </c>
+      <c r="C92" s="6" t="inlineStr">
+        <is>
+          <t>Fusionado de fibra óptica para conectar la casa club con la caseta de préstamo de bicicletas eléctricas del Meaztegi Golf (Bizkaia).</t>
+        </is>
+      </c>
+      <c r="D92" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E92" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F92" s="6" t="inlineStr"/>
+      <c r="G92" s="6" t="inlineStr"/>
+      <c r="H92" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I92" s="10" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J92" s="6" t="inlineStr"/>
+      <c r="K92" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L92" s="17" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M92" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="40" customHeight="1">
+      <c r="A93" s="16" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B93" s="6" t="inlineStr">
+        <is>
+          <t>EUS-17254</t>
+        </is>
+      </c>
+      <c r="C93" s="6" t="inlineStr">
+        <is>
+          <t>Material de albañilería para el módulo de mantenimiento de viviendas del imfpb de azitain.</t>
+        </is>
+      </c>
+      <c r="D93" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E93" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F93" s="6" t="inlineStr"/>
+      <c r="G93" s="6" t="inlineStr"/>
+      <c r="H93" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I93" s="10" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J93" s="6" t="inlineStr"/>
+      <c r="K93" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L93" s="17" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M93" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:M91"/>
+  <autoFilter ref="A4:M93"/>
   <mergeCells count="5">
     <mergeCell ref="A76:M76"/>
     <mergeCell ref="A1:M1"/>
@@ -5857,6 +5951,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M89" r:id="rId82"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M90" r:id="rId83"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M91" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M92" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M93" r:id="rId86"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5868,7 +5964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1259"/>
+  <dimension ref="A1:F1289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -11954,7 +12050,7 @@
     <row r="421" ht="30" customHeight="1">
       <c r="A421" s="18" t="inlineStr">
         <is>
-          <t>FICHA 29: HORIZON-CL5-2027-01-D1-08</t>
+          <t>FICHA 29: HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="B421" s="19" t="n"/>
@@ -11979,7 +12075,7 @@
       <c r="E422" s="22" t="n"/>
       <c r="F422" s="22" t="n"/>
     </row>
-    <row r="423" ht="20" customHeight="1">
+    <row r="423" ht="45" customHeight="1">
       <c r="A423" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -11987,7 +12083,7 @@
       </c>
       <c r="B423" s="21" t="inlineStr">
         <is>
-          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
+          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
         </is>
       </c>
       <c r="C423" s="22" t="n"/>
@@ -12003,7 +12099,7 @@
       </c>
       <c r="B424" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-08</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C424" s="22" t="n"/>
@@ -12115,7 +12211,7 @@
       </c>
       <c r="B431" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and interactions with ecosystems, leading to improved Earth system models;Future climate change scenarios produced in light of past changes in the Earth system, in particular warm climates/high sea-level situations, and abrupt transitions;Identification of thresholds in Earth system components and better characterisation of driving mechanisms and feedbacks that may be responsible for non-linear behaviours,</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Europe and globally, as well as the interaction between different hazards, their cumulative and/or cascading effects.Enhanced seamless prediction and projection modelling and attribution capabilities for extreme events and their likelihood to support preparedness, response and resilience to climate change by EU and national and regional actors. The EU Union Preparedness Strategy, the EU Adaptation Str</t>
         </is>
       </c>
       <c r="C431" s="22" t="n"/>
@@ -12159,7 +12255,7 @@
       </c>
       <c r="B434" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-08</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C434" s="22" t="n"/>
@@ -12602,7 +12698,7 @@
     <row r="466" ht="30" customHeight="1">
       <c r="A466" s="18" t="inlineStr">
         <is>
-          <t>FICHA 32: HORIZON-CL5-2027-01-D1-11</t>
+          <t>FICHA 32: HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="B466" s="19" t="n"/>
@@ -12627,7 +12723,7 @@
       <c r="E467" s="22" t="n"/>
       <c r="F467" s="22" t="n"/>
     </row>
-    <row r="468" ht="20" customHeight="1">
+    <row r="468" ht="45" customHeight="1">
       <c r="A468" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -12635,7 +12731,7 @@
       </c>
       <c r="B468" s="21" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
         </is>
       </c>
       <c r="C468" s="22" t="n"/>
@@ -12651,7 +12747,7 @@
       </c>
       <c r="B469" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C469" s="22" t="n"/>
@@ -12731,7 +12827,7 @@
       </c>
       <c r="B474" s="21" t="inlineStr">
         <is>
-          <t>Programme Cofund Actions</t>
+          <t xml:space="preserve"> Research and Innovation Actions</t>
         </is>
       </c>
       <c r="C474" s="22" t="n"/>
@@ -12763,7 +12859,7 @@
       </c>
       <c r="B476" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is established through development and implementation of the Climate Action pillar of the EU-AU Research and Innovation Partnership on Climate Change and Sustainable Energy (CCSE),[1] in co-design between African and European partners;Reduced fragmentation by aligning the EU, national and multilateral R&amp;amp;I efforts with increased leverage and impact of funding;African scientific, policy and practice com</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to inform mitigation action and policy improvements, ensuring a fair transition and social acceptability;Methodologies are developed and improved for ex-ante assessment and ex-post evaluation of greenhouse gas emission reductions from climate policies and measures;Strengthened collaboration and established networks between researchers, policy experts and government officials involved in designing and eva</t>
         </is>
       </c>
       <c r="C476" s="22" t="n"/>
@@ -12807,7 +12903,7 @@
       </c>
       <c r="B479" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-11</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C479" s="22" t="n"/>
@@ -12818,7 +12914,7 @@
     <row r="481" ht="30" customHeight="1">
       <c r="A481" s="18" t="inlineStr">
         <is>
-          <t>FICHA 33: HORIZON-CL5-2027-01-D1-10</t>
+          <t>FICHA 33: HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="B481" s="19" t="n"/>
@@ -12851,7 +12947,7 @@
       </c>
       <c r="B483" s="21" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
         </is>
       </c>
       <c r="C483" s="22" t="n"/>
@@ -12867,7 +12963,7 @@
       </c>
       <c r="B484" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="C484" s="22" t="n"/>
@@ -12979,7 +13075,7 @@
       </c>
       <c r="B491" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorporation into main EU repositories, such as Climate-ADAPT or the portal of the EU Mission on Adaptation to Climate Change;The risk and adaptation assessment frameworks are improved by better integrating the maladaptation dimension;Guidelines and tools for maladaptation prevention and correction strategies are made available to adaptation stakeholders at relevant scales and inform the design and impl</t>
+          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and interactions with ecosystems, leading to improved Earth system models;Future climate change scenarios produced in light of past changes in the Earth system, in particular warm climates/high sea-level situations, and abrupt transitions;Identification of thresholds in Earth system components and better characterisation of driving mechanisms and feedbacks that may be responsible for non-linear behaviours,</t>
         </is>
       </c>
       <c r="C491" s="22" t="n"/>
@@ -13023,7 +13119,7 @@
       </c>
       <c r="B494" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-10</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="C494" s="22" t="n"/>
@@ -13034,7 +13130,7 @@
     <row r="496" ht="30" customHeight="1">
       <c r="A496" s="18" t="inlineStr">
         <is>
-          <t>FICHA 34: HORIZON-CL5-2027-01-D1-09</t>
+          <t>FICHA 34: HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="B496" s="19" t="n"/>
@@ -13059,7 +13155,7 @@
       <c r="E497" s="22" t="n"/>
       <c r="F497" s="22" t="n"/>
     </row>
-    <row r="498" ht="45" customHeight="1">
+    <row r="498" ht="20" customHeight="1">
       <c r="A498" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -13067,7 +13163,7 @@
       </c>
       <c r="B498" s="21" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="C498" s="22" t="n"/>
@@ -13083,7 +13179,7 @@
       </c>
       <c r="B499" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C499" s="22" t="n"/>
@@ -13163,7 +13259,7 @@
       </c>
       <c r="B504" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Research and Innovation Actions</t>
+          <t>Programme Cofund Actions</t>
         </is>
       </c>
       <c r="C504" s="22" t="n"/>
@@ -13195,7 +13291,7 @@
       </c>
       <c r="B506" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to inform mitigation action and policy improvements, ensuring a fair transition and social acceptability;Methodologies are developed and improved for ex-ante assessment and ex-post evaluation of greenhouse gas emission reductions from climate policies and measures;Strengthened collaboration and established networks between researchers, policy experts and government officials involved in designing and eva</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is established through development and implementation of the Climate Action pillar of the EU-AU Research and Innovation Partnership on Climate Change and Sustainable Energy (CCSE),[1] in co-design between African and European partners;Reduced fragmentation by aligning the EU, national and multilateral R&amp;amp;I efforts with increased leverage and impact of funding;African scientific, policy and practice com</t>
         </is>
       </c>
       <c r="C506" s="22" t="n"/>
@@ -13239,7 +13335,7 @@
       </c>
       <c r="B509" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-09</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C509" s="22" t="n"/>
@@ -13250,7 +13346,7 @@
     <row r="511" ht="30" customHeight="1">
       <c r="A511" s="18" t="inlineStr">
         <is>
-          <t>FICHA 35: HORIZON-CL5-2027-01-D1-07</t>
+          <t>FICHA 35: HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="B511" s="19" t="n"/>
@@ -13275,7 +13371,7 @@
       <c r="E512" s="22" t="n"/>
       <c r="F512" s="22" t="n"/>
     </row>
-    <row r="513" ht="45" customHeight="1">
+    <row r="513" ht="20" customHeight="1">
       <c r="A513" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -13283,7 +13379,7 @@
       </c>
       <c r="B513" s="21" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="C513" s="22" t="n"/>
@@ -13299,7 +13395,7 @@
       </c>
       <c r="B514" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C514" s="22" t="n"/>
@@ -13411,7 +13507,7 @@
       </c>
       <c r="B521" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Europe and globally, as well as the interaction between different hazards, their cumulative and/or cascading effects.Enhanced seamless prediction and projection modelling and attribution capabilities for extreme events and their likelihood to support preparedness, response and resilience to climate change by EU and national and regional actors. The EU Union Preparedness Strategy, the EU Adaptation Str</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorporation into main EU repositories, such as Climate-ADAPT or the portal of the EU Mission on Adaptation to Climate Change;The risk and adaptation assessment frameworks are improved by better integrating the maladaptation dimension;Guidelines and tools for maladaptation prevention and correction strategies are made available to adaptation stakeholders at relevant scales and inform the design and impl</t>
         </is>
       </c>
       <c r="C521" s="22" t="n"/>
@@ -13455,7 +13551,7 @@
       </c>
       <c r="B524" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-07</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C524" s="22" t="n"/>
@@ -22266,7 +22362,7 @@
     <row r="1141" ht="30" customHeight="1">
       <c r="A1141" s="18" t="inlineStr">
         <is>
-          <t>FICHA 77: EUS-89440</t>
+          <t>FICHA 77: EUS-19519</t>
         </is>
       </c>
       <c r="B1141" s="19" t="n"/>
@@ -22299,7 +22395,7 @@
       </c>
       <c r="B1143" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
+          <t>Actualización  de servidores,  SAI y aislamiento acústico. Dravok. Escuela Ingeniería Bilbao.</t>
         </is>
       </c>
       <c r="C1143" s="22" t="n"/>
@@ -22315,7 +22411,7 @@
       </c>
       <c r="B1144" s="21" t="inlineStr">
         <is>
-          <t>EUS-89440</t>
+          <t>EUS-19519</t>
         </is>
       </c>
       <c r="C1144" s="22" t="n"/>
@@ -22391,7 +22487,7 @@
       </c>
       <c r="B1149" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C1149" s="22" t="n"/>
@@ -22449,9 +22545,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B1153" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ALTA — </t>
+      <c r="B1153" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MUY ALTA — </t>
         </is>
       </c>
       <c r="C1153" s="22" t="n"/>
@@ -22467,7 +22563,7 @@
       </c>
       <c r="B1154" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-con-incremento-de-capacidad-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/actualizacion-servidores-sai-y-aislamiento-acustico-dravok-escuela-ingenieria-bilbao/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1154" s="22" t="n"/>
@@ -22478,7 +22574,7 @@
     <row r="1156" ht="30" customHeight="1">
       <c r="A1156" s="18" t="inlineStr">
         <is>
-          <t>FICHA 78: EUS-95275</t>
+          <t>FICHA 78: EUS-37183</t>
         </is>
       </c>
       <c r="B1156" s="19" t="n"/>
@@ -22511,7 +22607,7 @@
       </c>
       <c r="B1158" s="21" t="inlineStr">
         <is>
-          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversidad, participación, principios de la UE. Eventos, difusiones e intercambios. Programa de Ciudadanos, Igualdad, Derechos y Valores de la UE (</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
         </is>
       </c>
       <c r="C1158" s="22" t="n"/>
@@ -22527,7 +22623,7 @@
       </c>
       <c r="B1159" s="21" t="inlineStr">
         <is>
-          <t>EUS-95275</t>
+          <t>EUS-37183</t>
         </is>
       </c>
       <c r="C1159" s="22" t="n"/>
@@ -22661,9 +22757,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B1168" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
+      <c r="B1168" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALTA — </t>
         </is>
       </c>
       <c r="C1168" s="22" t="n"/>
@@ -22679,7 +22775,7 @@
       </c>
       <c r="B1169" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260408cervhirisareak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-con-incremento-de-capacidad-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1169" s="22" t="n"/>
@@ -22690,7 +22786,7 @@
     <row r="1171" ht="30" customHeight="1">
       <c r="A1171" s="18" t="inlineStr">
         <is>
-          <t>FICHA 79: EUS-02578</t>
+          <t>FICHA 79: EUS-57324</t>
         </is>
       </c>
       <c r="B1171" s="19" t="n"/>
@@ -22723,7 +22819,7 @@
       </c>
       <c r="B1173" s="21" t="inlineStr">
         <is>
-          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el marco de la Intervención Sectorial Vitivinícola del Plan Estratégico (PEPAC) de la Política Agrícola Común de la UE 2023-2027</t>
+          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversidad, participación, principios de la UE. Eventos, difusiones e intercambios. Programa de Ciudadanos, Igualdad, Derechos y Valores de la UE (</t>
         </is>
       </c>
       <c r="C1173" s="22" t="n"/>
@@ -22739,7 +22835,7 @@
       </c>
       <c r="B1174" s="21" t="inlineStr">
         <is>
-          <t>EUS-02578</t>
+          <t>EUS-57324</t>
         </is>
       </c>
       <c r="C1174" s="22" t="n"/>
@@ -22891,7 +22987,7 @@
       </c>
       <c r="B1184" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/20260407mahastiardogintza/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260408cervhirisareak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1184" s="22" t="n"/>
@@ -22902,7 +22998,7 @@
     <row r="1186" ht="30" customHeight="1">
       <c r="A1186" s="18" t="inlineStr">
         <is>
-          <t>FICHA 80: EUS-34975</t>
+          <t>FICHA 80: EUS-46961</t>
         </is>
       </c>
       <c r="B1186" s="19" t="n"/>
@@ -22935,7 +23031,7 @@
       </c>
       <c r="B1188" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
+          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el marco de la Intervención Sectorial Vitivinícola del Plan Estratégico (PEPAC) de la Política Agrícola Común de la UE 2023-2027</t>
         </is>
       </c>
       <c r="C1188" s="22" t="n"/>
@@ -22951,7 +23047,7 @@
       </c>
       <c r="B1189" s="21" t="inlineStr">
         <is>
-          <t>EUS-34975</t>
+          <t>EUS-46961</t>
         </is>
       </c>
       <c r="C1189" s="22" t="n"/>
@@ -23103,7 +23199,7 @@
       </c>
       <c r="B1199" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-contribucion-de-la-acuicultura-al-buen-estado-ambiental-y-prestacion-de-servicios-ambientales-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/20260407mahastiardogintza/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1199" s="22" t="n"/>
@@ -23114,7 +23210,7 @@
     <row r="1201" ht="30" customHeight="1">
       <c r="A1201" s="18" t="inlineStr">
         <is>
-          <t>FICHA 81: EUS-76587</t>
+          <t>FICHA 81: EUS-97678</t>
         </is>
       </c>
       <c r="B1201" s="19" t="n"/>
@@ -23139,7 +23235,7 @@
       <c r="E1202" s="22" t="n"/>
       <c r="F1202" s="22" t="n"/>
     </row>
-    <row r="1203" ht="20" customHeight="1">
+    <row r="1203" ht="45" customHeight="1">
       <c r="A1203" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -23147,7 +23243,7 @@
       </c>
       <c r="B1203" s="21" t="inlineStr">
         <is>
-          <t>Reparacion averia por fallo electrico en imfpbe</t>
+          <t>Ayudas a la contribución de la acuicultura al buen estado ambiental y prestación de servicios ambientales 2026</t>
         </is>
       </c>
       <c r="C1203" s="22" t="n"/>
@@ -23163,7 +23259,7 @@
       </c>
       <c r="B1204" s="21" t="inlineStr">
         <is>
-          <t>EUS-76587</t>
+          <t>EUS-97678</t>
         </is>
       </c>
       <c r="C1204" s="22" t="n"/>
@@ -23239,7 +23335,7 @@
       </c>
       <c r="B1209" s="21" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C1209" s="22" t="n"/>
@@ -23315,7 +23411,7 @@
       </c>
       <c r="B1214" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/reparacion-averia-fallo-electrico-imfpbe/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-contribucion-de-la-acuicultura-al-buen-estado-ambiental-y-prestacion-de-servicios-ambientales-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1214" s="22" t="n"/>
@@ -23326,7 +23422,7 @@
     <row r="1216" ht="30" customHeight="1">
       <c r="A1216" s="18" t="inlineStr">
         <is>
-          <t>FICHA 82: EUS-98771</t>
+          <t>FICHA 82: EUS-08237</t>
         </is>
       </c>
       <c r="B1216" s="19" t="n"/>
@@ -23359,7 +23455,7 @@
       </c>
       <c r="B1218" s="21" t="inlineStr">
         <is>
-          <t>Transporte de las personas participantes en la campaña de verano Udalekuak 2026</t>
+          <t>PTO. Limpieza pintadas</t>
         </is>
       </c>
       <c r="C1218" s="22" t="n"/>
@@ -23375,7 +23471,7 @@
       </c>
       <c r="B1219" s="21" t="inlineStr">
         <is>
-          <t>EUS-98771</t>
+          <t>EUS-08237</t>
         </is>
       </c>
       <c r="C1219" s="22" t="n"/>
@@ -23527,7 +23623,7 @@
       </c>
       <c r="B1229" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/transporte-personas-participantes-campana-verano-udalekuak-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/pto-limpieza-pintadas/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1229" s="22" t="n"/>
@@ -23538,7 +23634,7 @@
     <row r="1231" ht="30" customHeight="1">
       <c r="A1231" s="18" t="inlineStr">
         <is>
-          <t>FICHA 83: EUS-50550</t>
+          <t>FICHA 83: EUS-22282</t>
         </is>
       </c>
       <c r="B1231" s="19" t="n"/>
@@ -23563,7 +23659,7 @@
       <c r="E1232" s="22" t="n"/>
       <c r="F1232" s="22" t="n"/>
     </row>
-    <row r="1233" ht="45" customHeight="1">
+    <row r="1233" ht="20" customHeight="1">
       <c r="A1233" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -23571,7 +23667,7 @@
       </c>
       <c r="B1233" s="21" t="inlineStr">
         <is>
-          <t>Auditoría de las instalaciones existentes en los edificios que conforman el Campo de Golf de Bizkaia - Meaztegi Golf.</t>
+          <t>Garbiketa eta higienerako produktuak/Productos de limpieza y aseo</t>
         </is>
       </c>
       <c r="C1233" s="22" t="n"/>
@@ -23587,7 +23683,7 @@
       </c>
       <c r="B1234" s="21" t="inlineStr">
         <is>
-          <t>EUS-50550</t>
+          <t>EUS-22282</t>
         </is>
       </c>
       <c r="C1234" s="22" t="n"/>
@@ -23739,7 +23835,7 @@
       </c>
       <c r="B1244" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/auditoria-instalaciones-existentes-edificios-que-conforman-campo-golf-bizkaia-meaztegi-golf/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/garbiketa-eta-higienerako-produktuak-productos-limpieza-y-aseo/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1244" s="22" t="n"/>
@@ -23750,7 +23846,7 @@
     <row r="1246" ht="30" customHeight="1">
       <c r="A1246" s="18" t="inlineStr">
         <is>
-          <t>FICHA 84: EUS-83048</t>
+          <t>FICHA 84: EUS-52631</t>
         </is>
       </c>
       <c r="B1246" s="19" t="n"/>
@@ -23783,7 +23879,7 @@
       </c>
       <c r="B1248" s="21" t="inlineStr">
         <is>
-          <t>Contrato de servicio de limpieza y desbroce de caminos públicos de Artea</t>
+          <t>Transporte de las personas participantes en la campaña de verano Udalekuak 2026</t>
         </is>
       </c>
       <c r="C1248" s="22" t="n"/>
@@ -23799,7 +23895,7 @@
       </c>
       <c r="B1249" s="21" t="inlineStr">
         <is>
-          <t>EUS-83048</t>
+          <t>EUS-52631</t>
         </is>
       </c>
       <c r="C1249" s="22" t="n"/>
@@ -23951,7 +24047,7 @@
       </c>
       <c r="B1259" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/contrato-servicio-limpieza-y-desbroce-caminos-publicos-artea/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/transporte-personas-participantes-campana-verano-udalekuak-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1259" s="22" t="n"/>
@@ -23959,8 +24055,432 @@
       <c r="E1259" s="22" t="n"/>
       <c r="F1259" s="22" t="n"/>
     </row>
+    <row r="1261" ht="30" customHeight="1">
+      <c r="A1261" s="18" t="inlineStr">
+        <is>
+          <t>FICHA 85: EUS-08085</t>
+        </is>
+      </c>
+      <c r="B1261" s="19" t="n"/>
+      <c r="C1261" s="19" t="n"/>
+      <c r="D1261" s="19" t="n"/>
+      <c r="E1261" s="19" t="n"/>
+      <c r="F1261" s="19" t="n"/>
+    </row>
+    <row r="1262" ht="20" customHeight="1">
+      <c r="A1262" s="20" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1262" s="21" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1262" s="22" t="n"/>
+      <c r="D1262" s="22" t="n"/>
+      <c r="E1262" s="22" t="n"/>
+      <c r="F1262" s="22" t="n"/>
+    </row>
+    <row r="1263" ht="45" customHeight="1">
+      <c r="A1263" s="20" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1263" s="21" t="inlineStr">
+        <is>
+          <t>Fusionado de fibra óptica para conectar la casa club con la caseta de préstamo de bicicletas eléctricas del Meaztegi Golf (Bizkaia).</t>
+        </is>
+      </c>
+      <c r="C1263" s="22" t="n"/>
+      <c r="D1263" s="22" t="n"/>
+      <c r="E1263" s="22" t="n"/>
+      <c r="F1263" s="22" t="n"/>
+    </row>
+    <row r="1264" ht="20" customHeight="1">
+      <c r="A1264" s="20" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1264" s="21" t="inlineStr">
+        <is>
+          <t>EUS-08085</t>
+        </is>
+      </c>
+      <c r="C1264" s="22" t="n"/>
+      <c r="D1264" s="22" t="n"/>
+      <c r="E1264" s="22" t="n"/>
+      <c r="F1264" s="22" t="n"/>
+    </row>
+    <row r="1265" ht="20" customHeight="1">
+      <c r="A1265" s="20" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1265" s="21" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1265" s="22" t="n"/>
+      <c r="D1265" s="22" t="n"/>
+      <c r="E1265" s="22" t="n"/>
+      <c r="F1265" s="22" t="n"/>
+    </row>
+    <row r="1266" ht="20" customHeight="1">
+      <c r="A1266" s="20" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1266" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1266" s="22" t="n"/>
+      <c r="D1266" s="22" t="n"/>
+      <c r="E1266" s="22" t="n"/>
+      <c r="F1266" s="22" t="n"/>
+    </row>
+    <row r="1267" ht="20" customHeight="1">
+      <c r="A1267" s="20" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1267" s="21" t="inlineStr"/>
+      <c r="C1267" s="22" t="n"/>
+      <c r="D1267" s="22" t="n"/>
+      <c r="E1267" s="22" t="n"/>
+      <c r="F1267" s="22" t="n"/>
+    </row>
+    <row r="1268" ht="20" customHeight="1">
+      <c r="A1268" s="20" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1268" s="21" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1268" s="22" t="n"/>
+      <c r="D1268" s="22" t="n"/>
+      <c r="E1268" s="22" t="n"/>
+      <c r="F1268" s="22" t="n"/>
+    </row>
+    <row r="1269" ht="20" customHeight="1">
+      <c r="A1269" s="20" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1269" s="21" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1269" s="22" t="n"/>
+      <c r="D1269" s="22" t="n"/>
+      <c r="E1269" s="22" t="n"/>
+      <c r="F1269" s="22" t="n"/>
+    </row>
+    <row r="1270" ht="20" customHeight="1">
+      <c r="A1270" s="20" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1270" s="21" t="inlineStr"/>
+      <c r="C1270" s="22" t="n"/>
+      <c r="D1270" s="22" t="n"/>
+      <c r="E1270" s="22" t="n"/>
+      <c r="F1270" s="22" t="n"/>
+    </row>
+    <row r="1271" ht="20" customHeight="1">
+      <c r="A1271" s="20" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1271" s="21" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1271" s="22" t="n"/>
+      <c r="D1271" s="22" t="n"/>
+      <c r="E1271" s="22" t="n"/>
+      <c r="F1271" s="22" t="n"/>
+    </row>
+    <row r="1272" ht="20" customHeight="1">
+      <c r="A1272" s="20" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1272" s="21" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1272" s="22" t="n"/>
+      <c r="D1272" s="22" t="n"/>
+      <c r="E1272" s="22" t="n"/>
+      <c r="F1272" s="22" t="n"/>
+    </row>
+    <row r="1273" ht="20" customHeight="1">
+      <c r="A1273" s="20" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1273" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1273" s="22" t="n"/>
+      <c r="D1273" s="22" t="n"/>
+      <c r="E1273" s="22" t="n"/>
+      <c r="F1273" s="22" t="n"/>
+    </row>
+    <row r="1274" ht="45" customHeight="1">
+      <c r="A1274" s="20" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1274" s="24" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/fusionado-fibra-optica-conectar-casa-club-caseta-prestamo-bicicletas-electricas-del-meaztegi-golf-bizkaia/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1274" s="22" t="n"/>
+      <c r="D1274" s="22" t="n"/>
+      <c r="E1274" s="22" t="n"/>
+      <c r="F1274" s="22" t="n"/>
+    </row>
+    <row r="1276" ht="30" customHeight="1">
+      <c r="A1276" s="18" t="inlineStr">
+        <is>
+          <t>FICHA 86: EUS-17254</t>
+        </is>
+      </c>
+      <c r="B1276" s="19" t="n"/>
+      <c r="C1276" s="19" t="n"/>
+      <c r="D1276" s="19" t="n"/>
+      <c r="E1276" s="19" t="n"/>
+      <c r="F1276" s="19" t="n"/>
+    </row>
+    <row r="1277" ht="20" customHeight="1">
+      <c r="A1277" s="20" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1277" s="21" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1277" s="22" t="n"/>
+      <c r="D1277" s="22" t="n"/>
+      <c r="E1277" s="22" t="n"/>
+      <c r="F1277" s="22" t="n"/>
+    </row>
+    <row r="1278" ht="45" customHeight="1">
+      <c r="A1278" s="20" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1278" s="21" t="inlineStr">
+        <is>
+          <t>Material de albañilería para el módulo de mantenimiento de viviendas del imfpb de azitain.</t>
+        </is>
+      </c>
+      <c r="C1278" s="22" t="n"/>
+      <c r="D1278" s="22" t="n"/>
+      <c r="E1278" s="22" t="n"/>
+      <c r="F1278" s="22" t="n"/>
+    </row>
+    <row r="1279" ht="20" customHeight="1">
+      <c r="A1279" s="20" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1279" s="21" t="inlineStr">
+        <is>
+          <t>EUS-17254</t>
+        </is>
+      </c>
+      <c r="C1279" s="22" t="n"/>
+      <c r="D1279" s="22" t="n"/>
+      <c r="E1279" s="22" t="n"/>
+      <c r="F1279" s="22" t="n"/>
+    </row>
+    <row r="1280" ht="20" customHeight="1">
+      <c r="A1280" s="20" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1280" s="21" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1280" s="22" t="n"/>
+      <c r="D1280" s="22" t="n"/>
+      <c r="E1280" s="22" t="n"/>
+      <c r="F1280" s="22" t="n"/>
+    </row>
+    <row r="1281" ht="20" customHeight="1">
+      <c r="A1281" s="20" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1281" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1281" s="22" t="n"/>
+      <c r="D1281" s="22" t="n"/>
+      <c r="E1281" s="22" t="n"/>
+      <c r="F1281" s="22" t="n"/>
+    </row>
+    <row r="1282" ht="20" customHeight="1">
+      <c r="A1282" s="20" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1282" s="21" t="inlineStr"/>
+      <c r="C1282" s="22" t="n"/>
+      <c r="D1282" s="22" t="n"/>
+      <c r="E1282" s="22" t="n"/>
+      <c r="F1282" s="22" t="n"/>
+    </row>
+    <row r="1283" ht="20" customHeight="1">
+      <c r="A1283" s="20" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1283" s="21" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1283" s="22" t="n"/>
+      <c r="D1283" s="22" t="n"/>
+      <c r="E1283" s="22" t="n"/>
+      <c r="F1283" s="22" t="n"/>
+    </row>
+    <row r="1284" ht="20" customHeight="1">
+      <c r="A1284" s="20" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1284" s="21" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1284" s="22" t="n"/>
+      <c r="D1284" s="22" t="n"/>
+      <c r="E1284" s="22" t="n"/>
+      <c r="F1284" s="22" t="n"/>
+    </row>
+    <row r="1285" ht="20" customHeight="1">
+      <c r="A1285" s="20" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1285" s="21" t="inlineStr"/>
+      <c r="C1285" s="22" t="n"/>
+      <c r="D1285" s="22" t="n"/>
+      <c r="E1285" s="22" t="n"/>
+      <c r="F1285" s="22" t="n"/>
+    </row>
+    <row r="1286" ht="20" customHeight="1">
+      <c r="A1286" s="20" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1286" s="21" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1286" s="22" t="n"/>
+      <c r="D1286" s="22" t="n"/>
+      <c r="E1286" s="22" t="n"/>
+      <c r="F1286" s="22" t="n"/>
+    </row>
+    <row r="1287" ht="20" customHeight="1">
+      <c r="A1287" s="20" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1287" s="21" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1287" s="22" t="n"/>
+      <c r="D1287" s="22" t="n"/>
+      <c r="E1287" s="22" t="n"/>
+      <c r="F1287" s="22" t="n"/>
+    </row>
+    <row r="1288" ht="20" customHeight="1">
+      <c r="A1288" s="20" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1288" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1288" s="22" t="n"/>
+      <c r="D1288" s="22" t="n"/>
+      <c r="E1288" s="22" t="n"/>
+      <c r="F1288" s="22" t="n"/>
+    </row>
+    <row r="1289" ht="45" customHeight="1">
+      <c r="A1289" s="20" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1289" s="24" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/material-albanileria-modulo-mantenimiento-viviendas-del-imfpb-azitain/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1289" s="22" t="n"/>
+      <c r="D1289" s="22" t="n"/>
+      <c r="E1289" s="22" t="n"/>
+      <c r="F1289" s="22" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="1176">
+  <mergeCells count="1204">
     <mergeCell ref="B679:F679"/>
     <mergeCell ref="B666:F666"/>
     <mergeCell ref="B964:F964"/>
@@ -23981,6 +24501,7 @@
     <mergeCell ref="B512:F512"/>
     <mergeCell ref="B238:F238"/>
     <mergeCell ref="B509:F509"/>
+    <mergeCell ref="B1264:F1264"/>
     <mergeCell ref="B303:F303"/>
     <mergeCell ref="B941:F941"/>
     <mergeCell ref="B797:F797"/>
@@ -24013,6 +24534,7 @@
     <mergeCell ref="B515:F515"/>
     <mergeCell ref="B1128:F1128"/>
     <mergeCell ref="B1193:F1193"/>
+    <mergeCell ref="B1279:F1279"/>
     <mergeCell ref="A841:F841"/>
     <mergeCell ref="B158:F158"/>
     <mergeCell ref="B1094:F1094"/>
@@ -24069,6 +24591,7 @@
     <mergeCell ref="B293:F293"/>
     <mergeCell ref="B657:F657"/>
     <mergeCell ref="B322:F322"/>
+    <mergeCell ref="B1270:F1270"/>
     <mergeCell ref="B1191:F1191"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B672:F672"/>
@@ -24077,6 +24600,7 @@
     <mergeCell ref="B148:F148"/>
     <mergeCell ref="B82:F82"/>
     <mergeCell ref="B446:F446"/>
+    <mergeCell ref="B1272:F1272"/>
     <mergeCell ref="B688:F688"/>
     <mergeCell ref="B622:F622"/>
     <mergeCell ref="B682:F682"/>
@@ -24159,6 +24683,7 @@
     <mergeCell ref="B1075:F1075"/>
     <mergeCell ref="B1197:F1197"/>
     <mergeCell ref="B678:F678"/>
+    <mergeCell ref="B1262:F1262"/>
     <mergeCell ref="B363:F363"/>
     <mergeCell ref="B534:F534"/>
     <mergeCell ref="B805:F805"/>
@@ -24185,6 +24710,7 @@
     <mergeCell ref="B1052:F1052"/>
     <mergeCell ref="B981:F981"/>
     <mergeCell ref="B846:F846"/>
+    <mergeCell ref="B1288:F1288"/>
     <mergeCell ref="B973:F973"/>
     <mergeCell ref="B389:F389"/>
     <mergeCell ref="B1044:F1044"/>
@@ -24235,8 +24761,10 @@
     <mergeCell ref="B1001:F1001"/>
     <mergeCell ref="B246:F246"/>
     <mergeCell ref="B1174:F1174"/>
+    <mergeCell ref="B1268:F1268"/>
     <mergeCell ref="B40:F40"/>
     <mergeCell ref="B338:F338"/>
+    <mergeCell ref="B1286:F1286"/>
     <mergeCell ref="B469:F469"/>
     <mergeCell ref="B767:F767"/>
     <mergeCell ref="B177:F177"/>
@@ -24251,6 +24779,8 @@
     <mergeCell ref="B978:F978"/>
     <mergeCell ref="B79:F79"/>
     <mergeCell ref="B1076:F1076"/>
+    <mergeCell ref="B1283:F1283"/>
+    <mergeCell ref="B1263:F1263"/>
     <mergeCell ref="B41:F41"/>
     <mergeCell ref="B35:F35"/>
     <mergeCell ref="B302:F302"/>
@@ -24272,12 +24802,14 @@
     <mergeCell ref="A1111:F1111"/>
     <mergeCell ref="B1084:F1084"/>
     <mergeCell ref="A976:F976"/>
+    <mergeCell ref="B1266:F1266"/>
     <mergeCell ref="B170:F170"/>
     <mergeCell ref="B157:F157"/>
     <mergeCell ref="B328:F328"/>
     <mergeCell ref="B455:F455"/>
     <mergeCell ref="B626:F626"/>
     <mergeCell ref="B697:F697"/>
+    <mergeCell ref="B1281:F1281"/>
     <mergeCell ref="B491:F491"/>
     <mergeCell ref="B762:F762"/>
     <mergeCell ref="B933:F933"/>
@@ -24309,6 +24841,7 @@
     <mergeCell ref="B1162:F1162"/>
     <mergeCell ref="B1233:F1233"/>
     <mergeCell ref="B692:F692"/>
+    <mergeCell ref="B1282:F1282"/>
     <mergeCell ref="A931:F931"/>
     <mergeCell ref="B486:F486"/>
     <mergeCell ref="B757:F757"/>
@@ -24370,6 +24903,7 @@
     <mergeCell ref="B171:F171"/>
     <mergeCell ref="B1168:F1168"/>
     <mergeCell ref="B407:F407"/>
+    <mergeCell ref="B1287:F1287"/>
     <mergeCell ref="A646:F646"/>
     <mergeCell ref="B972:F972"/>
     <mergeCell ref="B1208:F1208"/>
@@ -24400,6 +24934,7 @@
     <mergeCell ref="B507:F507"/>
     <mergeCell ref="B62:F62"/>
     <mergeCell ref="B700:F700"/>
+    <mergeCell ref="B1284:F1284"/>
     <mergeCell ref="B998:F998"/>
     <mergeCell ref="B792:F792"/>
     <mergeCell ref="B596:F596"/>
@@ -24418,6 +24953,7 @@
     <mergeCell ref="B39:F39"/>
     <mergeCell ref="B1092:F1092"/>
     <mergeCell ref="B508:F508"/>
+    <mergeCell ref="B1285:F1285"/>
     <mergeCell ref="B573:F573"/>
     <mergeCell ref="A961:F961"/>
     <mergeCell ref="B858:F858"/>
@@ -24453,6 +24989,7 @@
     <mergeCell ref="B222:F222"/>
     <mergeCell ref="B344:F344"/>
     <mergeCell ref="B415:F415"/>
+    <mergeCell ref="B1265:F1265"/>
     <mergeCell ref="B713:F713"/>
     <mergeCell ref="B884:F884"/>
     <mergeCell ref="B63:F63"/>
@@ -24527,6 +25064,7 @@
     <mergeCell ref="B169:F169"/>
     <mergeCell ref="B1166:F1166"/>
     <mergeCell ref="A706:F706"/>
+    <mergeCell ref="B1278:F1278"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B129:F129"/>
     <mergeCell ref="B200:F200"/>
@@ -24587,6 +25125,7 @@
     <mergeCell ref="B289:F289"/>
     <mergeCell ref="A721:F721"/>
     <mergeCell ref="B1259:F1259"/>
+    <mergeCell ref="A1261:F1261"/>
     <mergeCell ref="A31:F31"/>
     <mergeCell ref="B747:F747"/>
     <mergeCell ref="B1152:F1152"/>
@@ -24696,6 +25235,7 @@
     <mergeCell ref="A1156:F1156"/>
     <mergeCell ref="B232:F232"/>
     <mergeCell ref="B321:F321"/>
+    <mergeCell ref="B1274:F1274"/>
     <mergeCell ref="B215:F215"/>
     <mergeCell ref="B513:F513"/>
     <mergeCell ref="B684:F684"/>
@@ -24732,6 +25272,7 @@
     <mergeCell ref="B921:F921"/>
     <mergeCell ref="B550:F550"/>
     <mergeCell ref="B606:F606"/>
+    <mergeCell ref="B1269:F1269"/>
     <mergeCell ref="B544:F544"/>
     <mergeCell ref="B848:F848"/>
     <mergeCell ref="B87:F87"/>
@@ -24741,10 +25282,12 @@
     <mergeCell ref="B1206:F1206"/>
     <mergeCell ref="B245:F245"/>
     <mergeCell ref="B687:F687"/>
+    <mergeCell ref="B1271:F1271"/>
     <mergeCell ref="B543:F543"/>
     <mergeCell ref="B814:F814"/>
     <mergeCell ref="B456:F456"/>
     <mergeCell ref="B260:F260"/>
+    <mergeCell ref="A1276:F1276"/>
     <mergeCell ref="B545:F545"/>
     <mergeCell ref="A496:F496"/>
     <mergeCell ref="B36:F36"/>
@@ -24804,6 +25347,7 @@
     <mergeCell ref="A811:F811"/>
     <mergeCell ref="B1150:F1150"/>
     <mergeCell ref="B329:F329"/>
+    <mergeCell ref="B1277:F1277"/>
     <mergeCell ref="B627:F627"/>
     <mergeCell ref="A1201:F1201"/>
     <mergeCell ref="B49:F49"/>
@@ -24852,6 +25396,7 @@
     <mergeCell ref="B261:F261"/>
     <mergeCell ref="B1087:F1087"/>
     <mergeCell ref="B1149:F1149"/>
+    <mergeCell ref="B1280:F1280"/>
     <mergeCell ref="B1214:F1214"/>
     <mergeCell ref="B184:F184"/>
     <mergeCell ref="B1062:F1062"/>
@@ -24902,6 +25447,8 @@
     <mergeCell ref="B143:F143"/>
     <mergeCell ref="B118:F118"/>
     <mergeCell ref="B1202:F1202"/>
+    <mergeCell ref="B1273:F1273"/>
+    <mergeCell ref="B1267:F1267"/>
     <mergeCell ref="B683:F683"/>
     <mergeCell ref="A751:F751"/>
     <mergeCell ref="B477:F477"/>
@@ -25020,6 +25567,7 @@
     <mergeCell ref="B920:F920"/>
     <mergeCell ref="B1108:F1108"/>
     <mergeCell ref="B711:F711"/>
+    <mergeCell ref="B1289:F1289"/>
     <mergeCell ref="B1009:F1009"/>
     <mergeCell ref="B48:F48"/>
     <mergeCell ref="B1101:F1101"/>
@@ -25223,6 +25771,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1229" r:id="rId82"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1244" r:id="rId83"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1259" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1274" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1289" r:id="rId86"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -25234,7 +25784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J85"/>
+  <dimension ref="A1:J87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -26420,12 +26970,12 @@
     <row r="30" ht="28" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-08</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Palaeoclimate science for a better understanding of Earth sy</t>
+          <t>Advancing understanding, modelling and prediction of extreme</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -26540,12 +27090,12 @@
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Assessing the performance of policy instruments to inform cl</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -26580,12 +27130,12 @@
     <row r="34" ht="28" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Palaeoclimate science for a better understanding of Earth sy</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
@@ -26620,12 +27170,12 @@
     <row r="35" ht="28" customHeight="1">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform cl</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -26660,12 +27210,12 @@
     <row r="36" ht="28" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -28232,12 +28782,12 @@
     <row r="78" ht="28" customHeight="1">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>EUS-89440</t>
+          <t>EUS-19519</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
+          <t>Actualización  de servidores,  SAI y aislamiento acústico. D</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
@@ -28253,7 +28803,7 @@
       <c r="E78" s="6" t="inlineStr"/>
       <c r="F78" s="27" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>MUY ALTA</t>
         </is>
       </c>
       <c r="G78" s="6" t="inlineStr"/>
@@ -28268,12 +28818,12 @@
     <row r="79" ht="28" customHeight="1">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>EUS-95275</t>
+          <t>EUS-37183</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversi</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
@@ -28289,7 +28839,7 @@
       <c r="E79" s="6" t="inlineStr"/>
       <c r="F79" s="27" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="G79" s="6" t="inlineStr"/>
@@ -28304,12 +28854,12 @@
     <row r="80" ht="28" customHeight="1">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>EUS-02578</t>
+          <t>EUS-57324</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el ma</t>
+          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversi</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
@@ -28340,12 +28890,12 @@
     <row r="81" ht="28" customHeight="1">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>EUS-34975</t>
+          <t>EUS-46961</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la contribución de la acuicultura al buen estado am</t>
+          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el ma</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
@@ -28376,12 +28926,12 @@
     <row r="82" ht="28" customHeight="1">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>EUS-76587</t>
+          <t>EUS-97678</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>Reparacion averia por fallo electrico en imfpbe</t>
+          <t>Ayudas a la contribución de la acuicultura al buen estado am</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
@@ -28412,12 +28962,12 @@
     <row r="83" ht="28" customHeight="1">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>EUS-98771</t>
+          <t>EUS-08237</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>Transporte de las personas participantes en la campaña de ve</t>
+          <t>PTO. Limpieza pintadas</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
@@ -28448,12 +28998,12 @@
     <row r="84" ht="28" customHeight="1">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>EUS-50550</t>
+          <t>EUS-22282</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>Auditoría de las instalaciones existentes en los edificios q</t>
+          <t>Garbiketa eta higienerako produktuak/Productos de limpieza y</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
@@ -28484,12 +29034,12 @@
     <row r="85" ht="28" customHeight="1">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>EUS-83048</t>
+          <t>EUS-52631</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>Contrato de servicio de limpieza y desbroce de caminos públi</t>
+          <t>Transporte de las personas participantes en la campaña de ve</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
@@ -28517,8 +29067,80 @@
       <c r="I85" s="6" t="inlineStr"/>
       <c r="J85" s="6" t="inlineStr"/>
     </row>
+    <row r="86" ht="28" customHeight="1">
+      <c r="A86" s="6" t="inlineStr">
+        <is>
+          <t>EUS-08085</t>
+        </is>
+      </c>
+      <c r="B86" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fusionado de fibra óptica para conectar la casa club con la </t>
+        </is>
+      </c>
+      <c r="C86" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D86" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E86" s="6" t="inlineStr"/>
+      <c r="F86" s="27" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G86" s="6" t="inlineStr"/>
+      <c r="H86" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I86" s="6" t="inlineStr"/>
+      <c r="J86" s="6" t="inlineStr"/>
+    </row>
+    <row r="87" ht="28" customHeight="1">
+      <c r="A87" s="6" t="inlineStr">
+        <is>
+          <t>EUS-17254</t>
+        </is>
+      </c>
+      <c r="B87" s="6" t="inlineStr">
+        <is>
+          <t>Material de albañilería para el módulo de mantenimiento de v</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D87" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E87" s="6" t="inlineStr"/>
+      <c r="F87" s="27" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G87" s="6" t="inlineStr"/>
+      <c r="H87" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I87" s="6" t="inlineStr"/>
+      <c r="J87" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J85"/>
+  <autoFilter ref="A1:J87"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update funding data 2026-04-20
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Recursos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$93</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$85</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -679,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M93"/>
+  <dimension ref="A1:M91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -707,7 +707,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 19/04/2026 07:07 - 86 convocatorias - 10 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 20/04/2026 07:49 - 84 convocatorias - 8 nuevas</t>
         </is>
       </c>
     </row>
@@ -2529,12 +2529,12 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
+          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -2574,7 +2574,7 @@
       </c>
       <c r="K34" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Euro</t>
+          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and inter</t>
         </is>
       </c>
       <c r="L34" s="6" t="inlineStr"/>
@@ -2718,12 +2718,12 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
@@ -2748,7 +2748,7 @@
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Research and Innovation Actions</t>
+          <t>Programme Cofund Actions</t>
         </is>
       </c>
       <c r="I37" s="11" t="inlineStr">
@@ -2763,7 +2763,7 @@
       </c>
       <c r="K37" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to info</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is estab</t>
         </is>
       </c>
       <c r="L37" s="6" t="inlineStr"/>
@@ -2781,12 +2781,12 @@
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-08</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
@@ -2826,7 +2826,7 @@
       </c>
       <c r="K38" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and inter</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorpo</t>
         </is>
       </c>
       <c r="L38" s="6" t="inlineStr"/>
@@ -2844,12 +2844,12 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -2874,7 +2874,7 @@
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>Programme Cofund Actions</t>
+          <t xml:space="preserve"> Research and Innovation Actions</t>
         </is>
       </c>
       <c r="I39" s="11" t="inlineStr">
@@ -2889,7 +2889,7 @@
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is estab</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to info</t>
         </is>
       </c>
       <c r="L39" s="6" t="inlineStr"/>
@@ -2907,12 +2907,12 @@
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -2952,7 +2952,7 @@
       </c>
       <c r="K40" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorpo</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Euro</t>
         </is>
       </c>
       <c r="L40" s="6" t="inlineStr"/>
@@ -5315,7 +5315,7 @@
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>EUS-19519</t>
+          <t>EUS-15065</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
@@ -5370,7 +5370,7 @@
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>EUS-37183</t>
+          <t>EUS-35524</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
@@ -5425,7 +5425,7 @@
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>EUS-57324</t>
+          <t>EUS-92247</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
@@ -5480,7 +5480,7 @@
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>EUS-46961</t>
+          <t>EUS-01931</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
@@ -5535,7 +5535,7 @@
       </c>
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>EUS-97678</t>
+          <t>EUS-68899</t>
         </is>
       </c>
       <c r="C88" s="6" t="inlineStr">
@@ -5590,12 +5590,12 @@
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>EUS-08237</t>
+          <t>EUS-05501</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>PTO. Limpieza pintadas</t>
+          <t>Auditoría de las instalaciones existentes en los edificios que conforman el Campo de Golf de Bizkaia - Meaztegi Golf.</t>
         </is>
       </c>
       <c r="D89" s="6" t="inlineStr">
@@ -5645,12 +5645,12 @@
       </c>
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>EUS-22282</t>
+          <t>EUS-45127</t>
         </is>
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>Garbiketa eta higienerako produktuak/Productos de limpieza y aseo</t>
+          <t>Fusionado de fibra óptica para conectar la casa club con la caseta de préstamo de bicicletas eléctricas del Meaztegi Golf (Bizkaia).</t>
         </is>
       </c>
       <c r="D90" s="6" t="inlineStr">
@@ -5700,12 +5700,12 @@
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>EUS-52631</t>
+          <t>EUS-28844</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>Transporte de las personas participantes en la campaña de verano Udalekuak 2026</t>
+          <t>Servicio de transporte de Autobuses  Bengoetxea el 11/10/2025    de Donostia  a Donibane Lohitzune y vuelta a Donostia para  participantes del Congreso Ontológico 2025</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr">
@@ -5747,118 +5747,8 @@
         </is>
       </c>
     </row>
-    <row r="92" ht="40" customHeight="1">
-      <c r="A92" s="16" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="B92" s="6" t="inlineStr">
-        <is>
-          <t>EUS-08085</t>
-        </is>
-      </c>
-      <c r="C92" s="6" t="inlineStr">
-        <is>
-          <t>Fusionado de fibra óptica para conectar la casa club con la caseta de préstamo de bicicletas eléctricas del Meaztegi Golf (Bizkaia).</t>
-        </is>
-      </c>
-      <c r="D92" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="E92" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F92" s="6" t="inlineStr"/>
-      <c r="G92" s="6" t="inlineStr"/>
-      <c r="H92" s="6" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I92" s="10" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="J92" s="6" t="inlineStr"/>
-      <c r="K92" s="6" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="L92" s="17" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="M92" s="9" t="inlineStr">
-        <is>
-          <t>Ver</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="40" customHeight="1">
-      <c r="A93" s="16" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="B93" s="6" t="inlineStr">
-        <is>
-          <t>EUS-17254</t>
-        </is>
-      </c>
-      <c r="C93" s="6" t="inlineStr">
-        <is>
-          <t>Material de albañilería para el módulo de mantenimiento de viviendas del imfpb de azitain.</t>
-        </is>
-      </c>
-      <c r="D93" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="E93" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F93" s="6" t="inlineStr"/>
-      <c r="G93" s="6" t="inlineStr"/>
-      <c r="H93" s="6" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I93" s="10" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="J93" s="6" t="inlineStr"/>
-      <c r="K93" s="6" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="L93" s="17" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="M93" s="9" t="inlineStr">
-        <is>
-          <t>Ver</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:M93"/>
+  <autoFilter ref="A4:M91"/>
   <mergeCells count="5">
     <mergeCell ref="A76:M76"/>
     <mergeCell ref="A1:M1"/>
@@ -5951,8 +5841,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M89" r:id="rId82"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M90" r:id="rId83"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M91" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M92" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M93" r:id="rId86"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5964,7 +5852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1289"/>
+  <dimension ref="A1:F1259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -12050,7 +11938,7 @@
     <row r="421" ht="30" customHeight="1">
       <c r="A421" s="18" t="inlineStr">
         <is>
-          <t>FICHA 29: HORIZON-CL5-2027-01-D1-07</t>
+          <t>FICHA 29: HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="B421" s="19" t="n"/>
@@ -12075,7 +11963,7 @@
       <c r="E422" s="22" t="n"/>
       <c r="F422" s="22" t="n"/>
     </row>
-    <row r="423" ht="45" customHeight="1">
+    <row r="423" ht="20" customHeight="1">
       <c r="A423" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -12083,7 +11971,7 @@
       </c>
       <c r="B423" s="21" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
+          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
         </is>
       </c>
       <c r="C423" s="22" t="n"/>
@@ -12099,7 +11987,7 @@
       </c>
       <c r="B424" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="C424" s="22" t="n"/>
@@ -12211,7 +12099,7 @@
       </c>
       <c r="B431" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Europe and globally, as well as the interaction between different hazards, their cumulative and/or cascading effects.Enhanced seamless prediction and projection modelling and attribution capabilities for extreme events and their likelihood to support preparedness, response and resilience to climate change by EU and national and regional actors. The EU Union Preparedness Strategy, the EU Adaptation Str</t>
+          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and interactions with ecosystems, leading to improved Earth system models;Future climate change scenarios produced in light of past changes in the Earth system, in particular warm climates/high sea-level situations, and abrupt transitions;Identification of thresholds in Earth system components and better characterisation of driving mechanisms and feedbacks that may be responsible for non-linear behaviours,</t>
         </is>
       </c>
       <c r="C431" s="22" t="n"/>
@@ -12255,7 +12143,7 @@
       </c>
       <c r="B434" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-07</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="C434" s="22" t="n"/>
@@ -12698,7 +12586,7 @@
     <row r="466" ht="30" customHeight="1">
       <c r="A466" s="18" t="inlineStr">
         <is>
-          <t>FICHA 32: HORIZON-CL5-2027-01-D1-09</t>
+          <t>FICHA 32: HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="B466" s="19" t="n"/>
@@ -12723,7 +12611,7 @@
       <c r="E467" s="22" t="n"/>
       <c r="F467" s="22" t="n"/>
     </row>
-    <row r="468" ht="45" customHeight="1">
+    <row r="468" ht="20" customHeight="1">
       <c r="A468" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -12731,7 +12619,7 @@
       </c>
       <c r="B468" s="21" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="C468" s="22" t="n"/>
@@ -12747,7 +12635,7 @@
       </c>
       <c r="B469" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C469" s="22" t="n"/>
@@ -12827,7 +12715,7 @@
       </c>
       <c r="B474" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Research and Innovation Actions</t>
+          <t>Programme Cofund Actions</t>
         </is>
       </c>
       <c r="C474" s="22" t="n"/>
@@ -12859,7 +12747,7 @@
       </c>
       <c r="B476" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to inform mitigation action and policy improvements, ensuring a fair transition and social acceptability;Methodologies are developed and improved for ex-ante assessment and ex-post evaluation of greenhouse gas emission reductions from climate policies and measures;Strengthened collaboration and established networks between researchers, policy experts and government officials involved in designing and eva</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is established through development and implementation of the Climate Action pillar of the EU-AU Research and Innovation Partnership on Climate Change and Sustainable Energy (CCSE),[1] in co-design between African and European partners;Reduced fragmentation by aligning the EU, national and multilateral R&amp;amp;I efforts with increased leverage and impact of funding;African scientific, policy and practice com</t>
         </is>
       </c>
       <c r="C476" s="22" t="n"/>
@@ -12903,7 +12791,7 @@
       </c>
       <c r="B479" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-09</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C479" s="22" t="n"/>
@@ -12914,7 +12802,7 @@
     <row r="481" ht="30" customHeight="1">
       <c r="A481" s="18" t="inlineStr">
         <is>
-          <t>FICHA 33: HORIZON-CL5-2027-01-D1-08</t>
+          <t>FICHA 33: HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="B481" s="19" t="n"/>
@@ -12947,7 +12835,7 @@
       </c>
       <c r="B483" s="21" t="inlineStr">
         <is>
-          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="C483" s="22" t="n"/>
@@ -12963,7 +12851,7 @@
       </c>
       <c r="B484" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-08</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C484" s="22" t="n"/>
@@ -13075,7 +12963,7 @@
       </c>
       <c r="B491" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and interactions with ecosystems, leading to improved Earth system models;Future climate change scenarios produced in light of past changes in the Earth system, in particular warm climates/high sea-level situations, and abrupt transitions;Identification of thresholds in Earth system components and better characterisation of driving mechanisms and feedbacks that may be responsible for non-linear behaviours,</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorporation into main EU repositories, such as Climate-ADAPT or the portal of the EU Mission on Adaptation to Climate Change;The risk and adaptation assessment frameworks are improved by better integrating the maladaptation dimension;Guidelines and tools for maladaptation prevention and correction strategies are made available to adaptation stakeholders at relevant scales and inform the design and impl</t>
         </is>
       </c>
       <c r="C491" s="22" t="n"/>
@@ -13119,7 +13007,7 @@
       </c>
       <c r="B494" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-08</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C494" s="22" t="n"/>
@@ -13130,7 +13018,7 @@
     <row r="496" ht="30" customHeight="1">
       <c r="A496" s="18" t="inlineStr">
         <is>
-          <t>FICHA 34: HORIZON-CL5-2027-01-D1-11</t>
+          <t>FICHA 34: HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="B496" s="19" t="n"/>
@@ -13155,7 +13043,7 @@
       <c r="E497" s="22" t="n"/>
       <c r="F497" s="22" t="n"/>
     </row>
-    <row r="498" ht="20" customHeight="1">
+    <row r="498" ht="45" customHeight="1">
       <c r="A498" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -13163,7 +13051,7 @@
       </c>
       <c r="B498" s="21" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
         </is>
       </c>
       <c r="C498" s="22" t="n"/>
@@ -13179,7 +13067,7 @@
       </c>
       <c r="B499" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C499" s="22" t="n"/>
@@ -13259,7 +13147,7 @@
       </c>
       <c r="B504" s="21" t="inlineStr">
         <is>
-          <t>Programme Cofund Actions</t>
+          <t xml:space="preserve"> Research and Innovation Actions</t>
         </is>
       </c>
       <c r="C504" s="22" t="n"/>
@@ -13291,7 +13179,7 @@
       </c>
       <c r="B506" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is established through development and implementation of the Climate Action pillar of the EU-AU Research and Innovation Partnership on Climate Change and Sustainable Energy (CCSE),[1] in co-design between African and European partners;Reduced fragmentation by aligning the EU, national and multilateral R&amp;amp;I efforts with increased leverage and impact of funding;African scientific, policy and practice com</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to inform mitigation action and policy improvements, ensuring a fair transition and social acceptability;Methodologies are developed and improved for ex-ante assessment and ex-post evaluation of greenhouse gas emission reductions from climate policies and measures;Strengthened collaboration and established networks between researchers, policy experts and government officials involved in designing and eva</t>
         </is>
       </c>
       <c r="C506" s="22" t="n"/>
@@ -13335,7 +13223,7 @@
       </c>
       <c r="B509" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-11</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C509" s="22" t="n"/>
@@ -13346,7 +13234,7 @@
     <row r="511" ht="30" customHeight="1">
       <c r="A511" s="18" t="inlineStr">
         <is>
-          <t>FICHA 35: HORIZON-CL5-2027-01-D1-10</t>
+          <t>FICHA 35: HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="B511" s="19" t="n"/>
@@ -13371,7 +13259,7 @@
       <c r="E512" s="22" t="n"/>
       <c r="F512" s="22" t="n"/>
     </row>
-    <row r="513" ht="20" customHeight="1">
+    <row r="513" ht="45" customHeight="1">
       <c r="A513" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -13379,7 +13267,7 @@
       </c>
       <c r="B513" s="21" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
         </is>
       </c>
       <c r="C513" s="22" t="n"/>
@@ -13395,7 +13283,7 @@
       </c>
       <c r="B514" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C514" s="22" t="n"/>
@@ -13507,7 +13395,7 @@
       </c>
       <c r="B521" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorporation into main EU repositories, such as Climate-ADAPT or the portal of the EU Mission on Adaptation to Climate Change;The risk and adaptation assessment frameworks are improved by better integrating the maladaptation dimension;Guidelines and tools for maladaptation prevention and correction strategies are made available to adaptation stakeholders at relevant scales and inform the design and impl</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Europe and globally, as well as the interaction between different hazards, their cumulative and/or cascading effects.Enhanced seamless prediction and projection modelling and attribution capabilities for extreme events and their likelihood to support preparedness, response and resilience to climate change by EU and national and regional actors. The EU Union Preparedness Strategy, the EU Adaptation Str</t>
         </is>
       </c>
       <c r="C521" s="22" t="n"/>
@@ -13551,7 +13439,7 @@
       </c>
       <c r="B524" s="24" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-10</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C524" s="22" t="n"/>
@@ -22362,7 +22250,7 @@
     <row r="1141" ht="30" customHeight="1">
       <c r="A1141" s="18" t="inlineStr">
         <is>
-          <t>FICHA 77: EUS-19519</t>
+          <t>FICHA 77: EUS-15065</t>
         </is>
       </c>
       <c r="B1141" s="19" t="n"/>
@@ -22411,7 +22299,7 @@
       </c>
       <c r="B1144" s="21" t="inlineStr">
         <is>
-          <t>EUS-19519</t>
+          <t>EUS-15065</t>
         </is>
       </c>
       <c r="C1144" s="22" t="n"/>
@@ -22574,7 +22462,7 @@
     <row r="1156" ht="30" customHeight="1">
       <c r="A1156" s="18" t="inlineStr">
         <is>
-          <t>FICHA 78: EUS-37183</t>
+          <t>FICHA 78: EUS-35524</t>
         </is>
       </c>
       <c r="B1156" s="19" t="n"/>
@@ -22623,7 +22511,7 @@
       </c>
       <c r="B1159" s="21" t="inlineStr">
         <is>
-          <t>EUS-37183</t>
+          <t>EUS-35524</t>
         </is>
       </c>
       <c r="C1159" s="22" t="n"/>
@@ -22786,7 +22674,7 @@
     <row r="1171" ht="30" customHeight="1">
       <c r="A1171" s="18" t="inlineStr">
         <is>
-          <t>FICHA 79: EUS-57324</t>
+          <t>FICHA 79: EUS-92247</t>
         </is>
       </c>
       <c r="B1171" s="19" t="n"/>
@@ -22835,7 +22723,7 @@
       </c>
       <c r="B1174" s="21" t="inlineStr">
         <is>
-          <t>EUS-57324</t>
+          <t>EUS-92247</t>
         </is>
       </c>
       <c r="C1174" s="22" t="n"/>
@@ -22998,7 +22886,7 @@
     <row r="1186" ht="30" customHeight="1">
       <c r="A1186" s="18" t="inlineStr">
         <is>
-          <t>FICHA 80: EUS-46961</t>
+          <t>FICHA 80: EUS-01931</t>
         </is>
       </c>
       <c r="B1186" s="19" t="n"/>
@@ -23047,7 +22935,7 @@
       </c>
       <c r="B1189" s="21" t="inlineStr">
         <is>
-          <t>EUS-46961</t>
+          <t>EUS-01931</t>
         </is>
       </c>
       <c r="C1189" s="22" t="n"/>
@@ -23210,7 +23098,7 @@
     <row r="1201" ht="30" customHeight="1">
       <c r="A1201" s="18" t="inlineStr">
         <is>
-          <t>FICHA 81: EUS-97678</t>
+          <t>FICHA 81: EUS-68899</t>
         </is>
       </c>
       <c r="B1201" s="19" t="n"/>
@@ -23259,7 +23147,7 @@
       </c>
       <c r="B1204" s="21" t="inlineStr">
         <is>
-          <t>EUS-97678</t>
+          <t>EUS-68899</t>
         </is>
       </c>
       <c r="C1204" s="22" t="n"/>
@@ -23422,7 +23310,7 @@
     <row r="1216" ht="30" customHeight="1">
       <c r="A1216" s="18" t="inlineStr">
         <is>
-          <t>FICHA 82: EUS-08237</t>
+          <t>FICHA 82: EUS-05501</t>
         </is>
       </c>
       <c r="B1216" s="19" t="n"/>
@@ -23447,7 +23335,7 @@
       <c r="E1217" s="22" t="n"/>
       <c r="F1217" s="22" t="n"/>
     </row>
-    <row r="1218" ht="20" customHeight="1">
+    <row r="1218" ht="45" customHeight="1">
       <c r="A1218" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -23455,7 +23343,7 @@
       </c>
       <c r="B1218" s="21" t="inlineStr">
         <is>
-          <t>PTO. Limpieza pintadas</t>
+          <t>Auditoría de las instalaciones existentes en los edificios que conforman el Campo de Golf de Bizkaia - Meaztegi Golf.</t>
         </is>
       </c>
       <c r="C1218" s="22" t="n"/>
@@ -23471,7 +23359,7 @@
       </c>
       <c r="B1219" s="21" t="inlineStr">
         <is>
-          <t>EUS-08237</t>
+          <t>EUS-05501</t>
         </is>
       </c>
       <c r="C1219" s="22" t="n"/>
@@ -23623,7 +23511,7 @@
       </c>
       <c r="B1229" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/pto-limpieza-pintadas/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/auditoria-instalaciones-existentes-edificios-que-conforman-campo-golf-bizkaia-meaztegi-golf/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1229" s="22" t="n"/>
@@ -23634,7 +23522,7 @@
     <row r="1231" ht="30" customHeight="1">
       <c r="A1231" s="18" t="inlineStr">
         <is>
-          <t>FICHA 83: EUS-22282</t>
+          <t>FICHA 83: EUS-45127</t>
         </is>
       </c>
       <c r="B1231" s="19" t="n"/>
@@ -23659,7 +23547,7 @@
       <c r="E1232" s="22" t="n"/>
       <c r="F1232" s="22" t="n"/>
     </row>
-    <row r="1233" ht="20" customHeight="1">
+    <row r="1233" ht="45" customHeight="1">
       <c r="A1233" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -23667,7 +23555,7 @@
       </c>
       <c r="B1233" s="21" t="inlineStr">
         <is>
-          <t>Garbiketa eta higienerako produktuak/Productos de limpieza y aseo</t>
+          <t>Fusionado de fibra óptica para conectar la casa club con la caseta de préstamo de bicicletas eléctricas del Meaztegi Golf (Bizkaia).</t>
         </is>
       </c>
       <c r="C1233" s="22" t="n"/>
@@ -23683,7 +23571,7 @@
       </c>
       <c r="B1234" s="21" t="inlineStr">
         <is>
-          <t>EUS-22282</t>
+          <t>EUS-45127</t>
         </is>
       </c>
       <c r="C1234" s="22" t="n"/>
@@ -23835,7 +23723,7 @@
       </c>
       <c r="B1244" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/garbiketa-eta-higienerako-produktuak-productos-limpieza-y-aseo/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/fusionado-fibra-optica-conectar-casa-club-caseta-prestamo-bicicletas-electricas-del-meaztegi-golf-bizkaia/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1244" s="22" t="n"/>
@@ -23846,7 +23734,7 @@
     <row r="1246" ht="30" customHeight="1">
       <c r="A1246" s="18" t="inlineStr">
         <is>
-          <t>FICHA 84: EUS-52631</t>
+          <t>FICHA 84: EUS-28844</t>
         </is>
       </c>
       <c r="B1246" s="19" t="n"/>
@@ -23871,7 +23759,7 @@
       <c r="E1247" s="22" t="n"/>
       <c r="F1247" s="22" t="n"/>
     </row>
-    <row r="1248" ht="20" customHeight="1">
+    <row r="1248" ht="45" customHeight="1">
       <c r="A1248" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -23879,7 +23767,7 @@
       </c>
       <c r="B1248" s="21" t="inlineStr">
         <is>
-          <t>Transporte de las personas participantes en la campaña de verano Udalekuak 2026</t>
+          <t>Servicio de transporte de Autobuses  Bengoetxea el 11/10/2025    de Donostia  a Donibane Lohitzune y vuelta a Donostia para  participantes del Congreso Ontológico 2025</t>
         </is>
       </c>
       <c r="C1248" s="22" t="n"/>
@@ -23895,7 +23783,7 @@
       </c>
       <c r="B1249" s="21" t="inlineStr">
         <is>
-          <t>EUS-52631</t>
+          <t>EUS-28844</t>
         </is>
       </c>
       <c r="C1249" s="22" t="n"/>
@@ -24047,7 +23935,7 @@
       </c>
       <c r="B1259" s="24" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/transporte-personas-participantes-campana-verano-udalekuak-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-transporte-autobuses-bengoetxea-11-10-2025-donostia-donibane-lohitzune-y-vuelta-donostia-participantes-del-congreso-ontologico-2025/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1259" s="22" t="n"/>
@@ -24055,432 +23943,8 @@
       <c r="E1259" s="22" t="n"/>
       <c r="F1259" s="22" t="n"/>
     </row>
-    <row r="1261" ht="30" customHeight="1">
-      <c r="A1261" s="18" t="inlineStr">
-        <is>
-          <t>FICHA 85: EUS-08085</t>
-        </is>
-      </c>
-      <c r="B1261" s="19" t="n"/>
-      <c r="C1261" s="19" t="n"/>
-      <c r="D1261" s="19" t="n"/>
-      <c r="E1261" s="19" t="n"/>
-      <c r="F1261" s="19" t="n"/>
-    </row>
-    <row r="1262" ht="20" customHeight="1">
-      <c r="A1262" s="20" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-      <c r="B1262" s="21" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
-        </is>
-      </c>
-      <c r="C1262" s="22" t="n"/>
-      <c r="D1262" s="22" t="n"/>
-      <c r="E1262" s="22" t="n"/>
-      <c r="F1262" s="22" t="n"/>
-    </row>
-    <row r="1263" ht="45" customHeight="1">
-      <c r="A1263" s="20" t="inlineStr">
-        <is>
-          <t>Titulo</t>
-        </is>
-      </c>
-      <c r="B1263" s="21" t="inlineStr">
-        <is>
-          <t>Fusionado de fibra óptica para conectar la casa club con la caseta de préstamo de bicicletas eléctricas del Meaztegi Golf (Bizkaia).</t>
-        </is>
-      </c>
-      <c r="C1263" s="22" t="n"/>
-      <c r="D1263" s="22" t="n"/>
-      <c r="E1263" s="22" t="n"/>
-      <c r="F1263" s="22" t="n"/>
-    </row>
-    <row r="1264" ht="20" customHeight="1">
-      <c r="A1264" s="20" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1264" s="21" t="inlineStr">
-        <is>
-          <t>EUS-08085</t>
-        </is>
-      </c>
-      <c r="C1264" s="22" t="n"/>
-      <c r="D1264" s="22" t="n"/>
-      <c r="E1264" s="22" t="n"/>
-      <c r="F1264" s="22" t="n"/>
-    </row>
-    <row r="1265" ht="20" customHeight="1">
-      <c r="A1265" s="20" t="inlineStr">
-        <is>
-          <t>Programa</t>
-        </is>
-      </c>
-      <c r="B1265" s="21" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="C1265" s="22" t="n"/>
-      <c r="D1265" s="22" t="n"/>
-      <c r="E1265" s="22" t="n"/>
-      <c r="F1265" s="22" t="n"/>
-    </row>
-    <row r="1266" ht="20" customHeight="1">
-      <c r="A1266" s="20" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="B1266" s="21" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C1266" s="22" t="n"/>
-      <c r="D1266" s="22" t="n"/>
-      <c r="E1266" s="22" t="n"/>
-      <c r="F1266" s="22" t="n"/>
-    </row>
-    <row r="1267" ht="20" customHeight="1">
-      <c r="A1267" s="20" t="inlineStr">
-        <is>
-          <t>Deadline</t>
-        </is>
-      </c>
-      <c r="B1267" s="21" t="inlineStr"/>
-      <c r="C1267" s="22" t="n"/>
-      <c r="D1267" s="22" t="n"/>
-      <c r="E1267" s="22" t="n"/>
-      <c r="F1267" s="22" t="n"/>
-    </row>
-    <row r="1268" ht="20" customHeight="1">
-      <c r="A1268" s="20" t="inlineStr">
-        <is>
-          <t>Presupuesto (EUR)</t>
-        </is>
-      </c>
-      <c r="B1268" s="21" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="C1268" s="22" t="n"/>
-      <c r="D1268" s="22" t="n"/>
-      <c r="E1268" s="22" t="n"/>
-      <c r="F1268" s="22" t="n"/>
-    </row>
-    <row r="1269" ht="20" customHeight="1">
-      <c r="A1269" s="20" t="inlineStr">
-        <is>
-          <t>Tipo de Accion</t>
-        </is>
-      </c>
-      <c r="B1269" s="21" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="C1269" s="22" t="n"/>
-      <c r="D1269" s="22" t="n"/>
-      <c r="E1269" s="22" t="n"/>
-      <c r="F1269" s="22" t="n"/>
-    </row>
-    <row r="1270" ht="20" customHeight="1">
-      <c r="A1270" s="20" t="inlineStr">
-        <is>
-          <t>Call ID</t>
-        </is>
-      </c>
-      <c r="B1270" s="21" t="inlineStr"/>
-      <c r="C1270" s="22" t="n"/>
-      <c r="D1270" s="22" t="n"/>
-      <c r="E1270" s="22" t="n"/>
-      <c r="F1270" s="22" t="n"/>
-    </row>
-    <row r="1271" ht="20" customHeight="1">
-      <c r="A1271" s="20" t="inlineStr">
-        <is>
-          <t>Descripcion</t>
-        </is>
-      </c>
-      <c r="B1271" s="21" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="C1271" s="22" t="n"/>
-      <c r="D1271" s="22" t="n"/>
-      <c r="E1271" s="22" t="n"/>
-      <c r="F1271" s="22" t="n"/>
-    </row>
-    <row r="1272" ht="20" customHeight="1">
-      <c r="A1272" s="20" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-      <c r="B1272" s="21" t="inlineStr">
-        <is>
-          <t>energia</t>
-        </is>
-      </c>
-      <c r="C1272" s="22" t="n"/>
-      <c r="D1272" s="22" t="n"/>
-      <c r="E1272" s="22" t="n"/>
-      <c r="F1272" s="22" t="n"/>
-    </row>
-    <row r="1273" ht="20" customHeight="1">
-      <c r="A1273" s="20" t="inlineStr">
-        <is>
-          <t>Relevancia Bilbao</t>
-        </is>
-      </c>
-      <c r="B1273" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
-        </is>
-      </c>
-      <c r="C1273" s="22" t="n"/>
-      <c r="D1273" s="22" t="n"/>
-      <c r="E1273" s="22" t="n"/>
-      <c r="F1273" s="22" t="n"/>
-    </row>
-    <row r="1274" ht="45" customHeight="1">
-      <c r="A1274" s="20" t="inlineStr">
-        <is>
-          <t>Enlace al portal</t>
-        </is>
-      </c>
-      <c r="B1274" s="24" t="inlineStr">
-        <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/fusionado-fibra-optica-conectar-casa-club-caseta-prestamo-bicicletas-electricas-del-meaztegi-golf-bizkaia/web01-tramite/es/</t>
-        </is>
-      </c>
-      <c r="C1274" s="22" t="n"/>
-      <c r="D1274" s="22" t="n"/>
-      <c r="E1274" s="22" t="n"/>
-      <c r="F1274" s="22" t="n"/>
-    </row>
-    <row r="1276" ht="30" customHeight="1">
-      <c r="A1276" s="18" t="inlineStr">
-        <is>
-          <t>FICHA 86: EUS-17254</t>
-        </is>
-      </c>
-      <c r="B1276" s="19" t="n"/>
-      <c r="C1276" s="19" t="n"/>
-      <c r="D1276" s="19" t="n"/>
-      <c r="E1276" s="19" t="n"/>
-      <c r="F1276" s="19" t="n"/>
-    </row>
-    <row r="1277" ht="20" customHeight="1">
-      <c r="A1277" s="20" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-      <c r="B1277" s="21" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
-        </is>
-      </c>
-      <c r="C1277" s="22" t="n"/>
-      <c r="D1277" s="22" t="n"/>
-      <c r="E1277" s="22" t="n"/>
-      <c r="F1277" s="22" t="n"/>
-    </row>
-    <row r="1278" ht="45" customHeight="1">
-      <c r="A1278" s="20" t="inlineStr">
-        <is>
-          <t>Titulo</t>
-        </is>
-      </c>
-      <c r="B1278" s="21" t="inlineStr">
-        <is>
-          <t>Material de albañilería para el módulo de mantenimiento de viviendas del imfpb de azitain.</t>
-        </is>
-      </c>
-      <c r="C1278" s="22" t="n"/>
-      <c r="D1278" s="22" t="n"/>
-      <c r="E1278" s="22" t="n"/>
-      <c r="F1278" s="22" t="n"/>
-    </row>
-    <row r="1279" ht="20" customHeight="1">
-      <c r="A1279" s="20" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1279" s="21" t="inlineStr">
-        <is>
-          <t>EUS-17254</t>
-        </is>
-      </c>
-      <c r="C1279" s="22" t="n"/>
-      <c r="D1279" s="22" t="n"/>
-      <c r="E1279" s="22" t="n"/>
-      <c r="F1279" s="22" t="n"/>
-    </row>
-    <row r="1280" ht="20" customHeight="1">
-      <c r="A1280" s="20" t="inlineStr">
-        <is>
-          <t>Programa</t>
-        </is>
-      </c>
-      <c r="B1280" s="21" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="C1280" s="22" t="n"/>
-      <c r="D1280" s="22" t="n"/>
-      <c r="E1280" s="22" t="n"/>
-      <c r="F1280" s="22" t="n"/>
-    </row>
-    <row r="1281" ht="20" customHeight="1">
-      <c r="A1281" s="20" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="B1281" s="21" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C1281" s="22" t="n"/>
-      <c r="D1281" s="22" t="n"/>
-      <c r="E1281" s="22" t="n"/>
-      <c r="F1281" s="22" t="n"/>
-    </row>
-    <row r="1282" ht="20" customHeight="1">
-      <c r="A1282" s="20" t="inlineStr">
-        <is>
-          <t>Deadline</t>
-        </is>
-      </c>
-      <c r="B1282" s="21" t="inlineStr"/>
-      <c r="C1282" s="22" t="n"/>
-      <c r="D1282" s="22" t="n"/>
-      <c r="E1282" s="22" t="n"/>
-      <c r="F1282" s="22" t="n"/>
-    </row>
-    <row r="1283" ht="20" customHeight="1">
-      <c r="A1283" s="20" t="inlineStr">
-        <is>
-          <t>Presupuesto (EUR)</t>
-        </is>
-      </c>
-      <c r="B1283" s="21" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="C1283" s="22" t="n"/>
-      <c r="D1283" s="22" t="n"/>
-      <c r="E1283" s="22" t="n"/>
-      <c r="F1283" s="22" t="n"/>
-    </row>
-    <row r="1284" ht="20" customHeight="1">
-      <c r="A1284" s="20" t="inlineStr">
-        <is>
-          <t>Tipo de Accion</t>
-        </is>
-      </c>
-      <c r="B1284" s="21" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="C1284" s="22" t="n"/>
-      <c r="D1284" s="22" t="n"/>
-      <c r="E1284" s="22" t="n"/>
-      <c r="F1284" s="22" t="n"/>
-    </row>
-    <row r="1285" ht="20" customHeight="1">
-      <c r="A1285" s="20" t="inlineStr">
-        <is>
-          <t>Call ID</t>
-        </is>
-      </c>
-      <c r="B1285" s="21" t="inlineStr"/>
-      <c r="C1285" s="22" t="n"/>
-      <c r="D1285" s="22" t="n"/>
-      <c r="E1285" s="22" t="n"/>
-      <c r="F1285" s="22" t="n"/>
-    </row>
-    <row r="1286" ht="20" customHeight="1">
-      <c r="A1286" s="20" t="inlineStr">
-        <is>
-          <t>Descripcion</t>
-        </is>
-      </c>
-      <c r="B1286" s="21" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="C1286" s="22" t="n"/>
-      <c r="D1286" s="22" t="n"/>
-      <c r="E1286" s="22" t="n"/>
-      <c r="F1286" s="22" t="n"/>
-    </row>
-    <row r="1287" ht="20" customHeight="1">
-      <c r="A1287" s="20" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-      <c r="B1287" s="21" t="inlineStr">
-        <is>
-          <t>energia</t>
-        </is>
-      </c>
-      <c r="C1287" s="22" t="n"/>
-      <c r="D1287" s="22" t="n"/>
-      <c r="E1287" s="22" t="n"/>
-      <c r="F1287" s="22" t="n"/>
-    </row>
-    <row r="1288" ht="20" customHeight="1">
-      <c r="A1288" s="20" t="inlineStr">
-        <is>
-          <t>Relevancia Bilbao</t>
-        </is>
-      </c>
-      <c r="B1288" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
-        </is>
-      </c>
-      <c r="C1288" s="22" t="n"/>
-      <c r="D1288" s="22" t="n"/>
-      <c r="E1288" s="22" t="n"/>
-      <c r="F1288" s="22" t="n"/>
-    </row>
-    <row r="1289" ht="45" customHeight="1">
-      <c r="A1289" s="20" t="inlineStr">
-        <is>
-          <t>Enlace al portal</t>
-        </is>
-      </c>
-      <c r="B1289" s="24" t="inlineStr">
-        <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/material-albanileria-modulo-mantenimiento-viviendas-del-imfpb-azitain/web01-tramite/es/</t>
-        </is>
-      </c>
-      <c r="C1289" s="22" t="n"/>
-      <c r="D1289" s="22" t="n"/>
-      <c r="E1289" s="22" t="n"/>
-      <c r="F1289" s="22" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="1204">
+  <mergeCells count="1176">
     <mergeCell ref="B679:F679"/>
     <mergeCell ref="B666:F666"/>
     <mergeCell ref="B964:F964"/>
@@ -24501,7 +23965,6 @@
     <mergeCell ref="B512:F512"/>
     <mergeCell ref="B238:F238"/>
     <mergeCell ref="B509:F509"/>
-    <mergeCell ref="B1264:F1264"/>
     <mergeCell ref="B303:F303"/>
     <mergeCell ref="B941:F941"/>
     <mergeCell ref="B797:F797"/>
@@ -24534,7 +23997,6 @@
     <mergeCell ref="B515:F515"/>
     <mergeCell ref="B1128:F1128"/>
     <mergeCell ref="B1193:F1193"/>
-    <mergeCell ref="B1279:F1279"/>
     <mergeCell ref="A841:F841"/>
     <mergeCell ref="B158:F158"/>
     <mergeCell ref="B1094:F1094"/>
@@ -24591,7 +24053,6 @@
     <mergeCell ref="B293:F293"/>
     <mergeCell ref="B657:F657"/>
     <mergeCell ref="B322:F322"/>
-    <mergeCell ref="B1270:F1270"/>
     <mergeCell ref="B1191:F1191"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B672:F672"/>
@@ -24600,7 +24061,6 @@
     <mergeCell ref="B148:F148"/>
     <mergeCell ref="B82:F82"/>
     <mergeCell ref="B446:F446"/>
-    <mergeCell ref="B1272:F1272"/>
     <mergeCell ref="B688:F688"/>
     <mergeCell ref="B622:F622"/>
     <mergeCell ref="B682:F682"/>
@@ -24683,7 +24143,6 @@
     <mergeCell ref="B1075:F1075"/>
     <mergeCell ref="B1197:F1197"/>
     <mergeCell ref="B678:F678"/>
-    <mergeCell ref="B1262:F1262"/>
     <mergeCell ref="B363:F363"/>
     <mergeCell ref="B534:F534"/>
     <mergeCell ref="B805:F805"/>
@@ -24710,7 +24169,6 @@
     <mergeCell ref="B1052:F1052"/>
     <mergeCell ref="B981:F981"/>
     <mergeCell ref="B846:F846"/>
-    <mergeCell ref="B1288:F1288"/>
     <mergeCell ref="B973:F973"/>
     <mergeCell ref="B389:F389"/>
     <mergeCell ref="B1044:F1044"/>
@@ -24761,10 +24219,8 @@
     <mergeCell ref="B1001:F1001"/>
     <mergeCell ref="B246:F246"/>
     <mergeCell ref="B1174:F1174"/>
-    <mergeCell ref="B1268:F1268"/>
     <mergeCell ref="B40:F40"/>
     <mergeCell ref="B338:F338"/>
-    <mergeCell ref="B1286:F1286"/>
     <mergeCell ref="B469:F469"/>
     <mergeCell ref="B767:F767"/>
     <mergeCell ref="B177:F177"/>
@@ -24779,8 +24235,6 @@
     <mergeCell ref="B978:F978"/>
     <mergeCell ref="B79:F79"/>
     <mergeCell ref="B1076:F1076"/>
-    <mergeCell ref="B1283:F1283"/>
-    <mergeCell ref="B1263:F1263"/>
     <mergeCell ref="B41:F41"/>
     <mergeCell ref="B35:F35"/>
     <mergeCell ref="B302:F302"/>
@@ -24802,14 +24256,12 @@
     <mergeCell ref="A1111:F1111"/>
     <mergeCell ref="B1084:F1084"/>
     <mergeCell ref="A976:F976"/>
-    <mergeCell ref="B1266:F1266"/>
     <mergeCell ref="B170:F170"/>
     <mergeCell ref="B157:F157"/>
     <mergeCell ref="B328:F328"/>
     <mergeCell ref="B455:F455"/>
     <mergeCell ref="B626:F626"/>
     <mergeCell ref="B697:F697"/>
-    <mergeCell ref="B1281:F1281"/>
     <mergeCell ref="B491:F491"/>
     <mergeCell ref="B762:F762"/>
     <mergeCell ref="B933:F933"/>
@@ -24841,7 +24293,6 @@
     <mergeCell ref="B1162:F1162"/>
     <mergeCell ref="B1233:F1233"/>
     <mergeCell ref="B692:F692"/>
-    <mergeCell ref="B1282:F1282"/>
     <mergeCell ref="A931:F931"/>
     <mergeCell ref="B486:F486"/>
     <mergeCell ref="B757:F757"/>
@@ -24903,7 +24354,6 @@
     <mergeCell ref="B171:F171"/>
     <mergeCell ref="B1168:F1168"/>
     <mergeCell ref="B407:F407"/>
-    <mergeCell ref="B1287:F1287"/>
     <mergeCell ref="A646:F646"/>
     <mergeCell ref="B972:F972"/>
     <mergeCell ref="B1208:F1208"/>
@@ -24934,7 +24384,6 @@
     <mergeCell ref="B507:F507"/>
     <mergeCell ref="B62:F62"/>
     <mergeCell ref="B700:F700"/>
-    <mergeCell ref="B1284:F1284"/>
     <mergeCell ref="B998:F998"/>
     <mergeCell ref="B792:F792"/>
     <mergeCell ref="B596:F596"/>
@@ -24953,7 +24402,6 @@
     <mergeCell ref="B39:F39"/>
     <mergeCell ref="B1092:F1092"/>
     <mergeCell ref="B508:F508"/>
-    <mergeCell ref="B1285:F1285"/>
     <mergeCell ref="B573:F573"/>
     <mergeCell ref="A961:F961"/>
     <mergeCell ref="B858:F858"/>
@@ -24989,7 +24437,6 @@
     <mergeCell ref="B222:F222"/>
     <mergeCell ref="B344:F344"/>
     <mergeCell ref="B415:F415"/>
-    <mergeCell ref="B1265:F1265"/>
     <mergeCell ref="B713:F713"/>
     <mergeCell ref="B884:F884"/>
     <mergeCell ref="B63:F63"/>
@@ -25064,7 +24511,6 @@
     <mergeCell ref="B169:F169"/>
     <mergeCell ref="B1166:F1166"/>
     <mergeCell ref="A706:F706"/>
-    <mergeCell ref="B1278:F1278"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B129:F129"/>
     <mergeCell ref="B200:F200"/>
@@ -25125,7 +24571,6 @@
     <mergeCell ref="B289:F289"/>
     <mergeCell ref="A721:F721"/>
     <mergeCell ref="B1259:F1259"/>
-    <mergeCell ref="A1261:F1261"/>
     <mergeCell ref="A31:F31"/>
     <mergeCell ref="B747:F747"/>
     <mergeCell ref="B1152:F1152"/>
@@ -25235,7 +24680,6 @@
     <mergeCell ref="A1156:F1156"/>
     <mergeCell ref="B232:F232"/>
     <mergeCell ref="B321:F321"/>
-    <mergeCell ref="B1274:F1274"/>
     <mergeCell ref="B215:F215"/>
     <mergeCell ref="B513:F513"/>
     <mergeCell ref="B684:F684"/>
@@ -25272,7 +24716,6 @@
     <mergeCell ref="B921:F921"/>
     <mergeCell ref="B550:F550"/>
     <mergeCell ref="B606:F606"/>
-    <mergeCell ref="B1269:F1269"/>
     <mergeCell ref="B544:F544"/>
     <mergeCell ref="B848:F848"/>
     <mergeCell ref="B87:F87"/>
@@ -25282,12 +24725,10 @@
     <mergeCell ref="B1206:F1206"/>
     <mergeCell ref="B245:F245"/>
     <mergeCell ref="B687:F687"/>
-    <mergeCell ref="B1271:F1271"/>
     <mergeCell ref="B543:F543"/>
     <mergeCell ref="B814:F814"/>
     <mergeCell ref="B456:F456"/>
     <mergeCell ref="B260:F260"/>
-    <mergeCell ref="A1276:F1276"/>
     <mergeCell ref="B545:F545"/>
     <mergeCell ref="A496:F496"/>
     <mergeCell ref="B36:F36"/>
@@ -25347,7 +24788,6 @@
     <mergeCell ref="A811:F811"/>
     <mergeCell ref="B1150:F1150"/>
     <mergeCell ref="B329:F329"/>
-    <mergeCell ref="B1277:F1277"/>
     <mergeCell ref="B627:F627"/>
     <mergeCell ref="A1201:F1201"/>
     <mergeCell ref="B49:F49"/>
@@ -25396,7 +24836,6 @@
     <mergeCell ref="B261:F261"/>
     <mergeCell ref="B1087:F1087"/>
     <mergeCell ref="B1149:F1149"/>
-    <mergeCell ref="B1280:F1280"/>
     <mergeCell ref="B1214:F1214"/>
     <mergeCell ref="B184:F184"/>
     <mergeCell ref="B1062:F1062"/>
@@ -25447,8 +24886,6 @@
     <mergeCell ref="B143:F143"/>
     <mergeCell ref="B118:F118"/>
     <mergeCell ref="B1202:F1202"/>
-    <mergeCell ref="B1273:F1273"/>
-    <mergeCell ref="B1267:F1267"/>
     <mergeCell ref="B683:F683"/>
     <mergeCell ref="A751:F751"/>
     <mergeCell ref="B477:F477"/>
@@ -25567,7 +25004,6 @@
     <mergeCell ref="B920:F920"/>
     <mergeCell ref="B1108:F1108"/>
     <mergeCell ref="B711:F711"/>
-    <mergeCell ref="B1289:F1289"/>
     <mergeCell ref="B1009:F1009"/>
     <mergeCell ref="B48:F48"/>
     <mergeCell ref="B1101:F1101"/>
@@ -25771,8 +25207,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1229" r:id="rId82"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1244" r:id="rId83"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1259" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1274" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1289" r:id="rId86"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -25784,7 +25218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J87"/>
+  <dimension ref="A1:J85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -26970,12 +26404,12 @@
     <row r="30" ht="28" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme</t>
+          <t>Palaeoclimate science for a better understanding of Earth sy</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -27090,12 +26524,12 @@
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform cl</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -27130,12 +26564,12 @@
     <row r="34" ht="28" customHeight="1">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-08</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Palaeoclimate science for a better understanding of Earth sy</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
@@ -27170,12 +26604,12 @@
     <row r="35" ht="28" customHeight="1">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Assessing the performance of policy instruments to inform cl</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -27210,12 +26644,12 @@
     <row r="36" ht="28" customHeight="1">
       <c r="A36" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Advancing understanding, modelling and prediction of extreme</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -28782,7 +28216,7 @@
     <row r="78" ht="28" customHeight="1">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>EUS-19519</t>
+          <t>EUS-15065</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
@@ -28818,7 +28252,7 @@
     <row r="79" ht="28" customHeight="1">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>EUS-37183</t>
+          <t>EUS-35524</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
@@ -28854,7 +28288,7 @@
     <row r="80" ht="28" customHeight="1">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>EUS-57324</t>
+          <t>EUS-92247</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
@@ -28890,7 +28324,7 @@
     <row r="81" ht="28" customHeight="1">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>EUS-46961</t>
+          <t>EUS-01931</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
@@ -28926,7 +28360,7 @@
     <row r="82" ht="28" customHeight="1">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>EUS-97678</t>
+          <t>EUS-68899</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
@@ -28962,12 +28396,12 @@
     <row r="83" ht="28" customHeight="1">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>EUS-08237</t>
+          <t>EUS-05501</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>PTO. Limpieza pintadas</t>
+          <t>Auditoría de las instalaciones existentes en los edificios q</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
@@ -28998,12 +28432,12 @@
     <row r="84" ht="28" customHeight="1">
       <c r="A84" s="6" t="inlineStr">
         <is>
-          <t>EUS-22282</t>
+          <t>EUS-45127</t>
         </is>
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>Garbiketa eta higienerako produktuak/Productos de limpieza y</t>
+          <t xml:space="preserve">Fusionado de fibra óptica para conectar la casa club con la </t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
@@ -29034,12 +28468,12 @@
     <row r="85" ht="28" customHeight="1">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>EUS-52631</t>
+          <t>EUS-28844</t>
         </is>
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>Transporte de las personas participantes en la campaña de ve</t>
+          <t>Servicio de transporte de Autobuses  Bengoetxea el 11/10/202</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
@@ -29067,80 +28501,8 @@
       <c r="I85" s="6" t="inlineStr"/>
       <c r="J85" s="6" t="inlineStr"/>
     </row>
-    <row r="86" ht="28" customHeight="1">
-      <c r="A86" s="6" t="inlineStr">
-        <is>
-          <t>EUS-08085</t>
-        </is>
-      </c>
-      <c r="B86" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fusionado de fibra óptica para conectar la casa club con la </t>
-        </is>
-      </c>
-      <c r="C86" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="D86" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E86" s="6" t="inlineStr"/>
-      <c r="F86" s="27" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="G86" s="6" t="inlineStr"/>
-      <c r="H86" s="6" t="inlineStr">
-        <is>
-          <t>Por revisar</t>
-        </is>
-      </c>
-      <c r="I86" s="6" t="inlineStr"/>
-      <c r="J86" s="6" t="inlineStr"/>
-    </row>
-    <row r="87" ht="28" customHeight="1">
-      <c r="A87" s="6" t="inlineStr">
-        <is>
-          <t>EUS-17254</t>
-        </is>
-      </c>
-      <c r="B87" s="6" t="inlineStr">
-        <is>
-          <t>Material de albañilería para el módulo de mantenimiento de v</t>
-        </is>
-      </c>
-      <c r="C87" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="D87" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E87" s="6" t="inlineStr"/>
-      <c r="F87" s="27" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="G87" s="6" t="inlineStr"/>
-      <c r="H87" s="6" t="inlineStr">
-        <is>
-          <t>Por revisar</t>
-        </is>
-      </c>
-      <c r="I87" s="6" t="inlineStr"/>
-      <c r="J87" s="6" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J87"/>
+  <autoFilter ref="A1:J85"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update funding data 2026-04-26
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Recursos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$80</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$77</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -84,13 +84,13 @@
     <font>
       <name val="Leelawadee UI"/>
       <b val="1"/>
-      <color rgb="00DC2626"/>
+      <color rgb="00065F46"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Leelawadee UI"/>
       <b val="1"/>
-      <color rgb="00065F46"/>
+      <color rgb="00DC2626"/>
       <sz val="10"/>
     </font>
     <font>
@@ -166,17 +166,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00065F46"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -268,11 +268,11 @@
     <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -312,8 +312,8 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -679,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M80"/>
+  <dimension ref="A1:M83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -707,7 +707,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 25/04/2026 07:04 - 73 convocatorias - 8 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 26/04/2026 07:18 - 76 convocatorias - 10 nuevas</t>
         </is>
       </c>
     </row>
@@ -2155,12 +2155,12 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
+          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
@@ -2200,7 +2200,7 @@
       </c>
       <c r="K28" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Euro</t>
+          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and inter</t>
         </is>
       </c>
       <c r="L28" s="6" t="inlineStr"/>
@@ -2344,12 +2344,12 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Research and Innovation Actions</t>
+          <t>Programme Cofund Actions</t>
         </is>
       </c>
       <c r="I31" s="10" t="inlineStr">
@@ -2389,7 +2389,7 @@
       </c>
       <c r="K31" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to info</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is estab</t>
         </is>
       </c>
       <c r="L31" s="6" t="inlineStr"/>
@@ -2407,12 +2407,12 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-08</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -2452,7 +2452,7 @@
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and inter</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorpo</t>
         </is>
       </c>
       <c r="L32" s="6" t="inlineStr"/>
@@ -2470,12 +2470,12 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -2500,7 +2500,7 @@
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>Programme Cofund Actions</t>
+          <t xml:space="preserve"> Research and Innovation Actions</t>
         </is>
       </c>
       <c r="I33" s="10" t="inlineStr">
@@ -2515,7 +2515,7 @@
       </c>
       <c r="K33" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is estab</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to info</t>
         </is>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
@@ -2533,12 +2533,12 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="K34" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorpo</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Euro</t>
         </is>
       </c>
       <c r="L34" s="6" t="inlineStr"/>
@@ -4683,11 +4683,7 @@
           <t>PERSONAS JURÍDICAS QUE NO DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
         </is>
       </c>
-      <c r="L72" s="15" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
+      <c r="L72" s="6" t="inlineStr"/>
       <c r="M72" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
@@ -4695,21 +4691,21 @@
       </c>
     </row>
     <row r="73" ht="28" customHeight="1">
-      <c r="A73" s="16" t="inlineStr">
+      <c r="A73" s="15" t="inlineStr">
         <is>
           <t>🟢 Euskadi</t>
         </is>
       </c>
     </row>
     <row r="74" ht="40" customHeight="1">
-      <c r="A74" s="17" t="inlineStr">
+      <c r="A74" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>EUS-13680</t>
+          <t>EUS-39102</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
@@ -4745,7 +4741,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L74" s="15" t="inlineStr">
+      <c r="L74" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4757,14 +4753,14 @@
       </c>
     </row>
     <row r="75" ht="40" customHeight="1">
-      <c r="A75" s="17" t="inlineStr">
+      <c r="A75" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>EUS-61622</t>
+          <t>EUS-45913</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
@@ -4800,7 +4796,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L75" s="15" t="inlineStr">
+      <c r="L75" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4812,19 +4808,19 @@
       </c>
     </row>
     <row r="76" ht="40" customHeight="1">
-      <c r="A76" s="17" t="inlineStr">
+      <c r="A76" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>EUS-84974</t>
+          <t>EUS-94352</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>Servicios de transporte (excluido el transporte de residuos)</t>
+          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta el 01.10.26. Cribado de enfermedades con inteligencia artificial. Espacio de Datos Sanitarios de la UE. Red de Centros para Seguridad de la I</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr">
@@ -4841,12 +4837,12 @@
       <c r="G76" s="6" t="inlineStr"/>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I76" s="11" t="inlineStr">
-        <is>
-          <t>ALTA</t>
+          <t>Ayuda/Subvencion Euskadi</t>
+        </is>
+      </c>
+      <c r="I76" s="8" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
         </is>
       </c>
       <c r="J76" s="6" t="inlineStr"/>
@@ -4855,7 +4851,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L76" s="15" t="inlineStr">
+      <c r="L76" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4867,19 +4863,19 @@
       </c>
     </row>
     <row r="77" ht="40" customHeight="1">
-      <c r="A77" s="17" t="inlineStr">
+      <c r="A77" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>EUS-28416</t>
+          <t>EUS-59045</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta el 01.10.26. Cribado de enfermedades con inteligencia artificial. Espacio de Datos Sanitarios de la UE. Red de Centros para Seguridad de la I</t>
+          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversidad, participación, principios de la UE. Eventos, difusiones e intercambios. Programa de Ciudadanos, Igualdad, Derechos y Valores de la UE (</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
@@ -4910,7 +4906,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L77" s="15" t="inlineStr">
+      <c r="L77" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4922,19 +4918,19 @@
       </c>
     </row>
     <row r="78" ht="40" customHeight="1">
-      <c r="A78" s="17" t="inlineStr">
+      <c r="A78" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>EUS-00622</t>
+          <t>EUS-95978</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversidad, participación, principios de la UE. Eventos, difusiones e intercambios. Programa de Ciudadanos, Igualdad, Derechos y Valores de la UE (</t>
+          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el marco de la Intervención Sectorial Vitivinícola del Plan Estratégico (PEPAC) de la Política Agrícola Común de la UE 2023-2027</t>
         </is>
       </c>
       <c r="D78" s="6" t="inlineStr">
@@ -4965,7 +4961,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L78" s="15" t="inlineStr">
+      <c r="L78" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4977,19 +4973,19 @@
       </c>
     </row>
     <row r="79" ht="40" customHeight="1">
-      <c r="A79" s="17" t="inlineStr">
+      <c r="A79" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>EUS-46296</t>
+          <t>EUS-77155</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el marco de la Intervención Sectorial Vitivinícola del Plan Estratégico (PEPAC) de la Política Agrícola Común de la UE 2023-2027</t>
+          <t>Suministro Cajas transporte</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
@@ -5006,7 +5002,7 @@
       <c r="G79" s="6" t="inlineStr"/>
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="I79" s="8" t="inlineStr">
@@ -5020,7 +5016,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L79" s="15" t="inlineStr">
+      <c r="L79" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -5032,19 +5028,19 @@
       </c>
     </row>
     <row r="80" ht="40" customHeight="1">
-      <c r="A80" s="17" t="inlineStr">
+      <c r="A80" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>EUS-86487</t>
+          <t>EUS-03876</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>Servicios de transporte por carretera</t>
+          <t>Suministro Cajas transporte</t>
         </is>
       </c>
       <c r="D80" s="6" t="inlineStr">
@@ -5075,7 +5071,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L80" s="15" t="inlineStr">
+      <c r="L80" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -5086,8 +5082,173 @@
         </is>
       </c>
     </row>
+    <row r="81" ht="40" customHeight="1">
+      <c r="A81" s="16" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>EUS-59668</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>Suministros Agua</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F81" s="6" t="inlineStr"/>
+      <c r="G81" s="6" t="inlineStr"/>
+      <c r="H81" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I81" s="8" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J81" s="6" t="inlineStr"/>
+      <c r="K81" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L81" s="17" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M81" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="40" customHeight="1">
+      <c r="A82" s="16" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>EUS-79620</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>Suministros Agua</t>
+        </is>
+      </c>
+      <c r="D82" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F82" s="6" t="inlineStr"/>
+      <c r="G82" s="6" t="inlineStr"/>
+      <c r="H82" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I82" s="8" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J82" s="6" t="inlineStr"/>
+      <c r="K82" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L82" s="17" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M82" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="40" customHeight="1">
+      <c r="A83" s="16" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>EUS-89421</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="inlineStr">
+        <is>
+          <t>Suministros Agua</t>
+        </is>
+      </c>
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E83" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F83" s="6" t="inlineStr"/>
+      <c r="G83" s="6" t="inlineStr"/>
+      <c r="H83" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I83" s="8" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J83" s="6" t="inlineStr"/>
+      <c r="K83" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L83" s="17" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M83" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:M80"/>
+  <autoFilter ref="A4:M83"/>
   <mergeCells count="5">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A5:M5"/>
@@ -5169,6 +5330,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M78" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M79" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M80" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M81" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M82" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M83" r:id="rId76"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5180,7 +5344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1094"/>
+  <dimension ref="A1:F1139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -9958,7 +10122,7 @@
     <row r="331" ht="30" customHeight="1">
       <c r="A331" s="18" t="inlineStr">
         <is>
-          <t>FICHA 23: HORIZON-CL5-2027-01-D1-07</t>
+          <t>FICHA 23: HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="B331" s="19" t="n"/>
@@ -9983,7 +10147,7 @@
       <c r="E332" s="22" t="n"/>
       <c r="F332" s="22" t="n"/>
     </row>
-    <row r="333" ht="45" customHeight="1">
+    <row r="333" ht="20" customHeight="1">
       <c r="A333" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -9991,7 +10155,7 @@
       </c>
       <c r="B333" s="21" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
+          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
         </is>
       </c>
       <c r="C333" s="22" t="n"/>
@@ -10007,7 +10171,7 @@
       </c>
       <c r="B334" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="C334" s="22" t="n"/>
@@ -10119,7 +10283,7 @@
       </c>
       <c r="B341" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Europe and globally, as well as the interaction between different hazards, their cumulative and/or cascading effects.Enhanced seamless prediction and projection modelling and attribution capabilities for extreme events and their likelihood to support preparedness, response and resilience to climate change by EU and national and regional actors. The EU Union Preparedness Strategy, the EU Adaptation Str</t>
+          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and interactions with ecosystems, leading to improved Earth system models;Future climate change scenarios produced in light of past changes in the Earth system, in particular warm climates/high sea-level situations, and abrupt transitions;Identification of thresholds in Earth system components and better characterisation of driving mechanisms and feedbacks that may be responsible for non-linear behaviours,</t>
         </is>
       </c>
       <c r="C341" s="22" t="n"/>
@@ -10163,7 +10327,7 @@
       </c>
       <c r="B344" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-07</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="C344" s="22" t="n"/>
@@ -10606,7 +10770,7 @@
     <row r="376" ht="30" customHeight="1">
       <c r="A376" s="18" t="inlineStr">
         <is>
-          <t>FICHA 26: HORIZON-CL5-2027-01-D1-09</t>
+          <t>FICHA 26: HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="B376" s="19" t="n"/>
@@ -10631,7 +10795,7 @@
       <c r="E377" s="22" t="n"/>
       <c r="F377" s="22" t="n"/>
     </row>
-    <row r="378" ht="45" customHeight="1">
+    <row r="378" ht="20" customHeight="1">
       <c r="A378" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -10639,7 +10803,7 @@
       </c>
       <c r="B378" s="21" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="C378" s="22" t="n"/>
@@ -10655,7 +10819,7 @@
       </c>
       <c r="B379" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C379" s="22" t="n"/>
@@ -10735,7 +10899,7 @@
       </c>
       <c r="B384" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Research and Innovation Actions</t>
+          <t>Programme Cofund Actions</t>
         </is>
       </c>
       <c r="C384" s="22" t="n"/>
@@ -10767,7 +10931,7 @@
       </c>
       <c r="B386" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to inform mitigation action and policy improvements, ensuring a fair transition and social acceptability;Methodologies are developed and improved for ex-ante assessment and ex-post evaluation of greenhouse gas emission reductions from climate policies and measures;Strengthened collaboration and established networks between researchers, policy experts and government officials involved in designing and eva</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is established through development and implementation of the Climate Action pillar of the EU-AU Research and Innovation Partnership on Climate Change and Sustainable Energy (CCSE),[1] in co-design between African and European partners;Reduced fragmentation by aligning the EU, national and multilateral R&amp;amp;I efforts with increased leverage and impact of funding;African scientific, policy and practice com</t>
         </is>
       </c>
       <c r="C386" s="22" t="n"/>
@@ -10811,7 +10975,7 @@
       </c>
       <c r="B389" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-09</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C389" s="22" t="n"/>
@@ -10822,7 +10986,7 @@
     <row r="391" ht="30" customHeight="1">
       <c r="A391" s="18" t="inlineStr">
         <is>
-          <t>FICHA 27: HORIZON-CL5-2027-01-D1-08</t>
+          <t>FICHA 27: HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="B391" s="19" t="n"/>
@@ -10855,7 +11019,7 @@
       </c>
       <c r="B393" s="21" t="inlineStr">
         <is>
-          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="C393" s="22" t="n"/>
@@ -10871,7 +11035,7 @@
       </c>
       <c r="B394" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-08</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C394" s="22" t="n"/>
@@ -10983,7 +11147,7 @@
       </c>
       <c r="B401" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and interactions with ecosystems, leading to improved Earth system models;Future climate change scenarios produced in light of past changes in the Earth system, in particular warm climates/high sea-level situations, and abrupt transitions;Identification of thresholds in Earth system components and better characterisation of driving mechanisms and feedbacks that may be responsible for non-linear behaviours,</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorporation into main EU repositories, such as Climate-ADAPT or the portal of the EU Mission on Adaptation to Climate Change;The risk and adaptation assessment frameworks are improved by better integrating the maladaptation dimension;Guidelines and tools for maladaptation prevention and correction strategies are made available to adaptation stakeholders at relevant scales and inform the design and impl</t>
         </is>
       </c>
       <c r="C401" s="22" t="n"/>
@@ -11027,7 +11191,7 @@
       </c>
       <c r="B404" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-08</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C404" s="22" t="n"/>
@@ -11038,7 +11202,7 @@
     <row r="406" ht="30" customHeight="1">
       <c r="A406" s="18" t="inlineStr">
         <is>
-          <t>FICHA 28: HORIZON-CL5-2027-01-D1-11</t>
+          <t>FICHA 28: HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="B406" s="19" t="n"/>
@@ -11063,7 +11227,7 @@
       <c r="E407" s="22" t="n"/>
       <c r="F407" s="22" t="n"/>
     </row>
-    <row r="408" ht="20" customHeight="1">
+    <row r="408" ht="45" customHeight="1">
       <c r="A408" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -11071,7 +11235,7 @@
       </c>
       <c r="B408" s="21" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
         </is>
       </c>
       <c r="C408" s="22" t="n"/>
@@ -11087,7 +11251,7 @@
       </c>
       <c r="B409" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C409" s="22" t="n"/>
@@ -11167,7 +11331,7 @@
       </c>
       <c r="B414" s="21" t="inlineStr">
         <is>
-          <t>Programme Cofund Actions</t>
+          <t xml:space="preserve"> Research and Innovation Actions</t>
         </is>
       </c>
       <c r="C414" s="22" t="n"/>
@@ -11199,7 +11363,7 @@
       </c>
       <c r="B416" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is established through development and implementation of the Climate Action pillar of the EU-AU Research and Innovation Partnership on Climate Change and Sustainable Energy (CCSE),[1] in co-design between African and European partners;Reduced fragmentation by aligning the EU, national and multilateral R&amp;amp;I efforts with increased leverage and impact of funding;African scientific, policy and practice com</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to inform mitigation action and policy improvements, ensuring a fair transition and social acceptability;Methodologies are developed and improved for ex-ante assessment and ex-post evaluation of greenhouse gas emission reductions from climate policies and measures;Strengthened collaboration and established networks between researchers, policy experts and government officials involved in designing and eva</t>
         </is>
       </c>
       <c r="C416" s="22" t="n"/>
@@ -11243,7 +11407,7 @@
       </c>
       <c r="B419" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-11</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C419" s="22" t="n"/>
@@ -11254,7 +11418,7 @@
     <row r="421" ht="30" customHeight="1">
       <c r="A421" s="18" t="inlineStr">
         <is>
-          <t>FICHA 29: HORIZON-CL5-2027-01-D1-10</t>
+          <t>FICHA 29: HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="B421" s="19" t="n"/>
@@ -11279,7 +11443,7 @@
       <c r="E422" s="22" t="n"/>
       <c r="F422" s="22" t="n"/>
     </row>
-    <row r="423" ht="20" customHeight="1">
+    <row r="423" ht="45" customHeight="1">
       <c r="A423" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -11287,7 +11451,7 @@
       </c>
       <c r="B423" s="21" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
         </is>
       </c>
       <c r="C423" s="22" t="n"/>
@@ -11303,7 +11467,7 @@
       </c>
       <c r="B424" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C424" s="22" t="n"/>
@@ -11415,7 +11579,7 @@
       </c>
       <c r="B431" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorporation into main EU repositories, such as Climate-ADAPT or the portal of the EU Mission on Adaptation to Climate Change;The risk and adaptation assessment frameworks are improved by better integrating the maladaptation dimension;Guidelines and tools for maladaptation prevention and correction strategies are made available to adaptation stakeholders at relevant scales and inform the design and impl</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Europe and globally, as well as the interaction between different hazards, their cumulative and/or cascading effects.Enhanced seamless prediction and projection modelling and attribution capabilities for extreme events and their likelihood to support preparedness, response and resilience to climate change by EU and national and regional actors. The EU Union Preparedness Strategy, the EU Adaptation Str</t>
         </is>
       </c>
       <c r="C431" s="22" t="n"/>
@@ -11459,7 +11623,7 @@
       </c>
       <c r="B434" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-10</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C434" s="22" t="n"/>
@@ -19402,7 +19566,7 @@
     <row r="991" ht="30" customHeight="1">
       <c r="A991" s="18" t="inlineStr">
         <is>
-          <t>FICHA 67: EUS-13680</t>
+          <t>FICHA 67: EUS-39102</t>
         </is>
       </c>
       <c r="B991" s="19" t="n"/>
@@ -19451,7 +19615,7 @@
       </c>
       <c r="B994" s="21" t="inlineStr">
         <is>
-          <t>EUS-13680</t>
+          <t>EUS-39102</t>
         </is>
       </c>
       <c r="C994" s="22" t="n"/>
@@ -19614,7 +19778,7 @@
     <row r="1006" ht="30" customHeight="1">
       <c r="A1006" s="18" t="inlineStr">
         <is>
-          <t>FICHA 68: EUS-61622</t>
+          <t>FICHA 68: EUS-45913</t>
         </is>
       </c>
       <c r="B1006" s="19" t="n"/>
@@ -19663,7 +19827,7 @@
       </c>
       <c r="B1009" s="21" t="inlineStr">
         <is>
-          <t>EUS-61622</t>
+          <t>EUS-45913</t>
         </is>
       </c>
       <c r="C1009" s="22" t="n"/>
@@ -19826,7 +19990,7 @@
     <row r="1021" ht="30" customHeight="1">
       <c r="A1021" s="18" t="inlineStr">
         <is>
-          <t>FICHA 69: EUS-84974</t>
+          <t>FICHA 69: EUS-94352</t>
         </is>
       </c>
       <c r="B1021" s="19" t="n"/>
@@ -19851,7 +20015,7 @@
       <c r="E1022" s="22" t="n"/>
       <c r="F1022" s="22" t="n"/>
     </row>
-    <row r="1023" ht="20" customHeight="1">
+    <row r="1023" ht="45" customHeight="1">
       <c r="A1023" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -19859,7 +20023,7 @@
       </c>
       <c r="B1023" s="21" t="inlineStr">
         <is>
-          <t>Servicios de transporte (excluido el transporte de residuos)</t>
+          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta el 01.10.26. Cribado de enfermedades con inteligencia artificial. Espacio de Datos Sanitarios de la UE. Red de Centros para Seguridad de la I</t>
         </is>
       </c>
       <c r="C1023" s="22" t="n"/>
@@ -19875,7 +20039,7 @@
       </c>
       <c r="B1024" s="21" t="inlineStr">
         <is>
-          <t>EUS-84974</t>
+          <t>EUS-94352</t>
         </is>
       </c>
       <c r="C1024" s="22" t="n"/>
@@ -19951,7 +20115,7 @@
       </c>
       <c r="B1029" s="21" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C1029" s="22" t="n"/>
@@ -20009,9 +20173,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B1033" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ALTA — </t>
+      <c r="B1033" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
         </is>
       </c>
       <c r="C1033" s="22" t="n"/>
@@ -20027,7 +20191,7 @@
       </c>
       <c r="B1034" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/servicios-transporte-excluido-transporte-residuos/expcm506763/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260422digitaleuropekoak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1034" s="22" t="n"/>
@@ -20038,7 +20202,7 @@
     <row r="1036" ht="30" customHeight="1">
       <c r="A1036" s="18" t="inlineStr">
         <is>
-          <t>FICHA 70: EUS-28416</t>
+          <t>FICHA 70: EUS-59045</t>
         </is>
       </c>
       <c r="B1036" s="19" t="n"/>
@@ -20071,7 +20235,7 @@
       </c>
       <c r="B1038" s="21" t="inlineStr">
         <is>
-          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta el 01.10.26. Cribado de enfermedades con inteligencia artificial. Espacio de Datos Sanitarios de la UE. Red de Centros para Seguridad de la I</t>
+          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversidad, participación, principios de la UE. Eventos, difusiones e intercambios. Programa de Ciudadanos, Igualdad, Derechos y Valores de la UE (</t>
         </is>
       </c>
       <c r="C1038" s="22" t="n"/>
@@ -20087,7 +20251,7 @@
       </c>
       <c r="B1039" s="21" t="inlineStr">
         <is>
-          <t>EUS-28416</t>
+          <t>EUS-59045</t>
         </is>
       </c>
       <c r="C1039" s="22" t="n"/>
@@ -20239,7 +20403,7 @@
       </c>
       <c r="B1049" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260422digitaleuropekoak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260408cervhirisareak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1049" s="22" t="n"/>
@@ -20250,7 +20414,7 @@
     <row r="1051" ht="30" customHeight="1">
       <c r="A1051" s="18" t="inlineStr">
         <is>
-          <t>FICHA 71: EUS-00622</t>
+          <t>FICHA 71: EUS-95978</t>
         </is>
       </c>
       <c r="B1051" s="19" t="n"/>
@@ -20283,7 +20447,7 @@
       </c>
       <c r="B1053" s="21" t="inlineStr">
         <is>
-          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversidad, participación, principios de la UE. Eventos, difusiones e intercambios. Programa de Ciudadanos, Igualdad, Derechos y Valores de la UE (</t>
+          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el marco de la Intervención Sectorial Vitivinícola del Plan Estratégico (PEPAC) de la Política Agrícola Común de la UE 2023-2027</t>
         </is>
       </c>
       <c r="C1053" s="22" t="n"/>
@@ -20299,7 +20463,7 @@
       </c>
       <c r="B1054" s="21" t="inlineStr">
         <is>
-          <t>EUS-00622</t>
+          <t>EUS-95978</t>
         </is>
       </c>
       <c r="C1054" s="22" t="n"/>
@@ -20451,7 +20615,7 @@
       </c>
       <c r="B1064" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260408cervhirisareak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/20260407mahastiardogintza/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1064" s="22" t="n"/>
@@ -20462,7 +20626,7 @@
     <row r="1066" ht="30" customHeight="1">
       <c r="A1066" s="18" t="inlineStr">
         <is>
-          <t>FICHA 72: EUS-46296</t>
+          <t>FICHA 72: EUS-77155</t>
         </is>
       </c>
       <c r="B1066" s="19" t="n"/>
@@ -20487,7 +20651,7 @@
       <c r="E1067" s="22" t="n"/>
       <c r="F1067" s="22" t="n"/>
     </row>
-    <row r="1068" ht="45" customHeight="1">
+    <row r="1068" ht="20" customHeight="1">
       <c r="A1068" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -20495,7 +20659,7 @@
       </c>
       <c r="B1068" s="21" t="inlineStr">
         <is>
-          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el marco de la Intervención Sectorial Vitivinícola del Plan Estratégico (PEPAC) de la Política Agrícola Común de la UE 2023-2027</t>
+          <t>Suministro Cajas transporte</t>
         </is>
       </c>
       <c r="C1068" s="22" t="n"/>
@@ -20511,7 +20675,7 @@
       </c>
       <c r="B1069" s="21" t="inlineStr">
         <is>
-          <t>EUS-46296</t>
+          <t>EUS-77155</t>
         </is>
       </c>
       <c r="C1069" s="22" t="n"/>
@@ -20587,7 +20751,7 @@
       </c>
       <c r="B1074" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C1074" s="22" t="n"/>
@@ -20663,7 +20827,7 @@
       </c>
       <c r="B1079" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/20260407mahastiardogintza/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-cajas-transporte/expcm507348/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1079" s="22" t="n"/>
@@ -20674,7 +20838,7 @@
     <row r="1081" ht="30" customHeight="1">
       <c r="A1081" s="18" t="inlineStr">
         <is>
-          <t>FICHA 73: EUS-86487</t>
+          <t>FICHA 73: EUS-03876</t>
         </is>
       </c>
       <c r="B1081" s="19" t="n"/>
@@ -20707,7 +20871,7 @@
       </c>
       <c r="B1083" s="21" t="inlineStr">
         <is>
-          <t>Servicios de transporte por carretera</t>
+          <t>Suministro Cajas transporte</t>
         </is>
       </c>
       <c r="C1083" s="22" t="n"/>
@@ -20723,7 +20887,7 @@
       </c>
       <c r="B1084" s="21" t="inlineStr">
         <is>
-          <t>EUS-86487</t>
+          <t>EUS-03876</t>
         </is>
       </c>
       <c r="C1084" s="22" t="n"/>
@@ -20875,7 +21039,7 @@
       </c>
       <c r="B1094" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/servicios-transporte-carretera/expcm506733/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-cajas-transporte/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1094" s="22" t="n"/>
@@ -20883,8 +21047,644 @@
       <c r="E1094" s="22" t="n"/>
       <c r="F1094" s="22" t="n"/>
     </row>
+    <row r="1096" ht="30" customHeight="1">
+      <c r="A1096" s="18" t="inlineStr">
+        <is>
+          <t>FICHA 74: EUS-59668</t>
+        </is>
+      </c>
+      <c r="B1096" s="19" t="n"/>
+      <c r="C1096" s="19" t="n"/>
+      <c r="D1096" s="19" t="n"/>
+      <c r="E1096" s="19" t="n"/>
+      <c r="F1096" s="19" t="n"/>
+    </row>
+    <row r="1097" ht="20" customHeight="1">
+      <c r="A1097" s="20" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1097" s="21" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1097" s="22" t="n"/>
+      <c r="D1097" s="22" t="n"/>
+      <c r="E1097" s="22" t="n"/>
+      <c r="F1097" s="22" t="n"/>
+    </row>
+    <row r="1098" ht="20" customHeight="1">
+      <c r="A1098" s="20" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1098" s="21" t="inlineStr">
+        <is>
+          <t>Suministros Agua</t>
+        </is>
+      </c>
+      <c r="C1098" s="22" t="n"/>
+      <c r="D1098" s="22" t="n"/>
+      <c r="E1098" s="22" t="n"/>
+      <c r="F1098" s="22" t="n"/>
+    </row>
+    <row r="1099" ht="20" customHeight="1">
+      <c r="A1099" s="20" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1099" s="21" t="inlineStr">
+        <is>
+          <t>EUS-59668</t>
+        </is>
+      </c>
+      <c r="C1099" s="22" t="n"/>
+      <c r="D1099" s="22" t="n"/>
+      <c r="E1099" s="22" t="n"/>
+      <c r="F1099" s="22" t="n"/>
+    </row>
+    <row r="1100" ht="20" customHeight="1">
+      <c r="A1100" s="20" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1100" s="21" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1100" s="22" t="n"/>
+      <c r="D1100" s="22" t="n"/>
+      <c r="E1100" s="22" t="n"/>
+      <c r="F1100" s="22" t="n"/>
+    </row>
+    <row r="1101" ht="20" customHeight="1">
+      <c r="A1101" s="20" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1101" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1101" s="22" t="n"/>
+      <c r="D1101" s="22" t="n"/>
+      <c r="E1101" s="22" t="n"/>
+      <c r="F1101" s="22" t="n"/>
+    </row>
+    <row r="1102" ht="20" customHeight="1">
+      <c r="A1102" s="20" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1102" s="21" t="inlineStr"/>
+      <c r="C1102" s="22" t="n"/>
+      <c r="D1102" s="22" t="n"/>
+      <c r="E1102" s="22" t="n"/>
+      <c r="F1102" s="22" t="n"/>
+    </row>
+    <row r="1103" ht="20" customHeight="1">
+      <c r="A1103" s="20" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1103" s="21" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1103" s="22" t="n"/>
+      <c r="D1103" s="22" t="n"/>
+      <c r="E1103" s="22" t="n"/>
+      <c r="F1103" s="22" t="n"/>
+    </row>
+    <row r="1104" ht="20" customHeight="1">
+      <c r="A1104" s="20" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1104" s="21" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1104" s="22" t="n"/>
+      <c r="D1104" s="22" t="n"/>
+      <c r="E1104" s="22" t="n"/>
+      <c r="F1104" s="22" t="n"/>
+    </row>
+    <row r="1105" ht="20" customHeight="1">
+      <c r="A1105" s="20" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1105" s="21" t="inlineStr"/>
+      <c r="C1105" s="22" t="n"/>
+      <c r="D1105" s="22" t="n"/>
+      <c r="E1105" s="22" t="n"/>
+      <c r="F1105" s="22" t="n"/>
+    </row>
+    <row r="1106" ht="20" customHeight="1">
+      <c r="A1106" s="20" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1106" s="21" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1106" s="22" t="n"/>
+      <c r="D1106" s="22" t="n"/>
+      <c r="E1106" s="22" t="n"/>
+      <c r="F1106" s="22" t="n"/>
+    </row>
+    <row r="1107" ht="20" customHeight="1">
+      <c r="A1107" s="20" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1107" s="21" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1107" s="22" t="n"/>
+      <c r="D1107" s="22" t="n"/>
+      <c r="E1107" s="22" t="n"/>
+      <c r="F1107" s="22" t="n"/>
+    </row>
+    <row r="1108" ht="20" customHeight="1">
+      <c r="A1108" s="20" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1108" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1108" s="22" t="n"/>
+      <c r="D1108" s="22" t="n"/>
+      <c r="E1108" s="22" t="n"/>
+      <c r="F1108" s="22" t="n"/>
+    </row>
+    <row r="1109" ht="45" customHeight="1">
+      <c r="A1109" s="20" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1109" s="23" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/suministros-agua/expcm507335/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1109" s="22" t="n"/>
+      <c r="D1109" s="22" t="n"/>
+      <c r="E1109" s="22" t="n"/>
+      <c r="F1109" s="22" t="n"/>
+    </row>
+    <row r="1111" ht="30" customHeight="1">
+      <c r="A1111" s="18" t="inlineStr">
+        <is>
+          <t>FICHA 75: EUS-79620</t>
+        </is>
+      </c>
+      <c r="B1111" s="19" t="n"/>
+      <c r="C1111" s="19" t="n"/>
+      <c r="D1111" s="19" t="n"/>
+      <c r="E1111" s="19" t="n"/>
+      <c r="F1111" s="19" t="n"/>
+    </row>
+    <row r="1112" ht="20" customHeight="1">
+      <c r="A1112" s="20" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1112" s="21" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1112" s="22" t="n"/>
+      <c r="D1112" s="22" t="n"/>
+      <c r="E1112" s="22" t="n"/>
+      <c r="F1112" s="22" t="n"/>
+    </row>
+    <row r="1113" ht="20" customHeight="1">
+      <c r="A1113" s="20" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1113" s="21" t="inlineStr">
+        <is>
+          <t>Suministros Agua</t>
+        </is>
+      </c>
+      <c r="C1113" s="22" t="n"/>
+      <c r="D1113" s="22" t="n"/>
+      <c r="E1113" s="22" t="n"/>
+      <c r="F1113" s="22" t="n"/>
+    </row>
+    <row r="1114" ht="20" customHeight="1">
+      <c r="A1114" s="20" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1114" s="21" t="inlineStr">
+        <is>
+          <t>EUS-79620</t>
+        </is>
+      </c>
+      <c r="C1114" s="22" t="n"/>
+      <c r="D1114" s="22" t="n"/>
+      <c r="E1114" s="22" t="n"/>
+      <c r="F1114" s="22" t="n"/>
+    </row>
+    <row r="1115" ht="20" customHeight="1">
+      <c r="A1115" s="20" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1115" s="21" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1115" s="22" t="n"/>
+      <c r="D1115" s="22" t="n"/>
+      <c r="E1115" s="22" t="n"/>
+      <c r="F1115" s="22" t="n"/>
+    </row>
+    <row r="1116" ht="20" customHeight="1">
+      <c r="A1116" s="20" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1116" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1116" s="22" t="n"/>
+      <c r="D1116" s="22" t="n"/>
+      <c r="E1116" s="22" t="n"/>
+      <c r="F1116" s="22" t="n"/>
+    </row>
+    <row r="1117" ht="20" customHeight="1">
+      <c r="A1117" s="20" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1117" s="21" t="inlineStr"/>
+      <c r="C1117" s="22" t="n"/>
+      <c r="D1117" s="22" t="n"/>
+      <c r="E1117" s="22" t="n"/>
+      <c r="F1117" s="22" t="n"/>
+    </row>
+    <row r="1118" ht="20" customHeight="1">
+      <c r="A1118" s="20" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1118" s="21" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1118" s="22" t="n"/>
+      <c r="D1118" s="22" t="n"/>
+      <c r="E1118" s="22" t="n"/>
+      <c r="F1118" s="22" t="n"/>
+    </row>
+    <row r="1119" ht="20" customHeight="1">
+      <c r="A1119" s="20" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1119" s="21" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1119" s="22" t="n"/>
+      <c r="D1119" s="22" t="n"/>
+      <c r="E1119" s="22" t="n"/>
+      <c r="F1119" s="22" t="n"/>
+    </row>
+    <row r="1120" ht="20" customHeight="1">
+      <c r="A1120" s="20" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1120" s="21" t="inlineStr"/>
+      <c r="C1120" s="22" t="n"/>
+      <c r="D1120" s="22" t="n"/>
+      <c r="E1120" s="22" t="n"/>
+      <c r="F1120" s="22" t="n"/>
+    </row>
+    <row r="1121" ht="20" customHeight="1">
+      <c r="A1121" s="20" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1121" s="21" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1121" s="22" t="n"/>
+      <c r="D1121" s="22" t="n"/>
+      <c r="E1121" s="22" t="n"/>
+      <c r="F1121" s="22" t="n"/>
+    </row>
+    <row r="1122" ht="20" customHeight="1">
+      <c r="A1122" s="20" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1122" s="21" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1122" s="22" t="n"/>
+      <c r="D1122" s="22" t="n"/>
+      <c r="E1122" s="22" t="n"/>
+      <c r="F1122" s="22" t="n"/>
+    </row>
+    <row r="1123" ht="20" customHeight="1">
+      <c r="A1123" s="20" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1123" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1123" s="22" t="n"/>
+      <c r="D1123" s="22" t="n"/>
+      <c r="E1123" s="22" t="n"/>
+      <c r="F1123" s="22" t="n"/>
+    </row>
+    <row r="1124" ht="45" customHeight="1">
+      <c r="A1124" s="20" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1124" s="23" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/suministros-agua/expcm507334/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1124" s="22" t="n"/>
+      <c r="D1124" s="22" t="n"/>
+      <c r="E1124" s="22" t="n"/>
+      <c r="F1124" s="22" t="n"/>
+    </row>
+    <row r="1126" ht="30" customHeight="1">
+      <c r="A1126" s="18" t="inlineStr">
+        <is>
+          <t>FICHA 76: EUS-89421</t>
+        </is>
+      </c>
+      <c r="B1126" s="19" t="n"/>
+      <c r="C1126" s="19" t="n"/>
+      <c r="D1126" s="19" t="n"/>
+      <c r="E1126" s="19" t="n"/>
+      <c r="F1126" s="19" t="n"/>
+    </row>
+    <row r="1127" ht="20" customHeight="1">
+      <c r="A1127" s="20" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1127" s="21" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1127" s="22" t="n"/>
+      <c r="D1127" s="22" t="n"/>
+      <c r="E1127" s="22" t="n"/>
+      <c r="F1127" s="22" t="n"/>
+    </row>
+    <row r="1128" ht="20" customHeight="1">
+      <c r="A1128" s="20" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1128" s="21" t="inlineStr">
+        <is>
+          <t>Suministros Agua</t>
+        </is>
+      </c>
+      <c r="C1128" s="22" t="n"/>
+      <c r="D1128" s="22" t="n"/>
+      <c r="E1128" s="22" t="n"/>
+      <c r="F1128" s="22" t="n"/>
+    </row>
+    <row r="1129" ht="20" customHeight="1">
+      <c r="A1129" s="20" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1129" s="21" t="inlineStr">
+        <is>
+          <t>EUS-89421</t>
+        </is>
+      </c>
+      <c r="C1129" s="22" t="n"/>
+      <c r="D1129" s="22" t="n"/>
+      <c r="E1129" s="22" t="n"/>
+      <c r="F1129" s="22" t="n"/>
+    </row>
+    <row r="1130" ht="20" customHeight="1">
+      <c r="A1130" s="20" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1130" s="21" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1130" s="22" t="n"/>
+      <c r="D1130" s="22" t="n"/>
+      <c r="E1130" s="22" t="n"/>
+      <c r="F1130" s="22" t="n"/>
+    </row>
+    <row r="1131" ht="20" customHeight="1">
+      <c r="A1131" s="20" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1131" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1131" s="22" t="n"/>
+      <c r="D1131" s="22" t="n"/>
+      <c r="E1131" s="22" t="n"/>
+      <c r="F1131" s="22" t="n"/>
+    </row>
+    <row r="1132" ht="20" customHeight="1">
+      <c r="A1132" s="20" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1132" s="21" t="inlineStr"/>
+      <c r="C1132" s="22" t="n"/>
+      <c r="D1132" s="22" t="n"/>
+      <c r="E1132" s="22" t="n"/>
+      <c r="F1132" s="22" t="n"/>
+    </row>
+    <row r="1133" ht="20" customHeight="1">
+      <c r="A1133" s="20" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1133" s="21" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1133" s="22" t="n"/>
+      <c r="D1133" s="22" t="n"/>
+      <c r="E1133" s="22" t="n"/>
+      <c r="F1133" s="22" t="n"/>
+    </row>
+    <row r="1134" ht="20" customHeight="1">
+      <c r="A1134" s="20" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1134" s="21" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1134" s="22" t="n"/>
+      <c r="D1134" s="22" t="n"/>
+      <c r="E1134" s="22" t="n"/>
+      <c r="F1134" s="22" t="n"/>
+    </row>
+    <row r="1135" ht="20" customHeight="1">
+      <c r="A1135" s="20" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1135" s="21" t="inlineStr"/>
+      <c r="C1135" s="22" t="n"/>
+      <c r="D1135" s="22" t="n"/>
+      <c r="E1135" s="22" t="n"/>
+      <c r="F1135" s="22" t="n"/>
+    </row>
+    <row r="1136" ht="20" customHeight="1">
+      <c r="A1136" s="20" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1136" s="21" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1136" s="22" t="n"/>
+      <c r="D1136" s="22" t="n"/>
+      <c r="E1136" s="22" t="n"/>
+      <c r="F1136" s="22" t="n"/>
+    </row>
+    <row r="1137" ht="20" customHeight="1">
+      <c r="A1137" s="20" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1137" s="21" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1137" s="22" t="n"/>
+      <c r="D1137" s="22" t="n"/>
+      <c r="E1137" s="22" t="n"/>
+      <c r="F1137" s="22" t="n"/>
+    </row>
+    <row r="1138" ht="20" customHeight="1">
+      <c r="A1138" s="20" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1138" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1138" s="22" t="n"/>
+      <c r="D1138" s="22" t="n"/>
+      <c r="E1138" s="22" t="n"/>
+      <c r="F1138" s="22" t="n"/>
+    </row>
+    <row r="1139" ht="45" customHeight="1">
+      <c r="A1139" s="20" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1139" s="23" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/suministros-agua/expcm507333/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1139" s="22" t="n"/>
+      <c r="D1139" s="22" t="n"/>
+      <c r="E1139" s="22" t="n"/>
+      <c r="F1139" s="22" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="1022">
+  <mergeCells count="1064">
     <mergeCell ref="B679:F679"/>
     <mergeCell ref="B666:F666"/>
     <mergeCell ref="B964:F964"/>
@@ -20928,7 +21728,9 @@
     <mergeCell ref="B342:F342"/>
     <mergeCell ref="B578:F578"/>
     <mergeCell ref="A541:F541"/>
+    <mergeCell ref="B1099:F1099"/>
     <mergeCell ref="B515:F515"/>
+    <mergeCell ref="B1128:F1128"/>
     <mergeCell ref="A841:F841"/>
     <mergeCell ref="B158:F158"/>
     <mergeCell ref="B1094:F1094"/>
@@ -20937,6 +21739,7 @@
     <mergeCell ref="B894:F894"/>
     <mergeCell ref="B133:F133"/>
     <mergeCell ref="B959:F959"/>
+    <mergeCell ref="B1130:F1130"/>
     <mergeCell ref="B369:F369"/>
     <mergeCell ref="B667:F667"/>
     <mergeCell ref="B418:F418"/>
@@ -20963,11 +21766,13 @@
     <mergeCell ref="B662:F662"/>
     <mergeCell ref="B718:F718"/>
     <mergeCell ref="B889:F889"/>
+    <mergeCell ref="B1131:F1131"/>
     <mergeCell ref="B72:F72"/>
     <mergeCell ref="B954:F954"/>
     <mergeCell ref="B199:F199"/>
     <mergeCell ref="B370:F370"/>
     <mergeCell ref="B1025:F1025"/>
+    <mergeCell ref="B1112:F1112"/>
     <mergeCell ref="B291:F291"/>
     <mergeCell ref="B655:F655"/>
     <mergeCell ref="B974:F974"/>
@@ -21009,6 +21814,7 @@
     <mergeCell ref="B83:F83"/>
     <mergeCell ref="B254:F254"/>
     <mergeCell ref="B909:F909"/>
+    <mergeCell ref="B1105:F1105"/>
     <mergeCell ref="B319:F319"/>
     <mergeCell ref="B490:F490"/>
     <mergeCell ref="B604:F604"/>
@@ -21040,6 +21846,7 @@
     <mergeCell ref="B530:F530"/>
     <mergeCell ref="B726:F726"/>
     <mergeCell ref="B962:F962"/>
+    <mergeCell ref="B1133:F1133"/>
     <mergeCell ref="A886:F886"/>
     <mergeCell ref="B505:F505"/>
     <mergeCell ref="B1060:F1060"/>
@@ -21075,6 +21882,7 @@
     <mergeCell ref="B752:F752"/>
     <mergeCell ref="B1070:F1070"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B1115:F1115"/>
     <mergeCell ref="B325:F325"/>
     <mergeCell ref="B154:F154"/>
     <mergeCell ref="A271:F271"/>
@@ -21108,6 +21916,8 @@
     <mergeCell ref="B518:F518"/>
     <mergeCell ref="B562:F562"/>
     <mergeCell ref="B689:F689"/>
+    <mergeCell ref="B1121:F1121"/>
+    <mergeCell ref="B1123:F1123"/>
     <mergeCell ref="B86:F86"/>
     <mergeCell ref="B912:F912"/>
     <mergeCell ref="B1083:F1083"/>
@@ -21159,6 +21969,7 @@
     <mergeCell ref="B979:F979"/>
     <mergeCell ref="B381:F381"/>
     <mergeCell ref="B552:F552"/>
+    <mergeCell ref="A1111:F1111"/>
     <mergeCell ref="B1084:F1084"/>
     <mergeCell ref="A976:F976"/>
     <mergeCell ref="B170:F170"/>
@@ -21192,6 +22003,7 @@
     <mergeCell ref="B92:F92"/>
     <mergeCell ref="B984:F984"/>
     <mergeCell ref="A226:F226"/>
+    <mergeCell ref="B1124:F1124"/>
     <mergeCell ref="B394:F394"/>
     <mergeCell ref="B692:F692"/>
     <mergeCell ref="A931:F931"/>
@@ -21222,6 +22034,7 @@
     <mergeCell ref="B817:F817"/>
     <mergeCell ref="B944:F944"/>
     <mergeCell ref="B56:F56"/>
+    <mergeCell ref="B1102:F1102"/>
     <mergeCell ref="B43:F43"/>
     <mergeCell ref="B176:F176"/>
     <mergeCell ref="B347:F347"/>
@@ -21237,7 +22050,9 @@
     <mergeCell ref="B881:F881"/>
     <mergeCell ref="B1068:F1068"/>
     <mergeCell ref="B868:F868"/>
+    <mergeCell ref="B1117:F1117"/>
     <mergeCell ref="B107:F107"/>
+    <mergeCell ref="B1104:F1104"/>
     <mergeCell ref="B641:F641"/>
     <mergeCell ref="B57:F57"/>
     <mergeCell ref="B883:F883"/>
@@ -21263,6 +22078,7 @@
     <mergeCell ref="B999:F999"/>
     <mergeCell ref="B1061:F1061"/>
     <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B1097:F1097"/>
     <mergeCell ref="A46:F46"/>
     <mergeCell ref="B507:F507"/>
     <mergeCell ref="B62:F62"/>
@@ -21310,6 +22126,7 @@
     <mergeCell ref="B1018:F1018"/>
     <mergeCell ref="B624:F624"/>
     <mergeCell ref="B428:F428"/>
+    <mergeCell ref="B1118:F1118"/>
     <mergeCell ref="B284:F284"/>
     <mergeCell ref="B222:F222"/>
     <mergeCell ref="B344:F344"/>
@@ -21321,6 +22138,7 @@
     <mergeCell ref="B123:F123"/>
     <mergeCell ref="B949:F949"/>
     <mergeCell ref="B1011:F1011"/>
+    <mergeCell ref="B1120:F1120"/>
     <mergeCell ref="B50:F50"/>
     <mergeCell ref="B221:F221"/>
     <mergeCell ref="B110:F110"/>
@@ -21337,6 +22155,7 @@
     <mergeCell ref="B802:F802"/>
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B789:F789"/>
+    <mergeCell ref="B1136:F1136"/>
     <mergeCell ref="B248:F248"/>
     <mergeCell ref="B297:F297"/>
     <mergeCell ref="B813:F813"/>
@@ -21356,9 +22175,11 @@
     <mergeCell ref="B815:F815"/>
     <mergeCell ref="B597:F597"/>
     <mergeCell ref="B1064:F1064"/>
+    <mergeCell ref="B1113:F1113"/>
     <mergeCell ref="B103:F103"/>
     <mergeCell ref="B78:F78"/>
     <mergeCell ref="B833:F833"/>
+    <mergeCell ref="B1100:F1100"/>
     <mergeCell ref="B205:F205"/>
     <mergeCell ref="B339:F339"/>
     <mergeCell ref="B314:F314"/>
@@ -21454,6 +22275,7 @@
     <mergeCell ref="B305:F305"/>
     <mergeCell ref="B816:F816"/>
     <mergeCell ref="B918:F918"/>
+    <mergeCell ref="B1114:F1114"/>
     <mergeCell ref="B607:F607"/>
     <mergeCell ref="B663:F663"/>
     <mergeCell ref="B1049:F1049"/>
@@ -21464,6 +22286,7 @@
     <mergeCell ref="B442:F442"/>
     <mergeCell ref="B242:F242"/>
     <mergeCell ref="B880:F880"/>
+    <mergeCell ref="B1116:F1116"/>
     <mergeCell ref="B671:F671"/>
     <mergeCell ref="B969:F969"/>
     <mergeCell ref="B907:F907"/>
@@ -21481,12 +22304,15 @@
     <mergeCell ref="B760:F760"/>
     <mergeCell ref="B437:F437"/>
     <mergeCell ref="B852:F852"/>
+    <mergeCell ref="B1119:F1119"/>
     <mergeCell ref="B333:F333"/>
+    <mergeCell ref="B1098:F1098"/>
     <mergeCell ref="B898:F898"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="B520:F520"/>
     <mergeCell ref="B958:F958"/>
     <mergeCell ref="B308:F308"/>
+    <mergeCell ref="B1134:F1134"/>
     <mergeCell ref="B854:F854"/>
     <mergeCell ref="B99:F99"/>
     <mergeCell ref="B737:F737"/>
@@ -21505,12 +22331,14 @@
     <mergeCell ref="B372:F372"/>
     <mergeCell ref="B1071:F1071"/>
     <mergeCell ref="B608:F608"/>
+    <mergeCell ref="B1127:F1127"/>
     <mergeCell ref="B595:F595"/>
     <mergeCell ref="B1037:F1037"/>
     <mergeCell ref="B722:F722"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="A856:F856"/>
     <mergeCell ref="B893:F893"/>
+    <mergeCell ref="B1129:F1129"/>
     <mergeCell ref="B374:F374"/>
     <mergeCell ref="B659:F659"/>
     <mergeCell ref="B830:F830"/>
@@ -21579,6 +22407,7 @@
     <mergeCell ref="B309:F309"/>
     <mergeCell ref="A316:F316"/>
     <mergeCell ref="B380:F380"/>
+    <mergeCell ref="B1135:F1135"/>
     <mergeCell ref="A1081:F1081"/>
     <mergeCell ref="B100:F100"/>
     <mergeCell ref="B336:F336"/>
@@ -21588,10 +22417,12 @@
     <mergeCell ref="B140:F140"/>
     <mergeCell ref="B115:F115"/>
     <mergeCell ref="B382:F382"/>
+    <mergeCell ref="A1096:F1096"/>
     <mergeCell ref="B680:F680"/>
     <mergeCell ref="A376:F376"/>
     <mergeCell ref="B102:F102"/>
     <mergeCell ref="B674:F674"/>
+    <mergeCell ref="B1137:F1137"/>
     <mergeCell ref="B400:F400"/>
     <mergeCell ref="B698:F698"/>
     <mergeCell ref="B832:F832"/>
@@ -21604,6 +22435,7 @@
     <mergeCell ref="B598:F598"/>
     <mergeCell ref="B402:F402"/>
     <mergeCell ref="B669:F669"/>
+    <mergeCell ref="B1138:F1138"/>
     <mergeCell ref="B377:F377"/>
     <mergeCell ref="A451:F451"/>
     <mergeCell ref="B29:F29"/>
@@ -21810,11 +22642,14 @@
     <mergeCell ref="B409:F409"/>
     <mergeCell ref="B580:F580"/>
     <mergeCell ref="B920:F920"/>
+    <mergeCell ref="B1108:F1108"/>
     <mergeCell ref="B711:F711"/>
     <mergeCell ref="B1009:F1009"/>
     <mergeCell ref="B48:F48"/>
+    <mergeCell ref="B1101:F1101"/>
     <mergeCell ref="B582:F582"/>
     <mergeCell ref="B849:F849"/>
+    <mergeCell ref="B1132:F1132"/>
     <mergeCell ref="B73:F73"/>
     <mergeCell ref="B371:F371"/>
     <mergeCell ref="B638:F638"/>
@@ -21827,6 +22662,7 @@
     <mergeCell ref="A676:F676"/>
     <mergeCell ref="B137:F137"/>
     <mergeCell ref="B379:F379"/>
+    <mergeCell ref="B1106:F1106"/>
     <mergeCell ref="B702:F702"/>
     <mergeCell ref="B677:F677"/>
     <mergeCell ref="B640:F640"/>
@@ -21857,6 +22693,7 @@
     <mergeCell ref="B66:F66"/>
     <mergeCell ref="B326:F326"/>
     <mergeCell ref="B793:F793"/>
+    <mergeCell ref="B1103:F1103"/>
     <mergeCell ref="A406:F406"/>
     <mergeCell ref="B951:F951"/>
     <mergeCell ref="B130:F130"/>
@@ -21875,6 +22712,7 @@
     <mergeCell ref="B132:F132"/>
     <mergeCell ref="B425:F425"/>
     <mergeCell ref="B430:F430"/>
+    <mergeCell ref="B1107:F1107"/>
     <mergeCell ref="B1045:F1045"/>
     <mergeCell ref="B119:F119"/>
     <mergeCell ref="B290:F290"/>
@@ -21885,10 +22723,13 @@
     <mergeCell ref="B824:F824"/>
     <mergeCell ref="B1017:F1017"/>
     <mergeCell ref="B367:F367"/>
+    <mergeCell ref="B1122:F1122"/>
     <mergeCell ref="B427:F427"/>
+    <mergeCell ref="B1139:F1139"/>
     <mergeCell ref="B112:F112"/>
     <mergeCell ref="B283:F283"/>
     <mergeCell ref="B354:F354"/>
+    <mergeCell ref="B1109:F1109"/>
     <mergeCell ref="B348:F348"/>
     <mergeCell ref="B519:F519"/>
     <mergeCell ref="B419:F419"/>
@@ -21904,6 +22745,7 @@
     <mergeCell ref="B648:F648"/>
     <mergeCell ref="B64:F64"/>
     <mergeCell ref="B51:F51"/>
+    <mergeCell ref="A1126:F1126"/>
     <mergeCell ref="B443:F443"/>
     <mergeCell ref="A196:F196"/>
     <mergeCell ref="B237:F237"/>
@@ -21982,6 +22824,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1064" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1079" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1094" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1109" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1124" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1139" r:id="rId76"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -21993,7 +22838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J74"/>
+  <dimension ref="A1:J77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -22939,12 +23784,12 @@
     <row r="24" ht="28" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme</t>
+          <t>Palaeoclimate science for a better understanding of Earth sy</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -23059,12 +23904,12 @@
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform cl</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
@@ -23099,12 +23944,12 @@
     <row r="28" ht="28" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-08</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Palaeoclimate science for a better understanding of Earth sy</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -23139,12 +23984,12 @@
     <row r="29" ht="28" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Assessing the performance of policy instruments to inform cl</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
@@ -23179,12 +24024,12 @@
     <row r="30" ht="28" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Advancing understanding, modelling and prediction of extreme</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -24591,7 +25436,7 @@
     <row r="68" ht="28" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>EUS-13680</t>
+          <t>EUS-39102</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
@@ -24627,7 +25472,7 @@
     <row r="69" ht="28" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>EUS-61622</t>
+          <t>EUS-45913</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
@@ -24663,12 +25508,12 @@
     <row r="70" ht="28" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>EUS-84974</t>
+          <t>EUS-94352</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>Servicios de transporte (excluido el transporte de residuos)</t>
+          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta e</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -24684,7 +25529,7 @@
       <c r="E70" s="6" t="inlineStr"/>
       <c r="F70" s="27" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>MEDIA</t>
         </is>
       </c>
       <c r="G70" s="6" t="inlineStr"/>
@@ -24699,12 +25544,12 @@
     <row r="71" ht="28" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>EUS-28416</t>
+          <t>EUS-59045</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta e</t>
+          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversi</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -24735,12 +25580,12 @@
     <row r="72" ht="28" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>EUS-00622</t>
+          <t>EUS-95978</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversi</t>
+          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el ma</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -24771,12 +25616,12 @@
     <row r="73" ht="28" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>EUS-46296</t>
+          <t>EUS-77155</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el ma</t>
+          <t>Suministro Cajas transporte</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -24807,12 +25652,12 @@
     <row r="74" ht="28" customHeight="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>EUS-86487</t>
+          <t>EUS-03876</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>Servicios de transporte por carretera</t>
+          <t>Suministro Cajas transporte</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
@@ -24840,8 +25685,116 @@
       <c r="I74" s="6" t="inlineStr"/>
       <c r="J74" s="6" t="inlineStr"/>
     </row>
+    <row r="75" ht="28" customHeight="1">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>EUS-59668</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>Suministros Agua</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D75" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E75" s="6" t="inlineStr"/>
+      <c r="F75" s="27" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G75" s="6" t="inlineStr"/>
+      <c r="H75" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I75" s="6" t="inlineStr"/>
+      <c r="J75" s="6" t="inlineStr"/>
+    </row>
+    <row r="76" ht="28" customHeight="1">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>EUS-79620</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>Suministros Agua</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E76" s="6" t="inlineStr"/>
+      <c r="F76" s="27" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G76" s="6" t="inlineStr"/>
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I76" s="6" t="inlineStr"/>
+      <c r="J76" s="6" t="inlineStr"/>
+    </row>
+    <row r="77" ht="28" customHeight="1">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>EUS-89421</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>Suministros Agua</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="inlineStr"/>
+      <c r="F77" s="27" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G77" s="6" t="inlineStr"/>
+      <c r="H77" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I77" s="6" t="inlineStr"/>
+      <c r="J77" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J74"/>
+  <autoFilter ref="A1:J77"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update funding data 2026-04-28
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Recursos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$87</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$76</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -679,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M87"/>
+  <dimension ref="A1:M82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -707,7 +707,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 27/04/2026 08:04 - 80 convocatorias - 15 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 28/04/2026 08:10 - 75 convocatorias - 11 nuevas</t>
         </is>
       </c>
     </row>
@@ -2104,12 +2104,12 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-08</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
+          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and inter</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Euro</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr"/>
@@ -2293,12 +2293,12 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -2323,7 +2323,7 @@
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>Programme Cofund Actions</t>
+          <t xml:space="preserve"> Research and Innovation Actions</t>
         </is>
       </c>
       <c r="I30" s="10" t="inlineStr">
@@ -2338,7 +2338,7 @@
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is estab</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to info</t>
         </is>
       </c>
       <c r="L30" s="6" t="inlineStr"/>
@@ -2356,12 +2356,12 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -2401,7 +2401,7 @@
       </c>
       <c r="K31" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorpo</t>
+          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and inter</t>
         </is>
       </c>
       <c r="L31" s="6" t="inlineStr"/>
@@ -2419,12 +2419,12 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -2449,7 +2449,7 @@
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Research and Innovation Actions</t>
+          <t>Programme Cofund Actions</t>
         </is>
       </c>
       <c r="I32" s="10" t="inlineStr">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to info</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is estab</t>
         </is>
       </c>
       <c r="L32" s="6" t="inlineStr"/>
@@ -2482,12 +2482,12 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -2527,7 +2527,7 @@
       </c>
       <c r="K33" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Euro</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorpo</t>
         </is>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
@@ -4529,12 +4529,12 @@
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>BDNS-901096</t>
+          <t>BDNS-901505</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>Ayudas económicas al desarrollo y producción de proyectos audiovisuales y a la escritura de guiones. Año 2026</t>
+          <t>CONVENIO DE SUBVENCIÓN NOMINATIVA PARA LA ASOCIACIÓN KULTURA KALEAN PARA KORTERRAZA 2026</t>
         </is>
       </c>
       <c r="D70" s="6" t="inlineStr">
@@ -4549,12 +4549,12 @@
       </c>
       <c r="F70" s="6" t="inlineStr">
         <is>
-          <t>01/06/2026</t>
+          <t>31/12/2026</t>
         </is>
       </c>
       <c r="G70" s="6" t="inlineStr">
         <is>
-          <t>110,000.00 EUR</t>
+          <t>25,000.00 EUR</t>
         </is>
       </c>
       <c r="H70" s="6" t="inlineStr">
@@ -4570,7 +4570,7 @@
       <c r="J70" s="6" t="inlineStr"/>
       <c r="K70" s="6" t="inlineStr">
         <is>
-          <t>PYME Y PERSONAS FÍSICAS QUE DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
+          <t>PERSONAS JURÍDICAS QUE NO DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
         </is>
       </c>
       <c r="L70" s="6" t="inlineStr"/>
@@ -4580,69 +4580,65 @@
         </is>
       </c>
     </row>
-    <row r="71" ht="40" customHeight="1">
-      <c r="A71" s="14" t="inlineStr">
-        <is>
-          <t>España</t>
-        </is>
-      </c>
-      <c r="B71" s="6" t="inlineStr">
-        <is>
-          <t>BDNS-901505</t>
-        </is>
-      </c>
-      <c r="C71" s="6" t="inlineStr">
-        <is>
-          <t>CONVENIO DE SUBVENCIÓN NOMINATIVA PARA LA ASOCIACIÓN KULTURA KALEAN PARA KORTERRAZA 2026</t>
-        </is>
-      </c>
-      <c r="D71" s="6" t="inlineStr">
-        <is>
-          <t>VITORIA-GASTEIZ</t>
-        </is>
-      </c>
-      <c r="E71" s="7" t="inlineStr">
+    <row r="71" ht="28" customHeight="1">
+      <c r="A71" s="15" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="40" customHeight="1">
+      <c r="A72" s="16" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>EUS-74664</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>LIFE 2026. Medio ambiente. Ayudas de 4 subprogramas, de naturaleza y biodiversidad, circularidad y calidad de vida, cambio climático y transición energética. Con inscripción abierta para jornadas info</t>
+        </is>
+      </c>
+      <c r="D72" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F71" s="6" t="inlineStr">
-        <is>
-          <t>31/12/2026</t>
-        </is>
-      </c>
-      <c r="G71" s="6" t="inlineStr">
-        <is>
-          <t>25,000.00 EUR</t>
-        </is>
-      </c>
-      <c r="H71" s="6" t="inlineStr">
-        <is>
-          <t>Subvencion Nacional</t>
-        </is>
-      </c>
-      <c r="I71" s="8" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="J71" s="6" t="inlineStr"/>
-      <c r="K71" s="6" t="inlineStr">
-        <is>
-          <t>PERSONAS JURÍDICAS QUE NO DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
-        </is>
-      </c>
-      <c r="L71" s="6" t="inlineStr"/>
-      <c r="M71" s="9" t="inlineStr">
+      <c r="F72" s="6" t="inlineStr"/>
+      <c r="G72" s="6" t="inlineStr"/>
+      <c r="H72" s="6" t="inlineStr">
+        <is>
+          <t>Ayuda/Subvencion Euskadi</t>
+        </is>
+      </c>
+      <c r="I72" s="11" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J72" s="6" t="inlineStr"/>
+      <c r="K72" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L72" s="17" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M72" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="28" customHeight="1">
-      <c r="A72" s="15" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
         </is>
       </c>
     </row>
@@ -4654,12 +4650,12 @@
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>EUS-92454</t>
+          <t>EUS-70680</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Suministro de licencias de software para las plataformas Mailchimp, Zapier y SurveyMonkey, destinadas a la comunicación digital, automatización de procesos y gestión de encuestas de Bilbao Zerbitzuak </t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
@@ -4676,12 +4672,12 @@
       <c r="G73" s="6" t="inlineStr"/>
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I73" s="12" t="inlineStr">
-        <is>
-          <t>MUY ALTA</t>
+          <t>Ayuda/Subvencion Euskadi</t>
+        </is>
+      </c>
+      <c r="I73" s="11" t="inlineStr">
+        <is>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="J73" s="6" t="inlineStr"/>
@@ -4709,12 +4705,12 @@
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>EUS-75183</t>
+          <t>EUS-31421</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>LIFE 2026. Medio ambiente. Ayudas de 4 subprogramas, de naturaleza y biodiversidad, circularidad y calidad de vida, cambio climático y transición energética. Con inscripción abierta para jornadas info</t>
+          <t>Contrato mixto de suministro y obra para la sustitución y actualización de la instalación de climatización del polideportivo con piscina, Artebe, de Sondika.</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr">
@@ -4731,7 +4727,7 @@
       <c r="G74" s="6" t="inlineStr"/>
       <c r="H74" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="I74" s="11" t="inlineStr">
@@ -4764,12 +4760,12 @@
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>EUS-02830</t>
+          <t>EUS-13213</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
+          <t>Mantenimiento de las instalacioens  de climatización, ACS y grupo electrógeno del  centro de día Nafarroa, a excepción de los  equipos de climatización de la cafetería</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
@@ -4786,7 +4782,7 @@
       <c r="G75" s="6" t="inlineStr"/>
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="I75" s="11" t="inlineStr">
@@ -4819,12 +4815,13 @@
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>EUS-31407</t>
+          <t>EUS-28151</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>asistencia tecnica para el desarrollo de la campaña informativa para impulsar la recogida selectiva de residuos en Lasarte-Oria</t>
+          <t>Servicio de recogida separada y clasificación de residuos de productos textiles o de calzado posconsumo y el servicio de recogida separada de residuos de pilas y acumuladores portátiles usados
+(Contr</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr">
@@ -4874,7 +4871,7 @@
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>EUS-74304</t>
+          <t>EUS-86678</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
@@ -4929,7 +4926,7 @@
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>EUS-96161</t>
+          <t>EUS-71437</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
@@ -4984,7 +4981,7 @@
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>EUS-04369</t>
+          <t>EUS-71705</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
@@ -5039,12 +5036,12 @@
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>EUS-86318</t>
+          <t>EUS-79070</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>Contratación de los servicios de formación en materia ESG, realización de diagnósticos ESG y hojas de ruta en sostenibilidad, así como de los servicios de medición de impacto social en proyectos empre</t>
+          <t>Servicio de recogida de animales domésticos</t>
         </is>
       </c>
       <c r="D80" s="6" t="inlineStr">
@@ -5094,12 +5091,12 @@
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>EUS-63953</t>
+          <t>EUS-53277</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>Enajenación, mediante subasta, de la parcela urbana1-819 de Zambrana</t>
+          <t>Servicio de transporte para el programa Ibiliaz Ezagutu de primavera</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
@@ -5149,12 +5146,12 @@
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>EUS-29174</t>
+          <t>EUS-45140</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>Elaboración, transporte y entrega de comidas preparadas y prestaciones complementarias para el funcionamiento de los comedores de gestión directa en diversos centros públicos dependientes del Departam</t>
+          <t>Cubierta de patio CEIP BAGATZA HLHI, Barakaldo (Bizkaia)</t>
         </is>
       </c>
       <c r="D82" s="6" t="inlineStr">
@@ -5196,289 +5193,14 @@
         </is>
       </c>
     </row>
-    <row r="83" ht="40" customHeight="1">
-      <c r="A83" s="16" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="B83" s="6" t="inlineStr">
-        <is>
-          <t>EUS-05384</t>
-        </is>
-      </c>
-      <c r="C83" s="6" t="inlineStr">
-        <is>
-          <t>Suministro Cajas transporte</t>
-        </is>
-      </c>
-      <c r="D83" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="E83" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F83" s="6" t="inlineStr"/>
-      <c r="G83" s="6" t="inlineStr"/>
-      <c r="H83" s="6" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I83" s="8" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="J83" s="6" t="inlineStr"/>
-      <c r="K83" s="6" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="L83" s="17" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="M83" s="9" t="inlineStr">
-        <is>
-          <t>Ver</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="40" customHeight="1">
-      <c r="A84" s="16" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="B84" s="6" t="inlineStr">
-        <is>
-          <t>EUS-34859</t>
-        </is>
-      </c>
-      <c r="C84" s="6" t="inlineStr">
-        <is>
-          <t>Suministro Cajas transporte</t>
-        </is>
-      </c>
-      <c r="D84" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="E84" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F84" s="6" t="inlineStr"/>
-      <c r="G84" s="6" t="inlineStr"/>
-      <c r="H84" s="6" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I84" s="8" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="J84" s="6" t="inlineStr"/>
-      <c r="K84" s="6" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="L84" s="17" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="M84" s="9" t="inlineStr">
-        <is>
-          <t>Ver</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="40" customHeight="1">
-      <c r="A85" s="16" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="B85" s="6" t="inlineStr">
-        <is>
-          <t>EUS-38583</t>
-        </is>
-      </c>
-      <c r="C85" s="6" t="inlineStr">
-        <is>
-          <t>Suministros Agua</t>
-        </is>
-      </c>
-      <c r="D85" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="E85" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F85" s="6" t="inlineStr"/>
-      <c r="G85" s="6" t="inlineStr"/>
-      <c r="H85" s="6" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I85" s="8" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="J85" s="6" t="inlineStr"/>
-      <c r="K85" s="6" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="L85" s="17" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="M85" s="9" t="inlineStr">
-        <is>
-          <t>Ver</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="40" customHeight="1">
-      <c r="A86" s="16" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="B86" s="6" t="inlineStr">
-        <is>
-          <t>EUS-51111</t>
-        </is>
-      </c>
-      <c r="C86" s="6" t="inlineStr">
-        <is>
-          <t>Suministros Agua</t>
-        </is>
-      </c>
-      <c r="D86" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="E86" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F86" s="6" t="inlineStr"/>
-      <c r="G86" s="6" t="inlineStr"/>
-      <c r="H86" s="6" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I86" s="8" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="J86" s="6" t="inlineStr"/>
-      <c r="K86" s="6" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="L86" s="17" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="M86" s="9" t="inlineStr">
-        <is>
-          <t>Ver</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="40" customHeight="1">
-      <c r="A87" s="16" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="B87" s="6" t="inlineStr">
-        <is>
-          <t>EUS-50384</t>
-        </is>
-      </c>
-      <c r="C87" s="6" t="inlineStr">
-        <is>
-          <t>Suministros Agua</t>
-        </is>
-      </c>
-      <c r="D87" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="E87" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F87" s="6" t="inlineStr"/>
-      <c r="G87" s="6" t="inlineStr"/>
-      <c r="H87" s="6" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I87" s="8" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="J87" s="6" t="inlineStr"/>
-      <c r="K87" s="6" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="L87" s="17" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="M87" s="9" t="inlineStr">
-        <is>
-          <t>Ver</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:M87"/>
+  <autoFilter ref="A4:M82"/>
   <mergeCells count="5">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A5:M5"/>
-    <mergeCell ref="A72:M72"/>
     <mergeCell ref="A69:M69"/>
     <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A71:M71"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId1"/>
@@ -5545,7 +5267,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M67" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M68" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M70" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M71" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M72" r:id="rId65"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M73" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M74" r:id="rId67"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M75" r:id="rId68"/>
@@ -5556,11 +5278,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M80" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M81" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M82" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M83" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M84" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M85" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M86" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M87" r:id="rId80"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5572,7 +5289,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1199"/>
+  <dimension ref="A1:F1124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10138,7 +9855,7 @@
     <row r="316" ht="30" customHeight="1">
       <c r="A316" s="18" t="inlineStr">
         <is>
-          <t>FICHA 22: HORIZON-CL5-2027-01-D1-08</t>
+          <t>FICHA 22: HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="B316" s="19" t="n"/>
@@ -10163,7 +9880,7 @@
       <c r="E317" s="22" t="n"/>
       <c r="F317" s="22" t="n"/>
     </row>
-    <row r="318" ht="20" customHeight="1">
+    <row r="318" ht="45" customHeight="1">
       <c r="A318" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -10171,7 +9888,7 @@
       </c>
       <c r="B318" s="21" t="inlineStr">
         <is>
-          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
+          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
         </is>
       </c>
       <c r="C318" s="22" t="n"/>
@@ -10187,7 +9904,7 @@
       </c>
       <c r="B319" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-08</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C319" s="22" t="n"/>
@@ -10299,7 +10016,7 @@
       </c>
       <c r="B326" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and interactions with ecosystems, leading to improved Earth system models;Future climate change scenarios produced in light of past changes in the Earth system, in particular warm climates/high sea-level situations, and abrupt transitions;Identification of thresholds in Earth system components and better characterisation of driving mechanisms and feedbacks that may be responsible for non-linear behaviours,</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Europe and globally, as well as the interaction between different hazards, their cumulative and/or cascading effects.Enhanced seamless prediction and projection modelling and attribution capabilities for extreme events and their likelihood to support preparedness, response and resilience to climate change by EU and national and regional actors. The EU Union Preparedness Strategy, the EU Adaptation Str</t>
         </is>
       </c>
       <c r="C326" s="22" t="n"/>
@@ -10343,7 +10060,7 @@
       </c>
       <c r="B329" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-08</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C329" s="22" t="n"/>
@@ -10786,7 +10503,7 @@
     <row r="361" ht="30" customHeight="1">
       <c r="A361" s="18" t="inlineStr">
         <is>
-          <t>FICHA 25: HORIZON-CL5-2027-01-D1-11</t>
+          <t>FICHA 25: HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="B361" s="19" t="n"/>
@@ -10811,7 +10528,7 @@
       <c r="E362" s="22" t="n"/>
       <c r="F362" s="22" t="n"/>
     </row>
-    <row r="363" ht="20" customHeight="1">
+    <row r="363" ht="45" customHeight="1">
       <c r="A363" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -10819,7 +10536,7 @@
       </c>
       <c r="B363" s="21" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
         </is>
       </c>
       <c r="C363" s="22" t="n"/>
@@ -10835,7 +10552,7 @@
       </c>
       <c r="B364" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C364" s="22" t="n"/>
@@ -10915,7 +10632,7 @@
       </c>
       <c r="B369" s="21" t="inlineStr">
         <is>
-          <t>Programme Cofund Actions</t>
+          <t xml:space="preserve"> Research and Innovation Actions</t>
         </is>
       </c>
       <c r="C369" s="22" t="n"/>
@@ -10947,7 +10664,7 @@
       </c>
       <c r="B371" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is established through development and implementation of the Climate Action pillar of the EU-AU Research and Innovation Partnership on Climate Change and Sustainable Energy (CCSE),[1] in co-design between African and European partners;Reduced fragmentation by aligning the EU, national and multilateral R&amp;amp;I efforts with increased leverage and impact of funding;African scientific, policy and practice com</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to inform mitigation action and policy improvements, ensuring a fair transition and social acceptability;Methodologies are developed and improved for ex-ante assessment and ex-post evaluation of greenhouse gas emission reductions from climate policies and measures;Strengthened collaboration and established networks between researchers, policy experts and government officials involved in designing and eva</t>
         </is>
       </c>
       <c r="C371" s="22" t="n"/>
@@ -10991,7 +10708,7 @@
       </c>
       <c r="B374" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-11</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C374" s="22" t="n"/>
@@ -11002,7 +10719,7 @@
     <row r="376" ht="30" customHeight="1">
       <c r="A376" s="18" t="inlineStr">
         <is>
-          <t>FICHA 26: HORIZON-CL5-2027-01-D1-10</t>
+          <t>FICHA 26: HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="B376" s="19" t="n"/>
@@ -11035,7 +10752,7 @@
       </c>
       <c r="B378" s="21" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
         </is>
       </c>
       <c r="C378" s="22" t="n"/>
@@ -11051,7 +10768,7 @@
       </c>
       <c r="B379" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="C379" s="22" t="n"/>
@@ -11163,7 +10880,7 @@
       </c>
       <c r="B386" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorporation into main EU repositories, such as Climate-ADAPT or the portal of the EU Mission on Adaptation to Climate Change;The risk and adaptation assessment frameworks are improved by better integrating the maladaptation dimension;Guidelines and tools for maladaptation prevention and correction strategies are made available to adaptation stakeholders at relevant scales and inform the design and impl</t>
+          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and interactions with ecosystems, leading to improved Earth system models;Future climate change scenarios produced in light of past changes in the Earth system, in particular warm climates/high sea-level situations, and abrupt transitions;Identification of thresholds in Earth system components and better characterisation of driving mechanisms and feedbacks that may be responsible for non-linear behaviours,</t>
         </is>
       </c>
       <c r="C386" s="22" t="n"/>
@@ -11207,7 +10924,7 @@
       </c>
       <c r="B389" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-10</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="C389" s="22" t="n"/>
@@ -11218,7 +10935,7 @@
     <row r="391" ht="30" customHeight="1">
       <c r="A391" s="18" t="inlineStr">
         <is>
-          <t>FICHA 27: HORIZON-CL5-2027-01-D1-09</t>
+          <t>FICHA 27: HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="B391" s="19" t="n"/>
@@ -11243,7 +10960,7 @@
       <c r="E392" s="22" t="n"/>
       <c r="F392" s="22" t="n"/>
     </row>
-    <row r="393" ht="45" customHeight="1">
+    <row r="393" ht="20" customHeight="1">
       <c r="A393" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -11251,7 +10968,7 @@
       </c>
       <c r="B393" s="21" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="C393" s="22" t="n"/>
@@ -11267,7 +10984,7 @@
       </c>
       <c r="B394" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C394" s="22" t="n"/>
@@ -11347,7 +11064,7 @@
       </c>
       <c r="B399" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Research and Innovation Actions</t>
+          <t>Programme Cofund Actions</t>
         </is>
       </c>
       <c r="C399" s="22" t="n"/>
@@ -11379,7 +11096,7 @@
       </c>
       <c r="B401" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to inform mitigation action and policy improvements, ensuring a fair transition and social acceptability;Methodologies are developed and improved for ex-ante assessment and ex-post evaluation of greenhouse gas emission reductions from climate policies and measures;Strengthened collaboration and established networks between researchers, policy experts and government officials involved in designing and eva</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is established through development and implementation of the Climate Action pillar of the EU-AU Research and Innovation Partnership on Climate Change and Sustainable Energy (CCSE),[1] in co-design between African and European partners;Reduced fragmentation by aligning the EU, national and multilateral R&amp;amp;I efforts with increased leverage and impact of funding;African scientific, policy and practice com</t>
         </is>
       </c>
       <c r="C401" s="22" t="n"/>
@@ -11423,7 +11140,7 @@
       </c>
       <c r="B404" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-09</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C404" s="22" t="n"/>
@@ -11434,7 +11151,7 @@
     <row r="406" ht="30" customHeight="1">
       <c r="A406" s="18" t="inlineStr">
         <is>
-          <t>FICHA 28: HORIZON-CL5-2027-01-D1-07</t>
+          <t>FICHA 28: HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="B406" s="19" t="n"/>
@@ -11459,7 +11176,7 @@
       <c r="E407" s="22" t="n"/>
       <c r="F407" s="22" t="n"/>
     </row>
-    <row r="408" ht="45" customHeight="1">
+    <row r="408" ht="20" customHeight="1">
       <c r="A408" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -11467,7 +11184,7 @@
       </c>
       <c r="B408" s="21" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="C408" s="22" t="n"/>
@@ -11483,7 +11200,7 @@
       </c>
       <c r="B409" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C409" s="22" t="n"/>
@@ -11595,7 +11312,7 @@
       </c>
       <c r="B416" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Europe and globally, as well as the interaction between different hazards, their cumulative and/or cascading effects.Enhanced seamless prediction and projection modelling and attribution capabilities for extreme events and their likelihood to support preparedness, response and resilience to climate change by EU and national and regional actors. The EU Union Preparedness Strategy, the EU Adaptation Str</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorporation into main EU repositories, such as Climate-ADAPT or the portal of the EU Mission on Adaptation to Climate Change;The risk and adaptation assessment frameworks are improved by better integrating the maladaptation dimension;Guidelines and tools for maladaptation prevention and correction strategies are made available to adaptation stakeholders at relevant scales and inform the design and impl</t>
         </is>
       </c>
       <c r="C416" s="22" t="n"/>
@@ -11639,7 +11356,7 @@
       </c>
       <c r="B419" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-07</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C419" s="22" t="n"/>
@@ -19150,7 +18867,7 @@
     <row r="946" ht="30" customHeight="1">
       <c r="A946" s="18" t="inlineStr">
         <is>
-          <t>FICHA 64: BDNS-901096</t>
+          <t>FICHA 64: BDNS-901505</t>
         </is>
       </c>
       <c r="B946" s="19" t="n"/>
@@ -19183,7 +18900,7 @@
       </c>
       <c r="B948" s="21" t="inlineStr">
         <is>
-          <t>Ayudas económicas al desarrollo y producción de proyectos audiovisuales y a la escritura de guiones. Año 2026</t>
+          <t>CONVENIO DE SUBVENCIÓN NOMINATIVA PARA LA ASOCIACIÓN KULTURA KALEAN PARA KORTERRAZA 2026</t>
         </is>
       </c>
       <c r="C948" s="22" t="n"/>
@@ -19199,7 +18916,7 @@
       </c>
       <c r="B949" s="21" t="inlineStr">
         <is>
-          <t>BDNS-901096</t>
+          <t>BDNS-901505</t>
         </is>
       </c>
       <c r="C949" s="22" t="n"/>
@@ -19247,7 +18964,7 @@
       </c>
       <c r="B952" s="21" t="inlineStr">
         <is>
-          <t>01/06/2026</t>
+          <t>31/12/2026</t>
         </is>
       </c>
       <c r="C952" s="22" t="n"/>
@@ -19263,7 +18980,7 @@
       </c>
       <c r="B953" s="21" t="inlineStr">
         <is>
-          <t>110,000.00 EUR</t>
+          <t>25,000.00 EUR</t>
         </is>
       </c>
       <c r="C953" s="22" t="n"/>
@@ -19295,7 +19012,7 @@
       </c>
       <c r="B955" s="21" t="inlineStr">
         <is>
-          <t>BDNS 901096</t>
+          <t>BDNS 901505</t>
         </is>
       </c>
       <c r="C955" s="22" t="n"/>
@@ -19311,7 +19028,7 @@
       </c>
       <c r="B956" s="21" t="inlineStr">
         <is>
-          <t>PYME Y PERSONAS FÍSICAS QUE DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
+          <t>PERSONAS JURÍDICAS QUE NO DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
         </is>
       </c>
       <c r="C956" s="22" t="n"/>
@@ -19355,7 +19072,7 @@
       </c>
       <c r="B959" s="23" t="inlineStr">
         <is>
-          <t>https://www.infosubvenciones.es/bdnstrans/GE/es/convocatoria/901096</t>
+          <t>https://www.infosubvenciones.es/bdnstrans/GE/es/convocatoria/901505</t>
         </is>
       </c>
       <c r="C959" s="22" t="n"/>
@@ -19366,7 +19083,7 @@
     <row r="961" ht="30" customHeight="1">
       <c r="A961" s="18" t="inlineStr">
         <is>
-          <t>FICHA 65: BDNS-901505</t>
+          <t>FICHA 65: EUS-74664</t>
         </is>
       </c>
       <c r="B961" s="19" t="n"/>
@@ -19383,7 +19100,7 @@
       </c>
       <c r="B962" s="21" t="inlineStr">
         <is>
-          <t>🇪🇸 España</t>
+          <t>🟢 Euskadi</t>
         </is>
       </c>
       <c r="C962" s="22" t="n"/>
@@ -19399,7 +19116,7 @@
       </c>
       <c r="B963" s="21" t="inlineStr">
         <is>
-          <t>CONVENIO DE SUBVENCIÓN NOMINATIVA PARA LA ASOCIACIÓN KULTURA KALEAN PARA KORTERRAZA 2026</t>
+          <t>LIFE 2026. Medio ambiente. Ayudas de 4 subprogramas, de naturaleza y biodiversidad, circularidad y calidad de vida, cambio climático y transición energética. Con inscripción abierta para jornadas info</t>
         </is>
       </c>
       <c r="C963" s="22" t="n"/>
@@ -19415,7 +19132,7 @@
       </c>
       <c r="B964" s="21" t="inlineStr">
         <is>
-          <t>BDNS-901505</t>
+          <t>EUS-74664</t>
         </is>
       </c>
       <c r="C964" s="22" t="n"/>
@@ -19431,7 +19148,7 @@
       </c>
       <c r="B965" s="21" t="inlineStr">
         <is>
-          <t>VITORIA-GASTEIZ</t>
+          <t>Euskadi</t>
         </is>
       </c>
       <c r="C965" s="22" t="n"/>
@@ -19461,11 +19178,7 @@
           <t>Deadline</t>
         </is>
       </c>
-      <c r="B967" s="21" t="inlineStr">
-        <is>
-          <t>31/12/2026</t>
-        </is>
-      </c>
+      <c r="B967" s="21" t="inlineStr"/>
       <c r="C967" s="22" t="n"/>
       <c r="D967" s="22" t="n"/>
       <c r="E967" s="22" t="n"/>
@@ -19479,7 +19192,7 @@
       </c>
       <c r="B968" s="21" t="inlineStr">
         <is>
-          <t>25,000.00 EUR</t>
+          <t>No disponible</t>
         </is>
       </c>
       <c r="C968" s="22" t="n"/>
@@ -19495,7 +19208,7 @@
       </c>
       <c r="B969" s="21" t="inlineStr">
         <is>
-          <t>Subvencion Nacional</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C969" s="22" t="n"/>
@@ -19509,17 +19222,13 @@
           <t>Call ID</t>
         </is>
       </c>
-      <c r="B970" s="21" t="inlineStr">
-        <is>
-          <t>BDNS 901505</t>
-        </is>
-      </c>
+      <c r="B970" s="21" t="inlineStr"/>
       <c r="C970" s="22" t="n"/>
       <c r="D970" s="22" t="n"/>
       <c r="E970" s="22" t="n"/>
       <c r="F970" s="22" t="n"/>
     </row>
-    <row r="971" ht="45" customHeight="1">
+    <row r="971" ht="20" customHeight="1">
       <c r="A971" s="20" t="inlineStr">
         <is>
           <t>Descripcion</t>
@@ -19527,7 +19236,7 @@
       </c>
       <c r="B971" s="21" t="inlineStr">
         <is>
-          <t>PERSONAS JURÍDICAS QUE NO DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
       <c r="C971" s="22" t="n"/>
@@ -19541,7 +19250,11 @@
           <t>Tags</t>
         </is>
       </c>
-      <c r="B972" s="21" t="inlineStr"/>
+      <c r="B972" s="21" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
       <c r="C972" s="22" t="n"/>
       <c r="D972" s="22" t="n"/>
       <c r="E972" s="22" t="n"/>
@@ -19553,9 +19266,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B973" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
+      <c r="B973" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALTA — </t>
         </is>
       </c>
       <c r="C973" s="22" t="n"/>
@@ -19563,7 +19276,7 @@
       <c r="E973" s="22" t="n"/>
       <c r="F973" s="22" t="n"/>
     </row>
-    <row r="974" ht="20" customHeight="1">
+    <row r="974" ht="45" customHeight="1">
       <c r="A974" s="20" t="inlineStr">
         <is>
           <t>Enlace al portal</t>
@@ -19571,7 +19284,7 @@
       </c>
       <c r="B974" s="23" t="inlineStr">
         <is>
-          <t>https://www.infosubvenciones.es/bdnstrans/GE/es/convocatoria/901505</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260421life4lerrotajarduna/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C974" s="22" t="n"/>
@@ -19582,7 +19295,7 @@
     <row r="976" ht="30" customHeight="1">
       <c r="A976" s="18" t="inlineStr">
         <is>
-          <t>FICHA 66: EUS-92454</t>
+          <t>FICHA 66: EUS-70680</t>
         </is>
       </c>
       <c r="B976" s="19" t="n"/>
@@ -19615,7 +19328,7 @@
       </c>
       <c r="B978" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Suministro de licencias de software para las plataformas Mailchimp, Zapier y SurveyMonkey, destinadas a la comunicación digital, automatización de procesos y gestión de encuestas de Bilbao Zerbitzuak </t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
         </is>
       </c>
       <c r="C978" s="22" t="n"/>
@@ -19631,7 +19344,7 @@
       </c>
       <c r="B979" s="21" t="inlineStr">
         <is>
-          <t>EUS-92454</t>
+          <t>EUS-70680</t>
         </is>
       </c>
       <c r="C979" s="22" t="n"/>
@@ -19707,7 +19420,7 @@
       </c>
       <c r="B984" s="21" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C984" s="22" t="n"/>
@@ -19765,9 +19478,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B988" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MUY ALTA — </t>
+      <c r="B988" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALTA — </t>
         </is>
       </c>
       <c r="C988" s="22" t="n"/>
@@ -19783,7 +19496,7 @@
       </c>
       <c r="B989" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-licencias-software-plataformas-mailchimp-zapier-y-surveymonkey-destinadas-comunicacion-digital-automatizacion-procesos-y-gestion-encuestas-bilbao-zerbitzuak-modalidad-suscripcion-anual/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-con-incremento-de-capacidad-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C989" s="22" t="n"/>
@@ -19794,7 +19507,7 @@
     <row r="991" ht="30" customHeight="1">
       <c r="A991" s="18" t="inlineStr">
         <is>
-          <t>FICHA 67: EUS-75183</t>
+          <t>FICHA 67: EUS-31421</t>
         </is>
       </c>
       <c r="B991" s="19" t="n"/>
@@ -19827,7 +19540,7 @@
       </c>
       <c r="B993" s="21" t="inlineStr">
         <is>
-          <t>LIFE 2026. Medio ambiente. Ayudas de 4 subprogramas, de naturaleza y biodiversidad, circularidad y calidad de vida, cambio climático y transición energética. Con inscripción abierta para jornadas info</t>
+          <t>Contrato mixto de suministro y obra para la sustitución y actualización de la instalación de climatización del polideportivo con piscina, Artebe, de Sondika.</t>
         </is>
       </c>
       <c r="C993" s="22" t="n"/>
@@ -19843,7 +19556,7 @@
       </c>
       <c r="B994" s="21" t="inlineStr">
         <is>
-          <t>EUS-75183</t>
+          <t>EUS-31421</t>
         </is>
       </c>
       <c r="C994" s="22" t="n"/>
@@ -19919,7 +19632,7 @@
       </c>
       <c r="B999" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C999" s="22" t="n"/>
@@ -19995,7 +19708,7 @@
       </c>
       <c r="B1004" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260421life4lerrotajarduna/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/contrato-mixto-suministro-y-obra-sustitucion-y-actualizacion-instalacion-climatizacion-del-polideportivo-piscina-artebe-sondika/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1004" s="22" t="n"/>
@@ -20006,7 +19719,7 @@
     <row r="1006" ht="30" customHeight="1">
       <c r="A1006" s="18" t="inlineStr">
         <is>
-          <t>FICHA 68: EUS-02830</t>
+          <t>FICHA 68: EUS-13213</t>
         </is>
       </c>
       <c r="B1006" s="19" t="n"/>
@@ -20039,7 +19752,7 @@
       </c>
       <c r="B1008" s="21" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio climático con incremento de capacidad 2026</t>
+          <t>Mantenimiento de las instalacioens  de climatización, ACS y grupo electrógeno del  centro de día Nafarroa, a excepción de los  equipos de climatización de la cafetería</t>
         </is>
       </c>
       <c r="C1008" s="22" t="n"/>
@@ -20055,7 +19768,7 @@
       </c>
       <c r="B1009" s="21" t="inlineStr">
         <is>
-          <t>EUS-02830</t>
+          <t>EUS-13213</t>
         </is>
       </c>
       <c r="C1009" s="22" t="n"/>
@@ -20131,7 +19844,7 @@
       </c>
       <c r="B1014" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C1014" s="22" t="n"/>
@@ -20207,7 +19920,7 @@
       </c>
       <c r="B1019" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/fempa-eficiencia-energetica-y-mitigacion-del-cambio-climatico-con-incremento-de-capacidad-2026/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/mantenimiento-instalacioens-climatizacion-acs-y-grupo-electrogeno-del-centro-dia-nafarroa-excepcion-equipos-climatizacion-cafeteria/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1019" s="22" t="n"/>
@@ -20218,7 +19931,7 @@
     <row r="1021" ht="30" customHeight="1">
       <c r="A1021" s="18" t="inlineStr">
         <is>
-          <t>FICHA 69: EUS-31407</t>
+          <t>FICHA 69: EUS-28151</t>
         </is>
       </c>
       <c r="B1021" s="19" t="n"/>
@@ -20251,7 +19964,8 @@
       </c>
       <c r="B1023" s="21" t="inlineStr">
         <is>
-          <t>asistencia tecnica para el desarrollo de la campaña informativa para impulsar la recogida selectiva de residuos en Lasarte-Oria</t>
+          <t>Servicio de recogida separada y clasificación de residuos de productos textiles o de calzado posconsumo y el servicio de recogida separada de residuos de pilas y acumuladores portátiles usados
+(Contr</t>
         </is>
       </c>
       <c r="C1023" s="22" t="n"/>
@@ -20267,7 +19981,7 @@
       </c>
       <c r="B1024" s="21" t="inlineStr">
         <is>
-          <t>EUS-31407</t>
+          <t>EUS-28151</t>
         </is>
       </c>
       <c r="C1024" s="22" t="n"/>
@@ -20419,7 +20133,7 @@
       </c>
       <c r="B1034" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/asistencia-tecnica-desarrollo-campana-informativa-impulsar-recogida-selectiva-residuos-lasarte-oria/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-recogida-separada-y-clasificacion-residuos-productos-textiles-o-calzado-posconsumo-y-servicio-recogida-separada-residuos-pilas-y-acumuladores-portatiles-usados-contrato-reservado-dad-19-ley-7-2022-y-dad4-y-dad-48-lcsp/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1034" s="22" t="n"/>
@@ -20430,7 +20144,7 @@
     <row r="1036" ht="30" customHeight="1">
       <c r="A1036" s="18" t="inlineStr">
         <is>
-          <t>FICHA 70: EUS-74304</t>
+          <t>FICHA 70: EUS-86678</t>
         </is>
       </c>
       <c r="B1036" s="19" t="n"/>
@@ -20479,7 +20193,7 @@
       </c>
       <c r="B1039" s="21" t="inlineStr">
         <is>
-          <t>EUS-74304</t>
+          <t>EUS-86678</t>
         </is>
       </c>
       <c r="C1039" s="22" t="n"/>
@@ -20642,7 +20356,7 @@
     <row r="1051" ht="30" customHeight="1">
       <c r="A1051" s="18" t="inlineStr">
         <is>
-          <t>FICHA 71: EUS-96161</t>
+          <t>FICHA 71: EUS-71437</t>
         </is>
       </c>
       <c r="B1051" s="19" t="n"/>
@@ -20691,7 +20405,7 @@
       </c>
       <c r="B1054" s="21" t="inlineStr">
         <is>
-          <t>EUS-96161</t>
+          <t>EUS-71437</t>
         </is>
       </c>
       <c r="C1054" s="22" t="n"/>
@@ -20854,7 +20568,7 @@
     <row r="1066" ht="30" customHeight="1">
       <c r="A1066" s="18" t="inlineStr">
         <is>
-          <t>FICHA 72: EUS-04369</t>
+          <t>FICHA 72: EUS-71705</t>
         </is>
       </c>
       <c r="B1066" s="19" t="n"/>
@@ -20903,7 +20617,7 @@
       </c>
       <c r="B1069" s="21" t="inlineStr">
         <is>
-          <t>EUS-04369</t>
+          <t>EUS-71705</t>
         </is>
       </c>
       <c r="C1069" s="22" t="n"/>
@@ -21066,7 +20780,7 @@
     <row r="1081" ht="30" customHeight="1">
       <c r="A1081" s="18" t="inlineStr">
         <is>
-          <t>FICHA 73: EUS-86318</t>
+          <t>FICHA 73: EUS-79070</t>
         </is>
       </c>
       <c r="B1081" s="19" t="n"/>
@@ -21091,7 +20805,7 @@
       <c r="E1082" s="22" t="n"/>
       <c r="F1082" s="22" t="n"/>
     </row>
-    <row r="1083" ht="45" customHeight="1">
+    <row r="1083" ht="20" customHeight="1">
       <c r="A1083" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -21099,7 +20813,7 @@
       </c>
       <c r="B1083" s="21" t="inlineStr">
         <is>
-          <t>Contratación de los servicios de formación en materia ESG, realización de diagnósticos ESG y hojas de ruta en sostenibilidad, así como de los servicios de medición de impacto social en proyectos empre</t>
+          <t>Servicio de recogida de animales domésticos</t>
         </is>
       </c>
       <c r="C1083" s="22" t="n"/>
@@ -21115,7 +20829,7 @@
       </c>
       <c r="B1084" s="21" t="inlineStr">
         <is>
-          <t>EUS-86318</t>
+          <t>EUS-79070</t>
         </is>
       </c>
       <c r="C1084" s="22" t="n"/>
@@ -21267,7 +20981,7 @@
       </c>
       <c r="B1094" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/contratacion-servicios-formacion-materia-esg-realizacion-diagnosticos-esg-y-hojas-ruta-sostenibilidad-asi-como-servicios-medicion-impacto-social-proyectos-empresariales-innovadores-objeto-mejorar-su-acceso-financiacion-e-inversion/expjaso708863/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-recogida-animales-domesticos/expgebizkaia3436259/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1094" s="22" t="n"/>
@@ -21278,7 +20992,7 @@
     <row r="1096" ht="30" customHeight="1">
       <c r="A1096" s="18" t="inlineStr">
         <is>
-          <t>FICHA 74: EUS-63953</t>
+          <t>FICHA 74: EUS-53277</t>
         </is>
       </c>
       <c r="B1096" s="19" t="n"/>
@@ -21311,7 +21025,7 @@
       </c>
       <c r="B1098" s="21" t="inlineStr">
         <is>
-          <t>Enajenación, mediante subasta, de la parcela urbana1-819 de Zambrana</t>
+          <t>Servicio de transporte para el programa Ibiliaz Ezagutu de primavera</t>
         </is>
       </c>
       <c r="C1098" s="22" t="n"/>
@@ -21327,7 +21041,7 @@
       </c>
       <c r="B1099" s="21" t="inlineStr">
         <is>
-          <t>EUS-63953</t>
+          <t>EUS-53277</t>
         </is>
       </c>
       <c r="C1099" s="22" t="n"/>
@@ -21479,7 +21193,7 @@
       </c>
       <c r="B1109" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/enajenacion-mediante-subasta-parcela-urbana1-819-zambrana/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-transporte-programa-ibiliaz-ezagutu-primavera/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1109" s="22" t="n"/>
@@ -21490,7 +21204,7 @@
     <row r="1111" ht="30" customHeight="1">
       <c r="A1111" s="18" t="inlineStr">
         <is>
-          <t>FICHA 75: EUS-29174</t>
+          <t>FICHA 75: EUS-45140</t>
         </is>
       </c>
       <c r="B1111" s="19" t="n"/>
@@ -21515,7 +21229,7 @@
       <c r="E1112" s="22" t="n"/>
       <c r="F1112" s="22" t="n"/>
     </row>
-    <row r="1113" ht="45" customHeight="1">
+    <row r="1113" ht="20" customHeight="1">
       <c r="A1113" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -21523,7 +21237,7 @@
       </c>
       <c r="B1113" s="21" t="inlineStr">
         <is>
-          <t>Elaboración, transporte y entrega de comidas preparadas y prestaciones complementarias para el funcionamiento de los comedores de gestión directa en diversos centros públicos dependientes del Departam</t>
+          <t>Cubierta de patio CEIP BAGATZA HLHI, Barakaldo (Bizkaia)</t>
         </is>
       </c>
       <c r="C1113" s="22" t="n"/>
@@ -21539,7 +21253,7 @@
       </c>
       <c r="B1114" s="21" t="inlineStr">
         <is>
-          <t>EUS-29174</t>
+          <t>EUS-45140</t>
         </is>
       </c>
       <c r="C1114" s="22" t="n"/>
@@ -21691,7 +21405,7 @@
       </c>
       <c r="B1124" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/elaboracion-transporte-y-entrega-comidas-preparadas-y-prestaciones-complementarias-funcionamiento-comedores-gestion-directa-diversos-centros-publicos-dependientes-del-departamento-educacion-situados-comunidad-autonoma-del-pais-vasco/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/cubierta-patio-ceip-bagatza-hlhi-barakaldo-bizkaia/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1124" s="22" t="n"/>
@@ -21699,1068 +21413,8 @@
       <c r="E1124" s="22" t="n"/>
       <c r="F1124" s="22" t="n"/>
     </row>
-    <row r="1126" ht="30" customHeight="1">
-      <c r="A1126" s="18" t="inlineStr">
-        <is>
-          <t>FICHA 76: EUS-05384</t>
-        </is>
-      </c>
-      <c r="B1126" s="19" t="n"/>
-      <c r="C1126" s="19" t="n"/>
-      <c r="D1126" s="19" t="n"/>
-      <c r="E1126" s="19" t="n"/>
-      <c r="F1126" s="19" t="n"/>
-    </row>
-    <row r="1127" ht="20" customHeight="1">
-      <c r="A1127" s="20" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-      <c r="B1127" s="21" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
-        </is>
-      </c>
-      <c r="C1127" s="22" t="n"/>
-      <c r="D1127" s="22" t="n"/>
-      <c r="E1127" s="22" t="n"/>
-      <c r="F1127" s="22" t="n"/>
-    </row>
-    <row r="1128" ht="20" customHeight="1">
-      <c r="A1128" s="20" t="inlineStr">
-        <is>
-          <t>Titulo</t>
-        </is>
-      </c>
-      <c r="B1128" s="21" t="inlineStr">
-        <is>
-          <t>Suministro Cajas transporte</t>
-        </is>
-      </c>
-      <c r="C1128" s="22" t="n"/>
-      <c r="D1128" s="22" t="n"/>
-      <c r="E1128" s="22" t="n"/>
-      <c r="F1128" s="22" t="n"/>
-    </row>
-    <row r="1129" ht="20" customHeight="1">
-      <c r="A1129" s="20" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1129" s="21" t="inlineStr">
-        <is>
-          <t>EUS-05384</t>
-        </is>
-      </c>
-      <c r="C1129" s="22" t="n"/>
-      <c r="D1129" s="22" t="n"/>
-      <c r="E1129" s="22" t="n"/>
-      <c r="F1129" s="22" t="n"/>
-    </row>
-    <row r="1130" ht="20" customHeight="1">
-      <c r="A1130" s="20" t="inlineStr">
-        <is>
-          <t>Programa</t>
-        </is>
-      </c>
-      <c r="B1130" s="21" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="C1130" s="22" t="n"/>
-      <c r="D1130" s="22" t="n"/>
-      <c r="E1130" s="22" t="n"/>
-      <c r="F1130" s="22" t="n"/>
-    </row>
-    <row r="1131" ht="20" customHeight="1">
-      <c r="A1131" s="20" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="B1131" s="21" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C1131" s="22" t="n"/>
-      <c r="D1131" s="22" t="n"/>
-      <c r="E1131" s="22" t="n"/>
-      <c r="F1131" s="22" t="n"/>
-    </row>
-    <row r="1132" ht="20" customHeight="1">
-      <c r="A1132" s="20" t="inlineStr">
-        <is>
-          <t>Deadline</t>
-        </is>
-      </c>
-      <c r="B1132" s="21" t="inlineStr"/>
-      <c r="C1132" s="22" t="n"/>
-      <c r="D1132" s="22" t="n"/>
-      <c r="E1132" s="22" t="n"/>
-      <c r="F1132" s="22" t="n"/>
-    </row>
-    <row r="1133" ht="20" customHeight="1">
-      <c r="A1133" s="20" t="inlineStr">
-        <is>
-          <t>Presupuesto (EUR)</t>
-        </is>
-      </c>
-      <c r="B1133" s="21" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="C1133" s="22" t="n"/>
-      <c r="D1133" s="22" t="n"/>
-      <c r="E1133" s="22" t="n"/>
-      <c r="F1133" s="22" t="n"/>
-    </row>
-    <row r="1134" ht="20" customHeight="1">
-      <c r="A1134" s="20" t="inlineStr">
-        <is>
-          <t>Tipo de Accion</t>
-        </is>
-      </c>
-      <c r="B1134" s="21" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="C1134" s="22" t="n"/>
-      <c r="D1134" s="22" t="n"/>
-      <c r="E1134" s="22" t="n"/>
-      <c r="F1134" s="22" t="n"/>
-    </row>
-    <row r="1135" ht="20" customHeight="1">
-      <c r="A1135" s="20" t="inlineStr">
-        <is>
-          <t>Call ID</t>
-        </is>
-      </c>
-      <c r="B1135" s="21" t="inlineStr"/>
-      <c r="C1135" s="22" t="n"/>
-      <c r="D1135" s="22" t="n"/>
-      <c r="E1135" s="22" t="n"/>
-      <c r="F1135" s="22" t="n"/>
-    </row>
-    <row r="1136" ht="20" customHeight="1">
-      <c r="A1136" s="20" t="inlineStr">
-        <is>
-          <t>Descripcion</t>
-        </is>
-      </c>
-      <c r="B1136" s="21" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="C1136" s="22" t="n"/>
-      <c r="D1136" s="22" t="n"/>
-      <c r="E1136" s="22" t="n"/>
-      <c r="F1136" s="22" t="n"/>
-    </row>
-    <row r="1137" ht="20" customHeight="1">
-      <c r="A1137" s="20" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-      <c r="B1137" s="21" t="inlineStr">
-        <is>
-          <t>energia</t>
-        </is>
-      </c>
-      <c r="C1137" s="22" t="n"/>
-      <c r="D1137" s="22" t="n"/>
-      <c r="E1137" s="22" t="n"/>
-      <c r="F1137" s="22" t="n"/>
-    </row>
-    <row r="1138" ht="20" customHeight="1">
-      <c r="A1138" s="20" t="inlineStr">
-        <is>
-          <t>Relevancia Bilbao</t>
-        </is>
-      </c>
-      <c r="B1138" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
-        </is>
-      </c>
-      <c r="C1138" s="22" t="n"/>
-      <c r="D1138" s="22" t="n"/>
-      <c r="E1138" s="22" t="n"/>
-      <c r="F1138" s="22" t="n"/>
-    </row>
-    <row r="1139" ht="45" customHeight="1">
-      <c r="A1139" s="20" t="inlineStr">
-        <is>
-          <t>Enlace al portal</t>
-        </is>
-      </c>
-      <c r="B1139" s="23" t="inlineStr">
-        <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-cajas-transporte/expcm507348/web01-tramite/es/</t>
-        </is>
-      </c>
-      <c r="C1139" s="22" t="n"/>
-      <c r="D1139" s="22" t="n"/>
-      <c r="E1139" s="22" t="n"/>
-      <c r="F1139" s="22" t="n"/>
-    </row>
-    <row r="1141" ht="30" customHeight="1">
-      <c r="A1141" s="18" t="inlineStr">
-        <is>
-          <t>FICHA 77: EUS-34859</t>
-        </is>
-      </c>
-      <c r="B1141" s="19" t="n"/>
-      <c r="C1141" s="19" t="n"/>
-      <c r="D1141" s="19" t="n"/>
-      <c r="E1141" s="19" t="n"/>
-      <c r="F1141" s="19" t="n"/>
-    </row>
-    <row r="1142" ht="20" customHeight="1">
-      <c r="A1142" s="20" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-      <c r="B1142" s="21" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
-        </is>
-      </c>
-      <c r="C1142" s="22" t="n"/>
-      <c r="D1142" s="22" t="n"/>
-      <c r="E1142" s="22" t="n"/>
-      <c r="F1142" s="22" t="n"/>
-    </row>
-    <row r="1143" ht="20" customHeight="1">
-      <c r="A1143" s="20" t="inlineStr">
-        <is>
-          <t>Titulo</t>
-        </is>
-      </c>
-      <c r="B1143" s="21" t="inlineStr">
-        <is>
-          <t>Suministro Cajas transporte</t>
-        </is>
-      </c>
-      <c r="C1143" s="22" t="n"/>
-      <c r="D1143" s="22" t="n"/>
-      <c r="E1143" s="22" t="n"/>
-      <c r="F1143" s="22" t="n"/>
-    </row>
-    <row r="1144" ht="20" customHeight="1">
-      <c r="A1144" s="20" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1144" s="21" t="inlineStr">
-        <is>
-          <t>EUS-34859</t>
-        </is>
-      </c>
-      <c r="C1144" s="22" t="n"/>
-      <c r="D1144" s="22" t="n"/>
-      <c r="E1144" s="22" t="n"/>
-      <c r="F1144" s="22" t="n"/>
-    </row>
-    <row r="1145" ht="20" customHeight="1">
-      <c r="A1145" s="20" t="inlineStr">
-        <is>
-          <t>Programa</t>
-        </is>
-      </c>
-      <c r="B1145" s="21" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="C1145" s="22" t="n"/>
-      <c r="D1145" s="22" t="n"/>
-      <c r="E1145" s="22" t="n"/>
-      <c r="F1145" s="22" t="n"/>
-    </row>
-    <row r="1146" ht="20" customHeight="1">
-      <c r="A1146" s="20" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="B1146" s="21" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C1146" s="22" t="n"/>
-      <c r="D1146" s="22" t="n"/>
-      <c r="E1146" s="22" t="n"/>
-      <c r="F1146" s="22" t="n"/>
-    </row>
-    <row r="1147" ht="20" customHeight="1">
-      <c r="A1147" s="20" t="inlineStr">
-        <is>
-          <t>Deadline</t>
-        </is>
-      </c>
-      <c r="B1147" s="21" t="inlineStr"/>
-      <c r="C1147" s="22" t="n"/>
-      <c r="D1147" s="22" t="n"/>
-      <c r="E1147" s="22" t="n"/>
-      <c r="F1147" s="22" t="n"/>
-    </row>
-    <row r="1148" ht="20" customHeight="1">
-      <c r="A1148" s="20" t="inlineStr">
-        <is>
-          <t>Presupuesto (EUR)</t>
-        </is>
-      </c>
-      <c r="B1148" s="21" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="C1148" s="22" t="n"/>
-      <c r="D1148" s="22" t="n"/>
-      <c r="E1148" s="22" t="n"/>
-      <c r="F1148" s="22" t="n"/>
-    </row>
-    <row r="1149" ht="20" customHeight="1">
-      <c r="A1149" s="20" t="inlineStr">
-        <is>
-          <t>Tipo de Accion</t>
-        </is>
-      </c>
-      <c r="B1149" s="21" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="C1149" s="22" t="n"/>
-      <c r="D1149" s="22" t="n"/>
-      <c r="E1149" s="22" t="n"/>
-      <c r="F1149" s="22" t="n"/>
-    </row>
-    <row r="1150" ht="20" customHeight="1">
-      <c r="A1150" s="20" t="inlineStr">
-        <is>
-          <t>Call ID</t>
-        </is>
-      </c>
-      <c r="B1150" s="21" t="inlineStr"/>
-      <c r="C1150" s="22" t="n"/>
-      <c r="D1150" s="22" t="n"/>
-      <c r="E1150" s="22" t="n"/>
-      <c r="F1150" s="22" t="n"/>
-    </row>
-    <row r="1151" ht="20" customHeight="1">
-      <c r="A1151" s="20" t="inlineStr">
-        <is>
-          <t>Descripcion</t>
-        </is>
-      </c>
-      <c r="B1151" s="21" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="C1151" s="22" t="n"/>
-      <c r="D1151" s="22" t="n"/>
-      <c r="E1151" s="22" t="n"/>
-      <c r="F1151" s="22" t="n"/>
-    </row>
-    <row r="1152" ht="20" customHeight="1">
-      <c r="A1152" s="20" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-      <c r="B1152" s="21" t="inlineStr">
-        <is>
-          <t>energia</t>
-        </is>
-      </c>
-      <c r="C1152" s="22" t="n"/>
-      <c r="D1152" s="22" t="n"/>
-      <c r="E1152" s="22" t="n"/>
-      <c r="F1152" s="22" t="n"/>
-    </row>
-    <row r="1153" ht="20" customHeight="1">
-      <c r="A1153" s="20" t="inlineStr">
-        <is>
-          <t>Relevancia Bilbao</t>
-        </is>
-      </c>
-      <c r="B1153" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
-        </is>
-      </c>
-      <c r="C1153" s="22" t="n"/>
-      <c r="D1153" s="22" t="n"/>
-      <c r="E1153" s="22" t="n"/>
-      <c r="F1153" s="22" t="n"/>
-    </row>
-    <row r="1154" ht="45" customHeight="1">
-      <c r="A1154" s="20" t="inlineStr">
-        <is>
-          <t>Enlace al portal</t>
-        </is>
-      </c>
-      <c r="B1154" s="23" t="inlineStr">
-        <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-cajas-transporte/web01-tramite/es/</t>
-        </is>
-      </c>
-      <c r="C1154" s="22" t="n"/>
-      <c r="D1154" s="22" t="n"/>
-      <c r="E1154" s="22" t="n"/>
-      <c r="F1154" s="22" t="n"/>
-    </row>
-    <row r="1156" ht="30" customHeight="1">
-      <c r="A1156" s="18" t="inlineStr">
-        <is>
-          <t>FICHA 78: EUS-38583</t>
-        </is>
-      </c>
-      <c r="B1156" s="19" t="n"/>
-      <c r="C1156" s="19" t="n"/>
-      <c r="D1156" s="19" t="n"/>
-      <c r="E1156" s="19" t="n"/>
-      <c r="F1156" s="19" t="n"/>
-    </row>
-    <row r="1157" ht="20" customHeight="1">
-      <c r="A1157" s="20" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-      <c r="B1157" s="21" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
-        </is>
-      </c>
-      <c r="C1157" s="22" t="n"/>
-      <c r="D1157" s="22" t="n"/>
-      <c r="E1157" s="22" t="n"/>
-      <c r="F1157" s="22" t="n"/>
-    </row>
-    <row r="1158" ht="20" customHeight="1">
-      <c r="A1158" s="20" t="inlineStr">
-        <is>
-          <t>Titulo</t>
-        </is>
-      </c>
-      <c r="B1158" s="21" t="inlineStr">
-        <is>
-          <t>Suministros Agua</t>
-        </is>
-      </c>
-      <c r="C1158" s="22" t="n"/>
-      <c r="D1158" s="22" t="n"/>
-      <c r="E1158" s="22" t="n"/>
-      <c r="F1158" s="22" t="n"/>
-    </row>
-    <row r="1159" ht="20" customHeight="1">
-      <c r="A1159" s="20" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1159" s="21" t="inlineStr">
-        <is>
-          <t>EUS-38583</t>
-        </is>
-      </c>
-      <c r="C1159" s="22" t="n"/>
-      <c r="D1159" s="22" t="n"/>
-      <c r="E1159" s="22" t="n"/>
-      <c r="F1159" s="22" t="n"/>
-    </row>
-    <row r="1160" ht="20" customHeight="1">
-      <c r="A1160" s="20" t="inlineStr">
-        <is>
-          <t>Programa</t>
-        </is>
-      </c>
-      <c r="B1160" s="21" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="C1160" s="22" t="n"/>
-      <c r="D1160" s="22" t="n"/>
-      <c r="E1160" s="22" t="n"/>
-      <c r="F1160" s="22" t="n"/>
-    </row>
-    <row r="1161" ht="20" customHeight="1">
-      <c r="A1161" s="20" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="B1161" s="21" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C1161" s="22" t="n"/>
-      <c r="D1161" s="22" t="n"/>
-      <c r="E1161" s="22" t="n"/>
-      <c r="F1161" s="22" t="n"/>
-    </row>
-    <row r="1162" ht="20" customHeight="1">
-      <c r="A1162" s="20" t="inlineStr">
-        <is>
-          <t>Deadline</t>
-        </is>
-      </c>
-      <c r="B1162" s="21" t="inlineStr"/>
-      <c r="C1162" s="22" t="n"/>
-      <c r="D1162" s="22" t="n"/>
-      <c r="E1162" s="22" t="n"/>
-      <c r="F1162" s="22" t="n"/>
-    </row>
-    <row r="1163" ht="20" customHeight="1">
-      <c r="A1163" s="20" t="inlineStr">
-        <is>
-          <t>Presupuesto (EUR)</t>
-        </is>
-      </c>
-      <c r="B1163" s="21" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="C1163" s="22" t="n"/>
-      <c r="D1163" s="22" t="n"/>
-      <c r="E1163" s="22" t="n"/>
-      <c r="F1163" s="22" t="n"/>
-    </row>
-    <row r="1164" ht="20" customHeight="1">
-      <c r="A1164" s="20" t="inlineStr">
-        <is>
-          <t>Tipo de Accion</t>
-        </is>
-      </c>
-      <c r="B1164" s="21" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="C1164" s="22" t="n"/>
-      <c r="D1164" s="22" t="n"/>
-      <c r="E1164" s="22" t="n"/>
-      <c r="F1164" s="22" t="n"/>
-    </row>
-    <row r="1165" ht="20" customHeight="1">
-      <c r="A1165" s="20" t="inlineStr">
-        <is>
-          <t>Call ID</t>
-        </is>
-      </c>
-      <c r="B1165" s="21" t="inlineStr"/>
-      <c r="C1165" s="22" t="n"/>
-      <c r="D1165" s="22" t="n"/>
-      <c r="E1165" s="22" t="n"/>
-      <c r="F1165" s="22" t="n"/>
-    </row>
-    <row r="1166" ht="20" customHeight="1">
-      <c r="A1166" s="20" t="inlineStr">
-        <is>
-          <t>Descripcion</t>
-        </is>
-      </c>
-      <c r="B1166" s="21" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="C1166" s="22" t="n"/>
-      <c r="D1166" s="22" t="n"/>
-      <c r="E1166" s="22" t="n"/>
-      <c r="F1166" s="22" t="n"/>
-    </row>
-    <row r="1167" ht="20" customHeight="1">
-      <c r="A1167" s="20" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-      <c r="B1167" s="21" t="inlineStr">
-        <is>
-          <t>energia</t>
-        </is>
-      </c>
-      <c r="C1167" s="22" t="n"/>
-      <c r="D1167" s="22" t="n"/>
-      <c r="E1167" s="22" t="n"/>
-      <c r="F1167" s="22" t="n"/>
-    </row>
-    <row r="1168" ht="20" customHeight="1">
-      <c r="A1168" s="20" t="inlineStr">
-        <is>
-          <t>Relevancia Bilbao</t>
-        </is>
-      </c>
-      <c r="B1168" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
-        </is>
-      </c>
-      <c r="C1168" s="22" t="n"/>
-      <c r="D1168" s="22" t="n"/>
-      <c r="E1168" s="22" t="n"/>
-      <c r="F1168" s="22" t="n"/>
-    </row>
-    <row r="1169" ht="45" customHeight="1">
-      <c r="A1169" s="20" t="inlineStr">
-        <is>
-          <t>Enlace al portal</t>
-        </is>
-      </c>
-      <c r="B1169" s="23" t="inlineStr">
-        <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministros-agua/expcm507335/web01-tramite/es/</t>
-        </is>
-      </c>
-      <c r="C1169" s="22" t="n"/>
-      <c r="D1169" s="22" t="n"/>
-      <c r="E1169" s="22" t="n"/>
-      <c r="F1169" s="22" t="n"/>
-    </row>
-    <row r="1171" ht="30" customHeight="1">
-      <c r="A1171" s="18" t="inlineStr">
-        <is>
-          <t>FICHA 79: EUS-51111</t>
-        </is>
-      </c>
-      <c r="B1171" s="19" t="n"/>
-      <c r="C1171" s="19" t="n"/>
-      <c r="D1171" s="19" t="n"/>
-      <c r="E1171" s="19" t="n"/>
-      <c r="F1171" s="19" t="n"/>
-    </row>
-    <row r="1172" ht="20" customHeight="1">
-      <c r="A1172" s="20" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-      <c r="B1172" s="21" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
-        </is>
-      </c>
-      <c r="C1172" s="22" t="n"/>
-      <c r="D1172" s="22" t="n"/>
-      <c r="E1172" s="22" t="n"/>
-      <c r="F1172" s="22" t="n"/>
-    </row>
-    <row r="1173" ht="20" customHeight="1">
-      <c r="A1173" s="20" t="inlineStr">
-        <is>
-          <t>Titulo</t>
-        </is>
-      </c>
-      <c r="B1173" s="21" t="inlineStr">
-        <is>
-          <t>Suministros Agua</t>
-        </is>
-      </c>
-      <c r="C1173" s="22" t="n"/>
-      <c r="D1173" s="22" t="n"/>
-      <c r="E1173" s="22" t="n"/>
-      <c r="F1173" s="22" t="n"/>
-    </row>
-    <row r="1174" ht="20" customHeight="1">
-      <c r="A1174" s="20" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1174" s="21" t="inlineStr">
-        <is>
-          <t>EUS-51111</t>
-        </is>
-      </c>
-      <c r="C1174" s="22" t="n"/>
-      <c r="D1174" s="22" t="n"/>
-      <c r="E1174" s="22" t="n"/>
-      <c r="F1174" s="22" t="n"/>
-    </row>
-    <row r="1175" ht="20" customHeight="1">
-      <c r="A1175" s="20" t="inlineStr">
-        <is>
-          <t>Programa</t>
-        </is>
-      </c>
-      <c r="B1175" s="21" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="C1175" s="22" t="n"/>
-      <c r="D1175" s="22" t="n"/>
-      <c r="E1175" s="22" t="n"/>
-      <c r="F1175" s="22" t="n"/>
-    </row>
-    <row r="1176" ht="20" customHeight="1">
-      <c r="A1176" s="20" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="B1176" s="21" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C1176" s="22" t="n"/>
-      <c r="D1176" s="22" t="n"/>
-      <c r="E1176" s="22" t="n"/>
-      <c r="F1176" s="22" t="n"/>
-    </row>
-    <row r="1177" ht="20" customHeight="1">
-      <c r="A1177" s="20" t="inlineStr">
-        <is>
-          <t>Deadline</t>
-        </is>
-      </c>
-      <c r="B1177" s="21" t="inlineStr"/>
-      <c r="C1177" s="22" t="n"/>
-      <c r="D1177" s="22" t="n"/>
-      <c r="E1177" s="22" t="n"/>
-      <c r="F1177" s="22" t="n"/>
-    </row>
-    <row r="1178" ht="20" customHeight="1">
-      <c r="A1178" s="20" t="inlineStr">
-        <is>
-          <t>Presupuesto (EUR)</t>
-        </is>
-      </c>
-      <c r="B1178" s="21" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="C1178" s="22" t="n"/>
-      <c r="D1178" s="22" t="n"/>
-      <c r="E1178" s="22" t="n"/>
-      <c r="F1178" s="22" t="n"/>
-    </row>
-    <row r="1179" ht="20" customHeight="1">
-      <c r="A1179" s="20" t="inlineStr">
-        <is>
-          <t>Tipo de Accion</t>
-        </is>
-      </c>
-      <c r="B1179" s="21" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="C1179" s="22" t="n"/>
-      <c r="D1179" s="22" t="n"/>
-      <c r="E1179" s="22" t="n"/>
-      <c r="F1179" s="22" t="n"/>
-    </row>
-    <row r="1180" ht="20" customHeight="1">
-      <c r="A1180" s="20" t="inlineStr">
-        <is>
-          <t>Call ID</t>
-        </is>
-      </c>
-      <c r="B1180" s="21" t="inlineStr"/>
-      <c r="C1180" s="22" t="n"/>
-      <c r="D1180" s="22" t="n"/>
-      <c r="E1180" s="22" t="n"/>
-      <c r="F1180" s="22" t="n"/>
-    </row>
-    <row r="1181" ht="20" customHeight="1">
-      <c r="A1181" s="20" t="inlineStr">
-        <is>
-          <t>Descripcion</t>
-        </is>
-      </c>
-      <c r="B1181" s="21" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="C1181" s="22" t="n"/>
-      <c r="D1181" s="22" t="n"/>
-      <c r="E1181" s="22" t="n"/>
-      <c r="F1181" s="22" t="n"/>
-    </row>
-    <row r="1182" ht="20" customHeight="1">
-      <c r="A1182" s="20" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-      <c r="B1182" s="21" t="inlineStr">
-        <is>
-          <t>energia</t>
-        </is>
-      </c>
-      <c r="C1182" s="22" t="n"/>
-      <c r="D1182" s="22" t="n"/>
-      <c r="E1182" s="22" t="n"/>
-      <c r="F1182" s="22" t="n"/>
-    </row>
-    <row r="1183" ht="20" customHeight="1">
-      <c r="A1183" s="20" t="inlineStr">
-        <is>
-          <t>Relevancia Bilbao</t>
-        </is>
-      </c>
-      <c r="B1183" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
-        </is>
-      </c>
-      <c r="C1183" s="22" t="n"/>
-      <c r="D1183" s="22" t="n"/>
-      <c r="E1183" s="22" t="n"/>
-      <c r="F1183" s="22" t="n"/>
-    </row>
-    <row r="1184" ht="45" customHeight="1">
-      <c r="A1184" s="20" t="inlineStr">
-        <is>
-          <t>Enlace al portal</t>
-        </is>
-      </c>
-      <c r="B1184" s="23" t="inlineStr">
-        <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministros-agua/expcm507334/web01-tramite/es/</t>
-        </is>
-      </c>
-      <c r="C1184" s="22" t="n"/>
-      <c r="D1184" s="22" t="n"/>
-      <c r="E1184" s="22" t="n"/>
-      <c r="F1184" s="22" t="n"/>
-    </row>
-    <row r="1186" ht="30" customHeight="1">
-      <c r="A1186" s="18" t="inlineStr">
-        <is>
-          <t>FICHA 80: EUS-50384</t>
-        </is>
-      </c>
-      <c r="B1186" s="19" t="n"/>
-      <c r="C1186" s="19" t="n"/>
-      <c r="D1186" s="19" t="n"/>
-      <c r="E1186" s="19" t="n"/>
-      <c r="F1186" s="19" t="n"/>
-    </row>
-    <row r="1187" ht="20" customHeight="1">
-      <c r="A1187" s="20" t="inlineStr">
-        <is>
-          <t>Fuente</t>
-        </is>
-      </c>
-      <c r="B1187" s="21" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
-        </is>
-      </c>
-      <c r="C1187" s="22" t="n"/>
-      <c r="D1187" s="22" t="n"/>
-      <c r="E1187" s="22" t="n"/>
-      <c r="F1187" s="22" t="n"/>
-    </row>
-    <row r="1188" ht="20" customHeight="1">
-      <c r="A1188" s="20" t="inlineStr">
-        <is>
-          <t>Titulo</t>
-        </is>
-      </c>
-      <c r="B1188" s="21" t="inlineStr">
-        <is>
-          <t>Suministros Agua</t>
-        </is>
-      </c>
-      <c r="C1188" s="22" t="n"/>
-      <c r="D1188" s="22" t="n"/>
-      <c r="E1188" s="22" t="n"/>
-      <c r="F1188" s="22" t="n"/>
-    </row>
-    <row r="1189" ht="20" customHeight="1">
-      <c r="A1189" s="20" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B1189" s="21" t="inlineStr">
-        <is>
-          <t>EUS-50384</t>
-        </is>
-      </c>
-      <c r="C1189" s="22" t="n"/>
-      <c r="D1189" s="22" t="n"/>
-      <c r="E1189" s="22" t="n"/>
-      <c r="F1189" s="22" t="n"/>
-    </row>
-    <row r="1190" ht="20" customHeight="1">
-      <c r="A1190" s="20" t="inlineStr">
-        <is>
-          <t>Programa</t>
-        </is>
-      </c>
-      <c r="B1190" s="21" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="C1190" s="22" t="n"/>
-      <c r="D1190" s="22" t="n"/>
-      <c r="E1190" s="22" t="n"/>
-      <c r="F1190" s="22" t="n"/>
-    </row>
-    <row r="1191" ht="20" customHeight="1">
-      <c r="A1191" s="20" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="B1191" s="21" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="C1191" s="22" t="n"/>
-      <c r="D1191" s="22" t="n"/>
-      <c r="E1191" s="22" t="n"/>
-      <c r="F1191" s="22" t="n"/>
-    </row>
-    <row r="1192" ht="20" customHeight="1">
-      <c r="A1192" s="20" t="inlineStr">
-        <is>
-          <t>Deadline</t>
-        </is>
-      </c>
-      <c r="B1192" s="21" t="inlineStr"/>
-      <c r="C1192" s="22" t="n"/>
-      <c r="D1192" s="22" t="n"/>
-      <c r="E1192" s="22" t="n"/>
-      <c r="F1192" s="22" t="n"/>
-    </row>
-    <row r="1193" ht="20" customHeight="1">
-      <c r="A1193" s="20" t="inlineStr">
-        <is>
-          <t>Presupuesto (EUR)</t>
-        </is>
-      </c>
-      <c r="B1193" s="21" t="inlineStr">
-        <is>
-          <t>No disponible</t>
-        </is>
-      </c>
-      <c r="C1193" s="22" t="n"/>
-      <c r="D1193" s="22" t="n"/>
-      <c r="E1193" s="22" t="n"/>
-      <c r="F1193" s="22" t="n"/>
-    </row>
-    <row r="1194" ht="20" customHeight="1">
-      <c r="A1194" s="20" t="inlineStr">
-        <is>
-          <t>Tipo de Accion</t>
-        </is>
-      </c>
-      <c r="B1194" s="21" t="inlineStr">
-        <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="C1194" s="22" t="n"/>
-      <c r="D1194" s="22" t="n"/>
-      <c r="E1194" s="22" t="n"/>
-      <c r="F1194" s="22" t="n"/>
-    </row>
-    <row r="1195" ht="20" customHeight="1">
-      <c r="A1195" s="20" t="inlineStr">
-        <is>
-          <t>Call ID</t>
-        </is>
-      </c>
-      <c r="B1195" s="21" t="inlineStr"/>
-      <c r="C1195" s="22" t="n"/>
-      <c r="D1195" s="22" t="n"/>
-      <c r="E1195" s="22" t="n"/>
-      <c r="F1195" s="22" t="n"/>
-    </row>
-    <row r="1196" ht="20" customHeight="1">
-      <c r="A1196" s="20" t="inlineStr">
-        <is>
-          <t>Descripcion</t>
-        </is>
-      </c>
-      <c r="B1196" s="21" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="C1196" s="22" t="n"/>
-      <c r="D1196" s="22" t="n"/>
-      <c r="E1196" s="22" t="n"/>
-      <c r="F1196" s="22" t="n"/>
-    </row>
-    <row r="1197" ht="20" customHeight="1">
-      <c r="A1197" s="20" t="inlineStr">
-        <is>
-          <t>Tags</t>
-        </is>
-      </c>
-      <c r="B1197" s="21" t="inlineStr">
-        <is>
-          <t>energia</t>
-        </is>
-      </c>
-      <c r="C1197" s="22" t="n"/>
-      <c r="D1197" s="22" t="n"/>
-      <c r="E1197" s="22" t="n"/>
-      <c r="F1197" s="22" t="n"/>
-    </row>
-    <row r="1198" ht="20" customHeight="1">
-      <c r="A1198" s="20" t="inlineStr">
-        <is>
-          <t>Relevancia Bilbao</t>
-        </is>
-      </c>
-      <c r="B1198" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
-        </is>
-      </c>
-      <c r="C1198" s="22" t="n"/>
-      <c r="D1198" s="22" t="n"/>
-      <c r="E1198" s="22" t="n"/>
-      <c r="F1198" s="22" t="n"/>
-    </row>
-    <row r="1199" ht="45" customHeight="1">
-      <c r="A1199" s="20" t="inlineStr">
-        <is>
-          <t>Enlace al portal</t>
-        </is>
-      </c>
-      <c r="B1199" s="23" t="inlineStr">
-        <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministros-agua/expcm507333/web01-tramite/es/</t>
-        </is>
-      </c>
-      <c r="C1199" s="22" t="n"/>
-      <c r="D1199" s="22" t="n"/>
-      <c r="E1199" s="22" t="n"/>
-      <c r="F1199" s="22" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="1120">
+  <mergeCells count="1050">
     <mergeCell ref="B679:F679"/>
     <mergeCell ref="B666:F666"/>
     <mergeCell ref="B964:F964"/>
@@ -22787,7 +21441,6 @@
     <mergeCell ref="B1012:F1012"/>
     <mergeCell ref="B484:F484"/>
     <mergeCell ref="B794:F794"/>
-    <mergeCell ref="B1183:F1183"/>
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B278:F278"/>
     <mergeCell ref="B253:F253"/>
@@ -22797,7 +21450,6 @@
     <mergeCell ref="B707:F707"/>
     <mergeCell ref="B812:F812"/>
     <mergeCell ref="B538:F538"/>
-    <mergeCell ref="B1176:F1176"/>
     <mergeCell ref="B869:F869"/>
     <mergeCell ref="B532:F532"/>
     <mergeCell ref="B799:F799"/>
@@ -22806,11 +21458,8 @@
     <mergeCell ref="B342:F342"/>
     <mergeCell ref="B578:F578"/>
     <mergeCell ref="A541:F541"/>
-    <mergeCell ref="B1148:F1148"/>
     <mergeCell ref="B1099:F1099"/>
     <mergeCell ref="B515:F515"/>
-    <mergeCell ref="B1128:F1128"/>
-    <mergeCell ref="B1193:F1193"/>
     <mergeCell ref="A841:F841"/>
     <mergeCell ref="B158:F158"/>
     <mergeCell ref="B1094:F1094"/>
@@ -22819,11 +21468,9 @@
     <mergeCell ref="B894:F894"/>
     <mergeCell ref="B133:F133"/>
     <mergeCell ref="B959:F959"/>
-    <mergeCell ref="B1130:F1130"/>
     <mergeCell ref="B369:F369"/>
     <mergeCell ref="B667:F667"/>
     <mergeCell ref="B418:F418"/>
-    <mergeCell ref="B1142:F1142"/>
     <mergeCell ref="B356:F356"/>
     <mergeCell ref="B160:F160"/>
     <mergeCell ref="B489:F489"/>
@@ -22847,13 +21494,11 @@
     <mergeCell ref="B662:F662"/>
     <mergeCell ref="B718:F718"/>
     <mergeCell ref="B889:F889"/>
-    <mergeCell ref="B1131:F1131"/>
     <mergeCell ref="B72:F72"/>
     <mergeCell ref="B954:F954"/>
     <mergeCell ref="B199:F199"/>
     <mergeCell ref="B370:F370"/>
     <mergeCell ref="B1025:F1025"/>
-    <mergeCell ref="B1196:F1196"/>
     <mergeCell ref="B1112:F1112"/>
     <mergeCell ref="B291:F291"/>
     <mergeCell ref="B655:F655"/>
@@ -22865,7 +21510,6 @@
     <mergeCell ref="B293:F293"/>
     <mergeCell ref="B657:F657"/>
     <mergeCell ref="B322:F322"/>
-    <mergeCell ref="B1191:F1191"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B672:F672"/>
     <mergeCell ref="B88:F88"/>
@@ -22909,7 +21553,6 @@
     <mergeCell ref="A346:F346"/>
     <mergeCell ref="B904:F904"/>
     <mergeCell ref="B635:F635"/>
-    <mergeCell ref="A1141:F1141"/>
     <mergeCell ref="B141:F141"/>
     <mergeCell ref="B439:F439"/>
     <mergeCell ref="A136:F136"/>
@@ -22930,7 +21573,6 @@
     <mergeCell ref="B530:F530"/>
     <mergeCell ref="B726:F726"/>
     <mergeCell ref="B962:F962"/>
-    <mergeCell ref="B1133:F1133"/>
     <mergeCell ref="A886:F886"/>
     <mergeCell ref="B505:F505"/>
     <mergeCell ref="B1060:F1060"/>
@@ -22950,7 +21592,6 @@
     <mergeCell ref="B243:F243"/>
     <mergeCell ref="B1026:F1026"/>
     <mergeCell ref="B1075:F1075"/>
-    <mergeCell ref="B1197:F1197"/>
     <mergeCell ref="B678:F678"/>
     <mergeCell ref="B363:F363"/>
     <mergeCell ref="B534:F534"/>
@@ -22963,7 +21604,6 @@
     <mergeCell ref="B1055:F1055"/>
     <mergeCell ref="B536:F536"/>
     <mergeCell ref="B834:F834"/>
-    <mergeCell ref="B1143:F1143"/>
     <mergeCell ref="B899:F899"/>
     <mergeCell ref="B752:F752"/>
     <mergeCell ref="B1070:F1070"/>
@@ -22983,7 +21623,6 @@
     <mergeCell ref="B1044:F1044"/>
     <mergeCell ref="B156:F156"/>
     <mergeCell ref="B327:F327"/>
-    <mergeCell ref="B1144:F1144"/>
     <mergeCell ref="B454:F454"/>
     <mergeCell ref="B625:F625"/>
     <mergeCell ref="B923:F923"/>
@@ -23004,13 +21643,11 @@
     <mergeCell ref="B562:F562"/>
     <mergeCell ref="B689:F689"/>
     <mergeCell ref="B1121:F1121"/>
-    <mergeCell ref="B1146:F1146"/>
     <mergeCell ref="B1123:F1123"/>
     <mergeCell ref="B86:F86"/>
     <mergeCell ref="B912:F912"/>
     <mergeCell ref="B1083:F1083"/>
     <mergeCell ref="B262:F262"/>
-    <mergeCell ref="A1186:F1186"/>
     <mergeCell ref="B887:F887"/>
     <mergeCell ref="B862:F862"/>
     <mergeCell ref="B547:F547"/>
@@ -23024,7 +21661,6 @@
     <mergeCell ref="B1007:F1007"/>
     <mergeCell ref="B1001:F1001"/>
     <mergeCell ref="B246:F246"/>
-    <mergeCell ref="B1174:F1174"/>
     <mergeCell ref="B40:F40"/>
     <mergeCell ref="B338:F338"/>
     <mergeCell ref="B469:F469"/>
@@ -23095,7 +21731,6 @@
     <mergeCell ref="A226:F226"/>
     <mergeCell ref="B1124:F1124"/>
     <mergeCell ref="B394:F394"/>
-    <mergeCell ref="B1162:F1162"/>
     <mergeCell ref="B692:F692"/>
     <mergeCell ref="A931:F931"/>
     <mergeCell ref="B486:F486"/>
@@ -23111,7 +21746,6 @@
     <mergeCell ref="A526:F526"/>
     <mergeCell ref="B694:F694"/>
     <mergeCell ref="B786:F786"/>
-    <mergeCell ref="B1179:F1179"/>
     <mergeCell ref="B54:F54"/>
     <mergeCell ref="A286:F286"/>
     <mergeCell ref="B125:F125"/>
@@ -23119,7 +21753,6 @@
     <mergeCell ref="B185:F185"/>
     <mergeCell ref="A826:F826"/>
     <mergeCell ref="B483:F483"/>
-    <mergeCell ref="B1165:F1165"/>
     <mergeCell ref="B581:F581"/>
     <mergeCell ref="B1048:F1048"/>
     <mergeCell ref="B475:F475"/>
@@ -23146,23 +21779,19 @@
     <mergeCell ref="B1117:F1117"/>
     <mergeCell ref="B107:F107"/>
     <mergeCell ref="B1104:F1104"/>
-    <mergeCell ref="B1160:F1160"/>
     <mergeCell ref="B641:F641"/>
     <mergeCell ref="B57:F57"/>
     <mergeCell ref="B883:F883"/>
     <mergeCell ref="B908:F908"/>
     <mergeCell ref="B171:F171"/>
-    <mergeCell ref="B1168:F1168"/>
     <mergeCell ref="B407:F407"/>
     <mergeCell ref="A646:F646"/>
     <mergeCell ref="B972:F972"/>
     <mergeCell ref="B9:F9"/>
     <mergeCell ref="B463:F463"/>
     <mergeCell ref="B438:F438"/>
-    <mergeCell ref="B1145:F1145"/>
     <mergeCell ref="B359:F359"/>
     <mergeCell ref="B207:F207"/>
-    <mergeCell ref="B1194:F1194"/>
     <mergeCell ref="B788:F788"/>
     <mergeCell ref="B204:F204"/>
     <mergeCell ref="B198:F198"/>
@@ -23175,9 +21804,7 @@
     <mergeCell ref="B999:F999"/>
     <mergeCell ref="B1061:F1061"/>
     <mergeCell ref="B4:F4"/>
-    <mergeCell ref="B1188:F1188"/>
     <mergeCell ref="B1097:F1097"/>
-    <mergeCell ref="B1153:F1153"/>
     <mergeCell ref="A46:F46"/>
     <mergeCell ref="B507:F507"/>
     <mergeCell ref="B62:F62"/>
@@ -23193,7 +21820,6 @@
     <mergeCell ref="B857:F857"/>
     <mergeCell ref="B1063:F1063"/>
     <mergeCell ref="B1090:F1090"/>
-    <mergeCell ref="B1161:F1161"/>
     <mergeCell ref="B807:F807"/>
     <mergeCell ref="B1000:F1000"/>
     <mergeCell ref="B39:F39"/>
@@ -23211,7 +21837,6 @@
     <mergeCell ref="B818:F818"/>
     <mergeCell ref="B712:F712"/>
     <mergeCell ref="B128:F128"/>
-    <mergeCell ref="B1181:F1181"/>
     <mergeCell ref="B426:F426"/>
     <mergeCell ref="B364:F364"/>
     <mergeCell ref="B413:F413"/>
@@ -23229,7 +21854,6 @@
     <mergeCell ref="B428:F428"/>
     <mergeCell ref="B1118:F1118"/>
     <mergeCell ref="B284:F284"/>
-    <mergeCell ref="B1167:F1167"/>
     <mergeCell ref="B222:F222"/>
     <mergeCell ref="B344:F344"/>
     <mergeCell ref="B415:F415"/>
@@ -23252,13 +21876,11 @@
     <mergeCell ref="B948:F948"/>
     <mergeCell ref="B715:F715"/>
     <mergeCell ref="B1013:F1013"/>
-    <mergeCell ref="B1184:F1184"/>
     <mergeCell ref="B861:F861"/>
     <mergeCell ref="B504:F504"/>
     <mergeCell ref="B802:F802"/>
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B789:F789"/>
-    <mergeCell ref="B1136:F1136"/>
     <mergeCell ref="B248:F248"/>
     <mergeCell ref="B297:F297"/>
     <mergeCell ref="B813:F813"/>
@@ -23290,10 +21912,7 @@
     <mergeCell ref="B637:F637"/>
     <mergeCell ref="B808:F808"/>
     <mergeCell ref="B879:F879"/>
-    <mergeCell ref="B1177:F1177"/>
     <mergeCell ref="B897:F897"/>
-    <mergeCell ref="B1164:F1164"/>
-    <mergeCell ref="B1158:F1158"/>
     <mergeCell ref="B403:F403"/>
     <mergeCell ref="B574:F574"/>
     <mergeCell ref="B745:F745"/>
@@ -23301,7 +21920,6 @@
     <mergeCell ref="B55:F55"/>
     <mergeCell ref="B1003:F1003"/>
     <mergeCell ref="B169:F169"/>
-    <mergeCell ref="B1166:F1166"/>
     <mergeCell ref="A706:F706"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B129:F129"/>
@@ -23316,13 +21934,11 @@
     <mergeCell ref="B492:F492"/>
     <mergeCell ref="B734:F734"/>
     <mergeCell ref="B1082:F1082"/>
-    <mergeCell ref="B1189:F1189"/>
     <mergeCell ref="B528:F528"/>
     <mergeCell ref="B71:F71"/>
     <mergeCell ref="B1019:F1019"/>
     <mergeCell ref="B131:F131"/>
     <mergeCell ref="B236:F236"/>
-    <mergeCell ref="B1190:F1190"/>
     <mergeCell ref="B307:F307"/>
     <mergeCell ref="B58:F58"/>
     <mergeCell ref="B429:F429"/>
@@ -23342,7 +21958,6 @@
     <mergeCell ref="B890:F890"/>
     <mergeCell ref="B950:F950"/>
     <mergeCell ref="B1034:F1034"/>
-    <mergeCell ref="B1192:F1192"/>
     <mergeCell ref="B431:F431"/>
     <mergeCell ref="B231:F231"/>
     <mergeCell ref="B287:F287"/>
@@ -23362,7 +21977,6 @@
     <mergeCell ref="A721:F721"/>
     <mergeCell ref="A31:F31"/>
     <mergeCell ref="B747:F747"/>
-    <mergeCell ref="B1152:F1152"/>
     <mergeCell ref="B668:F668"/>
     <mergeCell ref="B84:F84"/>
     <mergeCell ref="A736:F736"/>
@@ -23399,13 +22013,11 @@
     <mergeCell ref="B880:F880"/>
     <mergeCell ref="B1116:F1116"/>
     <mergeCell ref="B671:F671"/>
-    <mergeCell ref="B1187:F1187"/>
     <mergeCell ref="B969:F969"/>
     <mergeCell ref="B907:F907"/>
     <mergeCell ref="B963:F963"/>
     <mergeCell ref="B208:F208"/>
     <mergeCell ref="B882:F882"/>
-    <mergeCell ref="B1180:F1180"/>
     <mergeCell ref="B219:F219"/>
     <mergeCell ref="B460:F460"/>
     <mergeCell ref="B517:F517"/>
@@ -23425,7 +22037,6 @@
     <mergeCell ref="B520:F520"/>
     <mergeCell ref="B958:F958"/>
     <mergeCell ref="B308:F308"/>
-    <mergeCell ref="B1134:F1134"/>
     <mergeCell ref="B854:F854"/>
     <mergeCell ref="B99:F99"/>
     <mergeCell ref="B737:F737"/>
@@ -23444,22 +22055,17 @@
     <mergeCell ref="B372:F372"/>
     <mergeCell ref="B1071:F1071"/>
     <mergeCell ref="B608:F608"/>
-    <mergeCell ref="B1127:F1127"/>
-    <mergeCell ref="B1198:F1198"/>
     <mergeCell ref="B595:F595"/>
     <mergeCell ref="B1037:F1037"/>
     <mergeCell ref="B722:F722"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="A856:F856"/>
     <mergeCell ref="B893:F893"/>
-    <mergeCell ref="B1195:F1195"/>
-    <mergeCell ref="B1129:F1129"/>
     <mergeCell ref="B374:F374"/>
     <mergeCell ref="B659:F659"/>
     <mergeCell ref="B830:F830"/>
     <mergeCell ref="A871:F871"/>
     <mergeCell ref="B895:F895"/>
-    <mergeCell ref="A1156:F1156"/>
     <mergeCell ref="B232:F232"/>
     <mergeCell ref="B321:F321"/>
     <mergeCell ref="B215:F215"/>
@@ -23523,13 +22129,11 @@
     <mergeCell ref="B309:F309"/>
     <mergeCell ref="A316:F316"/>
     <mergeCell ref="B380:F380"/>
-    <mergeCell ref="B1135:F1135"/>
     <mergeCell ref="A1081:F1081"/>
     <mergeCell ref="B100:F100"/>
     <mergeCell ref="B336:F336"/>
     <mergeCell ref="B634:F634"/>
     <mergeCell ref="B876:F876"/>
-    <mergeCell ref="B1199:F1199"/>
     <mergeCell ref="B311:F311"/>
     <mergeCell ref="B140:F140"/>
     <mergeCell ref="B115:F115"/>
@@ -23539,7 +22143,6 @@
     <mergeCell ref="A376:F376"/>
     <mergeCell ref="B102:F102"/>
     <mergeCell ref="B674:F674"/>
-    <mergeCell ref="B1137:F1137"/>
     <mergeCell ref="B400:F400"/>
     <mergeCell ref="B698:F698"/>
     <mergeCell ref="B832:F832"/>
@@ -23552,10 +22155,8 @@
     <mergeCell ref="B598:F598"/>
     <mergeCell ref="B402:F402"/>
     <mergeCell ref="B669:F669"/>
-    <mergeCell ref="B1138:F1138"/>
     <mergeCell ref="B377:F377"/>
     <mergeCell ref="A451:F451"/>
-    <mergeCell ref="A1171:F1171"/>
     <mergeCell ref="B29:F29"/>
     <mergeCell ref="A901:F901"/>
     <mergeCell ref="B563:F563"/>
@@ -23563,7 +22164,6 @@
     <mergeCell ref="B756:F756"/>
     <mergeCell ref="B992:F992"/>
     <mergeCell ref="A811:F811"/>
-    <mergeCell ref="B1150:F1150"/>
     <mergeCell ref="B329:F329"/>
     <mergeCell ref="B627:F627"/>
     <mergeCell ref="B49:F49"/>
@@ -23611,7 +22211,6 @@
     <mergeCell ref="B845:F845"/>
     <mergeCell ref="B261:F261"/>
     <mergeCell ref="B1087:F1087"/>
-    <mergeCell ref="B1149:F1149"/>
     <mergeCell ref="B184:F184"/>
     <mergeCell ref="B1062:F1062"/>
     <mergeCell ref="A301:F301"/>
@@ -23628,12 +22227,10 @@
     <mergeCell ref="B769:F769"/>
     <mergeCell ref="B940:F940"/>
     <mergeCell ref="B878:F878"/>
-    <mergeCell ref="B1182:F1182"/>
     <mergeCell ref="B179:F179"/>
     <mergeCell ref="B250:F250"/>
     <mergeCell ref="B927:F927"/>
     <mergeCell ref="B44:F44"/>
-    <mergeCell ref="B1163:F1163"/>
     <mergeCell ref="B408:F408"/>
     <mergeCell ref="B464:F464"/>
     <mergeCell ref="A916:F916"/>
@@ -23700,8 +22297,6 @@
     <mergeCell ref="B1024:F1024"/>
     <mergeCell ref="B396:F396"/>
     <mergeCell ref="B567:F567"/>
-    <mergeCell ref="B1151:F1151"/>
-    <mergeCell ref="B1157:F1157"/>
     <mergeCell ref="B632:F632"/>
     <mergeCell ref="B803:F803"/>
     <mergeCell ref="B996:F996"/>
@@ -23712,7 +22307,6 @@
     <mergeCell ref="B267:F267"/>
     <mergeCell ref="B798:F798"/>
     <mergeCell ref="B1088:F1088"/>
-    <mergeCell ref="B1159:F1159"/>
     <mergeCell ref="B398:F398"/>
     <mergeCell ref="B569:F569"/>
     <mergeCell ref="A466:F466"/>
@@ -23722,7 +22316,6 @@
     <mergeCell ref="B269:F269"/>
     <mergeCell ref="B187:F187"/>
     <mergeCell ref="B485:F485"/>
-    <mergeCell ref="B1154:F1154"/>
     <mergeCell ref="B124:F124"/>
     <mergeCell ref="B251:F251"/>
     <mergeCell ref="B806:F806"/>
@@ -23732,7 +22325,6 @@
     <mergeCell ref="B487:F487"/>
     <mergeCell ref="B1077:F1077"/>
     <mergeCell ref="B343:F343"/>
-    <mergeCell ref="B1169:F1169"/>
     <mergeCell ref="B414:F414"/>
     <mergeCell ref="B474:F474"/>
     <mergeCell ref="B772:F772"/>
@@ -23776,8 +22368,6 @@
     <mergeCell ref="B1101:F1101"/>
     <mergeCell ref="B582:F582"/>
     <mergeCell ref="B849:F849"/>
-    <mergeCell ref="B1147:F1147"/>
-    <mergeCell ref="B1132:F1132"/>
     <mergeCell ref="B73:F73"/>
     <mergeCell ref="B371:F371"/>
     <mergeCell ref="B638:F638"/>
@@ -23785,7 +22375,6 @@
     <mergeCell ref="B968:F968"/>
     <mergeCell ref="B874:F874"/>
     <mergeCell ref="B656:F656"/>
-    <mergeCell ref="B1172:F1172"/>
     <mergeCell ref="B727:F727"/>
     <mergeCell ref="A991:F991"/>
     <mergeCell ref="A676:F676"/>
@@ -23813,13 +22402,11 @@
     <mergeCell ref="B114:F114"/>
     <mergeCell ref="B498:F498"/>
     <mergeCell ref="B1002:F1002"/>
-    <mergeCell ref="B1173:F1173"/>
     <mergeCell ref="B212:F212"/>
     <mergeCell ref="B206:F206"/>
     <mergeCell ref="B399:F399"/>
     <mergeCell ref="B203:F203"/>
     <mergeCell ref="B1004:F1004"/>
-    <mergeCell ref="B1175:F1175"/>
     <mergeCell ref="B860:F860"/>
     <mergeCell ref="B66:F66"/>
     <mergeCell ref="B326:F326"/>
@@ -23847,7 +22434,6 @@
     <mergeCell ref="B1045:F1045"/>
     <mergeCell ref="B119:F119"/>
     <mergeCell ref="B290:F290"/>
-    <mergeCell ref="B1178:F1178"/>
     <mergeCell ref="B417:F417"/>
     <mergeCell ref="B588:F588"/>
     <mergeCell ref="B653:F653"/>
@@ -23857,7 +22443,6 @@
     <mergeCell ref="B367:F367"/>
     <mergeCell ref="B1122:F1122"/>
     <mergeCell ref="B427:F427"/>
-    <mergeCell ref="B1139:F1139"/>
     <mergeCell ref="B112:F112"/>
     <mergeCell ref="B283:F283"/>
     <mergeCell ref="B354:F354"/>
@@ -23877,7 +22462,6 @@
     <mergeCell ref="B648:F648"/>
     <mergeCell ref="B64:F64"/>
     <mergeCell ref="B51:F51"/>
-    <mergeCell ref="A1126:F1126"/>
     <mergeCell ref="B443:F443"/>
     <mergeCell ref="A196:F196"/>
     <mergeCell ref="B237:F237"/>
@@ -23958,11 +22542,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1094" r:id="rId73"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1109" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1124" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1139" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1154" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1169" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1184" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1199" r:id="rId80"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -23974,7 +22553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J81"/>
+  <dimension ref="A1:J76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -24884,12 +23463,12 @@
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-08</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Palaeoclimate science for a better understanding of Earth sy</t>
+          <t>Advancing understanding, modelling and prediction of extreme</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -25004,12 +23583,12 @@
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Assessing the performance of policy instruments to inform cl</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
@@ -25044,12 +23623,12 @@
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Palaeoclimate science for a better understanding of Earth sy</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
@@ -25084,12 +23663,12 @@
     <row r="28" ht="28" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform cl</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -25124,12 +23703,12 @@
     <row r="29" ht="28" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
@@ -26456,12 +25035,12 @@
     <row r="65" ht="28" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>BDNS-901096</t>
+          <t>BDNS-901505</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>Ayudas económicas al desarrollo y producción de proyectos au</t>
+          <t>CONVENIO DE SUBVENCIÓN NOMINATIVA PARA LA ASOCIACIÓN KULTURA</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -26476,7 +25055,7 @@
       </c>
       <c r="E65" s="6" t="inlineStr">
         <is>
-          <t>01/06/2026</t>
+          <t>31/12/2026</t>
         </is>
       </c>
       <c r="F65" s="27" t="inlineStr">
@@ -26496,17 +25075,17 @@
     <row r="66" ht="28" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>BDNS-901505</t>
+          <t>EUS-74664</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>CONVENIO DE SUBVENCIÓN NOMINATIVA PARA LA ASOCIACIÓN KULTURA</t>
+          <t>LIFE 2026. Medio ambiente. Ayudas de 4 subprogramas, de natu</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>VITORIA-GASTEIZ</t>
+          <t>Euskadi</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
@@ -26514,14 +25093,10 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="E66" s="6" t="inlineStr">
-        <is>
-          <t>31/12/2026</t>
-        </is>
-      </c>
+      <c r="E66" s="6" t="inlineStr"/>
       <c r="F66" s="27" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="G66" s="6" t="inlineStr"/>
@@ -26536,12 +25111,12 @@
     <row r="67" ht="28" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>EUS-92454</t>
+          <t>EUS-70680</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>Suministro de licencias de software para las plataformas Mai</t>
+          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
@@ -26557,7 +25132,7 @@
       <c r="E67" s="6" t="inlineStr"/>
       <c r="F67" s="27" t="inlineStr">
         <is>
-          <t>MUY ALTA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="G67" s="6" t="inlineStr"/>
@@ -26572,12 +25147,12 @@
     <row r="68" ht="28" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>EUS-75183</t>
+          <t>EUS-31421</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>LIFE 2026. Medio ambiente. Ayudas de 4 subprogramas, de natu</t>
+          <t>Contrato mixto de suministro y obra para la sustitución y ac</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -26608,12 +25183,12 @@
     <row r="69" ht="28" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>EUS-02830</t>
+          <t>EUS-13213</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>Ayudas a la eficiencia energética y mitigación del cambio cl</t>
+          <t xml:space="preserve">Mantenimiento de las instalacioens  de climatización, ACS y </t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -26644,12 +25219,12 @@
     <row r="70" ht="28" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>EUS-31407</t>
+          <t>EUS-28151</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>asistencia tecnica para el desarrollo de la campaña informat</t>
+          <t>Servicio de recogida separada y clasificación de residuos de</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -26680,7 +25255,7 @@
     <row r="71" ht="28" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>EUS-74304</t>
+          <t>EUS-86678</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
@@ -26716,7 +25291,7 @@
     <row r="72" ht="28" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>EUS-96161</t>
+          <t>EUS-71437</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
@@ -26752,7 +25327,7 @@
     <row r="73" ht="28" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>EUS-04369</t>
+          <t>EUS-71705</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
@@ -26788,12 +25363,12 @@
     <row r="74" ht="28" customHeight="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>EUS-86318</t>
+          <t>EUS-79070</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>Contratación de los servicios de formación en materia ESG, r</t>
+          <t>Servicio de recogida de animales domésticos</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
@@ -26824,12 +25399,12 @@
     <row r="75" ht="28" customHeight="1">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>EUS-63953</t>
+          <t>EUS-53277</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enajenación, mediante subasta, de la parcela urbana1-819 de </t>
+          <t>Servicio de transporte para el programa Ibiliaz Ezagutu de p</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
@@ -26860,12 +25435,12 @@
     <row r="76" ht="28" customHeight="1">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>EUS-29174</t>
+          <t>EUS-45140</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>Elaboración, transporte y entrega de comidas preparadas y pr</t>
+          <t>Cubierta de patio CEIP BAGATZA HLHI, Barakaldo (Bizkaia)</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
@@ -26893,188 +25468,8 @@
       <c r="I76" s="6" t="inlineStr"/>
       <c r="J76" s="6" t="inlineStr"/>
     </row>
-    <row r="77" ht="28" customHeight="1">
-      <c r="A77" s="6" t="inlineStr">
-        <is>
-          <t>EUS-05384</t>
-        </is>
-      </c>
-      <c r="B77" s="6" t="inlineStr">
-        <is>
-          <t>Suministro Cajas transporte</t>
-        </is>
-      </c>
-      <c r="C77" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="D77" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E77" s="6" t="inlineStr"/>
-      <c r="F77" s="27" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="G77" s="6" t="inlineStr"/>
-      <c r="H77" s="6" t="inlineStr">
-        <is>
-          <t>Por revisar</t>
-        </is>
-      </c>
-      <c r="I77" s="6" t="inlineStr"/>
-      <c r="J77" s="6" t="inlineStr"/>
-    </row>
-    <row r="78" ht="28" customHeight="1">
-      <c r="A78" s="6" t="inlineStr">
-        <is>
-          <t>EUS-34859</t>
-        </is>
-      </c>
-      <c r="B78" s="6" t="inlineStr">
-        <is>
-          <t>Suministro Cajas transporte</t>
-        </is>
-      </c>
-      <c r="C78" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="D78" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E78" s="6" t="inlineStr"/>
-      <c r="F78" s="27" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="G78" s="6" t="inlineStr"/>
-      <c r="H78" s="6" t="inlineStr">
-        <is>
-          <t>Por revisar</t>
-        </is>
-      </c>
-      <c r="I78" s="6" t="inlineStr"/>
-      <c r="J78" s="6" t="inlineStr"/>
-    </row>
-    <row r="79" ht="28" customHeight="1">
-      <c r="A79" s="6" t="inlineStr">
-        <is>
-          <t>EUS-38583</t>
-        </is>
-      </c>
-      <c r="B79" s="6" t="inlineStr">
-        <is>
-          <t>Suministros Agua</t>
-        </is>
-      </c>
-      <c r="C79" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="D79" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E79" s="6" t="inlineStr"/>
-      <c r="F79" s="27" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="G79" s="6" t="inlineStr"/>
-      <c r="H79" s="6" t="inlineStr">
-        <is>
-          <t>Por revisar</t>
-        </is>
-      </c>
-      <c r="I79" s="6" t="inlineStr"/>
-      <c r="J79" s="6" t="inlineStr"/>
-    </row>
-    <row r="80" ht="28" customHeight="1">
-      <c r="A80" s="6" t="inlineStr">
-        <is>
-          <t>EUS-51111</t>
-        </is>
-      </c>
-      <c r="B80" s="6" t="inlineStr">
-        <is>
-          <t>Suministros Agua</t>
-        </is>
-      </c>
-      <c r="C80" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="D80" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E80" s="6" t="inlineStr"/>
-      <c r="F80" s="27" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="G80" s="6" t="inlineStr"/>
-      <c r="H80" s="6" t="inlineStr">
-        <is>
-          <t>Por revisar</t>
-        </is>
-      </c>
-      <c r="I80" s="6" t="inlineStr"/>
-      <c r="J80" s="6" t="inlineStr"/>
-    </row>
-    <row r="81" ht="28" customHeight="1">
-      <c r="A81" s="6" t="inlineStr">
-        <is>
-          <t>EUS-50384</t>
-        </is>
-      </c>
-      <c r="B81" s="6" t="inlineStr">
-        <is>
-          <t>Suministros Agua</t>
-        </is>
-      </c>
-      <c r="C81" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="D81" s="6" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="E81" s="6" t="inlineStr"/>
-      <c r="F81" s="27" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
-        </is>
-      </c>
-      <c r="G81" s="6" t="inlineStr"/>
-      <c r="H81" s="6" t="inlineStr">
-        <is>
-          <t>Por revisar</t>
-        </is>
-      </c>
-      <c r="I81" s="6" t="inlineStr"/>
-      <c r="J81" s="6" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J81"/>
+  <autoFilter ref="A1:J76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update funding data 2026-05-02
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -84,13 +84,13 @@
     <font>
       <name val="Leelawadee UI"/>
       <b val="1"/>
-      <color rgb="00DC2626"/>
+      <color rgb="00065F46"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Leelawadee UI"/>
       <b val="1"/>
-      <color rgb="00065F46"/>
+      <color rgb="00DC2626"/>
       <sz val="10"/>
     </font>
     <font>
@@ -166,17 +166,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00065F46"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -268,11 +268,11 @@
     <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -312,8 +312,8 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -707,7 +707,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 01/05/2026 08:02 - 72 convocatorias - 9 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 02/05/2026 07:22 - 72 convocatorias - 8 nuevas</t>
         </is>
       </c>
     </row>
@@ -4573,11 +4573,7 @@
           <t>PERSONAS JURÍDICAS QUE NO DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
         </is>
       </c>
-      <c r="L70" s="15" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
+      <c r="L70" s="6" t="inlineStr"/>
       <c r="M70" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
@@ -4585,21 +4581,21 @@
       </c>
     </row>
     <row r="71" ht="28" customHeight="1">
-      <c r="A71" s="16" t="inlineStr">
+      <c r="A71" s="15" t="inlineStr">
         <is>
           <t>🟢 Euskadi</t>
         </is>
       </c>
     </row>
     <row r="72" ht="40" customHeight="1">
-      <c r="A72" s="17" t="inlineStr">
+      <c r="A72" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>EUS-20289</t>
+          <t>EUS-49329</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -4635,7 +4631,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L72" s="15" t="inlineStr">
+      <c r="L72" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4647,14 +4643,14 @@
       </c>
     </row>
     <row r="73" ht="40" customHeight="1">
-      <c r="A73" s="17" t="inlineStr">
+      <c r="A73" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>EUS-69486</t>
+          <t>EUS-81737</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -4690,7 +4686,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L73" s="15" t="inlineStr">
+      <c r="L73" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4702,14 +4698,14 @@
       </c>
     </row>
     <row r="74" ht="40" customHeight="1">
-      <c r="A74" s="17" t="inlineStr">
+      <c r="A74" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>EUS-04272</t>
+          <t>EUS-00039</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
@@ -4745,7 +4741,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L74" s="15" t="inlineStr">
+      <c r="L74" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4757,14 +4753,14 @@
       </c>
     </row>
     <row r="75" ht="40" customHeight="1">
-      <c r="A75" s="17" t="inlineStr">
+      <c r="A75" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>EUS-96111</t>
+          <t>EUS-28691</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
@@ -4800,7 +4796,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L75" s="15" t="inlineStr">
+      <c r="L75" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4812,14 +4808,14 @@
       </c>
     </row>
     <row r="76" ht="40" customHeight="1">
-      <c r="A76" s="17" t="inlineStr">
+      <c r="A76" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>EUS-61257</t>
+          <t>EUS-90174</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
@@ -4855,7 +4851,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L76" s="15" t="inlineStr">
+      <c r="L76" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4867,14 +4863,14 @@
       </c>
     </row>
     <row r="77" ht="40" customHeight="1">
-      <c r="A77" s="17" t="inlineStr">
+      <c r="A77" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>EUS-86924</t>
+          <t>EUS-64378</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
@@ -4910,7 +4906,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L77" s="15" t="inlineStr">
+      <c r="L77" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4922,14 +4918,14 @@
       </c>
     </row>
     <row r="78" ht="40" customHeight="1">
-      <c r="A78" s="17" t="inlineStr">
+      <c r="A78" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>EUS-47262</t>
+          <t>EUS-72310</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
@@ -4965,7 +4961,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L78" s="15" t="inlineStr">
+      <c r="L78" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4977,14 +4973,14 @@
       </c>
     </row>
     <row r="79" ht="40" customHeight="1">
-      <c r="A79" s="17" t="inlineStr">
+      <c r="A79" s="16" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>EUS-19829</t>
+          <t>EUS-62265</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
@@ -5020,7 +5016,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L79" s="15" t="inlineStr">
+      <c r="L79" s="17" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -18918,7 +18914,7 @@
     <row r="961" ht="30" customHeight="1">
       <c r="A961" s="18" t="inlineStr">
         <is>
-          <t>FICHA 65: EUS-20289</t>
+          <t>FICHA 65: EUS-49329</t>
         </is>
       </c>
       <c r="B961" s="19" t="n"/>
@@ -18967,7 +18963,7 @@
       </c>
       <c r="B964" s="21" t="inlineStr">
         <is>
-          <t>EUS-20289</t>
+          <t>EUS-49329</t>
         </is>
       </c>
       <c r="C964" s="22" t="n"/>
@@ -19130,7 +19126,7 @@
     <row r="976" ht="30" customHeight="1">
       <c r="A976" s="18" t="inlineStr">
         <is>
-          <t>FICHA 66: EUS-69486</t>
+          <t>FICHA 66: EUS-81737</t>
         </is>
       </c>
       <c r="B976" s="19" t="n"/>
@@ -19179,7 +19175,7 @@
       </c>
       <c r="B979" s="21" t="inlineStr">
         <is>
-          <t>EUS-69486</t>
+          <t>EUS-81737</t>
         </is>
       </c>
       <c r="C979" s="22" t="n"/>
@@ -19342,7 +19338,7 @@
     <row r="991" ht="30" customHeight="1">
       <c r="A991" s="18" t="inlineStr">
         <is>
-          <t>FICHA 67: EUS-04272</t>
+          <t>FICHA 67: EUS-00039</t>
         </is>
       </c>
       <c r="B991" s="19" t="n"/>
@@ -19391,7 +19387,7 @@
       </c>
       <c r="B994" s="21" t="inlineStr">
         <is>
-          <t>EUS-04272</t>
+          <t>EUS-00039</t>
         </is>
       </c>
       <c r="C994" s="22" t="n"/>
@@ -19554,7 +19550,7 @@
     <row r="1006" ht="30" customHeight="1">
       <c r="A1006" s="18" t="inlineStr">
         <is>
-          <t>FICHA 68: EUS-96111</t>
+          <t>FICHA 68: EUS-28691</t>
         </is>
       </c>
       <c r="B1006" s="19" t="n"/>
@@ -19603,7 +19599,7 @@
       </c>
       <c r="B1009" s="21" t="inlineStr">
         <is>
-          <t>EUS-96111</t>
+          <t>EUS-28691</t>
         </is>
       </c>
       <c r="C1009" s="22" t="n"/>
@@ -19766,7 +19762,7 @@
     <row r="1021" ht="30" customHeight="1">
       <c r="A1021" s="18" t="inlineStr">
         <is>
-          <t>FICHA 69: EUS-61257</t>
+          <t>FICHA 69: EUS-90174</t>
         </is>
       </c>
       <c r="B1021" s="19" t="n"/>
@@ -19815,7 +19811,7 @@
       </c>
       <c r="B1024" s="21" t="inlineStr">
         <is>
-          <t>EUS-61257</t>
+          <t>EUS-90174</t>
         </is>
       </c>
       <c r="C1024" s="22" t="n"/>
@@ -19978,7 +19974,7 @@
     <row r="1036" ht="30" customHeight="1">
       <c r="A1036" s="18" t="inlineStr">
         <is>
-          <t>FICHA 70: EUS-86924</t>
+          <t>FICHA 70: EUS-64378</t>
         </is>
       </c>
       <c r="B1036" s="19" t="n"/>
@@ -20027,7 +20023,7 @@
       </c>
       <c r="B1039" s="21" t="inlineStr">
         <is>
-          <t>EUS-86924</t>
+          <t>EUS-64378</t>
         </is>
       </c>
       <c r="C1039" s="22" t="n"/>
@@ -20190,7 +20186,7 @@
     <row r="1051" ht="30" customHeight="1">
       <c r="A1051" s="18" t="inlineStr">
         <is>
-          <t>FICHA 71: EUS-47262</t>
+          <t>FICHA 71: EUS-72310</t>
         </is>
       </c>
       <c r="B1051" s="19" t="n"/>
@@ -20239,7 +20235,7 @@
       </c>
       <c r="B1054" s="21" t="inlineStr">
         <is>
-          <t>EUS-47262</t>
+          <t>EUS-72310</t>
         </is>
       </c>
       <c r="C1054" s="22" t="n"/>
@@ -20402,7 +20398,7 @@
     <row r="1066" ht="30" customHeight="1">
       <c r="A1066" s="18" t="inlineStr">
         <is>
-          <t>FICHA 72: EUS-19829</t>
+          <t>FICHA 72: EUS-62265</t>
         </is>
       </c>
       <c r="B1066" s="19" t="n"/>
@@ -20451,7 +20447,7 @@
       </c>
       <c r="B1069" s="21" t="inlineStr">
         <is>
-          <t>EUS-19829</t>
+          <t>EUS-62265</t>
         </is>
       </c>
       <c r="C1069" s="22" t="n"/>
@@ -24228,7 +24224,7 @@
     <row r="66" ht="28" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>EUS-20289</t>
+          <t>EUS-49329</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
@@ -24264,7 +24260,7 @@
     <row r="67" ht="28" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>EUS-69486</t>
+          <t>EUS-81737</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
@@ -24300,7 +24296,7 @@
     <row r="68" ht="28" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>EUS-04272</t>
+          <t>EUS-00039</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
@@ -24336,7 +24332,7 @@
     <row r="69" ht="28" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>EUS-96111</t>
+          <t>EUS-28691</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
@@ -24372,7 +24368,7 @@
     <row r="70" ht="28" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>EUS-61257</t>
+          <t>EUS-90174</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
@@ -24408,7 +24404,7 @@
     <row r="71" ht="28" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>EUS-86924</t>
+          <t>EUS-64378</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
@@ -24444,7 +24440,7 @@
     <row r="72" ht="28" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>EUS-47262</t>
+          <t>EUS-72310</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
@@ -24480,7 +24476,7 @@
     <row r="73" ht="28" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>EUS-19829</t>
+          <t>EUS-62265</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Update funding data 2026-05-03
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Recursos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$79</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$74</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -679,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M79"/>
+  <dimension ref="A1:M80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -707,7 +707,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 02/05/2026 07:22 - 72 convocatorias - 8 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 03/05/2026 07:47 - 73 convocatorias - 9 nuevas</t>
         </is>
       </c>
     </row>
@@ -2041,12 +2041,12 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-08</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
+          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -2086,7 +2086,7 @@
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and inter</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Euro</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr"/>
@@ -2230,12 +2230,12 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>Programme Cofund Actions</t>
+          <t xml:space="preserve"> Research and Innovation Actions</t>
         </is>
       </c>
       <c r="I29" s="10" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="K29" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is estab</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to info</t>
         </is>
       </c>
       <c r="L29" s="6" t="inlineStr"/>
@@ -2293,12 +2293,12 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -2338,7 +2338,7 @@
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorpo</t>
+          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and inter</t>
         </is>
       </c>
       <c r="L30" s="6" t="inlineStr"/>
@@ -2356,12 +2356,12 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Research and Innovation Actions</t>
+          <t>Programme Cofund Actions</t>
         </is>
       </c>
       <c r="I31" s="10" t="inlineStr">
@@ -2401,7 +2401,7 @@
       </c>
       <c r="K31" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to info</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is estab</t>
         </is>
       </c>
       <c r="L31" s="6" t="inlineStr"/>
@@ -2419,12 +2419,12 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Euro</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorpo</t>
         </is>
       </c>
       <c r="L32" s="6" t="inlineStr"/>
@@ -4595,12 +4595,12 @@
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>EUS-49329</t>
+          <t>EUS-13454</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>LIFE 2026. Medio ambiente. Ayudas de 4 subprogramas, de naturaleza y biodiversidad, circularidad y calidad de vida, cambio climático y transición energética. Con inscripción abierta para jornadas info</t>
+          <t>Suministro de energia eléctrica a distintos puntos de consumo de los que es titular el Ayuntamiento.</t>
         </is>
       </c>
       <c r="D72" s="6" t="inlineStr">
@@ -4617,12 +4617,12 @@
       <c r="G72" s="6" t="inlineStr"/>
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
-        </is>
-      </c>
-      <c r="I72" s="11" t="inlineStr">
-        <is>
-          <t>ALTA</t>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I72" s="12" t="inlineStr">
+        <is>
+          <t>MUY ALTA</t>
         </is>
       </c>
       <c r="J72" s="6" t="inlineStr"/>
@@ -4650,12 +4650,12 @@
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>EUS-81737</t>
+          <t>EUS-59353</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>Ases. técnico diseño y plan de acción clima labora</t>
+          <t>LIFE 2026. Medio ambiente. Ayudas de 4 subprogramas, de naturaleza y biodiversidad, circularidad y calidad de vida, cambio climático y transición energética. Con inscripción abierta para jornadas info</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
@@ -4672,7 +4672,7 @@
       <c r="G73" s="6" t="inlineStr"/>
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="I73" s="11" t="inlineStr">
@@ -4705,12 +4705,12 @@
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>EUS-00039</t>
+          <t>EUS-00407</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>Plan de movilidad</t>
+          <t>Ases. técnico diseño y plan de acción clima labora</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr">
@@ -4760,12 +4760,12 @@
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>EUS-28691</t>
+          <t>EUS-78654</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta el 01.10.26. Cribado de enfermedades con inteligencia artificial. Espacio de Datos Sanitarios de la UE. Red de Centros para Seguridad de la I</t>
+          <t>Plan de movilidad</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
@@ -4782,12 +4782,12 @@
       <c r="G75" s="6" t="inlineStr"/>
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
-        </is>
-      </c>
-      <c r="I75" s="8" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I75" s="11" t="inlineStr">
+        <is>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="J75" s="6" t="inlineStr"/>
@@ -4815,12 +4815,12 @@
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>EUS-90174</t>
+          <t>EUS-15400</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversidad, participación, principios de la UE. Eventos, difusiones e intercambios. Programa de Ciudadanos, Igualdad, Derechos y Valores de la UE (</t>
+          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta el 01.10.26. Cribado de enfermedades con inteligencia artificial. Espacio de Datos Sanitarios de la UE. Red de Centros para Seguridad de la I</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr">
@@ -4870,12 +4870,12 @@
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>EUS-64378</t>
+          <t>EUS-82152</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el marco de la Intervención Sectorial Vitivinícola del Plan Estratégico (PEPAC) de la Política Agrícola Común de la UE 2023-2027</t>
+          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversidad, participación, principios de la UE. Eventos, difusiones e intercambios. Programa de Ciudadanos, Igualdad, Derechos y Valores de la UE (</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
@@ -4925,12 +4925,12 @@
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>EUS-72310</t>
+          <t>EUS-50992</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>Recogida de muestras de legionella mediante pcr en el acs de orbea</t>
+          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el marco de la Intervención Sectorial Vitivinícola del Plan Estratégico (PEPAC) de la Política Agrícola Común de la UE 2023-2027</t>
         </is>
       </c>
       <c r="D78" s="6" t="inlineStr">
@@ -4947,7 +4947,7 @@
       <c r="G78" s="6" t="inlineStr"/>
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="I78" s="8" t="inlineStr">
@@ -4980,12 +4980,12 @@
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>EUS-62265</t>
+          <t>EUS-73686</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>Coffee break Vititransfer Laguardia</t>
+          <t>Recogida de muestras de legionella mediante pcr en el acs de orbea</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
@@ -5027,8 +5027,63 @@
         </is>
       </c>
     </row>
+    <row r="80" ht="40" customHeight="1">
+      <c r="A80" s="16" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>EUS-57575</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>Coffee break Vititransfer Laguardia</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F80" s="6" t="inlineStr"/>
+      <c r="G80" s="6" t="inlineStr"/>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I80" s="8" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J80" s="6" t="inlineStr"/>
+      <c r="K80" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L80" s="17" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M80" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:M79"/>
+  <autoFilter ref="A4:M80"/>
   <mergeCells count="5">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A5:M5"/>
@@ -5109,6 +5164,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M77" r:id="rId70"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M78" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M79" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M80" r:id="rId73"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5120,7 +5176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1079"/>
+  <dimension ref="A1:F1094"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -9466,7 +9522,7 @@
     <row r="301" ht="30" customHeight="1">
       <c r="A301" s="18" t="inlineStr">
         <is>
-          <t>FICHA 21: HORIZON-CL5-2027-01-D1-08</t>
+          <t>FICHA 21: HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="B301" s="19" t="n"/>
@@ -9491,7 +9547,7 @@
       <c r="E302" s="22" t="n"/>
       <c r="F302" s="22" t="n"/>
     </row>
-    <row r="303" ht="20" customHeight="1">
+    <row r="303" ht="45" customHeight="1">
       <c r="A303" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -9499,7 +9555,7 @@
       </c>
       <c r="B303" s="21" t="inlineStr">
         <is>
-          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
+          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
         </is>
       </c>
       <c r="C303" s="22" t="n"/>
@@ -9515,7 +9571,7 @@
       </c>
       <c r="B304" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-08</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C304" s="22" t="n"/>
@@ -9627,7 +9683,7 @@
       </c>
       <c r="B311" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and interactions with ecosystems, leading to improved Earth system models;Future climate change scenarios produced in light of past changes in the Earth system, in particular warm climates/high sea-level situations, and abrupt transitions;Identification of thresholds in Earth system components and better characterisation of driving mechanisms and feedbacks that may be responsible for non-linear behaviours,</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Europe and globally, as well as the interaction between different hazards, their cumulative and/or cascading effects.Enhanced seamless prediction and projection modelling and attribution capabilities for extreme events and their likelihood to support preparedness, response and resilience to climate change by EU and national and regional actors. The EU Union Preparedness Strategy, the EU Adaptation Str</t>
         </is>
       </c>
       <c r="C311" s="22" t="n"/>
@@ -9671,7 +9727,7 @@
       </c>
       <c r="B314" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-08</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C314" s="22" t="n"/>
@@ -10114,7 +10170,7 @@
     <row r="346" ht="30" customHeight="1">
       <c r="A346" s="18" t="inlineStr">
         <is>
-          <t>FICHA 24: HORIZON-CL5-2027-01-D1-11</t>
+          <t>FICHA 24: HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="B346" s="19" t="n"/>
@@ -10139,7 +10195,7 @@
       <c r="E347" s="22" t="n"/>
       <c r="F347" s="22" t="n"/>
     </row>
-    <row r="348" ht="20" customHeight="1">
+    <row r="348" ht="45" customHeight="1">
       <c r="A348" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -10147,7 +10203,7 @@
       </c>
       <c r="B348" s="21" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
         </is>
       </c>
       <c r="C348" s="22" t="n"/>
@@ -10163,7 +10219,7 @@
       </c>
       <c r="B349" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C349" s="22" t="n"/>
@@ -10243,7 +10299,7 @@
       </c>
       <c r="B354" s="21" t="inlineStr">
         <is>
-          <t>Programme Cofund Actions</t>
+          <t xml:space="preserve"> Research and Innovation Actions</t>
         </is>
       </c>
       <c r="C354" s="22" t="n"/>
@@ -10275,7 +10331,7 @@
       </c>
       <c r="B356" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is established through development and implementation of the Climate Action pillar of the EU-AU Research and Innovation Partnership on Climate Change and Sustainable Energy (CCSE),[1] in co-design between African and European partners;Reduced fragmentation by aligning the EU, national and multilateral R&amp;amp;I efforts with increased leverage and impact of funding;African scientific, policy and practice com</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to inform mitigation action and policy improvements, ensuring a fair transition and social acceptability;Methodologies are developed and improved for ex-ante assessment and ex-post evaluation of greenhouse gas emission reductions from climate policies and measures;Strengthened collaboration and established networks between researchers, policy experts and government officials involved in designing and eva</t>
         </is>
       </c>
       <c r="C356" s="22" t="n"/>
@@ -10319,7 +10375,7 @@
       </c>
       <c r="B359" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-11</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C359" s="22" t="n"/>
@@ -10330,7 +10386,7 @@
     <row r="361" ht="30" customHeight="1">
       <c r="A361" s="18" t="inlineStr">
         <is>
-          <t>FICHA 25: HORIZON-CL5-2027-01-D1-10</t>
+          <t>FICHA 25: HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="B361" s="19" t="n"/>
@@ -10363,7 +10419,7 @@
       </c>
       <c r="B363" s="21" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
         </is>
       </c>
       <c r="C363" s="22" t="n"/>
@@ -10379,7 +10435,7 @@
       </c>
       <c r="B364" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="C364" s="22" t="n"/>
@@ -10491,7 +10547,7 @@
       </c>
       <c r="B371" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorporation into main EU repositories, such as Climate-ADAPT or the portal of the EU Mission on Adaptation to Climate Change;The risk and adaptation assessment frameworks are improved by better integrating the maladaptation dimension;Guidelines and tools for maladaptation prevention and correction strategies are made available to adaptation stakeholders at relevant scales and inform the design and impl</t>
+          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and interactions with ecosystems, leading to improved Earth system models;Future climate change scenarios produced in light of past changes in the Earth system, in particular warm climates/high sea-level situations, and abrupt transitions;Identification of thresholds in Earth system components and better characterisation of driving mechanisms and feedbacks that may be responsible for non-linear behaviours,</t>
         </is>
       </c>
       <c r="C371" s="22" t="n"/>
@@ -10535,7 +10591,7 @@
       </c>
       <c r="B374" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-10</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="C374" s="22" t="n"/>
@@ -10546,7 +10602,7 @@
     <row r="376" ht="30" customHeight="1">
       <c r="A376" s="18" t="inlineStr">
         <is>
-          <t>FICHA 26: HORIZON-CL5-2027-01-D1-09</t>
+          <t>FICHA 26: HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="B376" s="19" t="n"/>
@@ -10571,7 +10627,7 @@
       <c r="E377" s="22" t="n"/>
       <c r="F377" s="22" t="n"/>
     </row>
-    <row r="378" ht="45" customHeight="1">
+    <row r="378" ht="20" customHeight="1">
       <c r="A378" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -10579,7 +10635,7 @@
       </c>
       <c r="B378" s="21" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="C378" s="22" t="n"/>
@@ -10595,7 +10651,7 @@
       </c>
       <c r="B379" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C379" s="22" t="n"/>
@@ -10675,7 +10731,7 @@
       </c>
       <c r="B384" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Research and Innovation Actions</t>
+          <t>Programme Cofund Actions</t>
         </is>
       </c>
       <c r="C384" s="22" t="n"/>
@@ -10707,7 +10763,7 @@
       </c>
       <c r="B386" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to inform mitigation action and policy improvements, ensuring a fair transition and social acceptability;Methodologies are developed and improved for ex-ante assessment and ex-post evaluation of greenhouse gas emission reductions from climate policies and measures;Strengthened collaboration and established networks between researchers, policy experts and government officials involved in designing and eva</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is established through development and implementation of the Climate Action pillar of the EU-AU Research and Innovation Partnership on Climate Change and Sustainable Energy (CCSE),[1] in co-design between African and European partners;Reduced fragmentation by aligning the EU, national and multilateral R&amp;amp;I efforts with increased leverage and impact of funding;African scientific, policy and practice com</t>
         </is>
       </c>
       <c r="C386" s="22" t="n"/>
@@ -10751,7 +10807,7 @@
       </c>
       <c r="B389" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-09</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C389" s="22" t="n"/>
@@ -10762,7 +10818,7 @@
     <row r="391" ht="30" customHeight="1">
       <c r="A391" s="18" t="inlineStr">
         <is>
-          <t>FICHA 27: HORIZON-CL5-2027-01-D1-07</t>
+          <t>FICHA 27: HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="B391" s="19" t="n"/>
@@ -10787,7 +10843,7 @@
       <c r="E392" s="22" t="n"/>
       <c r="F392" s="22" t="n"/>
     </row>
-    <row r="393" ht="45" customHeight="1">
+    <row r="393" ht="20" customHeight="1">
       <c r="A393" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -10795,7 +10851,7 @@
       </c>
       <c r="B393" s="21" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="C393" s="22" t="n"/>
@@ -10811,7 +10867,7 @@
       </c>
       <c r="B394" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C394" s="22" t="n"/>
@@ -10923,7 +10979,7 @@
       </c>
       <c r="B401" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Europe and globally, as well as the interaction between different hazards, their cumulative and/or cascading effects.Enhanced seamless prediction and projection modelling and attribution capabilities for extreme events and their likelihood to support preparedness, response and resilience to climate change by EU and national and regional actors. The EU Union Preparedness Strategy, the EU Adaptation Str</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorporation into main EU repositories, such as Climate-ADAPT or the portal of the EU Mission on Adaptation to Climate Change;The risk and adaptation assessment frameworks are improved by better integrating the maladaptation dimension;Guidelines and tools for maladaptation prevention and correction strategies are made available to adaptation stakeholders at relevant scales and inform the design and impl</t>
         </is>
       </c>
       <c r="C401" s="22" t="n"/>
@@ -10967,7 +11023,7 @@
       </c>
       <c r="B404" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-07</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C404" s="22" t="n"/>
@@ -18914,7 +18970,7 @@
     <row r="961" ht="30" customHeight="1">
       <c r="A961" s="18" t="inlineStr">
         <is>
-          <t>FICHA 65: EUS-49329</t>
+          <t>FICHA 65: EUS-13454</t>
         </is>
       </c>
       <c r="B961" s="19" t="n"/>
@@ -18947,7 +19003,7 @@
       </c>
       <c r="B963" s="21" t="inlineStr">
         <is>
-          <t>LIFE 2026. Medio ambiente. Ayudas de 4 subprogramas, de naturaleza y biodiversidad, circularidad y calidad de vida, cambio climático y transición energética. Con inscripción abierta para jornadas info</t>
+          <t>Suministro de energia eléctrica a distintos puntos de consumo de los que es titular el Ayuntamiento.</t>
         </is>
       </c>
       <c r="C963" s="22" t="n"/>
@@ -18963,7 +19019,7 @@
       </c>
       <c r="B964" s="21" t="inlineStr">
         <is>
-          <t>EUS-49329</t>
+          <t>EUS-13454</t>
         </is>
       </c>
       <c r="C964" s="22" t="n"/>
@@ -19039,7 +19095,7 @@
       </c>
       <c r="B969" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C969" s="22" t="n"/>
@@ -19097,9 +19153,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B973" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ALTA — </t>
+      <c r="B973" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MUY ALTA — </t>
         </is>
       </c>
       <c r="C973" s="22" t="n"/>
@@ -19115,7 +19171,7 @@
       </c>
       <c r="B974" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260421life4lerrotajarduna/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-energia-electrica-distintos-puntos-consumo-que-es-titular-ayuntamiento/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C974" s="22" t="n"/>
@@ -19126,7 +19182,7 @@
     <row r="976" ht="30" customHeight="1">
       <c r="A976" s="18" t="inlineStr">
         <is>
-          <t>FICHA 66: EUS-81737</t>
+          <t>FICHA 66: EUS-59353</t>
         </is>
       </c>
       <c r="B976" s="19" t="n"/>
@@ -19151,7 +19207,7 @@
       <c r="E977" s="22" t="n"/>
       <c r="F977" s="22" t="n"/>
     </row>
-    <row r="978" ht="20" customHeight="1">
+    <row r="978" ht="45" customHeight="1">
       <c r="A978" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -19159,7 +19215,7 @@
       </c>
       <c r="B978" s="21" t="inlineStr">
         <is>
-          <t>Ases. técnico diseño y plan de acción clima labora</t>
+          <t>LIFE 2026. Medio ambiente. Ayudas de 4 subprogramas, de naturaleza y biodiversidad, circularidad y calidad de vida, cambio climático y transición energética. Con inscripción abierta para jornadas info</t>
         </is>
       </c>
       <c r="C978" s="22" t="n"/>
@@ -19175,7 +19231,7 @@
       </c>
       <c r="B979" s="21" t="inlineStr">
         <is>
-          <t>EUS-81737</t>
+          <t>EUS-59353</t>
         </is>
       </c>
       <c r="C979" s="22" t="n"/>
@@ -19251,7 +19307,7 @@
       </c>
       <c r="B984" s="21" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C984" s="22" t="n"/>
@@ -19327,7 +19383,7 @@
       </c>
       <c r="B989" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/ases-tecnico-diseno-y-plan-accion-clima-labora/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260421life4lerrotajarduna/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C989" s="22" t="n"/>
@@ -19338,7 +19394,7 @@
     <row r="991" ht="30" customHeight="1">
       <c r="A991" s="18" t="inlineStr">
         <is>
-          <t>FICHA 67: EUS-00039</t>
+          <t>FICHA 67: EUS-00407</t>
         </is>
       </c>
       <c r="B991" s="19" t="n"/>
@@ -19371,7 +19427,7 @@
       </c>
       <c r="B993" s="21" t="inlineStr">
         <is>
-          <t>Plan de movilidad</t>
+          <t>Ases. técnico diseño y plan de acción clima labora</t>
         </is>
       </c>
       <c r="C993" s="22" t="n"/>
@@ -19387,7 +19443,7 @@
       </c>
       <c r="B994" s="21" t="inlineStr">
         <is>
-          <t>EUS-00039</t>
+          <t>EUS-00407</t>
         </is>
       </c>
       <c r="C994" s="22" t="n"/>
@@ -19539,7 +19595,7 @@
       </c>
       <c r="B1004" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/plan-movilidad/expcm508889/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/ases-tecnico-diseno-y-plan-accion-clima-labora/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1004" s="22" t="n"/>
@@ -19550,7 +19606,7 @@
     <row r="1006" ht="30" customHeight="1">
       <c r="A1006" s="18" t="inlineStr">
         <is>
-          <t>FICHA 68: EUS-28691</t>
+          <t>FICHA 68: EUS-78654</t>
         </is>
       </c>
       <c r="B1006" s="19" t="n"/>
@@ -19575,7 +19631,7 @@
       <c r="E1007" s="22" t="n"/>
       <c r="F1007" s="22" t="n"/>
     </row>
-    <row r="1008" ht="45" customHeight="1">
+    <row r="1008" ht="20" customHeight="1">
       <c r="A1008" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -19583,7 +19639,7 @@
       </c>
       <c r="B1008" s="21" t="inlineStr">
         <is>
-          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta el 01.10.26. Cribado de enfermedades con inteligencia artificial. Espacio de Datos Sanitarios de la UE. Red de Centros para Seguridad de la I</t>
+          <t>Plan de movilidad</t>
         </is>
       </c>
       <c r="C1008" s="22" t="n"/>
@@ -19599,7 +19655,7 @@
       </c>
       <c r="B1009" s="21" t="inlineStr">
         <is>
-          <t>EUS-28691</t>
+          <t>EUS-78654</t>
         </is>
       </c>
       <c r="C1009" s="22" t="n"/>
@@ -19675,7 +19731,7 @@
       </c>
       <c r="B1014" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C1014" s="22" t="n"/>
@@ -19733,9 +19789,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B1018" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
+      <c r="B1018" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALTA — </t>
         </is>
       </c>
       <c r="C1018" s="22" t="n"/>
@@ -19751,7 +19807,7 @@
       </c>
       <c r="B1019" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260422digitaleuropekoak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/plan-movilidad/expcm508889/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1019" s="22" t="n"/>
@@ -19762,7 +19818,7 @@
     <row r="1021" ht="30" customHeight="1">
       <c r="A1021" s="18" t="inlineStr">
         <is>
-          <t>FICHA 69: EUS-90174</t>
+          <t>FICHA 69: EUS-15400</t>
         </is>
       </c>
       <c r="B1021" s="19" t="n"/>
@@ -19795,7 +19851,7 @@
       </c>
       <c r="B1023" s="21" t="inlineStr">
         <is>
-          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversidad, participación, principios de la UE. Eventos, difusiones e intercambios. Programa de Ciudadanos, Igualdad, Derechos y Valores de la UE (</t>
+          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta el 01.10.26. Cribado de enfermedades con inteligencia artificial. Espacio de Datos Sanitarios de la UE. Red de Centros para Seguridad de la I</t>
         </is>
       </c>
       <c r="C1023" s="22" t="n"/>
@@ -19811,7 +19867,7 @@
       </c>
       <c r="B1024" s="21" t="inlineStr">
         <is>
-          <t>EUS-90174</t>
+          <t>EUS-15400</t>
         </is>
       </c>
       <c r="C1024" s="22" t="n"/>
@@ -19963,7 +20019,7 @@
       </c>
       <c r="B1034" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260408cervhirisareak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260422digitaleuropekoak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1034" s="22" t="n"/>
@@ -19974,7 +20030,7 @@
     <row r="1036" ht="30" customHeight="1">
       <c r="A1036" s="18" t="inlineStr">
         <is>
-          <t>FICHA 70: EUS-64378</t>
+          <t>FICHA 70: EUS-82152</t>
         </is>
       </c>
       <c r="B1036" s="19" t="n"/>
@@ -20007,7 +20063,7 @@
       </c>
       <c r="B1038" s="21" t="inlineStr">
         <is>
-          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el marco de la Intervención Sectorial Vitivinícola del Plan Estratégico (PEPAC) de la Política Agrícola Común de la UE 2023-2027</t>
+          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversidad, participación, principios de la UE. Eventos, difusiones e intercambios. Programa de Ciudadanos, Igualdad, Derechos y Valores de la UE (</t>
         </is>
       </c>
       <c r="C1038" s="22" t="n"/>
@@ -20023,7 +20079,7 @@
       </c>
       <c r="B1039" s="21" t="inlineStr">
         <is>
-          <t>EUS-64378</t>
+          <t>EUS-82152</t>
         </is>
       </c>
       <c r="C1039" s="22" t="n"/>
@@ -20175,7 +20231,7 @@
       </c>
       <c r="B1049" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/20260407mahastiardogintza/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260408cervhirisareak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1049" s="22" t="n"/>
@@ -20186,7 +20242,7 @@
     <row r="1051" ht="30" customHeight="1">
       <c r="A1051" s="18" t="inlineStr">
         <is>
-          <t>FICHA 71: EUS-72310</t>
+          <t>FICHA 71: EUS-50992</t>
         </is>
       </c>
       <c r="B1051" s="19" t="n"/>
@@ -20211,7 +20267,7 @@
       <c r="E1052" s="22" t="n"/>
       <c r="F1052" s="22" t="n"/>
     </row>
-    <row r="1053" ht="20" customHeight="1">
+    <row r="1053" ht="45" customHeight="1">
       <c r="A1053" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -20219,7 +20275,7 @@
       </c>
       <c r="B1053" s="21" t="inlineStr">
         <is>
-          <t>Recogida de muestras de legionella mediante pcr en el acs de orbea</t>
+          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el marco de la Intervención Sectorial Vitivinícola del Plan Estratégico (PEPAC) de la Política Agrícola Común de la UE 2023-2027</t>
         </is>
       </c>
       <c r="C1053" s="22" t="n"/>
@@ -20235,7 +20291,7 @@
       </c>
       <c r="B1054" s="21" t="inlineStr">
         <is>
-          <t>EUS-72310</t>
+          <t>EUS-50992</t>
         </is>
       </c>
       <c r="C1054" s="22" t="n"/>
@@ -20311,7 +20367,7 @@
       </c>
       <c r="B1059" s="21" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C1059" s="22" t="n"/>
@@ -20387,7 +20443,7 @@
       </c>
       <c r="B1064" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/recogida-muestras-legionella-mediante-pcr-acs-orbea/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/20260407mahastiardogintza/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1064" s="22" t="n"/>
@@ -20398,7 +20454,7 @@
     <row r="1066" ht="30" customHeight="1">
       <c r="A1066" s="18" t="inlineStr">
         <is>
-          <t>FICHA 72: EUS-62265</t>
+          <t>FICHA 72: EUS-73686</t>
         </is>
       </c>
       <c r="B1066" s="19" t="n"/>
@@ -20431,7 +20487,7 @@
       </c>
       <c r="B1068" s="21" t="inlineStr">
         <is>
-          <t>Coffee break Vititransfer Laguardia</t>
+          <t>Recogida de muestras de legionella mediante pcr en el acs de orbea</t>
         </is>
       </c>
       <c r="C1068" s="22" t="n"/>
@@ -20447,7 +20503,7 @@
       </c>
       <c r="B1069" s="21" t="inlineStr">
         <is>
-          <t>EUS-62265</t>
+          <t>EUS-73686</t>
         </is>
       </c>
       <c r="C1069" s="22" t="n"/>
@@ -20599,7 +20655,7 @@
       </c>
       <c r="B1079" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/coffee-break-vititransfer-laguardia/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/recogida-muestras-legionella-mediante-pcr-acs-orbea/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1079" s="22" t="n"/>
@@ -20607,8 +20663,220 @@
       <c r="E1079" s="22" t="n"/>
       <c r="F1079" s="22" t="n"/>
     </row>
+    <row r="1081" ht="30" customHeight="1">
+      <c r="A1081" s="18" t="inlineStr">
+        <is>
+          <t>FICHA 73: EUS-57575</t>
+        </is>
+      </c>
+      <c r="B1081" s="19" t="n"/>
+      <c r="C1081" s="19" t="n"/>
+      <c r="D1081" s="19" t="n"/>
+      <c r="E1081" s="19" t="n"/>
+      <c r="F1081" s="19" t="n"/>
+    </row>
+    <row r="1082" ht="20" customHeight="1">
+      <c r="A1082" s="20" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1082" s="21" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1082" s="22" t="n"/>
+      <c r="D1082" s="22" t="n"/>
+      <c r="E1082" s="22" t="n"/>
+      <c r="F1082" s="22" t="n"/>
+    </row>
+    <row r="1083" ht="20" customHeight="1">
+      <c r="A1083" s="20" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1083" s="21" t="inlineStr">
+        <is>
+          <t>Coffee break Vititransfer Laguardia</t>
+        </is>
+      </c>
+      <c r="C1083" s="22" t="n"/>
+      <c r="D1083" s="22" t="n"/>
+      <c r="E1083" s="22" t="n"/>
+      <c r="F1083" s="22" t="n"/>
+    </row>
+    <row r="1084" ht="20" customHeight="1">
+      <c r="A1084" s="20" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1084" s="21" t="inlineStr">
+        <is>
+          <t>EUS-57575</t>
+        </is>
+      </c>
+      <c r="C1084" s="22" t="n"/>
+      <c r="D1084" s="22" t="n"/>
+      <c r="E1084" s="22" t="n"/>
+      <c r="F1084" s="22" t="n"/>
+    </row>
+    <row r="1085" ht="20" customHeight="1">
+      <c r="A1085" s="20" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1085" s="21" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1085" s="22" t="n"/>
+      <c r="D1085" s="22" t="n"/>
+      <c r="E1085" s="22" t="n"/>
+      <c r="F1085" s="22" t="n"/>
+    </row>
+    <row r="1086" ht="20" customHeight="1">
+      <c r="A1086" s="20" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1086" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1086" s="22" t="n"/>
+      <c r="D1086" s="22" t="n"/>
+      <c r="E1086" s="22" t="n"/>
+      <c r="F1086" s="22" t="n"/>
+    </row>
+    <row r="1087" ht="20" customHeight="1">
+      <c r="A1087" s="20" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1087" s="21" t="inlineStr"/>
+      <c r="C1087" s="22" t="n"/>
+      <c r="D1087" s="22" t="n"/>
+      <c r="E1087" s="22" t="n"/>
+      <c r="F1087" s="22" t="n"/>
+    </row>
+    <row r="1088" ht="20" customHeight="1">
+      <c r="A1088" s="20" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1088" s="21" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1088" s="22" t="n"/>
+      <c r="D1088" s="22" t="n"/>
+      <c r="E1088" s="22" t="n"/>
+      <c r="F1088" s="22" t="n"/>
+    </row>
+    <row r="1089" ht="20" customHeight="1">
+      <c r="A1089" s="20" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1089" s="21" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1089" s="22" t="n"/>
+      <c r="D1089" s="22" t="n"/>
+      <c r="E1089" s="22" t="n"/>
+      <c r="F1089" s="22" t="n"/>
+    </row>
+    <row r="1090" ht="20" customHeight="1">
+      <c r="A1090" s="20" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1090" s="21" t="inlineStr"/>
+      <c r="C1090" s="22" t="n"/>
+      <c r="D1090" s="22" t="n"/>
+      <c r="E1090" s="22" t="n"/>
+      <c r="F1090" s="22" t="n"/>
+    </row>
+    <row r="1091" ht="20" customHeight="1">
+      <c r="A1091" s="20" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1091" s="21" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1091" s="22" t="n"/>
+      <c r="D1091" s="22" t="n"/>
+      <c r="E1091" s="22" t="n"/>
+      <c r="F1091" s="22" t="n"/>
+    </row>
+    <row r="1092" ht="20" customHeight="1">
+      <c r="A1092" s="20" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1092" s="21" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1092" s="22" t="n"/>
+      <c r="D1092" s="22" t="n"/>
+      <c r="E1092" s="22" t="n"/>
+      <c r="F1092" s="22" t="n"/>
+    </row>
+    <row r="1093" ht="20" customHeight="1">
+      <c r="A1093" s="20" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1093" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1093" s="22" t="n"/>
+      <c r="D1093" s="22" t="n"/>
+      <c r="E1093" s="22" t="n"/>
+      <c r="F1093" s="22" t="n"/>
+    </row>
+    <row r="1094" ht="45" customHeight="1">
+      <c r="A1094" s="20" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1094" s="23" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/coffee-break-vititransfer-laguardia/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1094" s="22" t="n"/>
+      <c r="D1094" s="22" t="n"/>
+      <c r="E1094" s="22" t="n"/>
+      <c r="F1094" s="22" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="1008">
+  <mergeCells count="1022">
     <mergeCell ref="B679:F679"/>
     <mergeCell ref="B666:F666"/>
     <mergeCell ref="B964:F964"/>
@@ -20655,6 +20923,7 @@
     <mergeCell ref="B515:F515"/>
     <mergeCell ref="A841:F841"/>
     <mergeCell ref="B158:F158"/>
+    <mergeCell ref="B1094:F1094"/>
     <mergeCell ref="B723:F723"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="B894:F894"/>
@@ -20678,6 +20947,7 @@
     <mergeCell ref="B433:F433"/>
     <mergeCell ref="B233:F233"/>
     <mergeCell ref="B1067:F1067"/>
+    <mergeCell ref="B1085:F1085"/>
     <mergeCell ref="B227:F227"/>
     <mergeCell ref="B531:F531"/>
     <mergeCell ref="B591:F591"/>
@@ -20832,6 +21102,7 @@
     <mergeCell ref="B689:F689"/>
     <mergeCell ref="B86:F86"/>
     <mergeCell ref="B912:F912"/>
+    <mergeCell ref="B1083:F1083"/>
     <mergeCell ref="B262:F262"/>
     <mergeCell ref="B887:F887"/>
     <mergeCell ref="B862:F862"/>
@@ -20880,6 +21151,7 @@
     <mergeCell ref="B979:F979"/>
     <mergeCell ref="B381:F381"/>
     <mergeCell ref="B552:F552"/>
+    <mergeCell ref="B1084:F1084"/>
     <mergeCell ref="A976:F976"/>
     <mergeCell ref="B170:F170"/>
     <mergeCell ref="B157:F157"/>
@@ -20924,6 +21196,7 @@
     <mergeCell ref="B265:F265"/>
     <mergeCell ref="B458:F458"/>
     <mergeCell ref="B773:F773"/>
+    <mergeCell ref="B1091:F1091"/>
     <mergeCell ref="A526:F526"/>
     <mergeCell ref="B694:F694"/>
     <mergeCell ref="B786:F786"/>
@@ -20996,9 +21269,11 @@
     <mergeCell ref="B273:F273"/>
     <mergeCell ref="B857:F857"/>
     <mergeCell ref="B1063:F1063"/>
+    <mergeCell ref="B1090:F1090"/>
     <mergeCell ref="B807:F807"/>
     <mergeCell ref="B1000:F1000"/>
     <mergeCell ref="B39:F39"/>
+    <mergeCell ref="B1092:F1092"/>
     <mergeCell ref="B508:F508"/>
     <mergeCell ref="B573:F573"/>
     <mergeCell ref="A961:F961"/>
@@ -21067,6 +21342,7 @@
     <mergeCell ref="B337:F337"/>
     <mergeCell ref="B312:F312"/>
     <mergeCell ref="B579:F579"/>
+    <mergeCell ref="B1089:F1089"/>
     <mergeCell ref="B610:F610"/>
     <mergeCell ref="B877:F877"/>
     <mergeCell ref="B815:F815"/>
@@ -21103,6 +21379,7 @@
     <mergeCell ref="B292:F292"/>
     <mergeCell ref="B492:F492"/>
     <mergeCell ref="B734:F734"/>
+    <mergeCell ref="B1082:F1082"/>
     <mergeCell ref="B528:F528"/>
     <mergeCell ref="B71:F71"/>
     <mergeCell ref="B1019:F1019"/>
@@ -21294,6 +21571,7 @@
     <mergeCell ref="B309:F309"/>
     <mergeCell ref="A316:F316"/>
     <mergeCell ref="B380:F380"/>
+    <mergeCell ref="A1081:F1081"/>
     <mergeCell ref="B100:F100"/>
     <mergeCell ref="B336:F336"/>
     <mergeCell ref="B634:F634"/>
@@ -21373,6 +21651,7 @@
     <mergeCell ref="B851:F851"/>
     <mergeCell ref="B845:F845"/>
     <mergeCell ref="B261:F261"/>
+    <mergeCell ref="B1087:F1087"/>
     <mergeCell ref="B184:F184"/>
     <mergeCell ref="B1062:F1062"/>
     <mergeCell ref="A301:F301"/>
@@ -21441,6 +21720,7 @@
     <mergeCell ref="B96:F96"/>
     <mergeCell ref="B922:F922"/>
     <mergeCell ref="B167:F167"/>
+    <mergeCell ref="B1093:F1093"/>
     <mergeCell ref="B332:F332"/>
     <mergeCell ref="B503:F503"/>
     <mergeCell ref="B701:F701"/>
@@ -21451,6 +21731,7 @@
     <mergeCell ref="B617:F617"/>
     <mergeCell ref="B937:F937"/>
     <mergeCell ref="B1059:F1059"/>
+    <mergeCell ref="B1086:F1086"/>
     <mergeCell ref="B853:F853"/>
     <mergeCell ref="B98:F98"/>
     <mergeCell ref="B986:F986"/>
@@ -21466,6 +21747,7 @@
     <mergeCell ref="B162:F162"/>
     <mergeCell ref="B267:F267"/>
     <mergeCell ref="B798:F798"/>
+    <mergeCell ref="B1088:F1088"/>
     <mergeCell ref="B398:F398"/>
     <mergeCell ref="B569:F569"/>
     <mergeCell ref="A466:F466"/>
@@ -21691,6 +21973,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1049" r:id="rId70"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1064" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1079" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1094" r:id="rId73"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -21702,7 +21985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J73"/>
+  <dimension ref="A1:J74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -22572,12 +22855,12 @@
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-08</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Palaeoclimate science for a better understanding of Earth sy</t>
+          <t>Advancing understanding, modelling and prediction of extreme</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -22692,12 +22975,12 @@
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Assessing the performance of policy instruments to inform cl</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
@@ -22732,12 +23015,12 @@
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Palaeoclimate science for a better understanding of Earth sy</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
@@ -22772,12 +23055,12 @@
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform cl</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
@@ -22812,12 +23095,12 @@
     <row r="28" ht="28" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -24224,12 +24507,12 @@
     <row r="66" ht="28" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>EUS-49329</t>
+          <t>EUS-13454</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>LIFE 2026. Medio ambiente. Ayudas de 4 subprogramas, de natu</t>
+          <t>Suministro de energia eléctrica a distintos puntos de consum</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
@@ -24245,7 +24528,7 @@
       <c r="E66" s="6" t="inlineStr"/>
       <c r="F66" s="27" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>MUY ALTA</t>
         </is>
       </c>
       <c r="G66" s="6" t="inlineStr"/>
@@ -24260,12 +24543,12 @@
     <row r="67" ht="28" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>EUS-81737</t>
+          <t>EUS-59353</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>Ases. técnico diseño y plan de acción clima labora</t>
+          <t>LIFE 2026. Medio ambiente. Ayudas de 4 subprogramas, de natu</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
@@ -24296,12 +24579,12 @@
     <row r="68" ht="28" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>EUS-00039</t>
+          <t>EUS-00407</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>Plan de movilidad</t>
+          <t>Ases. técnico diseño y plan de acción clima labora</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -24332,12 +24615,12 @@
     <row r="69" ht="28" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>EUS-28691</t>
+          <t>EUS-78654</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta e</t>
+          <t>Plan de movilidad</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -24353,7 +24636,7 @@
       <c r="E69" s="6" t="inlineStr"/>
       <c r="F69" s="27" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="G69" s="6" t="inlineStr"/>
@@ -24368,12 +24651,12 @@
     <row r="70" ht="28" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>EUS-90174</t>
+          <t>EUS-15400</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversi</t>
+          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta e</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -24404,12 +24687,12 @@
     <row r="71" ht="28" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>EUS-64378</t>
+          <t>EUS-82152</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el ma</t>
+          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversi</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -24440,12 +24723,12 @@
     <row r="72" ht="28" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>EUS-72310</t>
+          <t>EUS-50992</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>Recogida de muestras de legionella mediante pcr en el acs de</t>
+          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el ma</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -24476,12 +24759,12 @@
     <row r="73" ht="28" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>EUS-62265</t>
+          <t>EUS-73686</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>Coffee break Vititransfer Laguardia</t>
+          <t>Recogida de muestras de legionella mediante pcr en el acs de</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -24509,8 +24792,44 @@
       <c r="I73" s="6" t="inlineStr"/>
       <c r="J73" s="6" t="inlineStr"/>
     </row>
+    <row r="74" ht="28" customHeight="1">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>EUS-57575</t>
+        </is>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>Coffee break Vititransfer Laguardia</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D74" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E74" s="6" t="inlineStr"/>
+      <c r="F74" s="27" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G74" s="6" t="inlineStr"/>
+      <c r="H74" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I74" s="6" t="inlineStr"/>
+      <c r="J74" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J73"/>
+  <autoFilter ref="A1:J74"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update funding data 2026-05-04
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Recursos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$80</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$77</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -679,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M80"/>
+  <dimension ref="A1:M83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -707,7 +707,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 03/05/2026 07:47 - 73 convocatorias - 9 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 04/05/2026 08:15 - 76 convocatorias - 12 nuevas</t>
         </is>
       </c>
     </row>
@@ -1222,12 +1222,12 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-04</t>
+          <t>HORIZON-CL5-2026-11-D3-23</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>De-risking renewable fuel technologies through transnational pre-commercial procurement of renewable fuel industrial value chains</t>
+          <t>Data sharing to support the training and development of AI foundation models in the energy sector</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>Pre-commercial Procurement</t>
+          <t>Innovation Actions</t>
         </is>
       </c>
       <c r="I13" s="10" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Public authorities, industry, technology providers, energy producers and consumers profit from de-</t>
+          <t>Expected Outcome:Projects are expected to contribute to all the following expected outcomes:Effective and innovative methods for gathering, sharing and using large data sets in energy applications for</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr"/>
@@ -1285,12 +1285,12 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-05</t>
+          <t>HORIZON-CL5-2026-11-D3-06</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Demonstration of solid biofuel supply and conversion to high efficiency CHP from fully sustainable regional value chains</t>
+          <t>Resource assessment for deep sedimentary and basement reservoirs</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -1315,7 +1315,7 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>Innovation Actions</t>
+          <t xml:space="preserve"> Research and Innovation Actions</t>
         </is>
       </c>
       <c r="I14" s="10" t="inlineStr">
@@ -1330,7 +1330,7 @@
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Fully sustainable regional bioenergy value chains and efficient conversion can play an important role in renewable efficient power and heating generation and for reaching the EU clima</t>
+          <t>Expected Outcome:Deep sedimentary/basement reservoirs are usually characterized by low permeability, high drilling cost and a scarcity of data, as they are typically ignored by hydrocarbon exploration</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr"/>
@@ -1348,12 +1348,12 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-23</t>
+          <t>HORIZON-CL5-2026-11-D3-14</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Data sharing to support the training and development of AI foundation models in the energy sector</t>
+          <t>Improved system design for innovative PV applications (EUPI-PV Partnership)</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Projects are expected to contribute to all the following expected outcomes:Effective and innovative methods for gathering, sharing and using large data sets in energy applications for</t>
+          <t>Expected Outcome:Agrivoltaics or the co-location of agricultural activity and PV electricity production is a novel form of PV deployment which could provide farmers with diversified revenue sources an</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr"/>
@@ -1411,12 +1411,12 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-06</t>
+          <t>HORIZON-CL5-2026-11-D3-05</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Resource assessment for deep sedimentary and basement reservoirs</t>
+          <t>Demonstration of solid biofuel supply and conversion to high efficiency CHP from fully sustainable regional value chains</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Research and Innovation Actions</t>
+          <t>Innovation Actions</t>
         </is>
       </c>
       <c r="I16" s="10" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Deep sedimentary/basement reservoirs are usually characterized by low permeability, high drilling cost and a scarcity of data, as they are typically ignored by hydrocarbon exploration</t>
+          <t>Expected Outcome:Fully sustainable regional bioenergy value chains and efficient conversion can play an important role in renewable efficient power and heating generation and for reaching the EU clima</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr"/>
@@ -1474,12 +1474,12 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-14</t>
+          <t>HORIZON-CL5-2026-11-D3-04</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Improved system design for innovative PV applications (EUPI-PV Partnership)</t>
+          <t>De-risking renewable fuel technologies through transnational pre-commercial procurement of renewable fuel industrial value chains</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -1504,7 +1504,7 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>Innovation Actions</t>
+          <t>Pre-commercial Procurement</t>
         </is>
       </c>
       <c r="I17" s="10" t="inlineStr">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Agrivoltaics or the co-location of agricultural activity and PV electricity production is a novel form of PV deployment which could provide farmers with diversified revenue sources an</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Public authorities, industry, technology providers, energy producers and consumers profit from de-</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr"/>
@@ -1537,12 +1537,12 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-16</t>
+          <t>HORIZON-CL5-2027-07-D3-27</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Industrial processes and equipment for innovative, reliable and scalable tandem technologies (EUPI-PV Partnership)</t>
+          <t>Integrated Approaches for Retrofitting Infrastructures with Innovative Energy Storage Technologies</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:The REPowerEU plan and the EU Solar Energy Strategy introduced targets for the deployment of solar PV amounting to 600 GWac by 2030. Complying with these targets will be crucial for t</t>
+          <t xml:space="preserve">Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Improved energy security of the energy system by offering cost-effective and efficient solutions for </t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr"/>
@@ -1600,12 +1600,12 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-11</t>
+          <t>HORIZON-CL5-2027-07-D3-26</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Demonstration of hydropower technologies for efficient and forward-looking refurbishment of existing hydropower plants</t>
+          <t>Advanced Distribution Management Systems (ADSM) for more efficient and flexible distribution grids</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -1645,7 +1645,7 @@
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:For a renewables-based electricity system sufficient flexible and also in the long-run fully sustainable hydropower capacity is pivotal.Project results are expected to contribute to a</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced reliability, resilience, controllability and efficiency of electricity distribution grids. C</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr"/>
@@ -1726,12 +1726,12 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-26</t>
+          <t>HORIZON-CL5-2027-07-D3-28</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Advanced Distribution Management Systems (ADSM) for more efficient and flexible distribution grids</t>
+          <t>Community of practice - Data-Driven Decision-Making in Energy</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -1756,7 +1756,7 @@
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>Innovation Actions</t>
+          <t>Coordination and Support Actions</t>
         </is>
       </c>
       <c r="I21" s="10" t="inlineStr">
@@ -1771,7 +1771,7 @@
       </c>
       <c r="K21" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced reliability, resilience, controllability and efficiency of electricity distribution grids. C</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced EU cooperation to generate knowledge sharing on data and analytics used for the planning and</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr"/>
@@ -1789,12 +1789,12 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-27</t>
+          <t>HORIZON-CL5-2027-07-D3-16</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Integrated Approaches for Retrofitting Infrastructures with Innovative Energy Storage Technologies</t>
+          <t>Industrial processes and equipment for innovative, reliable and scalable tandem technologies (EUPI-PV Partnership)</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Improved energy security of the energy system by offering cost-effective and efficient solutions for </t>
+          <t>Expected Outcome:The REPowerEU plan and the EU Solar Energy Strategy introduced targets for the deployment of solar PV amounting to 600 GWac by 2030. Complying with these targets will be crucial for t</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr"/>
@@ -1852,12 +1852,12 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-28</t>
+          <t>HORIZON-CL5-2027-07-D3-25</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Community of practice - Data-Driven Decision-Making in Energy</t>
+          <t>Advanced TSO control rooms to enhance grid observability, stability and resilience</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -1882,7 +1882,7 @@
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>Coordination and Support Actions</t>
+          <t>Innovation Actions</t>
         </is>
       </c>
       <c r="I23" s="10" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="K23" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced EU cooperation to generate knowledge sharing on data and analytics used for the planning and</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced reliability, resilience, and efficiency of electricity transmission grids. Grid congestion i</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr"/>
@@ -1915,12 +1915,12 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-25</t>
+          <t>HORIZON-CL5-2027-07-D3-17</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Advanced TSO control rooms to enhance grid observability, stability and resilience</t>
+          <t>PV based electrification of the economy: Designing &amp; optimising PV systems supporting industrial electrification and promoting participation in electricity markets (EUPI-PV Partnership)</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -1960,7 +1960,7 @@
       </c>
       <c r="K24" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced reliability, resilience, and efficiency of electricity transmission grids. Grid congestion i</t>
+          <t>Expected Outcome:Large PV systems such as utility scale PV are evolving towards higher voltage architecture (&amp;gt;=3kV) with the objective to minimize losses and improve system efficiency at lower cost</t>
         </is>
       </c>
       <c r="L24" s="6" t="inlineStr"/>
@@ -1978,12 +1978,12 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-17</t>
+          <t>HORIZON-CL5-2027-07-D3-11</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>PV based electrification of the economy: Designing &amp; optimising PV systems supporting industrial electrification and promoting participation in electricity markets (EUPI-PV Partnership)</t>
+          <t>Demonstration of hydropower technologies for efficient and forward-looking refurbishment of existing hydropower plants</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -2023,7 +2023,7 @@
       </c>
       <c r="K25" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Large PV systems such as utility scale PV are evolving towards higher voltage architecture (&amp;gt;=3kV) with the objective to minimize losses and improve system efficiency at lower cost</t>
+          <t>Expected Outcome:For a renewables-based electricity system sufficient flexible and also in the long-run fully sustainable hydropower capacity is pivotal.Project results are expected to contribute to a</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr"/>
@@ -2041,12 +2041,12 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
+          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -2086,7 +2086,7 @@
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Euro</t>
+          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and inter</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr"/>
@@ -2230,12 +2230,12 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Research and Innovation Actions</t>
+          <t>Programme Cofund Actions</t>
         </is>
       </c>
       <c r="I29" s="10" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="K29" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to info</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is estab</t>
         </is>
       </c>
       <c r="L29" s="6" t="inlineStr"/>
@@ -2293,12 +2293,12 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-08</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -2338,7 +2338,7 @@
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and inter</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorpo</t>
         </is>
       </c>
       <c r="L30" s="6" t="inlineStr"/>
@@ -2356,12 +2356,12 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>Programme Cofund Actions</t>
+          <t xml:space="preserve"> Research and Innovation Actions</t>
         </is>
       </c>
       <c r="I31" s="10" t="inlineStr">
@@ -2401,7 +2401,7 @@
       </c>
       <c r="K31" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is estab</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to info</t>
         </is>
       </c>
       <c r="L31" s="6" t="inlineStr"/>
@@ -2419,12 +2419,12 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorpo</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Euro</t>
         </is>
       </c>
       <c r="L32" s="6" t="inlineStr"/>
@@ -3364,12 +3364,12 @@
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-08</t>
+          <t>HORIZON-CL5-2027-02-D3-31</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Co-funding Strategic Energy Technology (SET) Plan renewable fuel value chains at EU, national, regional, and local level</t>
+          <t>Support to the implementation of an EU policy framework for CO2 transport and storage infrastructure</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="H47" s="6" t="inlineStr">
         <is>
-          <t>Programme Cofund Actions</t>
+          <t>Coordination and Support Actions</t>
         </is>
       </c>
       <c r="I47" s="10" t="inlineStr">
@@ -3409,7 +3409,7 @@
       </c>
       <c r="K47" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Advance in the realisation of the Strategic Energy Technology (SET) Plan Action of Renewable fuels</t>
+          <t>Expected Outcome:Project results are expected to contribute to the following outcome:Stakeholders involved in the CO2 infrastructure network are in a position to implement the upcoming legislative fra</t>
         </is>
       </c>
       <c r="L47" s="6" t="inlineStr"/>
@@ -3427,12 +3427,12 @@
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-09</t>
+          <t>HORIZON-CL5-2027-02-D3-24</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Innovative technologies and solutions to improve wave and tidal energy systems</t>
+          <t>Large scale operational validation and upscaling of state-of-the-art (Generative) AI tools and models powering a next generation digital energy system</t>
         </is>
       </c>
       <c r="D48" s="6" t="inlineStr">
@@ -3472,7 +3472,7 @@
       </c>
       <c r="K48" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all following expected outcomes:Advance in the realisation of the Strategic Energy Technology (SET) Plan’s research and innovation priori</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Advanced, secure frugal (energy-, resource-, data- and cost-efficient, sustainable) AI tools for real</t>
         </is>
       </c>
       <c r="L48" s="6" t="inlineStr"/>
@@ -3553,12 +3553,12 @@
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-24</t>
+          <t>HORIZON-CL5-2027-02-D3-15</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>Large scale operational validation and upscaling of state-of-the-art (Generative) AI tools and models powering a next generation digital energy system</t>
+          <t>Production technologies for solar photovoltaics beyond the state-of-the-art (EUPI-PV Partnership)</t>
         </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </c>
       <c r="K50" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Advanced, secure frugal (energy-, resource-, data- and cost-efficient, sustainable) AI tools for real</t>
+          <t>Expected Outcome:The REPowerEU plan and the EU Solar Energy Strategy introduced targets for the deployment of solar PV amounting to 600 GWac by 2030. Complying with these targets will be crucial for t</t>
         </is>
       </c>
       <c r="L50" s="6" t="inlineStr"/>
@@ -3616,12 +3616,12 @@
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-31</t>
+          <t>HORIZON-CL5-2027-02-D3-07</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>Support to the implementation of an EU policy framework for CO2 transport and storage infrastructure</t>
+          <t>Concentrated solar thermal systems for decarbonising industrial processes</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
@@ -3646,7 +3646,7 @@
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>Coordination and Support Actions</t>
+          <t>Innovation Actions</t>
         </is>
       </c>
       <c r="I51" s="10" t="inlineStr">
@@ -3661,7 +3661,7 @@
       </c>
       <c r="K51" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to the following outcome:Stakeholders involved in the CO2 infrastructure network are in a position to implement the upcoming legislative fra</t>
+          <t>Expected Outcome:Renewable heating can be directly used to efficiently decarbonise industrial processes. Concentrated solar thermal technologies offer a great potential to supply renewable heat for in</t>
         </is>
       </c>
       <c r="L51" s="6" t="inlineStr"/>
@@ -3679,12 +3679,12 @@
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-15</t>
+          <t>HORIZON-CL5-2027-02-D3-08</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>Production technologies for solar photovoltaics beyond the state-of-the-art (EUPI-PV Partnership)</t>
+          <t>Co-funding Strategic Energy Technology (SET) Plan renewable fuel value chains at EU, national, regional, and local level</t>
         </is>
       </c>
       <c r="D52" s="6" t="inlineStr">
@@ -3709,7 +3709,7 @@
       </c>
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>Innovation Actions</t>
+          <t>Programme Cofund Actions</t>
         </is>
       </c>
       <c r="I52" s="10" t="inlineStr">
@@ -3724,7 +3724,7 @@
       </c>
       <c r="K52" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:The REPowerEU plan and the EU Solar Energy Strategy introduced targets for the deployment of solar PV amounting to 600 GWac by 2030. Complying with these targets will be crucial for t</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Advance in the realisation of the Strategic Energy Technology (SET) Plan Action of Renewable fuels</t>
         </is>
       </c>
       <c r="L52" s="6" t="inlineStr"/>
@@ -4595,7 +4595,7 @@
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>EUS-13454</t>
+          <t>EUS-41373</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -4650,7 +4650,7 @@
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>EUS-59353</t>
+          <t>EUS-68354</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -4705,12 +4705,12 @@
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>EUS-00407</t>
+          <t>EUS-84214</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>Ases. técnico diseño y plan de acción clima labora</t>
+          <t>Mantenimiento preventivo y correctivo de los equipos de climatización de los despachos y otras estancias de los cinco edificios y el suministro de nuevos equipos</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr">
@@ -4760,12 +4760,12 @@
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>EUS-78654</t>
+          <t>EUS-43982</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>Plan de movilidad</t>
+          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta el 01.10.26. Cribado de enfermedades con inteligencia artificial. Espacio de Datos Sanitarios de la UE. Red de Centros para Seguridad de la I</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
@@ -4782,12 +4782,12 @@
       <c r="G75" s="6" t="inlineStr"/>
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I75" s="11" t="inlineStr">
-        <is>
-          <t>ALTA</t>
+          <t>Ayuda/Subvencion Euskadi</t>
+        </is>
+      </c>
+      <c r="I75" s="8" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
         </is>
       </c>
       <c r="J75" s="6" t="inlineStr"/>
@@ -4815,12 +4815,12 @@
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>EUS-15400</t>
+          <t>EUS-33357</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta el 01.10.26. Cribado de enfermedades con inteligencia artificial. Espacio de Datos Sanitarios de la UE. Red de Centros para Seguridad de la I</t>
+          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversidad, participación, principios de la UE. Eventos, difusiones e intercambios. Programa de Ciudadanos, Igualdad, Derechos y Valores de la UE (</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr">
@@ -4870,12 +4870,12 @@
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>EUS-82152</t>
+          <t>EUS-05202</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversidad, participación, principios de la UE. Eventos, difusiones e intercambios. Programa de Ciudadanos, Igualdad, Derechos y Valores de la UE (</t>
+          <t>Servicio de control antidopaje (recogida de muestras) a través del personal habilitado para la Agencia Vasca Antidopaje, período 2026-2027.</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
@@ -4892,7 +4892,7 @@
       <c r="G77" s="6" t="inlineStr"/>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="I77" s="8" t="inlineStr">
@@ -4925,12 +4925,12 @@
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>EUS-50992</t>
+          <t>EUS-40531</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el marco de la Intervención Sectorial Vitivinícola del Plan Estratégico (PEPAC) de la Política Agrícola Común de la UE 2023-2027</t>
+          <t>Reparación humedades en cubierta en el centro IES Angela Figuera BHI</t>
         </is>
       </c>
       <c r="D78" s="6" t="inlineStr">
@@ -4947,7 +4947,7 @@
       <c r="G78" s="6" t="inlineStr"/>
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="I78" s="8" t="inlineStr">
@@ -4980,12 +4980,12 @@
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>EUS-73686</t>
+          <t>EUS-11190</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>Recogida de muestras de legionella mediante pcr en el acs de orbea</t>
+          <t>Reparación murete de cubierta fachada principal en el centro IES Antonio Trueba BHI (edificio Minería UE)</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
@@ -5035,12 +5035,12 @@
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>EUS-57575</t>
+          <t>EUS-51778</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>Coffee break Vititransfer Laguardia</t>
+          <t>Gestión del programa Hiriko Udalekuak / Colonias Urbanas de Verano y Gabonetako Koloniak / Colonias de Navidad en 2026.</t>
         </is>
       </c>
       <c r="D80" s="6" t="inlineStr">
@@ -5082,8 +5082,173 @@
         </is>
       </c>
     </row>
+    <row r="81" ht="40" customHeight="1">
+      <c r="A81" s="16" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>EUS-15302</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>Contratacion Conjunta de servicio de seguridad y servicios auxiliares en diversos edificios del Gobierno Vasco</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F81" s="6" t="inlineStr"/>
+      <c r="G81" s="6" t="inlineStr"/>
+      <c r="H81" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I81" s="8" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J81" s="6" t="inlineStr"/>
+      <c r="K81" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L81" s="17" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M81" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="40" customHeight="1">
+      <c r="A82" s="16" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>EUS-69233</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>Suministro y obra para instalación de la infraestructura de cuatro puntos de recarga de vehículos eléctricos</t>
+        </is>
+      </c>
+      <c r="D82" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F82" s="6" t="inlineStr"/>
+      <c r="G82" s="6" t="inlineStr"/>
+      <c r="H82" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I82" s="8" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J82" s="6" t="inlineStr"/>
+      <c r="K82" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L82" s="17" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M82" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="40" customHeight="1">
+      <c r="A83" s="16" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>EUS-38333</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="inlineStr">
+        <is>
+          <t>Recogida de muestras de legionella mediante pcr en el acs de orbea</t>
+        </is>
+      </c>
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E83" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F83" s="6" t="inlineStr"/>
+      <c r="G83" s="6" t="inlineStr"/>
+      <c r="H83" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I83" s="8" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J83" s="6" t="inlineStr"/>
+      <c r="K83" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L83" s="17" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M83" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:M80"/>
+  <autoFilter ref="A4:M83"/>
   <mergeCells count="5">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A5:M5"/>
@@ -5165,6 +5330,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M78" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M79" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M80" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M81" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M82" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M83" r:id="rId76"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5176,7 +5344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1094"/>
+  <dimension ref="A1:F1139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6714,7 +6882,7 @@
     <row r="106" ht="30" customHeight="1">
       <c r="A106" s="18" t="inlineStr">
         <is>
-          <t>FICHA 8: HORIZON-CL5-2026-11-D3-04</t>
+          <t>FICHA 8: HORIZON-CL5-2026-11-D3-23</t>
         </is>
       </c>
       <c r="B106" s="19" t="n"/>
@@ -6747,7 +6915,7 @@
       </c>
       <c r="B108" s="21" t="inlineStr">
         <is>
-          <t>De-risking renewable fuel technologies through transnational pre-commercial procurement of renewable fuel industrial value chains</t>
+          <t>Data sharing to support the training and development of AI foundation models in the energy sector</t>
         </is>
       </c>
       <c r="C108" s="22" t="n"/>
@@ -6763,7 +6931,7 @@
       </c>
       <c r="B109" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-04</t>
+          <t>HORIZON-CL5-2026-11-D3-23</t>
         </is>
       </c>
       <c r="C109" s="22" t="n"/>
@@ -6843,7 +7011,7 @@
       </c>
       <c r="B114" s="21" t="inlineStr">
         <is>
-          <t>Pre-commercial Procurement</t>
+          <t>Innovation Actions</t>
         </is>
       </c>
       <c r="C114" s="22" t="n"/>
@@ -6875,7 +7043,7 @@
       </c>
       <c r="B116" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Public authorities, industry, technology providers, energy producers and consumers profit from de-risking of cost-effective essential value chains of those renewable fuel technologies that can contribute to domestic commercial fuel production beyond 2030 customized to their needs, from improved access to better financing exploiting synergies across funding schemes, and from more effective market uptake, business models, increased competitiveness, and commercialization opportunities.Energy prod</t>
+          <t>Expected Outcome:Projects are expected to contribute to all the following expected outcomes:Effective and innovative methods for gathering, sharing and using large data sets in energy applications for the purpose of training AI models while ensuring privacy and security.Advanced and - wherever possible - open-source AI foundation models to support the digitalisation of the energy system, through improved grid observability, forecasting of supply and demand, advanced storage and renewables integration, demand side flexibility and energy efficiency.Enhanced cooperation, knowledge sharing and int</t>
         </is>
       </c>
       <c r="C116" s="22" t="n"/>
@@ -6919,7 +7087,7 @@
       </c>
       <c r="B119" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-04</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-23</t>
         </is>
       </c>
       <c r="C119" s="22" t="n"/>
@@ -6930,7 +7098,7 @@
     <row r="121" ht="30" customHeight="1">
       <c r="A121" s="18" t="inlineStr">
         <is>
-          <t>FICHA 9: HORIZON-CL5-2026-11-D3-05</t>
+          <t>FICHA 9: HORIZON-CL5-2026-11-D3-06</t>
         </is>
       </c>
       <c r="B121" s="19" t="n"/>
@@ -6955,7 +7123,7 @@
       <c r="E122" s="22" t="n"/>
       <c r="F122" s="22" t="n"/>
     </row>
-    <row r="123" ht="45" customHeight="1">
+    <row r="123" ht="20" customHeight="1">
       <c r="A123" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -6963,7 +7131,7 @@
       </c>
       <c r="B123" s="21" t="inlineStr">
         <is>
-          <t>Demonstration of solid biofuel supply and conversion to high efficiency CHP from fully sustainable regional value chains</t>
+          <t>Resource assessment for deep sedimentary and basement reservoirs</t>
         </is>
       </c>
       <c r="C123" s="22" t="n"/>
@@ -6979,7 +7147,7 @@
       </c>
       <c r="B124" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-05</t>
+          <t>HORIZON-CL5-2026-11-D3-06</t>
         </is>
       </c>
       <c r="C124" s="22" t="n"/>
@@ -7059,7 +7227,7 @@
       </c>
       <c r="B129" s="21" t="inlineStr">
         <is>
-          <t>Innovation Actions</t>
+          <t xml:space="preserve"> Research and Innovation Actions</t>
         </is>
       </c>
       <c r="C129" s="22" t="n"/>
@@ -7091,7 +7259,7 @@
       </c>
       <c r="B131" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Fully sustainable regional bioenergy value chains and efficient conversion can play an important role in renewable efficient power and heating generation and for reaching the EU climate and energy targets and contribute to European competitiveness and energy security.Project results are expected to contribute to at all of the following expected outcomes:The demonstration of regional value chains for the use of locally to regionally sourced sustainable and cheap solid biofuel from upgraded biogenic residues and wastes in line with the provisions of the Renewable Energy Directiv</t>
+          <t>Expected Outcome:Deep sedimentary/basement reservoirs are usually characterized by low permeability, high drilling cost and a scarcity of data, as they are typically ignored by hydrocarbon exploration. Major exploration challenges relate to predicting deep sedimentary and basement reservoir structures and properties to identify suitable locations for reservoir-independent approaches, capable of overcoming the low permeability obstacle, such as Enhanced Geothermal Systems (EGS) or closed-loop geothermal systems.Project results are expected to contribute to all of the following expected outcomes</t>
         </is>
       </c>
       <c r="C131" s="22" t="n"/>
@@ -7135,7 +7303,7 @@
       </c>
       <c r="B134" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-05</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-06</t>
         </is>
       </c>
       <c r="C134" s="22" t="n"/>
@@ -7146,7 +7314,7 @@
     <row r="136" ht="30" customHeight="1">
       <c r="A136" s="18" t="inlineStr">
         <is>
-          <t>FICHA 10: HORIZON-CL5-2026-11-D3-23</t>
+          <t>FICHA 10: HORIZON-CL5-2026-11-D3-14</t>
         </is>
       </c>
       <c r="B136" s="19" t="n"/>
@@ -7171,7 +7339,7 @@
       <c r="E137" s="22" t="n"/>
       <c r="F137" s="22" t="n"/>
     </row>
-    <row r="138" ht="45" customHeight="1">
+    <row r="138" ht="20" customHeight="1">
       <c r="A138" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -7179,7 +7347,7 @@
       </c>
       <c r="B138" s="21" t="inlineStr">
         <is>
-          <t>Data sharing to support the training and development of AI foundation models in the energy sector</t>
+          <t>Improved system design for innovative PV applications (EUPI-PV Partnership)</t>
         </is>
       </c>
       <c r="C138" s="22" t="n"/>
@@ -7195,7 +7363,7 @@
       </c>
       <c r="B139" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-23</t>
+          <t>HORIZON-CL5-2026-11-D3-14</t>
         </is>
       </c>
       <c r="C139" s="22" t="n"/>
@@ -7307,7 +7475,7 @@
       </c>
       <c r="B146" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Projects are expected to contribute to all the following expected outcomes:Effective and innovative methods for gathering, sharing and using large data sets in energy applications for the purpose of training AI models while ensuring privacy and security.Advanced and - wherever possible - open-source AI foundation models to support the digitalisation of the energy system, through improved grid observability, forecasting of supply and demand, advanced storage and renewables integration, demand side flexibility and energy efficiency.Enhanced cooperation, knowledge sharing and int</t>
+          <t>Expected Outcome:Agrivoltaics or the co-location of agricultural activity and PV electricity production is a novel form of PV deployment which could provide farmers with diversified revenue sources and ecological benefits, while reducing land use competition, siting restrictions or adverse impacts on biodiversity and agricultural production. Optimizing system designs and business practices will help to enable simultaneous land use creating synergy for both agriculture and electricity production; this can benefit farmers, lower PV costs and enable the European Union to reach the goals of the EU</t>
         </is>
       </c>
       <c r="C146" s="22" t="n"/>
@@ -7351,7 +7519,7 @@
       </c>
       <c r="B149" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-23</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-14</t>
         </is>
       </c>
       <c r="C149" s="22" t="n"/>
@@ -7362,7 +7530,7 @@
     <row r="151" ht="30" customHeight="1">
       <c r="A151" s="18" t="inlineStr">
         <is>
-          <t>FICHA 11: HORIZON-CL5-2026-11-D3-06</t>
+          <t>FICHA 11: HORIZON-CL5-2026-11-D3-05</t>
         </is>
       </c>
       <c r="B151" s="19" t="n"/>
@@ -7387,7 +7555,7 @@
       <c r="E152" s="22" t="n"/>
       <c r="F152" s="22" t="n"/>
     </row>
-    <row r="153" ht="20" customHeight="1">
+    <row r="153" ht="45" customHeight="1">
       <c r="A153" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -7395,7 +7563,7 @@
       </c>
       <c r="B153" s="21" t="inlineStr">
         <is>
-          <t>Resource assessment for deep sedimentary and basement reservoirs</t>
+          <t>Demonstration of solid biofuel supply and conversion to high efficiency CHP from fully sustainable regional value chains</t>
         </is>
       </c>
       <c r="C153" s="22" t="n"/>
@@ -7411,7 +7579,7 @@
       </c>
       <c r="B154" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-06</t>
+          <t>HORIZON-CL5-2026-11-D3-05</t>
         </is>
       </c>
       <c r="C154" s="22" t="n"/>
@@ -7491,7 +7659,7 @@
       </c>
       <c r="B159" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Research and Innovation Actions</t>
+          <t>Innovation Actions</t>
         </is>
       </c>
       <c r="C159" s="22" t="n"/>
@@ -7523,7 +7691,7 @@
       </c>
       <c r="B161" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Deep sedimentary/basement reservoirs are usually characterized by low permeability, high drilling cost and a scarcity of data, as they are typically ignored by hydrocarbon exploration. Major exploration challenges relate to predicting deep sedimentary and basement reservoir structures and properties to identify suitable locations for reservoir-independent approaches, capable of overcoming the low permeability obstacle, such as Enhanced Geothermal Systems (EGS) or closed-loop geothermal systems.Project results are expected to contribute to all of the following expected outcomes</t>
+          <t>Expected Outcome:Fully sustainable regional bioenergy value chains and efficient conversion can play an important role in renewable efficient power and heating generation and for reaching the EU climate and energy targets and contribute to European competitiveness and energy security.Project results are expected to contribute to at all of the following expected outcomes:The demonstration of regional value chains for the use of locally to regionally sourced sustainable and cheap solid biofuel from upgraded biogenic residues and wastes in line with the provisions of the Renewable Energy Directiv</t>
         </is>
       </c>
       <c r="C161" s="22" t="n"/>
@@ -7567,7 +7735,7 @@
       </c>
       <c r="B164" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-06</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-05</t>
         </is>
       </c>
       <c r="C164" s="22" t="n"/>
@@ -7578,7 +7746,7 @@
     <row r="166" ht="30" customHeight="1">
       <c r="A166" s="18" t="inlineStr">
         <is>
-          <t>FICHA 12: HORIZON-CL5-2026-11-D3-14</t>
+          <t>FICHA 12: HORIZON-CL5-2026-11-D3-04</t>
         </is>
       </c>
       <c r="B166" s="19" t="n"/>
@@ -7603,7 +7771,7 @@
       <c r="E167" s="22" t="n"/>
       <c r="F167" s="22" t="n"/>
     </row>
-    <row r="168" ht="20" customHeight="1">
+    <row r="168" ht="45" customHeight="1">
       <c r="A168" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -7611,7 +7779,7 @@
       </c>
       <c r="B168" s="21" t="inlineStr">
         <is>
-          <t>Improved system design for innovative PV applications (EUPI-PV Partnership)</t>
+          <t>De-risking renewable fuel technologies through transnational pre-commercial procurement of renewable fuel industrial value chains</t>
         </is>
       </c>
       <c r="C168" s="22" t="n"/>
@@ -7627,7 +7795,7 @@
       </c>
       <c r="B169" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-14</t>
+          <t>HORIZON-CL5-2026-11-D3-04</t>
         </is>
       </c>
       <c r="C169" s="22" t="n"/>
@@ -7707,7 +7875,7 @@
       </c>
       <c r="B174" s="21" t="inlineStr">
         <is>
-          <t>Innovation Actions</t>
+          <t>Pre-commercial Procurement</t>
         </is>
       </c>
       <c r="C174" s="22" t="n"/>
@@ -7739,7 +7907,7 @@
       </c>
       <c r="B176" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Agrivoltaics or the co-location of agricultural activity and PV electricity production is a novel form of PV deployment which could provide farmers with diversified revenue sources and ecological benefits, while reducing land use competition, siting restrictions or adverse impacts on biodiversity and agricultural production. Optimizing system designs and business practices will help to enable simultaneous land use creating synergy for both agriculture and electricity production; this can benefit farmers, lower PV costs and enable the European Union to reach the goals of the EU</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Public authorities, industry, technology providers, energy producers and consumers profit from de-risking of cost-effective essential value chains of those renewable fuel technologies that can contribute to domestic commercial fuel production beyond 2030 customized to their needs, from improved access to better financing exploiting synergies across funding schemes, and from more effective market uptake, business models, increased competitiveness, and commercialization opportunities.Energy prod</t>
         </is>
       </c>
       <c r="C176" s="22" t="n"/>
@@ -7783,7 +7951,7 @@
       </c>
       <c r="B179" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-14</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-04</t>
         </is>
       </c>
       <c r="C179" s="22" t="n"/>
@@ -7794,7 +7962,7 @@
     <row r="181" ht="30" customHeight="1">
       <c r="A181" s="18" t="inlineStr">
         <is>
-          <t>FICHA 13: HORIZON-CL5-2027-07-D3-16</t>
+          <t>FICHA 13: HORIZON-CL5-2027-07-D3-27</t>
         </is>
       </c>
       <c r="B181" s="19" t="n"/>
@@ -7827,7 +7995,7 @@
       </c>
       <c r="B183" s="21" t="inlineStr">
         <is>
-          <t>Industrial processes and equipment for innovative, reliable and scalable tandem technologies (EUPI-PV Partnership)</t>
+          <t>Integrated Approaches for Retrofitting Infrastructures with Innovative Energy Storage Technologies</t>
         </is>
       </c>
       <c r="C183" s="22" t="n"/>
@@ -7843,7 +8011,7 @@
       </c>
       <c r="B184" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-16</t>
+          <t>HORIZON-CL5-2027-07-D3-27</t>
         </is>
       </c>
       <c r="C184" s="22" t="n"/>
@@ -7955,7 +8123,7 @@
       </c>
       <c r="B191" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:The REPowerEU plan and the EU Solar Energy Strategy introduced targets for the deployment of solar PV amounting to 600 GWac by 2030. Complying with these targets will be crucial for the European Union to reach its climate targets and free itself from import dependency on fossil fuels and the costs this imposes on Europe’s competitiveness in terms of high energy prices. The Solar Strategy also introduces a target, which has been enshrined into the Net-Zero Industry Act, to re-consolidate the European solar manufacturing sector and scale up European manufacturing capacity across</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Improved energy security of the energy system by offering cost-effective and efficient solutions for additional diverse and flexible energy storage capacities.Improve the sustainability and circularity of energy storage systems.Enhanced economic viability of energy storage by utilizing existing infrastructures.  Scope:Demonstration of novel or improved technological solutions for cost-efficient, circular and sustainable energy storage, which contribute to grid flexibility and make use of existing</t>
         </is>
       </c>
       <c r="C191" s="22" t="n"/>
@@ -7999,7 +8167,7 @@
       </c>
       <c r="B194" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-16</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-27</t>
         </is>
       </c>
       <c r="C194" s="22" t="n"/>
@@ -8010,7 +8178,7 @@
     <row r="196" ht="30" customHeight="1">
       <c r="A196" s="18" t="inlineStr">
         <is>
-          <t>FICHA 14: HORIZON-CL5-2027-07-D3-11</t>
+          <t>FICHA 14: HORIZON-CL5-2027-07-D3-26</t>
         </is>
       </c>
       <c r="B196" s="19" t="n"/>
@@ -8043,7 +8211,7 @@
       </c>
       <c r="B198" s="21" t="inlineStr">
         <is>
-          <t>Demonstration of hydropower technologies for efficient and forward-looking refurbishment of existing hydropower plants</t>
+          <t>Advanced Distribution Management Systems (ADSM) for more efficient and flexible distribution grids</t>
         </is>
       </c>
       <c r="C198" s="22" t="n"/>
@@ -8059,7 +8227,7 @@
       </c>
       <c r="B199" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-11</t>
+          <t>HORIZON-CL5-2027-07-D3-26</t>
         </is>
       </c>
       <c r="C199" s="22" t="n"/>
@@ -8171,7 +8339,7 @@
       </c>
       <c r="B206" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:For a renewables-based electricity system sufficient flexible and also in the long-run fully sustainable hydropower capacity is pivotal.Project results are expected to contribute to all of the following expected outcomes:Enhancing the capacities of the hydropower fleet to contribute with variable renewables base load to a secure and stable electricity system, including by modernising grid integration and hydropower fleet control.Increase technology leadership, competitiveness and technology export potential of European hydropower industry.Address challenges of climate change a</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced reliability, resilience, controllability and efficiency of electricity distribution grids. Congestion in distribution grids is managed effectively;Distribution system operators (DSO) leverage modern digital solutions and employ improved systems to effectively manage their grids and improve interoperability with TSOs and other DSOs;Vendor-agnostic reference architectures, solutions and tools are developed to help advancing the ADSM design and operation and effectively manage a broad range</t>
         </is>
       </c>
       <c r="C206" s="22" t="n"/>
@@ -8215,7 +8383,7 @@
       </c>
       <c r="B209" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-11</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-26</t>
         </is>
       </c>
       <c r="C209" s="22" t="n"/>
@@ -8442,7 +8610,7 @@
     <row r="226" ht="30" customHeight="1">
       <c r="A226" s="18" t="inlineStr">
         <is>
-          <t>FICHA 16: HORIZON-CL5-2027-07-D3-26</t>
+          <t>FICHA 16: HORIZON-CL5-2027-07-D3-28</t>
         </is>
       </c>
       <c r="B226" s="19" t="n"/>
@@ -8467,7 +8635,7 @@
       <c r="E227" s="22" t="n"/>
       <c r="F227" s="22" t="n"/>
     </row>
-    <row r="228" ht="45" customHeight="1">
+    <row r="228" ht="20" customHeight="1">
       <c r="A228" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -8475,7 +8643,7 @@
       </c>
       <c r="B228" s="21" t="inlineStr">
         <is>
-          <t>Advanced Distribution Management Systems (ADSM) for more efficient and flexible distribution grids</t>
+          <t>Community of practice - Data-Driven Decision-Making in Energy</t>
         </is>
       </c>
       <c r="C228" s="22" t="n"/>
@@ -8491,7 +8659,7 @@
       </c>
       <c r="B229" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-26</t>
+          <t>HORIZON-CL5-2027-07-D3-28</t>
         </is>
       </c>
       <c r="C229" s="22" t="n"/>
@@ -8571,7 +8739,7 @@
       </c>
       <c r="B234" s="21" t="inlineStr">
         <is>
-          <t>Innovation Actions</t>
+          <t>Coordination and Support Actions</t>
         </is>
       </c>
       <c r="C234" s="22" t="n"/>
@@ -8603,7 +8771,7 @@
       </c>
       <c r="B236" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced reliability, resilience, controllability and efficiency of electricity distribution grids. Congestion in distribution grids is managed effectively;Distribution system operators (DSO) leverage modern digital solutions and employ improved systems to effectively manage their grids and improve interoperability with TSOs and other DSOs;Vendor-agnostic reference architectures, solutions and tools are developed to help advancing the ADSM design and operation and effectively manage a broad range</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced EU cooperation to generate knowledge sharing on data and analytics used for the planning and operation of European grids, and market integration;Better EU coordination with regard to planning and simulation tools to support the development of electricity grids and integration of RES are made available to the research, academia, grid operators, and key actors in the energy value chains;Coordinated processes to generate new and innovative open-source solutions, software modules etc. that a</t>
         </is>
       </c>
       <c r="C236" s="22" t="n"/>
@@ -8647,7 +8815,7 @@
       </c>
       <c r="B239" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-26</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-28</t>
         </is>
       </c>
       <c r="C239" s="22" t="n"/>
@@ -8658,7 +8826,7 @@
     <row r="241" ht="30" customHeight="1">
       <c r="A241" s="18" t="inlineStr">
         <is>
-          <t>FICHA 17: HORIZON-CL5-2027-07-D3-27</t>
+          <t>FICHA 17: HORIZON-CL5-2027-07-D3-16</t>
         </is>
       </c>
       <c r="B241" s="19" t="n"/>
@@ -8691,7 +8859,7 @@
       </c>
       <c r="B243" s="21" t="inlineStr">
         <is>
-          <t>Integrated Approaches for Retrofitting Infrastructures with Innovative Energy Storage Technologies</t>
+          <t>Industrial processes and equipment for innovative, reliable and scalable tandem technologies (EUPI-PV Partnership)</t>
         </is>
       </c>
       <c r="C243" s="22" t="n"/>
@@ -8707,7 +8875,7 @@
       </c>
       <c r="B244" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-27</t>
+          <t>HORIZON-CL5-2027-07-D3-16</t>
         </is>
       </c>
       <c r="C244" s="22" t="n"/>
@@ -8819,7 +8987,7 @@
       </c>
       <c r="B251" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Improved energy security of the energy system by offering cost-effective and efficient solutions for additional diverse and flexible energy storage capacities.Improve the sustainability and circularity of energy storage systems.Enhanced economic viability of energy storage by utilizing existing infrastructures.  Scope:Demonstration of novel or improved technological solutions for cost-efficient, circular and sustainable energy storage, which contribute to grid flexibility and make use of existing</t>
+          <t>Expected Outcome:The REPowerEU plan and the EU Solar Energy Strategy introduced targets for the deployment of solar PV amounting to 600 GWac by 2030. Complying with these targets will be crucial for the European Union to reach its climate targets and free itself from import dependency on fossil fuels and the costs this imposes on Europe’s competitiveness in terms of high energy prices. The Solar Strategy also introduces a target, which has been enshrined into the Net-Zero Industry Act, to re-consolidate the European solar manufacturing sector and scale up European manufacturing capacity across</t>
         </is>
       </c>
       <c r="C251" s="22" t="n"/>
@@ -8863,7 +9031,7 @@
       </c>
       <c r="B254" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-27</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-16</t>
         </is>
       </c>
       <c r="C254" s="22" t="n"/>
@@ -8874,7 +9042,7 @@
     <row r="256" ht="30" customHeight="1">
       <c r="A256" s="18" t="inlineStr">
         <is>
-          <t>FICHA 18: HORIZON-CL5-2027-07-D3-28</t>
+          <t>FICHA 18: HORIZON-CL5-2027-07-D3-25</t>
         </is>
       </c>
       <c r="B256" s="19" t="n"/>
@@ -8899,7 +9067,7 @@
       <c r="E257" s="22" t="n"/>
       <c r="F257" s="22" t="n"/>
     </row>
-    <row r="258" ht="20" customHeight="1">
+    <row r="258" ht="45" customHeight="1">
       <c r="A258" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -8907,7 +9075,7 @@
       </c>
       <c r="B258" s="21" t="inlineStr">
         <is>
-          <t>Community of practice - Data-Driven Decision-Making in Energy</t>
+          <t>Advanced TSO control rooms to enhance grid observability, stability and resilience</t>
         </is>
       </c>
       <c r="C258" s="22" t="n"/>
@@ -8923,7 +9091,7 @@
       </c>
       <c r="B259" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-28</t>
+          <t>HORIZON-CL5-2027-07-D3-25</t>
         </is>
       </c>
       <c r="C259" s="22" t="n"/>
@@ -9003,7 +9171,7 @@
       </c>
       <c r="B264" s="21" t="inlineStr">
         <is>
-          <t>Coordination and Support Actions</t>
+          <t>Innovation Actions</t>
         </is>
       </c>
       <c r="C264" s="22" t="n"/>
@@ -9035,7 +9203,7 @@
       </c>
       <c r="B266" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced EU cooperation to generate knowledge sharing on data and analytics used for the planning and operation of European grids, and market integration;Better EU coordination with regard to planning and simulation tools to support the development of electricity grids and integration of RES are made available to the research, academia, grid operators, and key actors in the energy value chains;Coordinated processes to generate new and innovative open-source solutions, software modules etc. that a</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced reliability, resilience, and efficiency of electricity transmission grids. Grid congestion is managed efficiently;Enhanced observability of grids and improved forecasting of supply, demand, grid capacity availability, and flexibility;Transmission system operators (TSO) leverage modern digital solutions and employ improved systems to effectively manage their grids and improve interoperability with other TSOs;Vendor-agnostic reference architectures, solutions and tools are developed to hel</t>
         </is>
       </c>
       <c r="C266" s="22" t="n"/>
@@ -9079,7 +9247,7 @@
       </c>
       <c r="B269" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-28</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-25</t>
         </is>
       </c>
       <c r="C269" s="22" t="n"/>
@@ -9090,7 +9258,7 @@
     <row r="271" ht="30" customHeight="1">
       <c r="A271" s="18" t="inlineStr">
         <is>
-          <t>FICHA 19: HORIZON-CL5-2027-07-D3-25</t>
+          <t>FICHA 19: HORIZON-CL5-2027-07-D3-17</t>
         </is>
       </c>
       <c r="B271" s="19" t="n"/>
@@ -9123,7 +9291,7 @@
       </c>
       <c r="B273" s="21" t="inlineStr">
         <is>
-          <t>Advanced TSO control rooms to enhance grid observability, stability and resilience</t>
+          <t>PV based electrification of the economy: Designing &amp; optimising PV systems supporting industrial electrification and promoting participation in electricity markets (EUPI-PV Partnership)</t>
         </is>
       </c>
       <c r="C273" s="22" t="n"/>
@@ -9139,7 +9307,7 @@
       </c>
       <c r="B274" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-25</t>
+          <t>HORIZON-CL5-2027-07-D3-17</t>
         </is>
       </c>
       <c r="C274" s="22" t="n"/>
@@ -9251,7 +9419,7 @@
       </c>
       <c r="B281" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced reliability, resilience, and efficiency of electricity transmission grids. Grid congestion is managed efficiently;Enhanced observability of grids and improved forecasting of supply, demand, grid capacity availability, and flexibility;Transmission system operators (TSO) leverage modern digital solutions and employ improved systems to effectively manage their grids and improve interoperability with other TSOs;Vendor-agnostic reference architectures, solutions and tools are developed to hel</t>
+          <t>Expected Outcome:Large PV systems such as utility scale PV are evolving towards higher voltage architecture (&amp;gt;=3kV) with the objective to minimize losses and improve system efficiency at lower costs. The intention is to integrate also storage into such (hybrid) PV systems offering flexibility. It is consequently essential to build a blueprint for the implementation of high voltage large PV systems and the development of Direct Current (DC) networks around strategic end users for high voltage demand (industrial sites, servers, electric vehicle charging stations…). Understanding the factors t</t>
         </is>
       </c>
       <c r="C281" s="22" t="n"/>
@@ -9295,7 +9463,7 @@
       </c>
       <c r="B284" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-25</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-17</t>
         </is>
       </c>
       <c r="C284" s="22" t="n"/>
@@ -9306,7 +9474,7 @@
     <row r="286" ht="30" customHeight="1">
       <c r="A286" s="18" t="inlineStr">
         <is>
-          <t>FICHA 20: HORIZON-CL5-2027-07-D3-17</t>
+          <t>FICHA 20: HORIZON-CL5-2027-07-D3-11</t>
         </is>
       </c>
       <c r="B286" s="19" t="n"/>
@@ -9339,7 +9507,7 @@
       </c>
       <c r="B288" s="21" t="inlineStr">
         <is>
-          <t>PV based electrification of the economy: Designing &amp; optimising PV systems supporting industrial electrification and promoting participation in electricity markets (EUPI-PV Partnership)</t>
+          <t>Demonstration of hydropower technologies for efficient and forward-looking refurbishment of existing hydropower plants</t>
         </is>
       </c>
       <c r="C288" s="22" t="n"/>
@@ -9355,7 +9523,7 @@
       </c>
       <c r="B289" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-17</t>
+          <t>HORIZON-CL5-2027-07-D3-11</t>
         </is>
       </c>
       <c r="C289" s="22" t="n"/>
@@ -9467,7 +9635,7 @@
       </c>
       <c r="B296" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Large PV systems such as utility scale PV are evolving towards higher voltage architecture (&amp;gt;=3kV) with the objective to minimize losses and improve system efficiency at lower costs. The intention is to integrate also storage into such (hybrid) PV systems offering flexibility. It is consequently essential to build a blueprint for the implementation of high voltage large PV systems and the development of Direct Current (DC) networks around strategic end users for high voltage demand (industrial sites, servers, electric vehicle charging stations…). Understanding the factors t</t>
+          <t>Expected Outcome:For a renewables-based electricity system sufficient flexible and also in the long-run fully sustainable hydropower capacity is pivotal.Project results are expected to contribute to all of the following expected outcomes:Enhancing the capacities of the hydropower fleet to contribute with variable renewables base load to a secure and stable electricity system, including by modernising grid integration and hydropower fleet control.Increase technology leadership, competitiveness and technology export potential of European hydropower industry.Address challenges of climate change a</t>
         </is>
       </c>
       <c r="C296" s="22" t="n"/>
@@ -9511,7 +9679,7 @@
       </c>
       <c r="B299" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-17</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-11</t>
         </is>
       </c>
       <c r="C299" s="22" t="n"/>
@@ -9522,7 +9690,7 @@
     <row r="301" ht="30" customHeight="1">
       <c r="A301" s="18" t="inlineStr">
         <is>
-          <t>FICHA 21: HORIZON-CL5-2027-01-D1-07</t>
+          <t>FICHA 21: HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="B301" s="19" t="n"/>
@@ -9547,7 +9715,7 @@
       <c r="E302" s="22" t="n"/>
       <c r="F302" s="22" t="n"/>
     </row>
-    <row r="303" ht="45" customHeight="1">
+    <row r="303" ht="20" customHeight="1">
       <c r="A303" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -9555,7 +9723,7 @@
       </c>
       <c r="B303" s="21" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
+          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
         </is>
       </c>
       <c r="C303" s="22" t="n"/>
@@ -9571,7 +9739,7 @@
       </c>
       <c r="B304" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="C304" s="22" t="n"/>
@@ -9683,7 +9851,7 @@
       </c>
       <c r="B311" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Europe and globally, as well as the interaction between different hazards, their cumulative and/or cascading effects.Enhanced seamless prediction and projection modelling and attribution capabilities for extreme events and their likelihood to support preparedness, response and resilience to climate change by EU and national and regional actors. The EU Union Preparedness Strategy, the EU Adaptation Str</t>
+          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and interactions with ecosystems, leading to improved Earth system models;Future climate change scenarios produced in light of past changes in the Earth system, in particular warm climates/high sea-level situations, and abrupt transitions;Identification of thresholds in Earth system components and better characterisation of driving mechanisms and feedbacks that may be responsible for non-linear behaviours,</t>
         </is>
       </c>
       <c r="C311" s="22" t="n"/>
@@ -9727,7 +9895,7 @@
       </c>
       <c r="B314" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-07</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="C314" s="22" t="n"/>
@@ -10170,7 +10338,7 @@
     <row r="346" ht="30" customHeight="1">
       <c r="A346" s="18" t="inlineStr">
         <is>
-          <t>FICHA 24: HORIZON-CL5-2027-01-D1-09</t>
+          <t>FICHA 24: HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="B346" s="19" t="n"/>
@@ -10195,7 +10363,7 @@
       <c r="E347" s="22" t="n"/>
       <c r="F347" s="22" t="n"/>
     </row>
-    <row r="348" ht="45" customHeight="1">
+    <row r="348" ht="20" customHeight="1">
       <c r="A348" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -10203,7 +10371,7 @@
       </c>
       <c r="B348" s="21" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="C348" s="22" t="n"/>
@@ -10219,7 +10387,7 @@
       </c>
       <c r="B349" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C349" s="22" t="n"/>
@@ -10299,7 +10467,7 @@
       </c>
       <c r="B354" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Research and Innovation Actions</t>
+          <t>Programme Cofund Actions</t>
         </is>
       </c>
       <c r="C354" s="22" t="n"/>
@@ -10331,7 +10499,7 @@
       </c>
       <c r="B356" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to inform mitigation action and policy improvements, ensuring a fair transition and social acceptability;Methodologies are developed and improved for ex-ante assessment and ex-post evaluation of greenhouse gas emission reductions from climate policies and measures;Strengthened collaboration and established networks between researchers, policy experts and government officials involved in designing and eva</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is established through development and implementation of the Climate Action pillar of the EU-AU Research and Innovation Partnership on Climate Change and Sustainable Energy (CCSE),[1] in co-design between African and European partners;Reduced fragmentation by aligning the EU, national and multilateral R&amp;amp;I efforts with increased leverage and impact of funding;African scientific, policy and practice com</t>
         </is>
       </c>
       <c r="C356" s="22" t="n"/>
@@ -10375,7 +10543,7 @@
       </c>
       <c r="B359" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-09</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C359" s="22" t="n"/>
@@ -10386,7 +10554,7 @@
     <row r="361" ht="30" customHeight="1">
       <c r="A361" s="18" t="inlineStr">
         <is>
-          <t>FICHA 25: HORIZON-CL5-2027-01-D1-08</t>
+          <t>FICHA 25: HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="B361" s="19" t="n"/>
@@ -10419,7 +10587,7 @@
       </c>
       <c r="B363" s="21" t="inlineStr">
         <is>
-          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="C363" s="22" t="n"/>
@@ -10435,7 +10603,7 @@
       </c>
       <c r="B364" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-08</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C364" s="22" t="n"/>
@@ -10547,7 +10715,7 @@
       </c>
       <c r="B371" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and interactions with ecosystems, leading to improved Earth system models;Future climate change scenarios produced in light of past changes in the Earth system, in particular warm climates/high sea-level situations, and abrupt transitions;Identification of thresholds in Earth system components and better characterisation of driving mechanisms and feedbacks that may be responsible for non-linear behaviours,</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorporation into main EU repositories, such as Climate-ADAPT or the portal of the EU Mission on Adaptation to Climate Change;The risk and adaptation assessment frameworks are improved by better integrating the maladaptation dimension;Guidelines and tools for maladaptation prevention and correction strategies are made available to adaptation stakeholders at relevant scales and inform the design and impl</t>
         </is>
       </c>
       <c r="C371" s="22" t="n"/>
@@ -10591,7 +10759,7 @@
       </c>
       <c r="B374" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-08</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C374" s="22" t="n"/>
@@ -10602,7 +10770,7 @@
     <row r="376" ht="30" customHeight="1">
       <c r="A376" s="18" t="inlineStr">
         <is>
-          <t>FICHA 26: HORIZON-CL5-2027-01-D1-11</t>
+          <t>FICHA 26: HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="B376" s="19" t="n"/>
@@ -10627,7 +10795,7 @@
       <c r="E377" s="22" t="n"/>
       <c r="F377" s="22" t="n"/>
     </row>
-    <row r="378" ht="20" customHeight="1">
+    <row r="378" ht="45" customHeight="1">
       <c r="A378" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -10635,7 +10803,7 @@
       </c>
       <c r="B378" s="21" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
         </is>
       </c>
       <c r="C378" s="22" t="n"/>
@@ -10651,7 +10819,7 @@
       </c>
       <c r="B379" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C379" s="22" t="n"/>
@@ -10731,7 +10899,7 @@
       </c>
       <c r="B384" s="21" t="inlineStr">
         <is>
-          <t>Programme Cofund Actions</t>
+          <t xml:space="preserve"> Research and Innovation Actions</t>
         </is>
       </c>
       <c r="C384" s="22" t="n"/>
@@ -10763,7 +10931,7 @@
       </c>
       <c r="B386" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is established through development and implementation of the Climate Action pillar of the EU-AU Research and Innovation Partnership on Climate Change and Sustainable Energy (CCSE),[1] in co-design between African and European partners;Reduced fragmentation by aligning the EU, national and multilateral R&amp;amp;I efforts with increased leverage and impact of funding;African scientific, policy and practice com</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to inform mitigation action and policy improvements, ensuring a fair transition and social acceptability;Methodologies are developed and improved for ex-ante assessment and ex-post evaluation of greenhouse gas emission reductions from climate policies and measures;Strengthened collaboration and established networks between researchers, policy experts and government officials involved in designing and eva</t>
         </is>
       </c>
       <c r="C386" s="22" t="n"/>
@@ -10807,7 +10975,7 @@
       </c>
       <c r="B389" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-11</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C389" s="22" t="n"/>
@@ -10818,7 +10986,7 @@
     <row r="391" ht="30" customHeight="1">
       <c r="A391" s="18" t="inlineStr">
         <is>
-          <t>FICHA 27: HORIZON-CL5-2027-01-D1-10</t>
+          <t>FICHA 27: HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="B391" s="19" t="n"/>
@@ -10843,7 +11011,7 @@
       <c r="E392" s="22" t="n"/>
       <c r="F392" s="22" t="n"/>
     </row>
-    <row r="393" ht="20" customHeight="1">
+    <row r="393" ht="45" customHeight="1">
       <c r="A393" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -10851,7 +11019,7 @@
       </c>
       <c r="B393" s="21" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
         </is>
       </c>
       <c r="C393" s="22" t="n"/>
@@ -10867,7 +11035,7 @@
       </c>
       <c r="B394" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C394" s="22" t="n"/>
@@ -10979,7 +11147,7 @@
       </c>
       <c r="B401" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorporation into main EU repositories, such as Climate-ADAPT or the portal of the EU Mission on Adaptation to Climate Change;The risk and adaptation assessment frameworks are improved by better integrating the maladaptation dimension;Guidelines and tools for maladaptation prevention and correction strategies are made available to adaptation stakeholders at relevant scales and inform the design and impl</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Europe and globally, as well as the interaction between different hazards, their cumulative and/or cascading effects.Enhanced seamless prediction and projection modelling and attribution capabilities for extreme events and their likelihood to support preparedness, response and resilience to climate change by EU and national and regional actors. The EU Union Preparedness Strategy, the EU Adaptation Str</t>
         </is>
       </c>
       <c r="C401" s="22" t="n"/>
@@ -11023,7 +11191,7 @@
       </c>
       <c r="B404" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-10</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C404" s="22" t="n"/>
@@ -14110,7 +14278,7 @@
     <row r="616" ht="30" customHeight="1">
       <c r="A616" s="18" t="inlineStr">
         <is>
-          <t>FICHA 42: HORIZON-CL5-2027-02-D3-08</t>
+          <t>FICHA 42: HORIZON-CL5-2027-02-D3-31</t>
         </is>
       </c>
       <c r="B616" s="19" t="n"/>
@@ -14143,7 +14311,7 @@
       </c>
       <c r="B618" s="21" t="inlineStr">
         <is>
-          <t>Co-funding Strategic Energy Technology (SET) Plan renewable fuel value chains at EU, national, regional, and local level</t>
+          <t>Support to the implementation of an EU policy framework for CO2 transport and storage infrastructure</t>
         </is>
       </c>
       <c r="C618" s="22" t="n"/>
@@ -14159,7 +14327,7 @@
       </c>
       <c r="B619" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-08</t>
+          <t>HORIZON-CL5-2027-02-D3-31</t>
         </is>
       </c>
       <c r="C619" s="22" t="n"/>
@@ -14239,7 +14407,7 @@
       </c>
       <c r="B624" s="21" t="inlineStr">
         <is>
-          <t>Programme Cofund Actions</t>
+          <t>Coordination and Support Actions</t>
         </is>
       </c>
       <c r="C624" s="22" t="n"/>
@@ -14271,7 +14439,7 @@
       </c>
       <c r="B626" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Advance in the realisation of the Strategic Energy Technology (SET) Plan Action of Renewable fuels and Bioenergy (for the fuels part) is supported, overcoming fragmentation by mobilizing resources and establishing across EU interregional value chains of renewable fuel technologies and by better alignment of public and private R&amp;amp;I priorities and of funding mechanisms.All sector stakeholders benefit from establishment of renewable fuels value chains at EU, national, regional, and local level</t>
+          <t>Expected Outcome:Project results are expected to contribute to the following outcome:Stakeholders involved in the CO2 infrastructure network are in a position to implement the upcoming legislative framework for CO2 infrastructure.  Scope:The project is expected to assist stakeholders involved in the CO2 infrastructure network in implementing the upcoming legislative framework for CO2 infrastructure.Issues to address include market and cost structure, cross-border integration, interoperability and planning, technical harmonisation and investment incentives for new infrastructure, third-party ac</t>
         </is>
       </c>
       <c r="C626" s="22" t="n"/>
@@ -14315,7 +14483,7 @@
       </c>
       <c r="B629" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-08</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-31</t>
         </is>
       </c>
       <c r="C629" s="22" t="n"/>
@@ -14326,7 +14494,7 @@
     <row r="631" ht="30" customHeight="1">
       <c r="A631" s="18" t="inlineStr">
         <is>
-          <t>FICHA 43: HORIZON-CL5-2027-02-D3-09</t>
+          <t>FICHA 43: HORIZON-CL5-2027-02-D3-24</t>
         </is>
       </c>
       <c r="B631" s="19" t="n"/>
@@ -14351,7 +14519,7 @@
       <c r="E632" s="22" t="n"/>
       <c r="F632" s="22" t="n"/>
     </row>
-    <row r="633" ht="20" customHeight="1">
+    <row r="633" ht="45" customHeight="1">
       <c r="A633" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -14359,7 +14527,7 @@
       </c>
       <c r="B633" s="21" t="inlineStr">
         <is>
-          <t>Innovative technologies and solutions to improve wave and tidal energy systems</t>
+          <t>Large scale operational validation and upscaling of state-of-the-art (Generative) AI tools and models powering a next generation digital energy system</t>
         </is>
       </c>
       <c r="C633" s="22" t="n"/>
@@ -14375,7 +14543,7 @@
       </c>
       <c r="B634" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-09</t>
+          <t>HORIZON-CL5-2027-02-D3-24</t>
         </is>
       </c>
       <c r="C634" s="22" t="n"/>
@@ -14487,7 +14655,7 @@
       </c>
       <c r="B641" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all following expected outcomes:Advance in the realisation of the Strategic Energy Technology (SET) Plan’s research and innovation priorities and targets for ocean energy;Energy producers and consumers benefit from increased performance of wave and tidal energy technologies with the focus on efficiency and flexibility, reduced cost, improved reliability and sustainability, operation and maintenance, robustness and security during all stages of the lifetime of an ocean energy farm from installation, operation and maintenance to deco</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Advanced, secure frugal (energy-, resource-, data- and cost-efficient, sustainable) AI tools for real-time grid operations (including protection), market operations (if relevant) and consumer empowerment in distributed energy systems.A demonstrated AI development environment integrated with the upgraded digital spine of the energy system and energy-saving consumer applications.Scaled-up capabilities for learning at edge nodes and federated systems using agent-based architectures.A governance fram</t>
         </is>
       </c>
       <c r="C641" s="22" t="n"/>
@@ -14531,7 +14699,7 @@
       </c>
       <c r="B644" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-09</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-24</t>
         </is>
       </c>
       <c r="C644" s="22" t="n"/>
@@ -14758,7 +14926,7 @@
     <row r="661" ht="30" customHeight="1">
       <c r="A661" s="18" t="inlineStr">
         <is>
-          <t>FICHA 45: HORIZON-CL5-2027-02-D3-24</t>
+          <t>FICHA 45: HORIZON-CL5-2027-02-D3-15</t>
         </is>
       </c>
       <c r="B661" s="19" t="n"/>
@@ -14791,7 +14959,7 @@
       </c>
       <c r="B663" s="21" t="inlineStr">
         <is>
-          <t>Large scale operational validation and upscaling of state-of-the-art (Generative) AI tools and models powering a next generation digital energy system</t>
+          <t>Production technologies for solar photovoltaics beyond the state-of-the-art (EUPI-PV Partnership)</t>
         </is>
       </c>
       <c r="C663" s="22" t="n"/>
@@ -14807,7 +14975,7 @@
       </c>
       <c r="B664" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-24</t>
+          <t>HORIZON-CL5-2027-02-D3-15</t>
         </is>
       </c>
       <c r="C664" s="22" t="n"/>
@@ -14919,7 +15087,7 @@
       </c>
       <c r="B671" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Advanced, secure frugal (energy-, resource-, data- and cost-efficient, sustainable) AI tools for real-time grid operations (including protection), market operations (if relevant) and consumer empowerment in distributed energy systems.A demonstrated AI development environment integrated with the upgraded digital spine of the energy system and energy-saving consumer applications.Scaled-up capabilities for learning at edge nodes and federated systems using agent-based architectures.A governance fram</t>
+          <t>Expected Outcome:The REPowerEU plan and the EU Solar Energy Strategy introduced targets for the deployment of solar PV amounting to 600 GWac by 2030. Complying with these targets will be crucial for the European Union to reach its climate targets and free itself from import dependency on fossil fuels and the costs this imposes on Europe’s competitiveness in terms of high energy prices. The Solar Strategy also introduces a target, which has been enshrined into the Net-Zero Industry Act, to re-consolidate the European solar manufacturing sector and scale up European manufacturing capacity across</t>
         </is>
       </c>
       <c r="C671" s="22" t="n"/>
@@ -14963,7 +15131,7 @@
       </c>
       <c r="B674" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-24</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-15</t>
         </is>
       </c>
       <c r="C674" s="22" t="n"/>
@@ -14974,7 +15142,7 @@
     <row r="676" ht="30" customHeight="1">
       <c r="A676" s="18" t="inlineStr">
         <is>
-          <t>FICHA 46: HORIZON-CL5-2027-02-D3-31</t>
+          <t>FICHA 46: HORIZON-CL5-2027-02-D3-07</t>
         </is>
       </c>
       <c r="B676" s="19" t="n"/>
@@ -14999,7 +15167,7 @@
       <c r="E677" s="22" t="n"/>
       <c r="F677" s="22" t="n"/>
     </row>
-    <row r="678" ht="45" customHeight="1">
+    <row r="678" ht="20" customHeight="1">
       <c r="A678" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -15007,7 +15175,7 @@
       </c>
       <c r="B678" s="21" t="inlineStr">
         <is>
-          <t>Support to the implementation of an EU policy framework for CO2 transport and storage infrastructure</t>
+          <t>Concentrated solar thermal systems for decarbonising industrial processes</t>
         </is>
       </c>
       <c r="C678" s="22" t="n"/>
@@ -15023,7 +15191,7 @@
       </c>
       <c r="B679" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-31</t>
+          <t>HORIZON-CL5-2027-02-D3-07</t>
         </is>
       </c>
       <c r="C679" s="22" t="n"/>
@@ -15103,7 +15271,7 @@
       </c>
       <c r="B684" s="21" t="inlineStr">
         <is>
-          <t>Coordination and Support Actions</t>
+          <t>Innovation Actions</t>
         </is>
       </c>
       <c r="C684" s="22" t="n"/>
@@ -15135,7 +15303,7 @@
       </c>
       <c r="B686" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to the following outcome:Stakeholders involved in the CO2 infrastructure network are in a position to implement the upcoming legislative framework for CO2 infrastructure.  Scope:The project is expected to assist stakeholders involved in the CO2 infrastructure network in implementing the upcoming legislative framework for CO2 infrastructure.Issues to address include market and cost structure, cross-border integration, interoperability and planning, technical harmonisation and investment incentives for new infrastructure, third-party ac</t>
+          <t>Expected Outcome:Renewable heating can be directly used to efficiently decarbonise industrial processes. Concentrated solar thermal technologies offer a great potential to supply renewable heat for industry for temperatures between 150°C - 400°C. Nevertheless, efforts are still required to demonstrate these technologies for a variety of industrial processes.Proposals are expected to contribute to all the following outcomes:Showcase the capacity of concentrated solar thermal systems to largely meet the heat demand of industrial processes and to achieve a yearly solar fraction of at least 50%.In</t>
         </is>
       </c>
       <c r="C686" s="22" t="n"/>
@@ -15179,7 +15347,7 @@
       </c>
       <c r="B689" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-31</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-07</t>
         </is>
       </c>
       <c r="C689" s="22" t="n"/>
@@ -15190,7 +15358,7 @@
     <row r="691" ht="30" customHeight="1">
       <c r="A691" s="18" t="inlineStr">
         <is>
-          <t>FICHA 47: HORIZON-CL5-2027-02-D3-15</t>
+          <t>FICHA 47: HORIZON-CL5-2027-02-D3-08</t>
         </is>
       </c>
       <c r="B691" s="19" t="n"/>
@@ -15223,7 +15391,7 @@
       </c>
       <c r="B693" s="21" t="inlineStr">
         <is>
-          <t>Production technologies for solar photovoltaics beyond the state-of-the-art (EUPI-PV Partnership)</t>
+          <t>Co-funding Strategic Energy Technology (SET) Plan renewable fuel value chains at EU, national, regional, and local level</t>
         </is>
       </c>
       <c r="C693" s="22" t="n"/>
@@ -15239,7 +15407,7 @@
       </c>
       <c r="B694" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-15</t>
+          <t>HORIZON-CL5-2027-02-D3-08</t>
         </is>
       </c>
       <c r="C694" s="22" t="n"/>
@@ -15319,7 +15487,7 @@
       </c>
       <c r="B699" s="21" t="inlineStr">
         <is>
-          <t>Innovation Actions</t>
+          <t>Programme Cofund Actions</t>
         </is>
       </c>
       <c r="C699" s="22" t="n"/>
@@ -15351,7 +15519,7 @@
       </c>
       <c r="B701" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:The REPowerEU plan and the EU Solar Energy Strategy introduced targets for the deployment of solar PV amounting to 600 GWac by 2030. Complying with these targets will be crucial for the European Union to reach its climate targets and free itself from import dependency on fossil fuels and the costs this imposes on Europe’s competitiveness in terms of high energy prices. The Solar Strategy also introduces a target, which has been enshrined into the Net-Zero Industry Act, to re-consolidate the European solar manufacturing sector and scale up European manufacturing capacity across</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Advance in the realisation of the Strategic Energy Technology (SET) Plan Action of Renewable fuels and Bioenergy (for the fuels part) is supported, overcoming fragmentation by mobilizing resources and establishing across EU interregional value chains of renewable fuel technologies and by better alignment of public and private R&amp;amp;I priorities and of funding mechanisms.All sector stakeholders benefit from establishment of renewable fuels value chains at EU, national, regional, and local level</t>
         </is>
       </c>
       <c r="C701" s="22" t="n"/>
@@ -15395,7 +15563,7 @@
       </c>
       <c r="B704" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-15</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-08</t>
         </is>
       </c>
       <c r="C704" s="22" t="n"/>
@@ -18970,7 +19138,7 @@
     <row r="961" ht="30" customHeight="1">
       <c r="A961" s="18" t="inlineStr">
         <is>
-          <t>FICHA 65: EUS-13454</t>
+          <t>FICHA 65: EUS-41373</t>
         </is>
       </c>
       <c r="B961" s="19" t="n"/>
@@ -19019,7 +19187,7 @@
       </c>
       <c r="B964" s="21" t="inlineStr">
         <is>
-          <t>EUS-13454</t>
+          <t>EUS-41373</t>
         </is>
       </c>
       <c r="C964" s="22" t="n"/>
@@ -19182,7 +19350,7 @@
     <row r="976" ht="30" customHeight="1">
       <c r="A976" s="18" t="inlineStr">
         <is>
-          <t>FICHA 66: EUS-59353</t>
+          <t>FICHA 66: EUS-68354</t>
         </is>
       </c>
       <c r="B976" s="19" t="n"/>
@@ -19231,7 +19399,7 @@
       </c>
       <c r="B979" s="21" t="inlineStr">
         <is>
-          <t>EUS-59353</t>
+          <t>EUS-68354</t>
         </is>
       </c>
       <c r="C979" s="22" t="n"/>
@@ -19394,7 +19562,7 @@
     <row r="991" ht="30" customHeight="1">
       <c r="A991" s="18" t="inlineStr">
         <is>
-          <t>FICHA 67: EUS-00407</t>
+          <t>FICHA 67: EUS-84214</t>
         </is>
       </c>
       <c r="B991" s="19" t="n"/>
@@ -19419,7 +19587,7 @@
       <c r="E992" s="22" t="n"/>
       <c r="F992" s="22" t="n"/>
     </row>
-    <row r="993" ht="20" customHeight="1">
+    <row r="993" ht="45" customHeight="1">
       <c r="A993" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -19427,7 +19595,7 @@
       </c>
       <c r="B993" s="21" t="inlineStr">
         <is>
-          <t>Ases. técnico diseño y plan de acción clima labora</t>
+          <t>Mantenimiento preventivo y correctivo de los equipos de climatización de los despachos y otras estancias de los cinco edificios y el suministro de nuevos equipos</t>
         </is>
       </c>
       <c r="C993" s="22" t="n"/>
@@ -19443,7 +19611,7 @@
       </c>
       <c r="B994" s="21" t="inlineStr">
         <is>
-          <t>EUS-00407</t>
+          <t>EUS-84214</t>
         </is>
       </c>
       <c r="C994" s="22" t="n"/>
@@ -19595,7 +19763,7 @@
       </c>
       <c r="B1004" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/ases-tecnico-diseno-y-plan-accion-clima-labora/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/mantenimiento-preventivo-y-correctivo-equipos-climatizacion-despachos-y-otras-estancias-cinco-edificios-y-suministro-nuevos-equipos/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1004" s="22" t="n"/>
@@ -19606,7 +19774,7 @@
     <row r="1006" ht="30" customHeight="1">
       <c r="A1006" s="18" t="inlineStr">
         <is>
-          <t>FICHA 68: EUS-78654</t>
+          <t>FICHA 68: EUS-43982</t>
         </is>
       </c>
       <c r="B1006" s="19" t="n"/>
@@ -19631,7 +19799,7 @@
       <c r="E1007" s="22" t="n"/>
       <c r="F1007" s="22" t="n"/>
     </row>
-    <row r="1008" ht="20" customHeight="1">
+    <row r="1008" ht="45" customHeight="1">
       <c r="A1008" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -19639,7 +19807,7 @@
       </c>
       <c r="B1008" s="21" t="inlineStr">
         <is>
-          <t>Plan de movilidad</t>
+          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta el 01.10.26. Cribado de enfermedades con inteligencia artificial. Espacio de Datos Sanitarios de la UE. Red de Centros para Seguridad de la I</t>
         </is>
       </c>
       <c r="C1008" s="22" t="n"/>
@@ -19655,7 +19823,7 @@
       </c>
       <c r="B1009" s="21" t="inlineStr">
         <is>
-          <t>EUS-78654</t>
+          <t>EUS-43982</t>
         </is>
       </c>
       <c r="C1009" s="22" t="n"/>
@@ -19731,7 +19899,7 @@
       </c>
       <c r="B1014" s="21" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C1014" s="22" t="n"/>
@@ -19789,9 +19957,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B1018" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ALTA — </t>
+      <c r="B1018" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
         </is>
       </c>
       <c r="C1018" s="22" t="n"/>
@@ -19807,7 +19975,7 @@
       </c>
       <c r="B1019" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/plan-movilidad/expcm508889/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260422digitaleuropekoak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1019" s="22" t="n"/>
@@ -19818,7 +19986,7 @@
     <row r="1021" ht="30" customHeight="1">
       <c r="A1021" s="18" t="inlineStr">
         <is>
-          <t>FICHA 69: EUS-15400</t>
+          <t>FICHA 69: EUS-33357</t>
         </is>
       </c>
       <c r="B1021" s="19" t="n"/>
@@ -19851,7 +20019,7 @@
       </c>
       <c r="B1023" s="21" t="inlineStr">
         <is>
-          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta el 01.10.26. Cribado de enfermedades con inteligencia artificial. Espacio de Datos Sanitarios de la UE. Red de Centros para Seguridad de la I</t>
+          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversidad, participación, principios de la UE. Eventos, difusiones e intercambios. Programa de Ciudadanos, Igualdad, Derechos y Valores de la UE (</t>
         </is>
       </c>
       <c r="C1023" s="22" t="n"/>
@@ -19867,7 +20035,7 @@
       </c>
       <c r="B1024" s="21" t="inlineStr">
         <is>
-          <t>EUS-15400</t>
+          <t>EUS-33357</t>
         </is>
       </c>
       <c r="C1024" s="22" t="n"/>
@@ -20019,7 +20187,7 @@
       </c>
       <c r="B1034" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260422digitaleuropekoak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260408cervhirisareak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1034" s="22" t="n"/>
@@ -20030,7 +20198,7 @@
     <row r="1036" ht="30" customHeight="1">
       <c r="A1036" s="18" t="inlineStr">
         <is>
-          <t>FICHA 70: EUS-82152</t>
+          <t>FICHA 70: EUS-05202</t>
         </is>
       </c>
       <c r="B1036" s="19" t="n"/>
@@ -20063,7 +20231,7 @@
       </c>
       <c r="B1038" s="21" t="inlineStr">
         <is>
-          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversidad, participación, principios de la UE. Eventos, difusiones e intercambios. Programa de Ciudadanos, Igualdad, Derechos y Valores de la UE (</t>
+          <t>Servicio de control antidopaje (recogida de muestras) a través del personal habilitado para la Agencia Vasca Antidopaje, período 2026-2027.</t>
         </is>
       </c>
       <c r="C1038" s="22" t="n"/>
@@ -20079,7 +20247,7 @@
       </c>
       <c r="B1039" s="21" t="inlineStr">
         <is>
-          <t>EUS-82152</t>
+          <t>EUS-05202</t>
         </is>
       </c>
       <c r="C1039" s="22" t="n"/>
@@ -20155,7 +20323,7 @@
       </c>
       <c r="B1044" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C1044" s="22" t="n"/>
@@ -20231,7 +20399,7 @@
       </c>
       <c r="B1049" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260408cervhirisareak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-control-antidopaje-recogida-muestras-traves-del-personal-habilitado-agencia-vasca-antidopaje-periodo-2026-2027/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1049" s="22" t="n"/>
@@ -20242,7 +20410,7 @@
     <row r="1051" ht="30" customHeight="1">
       <c r="A1051" s="18" t="inlineStr">
         <is>
-          <t>FICHA 71: EUS-50992</t>
+          <t>FICHA 71: EUS-40531</t>
         </is>
       </c>
       <c r="B1051" s="19" t="n"/>
@@ -20267,7 +20435,7 @@
       <c r="E1052" s="22" t="n"/>
       <c r="F1052" s="22" t="n"/>
     </row>
-    <row r="1053" ht="45" customHeight="1">
+    <row r="1053" ht="20" customHeight="1">
       <c r="A1053" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -20275,7 +20443,7 @@
       </c>
       <c r="B1053" s="21" t="inlineStr">
         <is>
-          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el marco de la Intervención Sectorial Vitivinícola del Plan Estratégico (PEPAC) de la Política Agrícola Común de la UE 2023-2027</t>
+          <t>Reparación humedades en cubierta en el centro IES Angela Figuera BHI</t>
         </is>
       </c>
       <c r="C1053" s="22" t="n"/>
@@ -20291,7 +20459,7 @@
       </c>
       <c r="B1054" s="21" t="inlineStr">
         <is>
-          <t>EUS-50992</t>
+          <t>EUS-40531</t>
         </is>
       </c>
       <c r="C1054" s="22" t="n"/>
@@ -20367,7 +20535,7 @@
       </c>
       <c r="B1059" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C1059" s="22" t="n"/>
@@ -20443,7 +20611,7 @@
       </c>
       <c r="B1064" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/20260407mahastiardogintza/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/reparacion-humedades-cubierta-centro-ies-angela-figuera-bhi/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1064" s="22" t="n"/>
@@ -20454,7 +20622,7 @@
     <row r="1066" ht="30" customHeight="1">
       <c r="A1066" s="18" t="inlineStr">
         <is>
-          <t>FICHA 72: EUS-73686</t>
+          <t>FICHA 72: EUS-11190</t>
         </is>
       </c>
       <c r="B1066" s="19" t="n"/>
@@ -20479,7 +20647,7 @@
       <c r="E1067" s="22" t="n"/>
       <c r="F1067" s="22" t="n"/>
     </row>
-    <row r="1068" ht="20" customHeight="1">
+    <row r="1068" ht="45" customHeight="1">
       <c r="A1068" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -20487,7 +20655,7 @@
       </c>
       <c r="B1068" s="21" t="inlineStr">
         <is>
-          <t>Recogida de muestras de legionella mediante pcr en el acs de orbea</t>
+          <t>Reparación murete de cubierta fachada principal en el centro IES Antonio Trueba BHI (edificio Minería UE)</t>
         </is>
       </c>
       <c r="C1068" s="22" t="n"/>
@@ -20503,7 +20671,7 @@
       </c>
       <c r="B1069" s="21" t="inlineStr">
         <is>
-          <t>EUS-73686</t>
+          <t>EUS-11190</t>
         </is>
       </c>
       <c r="C1069" s="22" t="n"/>
@@ -20655,7 +20823,7 @@
       </c>
       <c r="B1079" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/recogida-muestras-legionella-mediante-pcr-acs-orbea/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/reparacion-murete-cubierta-fachada-principal-centro-ies-antonio-trueba-bhi-edificio-mineria-ue/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1079" s="22" t="n"/>
@@ -20666,7 +20834,7 @@
     <row r="1081" ht="30" customHeight="1">
       <c r="A1081" s="18" t="inlineStr">
         <is>
-          <t>FICHA 73: EUS-57575</t>
+          <t>FICHA 73: EUS-51778</t>
         </is>
       </c>
       <c r="B1081" s="19" t="n"/>
@@ -20691,7 +20859,7 @@
       <c r="E1082" s="22" t="n"/>
       <c r="F1082" s="22" t="n"/>
     </row>
-    <row r="1083" ht="20" customHeight="1">
+    <row r="1083" ht="45" customHeight="1">
       <c r="A1083" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -20699,7 +20867,7 @@
       </c>
       <c r="B1083" s="21" t="inlineStr">
         <is>
-          <t>Coffee break Vititransfer Laguardia</t>
+          <t>Gestión del programa Hiriko Udalekuak / Colonias Urbanas de Verano y Gabonetako Koloniak / Colonias de Navidad en 2026.</t>
         </is>
       </c>
       <c r="C1083" s="22" t="n"/>
@@ -20715,7 +20883,7 @@
       </c>
       <c r="B1084" s="21" t="inlineStr">
         <is>
-          <t>EUS-57575</t>
+          <t>EUS-51778</t>
         </is>
       </c>
       <c r="C1084" s="22" t="n"/>
@@ -20867,7 +21035,7 @@
       </c>
       <c r="B1094" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/coffee-break-vititransfer-laguardia/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/gestion-del-programa-hiriko-udalekuak-colonias-urbanas-verano-y-gabonetako-koloniak-colonias-navidad-2026/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1094" s="22" t="n"/>
@@ -20875,8 +21043,644 @@
       <c r="E1094" s="22" t="n"/>
       <c r="F1094" s="22" t="n"/>
     </row>
+    <row r="1096" ht="30" customHeight="1">
+      <c r="A1096" s="18" t="inlineStr">
+        <is>
+          <t>FICHA 74: EUS-15302</t>
+        </is>
+      </c>
+      <c r="B1096" s="19" t="n"/>
+      <c r="C1096" s="19" t="n"/>
+      <c r="D1096" s="19" t="n"/>
+      <c r="E1096" s="19" t="n"/>
+      <c r="F1096" s="19" t="n"/>
+    </row>
+    <row r="1097" ht="20" customHeight="1">
+      <c r="A1097" s="20" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1097" s="21" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1097" s="22" t="n"/>
+      <c r="D1097" s="22" t="n"/>
+      <c r="E1097" s="22" t="n"/>
+      <c r="F1097" s="22" t="n"/>
+    </row>
+    <row r="1098" ht="45" customHeight="1">
+      <c r="A1098" s="20" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1098" s="21" t="inlineStr">
+        <is>
+          <t>Contratacion Conjunta de servicio de seguridad y servicios auxiliares en diversos edificios del Gobierno Vasco</t>
+        </is>
+      </c>
+      <c r="C1098" s="22" t="n"/>
+      <c r="D1098" s="22" t="n"/>
+      <c r="E1098" s="22" t="n"/>
+      <c r="F1098" s="22" t="n"/>
+    </row>
+    <row r="1099" ht="20" customHeight="1">
+      <c r="A1099" s="20" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1099" s="21" t="inlineStr">
+        <is>
+          <t>EUS-15302</t>
+        </is>
+      </c>
+      <c r="C1099" s="22" t="n"/>
+      <c r="D1099" s="22" t="n"/>
+      <c r="E1099" s="22" t="n"/>
+      <c r="F1099" s="22" t="n"/>
+    </row>
+    <row r="1100" ht="20" customHeight="1">
+      <c r="A1100" s="20" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1100" s="21" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1100" s="22" t="n"/>
+      <c r="D1100" s="22" t="n"/>
+      <c r="E1100" s="22" t="n"/>
+      <c r="F1100" s="22" t="n"/>
+    </row>
+    <row r="1101" ht="20" customHeight="1">
+      <c r="A1101" s="20" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1101" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1101" s="22" t="n"/>
+      <c r="D1101" s="22" t="n"/>
+      <c r="E1101" s="22" t="n"/>
+      <c r="F1101" s="22" t="n"/>
+    </row>
+    <row r="1102" ht="20" customHeight="1">
+      <c r="A1102" s="20" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1102" s="21" t="inlineStr"/>
+      <c r="C1102" s="22" t="n"/>
+      <c r="D1102" s="22" t="n"/>
+      <c r="E1102" s="22" t="n"/>
+      <c r="F1102" s="22" t="n"/>
+    </row>
+    <row r="1103" ht="20" customHeight="1">
+      <c r="A1103" s="20" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1103" s="21" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1103" s="22" t="n"/>
+      <c r="D1103" s="22" t="n"/>
+      <c r="E1103" s="22" t="n"/>
+      <c r="F1103" s="22" t="n"/>
+    </row>
+    <row r="1104" ht="20" customHeight="1">
+      <c r="A1104" s="20" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1104" s="21" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1104" s="22" t="n"/>
+      <c r="D1104" s="22" t="n"/>
+      <c r="E1104" s="22" t="n"/>
+      <c r="F1104" s="22" t="n"/>
+    </row>
+    <row r="1105" ht="20" customHeight="1">
+      <c r="A1105" s="20" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1105" s="21" t="inlineStr"/>
+      <c r="C1105" s="22" t="n"/>
+      <c r="D1105" s="22" t="n"/>
+      <c r="E1105" s="22" t="n"/>
+      <c r="F1105" s="22" t="n"/>
+    </row>
+    <row r="1106" ht="20" customHeight="1">
+      <c r="A1106" s="20" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1106" s="21" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1106" s="22" t="n"/>
+      <c r="D1106" s="22" t="n"/>
+      <c r="E1106" s="22" t="n"/>
+      <c r="F1106" s="22" t="n"/>
+    </row>
+    <row r="1107" ht="20" customHeight="1">
+      <c r="A1107" s="20" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1107" s="21" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1107" s="22" t="n"/>
+      <c r="D1107" s="22" t="n"/>
+      <c r="E1107" s="22" t="n"/>
+      <c r="F1107" s="22" t="n"/>
+    </row>
+    <row r="1108" ht="20" customHeight="1">
+      <c r="A1108" s="20" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1108" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1108" s="22" t="n"/>
+      <c r="D1108" s="22" t="n"/>
+      <c r="E1108" s="22" t="n"/>
+      <c r="F1108" s="22" t="n"/>
+    </row>
+    <row r="1109" ht="45" customHeight="1">
+      <c r="A1109" s="20" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1109" s="23" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/contratacion-conjunta-servicio-seguridad-y-servicios-auxiliares-diversos-edificios-del-gobierno-vasco/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1109" s="22" t="n"/>
+      <c r="D1109" s="22" t="n"/>
+      <c r="E1109" s="22" t="n"/>
+      <c r="F1109" s="22" t="n"/>
+    </row>
+    <row r="1111" ht="30" customHeight="1">
+      <c r="A1111" s="18" t="inlineStr">
+        <is>
+          <t>FICHA 75: EUS-69233</t>
+        </is>
+      </c>
+      <c r="B1111" s="19" t="n"/>
+      <c r="C1111" s="19" t="n"/>
+      <c r="D1111" s="19" t="n"/>
+      <c r="E1111" s="19" t="n"/>
+      <c r="F1111" s="19" t="n"/>
+    </row>
+    <row r="1112" ht="20" customHeight="1">
+      <c r="A1112" s="20" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1112" s="21" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1112" s="22" t="n"/>
+      <c r="D1112" s="22" t="n"/>
+      <c r="E1112" s="22" t="n"/>
+      <c r="F1112" s="22" t="n"/>
+    </row>
+    <row r="1113" ht="45" customHeight="1">
+      <c r="A1113" s="20" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1113" s="21" t="inlineStr">
+        <is>
+          <t>Suministro y obra para instalación de la infraestructura de cuatro puntos de recarga de vehículos eléctricos</t>
+        </is>
+      </c>
+      <c r="C1113" s="22" t="n"/>
+      <c r="D1113" s="22" t="n"/>
+      <c r="E1113" s="22" t="n"/>
+      <c r="F1113" s="22" t="n"/>
+    </row>
+    <row r="1114" ht="20" customHeight="1">
+      <c r="A1114" s="20" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1114" s="21" t="inlineStr">
+        <is>
+          <t>EUS-69233</t>
+        </is>
+      </c>
+      <c r="C1114" s="22" t="n"/>
+      <c r="D1114" s="22" t="n"/>
+      <c r="E1114" s="22" t="n"/>
+      <c r="F1114" s="22" t="n"/>
+    </row>
+    <row r="1115" ht="20" customHeight="1">
+      <c r="A1115" s="20" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1115" s="21" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1115" s="22" t="n"/>
+      <c r="D1115" s="22" t="n"/>
+      <c r="E1115" s="22" t="n"/>
+      <c r="F1115" s="22" t="n"/>
+    </row>
+    <row r="1116" ht="20" customHeight="1">
+      <c r="A1116" s="20" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1116" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1116" s="22" t="n"/>
+      <c r="D1116" s="22" t="n"/>
+      <c r="E1116" s="22" t="n"/>
+      <c r="F1116" s="22" t="n"/>
+    </row>
+    <row r="1117" ht="20" customHeight="1">
+      <c r="A1117" s="20" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1117" s="21" t="inlineStr"/>
+      <c r="C1117" s="22" t="n"/>
+      <c r="D1117" s="22" t="n"/>
+      <c r="E1117" s="22" t="n"/>
+      <c r="F1117" s="22" t="n"/>
+    </row>
+    <row r="1118" ht="20" customHeight="1">
+      <c r="A1118" s="20" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1118" s="21" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1118" s="22" t="n"/>
+      <c r="D1118" s="22" t="n"/>
+      <c r="E1118" s="22" t="n"/>
+      <c r="F1118" s="22" t="n"/>
+    </row>
+    <row r="1119" ht="20" customHeight="1">
+      <c r="A1119" s="20" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1119" s="21" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1119" s="22" t="n"/>
+      <c r="D1119" s="22" t="n"/>
+      <c r="E1119" s="22" t="n"/>
+      <c r="F1119" s="22" t="n"/>
+    </row>
+    <row r="1120" ht="20" customHeight="1">
+      <c r="A1120" s="20" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1120" s="21" t="inlineStr"/>
+      <c r="C1120" s="22" t="n"/>
+      <c r="D1120" s="22" t="n"/>
+      <c r="E1120" s="22" t="n"/>
+      <c r="F1120" s="22" t="n"/>
+    </row>
+    <row r="1121" ht="20" customHeight="1">
+      <c r="A1121" s="20" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1121" s="21" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1121" s="22" t="n"/>
+      <c r="D1121" s="22" t="n"/>
+      <c r="E1121" s="22" t="n"/>
+      <c r="F1121" s="22" t="n"/>
+    </row>
+    <row r="1122" ht="20" customHeight="1">
+      <c r="A1122" s="20" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1122" s="21" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1122" s="22" t="n"/>
+      <c r="D1122" s="22" t="n"/>
+      <c r="E1122" s="22" t="n"/>
+      <c r="F1122" s="22" t="n"/>
+    </row>
+    <row r="1123" ht="20" customHeight="1">
+      <c r="A1123" s="20" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1123" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1123" s="22" t="n"/>
+      <c r="D1123" s="22" t="n"/>
+      <c r="E1123" s="22" t="n"/>
+      <c r="F1123" s="22" t="n"/>
+    </row>
+    <row r="1124" ht="45" customHeight="1">
+      <c r="A1124" s="20" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1124" s="23" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-y-obra-instalacion-infraestructura-cuatro-puntos-recarga-vehiculos-electricos/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1124" s="22" t="n"/>
+      <c r="D1124" s="22" t="n"/>
+      <c r="E1124" s="22" t="n"/>
+      <c r="F1124" s="22" t="n"/>
+    </row>
+    <row r="1126" ht="30" customHeight="1">
+      <c r="A1126" s="18" t="inlineStr">
+        <is>
+          <t>FICHA 76: EUS-38333</t>
+        </is>
+      </c>
+      <c r="B1126" s="19" t="n"/>
+      <c r="C1126" s="19" t="n"/>
+      <c r="D1126" s="19" t="n"/>
+      <c r="E1126" s="19" t="n"/>
+      <c r="F1126" s="19" t="n"/>
+    </row>
+    <row r="1127" ht="20" customHeight="1">
+      <c r="A1127" s="20" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1127" s="21" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1127" s="22" t="n"/>
+      <c r="D1127" s="22" t="n"/>
+      <c r="E1127" s="22" t="n"/>
+      <c r="F1127" s="22" t="n"/>
+    </row>
+    <row r="1128" ht="20" customHeight="1">
+      <c r="A1128" s="20" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1128" s="21" t="inlineStr">
+        <is>
+          <t>Recogida de muestras de legionella mediante pcr en el acs de orbea</t>
+        </is>
+      </c>
+      <c r="C1128" s="22" t="n"/>
+      <c r="D1128" s="22" t="n"/>
+      <c r="E1128" s="22" t="n"/>
+      <c r="F1128" s="22" t="n"/>
+    </row>
+    <row r="1129" ht="20" customHeight="1">
+      <c r="A1129" s="20" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1129" s="21" t="inlineStr">
+        <is>
+          <t>EUS-38333</t>
+        </is>
+      </c>
+      <c r="C1129" s="22" t="n"/>
+      <c r="D1129" s="22" t="n"/>
+      <c r="E1129" s="22" t="n"/>
+      <c r="F1129" s="22" t="n"/>
+    </row>
+    <row r="1130" ht="20" customHeight="1">
+      <c r="A1130" s="20" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1130" s="21" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1130" s="22" t="n"/>
+      <c r="D1130" s="22" t="n"/>
+      <c r="E1130" s="22" t="n"/>
+      <c r="F1130" s="22" t="n"/>
+    </row>
+    <row r="1131" ht="20" customHeight="1">
+      <c r="A1131" s="20" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1131" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1131" s="22" t="n"/>
+      <c r="D1131" s="22" t="n"/>
+      <c r="E1131" s="22" t="n"/>
+      <c r="F1131" s="22" t="n"/>
+    </row>
+    <row r="1132" ht="20" customHeight="1">
+      <c r="A1132" s="20" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1132" s="21" t="inlineStr"/>
+      <c r="C1132" s="22" t="n"/>
+      <c r="D1132" s="22" t="n"/>
+      <c r="E1132" s="22" t="n"/>
+      <c r="F1132" s="22" t="n"/>
+    </row>
+    <row r="1133" ht="20" customHeight="1">
+      <c r="A1133" s="20" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1133" s="21" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1133" s="22" t="n"/>
+      <c r="D1133" s="22" t="n"/>
+      <c r="E1133" s="22" t="n"/>
+      <c r="F1133" s="22" t="n"/>
+    </row>
+    <row r="1134" ht="20" customHeight="1">
+      <c r="A1134" s="20" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1134" s="21" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1134" s="22" t="n"/>
+      <c r="D1134" s="22" t="n"/>
+      <c r="E1134" s="22" t="n"/>
+      <c r="F1134" s="22" t="n"/>
+    </row>
+    <row r="1135" ht="20" customHeight="1">
+      <c r="A1135" s="20" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1135" s="21" t="inlineStr"/>
+      <c r="C1135" s="22" t="n"/>
+      <c r="D1135" s="22" t="n"/>
+      <c r="E1135" s="22" t="n"/>
+      <c r="F1135" s="22" t="n"/>
+    </row>
+    <row r="1136" ht="20" customHeight="1">
+      <c r="A1136" s="20" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1136" s="21" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1136" s="22" t="n"/>
+      <c r="D1136" s="22" t="n"/>
+      <c r="E1136" s="22" t="n"/>
+      <c r="F1136" s="22" t="n"/>
+    </row>
+    <row r="1137" ht="20" customHeight="1">
+      <c r="A1137" s="20" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1137" s="21" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1137" s="22" t="n"/>
+      <c r="D1137" s="22" t="n"/>
+      <c r="E1137" s="22" t="n"/>
+      <c r="F1137" s="22" t="n"/>
+    </row>
+    <row r="1138" ht="20" customHeight="1">
+      <c r="A1138" s="20" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1138" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1138" s="22" t="n"/>
+      <c r="D1138" s="22" t="n"/>
+      <c r="E1138" s="22" t="n"/>
+      <c r="F1138" s="22" t="n"/>
+    </row>
+    <row r="1139" ht="45" customHeight="1">
+      <c r="A1139" s="20" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1139" s="23" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/recogida-muestras-legionella-mediante-pcr-acs-orbea/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1139" s="22" t="n"/>
+      <c r="D1139" s="22" t="n"/>
+      <c r="E1139" s="22" t="n"/>
+      <c r="F1139" s="22" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="1022">
+  <mergeCells count="1064">
     <mergeCell ref="B679:F679"/>
     <mergeCell ref="B666:F666"/>
     <mergeCell ref="B964:F964"/>
@@ -20920,7 +21724,9 @@
     <mergeCell ref="B342:F342"/>
     <mergeCell ref="B578:F578"/>
     <mergeCell ref="A541:F541"/>
+    <mergeCell ref="B1099:F1099"/>
     <mergeCell ref="B515:F515"/>
+    <mergeCell ref="B1128:F1128"/>
     <mergeCell ref="A841:F841"/>
     <mergeCell ref="B158:F158"/>
     <mergeCell ref="B1094:F1094"/>
@@ -20929,6 +21735,7 @@
     <mergeCell ref="B894:F894"/>
     <mergeCell ref="B133:F133"/>
     <mergeCell ref="B959:F959"/>
+    <mergeCell ref="B1130:F1130"/>
     <mergeCell ref="B369:F369"/>
     <mergeCell ref="B667:F667"/>
     <mergeCell ref="B418:F418"/>
@@ -20955,11 +21762,13 @@
     <mergeCell ref="B662:F662"/>
     <mergeCell ref="B718:F718"/>
     <mergeCell ref="B889:F889"/>
+    <mergeCell ref="B1131:F1131"/>
     <mergeCell ref="B72:F72"/>
     <mergeCell ref="B954:F954"/>
     <mergeCell ref="B199:F199"/>
     <mergeCell ref="B370:F370"/>
     <mergeCell ref="B1025:F1025"/>
+    <mergeCell ref="B1112:F1112"/>
     <mergeCell ref="B291:F291"/>
     <mergeCell ref="B655:F655"/>
     <mergeCell ref="B974:F974"/>
@@ -21001,6 +21810,7 @@
     <mergeCell ref="B83:F83"/>
     <mergeCell ref="B254:F254"/>
     <mergeCell ref="B909:F909"/>
+    <mergeCell ref="B1105:F1105"/>
     <mergeCell ref="B319:F319"/>
     <mergeCell ref="B490:F490"/>
     <mergeCell ref="B604:F604"/>
@@ -21032,6 +21842,7 @@
     <mergeCell ref="B530:F530"/>
     <mergeCell ref="B726:F726"/>
     <mergeCell ref="B962:F962"/>
+    <mergeCell ref="B1133:F1133"/>
     <mergeCell ref="A886:F886"/>
     <mergeCell ref="B505:F505"/>
     <mergeCell ref="B1060:F1060"/>
@@ -21067,6 +21878,7 @@
     <mergeCell ref="B752:F752"/>
     <mergeCell ref="B1070:F1070"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B1115:F1115"/>
     <mergeCell ref="B325:F325"/>
     <mergeCell ref="B154:F154"/>
     <mergeCell ref="A271:F271"/>
@@ -21100,6 +21912,8 @@
     <mergeCell ref="B518:F518"/>
     <mergeCell ref="B562:F562"/>
     <mergeCell ref="B689:F689"/>
+    <mergeCell ref="B1121:F1121"/>
+    <mergeCell ref="B1123:F1123"/>
     <mergeCell ref="B86:F86"/>
     <mergeCell ref="B912:F912"/>
     <mergeCell ref="B1083:F1083"/>
@@ -21151,6 +21965,7 @@
     <mergeCell ref="B979:F979"/>
     <mergeCell ref="B381:F381"/>
     <mergeCell ref="B552:F552"/>
+    <mergeCell ref="A1111:F1111"/>
     <mergeCell ref="B1084:F1084"/>
     <mergeCell ref="A976:F976"/>
     <mergeCell ref="B170:F170"/>
@@ -21184,6 +21999,7 @@
     <mergeCell ref="B92:F92"/>
     <mergeCell ref="B984:F984"/>
     <mergeCell ref="A226:F226"/>
+    <mergeCell ref="B1124:F1124"/>
     <mergeCell ref="B394:F394"/>
     <mergeCell ref="B692:F692"/>
     <mergeCell ref="A931:F931"/>
@@ -21214,6 +22030,7 @@
     <mergeCell ref="B817:F817"/>
     <mergeCell ref="B944:F944"/>
     <mergeCell ref="B56:F56"/>
+    <mergeCell ref="B1102:F1102"/>
     <mergeCell ref="B43:F43"/>
     <mergeCell ref="B176:F176"/>
     <mergeCell ref="B347:F347"/>
@@ -21229,7 +22046,9 @@
     <mergeCell ref="B881:F881"/>
     <mergeCell ref="B1068:F1068"/>
     <mergeCell ref="B868:F868"/>
+    <mergeCell ref="B1117:F1117"/>
     <mergeCell ref="B107:F107"/>
+    <mergeCell ref="B1104:F1104"/>
     <mergeCell ref="B641:F641"/>
     <mergeCell ref="B57:F57"/>
     <mergeCell ref="B883:F883"/>
@@ -21255,6 +22074,7 @@
     <mergeCell ref="B999:F999"/>
     <mergeCell ref="B1061:F1061"/>
     <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B1097:F1097"/>
     <mergeCell ref="A46:F46"/>
     <mergeCell ref="B507:F507"/>
     <mergeCell ref="B62:F62"/>
@@ -21302,6 +22122,7 @@
     <mergeCell ref="B1018:F1018"/>
     <mergeCell ref="B624:F624"/>
     <mergeCell ref="B428:F428"/>
+    <mergeCell ref="B1118:F1118"/>
     <mergeCell ref="B284:F284"/>
     <mergeCell ref="B222:F222"/>
     <mergeCell ref="B344:F344"/>
@@ -21313,6 +22134,7 @@
     <mergeCell ref="B123:F123"/>
     <mergeCell ref="B949:F949"/>
     <mergeCell ref="B1011:F1011"/>
+    <mergeCell ref="B1120:F1120"/>
     <mergeCell ref="B50:F50"/>
     <mergeCell ref="B221:F221"/>
     <mergeCell ref="B110:F110"/>
@@ -21329,6 +22151,7 @@
     <mergeCell ref="B802:F802"/>
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B789:F789"/>
+    <mergeCell ref="B1136:F1136"/>
     <mergeCell ref="B248:F248"/>
     <mergeCell ref="B297:F297"/>
     <mergeCell ref="B813:F813"/>
@@ -21348,9 +22171,11 @@
     <mergeCell ref="B815:F815"/>
     <mergeCell ref="B597:F597"/>
     <mergeCell ref="B1064:F1064"/>
+    <mergeCell ref="B1113:F1113"/>
     <mergeCell ref="B103:F103"/>
     <mergeCell ref="B78:F78"/>
     <mergeCell ref="B833:F833"/>
+    <mergeCell ref="B1100:F1100"/>
     <mergeCell ref="B205:F205"/>
     <mergeCell ref="B339:F339"/>
     <mergeCell ref="B314:F314"/>
@@ -21446,6 +22271,7 @@
     <mergeCell ref="B305:F305"/>
     <mergeCell ref="B816:F816"/>
     <mergeCell ref="B918:F918"/>
+    <mergeCell ref="B1114:F1114"/>
     <mergeCell ref="B607:F607"/>
     <mergeCell ref="B663:F663"/>
     <mergeCell ref="B1049:F1049"/>
@@ -21456,6 +22282,7 @@
     <mergeCell ref="B442:F442"/>
     <mergeCell ref="B242:F242"/>
     <mergeCell ref="B880:F880"/>
+    <mergeCell ref="B1116:F1116"/>
     <mergeCell ref="B671:F671"/>
     <mergeCell ref="B969:F969"/>
     <mergeCell ref="B907:F907"/>
@@ -21473,12 +22300,15 @@
     <mergeCell ref="B760:F760"/>
     <mergeCell ref="B437:F437"/>
     <mergeCell ref="B852:F852"/>
+    <mergeCell ref="B1119:F1119"/>
     <mergeCell ref="B333:F333"/>
+    <mergeCell ref="B1098:F1098"/>
     <mergeCell ref="B898:F898"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="B520:F520"/>
     <mergeCell ref="B958:F958"/>
     <mergeCell ref="B308:F308"/>
+    <mergeCell ref="B1134:F1134"/>
     <mergeCell ref="B854:F854"/>
     <mergeCell ref="B99:F99"/>
     <mergeCell ref="B737:F737"/>
@@ -21497,12 +22327,14 @@
     <mergeCell ref="B372:F372"/>
     <mergeCell ref="B1071:F1071"/>
     <mergeCell ref="B608:F608"/>
+    <mergeCell ref="B1127:F1127"/>
     <mergeCell ref="B595:F595"/>
     <mergeCell ref="B1037:F1037"/>
     <mergeCell ref="B722:F722"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="A856:F856"/>
     <mergeCell ref="B893:F893"/>
+    <mergeCell ref="B1129:F1129"/>
     <mergeCell ref="B374:F374"/>
     <mergeCell ref="B659:F659"/>
     <mergeCell ref="B830:F830"/>
@@ -21571,6 +22403,7 @@
     <mergeCell ref="B309:F309"/>
     <mergeCell ref="A316:F316"/>
     <mergeCell ref="B380:F380"/>
+    <mergeCell ref="B1135:F1135"/>
     <mergeCell ref="A1081:F1081"/>
     <mergeCell ref="B100:F100"/>
     <mergeCell ref="B336:F336"/>
@@ -21580,10 +22413,12 @@
     <mergeCell ref="B140:F140"/>
     <mergeCell ref="B115:F115"/>
     <mergeCell ref="B382:F382"/>
+    <mergeCell ref="A1096:F1096"/>
     <mergeCell ref="B680:F680"/>
     <mergeCell ref="A376:F376"/>
     <mergeCell ref="B102:F102"/>
     <mergeCell ref="B674:F674"/>
+    <mergeCell ref="B1137:F1137"/>
     <mergeCell ref="B400:F400"/>
     <mergeCell ref="B698:F698"/>
     <mergeCell ref="B832:F832"/>
@@ -21596,6 +22431,7 @@
     <mergeCell ref="B598:F598"/>
     <mergeCell ref="B402:F402"/>
     <mergeCell ref="B669:F669"/>
+    <mergeCell ref="B1138:F1138"/>
     <mergeCell ref="B377:F377"/>
     <mergeCell ref="A451:F451"/>
     <mergeCell ref="B29:F29"/>
@@ -21802,11 +22638,14 @@
     <mergeCell ref="B409:F409"/>
     <mergeCell ref="B580:F580"/>
     <mergeCell ref="B920:F920"/>
+    <mergeCell ref="B1108:F1108"/>
     <mergeCell ref="B711:F711"/>
     <mergeCell ref="B1009:F1009"/>
     <mergeCell ref="B48:F48"/>
+    <mergeCell ref="B1101:F1101"/>
     <mergeCell ref="B582:F582"/>
     <mergeCell ref="B849:F849"/>
+    <mergeCell ref="B1132:F1132"/>
     <mergeCell ref="B73:F73"/>
     <mergeCell ref="B371:F371"/>
     <mergeCell ref="B638:F638"/>
@@ -21819,6 +22658,7 @@
     <mergeCell ref="A676:F676"/>
     <mergeCell ref="B137:F137"/>
     <mergeCell ref="B379:F379"/>
+    <mergeCell ref="B1106:F1106"/>
     <mergeCell ref="B702:F702"/>
     <mergeCell ref="B677:F677"/>
     <mergeCell ref="B640:F640"/>
@@ -21849,6 +22689,7 @@
     <mergeCell ref="B66:F66"/>
     <mergeCell ref="B326:F326"/>
     <mergeCell ref="B793:F793"/>
+    <mergeCell ref="B1103:F1103"/>
     <mergeCell ref="A406:F406"/>
     <mergeCell ref="B951:F951"/>
     <mergeCell ref="B130:F130"/>
@@ -21867,6 +22708,7 @@
     <mergeCell ref="B132:F132"/>
     <mergeCell ref="B425:F425"/>
     <mergeCell ref="B430:F430"/>
+    <mergeCell ref="B1107:F1107"/>
     <mergeCell ref="B1045:F1045"/>
     <mergeCell ref="B119:F119"/>
     <mergeCell ref="B290:F290"/>
@@ -21877,10 +22719,13 @@
     <mergeCell ref="B824:F824"/>
     <mergeCell ref="B1017:F1017"/>
     <mergeCell ref="B367:F367"/>
+    <mergeCell ref="B1122:F1122"/>
     <mergeCell ref="B427:F427"/>
+    <mergeCell ref="B1139:F1139"/>
     <mergeCell ref="B112:F112"/>
     <mergeCell ref="B283:F283"/>
     <mergeCell ref="B354:F354"/>
+    <mergeCell ref="B1109:F1109"/>
     <mergeCell ref="B348:F348"/>
     <mergeCell ref="B519:F519"/>
     <mergeCell ref="B419:F419"/>
@@ -21896,6 +22741,7 @@
     <mergeCell ref="B648:F648"/>
     <mergeCell ref="B64:F64"/>
     <mergeCell ref="B51:F51"/>
+    <mergeCell ref="A1126:F1126"/>
     <mergeCell ref="B443:F443"/>
     <mergeCell ref="A196:F196"/>
     <mergeCell ref="B237:F237"/>
@@ -21974,6 +22820,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1064" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1079" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1094" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1109" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1124" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1139" r:id="rId76"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -21985,7 +22834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J74"/>
+  <dimension ref="A1:J77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -22335,12 +23184,12 @@
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-04</t>
+          <t>HORIZON-CL5-2026-11-D3-23</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>De-risking renewable fuel technologies through transnational</t>
+          <t>Data sharing to support the training and development of AI f</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -22375,12 +23224,12 @@
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-05</t>
+          <t>HORIZON-CL5-2026-11-D3-06</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Demonstration of solid biofuel supply and conversion to high</t>
+          <t>Resource assessment for deep sedimentary and basement reserv</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -22415,12 +23264,12 @@
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-23</t>
+          <t>HORIZON-CL5-2026-11-D3-14</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Data sharing to support the training and development of AI f</t>
+          <t>Improved system design for innovative PV applications (EUPI-</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -22455,12 +23304,12 @@
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-06</t>
+          <t>HORIZON-CL5-2026-11-D3-05</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Resource assessment for deep sedimentary and basement reserv</t>
+          <t>Demonstration of solid biofuel supply and conversion to high</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -22495,12 +23344,12 @@
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-14</t>
+          <t>HORIZON-CL5-2026-11-D3-04</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Improved system design for innovative PV applications (EUPI-</t>
+          <t>De-risking renewable fuel technologies through transnational</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -22535,12 +23384,12 @@
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-16</t>
+          <t>HORIZON-CL5-2027-07-D3-27</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Industrial processes and equipment for innovative, reliable </t>
+          <t xml:space="preserve">Integrated Approaches for Retrofitting Infrastructures with </t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -22575,12 +23424,12 @@
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-11</t>
+          <t>HORIZON-CL5-2027-07-D3-26</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Demonstration of hydropower technologies for efficient and f</t>
+          <t>Advanced Distribution Management Systems (ADSM) for more eff</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -22655,12 +23504,12 @@
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-26</t>
+          <t>HORIZON-CL5-2027-07-D3-28</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Advanced Distribution Management Systems (ADSM) for more eff</t>
+          <t>Community of practice - Data-Driven Decision-Making in Energ</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -22695,12 +23544,12 @@
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-27</t>
+          <t>HORIZON-CL5-2027-07-D3-16</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Integrated Approaches for Retrofitting Infrastructures with </t>
+          <t xml:space="preserve">Industrial processes and equipment for innovative, reliable </t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -22735,12 +23584,12 @@
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-28</t>
+          <t>HORIZON-CL5-2027-07-D3-25</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Community of practice - Data-Driven Decision-Making in Energ</t>
+          <t>Advanced TSO control rooms to enhance grid observability, st</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -22775,12 +23624,12 @@
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-25</t>
+          <t>HORIZON-CL5-2027-07-D3-17</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Advanced TSO control rooms to enhance grid observability, st</t>
+          <t>PV based electrification of the economy: Designing &amp; optimis</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -22815,12 +23664,12 @@
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-17</t>
+          <t>HORIZON-CL5-2027-07-D3-11</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>PV based electrification of the economy: Designing &amp; optimis</t>
+          <t>Demonstration of hydropower technologies for efficient and f</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -22855,12 +23704,12 @@
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme</t>
+          <t>Palaeoclimate science for a better understanding of Earth sy</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -22975,12 +23824,12 @@
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform cl</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
@@ -23015,12 +23864,12 @@
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-08</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Palaeoclimate science for a better understanding of Earth sy</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
@@ -23055,12 +23904,12 @@
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Assessing the performance of policy instruments to inform cl</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
@@ -23095,12 +23944,12 @@
     <row r="28" ht="28" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Advancing understanding, modelling and prediction of extreme</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -23695,12 +24544,12 @@
     <row r="43" ht="28" customHeight="1">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-08</t>
+          <t>HORIZON-CL5-2027-02-D3-31</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Co-funding Strategic Energy Technology (SET) Plan renewable </t>
+          <t xml:space="preserve">Support to the implementation of an EU policy framework for </t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
@@ -23735,12 +24584,12 @@
     <row r="44" ht="28" customHeight="1">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-09</t>
+          <t>HORIZON-CL5-2027-02-D3-24</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>Innovative technologies and solutions to improve wave and ti</t>
+          <t>Large scale operational validation and upscaling of state-of</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
@@ -23815,12 +24664,12 @@
     <row r="46" ht="28" customHeight="1">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-24</t>
+          <t>HORIZON-CL5-2027-02-D3-15</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>Large scale operational validation and upscaling of state-of</t>
+          <t>Production technologies for solar photovoltaics beyond the s</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
@@ -23855,12 +24704,12 @@
     <row r="47" ht="28" customHeight="1">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-31</t>
+          <t>HORIZON-CL5-2027-02-D3-07</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support to the implementation of an EU policy framework for </t>
+          <t>Concentrated solar thermal systems for decarbonising industr</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
@@ -23895,12 +24744,12 @@
     <row r="48" ht="28" customHeight="1">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-15</t>
+          <t>HORIZON-CL5-2027-02-D3-08</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>Production technologies for solar photovoltaics beyond the s</t>
+          <t xml:space="preserve">Co-funding Strategic Energy Technology (SET) Plan renewable </t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
@@ -24507,7 +25356,7 @@
     <row r="66" ht="28" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>EUS-13454</t>
+          <t>EUS-41373</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
@@ -24543,7 +25392,7 @@
     <row r="67" ht="28" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>EUS-59353</t>
+          <t>EUS-68354</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
@@ -24579,12 +25428,12 @@
     <row r="68" ht="28" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>EUS-00407</t>
+          <t>EUS-84214</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>Ases. técnico diseño y plan de acción clima labora</t>
+          <t>Mantenimiento preventivo y correctivo de los equipos de clim</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -24615,12 +25464,12 @@
     <row r="69" ht="28" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>EUS-78654</t>
+          <t>EUS-43982</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>Plan de movilidad</t>
+          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta e</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -24636,7 +25485,7 @@
       <c r="E69" s="6" t="inlineStr"/>
       <c r="F69" s="27" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>MEDIA</t>
         </is>
       </c>
       <c r="G69" s="6" t="inlineStr"/>
@@ -24651,12 +25500,12 @@
     <row r="70" ht="28" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>EUS-15400</t>
+          <t>EUS-33357</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta e</t>
+          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversi</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -24687,12 +25536,12 @@
     <row r="71" ht="28" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>EUS-82152</t>
+          <t>EUS-05202</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>Redes de ciudades 2026. Sostenibilidad, cooperación, diversi</t>
+          <t>Servicio de control antidopaje (recogida de muestras) a trav</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -24723,12 +25572,12 @@
     <row r="72" ht="28" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>EUS-50992</t>
+          <t>EUS-40531</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>Ayudas de 2026 para la cosecha en verde de viñedos, en el ma</t>
+          <t>Reparación humedades en cubierta en el centro IES Angela Fig</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -24759,12 +25608,12 @@
     <row r="73" ht="28" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>EUS-73686</t>
+          <t>EUS-11190</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>Recogida de muestras de legionella mediante pcr en el acs de</t>
+          <t>Reparación murete de cubierta fachada principal en el centro</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -24795,12 +25644,12 @@
     <row r="74" ht="28" customHeight="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>EUS-57575</t>
+          <t>EUS-51778</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>Coffee break Vititransfer Laguardia</t>
+          <t xml:space="preserve">Gestión del programa Hiriko Udalekuak / Colonias Urbanas de </t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
@@ -24828,8 +25677,116 @@
       <c r="I74" s="6" t="inlineStr"/>
       <c r="J74" s="6" t="inlineStr"/>
     </row>
+    <row r="75" ht="28" customHeight="1">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>EUS-15302</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>Contratacion Conjunta de servicio de seguridad y servicios a</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D75" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E75" s="6" t="inlineStr"/>
+      <c r="F75" s="27" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G75" s="6" t="inlineStr"/>
+      <c r="H75" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I75" s="6" t="inlineStr"/>
+      <c r="J75" s="6" t="inlineStr"/>
+    </row>
+    <row r="76" ht="28" customHeight="1">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>EUS-69233</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Suministro y obra para instalación de la infraestructura de </t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E76" s="6" t="inlineStr"/>
+      <c r="F76" s="27" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G76" s="6" t="inlineStr"/>
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I76" s="6" t="inlineStr"/>
+      <c r="J76" s="6" t="inlineStr"/>
+    </row>
+    <row r="77" ht="28" customHeight="1">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>EUS-38333</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>Recogida de muestras de legionella mediante pcr en el acs de</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="inlineStr"/>
+      <c r="F77" s="27" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G77" s="6" t="inlineStr"/>
+      <c r="H77" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I77" s="6" t="inlineStr"/>
+      <c r="J77" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J74"/>
+  <autoFilter ref="A1:J77"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update funding data 2026-05-11
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Recursos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$80</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$77</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -679,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M80"/>
+  <dimension ref="A1:M83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -707,7 +707,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 10/05/2026 07:57 - 73 convocatorias - 11 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 11/05/2026 09:01 - 76 convocatorias - 14 nuevas</t>
         </is>
       </c>
     </row>
@@ -857,7 +857,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Security challenges of the green transition in urban und peri urban areas</t>
+          <t>Défis en matière de sécurité de la transition écologique dans les zones urbaines et périurbaines</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -897,7 +897,7 @@
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to some or all of the following outcomes:Identification and analysis of potential new security risks related to innovative technologies bein</t>
+          <t>Résultat escompté:On s&amp;#39;attend à ce que les résultats du projet contribuent à certains ou à la totalité des résultats suivants:Identification et analyse des nouveaux risques potentiels pour la sécu</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr"/>
@@ -1289,12 +1289,12 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-23</t>
+          <t>HORIZON-CL5-2026-11-D3-04</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Data sharing to support the training and development of AI foundation models in the energy sector</t>
+          <t>De-risking renewable fuel technologies through transnational pre-commercial procurement of renewable fuel industrial value chains</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>Innovation Actions</t>
+          <t>Pre-commercial Procurement</t>
         </is>
       </c>
       <c r="I14" s="10" t="inlineStr">
@@ -1334,7 +1334,7 @@
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Projects are expected to contribute to all the following expected outcomes:Effective and innovative methods for gathering, sharing and using large data sets in energy applications for</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Public authorities, industry, technology providers, energy producers and consumers profit from de-</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr"/>
@@ -1352,12 +1352,12 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-06</t>
+          <t>HORIZON-CL5-2026-11-D3-05</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Resource assessment for deep sedimentary and basement reservoirs</t>
+          <t>Demonstration of solid biofuel supply and conversion to high efficiency CHP from fully sustainable regional value chains</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Research and Innovation Actions</t>
+          <t>Innovation Actions</t>
         </is>
       </c>
       <c r="I15" s="10" t="inlineStr">
@@ -1397,7 +1397,7 @@
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Deep sedimentary/basement reservoirs are usually characterized by low permeability, high drilling cost and a scarcity of data, as they are typically ignored by hydrocarbon exploration</t>
+          <t>Expected Outcome:Fully sustainable regional bioenergy value chains and efficient conversion can play an important role in renewable efficient power and heating generation and for reaching the EU clima</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr"/>
@@ -1415,12 +1415,12 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-14</t>
+          <t>HORIZON-CL5-2026-11-D3-23</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Improved system design for innovative PV applications (EUPI-PV Partnership)</t>
+          <t>Data sharing to support the training and development of AI foundation models in the energy sector</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Agrivoltaics or the co-location of agricultural activity and PV electricity production is a novel form of PV deployment which could provide farmers with diversified revenue sources an</t>
+          <t>Expected Outcome:Projects are expected to contribute to all the following expected outcomes:Effective and innovative methods for gathering, sharing and using large data sets in energy applications for</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr"/>
@@ -1478,12 +1478,12 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-05</t>
+          <t>HORIZON-CL5-2026-11-D3-06</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Demonstration of solid biofuel supply and conversion to high efficiency CHP from fully sustainable regional value chains</t>
+          <t>Resource assessment for deep sedimentary and basement reservoirs</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>Innovation Actions</t>
+          <t xml:space="preserve"> Research and Innovation Actions</t>
         </is>
       </c>
       <c r="I17" s="10" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Fully sustainable regional bioenergy value chains and efficient conversion can play an important role in renewable efficient power and heating generation and for reaching the EU clima</t>
+          <t>Expected Outcome:Deep sedimentary/basement reservoirs are usually characterized by low permeability, high drilling cost and a scarcity of data, as they are typically ignored by hydrocarbon exploration</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr"/>
@@ -1541,12 +1541,12 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-04</t>
+          <t>HORIZON-CL5-2026-11-D3-14</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>De-risking renewable fuel technologies through transnational pre-commercial procurement of renewable fuel industrial value chains</t>
+          <t>Improved system design for innovative PV applications (EUPI-PV Partnership)</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -1571,7 +1571,7 @@
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>Pre-commercial Procurement</t>
+          <t>Innovation Actions</t>
         </is>
       </c>
       <c r="I18" s="10" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Public authorities, industry, technology providers, energy producers and consumers profit from de-</t>
+          <t>Expected Outcome:Agrivoltaics or the co-location of agricultural activity and PV electricity production is a novel form of PV deployment which could provide farmers with diversified revenue sources an</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr"/>
@@ -1604,12 +1604,12 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-27</t>
+          <t>HORIZON-CL5-2027-07-D3-16</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Integrated Approaches for Retrofitting Infrastructures with Innovative Energy Storage Technologies</t>
+          <t>Industrial processes and equipment for innovative, reliable and scalable tandem technologies (EUPI-PV Partnership)</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Improved energy security of the energy system by offering cost-effective and efficient solutions for </t>
+          <t>Expected Outcome:The REPowerEU plan and the EU Solar Energy Strategy introduced targets for the deployment of solar PV amounting to 600 GWac by 2030. Complying with these targets will be crucial for t</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr"/>
@@ -1667,12 +1667,12 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-26</t>
+          <t>HORIZON-CL5-2027-07-D3-11</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Advanced Distribution Management Systems (ADSM) for more efficient and flexible distribution grids</t>
+          <t>Demonstration of hydropower technologies for efficient and forward-looking refurbishment of existing hydropower plants</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced reliability, resilience, controllability and efficiency of electricity distribution grids. C</t>
+          <t>Expected Outcome:For a renewables-based electricity system sufficient flexible and also in the long-run fully sustainable hydropower capacity is pivotal.Project results are expected to contribute to a</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr"/>
@@ -1793,12 +1793,12 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-28</t>
+          <t>HORIZON-CL5-2027-07-D3-26</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Community of practice - Data-Driven Decision-Making in Energy</t>
+          <t>Advanced Distribution Management Systems (ADSM) for more efficient and flexible distribution grids</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>Coordination and Support Actions</t>
+          <t>Innovation Actions</t>
         </is>
       </c>
       <c r="I22" s="10" t="inlineStr">
@@ -1838,7 +1838,7 @@
       </c>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced EU cooperation to generate knowledge sharing on data and analytics used for the planning and</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced reliability, resilience, controllability and efficiency of electricity distribution grids. C</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr"/>
@@ -1856,12 +1856,12 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-16</t>
+          <t>HORIZON-CL5-2027-07-D3-27</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Industrial processes and equipment for innovative, reliable and scalable tandem technologies (EUPI-PV Partnership)</t>
+          <t>Integrated Approaches for Retrofitting Infrastructures with Innovative Energy Storage Technologies</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="K23" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:The REPowerEU plan and the EU Solar Energy Strategy introduced targets for the deployment of solar PV amounting to 600 GWac by 2030. Complying with these targets will be crucial for t</t>
+          <t xml:space="preserve">Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Improved energy security of the energy system by offering cost-effective and efficient solutions for </t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr"/>
@@ -1919,12 +1919,12 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-25</t>
+          <t>HORIZON-CL5-2027-07-D3-28</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Advanced TSO control rooms to enhance grid observability, stability and resilience</t>
+          <t>Community of practice - Data-Driven Decision-Making in Energy</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -1949,7 +1949,7 @@
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>Innovation Actions</t>
+          <t>Coordination and Support Actions</t>
         </is>
       </c>
       <c r="I24" s="10" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="K24" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced reliability, resilience, and efficiency of electricity transmission grids. Grid congestion i</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced EU cooperation to generate knowledge sharing on data and analytics used for the planning and</t>
         </is>
       </c>
       <c r="L24" s="6" t="inlineStr"/>
@@ -1982,12 +1982,12 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-17</t>
+          <t>HORIZON-CL5-2027-07-D3-25</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>PV based electrification of the economy: Designing &amp; optimising PV systems supporting industrial electrification and promoting participation in electricity markets (EUPI-PV Partnership)</t>
+          <t>Advanced TSO control rooms to enhance grid observability, stability and resilience</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -2027,7 +2027,7 @@
       </c>
       <c r="K25" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Large PV systems such as utility scale PV are evolving towards higher voltage architecture (&amp;gt;=3kV) with the objective to minimize losses and improve system efficiency at lower cost</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced reliability, resilience, and efficiency of electricity transmission grids. Grid congestion i</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr"/>
@@ -2045,12 +2045,12 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-11</t>
+          <t>HORIZON-CL5-2027-07-D3-17</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Demonstration of hydropower technologies for efficient and forward-looking refurbishment of existing hydropower plants</t>
+          <t>PV based electrification of the economy: Designing &amp; optimising PV systems supporting industrial electrification and promoting participation in electricity markets (EUPI-PV Partnership)</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -2090,7 +2090,7 @@
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:For a renewables-based electricity system sufficient flexible and also in the long-run fully sustainable hydropower capacity is pivotal.Project results are expected to contribute to a</t>
+          <t>Expected Outcome:Large PV systems such as utility scale PV are evolving towards higher voltage architecture (&amp;gt;=3kV) with the objective to minimize losses and improve system efficiency at lower cost</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr"/>
@@ -3242,12 +3242,12 @@
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-31</t>
+          <t>HORIZON-CL5-2027-02-D3-08</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>Support to the implementation of an EU policy framework for CO2 transport and storage infrastructure</t>
+          <t>Co-funding Strategic Energy Technology (SET) Plan renewable fuel value chains at EU, national, regional, and local level</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
@@ -3272,7 +3272,7 @@
       </c>
       <c r="H45" s="6" t="inlineStr">
         <is>
-          <t>Coordination and Support Actions</t>
+          <t>Programme Cofund Actions</t>
         </is>
       </c>
       <c r="I45" s="10" t="inlineStr">
@@ -3287,7 +3287,7 @@
       </c>
       <c r="K45" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to the following outcome:Stakeholders involved in the CO2 infrastructure network are in a position to implement the upcoming legislative fra</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Advance in the realisation of the Strategic Energy Technology (SET) Plan Action of Renewable fuels</t>
         </is>
       </c>
       <c r="L45" s="6" t="inlineStr"/>
@@ -3305,12 +3305,12 @@
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-24</t>
+          <t>HORIZON-CL5-2027-02-D3-09</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Large scale operational validation and upscaling of state-of-the-art (Generative) AI tools and models powering a next generation digital energy system</t>
+          <t>Innovative technologies and solutions to improve wave and tidal energy systems</t>
         </is>
       </c>
       <c r="D46" s="6" t="inlineStr">
@@ -3350,7 +3350,7 @@
       </c>
       <c r="K46" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Advanced, secure frugal (energy-, resource-, data- and cost-efficient, sustainable) AI tools for real</t>
+          <t>Expected Outcome:Project results are expected to contribute to all following expected outcomes:Advance in the realisation of the Strategic Energy Technology (SET) Plan’s research and innovation priori</t>
         </is>
       </c>
       <c r="L46" s="6" t="inlineStr"/>
@@ -3431,12 +3431,12 @@
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-15</t>
+          <t>HORIZON-CL5-2027-02-D3-24</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Production technologies for solar photovoltaics beyond the state-of-the-art (EUPI-PV Partnership)</t>
+          <t>Large scale operational validation and upscaling of state-of-the-art (Generative) AI tools and models powering a next generation digital energy system</t>
         </is>
       </c>
       <c r="D48" s="6" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="K48" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:The REPowerEU plan and the EU Solar Energy Strategy introduced targets for the deployment of solar PV amounting to 600 GWac by 2030. Complying with these targets will be crucial for t</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Advanced, secure frugal (energy-, resource-, data- and cost-efficient, sustainable) AI tools for real</t>
         </is>
       </c>
       <c r="L48" s="6" t="inlineStr"/>
@@ -3494,12 +3494,12 @@
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-07</t>
+          <t>HORIZON-CL5-2027-02-D3-31</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>Concentrated solar thermal systems for decarbonising industrial processes</t>
+          <t>Support to the implementation of an EU policy framework for CO2 transport and storage infrastructure</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
@@ -3524,7 +3524,7 @@
       </c>
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>Innovation Actions</t>
+          <t>Coordination and Support Actions</t>
         </is>
       </c>
       <c r="I49" s="10" t="inlineStr">
@@ -3539,7 +3539,7 @@
       </c>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Renewable heating can be directly used to efficiently decarbonise industrial processes. Concentrated solar thermal technologies offer a great potential to supply renewable heat for in</t>
+          <t>Expected Outcome:Project results are expected to contribute to the following outcome:Stakeholders involved in the CO2 infrastructure network are in a position to implement the upcoming legislative fra</t>
         </is>
       </c>
       <c r="L49" s="6" t="inlineStr"/>
@@ -3557,12 +3557,12 @@
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-08</t>
+          <t>HORIZON-CL5-2027-02-D3-15</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>Co-funding Strategic Energy Technology (SET) Plan renewable fuel value chains at EU, national, regional, and local level</t>
+          <t>Production technologies for solar photovoltaics beyond the state-of-the-art (EUPI-PV Partnership)</t>
         </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>Programme Cofund Actions</t>
+          <t>Innovation Actions</t>
         </is>
       </c>
       <c r="I50" s="10" t="inlineStr">
@@ -3602,7 +3602,7 @@
       </c>
       <c r="K50" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Advance in the realisation of the Strategic Energy Technology (SET) Plan Action of Renewable fuels</t>
+          <t>Expected Outcome:The REPowerEU plan and the EU Solar Energy Strategy introduced targets for the deployment of solar PV amounting to 600 GWac by 2030. Complying with these targets will be crucial for t</t>
         </is>
       </c>
       <c r="L50" s="6" t="inlineStr"/>
@@ -4473,7 +4473,7 @@
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>EUS-57677</t>
+          <t>EUS-97378</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -4528,7 +4528,7 @@
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>EUS-13853</t>
+          <t>EUS-04117</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -4583,7 +4583,7 @@
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>EUS-25004</t>
+          <t>EUS-87863</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -4638,7 +4638,7 @@
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>EUS-93927</t>
+          <t>EUS-85070</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -4693,12 +4693,12 @@
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>EUS-34980</t>
+          <t>EUS-86334</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>I+D.  Red Eureka, o programas financiados por el marco de innovación Horizon, como Eurostars (pymes) PRIMA (Mediterráneo) CETP (Energía) o DUT (Transformación Urbana). Evento del 12.05.26 sobre consor</t>
+          <t>Enajenación mediante subasta de diversos materiales que se encuentran en el almacén municipal para su achatarramiento y tratamiento como residuos sólidos urbanos</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr">
@@ -4715,12 +4715,12 @@
       <c r="G74" s="6" t="inlineStr"/>
       <c r="H74" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
-        </is>
-      </c>
-      <c r="I74" s="8" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I74" s="11" t="inlineStr">
+        <is>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="J74" s="6" t="inlineStr"/>
@@ -4748,12 +4748,12 @@
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>EUS-01747</t>
+          <t>EUS-05833</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>CEF-E. Línea de infraestructuras energéticas del Mecanismo Conectar Europa. Alineado con planes de Redes Transeuropeas (RTE-E) plan de choque anticrisis de la Unión de la Energía (AccelerateEU). Proye</t>
+          <t>I+D.  Red Eureka, o programas financiados por el marco de innovación Horizon, como Eurostars (pymes) PRIMA (Mediterráneo) CETP (Energía) o DUT (Transformación Urbana). Evento del 12.05.26 sobre consor</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
@@ -4803,12 +4803,12 @@
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>EUS-42478</t>
+          <t>EUS-20593</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta el 01.10.26. Cribado de enfermedades con inteligencia artificial. Espacio de Datos Sanitarios de la UE. Red de Centros para Seguridad de la I</t>
+          <t>CEF-E. Línea de infraestructuras energéticas del Mecanismo Conectar Europa. Alineado con planes de Redes Transeuropeas (RTE-E) plan de choque anticrisis de la Unión de la Energía (AccelerateEU). Proye</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr">
@@ -4858,12 +4858,12 @@
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>EUS-35761</t>
+          <t>EUS-82373</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>Suministro, implantación, mantenimiento, gestión y operación del nuevo servicio de bicicleta pública de Bizkaia BizkaiBizi</t>
+          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta el 01.10.26. Cribado de enfermedades con inteligencia artificial. Espacio de Datos Sanitarios de la UE. Red de Centros para Seguridad de la I</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
@@ -4880,7 +4880,7 @@
       <c r="G77" s="6" t="inlineStr"/>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="I77" s="8" t="inlineStr">
@@ -4913,12 +4913,12 @@
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>EUS-32315</t>
+          <t>EUS-56939</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>Servicio de transporte urbano de viajeros- experiencia piloto</t>
+          <t>Adquisición de paraguas corporativos del 90 aniversario del Gobierno Vasco</t>
         </is>
       </c>
       <c r="D78" s="6" t="inlineStr">
@@ -4968,12 +4968,12 @@
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>EUS-36844</t>
+          <t>EUS-37445</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>Prestación de servicios de apoyo a la secretaría técnica en el diseño, despliegue y seguimiento de la Estrategia para la Transformación Digital de Euskadi 2030.</t>
+          <t>Suministro, instalación y puesta en marcha de un conjunto de grupos electrógenos y depósitos auxiliares del sistema PEMEL de la red de saneamiento y abastecimiento de Aguas del Añarbe</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
@@ -5023,12 +5023,12 @@
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>EUS-88203</t>
+          <t>EUS-17618</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>Mantenimiento limpieza de la red de arquetas y tuberías de saneamiento en villamonte</t>
+          <t>Obras de reparación de la caldera en el colegio Mendiko</t>
         </is>
       </c>
       <c r="D80" s="6" t="inlineStr">
@@ -5070,8 +5070,173 @@
         </is>
       </c>
     </row>
+    <row r="81" ht="40" customHeight="1">
+      <c r="A81" s="16" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>EUS-83776</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>Suministro, instalación, puesta en marcha y mantenimiento de un sistema analítico para la determinación de la concentración de compuestos organohalogenados adsorbibles (AOX) en el laboratorio de contr</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F81" s="6" t="inlineStr"/>
+      <c r="G81" s="6" t="inlineStr"/>
+      <c r="H81" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I81" s="8" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J81" s="6" t="inlineStr"/>
+      <c r="K81" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L81" s="17" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M81" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="40" customHeight="1">
+      <c r="A82" s="16" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>EUS-27600</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>Gestión de incidencias en las viviendas dependientes de servicios sociales</t>
+        </is>
+      </c>
+      <c r="D82" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F82" s="6" t="inlineStr"/>
+      <c r="G82" s="6" t="inlineStr"/>
+      <c r="H82" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I82" s="8" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J82" s="6" t="inlineStr"/>
+      <c r="K82" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L82" s="17" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M82" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="40" customHeight="1">
+      <c r="A83" s="16" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>EUS-44604</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="inlineStr">
+        <is>
+          <t>Trabajos sobrevenidos de renovación integral de zonas verdes aledañas a rampas 1 y 2 bidezabal</t>
+        </is>
+      </c>
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E83" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F83" s="6" t="inlineStr"/>
+      <c r="G83" s="6" t="inlineStr"/>
+      <c r="H83" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I83" s="8" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J83" s="6" t="inlineStr"/>
+      <c r="K83" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L83" s="17" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M83" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:M80"/>
+  <autoFilter ref="A4:M83"/>
   <mergeCells count="5">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A5:M5"/>
@@ -5153,6 +5318,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M78" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M79" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M80" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M81" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M82" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M83" r:id="rId76"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5164,7 +5332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1094"/>
+  <dimension ref="A1:F1139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5419,7 +5587,7 @@
       <c r="E17" s="22" t="n"/>
       <c r="F17" s="22" t="n"/>
     </row>
-    <row r="18" ht="20" customHeight="1">
+    <row r="18" ht="45" customHeight="1">
       <c r="A18" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -5427,7 +5595,7 @@
       </c>
       <c r="B18" s="21" t="inlineStr">
         <is>
-          <t>Security challenges of the green transition in urban und peri urban areas</t>
+          <t>Défis en matière de sécurité de la transition écologique dans les zones urbaines et périurbaines</t>
         </is>
       </c>
       <c r="C18" s="22" t="n"/>
@@ -5555,7 +5723,7 @@
       </c>
       <c r="B26" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to some or all of the following outcomes:Identification and analysis of potential new security risks related to innovative technologies being deployed in the urban and peri-urban environments;Innovative and modern tools to identify and measure changes in urban and peri-urban areas caused by the green transition, insofar as they concern security and possible resilience approaches;Verification of measures countering potential safety and security risks, hazards and challenges arising in areas hosting green technologies;Contribution to bu</t>
+          <t>Résultat escompté:On s&amp;#39;attend à ce que les résultats du projet contribuent à certains ou à la totalité des résultats suivants:Identification et analyse des nouveaux risques potentiels pour la sécurité liés aux technologies innovantes déployées dans les environnements urbains et périurbains;des outils innovants et modernes pour identifier et mesurer les changements dans les zones urbaines et périurbaines causés par la transition écologique, dans la mesure où ils concernent la sécurité et les approches possibles en matière de résilience;la vérification des mesures de lutte contre les risques</t>
         </is>
       </c>
       <c r="C26" s="22" t="n"/>
@@ -6926,7 +7094,7 @@
     <row r="121" ht="30" customHeight="1">
       <c r="A121" s="18" t="inlineStr">
         <is>
-          <t>FICHA 9: HORIZON-CL5-2026-11-D3-23</t>
+          <t>FICHA 9: HORIZON-CL5-2026-11-D3-04</t>
         </is>
       </c>
       <c r="B121" s="19" t="n"/>
@@ -6959,7 +7127,7 @@
       </c>
       <c r="B123" s="21" t="inlineStr">
         <is>
-          <t>Data sharing to support the training and development of AI foundation models in the energy sector</t>
+          <t>De-risking renewable fuel technologies through transnational pre-commercial procurement of renewable fuel industrial value chains</t>
         </is>
       </c>
       <c r="C123" s="22" t="n"/>
@@ -6975,7 +7143,7 @@
       </c>
       <c r="B124" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-23</t>
+          <t>HORIZON-CL5-2026-11-D3-04</t>
         </is>
       </c>
       <c r="C124" s="22" t="n"/>
@@ -7055,7 +7223,7 @@
       </c>
       <c r="B129" s="21" t="inlineStr">
         <is>
-          <t>Innovation Actions</t>
+          <t>Pre-commercial Procurement</t>
         </is>
       </c>
       <c r="C129" s="22" t="n"/>
@@ -7087,7 +7255,7 @@
       </c>
       <c r="B131" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Projects are expected to contribute to all the following expected outcomes:Effective and innovative methods for gathering, sharing and using large data sets in energy applications for the purpose of training AI models while ensuring privacy and security.Advanced and - wherever possible - open-source AI foundation models to support the digitalisation of the energy system, through improved grid observability, forecasting of supply and demand, advanced storage and renewables integration, demand side flexibility and energy efficiency.Enhanced cooperation, knowledge sharing and int</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Public authorities, industry, technology providers, energy producers and consumers profit from de-risking of cost-effective essential value chains of those renewable fuel technologies that can contribute to domestic commercial fuel production beyond 2030 customized to their needs, from improved access to better financing exploiting synergies across funding schemes, and from more effective market uptake, business models, increased competitiveness, and commercialization opportunities.Energy prod</t>
         </is>
       </c>
       <c r="C131" s="22" t="n"/>
@@ -7131,7 +7299,7 @@
       </c>
       <c r="B134" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-23</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-04</t>
         </is>
       </c>
       <c r="C134" s="22" t="n"/>
@@ -7142,7 +7310,7 @@
     <row r="136" ht="30" customHeight="1">
       <c r="A136" s="18" t="inlineStr">
         <is>
-          <t>FICHA 10: HORIZON-CL5-2026-11-D3-06</t>
+          <t>FICHA 10: HORIZON-CL5-2026-11-D3-05</t>
         </is>
       </c>
       <c r="B136" s="19" t="n"/>
@@ -7167,7 +7335,7 @@
       <c r="E137" s="22" t="n"/>
       <c r="F137" s="22" t="n"/>
     </row>
-    <row r="138" ht="20" customHeight="1">
+    <row r="138" ht="45" customHeight="1">
       <c r="A138" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -7175,7 +7343,7 @@
       </c>
       <c r="B138" s="21" t="inlineStr">
         <is>
-          <t>Resource assessment for deep sedimentary and basement reservoirs</t>
+          <t>Demonstration of solid biofuel supply and conversion to high efficiency CHP from fully sustainable regional value chains</t>
         </is>
       </c>
       <c r="C138" s="22" t="n"/>
@@ -7191,7 +7359,7 @@
       </c>
       <c r="B139" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-06</t>
+          <t>HORIZON-CL5-2026-11-D3-05</t>
         </is>
       </c>
       <c r="C139" s="22" t="n"/>
@@ -7271,7 +7439,7 @@
       </c>
       <c r="B144" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Research and Innovation Actions</t>
+          <t>Innovation Actions</t>
         </is>
       </c>
       <c r="C144" s="22" t="n"/>
@@ -7303,7 +7471,7 @@
       </c>
       <c r="B146" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Deep sedimentary/basement reservoirs are usually characterized by low permeability, high drilling cost and a scarcity of data, as they are typically ignored by hydrocarbon exploration. Major exploration challenges relate to predicting deep sedimentary and basement reservoir structures and properties to identify suitable locations for reservoir-independent approaches, capable of overcoming the low permeability obstacle, such as Enhanced Geothermal Systems (EGS) or closed-loop geothermal systems.Project results are expected to contribute to all of the following expected outcomes</t>
+          <t>Expected Outcome:Fully sustainable regional bioenergy value chains and efficient conversion can play an important role in renewable efficient power and heating generation and for reaching the EU climate and energy targets and contribute to European competitiveness and energy security.Project results are expected to contribute to at all of the following expected outcomes:The demonstration of regional value chains for the use of locally to regionally sourced sustainable and cheap solid biofuel from upgraded biogenic residues and wastes in line with the provisions of the Renewable Energy Directiv</t>
         </is>
       </c>
       <c r="C146" s="22" t="n"/>
@@ -7347,7 +7515,7 @@
       </c>
       <c r="B149" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-06</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-05</t>
         </is>
       </c>
       <c r="C149" s="22" t="n"/>
@@ -7358,7 +7526,7 @@
     <row r="151" ht="30" customHeight="1">
       <c r="A151" s="18" t="inlineStr">
         <is>
-          <t>FICHA 11: HORIZON-CL5-2026-11-D3-14</t>
+          <t>FICHA 11: HORIZON-CL5-2026-11-D3-23</t>
         </is>
       </c>
       <c r="B151" s="19" t="n"/>
@@ -7383,7 +7551,7 @@
       <c r="E152" s="22" t="n"/>
       <c r="F152" s="22" t="n"/>
     </row>
-    <row r="153" ht="20" customHeight="1">
+    <row r="153" ht="45" customHeight="1">
       <c r="A153" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -7391,7 +7559,7 @@
       </c>
       <c r="B153" s="21" t="inlineStr">
         <is>
-          <t>Improved system design for innovative PV applications (EUPI-PV Partnership)</t>
+          <t>Data sharing to support the training and development of AI foundation models in the energy sector</t>
         </is>
       </c>
       <c r="C153" s="22" t="n"/>
@@ -7407,7 +7575,7 @@
       </c>
       <c r="B154" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-14</t>
+          <t>HORIZON-CL5-2026-11-D3-23</t>
         </is>
       </c>
       <c r="C154" s="22" t="n"/>
@@ -7519,7 +7687,7 @@
       </c>
       <c r="B161" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Agrivoltaics or the co-location of agricultural activity and PV electricity production is a novel form of PV deployment which could provide farmers with diversified revenue sources and ecological benefits, while reducing land use competition, siting restrictions or adverse impacts on biodiversity and agricultural production. Optimizing system designs and business practices will help to enable simultaneous land use creating synergy for both agriculture and electricity production; this can benefit farmers, lower PV costs and enable the European Union to reach the goals of the EU</t>
+          <t>Expected Outcome:Projects are expected to contribute to all the following expected outcomes:Effective and innovative methods for gathering, sharing and using large data sets in energy applications for the purpose of training AI models while ensuring privacy and security.Advanced and - wherever possible - open-source AI foundation models to support the digitalisation of the energy system, through improved grid observability, forecasting of supply and demand, advanced storage and renewables integration, demand side flexibility and energy efficiency.Enhanced cooperation, knowledge sharing and int</t>
         </is>
       </c>
       <c r="C161" s="22" t="n"/>
@@ -7563,7 +7731,7 @@
       </c>
       <c r="B164" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-14</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-23</t>
         </is>
       </c>
       <c r="C164" s="22" t="n"/>
@@ -7574,7 +7742,7 @@
     <row r="166" ht="30" customHeight="1">
       <c r="A166" s="18" t="inlineStr">
         <is>
-          <t>FICHA 12: HORIZON-CL5-2026-11-D3-05</t>
+          <t>FICHA 12: HORIZON-CL5-2026-11-D3-06</t>
         </is>
       </c>
       <c r="B166" s="19" t="n"/>
@@ -7599,7 +7767,7 @@
       <c r="E167" s="22" t="n"/>
       <c r="F167" s="22" t="n"/>
     </row>
-    <row r="168" ht="45" customHeight="1">
+    <row r="168" ht="20" customHeight="1">
       <c r="A168" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -7607,7 +7775,7 @@
       </c>
       <c r="B168" s="21" t="inlineStr">
         <is>
-          <t>Demonstration of solid biofuel supply and conversion to high efficiency CHP from fully sustainable regional value chains</t>
+          <t>Resource assessment for deep sedimentary and basement reservoirs</t>
         </is>
       </c>
       <c r="C168" s="22" t="n"/>
@@ -7623,7 +7791,7 @@
       </c>
       <c r="B169" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-05</t>
+          <t>HORIZON-CL5-2026-11-D3-06</t>
         </is>
       </c>
       <c r="C169" s="22" t="n"/>
@@ -7703,7 +7871,7 @@
       </c>
       <c r="B174" s="21" t="inlineStr">
         <is>
-          <t>Innovation Actions</t>
+          <t xml:space="preserve"> Research and Innovation Actions</t>
         </is>
       </c>
       <c r="C174" s="22" t="n"/>
@@ -7735,7 +7903,7 @@
       </c>
       <c r="B176" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Fully sustainable regional bioenergy value chains and efficient conversion can play an important role in renewable efficient power and heating generation and for reaching the EU climate and energy targets and contribute to European competitiveness and energy security.Project results are expected to contribute to at all of the following expected outcomes:The demonstration of regional value chains for the use of locally to regionally sourced sustainable and cheap solid biofuel from upgraded biogenic residues and wastes in line with the provisions of the Renewable Energy Directiv</t>
+          <t>Expected Outcome:Deep sedimentary/basement reservoirs are usually characterized by low permeability, high drilling cost and a scarcity of data, as they are typically ignored by hydrocarbon exploration. Major exploration challenges relate to predicting deep sedimentary and basement reservoir structures and properties to identify suitable locations for reservoir-independent approaches, capable of overcoming the low permeability obstacle, such as Enhanced Geothermal Systems (EGS) or closed-loop geothermal systems.Project results are expected to contribute to all of the following expected outcomes</t>
         </is>
       </c>
       <c r="C176" s="22" t="n"/>
@@ -7779,7 +7947,7 @@
       </c>
       <c r="B179" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-05</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-06</t>
         </is>
       </c>
       <c r="C179" s="22" t="n"/>
@@ -7790,7 +7958,7 @@
     <row r="181" ht="30" customHeight="1">
       <c r="A181" s="18" t="inlineStr">
         <is>
-          <t>FICHA 13: HORIZON-CL5-2026-11-D3-04</t>
+          <t>FICHA 13: HORIZON-CL5-2026-11-D3-14</t>
         </is>
       </c>
       <c r="B181" s="19" t="n"/>
@@ -7815,7 +7983,7 @@
       <c r="E182" s="22" t="n"/>
       <c r="F182" s="22" t="n"/>
     </row>
-    <row r="183" ht="45" customHeight="1">
+    <row r="183" ht="20" customHeight="1">
       <c r="A183" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -7823,7 +7991,7 @@
       </c>
       <c r="B183" s="21" t="inlineStr">
         <is>
-          <t>De-risking renewable fuel technologies through transnational pre-commercial procurement of renewable fuel industrial value chains</t>
+          <t>Improved system design for innovative PV applications (EUPI-PV Partnership)</t>
         </is>
       </c>
       <c r="C183" s="22" t="n"/>
@@ -7839,7 +8007,7 @@
       </c>
       <c r="B184" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-04</t>
+          <t>HORIZON-CL5-2026-11-D3-14</t>
         </is>
       </c>
       <c r="C184" s="22" t="n"/>
@@ -7919,7 +8087,7 @@
       </c>
       <c r="B189" s="21" t="inlineStr">
         <is>
-          <t>Pre-commercial Procurement</t>
+          <t>Innovation Actions</t>
         </is>
       </c>
       <c r="C189" s="22" t="n"/>
@@ -7951,7 +8119,7 @@
       </c>
       <c r="B191" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Public authorities, industry, technology providers, energy producers and consumers profit from de-risking of cost-effective essential value chains of those renewable fuel technologies that can contribute to domestic commercial fuel production beyond 2030 customized to their needs, from improved access to better financing exploiting synergies across funding schemes, and from more effective market uptake, business models, increased competitiveness, and commercialization opportunities.Energy prod</t>
+          <t>Expected Outcome:Agrivoltaics or the co-location of agricultural activity and PV electricity production is a novel form of PV deployment which could provide farmers with diversified revenue sources and ecological benefits, while reducing land use competition, siting restrictions or adverse impacts on biodiversity and agricultural production. Optimizing system designs and business practices will help to enable simultaneous land use creating synergy for both agriculture and electricity production; this can benefit farmers, lower PV costs and enable the European Union to reach the goals of the EU</t>
         </is>
       </c>
       <c r="C191" s="22" t="n"/>
@@ -7995,7 +8163,7 @@
       </c>
       <c r="B194" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-04</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-14</t>
         </is>
       </c>
       <c r="C194" s="22" t="n"/>
@@ -8006,7 +8174,7 @@
     <row r="196" ht="30" customHeight="1">
       <c r="A196" s="18" t="inlineStr">
         <is>
-          <t>FICHA 14: HORIZON-CL5-2027-07-D3-27</t>
+          <t>FICHA 14: HORIZON-CL5-2027-07-D3-16</t>
         </is>
       </c>
       <c r="B196" s="19" t="n"/>
@@ -8039,7 +8207,7 @@
       </c>
       <c r="B198" s="21" t="inlineStr">
         <is>
-          <t>Integrated Approaches for Retrofitting Infrastructures with Innovative Energy Storage Technologies</t>
+          <t>Industrial processes and equipment for innovative, reliable and scalable tandem technologies (EUPI-PV Partnership)</t>
         </is>
       </c>
       <c r="C198" s="22" t="n"/>
@@ -8055,7 +8223,7 @@
       </c>
       <c r="B199" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-27</t>
+          <t>HORIZON-CL5-2027-07-D3-16</t>
         </is>
       </c>
       <c r="C199" s="22" t="n"/>
@@ -8167,7 +8335,7 @@
       </c>
       <c r="B206" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Improved energy security of the energy system by offering cost-effective and efficient solutions for additional diverse and flexible energy storage capacities.Improve the sustainability and circularity of energy storage systems.Enhanced economic viability of energy storage by utilizing existing infrastructures.  Scope:Demonstration of novel or improved technological solutions for cost-efficient, circular and sustainable energy storage, which contribute to grid flexibility and make use of existing</t>
+          <t>Expected Outcome:The REPowerEU plan and the EU Solar Energy Strategy introduced targets for the deployment of solar PV amounting to 600 GWac by 2030. Complying with these targets will be crucial for the European Union to reach its climate targets and free itself from import dependency on fossil fuels and the costs this imposes on Europe’s competitiveness in terms of high energy prices. The Solar Strategy also introduces a target, which has been enshrined into the Net-Zero Industry Act, to re-consolidate the European solar manufacturing sector and scale up European manufacturing capacity across</t>
         </is>
       </c>
       <c r="C206" s="22" t="n"/>
@@ -8211,7 +8379,7 @@
       </c>
       <c r="B209" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-27</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-16</t>
         </is>
       </c>
       <c r="C209" s="22" t="n"/>
@@ -8222,7 +8390,7 @@
     <row r="211" ht="30" customHeight="1">
       <c r="A211" s="18" t="inlineStr">
         <is>
-          <t>FICHA 15: HORIZON-CL5-2027-07-D3-26</t>
+          <t>FICHA 15: HORIZON-CL5-2027-07-D3-11</t>
         </is>
       </c>
       <c r="B211" s="19" t="n"/>
@@ -8255,7 +8423,7 @@
       </c>
       <c r="B213" s="21" t="inlineStr">
         <is>
-          <t>Advanced Distribution Management Systems (ADSM) for more efficient and flexible distribution grids</t>
+          <t>Demonstration of hydropower technologies for efficient and forward-looking refurbishment of existing hydropower plants</t>
         </is>
       </c>
       <c r="C213" s="22" t="n"/>
@@ -8271,7 +8439,7 @@
       </c>
       <c r="B214" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-26</t>
+          <t>HORIZON-CL5-2027-07-D3-11</t>
         </is>
       </c>
       <c r="C214" s="22" t="n"/>
@@ -8383,7 +8551,7 @@
       </c>
       <c r="B221" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced reliability, resilience, controllability and efficiency of electricity distribution grids. Congestion in distribution grids is managed effectively;Distribution system operators (DSO) leverage modern digital solutions and employ improved systems to effectively manage their grids and improve interoperability with TSOs and other DSOs;Vendor-agnostic reference architectures, solutions and tools are developed to help advancing the ADSM design and operation and effectively manage a broad range</t>
+          <t>Expected Outcome:For a renewables-based electricity system sufficient flexible and also in the long-run fully sustainable hydropower capacity is pivotal.Project results are expected to contribute to all of the following expected outcomes:Enhancing the capacities of the hydropower fleet to contribute with variable renewables base load to a secure and stable electricity system, including by modernising grid integration and hydropower fleet control.Increase technology leadership, competitiveness and technology export potential of European hydropower industry.Address challenges of climate change a</t>
         </is>
       </c>
       <c r="C221" s="22" t="n"/>
@@ -8427,7 +8595,7 @@
       </c>
       <c r="B224" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-26</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-11</t>
         </is>
       </c>
       <c r="C224" s="22" t="n"/>
@@ -8654,7 +8822,7 @@
     <row r="241" ht="30" customHeight="1">
       <c r="A241" s="18" t="inlineStr">
         <is>
-          <t>FICHA 17: HORIZON-CL5-2027-07-D3-28</t>
+          <t>FICHA 17: HORIZON-CL5-2027-07-D3-26</t>
         </is>
       </c>
       <c r="B241" s="19" t="n"/>
@@ -8679,7 +8847,7 @@
       <c r="E242" s="22" t="n"/>
       <c r="F242" s="22" t="n"/>
     </row>
-    <row r="243" ht="20" customHeight="1">
+    <row r="243" ht="45" customHeight="1">
       <c r="A243" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -8687,7 +8855,7 @@
       </c>
       <c r="B243" s="21" t="inlineStr">
         <is>
-          <t>Community of practice - Data-Driven Decision-Making in Energy</t>
+          <t>Advanced Distribution Management Systems (ADSM) for more efficient and flexible distribution grids</t>
         </is>
       </c>
       <c r="C243" s="22" t="n"/>
@@ -8703,7 +8871,7 @@
       </c>
       <c r="B244" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-28</t>
+          <t>HORIZON-CL5-2027-07-D3-26</t>
         </is>
       </c>
       <c r="C244" s="22" t="n"/>
@@ -8783,7 +8951,7 @@
       </c>
       <c r="B249" s="21" t="inlineStr">
         <is>
-          <t>Coordination and Support Actions</t>
+          <t>Innovation Actions</t>
         </is>
       </c>
       <c r="C249" s="22" t="n"/>
@@ -8815,7 +8983,7 @@
       </c>
       <c r="B251" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced EU cooperation to generate knowledge sharing on data and analytics used for the planning and operation of European grids, and market integration;Better EU coordination with regard to planning and simulation tools to support the development of electricity grids and integration of RES are made available to the research, academia, grid operators, and key actors in the energy value chains;Coordinated processes to generate new and innovative open-source solutions, software modules etc. that a</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced reliability, resilience, controllability and efficiency of electricity distribution grids. Congestion in distribution grids is managed effectively;Distribution system operators (DSO) leverage modern digital solutions and employ improved systems to effectively manage their grids and improve interoperability with TSOs and other DSOs;Vendor-agnostic reference architectures, solutions and tools are developed to help advancing the ADSM design and operation and effectively manage a broad range</t>
         </is>
       </c>
       <c r="C251" s="22" t="n"/>
@@ -8859,7 +9027,7 @@
       </c>
       <c r="B254" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-28</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-26</t>
         </is>
       </c>
       <c r="C254" s="22" t="n"/>
@@ -8870,7 +9038,7 @@
     <row r="256" ht="30" customHeight="1">
       <c r="A256" s="18" t="inlineStr">
         <is>
-          <t>FICHA 18: HORIZON-CL5-2027-07-D3-16</t>
+          <t>FICHA 18: HORIZON-CL5-2027-07-D3-27</t>
         </is>
       </c>
       <c r="B256" s="19" t="n"/>
@@ -8903,7 +9071,7 @@
       </c>
       <c r="B258" s="21" t="inlineStr">
         <is>
-          <t>Industrial processes and equipment for innovative, reliable and scalable tandem technologies (EUPI-PV Partnership)</t>
+          <t>Integrated Approaches for Retrofitting Infrastructures with Innovative Energy Storage Technologies</t>
         </is>
       </c>
       <c r="C258" s="22" t="n"/>
@@ -8919,7 +9087,7 @@
       </c>
       <c r="B259" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-16</t>
+          <t>HORIZON-CL5-2027-07-D3-27</t>
         </is>
       </c>
       <c r="C259" s="22" t="n"/>
@@ -9031,7 +9199,7 @@
       </c>
       <c r="B266" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:The REPowerEU plan and the EU Solar Energy Strategy introduced targets for the deployment of solar PV amounting to 600 GWac by 2030. Complying with these targets will be crucial for the European Union to reach its climate targets and free itself from import dependency on fossil fuels and the costs this imposes on Europe’s competitiveness in terms of high energy prices. The Solar Strategy also introduces a target, which has been enshrined into the Net-Zero Industry Act, to re-consolidate the European solar manufacturing sector and scale up European manufacturing capacity across</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Improved energy security of the energy system by offering cost-effective and efficient solutions for additional diverse and flexible energy storage capacities.Improve the sustainability and circularity of energy storage systems.Enhanced economic viability of energy storage by utilizing existing infrastructures.  Scope:Demonstration of novel or improved technological solutions for cost-efficient, circular and sustainable energy storage, which contribute to grid flexibility and make use of existing</t>
         </is>
       </c>
       <c r="C266" s="22" t="n"/>
@@ -9075,7 +9243,7 @@
       </c>
       <c r="B269" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-16</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-27</t>
         </is>
       </c>
       <c r="C269" s="22" t="n"/>
@@ -9086,7 +9254,7 @@
     <row r="271" ht="30" customHeight="1">
       <c r="A271" s="18" t="inlineStr">
         <is>
-          <t>FICHA 19: HORIZON-CL5-2027-07-D3-25</t>
+          <t>FICHA 19: HORIZON-CL5-2027-07-D3-28</t>
         </is>
       </c>
       <c r="B271" s="19" t="n"/>
@@ -9111,7 +9279,7 @@
       <c r="E272" s="22" t="n"/>
       <c r="F272" s="22" t="n"/>
     </row>
-    <row r="273" ht="45" customHeight="1">
+    <row r="273" ht="20" customHeight="1">
       <c r="A273" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -9119,7 +9287,7 @@
       </c>
       <c r="B273" s="21" t="inlineStr">
         <is>
-          <t>Advanced TSO control rooms to enhance grid observability, stability and resilience</t>
+          <t>Community of practice - Data-Driven Decision-Making in Energy</t>
         </is>
       </c>
       <c r="C273" s="22" t="n"/>
@@ -9135,7 +9303,7 @@
       </c>
       <c r="B274" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-25</t>
+          <t>HORIZON-CL5-2027-07-D3-28</t>
         </is>
       </c>
       <c r="C274" s="22" t="n"/>
@@ -9215,7 +9383,7 @@
       </c>
       <c r="B279" s="21" t="inlineStr">
         <is>
-          <t>Innovation Actions</t>
+          <t>Coordination and Support Actions</t>
         </is>
       </c>
       <c r="C279" s="22" t="n"/>
@@ -9247,7 +9415,7 @@
       </c>
       <c r="B281" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced reliability, resilience, and efficiency of electricity transmission grids. Grid congestion is managed efficiently;Enhanced observability of grids and improved forecasting of supply, demand, grid capacity availability, and flexibility;Transmission system operators (TSO) leverage modern digital solutions and employ improved systems to effectively manage their grids and improve interoperability with other TSOs;Vendor-agnostic reference architectures, solutions and tools are developed to hel</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced EU cooperation to generate knowledge sharing on data and analytics used for the planning and operation of European grids, and market integration;Better EU coordination with regard to planning and simulation tools to support the development of electricity grids and integration of RES are made available to the research, academia, grid operators, and key actors in the energy value chains;Coordinated processes to generate new and innovative open-source solutions, software modules etc. that a</t>
         </is>
       </c>
       <c r="C281" s="22" t="n"/>
@@ -9291,7 +9459,7 @@
       </c>
       <c r="B284" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-25</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-28</t>
         </is>
       </c>
       <c r="C284" s="22" t="n"/>
@@ -9302,7 +9470,7 @@
     <row r="286" ht="30" customHeight="1">
       <c r="A286" s="18" t="inlineStr">
         <is>
-          <t>FICHA 20: HORIZON-CL5-2027-07-D3-17</t>
+          <t>FICHA 20: HORIZON-CL5-2027-07-D3-25</t>
         </is>
       </c>
       <c r="B286" s="19" t="n"/>
@@ -9335,7 +9503,7 @@
       </c>
       <c r="B288" s="21" t="inlineStr">
         <is>
-          <t>PV based electrification of the economy: Designing &amp; optimising PV systems supporting industrial electrification and promoting participation in electricity markets (EUPI-PV Partnership)</t>
+          <t>Advanced TSO control rooms to enhance grid observability, stability and resilience</t>
         </is>
       </c>
       <c r="C288" s="22" t="n"/>
@@ -9351,7 +9519,7 @@
       </c>
       <c r="B289" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-17</t>
+          <t>HORIZON-CL5-2027-07-D3-25</t>
         </is>
       </c>
       <c r="C289" s="22" t="n"/>
@@ -9463,7 +9631,7 @@
       </c>
       <c r="B296" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Large PV systems such as utility scale PV are evolving towards higher voltage architecture (&amp;gt;=3kV) with the objective to minimize losses and improve system efficiency at lower costs. The intention is to integrate also storage into such (hybrid) PV systems offering flexibility. It is consequently essential to build a blueprint for the implementation of high voltage large PV systems and the development of Direct Current (DC) networks around strategic end users for high voltage demand (industrial sites, servers, electric vehicle charging stations…). Understanding the factors t</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced reliability, resilience, and efficiency of electricity transmission grids. Grid congestion is managed efficiently;Enhanced observability of grids and improved forecasting of supply, demand, grid capacity availability, and flexibility;Transmission system operators (TSO) leverage modern digital solutions and employ improved systems to effectively manage their grids and improve interoperability with other TSOs;Vendor-agnostic reference architectures, solutions and tools are developed to hel</t>
         </is>
       </c>
       <c r="C296" s="22" t="n"/>
@@ -9507,7 +9675,7 @@
       </c>
       <c r="B299" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-17</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-25</t>
         </is>
       </c>
       <c r="C299" s="22" t="n"/>
@@ -9518,7 +9686,7 @@
     <row r="301" ht="30" customHeight="1">
       <c r="A301" s="18" t="inlineStr">
         <is>
-          <t>FICHA 21: HORIZON-CL5-2027-07-D3-11</t>
+          <t>FICHA 21: HORIZON-CL5-2027-07-D3-17</t>
         </is>
       </c>
       <c r="B301" s="19" t="n"/>
@@ -9551,7 +9719,7 @@
       </c>
       <c r="B303" s="21" t="inlineStr">
         <is>
-          <t>Demonstration of hydropower technologies for efficient and forward-looking refurbishment of existing hydropower plants</t>
+          <t>PV based electrification of the economy: Designing &amp; optimising PV systems supporting industrial electrification and promoting participation in electricity markets (EUPI-PV Partnership)</t>
         </is>
       </c>
       <c r="C303" s="22" t="n"/>
@@ -9567,7 +9735,7 @@
       </c>
       <c r="B304" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-11</t>
+          <t>HORIZON-CL5-2027-07-D3-17</t>
         </is>
       </c>
       <c r="C304" s="22" t="n"/>
@@ -9679,7 +9847,7 @@
       </c>
       <c r="B311" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:For a renewables-based electricity system sufficient flexible and also in the long-run fully sustainable hydropower capacity is pivotal.Project results are expected to contribute to all of the following expected outcomes:Enhancing the capacities of the hydropower fleet to contribute with variable renewables base load to a secure and stable electricity system, including by modernising grid integration and hydropower fleet control.Increase technology leadership, competitiveness and technology export potential of European hydropower industry.Address challenges of climate change a</t>
+          <t>Expected Outcome:Large PV systems such as utility scale PV are evolving towards higher voltage architecture (&amp;gt;=3kV) with the objective to minimize losses and improve system efficiency at lower costs. The intention is to integrate also storage into such (hybrid) PV systems offering flexibility. It is consequently essential to build a blueprint for the implementation of high voltage large PV systems and the development of Direct Current (DC) networks around strategic end users for high voltage demand (industrial sites, servers, electric vehicle charging stations…). Understanding the factors t</t>
         </is>
       </c>
       <c r="C311" s="22" t="n"/>
@@ -9723,7 +9891,7 @@
       </c>
       <c r="B314" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-11</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-17</t>
         </is>
       </c>
       <c r="C314" s="22" t="n"/>
@@ -13666,7 +13834,7 @@
     <row r="586" ht="30" customHeight="1">
       <c r="A586" s="18" t="inlineStr">
         <is>
-          <t>FICHA 40: HORIZON-CL5-2027-02-D3-31</t>
+          <t>FICHA 40: HORIZON-CL5-2027-02-D3-08</t>
         </is>
       </c>
       <c r="B586" s="19" t="n"/>
@@ -13699,7 +13867,7 @@
       </c>
       <c r="B588" s="21" t="inlineStr">
         <is>
-          <t>Support to the implementation of an EU policy framework for CO2 transport and storage infrastructure</t>
+          <t>Co-funding Strategic Energy Technology (SET) Plan renewable fuel value chains at EU, national, regional, and local level</t>
         </is>
       </c>
       <c r="C588" s="22" t="n"/>
@@ -13715,7 +13883,7 @@
       </c>
       <c r="B589" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-31</t>
+          <t>HORIZON-CL5-2027-02-D3-08</t>
         </is>
       </c>
       <c r="C589" s="22" t="n"/>
@@ -13795,7 +13963,7 @@
       </c>
       <c r="B594" s="21" t="inlineStr">
         <is>
-          <t>Coordination and Support Actions</t>
+          <t>Programme Cofund Actions</t>
         </is>
       </c>
       <c r="C594" s="22" t="n"/>
@@ -13827,7 +13995,7 @@
       </c>
       <c r="B596" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to the following outcome:Stakeholders involved in the CO2 infrastructure network are in a position to implement the upcoming legislative framework for CO2 infrastructure.  Scope:The project is expected to assist stakeholders involved in the CO2 infrastructure network in implementing the upcoming legislative framework for CO2 infrastructure.Issues to address include market and cost structure, cross-border integration, interoperability and planning, technical harmonisation and investment incentives for new infrastructure, third-party ac</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Advance in the realisation of the Strategic Energy Technology (SET) Plan Action of Renewable fuels and Bioenergy (for the fuels part) is supported, overcoming fragmentation by mobilizing resources and establishing across EU interregional value chains of renewable fuel technologies and by better alignment of public and private R&amp;amp;I priorities and of funding mechanisms.All sector stakeholders benefit from establishment of renewable fuels value chains at EU, national, regional, and local level</t>
         </is>
       </c>
       <c r="C596" s="22" t="n"/>
@@ -13871,7 +14039,7 @@
       </c>
       <c r="B599" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-31</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-08</t>
         </is>
       </c>
       <c r="C599" s="22" t="n"/>
@@ -13882,7 +14050,7 @@
     <row r="601" ht="30" customHeight="1">
       <c r="A601" s="18" t="inlineStr">
         <is>
-          <t>FICHA 41: HORIZON-CL5-2027-02-D3-24</t>
+          <t>FICHA 41: HORIZON-CL5-2027-02-D3-09</t>
         </is>
       </c>
       <c r="B601" s="19" t="n"/>
@@ -13907,7 +14075,7 @@
       <c r="E602" s="22" t="n"/>
       <c r="F602" s="22" t="n"/>
     </row>
-    <row r="603" ht="45" customHeight="1">
+    <row r="603" ht="20" customHeight="1">
       <c r="A603" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -13915,7 +14083,7 @@
       </c>
       <c r="B603" s="21" t="inlineStr">
         <is>
-          <t>Large scale operational validation and upscaling of state-of-the-art (Generative) AI tools and models powering a next generation digital energy system</t>
+          <t>Innovative technologies and solutions to improve wave and tidal energy systems</t>
         </is>
       </c>
       <c r="C603" s="22" t="n"/>
@@ -13931,7 +14099,7 @@
       </c>
       <c r="B604" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-24</t>
+          <t>HORIZON-CL5-2027-02-D3-09</t>
         </is>
       </c>
       <c r="C604" s="22" t="n"/>
@@ -14043,7 +14211,7 @@
       </c>
       <c r="B611" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Advanced, secure frugal (energy-, resource-, data- and cost-efficient, sustainable) AI tools for real-time grid operations (including protection), market operations (if relevant) and consumer empowerment in distributed energy systems.A demonstrated AI development environment integrated with the upgraded digital spine of the energy system and energy-saving consumer applications.Scaled-up capabilities for learning at edge nodes and federated systems using agent-based architectures.A governance fram</t>
+          <t>Expected Outcome:Project results are expected to contribute to all following expected outcomes:Advance in the realisation of the Strategic Energy Technology (SET) Plan’s research and innovation priorities and targets for ocean energy;Energy producers and consumers benefit from increased performance of wave and tidal energy technologies with the focus on efficiency and flexibility, reduced cost, improved reliability and sustainability, operation and maintenance, robustness and security during all stages of the lifetime of an ocean energy farm from installation, operation and maintenance to deco</t>
         </is>
       </c>
       <c r="C611" s="22" t="n"/>
@@ -14087,7 +14255,7 @@
       </c>
       <c r="B614" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-24</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-09</t>
         </is>
       </c>
       <c r="C614" s="22" t="n"/>
@@ -14314,7 +14482,7 @@
     <row r="631" ht="30" customHeight="1">
       <c r="A631" s="18" t="inlineStr">
         <is>
-          <t>FICHA 43: HORIZON-CL5-2027-02-D3-15</t>
+          <t>FICHA 43: HORIZON-CL5-2027-02-D3-24</t>
         </is>
       </c>
       <c r="B631" s="19" t="n"/>
@@ -14347,7 +14515,7 @@
       </c>
       <c r="B633" s="21" t="inlineStr">
         <is>
-          <t>Production technologies for solar photovoltaics beyond the state-of-the-art (EUPI-PV Partnership)</t>
+          <t>Large scale operational validation and upscaling of state-of-the-art (Generative) AI tools and models powering a next generation digital energy system</t>
         </is>
       </c>
       <c r="C633" s="22" t="n"/>
@@ -14363,7 +14531,7 @@
       </c>
       <c r="B634" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-15</t>
+          <t>HORIZON-CL5-2027-02-D3-24</t>
         </is>
       </c>
       <c r="C634" s="22" t="n"/>
@@ -14475,7 +14643,7 @@
       </c>
       <c r="B641" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:The REPowerEU plan and the EU Solar Energy Strategy introduced targets for the deployment of solar PV amounting to 600 GWac by 2030. Complying with these targets will be crucial for the European Union to reach its climate targets and free itself from import dependency on fossil fuels and the costs this imposes on Europe’s competitiveness in terms of high energy prices. The Solar Strategy also introduces a target, which has been enshrined into the Net-Zero Industry Act, to re-consolidate the European solar manufacturing sector and scale up European manufacturing capacity across</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Advanced, secure frugal (energy-, resource-, data- and cost-efficient, sustainable) AI tools for real-time grid operations (including protection), market operations (if relevant) and consumer empowerment in distributed energy systems.A demonstrated AI development environment integrated with the upgraded digital spine of the energy system and energy-saving consumer applications.Scaled-up capabilities for learning at edge nodes and federated systems using agent-based architectures.A governance fram</t>
         </is>
       </c>
       <c r="C641" s="22" t="n"/>
@@ -14519,7 +14687,7 @@
       </c>
       <c r="B644" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-15</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-24</t>
         </is>
       </c>
       <c r="C644" s="22" t="n"/>
@@ -14530,7 +14698,7 @@
     <row r="646" ht="30" customHeight="1">
       <c r="A646" s="18" t="inlineStr">
         <is>
-          <t>FICHA 44: HORIZON-CL5-2027-02-D3-07</t>
+          <t>FICHA 44: HORIZON-CL5-2027-02-D3-31</t>
         </is>
       </c>
       <c r="B646" s="19" t="n"/>
@@ -14555,7 +14723,7 @@
       <c r="E647" s="22" t="n"/>
       <c r="F647" s="22" t="n"/>
     </row>
-    <row r="648" ht="20" customHeight="1">
+    <row r="648" ht="45" customHeight="1">
       <c r="A648" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -14563,7 +14731,7 @@
       </c>
       <c r="B648" s="21" t="inlineStr">
         <is>
-          <t>Concentrated solar thermal systems for decarbonising industrial processes</t>
+          <t>Support to the implementation of an EU policy framework for CO2 transport and storage infrastructure</t>
         </is>
       </c>
       <c r="C648" s="22" t="n"/>
@@ -14579,7 +14747,7 @@
       </c>
       <c r="B649" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-07</t>
+          <t>HORIZON-CL5-2027-02-D3-31</t>
         </is>
       </c>
       <c r="C649" s="22" t="n"/>
@@ -14659,7 +14827,7 @@
       </c>
       <c r="B654" s="21" t="inlineStr">
         <is>
-          <t>Innovation Actions</t>
+          <t>Coordination and Support Actions</t>
         </is>
       </c>
       <c r="C654" s="22" t="n"/>
@@ -14691,7 +14859,7 @@
       </c>
       <c r="B656" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Renewable heating can be directly used to efficiently decarbonise industrial processes. Concentrated solar thermal technologies offer a great potential to supply renewable heat for industry for temperatures between 150°C - 400°C. Nevertheless, efforts are still required to demonstrate these technologies for a variety of industrial processes.Proposals are expected to contribute to all the following outcomes:Showcase the capacity of concentrated solar thermal systems to largely meet the heat demand of industrial processes and to achieve a yearly solar fraction of at least 50%.In</t>
+          <t>Expected Outcome:Project results are expected to contribute to the following outcome:Stakeholders involved in the CO2 infrastructure network are in a position to implement the upcoming legislative framework for CO2 infrastructure.  Scope:The project is expected to assist stakeholders involved in the CO2 infrastructure network in implementing the upcoming legislative framework for CO2 infrastructure.Issues to address include market and cost structure, cross-border integration, interoperability and planning, technical harmonisation and investment incentives for new infrastructure, third-party ac</t>
         </is>
       </c>
       <c r="C656" s="22" t="n"/>
@@ -14735,7 +14903,7 @@
       </c>
       <c r="B659" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-07</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-31</t>
         </is>
       </c>
       <c r="C659" s="22" t="n"/>
@@ -14746,7 +14914,7 @@
     <row r="661" ht="30" customHeight="1">
       <c r="A661" s="18" t="inlineStr">
         <is>
-          <t>FICHA 45: HORIZON-CL5-2027-02-D3-08</t>
+          <t>FICHA 45: HORIZON-CL5-2027-02-D3-15</t>
         </is>
       </c>
       <c r="B661" s="19" t="n"/>
@@ -14779,7 +14947,7 @@
       </c>
       <c r="B663" s="21" t="inlineStr">
         <is>
-          <t>Co-funding Strategic Energy Technology (SET) Plan renewable fuel value chains at EU, national, regional, and local level</t>
+          <t>Production technologies for solar photovoltaics beyond the state-of-the-art (EUPI-PV Partnership)</t>
         </is>
       </c>
       <c r="C663" s="22" t="n"/>
@@ -14795,7 +14963,7 @@
       </c>
       <c r="B664" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-08</t>
+          <t>HORIZON-CL5-2027-02-D3-15</t>
         </is>
       </c>
       <c r="C664" s="22" t="n"/>
@@ -14875,7 +15043,7 @@
       </c>
       <c r="B669" s="21" t="inlineStr">
         <is>
-          <t>Programme Cofund Actions</t>
+          <t>Innovation Actions</t>
         </is>
       </c>
       <c r="C669" s="22" t="n"/>
@@ -14907,7 +15075,7 @@
       </c>
       <c r="B671" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Advance in the realisation of the Strategic Energy Technology (SET) Plan Action of Renewable fuels and Bioenergy (for the fuels part) is supported, overcoming fragmentation by mobilizing resources and establishing across EU interregional value chains of renewable fuel technologies and by better alignment of public and private R&amp;amp;I priorities and of funding mechanisms.All sector stakeholders benefit from establishment of renewable fuels value chains at EU, national, regional, and local level</t>
+          <t>Expected Outcome:The REPowerEU plan and the EU Solar Energy Strategy introduced targets for the deployment of solar PV amounting to 600 GWac by 2030. Complying with these targets will be crucial for the European Union to reach its climate targets and free itself from import dependency on fossil fuels and the costs this imposes on Europe’s competitiveness in terms of high energy prices. The Solar Strategy also introduces a target, which has been enshrined into the Net-Zero Industry Act, to re-consolidate the European solar manufacturing sector and scale up European manufacturing capacity across</t>
         </is>
       </c>
       <c r="C671" s="22" t="n"/>
@@ -14951,7 +15119,7 @@
       </c>
       <c r="B674" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-08</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-15</t>
         </is>
       </c>
       <c r="C674" s="22" t="n"/>
@@ -18526,7 +18694,7 @@
     <row r="931" ht="30" customHeight="1">
       <c r="A931" s="18" t="inlineStr">
         <is>
-          <t>FICHA 63: EUS-57677</t>
+          <t>FICHA 63: EUS-97378</t>
         </is>
       </c>
       <c r="B931" s="19" t="n"/>
@@ -18575,7 +18743,7 @@
       </c>
       <c r="B934" s="21" t="inlineStr">
         <is>
-          <t>EUS-57677</t>
+          <t>EUS-97378</t>
         </is>
       </c>
       <c r="C934" s="22" t="n"/>
@@ -18738,7 +18906,7 @@
     <row r="946" ht="30" customHeight="1">
       <c r="A946" s="18" t="inlineStr">
         <is>
-          <t>FICHA 64: EUS-13853</t>
+          <t>FICHA 64: EUS-04117</t>
         </is>
       </c>
       <c r="B946" s="19" t="n"/>
@@ -18787,7 +18955,7 @@
       </c>
       <c r="B949" s="21" t="inlineStr">
         <is>
-          <t>EUS-13853</t>
+          <t>EUS-04117</t>
         </is>
       </c>
       <c r="C949" s="22" t="n"/>
@@ -18950,7 +19118,7 @@
     <row r="961" ht="30" customHeight="1">
       <c r="A961" s="18" t="inlineStr">
         <is>
-          <t>FICHA 65: EUS-25004</t>
+          <t>FICHA 65: EUS-87863</t>
         </is>
       </c>
       <c r="B961" s="19" t="n"/>
@@ -18999,7 +19167,7 @@
       </c>
       <c r="B964" s="21" t="inlineStr">
         <is>
-          <t>EUS-25004</t>
+          <t>EUS-87863</t>
         </is>
       </c>
       <c r="C964" s="22" t="n"/>
@@ -19162,7 +19330,7 @@
     <row r="976" ht="30" customHeight="1">
       <c r="A976" s="18" t="inlineStr">
         <is>
-          <t>FICHA 66: EUS-93927</t>
+          <t>FICHA 66: EUS-85070</t>
         </is>
       </c>
       <c r="B976" s="19" t="n"/>
@@ -19211,7 +19379,7 @@
       </c>
       <c r="B979" s="21" t="inlineStr">
         <is>
-          <t>EUS-93927</t>
+          <t>EUS-85070</t>
         </is>
       </c>
       <c r="C979" s="22" t="n"/>
@@ -19374,7 +19542,7 @@
     <row r="991" ht="30" customHeight="1">
       <c r="A991" s="18" t="inlineStr">
         <is>
-          <t>FICHA 67: EUS-34980</t>
+          <t>FICHA 67: EUS-86334</t>
         </is>
       </c>
       <c r="B991" s="19" t="n"/>
@@ -19407,7 +19575,7 @@
       </c>
       <c r="B993" s="21" t="inlineStr">
         <is>
-          <t>I+D.  Red Eureka, o programas financiados por el marco de innovación Horizon, como Eurostars (pymes) PRIMA (Mediterráneo) CETP (Energía) o DUT (Transformación Urbana). Evento del 12.05.26 sobre consor</t>
+          <t>Enajenación mediante subasta de diversos materiales que se encuentran en el almacén municipal para su achatarramiento y tratamiento como residuos sólidos urbanos</t>
         </is>
       </c>
       <c r="C993" s="22" t="n"/>
@@ -19423,7 +19591,7 @@
       </c>
       <c r="B994" s="21" t="inlineStr">
         <is>
-          <t>EUS-34980</t>
+          <t>EUS-86334</t>
         </is>
       </c>
       <c r="C994" s="22" t="n"/>
@@ -19499,7 +19667,7 @@
       </c>
       <c r="B999" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C999" s="22" t="n"/>
@@ -19557,9 +19725,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B1003" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
+      <c r="B1003" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALTA — </t>
         </is>
       </c>
       <c r="C1003" s="22" t="n"/>
@@ -19575,7 +19743,7 @@
       </c>
       <c r="B1004" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/2605eurekaeurostarsdutpri/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/enajenacion-mediante-subasta-diversos-materiales-que-se-encuentran-almacen-municipal-su-achatarramiento-y-tratamiento-como-residuos-solidos-urbanos/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1004" s="22" t="n"/>
@@ -19586,7 +19754,7 @@
     <row r="1006" ht="30" customHeight="1">
       <c r="A1006" s="18" t="inlineStr">
         <is>
-          <t>FICHA 68: EUS-01747</t>
+          <t>FICHA 68: EUS-05833</t>
         </is>
       </c>
       <c r="B1006" s="19" t="n"/>
@@ -19619,7 +19787,7 @@
       </c>
       <c r="B1008" s="21" t="inlineStr">
         <is>
-          <t>CEF-E. Línea de infraestructuras energéticas del Mecanismo Conectar Europa. Alineado con planes de Redes Transeuropeas (RTE-E) plan de choque anticrisis de la Unión de la Energía (AccelerateEU). Proye</t>
+          <t>I+D.  Red Eureka, o programas financiados por el marco de innovación Horizon, como Eurostars (pymes) PRIMA (Mediterráneo) CETP (Energía) o DUT (Transformación Urbana). Evento del 12.05.26 sobre consor</t>
         </is>
       </c>
       <c r="C1008" s="22" t="n"/>
@@ -19635,7 +19803,7 @@
       </c>
       <c r="B1009" s="21" t="inlineStr">
         <is>
-          <t>EUS-01747</t>
+          <t>EUS-05833</t>
         </is>
       </c>
       <c r="C1009" s="22" t="n"/>
@@ -19787,7 +19955,7 @@
       </c>
       <c r="B1019" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/2605ceferteepcipmiacceler/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/2605eurekaeurostarsdutpri/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1019" s="22" t="n"/>
@@ -19798,7 +19966,7 @@
     <row r="1021" ht="30" customHeight="1">
       <c r="A1021" s="18" t="inlineStr">
         <is>
-          <t>FICHA 69: EUS-42478</t>
+          <t>FICHA 69: EUS-20593</t>
         </is>
       </c>
       <c r="B1021" s="19" t="n"/>
@@ -19831,7 +19999,7 @@
       </c>
       <c r="B1023" s="21" t="inlineStr">
         <is>
-          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta el 01.10.26. Cribado de enfermedades con inteligencia artificial. Espacio de Datos Sanitarios de la UE. Red de Centros para Seguridad de la I</t>
+          <t>CEF-E. Línea de infraestructuras energéticas del Mecanismo Conectar Europa. Alineado con planes de Redes Transeuropeas (RTE-E) plan de choque anticrisis de la Unión de la Energía (AccelerateEU). Proye</t>
         </is>
       </c>
       <c r="C1023" s="22" t="n"/>
@@ -19847,7 +20015,7 @@
       </c>
       <c r="B1024" s="21" t="inlineStr">
         <is>
-          <t>EUS-42478</t>
+          <t>EUS-20593</t>
         </is>
       </c>
       <c r="C1024" s="22" t="n"/>
@@ -19999,7 +20167,7 @@
       </c>
       <c r="B1034" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260422digitaleuropekoak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/2605ceferteepcipmiacceler/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1034" s="22" t="n"/>
@@ -20010,7 +20178,7 @@
     <row r="1036" ht="30" customHeight="1">
       <c r="A1036" s="18" t="inlineStr">
         <is>
-          <t>FICHA 70: EUS-35761</t>
+          <t>FICHA 70: EUS-82373</t>
         </is>
       </c>
       <c r="B1036" s="19" t="n"/>
@@ -20043,7 +20211,7 @@
       </c>
       <c r="B1038" s="21" t="inlineStr">
         <is>
-          <t>Suministro, implantación, mantenimiento, gestión y operación del nuevo servicio de bicicleta pública de Bizkaia BizkaiBizi</t>
+          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta el 01.10.26. Cribado de enfermedades con inteligencia artificial. Espacio de Datos Sanitarios de la UE. Red de Centros para Seguridad de la I</t>
         </is>
       </c>
       <c r="C1038" s="22" t="n"/>
@@ -20059,7 +20227,7 @@
       </c>
       <c r="B1039" s="21" t="inlineStr">
         <is>
-          <t>EUS-35761</t>
+          <t>EUS-82373</t>
         </is>
       </c>
       <c r="C1039" s="22" t="n"/>
@@ -20135,7 +20303,7 @@
       </c>
       <c r="B1044" s="21" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C1044" s="22" t="n"/>
@@ -20211,7 +20379,7 @@
       </c>
       <c r="B1049" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-implantacion-mantenimiento-gestion-y-operacion-del-nuevo-servicio-bicicleta-publica-bizkaia-bizkaibizi/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260422digitaleuropekoak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1049" s="22" t="n"/>
@@ -20222,7 +20390,7 @@
     <row r="1051" ht="30" customHeight="1">
       <c r="A1051" s="18" t="inlineStr">
         <is>
-          <t>FICHA 71: EUS-32315</t>
+          <t>FICHA 71: EUS-56939</t>
         </is>
       </c>
       <c r="B1051" s="19" t="n"/>
@@ -20255,7 +20423,7 @@
       </c>
       <c r="B1053" s="21" t="inlineStr">
         <is>
-          <t>Servicio de transporte urbano de viajeros- experiencia piloto</t>
+          <t>Adquisición de paraguas corporativos del 90 aniversario del Gobierno Vasco</t>
         </is>
       </c>
       <c r="C1053" s="22" t="n"/>
@@ -20271,7 +20439,7 @@
       </c>
       <c r="B1054" s="21" t="inlineStr">
         <is>
-          <t>EUS-32315</t>
+          <t>EUS-56939</t>
         </is>
       </c>
       <c r="C1054" s="22" t="n"/>
@@ -20423,7 +20591,7 @@
       </c>
       <c r="B1064" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/servicio-transporte-urbano-viajeros-experiencia-piloto/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/adquisicion-paraguas-corporativos-del-90-aniversario-del-gobierno-vasco/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1064" s="22" t="n"/>
@@ -20434,7 +20602,7 @@
     <row r="1066" ht="30" customHeight="1">
       <c r="A1066" s="18" t="inlineStr">
         <is>
-          <t>FICHA 72: EUS-36844</t>
+          <t>FICHA 72: EUS-37445</t>
         </is>
       </c>
       <c r="B1066" s="19" t="n"/>
@@ -20467,7 +20635,7 @@
       </c>
       <c r="B1068" s="21" t="inlineStr">
         <is>
-          <t>Prestación de servicios de apoyo a la secretaría técnica en el diseño, despliegue y seguimiento de la Estrategia para la Transformación Digital de Euskadi 2030.</t>
+          <t>Suministro, instalación y puesta en marcha de un conjunto de grupos electrógenos y depósitos auxiliares del sistema PEMEL de la red de saneamiento y abastecimiento de Aguas del Añarbe</t>
         </is>
       </c>
       <c r="C1068" s="22" t="n"/>
@@ -20483,7 +20651,7 @@
       </c>
       <c r="B1069" s="21" t="inlineStr">
         <is>
-          <t>EUS-36844</t>
+          <t>EUS-37445</t>
         </is>
       </c>
       <c r="C1069" s="22" t="n"/>
@@ -20635,7 +20803,7 @@
       </c>
       <c r="B1079" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/prestacion-servicios-apoyo-secretaria-tecnica-diseno-despliegue-y-seguimiento-estrategia-transformacion-digital-euskadi-2030/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-instalacion-y-puesta-marcha-conjunto-grupos-electrogenos-y-depositos-auxiliares-del-sistema-pemel-red-saneamiento-y-abastecimiento-aguas-del-anarbe/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1079" s="22" t="n"/>
@@ -20646,7 +20814,7 @@
     <row r="1081" ht="30" customHeight="1">
       <c r="A1081" s="18" t="inlineStr">
         <is>
-          <t>FICHA 73: EUS-88203</t>
+          <t>FICHA 73: EUS-17618</t>
         </is>
       </c>
       <c r="B1081" s="19" t="n"/>
@@ -20671,7 +20839,7 @@
       <c r="E1082" s="22" t="n"/>
       <c r="F1082" s="22" t="n"/>
     </row>
-    <row r="1083" ht="45" customHeight="1">
+    <row r="1083" ht="20" customHeight="1">
       <c r="A1083" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -20679,7 +20847,7 @@
       </c>
       <c r="B1083" s="21" t="inlineStr">
         <is>
-          <t>Mantenimiento limpieza de la red de arquetas y tuberías de saneamiento en villamonte</t>
+          <t>Obras de reparación de la caldera en el colegio Mendiko</t>
         </is>
       </c>
       <c r="C1083" s="22" t="n"/>
@@ -20695,7 +20863,7 @@
       </c>
       <c r="B1084" s="21" t="inlineStr">
         <is>
-          <t>EUS-88203</t>
+          <t>EUS-17618</t>
         </is>
       </c>
       <c r="C1084" s="22" t="n"/>
@@ -20847,7 +21015,7 @@
       </c>
       <c r="B1094" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/mantenimiento-limpieza-red-arquetas-y-tuberias-saneamiento-villamonte/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/obras-reparacion-caldera-colegio-mendiko/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1094" s="22" t="n"/>
@@ -20855,8 +21023,644 @@
       <c r="E1094" s="22" t="n"/>
       <c r="F1094" s="22" t="n"/>
     </row>
+    <row r="1096" ht="30" customHeight="1">
+      <c r="A1096" s="18" t="inlineStr">
+        <is>
+          <t>FICHA 74: EUS-83776</t>
+        </is>
+      </c>
+      <c r="B1096" s="19" t="n"/>
+      <c r="C1096" s="19" t="n"/>
+      <c r="D1096" s="19" t="n"/>
+      <c r="E1096" s="19" t="n"/>
+      <c r="F1096" s="19" t="n"/>
+    </row>
+    <row r="1097" ht="20" customHeight="1">
+      <c r="A1097" s="20" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1097" s="21" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1097" s="22" t="n"/>
+      <c r="D1097" s="22" t="n"/>
+      <c r="E1097" s="22" t="n"/>
+      <c r="F1097" s="22" t="n"/>
+    </row>
+    <row r="1098" ht="45" customHeight="1">
+      <c r="A1098" s="20" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1098" s="21" t="inlineStr">
+        <is>
+          <t>Suministro, instalación, puesta en marcha y mantenimiento de un sistema analítico para la determinación de la concentración de compuestos organohalogenados adsorbibles (AOX) en el laboratorio de contr</t>
+        </is>
+      </c>
+      <c r="C1098" s="22" t="n"/>
+      <c r="D1098" s="22" t="n"/>
+      <c r="E1098" s="22" t="n"/>
+      <c r="F1098" s="22" t="n"/>
+    </row>
+    <row r="1099" ht="20" customHeight="1">
+      <c r="A1099" s="20" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1099" s="21" t="inlineStr">
+        <is>
+          <t>EUS-83776</t>
+        </is>
+      </c>
+      <c r="C1099" s="22" t="n"/>
+      <c r="D1099" s="22" t="n"/>
+      <c r="E1099" s="22" t="n"/>
+      <c r="F1099" s="22" t="n"/>
+    </row>
+    <row r="1100" ht="20" customHeight="1">
+      <c r="A1100" s="20" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1100" s="21" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1100" s="22" t="n"/>
+      <c r="D1100" s="22" t="n"/>
+      <c r="E1100" s="22" t="n"/>
+      <c r="F1100" s="22" t="n"/>
+    </row>
+    <row r="1101" ht="20" customHeight="1">
+      <c r="A1101" s="20" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1101" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1101" s="22" t="n"/>
+      <c r="D1101" s="22" t="n"/>
+      <c r="E1101" s="22" t="n"/>
+      <c r="F1101" s="22" t="n"/>
+    </row>
+    <row r="1102" ht="20" customHeight="1">
+      <c r="A1102" s="20" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1102" s="21" t="inlineStr"/>
+      <c r="C1102" s="22" t="n"/>
+      <c r="D1102" s="22" t="n"/>
+      <c r="E1102" s="22" t="n"/>
+      <c r="F1102" s="22" t="n"/>
+    </row>
+    <row r="1103" ht="20" customHeight="1">
+      <c r="A1103" s="20" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1103" s="21" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1103" s="22" t="n"/>
+      <c r="D1103" s="22" t="n"/>
+      <c r="E1103" s="22" t="n"/>
+      <c r="F1103" s="22" t="n"/>
+    </row>
+    <row r="1104" ht="20" customHeight="1">
+      <c r="A1104" s="20" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1104" s="21" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1104" s="22" t="n"/>
+      <c r="D1104" s="22" t="n"/>
+      <c r="E1104" s="22" t="n"/>
+      <c r="F1104" s="22" t="n"/>
+    </row>
+    <row r="1105" ht="20" customHeight="1">
+      <c r="A1105" s="20" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1105" s="21" t="inlineStr"/>
+      <c r="C1105" s="22" t="n"/>
+      <c r="D1105" s="22" t="n"/>
+      <c r="E1105" s="22" t="n"/>
+      <c r="F1105" s="22" t="n"/>
+    </row>
+    <row r="1106" ht="20" customHeight="1">
+      <c r="A1106" s="20" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1106" s="21" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1106" s="22" t="n"/>
+      <c r="D1106" s="22" t="n"/>
+      <c r="E1106" s="22" t="n"/>
+      <c r="F1106" s="22" t="n"/>
+    </row>
+    <row r="1107" ht="20" customHeight="1">
+      <c r="A1107" s="20" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1107" s="21" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1107" s="22" t="n"/>
+      <c r="D1107" s="22" t="n"/>
+      <c r="E1107" s="22" t="n"/>
+      <c r="F1107" s="22" t="n"/>
+    </row>
+    <row r="1108" ht="20" customHeight="1">
+      <c r="A1108" s="20" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1108" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1108" s="22" t="n"/>
+      <c r="D1108" s="22" t="n"/>
+      <c r="E1108" s="22" t="n"/>
+      <c r="F1108" s="22" t="n"/>
+    </row>
+    <row r="1109" ht="45" customHeight="1">
+      <c r="A1109" s="20" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1109" s="23" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-instalacion-puesta-marcha-y-mantenimiento-sistema-analitico-determinacion-concentracion-compuestos-organohalogenados-adsorbibles-aox-laboratorio-control-calidad-aguas-residuales-agasa/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1109" s="22" t="n"/>
+      <c r="D1109" s="22" t="n"/>
+      <c r="E1109" s="22" t="n"/>
+      <c r="F1109" s="22" t="n"/>
+    </row>
+    <row r="1111" ht="30" customHeight="1">
+      <c r="A1111" s="18" t="inlineStr">
+        <is>
+          <t>FICHA 75: EUS-27600</t>
+        </is>
+      </c>
+      <c r="B1111" s="19" t="n"/>
+      <c r="C1111" s="19" t="n"/>
+      <c r="D1111" s="19" t="n"/>
+      <c r="E1111" s="19" t="n"/>
+      <c r="F1111" s="19" t="n"/>
+    </row>
+    <row r="1112" ht="20" customHeight="1">
+      <c r="A1112" s="20" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1112" s="21" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1112" s="22" t="n"/>
+      <c r="D1112" s="22" t="n"/>
+      <c r="E1112" s="22" t="n"/>
+      <c r="F1112" s="22" t="n"/>
+    </row>
+    <row r="1113" ht="20" customHeight="1">
+      <c r="A1113" s="20" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1113" s="21" t="inlineStr">
+        <is>
+          <t>Gestión de incidencias en las viviendas dependientes de servicios sociales</t>
+        </is>
+      </c>
+      <c r="C1113" s="22" t="n"/>
+      <c r="D1113" s="22" t="n"/>
+      <c r="E1113" s="22" t="n"/>
+      <c r="F1113" s="22" t="n"/>
+    </row>
+    <row r="1114" ht="20" customHeight="1">
+      <c r="A1114" s="20" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1114" s="21" t="inlineStr">
+        <is>
+          <t>EUS-27600</t>
+        </is>
+      </c>
+      <c r="C1114" s="22" t="n"/>
+      <c r="D1114" s="22" t="n"/>
+      <c r="E1114" s="22" t="n"/>
+      <c r="F1114" s="22" t="n"/>
+    </row>
+    <row r="1115" ht="20" customHeight="1">
+      <c r="A1115" s="20" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1115" s="21" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1115" s="22" t="n"/>
+      <c r="D1115" s="22" t="n"/>
+      <c r="E1115" s="22" t="n"/>
+      <c r="F1115" s="22" t="n"/>
+    </row>
+    <row r="1116" ht="20" customHeight="1">
+      <c r="A1116" s="20" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1116" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1116" s="22" t="n"/>
+      <c r="D1116" s="22" t="n"/>
+      <c r="E1116" s="22" t="n"/>
+      <c r="F1116" s="22" t="n"/>
+    </row>
+    <row r="1117" ht="20" customHeight="1">
+      <c r="A1117" s="20" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1117" s="21" t="inlineStr"/>
+      <c r="C1117" s="22" t="n"/>
+      <c r="D1117" s="22" t="n"/>
+      <c r="E1117" s="22" t="n"/>
+      <c r="F1117" s="22" t="n"/>
+    </row>
+    <row r="1118" ht="20" customHeight="1">
+      <c r="A1118" s="20" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1118" s="21" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1118" s="22" t="n"/>
+      <c r="D1118" s="22" t="n"/>
+      <c r="E1118" s="22" t="n"/>
+      <c r="F1118" s="22" t="n"/>
+    </row>
+    <row r="1119" ht="20" customHeight="1">
+      <c r="A1119" s="20" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1119" s="21" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1119" s="22" t="n"/>
+      <c r="D1119" s="22" t="n"/>
+      <c r="E1119" s="22" t="n"/>
+      <c r="F1119" s="22" t="n"/>
+    </row>
+    <row r="1120" ht="20" customHeight="1">
+      <c r="A1120" s="20" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1120" s="21" t="inlineStr"/>
+      <c r="C1120" s="22" t="n"/>
+      <c r="D1120" s="22" t="n"/>
+      <c r="E1120" s="22" t="n"/>
+      <c r="F1120" s="22" t="n"/>
+    </row>
+    <row r="1121" ht="20" customHeight="1">
+      <c r="A1121" s="20" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1121" s="21" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1121" s="22" t="n"/>
+      <c r="D1121" s="22" t="n"/>
+      <c r="E1121" s="22" t="n"/>
+      <c r="F1121" s="22" t="n"/>
+    </row>
+    <row r="1122" ht="20" customHeight="1">
+      <c r="A1122" s="20" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1122" s="21" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1122" s="22" t="n"/>
+      <c r="D1122" s="22" t="n"/>
+      <c r="E1122" s="22" t="n"/>
+      <c r="F1122" s="22" t="n"/>
+    </row>
+    <row r="1123" ht="20" customHeight="1">
+      <c r="A1123" s="20" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1123" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1123" s="22" t="n"/>
+      <c r="D1123" s="22" t="n"/>
+      <c r="E1123" s="22" t="n"/>
+      <c r="F1123" s="22" t="n"/>
+    </row>
+    <row r="1124" ht="45" customHeight="1">
+      <c r="A1124" s="20" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1124" s="23" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/gestion-incidencias-viviendas-dependientes-servicios-sociales/expgegetxo12025002732/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1124" s="22" t="n"/>
+      <c r="D1124" s="22" t="n"/>
+      <c r="E1124" s="22" t="n"/>
+      <c r="F1124" s="22" t="n"/>
+    </row>
+    <row r="1126" ht="30" customHeight="1">
+      <c r="A1126" s="18" t="inlineStr">
+        <is>
+          <t>FICHA 76: EUS-44604</t>
+        </is>
+      </c>
+      <c r="B1126" s="19" t="n"/>
+      <c r="C1126" s="19" t="n"/>
+      <c r="D1126" s="19" t="n"/>
+      <c r="E1126" s="19" t="n"/>
+      <c r="F1126" s="19" t="n"/>
+    </row>
+    <row r="1127" ht="20" customHeight="1">
+      <c r="A1127" s="20" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1127" s="21" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1127" s="22" t="n"/>
+      <c r="D1127" s="22" t="n"/>
+      <c r="E1127" s="22" t="n"/>
+      <c r="F1127" s="22" t="n"/>
+    </row>
+    <row r="1128" ht="45" customHeight="1">
+      <c r="A1128" s="20" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1128" s="21" t="inlineStr">
+        <is>
+          <t>Trabajos sobrevenidos de renovación integral de zonas verdes aledañas a rampas 1 y 2 bidezabal</t>
+        </is>
+      </c>
+      <c r="C1128" s="22" t="n"/>
+      <c r="D1128" s="22" t="n"/>
+      <c r="E1128" s="22" t="n"/>
+      <c r="F1128" s="22" t="n"/>
+    </row>
+    <row r="1129" ht="20" customHeight="1">
+      <c r="A1129" s="20" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1129" s="21" t="inlineStr">
+        <is>
+          <t>EUS-44604</t>
+        </is>
+      </c>
+      <c r="C1129" s="22" t="n"/>
+      <c r="D1129" s="22" t="n"/>
+      <c r="E1129" s="22" t="n"/>
+      <c r="F1129" s="22" t="n"/>
+    </row>
+    <row r="1130" ht="20" customHeight="1">
+      <c r="A1130" s="20" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1130" s="21" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1130" s="22" t="n"/>
+      <c r="D1130" s="22" t="n"/>
+      <c r="E1130" s="22" t="n"/>
+      <c r="F1130" s="22" t="n"/>
+    </row>
+    <row r="1131" ht="20" customHeight="1">
+      <c r="A1131" s="20" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1131" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1131" s="22" t="n"/>
+      <c r="D1131" s="22" t="n"/>
+      <c r="E1131" s="22" t="n"/>
+      <c r="F1131" s="22" t="n"/>
+    </row>
+    <row r="1132" ht="20" customHeight="1">
+      <c r="A1132" s="20" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1132" s="21" t="inlineStr"/>
+      <c r="C1132" s="22" t="n"/>
+      <c r="D1132" s="22" t="n"/>
+      <c r="E1132" s="22" t="n"/>
+      <c r="F1132" s="22" t="n"/>
+    </row>
+    <row r="1133" ht="20" customHeight="1">
+      <c r="A1133" s="20" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1133" s="21" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1133" s="22" t="n"/>
+      <c r="D1133" s="22" t="n"/>
+      <c r="E1133" s="22" t="n"/>
+      <c r="F1133" s="22" t="n"/>
+    </row>
+    <row r="1134" ht="20" customHeight="1">
+      <c r="A1134" s="20" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1134" s="21" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1134" s="22" t="n"/>
+      <c r="D1134" s="22" t="n"/>
+      <c r="E1134" s="22" t="n"/>
+      <c r="F1134" s="22" t="n"/>
+    </row>
+    <row r="1135" ht="20" customHeight="1">
+      <c r="A1135" s="20" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1135" s="21" t="inlineStr"/>
+      <c r="C1135" s="22" t="n"/>
+      <c r="D1135" s="22" t="n"/>
+      <c r="E1135" s="22" t="n"/>
+      <c r="F1135" s="22" t="n"/>
+    </row>
+    <row r="1136" ht="20" customHeight="1">
+      <c r="A1136" s="20" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1136" s="21" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1136" s="22" t="n"/>
+      <c r="D1136" s="22" t="n"/>
+      <c r="E1136" s="22" t="n"/>
+      <c r="F1136" s="22" t="n"/>
+    </row>
+    <row r="1137" ht="20" customHeight="1">
+      <c r="A1137" s="20" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1137" s="21" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1137" s="22" t="n"/>
+      <c r="D1137" s="22" t="n"/>
+      <c r="E1137" s="22" t="n"/>
+      <c r="F1137" s="22" t="n"/>
+    </row>
+    <row r="1138" ht="20" customHeight="1">
+      <c r="A1138" s="20" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1138" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1138" s="22" t="n"/>
+      <c r="D1138" s="22" t="n"/>
+      <c r="E1138" s="22" t="n"/>
+      <c r="F1138" s="22" t="n"/>
+    </row>
+    <row r="1139" ht="45" customHeight="1">
+      <c r="A1139" s="20" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1139" s="23" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/trabajos-sobrevenidos-renovacion-integral-zonas-verdes-aledanas-rampas-1-y-2-bidezabal/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1139" s="22" t="n"/>
+      <c r="D1139" s="22" t="n"/>
+      <c r="E1139" s="22" t="n"/>
+      <c r="F1139" s="22" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="1022">
+  <mergeCells count="1064">
     <mergeCell ref="B679:F679"/>
     <mergeCell ref="B666:F666"/>
     <mergeCell ref="B964:F964"/>
@@ -20900,7 +21704,9 @@
     <mergeCell ref="B342:F342"/>
     <mergeCell ref="B578:F578"/>
     <mergeCell ref="A541:F541"/>
+    <mergeCell ref="B1099:F1099"/>
     <mergeCell ref="B515:F515"/>
+    <mergeCell ref="B1128:F1128"/>
     <mergeCell ref="A841:F841"/>
     <mergeCell ref="B158:F158"/>
     <mergeCell ref="B1094:F1094"/>
@@ -20909,6 +21715,7 @@
     <mergeCell ref="B894:F894"/>
     <mergeCell ref="B133:F133"/>
     <mergeCell ref="B959:F959"/>
+    <mergeCell ref="B1130:F1130"/>
     <mergeCell ref="B369:F369"/>
     <mergeCell ref="B667:F667"/>
     <mergeCell ref="B418:F418"/>
@@ -20935,11 +21742,13 @@
     <mergeCell ref="B662:F662"/>
     <mergeCell ref="B718:F718"/>
     <mergeCell ref="B889:F889"/>
+    <mergeCell ref="B1131:F1131"/>
     <mergeCell ref="B72:F72"/>
     <mergeCell ref="B954:F954"/>
     <mergeCell ref="B199:F199"/>
     <mergeCell ref="B370:F370"/>
     <mergeCell ref="B1025:F1025"/>
+    <mergeCell ref="B1112:F1112"/>
     <mergeCell ref="B291:F291"/>
     <mergeCell ref="B655:F655"/>
     <mergeCell ref="B974:F974"/>
@@ -20981,6 +21790,7 @@
     <mergeCell ref="B83:F83"/>
     <mergeCell ref="B254:F254"/>
     <mergeCell ref="B909:F909"/>
+    <mergeCell ref="B1105:F1105"/>
     <mergeCell ref="B319:F319"/>
     <mergeCell ref="B490:F490"/>
     <mergeCell ref="B604:F604"/>
@@ -21012,6 +21822,7 @@
     <mergeCell ref="B530:F530"/>
     <mergeCell ref="B726:F726"/>
     <mergeCell ref="B962:F962"/>
+    <mergeCell ref="B1133:F1133"/>
     <mergeCell ref="A886:F886"/>
     <mergeCell ref="B505:F505"/>
     <mergeCell ref="B1060:F1060"/>
@@ -21047,6 +21858,7 @@
     <mergeCell ref="B752:F752"/>
     <mergeCell ref="B1070:F1070"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B1115:F1115"/>
     <mergeCell ref="B325:F325"/>
     <mergeCell ref="B154:F154"/>
     <mergeCell ref="A271:F271"/>
@@ -21080,6 +21892,8 @@
     <mergeCell ref="B518:F518"/>
     <mergeCell ref="B562:F562"/>
     <mergeCell ref="B689:F689"/>
+    <mergeCell ref="B1121:F1121"/>
+    <mergeCell ref="B1123:F1123"/>
     <mergeCell ref="B86:F86"/>
     <mergeCell ref="B912:F912"/>
     <mergeCell ref="B1083:F1083"/>
@@ -21131,6 +21945,7 @@
     <mergeCell ref="B979:F979"/>
     <mergeCell ref="B381:F381"/>
     <mergeCell ref="B552:F552"/>
+    <mergeCell ref="A1111:F1111"/>
     <mergeCell ref="B1084:F1084"/>
     <mergeCell ref="A976:F976"/>
     <mergeCell ref="B170:F170"/>
@@ -21164,6 +21979,7 @@
     <mergeCell ref="B92:F92"/>
     <mergeCell ref="B984:F984"/>
     <mergeCell ref="A226:F226"/>
+    <mergeCell ref="B1124:F1124"/>
     <mergeCell ref="B394:F394"/>
     <mergeCell ref="B692:F692"/>
     <mergeCell ref="A931:F931"/>
@@ -21194,6 +22010,7 @@
     <mergeCell ref="B817:F817"/>
     <mergeCell ref="B944:F944"/>
     <mergeCell ref="B56:F56"/>
+    <mergeCell ref="B1102:F1102"/>
     <mergeCell ref="B43:F43"/>
     <mergeCell ref="B176:F176"/>
     <mergeCell ref="B347:F347"/>
@@ -21209,7 +22026,9 @@
     <mergeCell ref="B881:F881"/>
     <mergeCell ref="B1068:F1068"/>
     <mergeCell ref="B868:F868"/>
+    <mergeCell ref="B1117:F1117"/>
     <mergeCell ref="B107:F107"/>
+    <mergeCell ref="B1104:F1104"/>
     <mergeCell ref="B641:F641"/>
     <mergeCell ref="B57:F57"/>
     <mergeCell ref="B883:F883"/>
@@ -21235,6 +22054,7 @@
     <mergeCell ref="B999:F999"/>
     <mergeCell ref="B1061:F1061"/>
     <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B1097:F1097"/>
     <mergeCell ref="A46:F46"/>
     <mergeCell ref="B507:F507"/>
     <mergeCell ref="B62:F62"/>
@@ -21282,6 +22102,7 @@
     <mergeCell ref="B1018:F1018"/>
     <mergeCell ref="B624:F624"/>
     <mergeCell ref="B428:F428"/>
+    <mergeCell ref="B1118:F1118"/>
     <mergeCell ref="B284:F284"/>
     <mergeCell ref="B222:F222"/>
     <mergeCell ref="B344:F344"/>
@@ -21293,6 +22114,7 @@
     <mergeCell ref="B123:F123"/>
     <mergeCell ref="B949:F949"/>
     <mergeCell ref="B1011:F1011"/>
+    <mergeCell ref="B1120:F1120"/>
     <mergeCell ref="B50:F50"/>
     <mergeCell ref="B221:F221"/>
     <mergeCell ref="B110:F110"/>
@@ -21309,6 +22131,7 @@
     <mergeCell ref="B802:F802"/>
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B789:F789"/>
+    <mergeCell ref="B1136:F1136"/>
     <mergeCell ref="B248:F248"/>
     <mergeCell ref="B297:F297"/>
     <mergeCell ref="B813:F813"/>
@@ -21328,9 +22151,11 @@
     <mergeCell ref="B815:F815"/>
     <mergeCell ref="B597:F597"/>
     <mergeCell ref="B1064:F1064"/>
+    <mergeCell ref="B1113:F1113"/>
     <mergeCell ref="B103:F103"/>
     <mergeCell ref="B78:F78"/>
     <mergeCell ref="B833:F833"/>
+    <mergeCell ref="B1100:F1100"/>
     <mergeCell ref="B205:F205"/>
     <mergeCell ref="B339:F339"/>
     <mergeCell ref="B314:F314"/>
@@ -21426,6 +22251,7 @@
     <mergeCell ref="B305:F305"/>
     <mergeCell ref="B816:F816"/>
     <mergeCell ref="B918:F918"/>
+    <mergeCell ref="B1114:F1114"/>
     <mergeCell ref="B607:F607"/>
     <mergeCell ref="B663:F663"/>
     <mergeCell ref="B1049:F1049"/>
@@ -21436,6 +22262,7 @@
     <mergeCell ref="B442:F442"/>
     <mergeCell ref="B242:F242"/>
     <mergeCell ref="B880:F880"/>
+    <mergeCell ref="B1116:F1116"/>
     <mergeCell ref="B671:F671"/>
     <mergeCell ref="B969:F969"/>
     <mergeCell ref="B907:F907"/>
@@ -21453,12 +22280,15 @@
     <mergeCell ref="B760:F760"/>
     <mergeCell ref="B437:F437"/>
     <mergeCell ref="B852:F852"/>
+    <mergeCell ref="B1119:F1119"/>
     <mergeCell ref="B333:F333"/>
+    <mergeCell ref="B1098:F1098"/>
     <mergeCell ref="B898:F898"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="B520:F520"/>
     <mergeCell ref="B958:F958"/>
     <mergeCell ref="B308:F308"/>
+    <mergeCell ref="B1134:F1134"/>
     <mergeCell ref="B854:F854"/>
     <mergeCell ref="B99:F99"/>
     <mergeCell ref="B737:F737"/>
@@ -21477,12 +22307,14 @@
     <mergeCell ref="B372:F372"/>
     <mergeCell ref="B1071:F1071"/>
     <mergeCell ref="B608:F608"/>
+    <mergeCell ref="B1127:F1127"/>
     <mergeCell ref="B595:F595"/>
     <mergeCell ref="B1037:F1037"/>
     <mergeCell ref="B722:F722"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="A856:F856"/>
     <mergeCell ref="B893:F893"/>
+    <mergeCell ref="B1129:F1129"/>
     <mergeCell ref="B374:F374"/>
     <mergeCell ref="B659:F659"/>
     <mergeCell ref="B830:F830"/>
@@ -21551,6 +22383,7 @@
     <mergeCell ref="B309:F309"/>
     <mergeCell ref="A316:F316"/>
     <mergeCell ref="B380:F380"/>
+    <mergeCell ref="B1135:F1135"/>
     <mergeCell ref="A1081:F1081"/>
     <mergeCell ref="B100:F100"/>
     <mergeCell ref="B336:F336"/>
@@ -21560,10 +22393,12 @@
     <mergeCell ref="B140:F140"/>
     <mergeCell ref="B115:F115"/>
     <mergeCell ref="B382:F382"/>
+    <mergeCell ref="A1096:F1096"/>
     <mergeCell ref="B680:F680"/>
     <mergeCell ref="A376:F376"/>
     <mergeCell ref="B102:F102"/>
     <mergeCell ref="B674:F674"/>
+    <mergeCell ref="B1137:F1137"/>
     <mergeCell ref="B400:F400"/>
     <mergeCell ref="B698:F698"/>
     <mergeCell ref="B832:F832"/>
@@ -21576,6 +22411,7 @@
     <mergeCell ref="B598:F598"/>
     <mergeCell ref="B402:F402"/>
     <mergeCell ref="B669:F669"/>
+    <mergeCell ref="B1138:F1138"/>
     <mergeCell ref="B377:F377"/>
     <mergeCell ref="A451:F451"/>
     <mergeCell ref="B29:F29"/>
@@ -21782,11 +22618,14 @@
     <mergeCell ref="B409:F409"/>
     <mergeCell ref="B580:F580"/>
     <mergeCell ref="B920:F920"/>
+    <mergeCell ref="B1108:F1108"/>
     <mergeCell ref="B711:F711"/>
     <mergeCell ref="B1009:F1009"/>
     <mergeCell ref="B48:F48"/>
+    <mergeCell ref="B1101:F1101"/>
     <mergeCell ref="B582:F582"/>
     <mergeCell ref="B849:F849"/>
+    <mergeCell ref="B1132:F1132"/>
     <mergeCell ref="B73:F73"/>
     <mergeCell ref="B371:F371"/>
     <mergeCell ref="B638:F638"/>
@@ -21799,6 +22638,7 @@
     <mergeCell ref="A676:F676"/>
     <mergeCell ref="B137:F137"/>
     <mergeCell ref="B379:F379"/>
+    <mergeCell ref="B1106:F1106"/>
     <mergeCell ref="B702:F702"/>
     <mergeCell ref="B677:F677"/>
     <mergeCell ref="B640:F640"/>
@@ -21829,6 +22669,7 @@
     <mergeCell ref="B66:F66"/>
     <mergeCell ref="B326:F326"/>
     <mergeCell ref="B793:F793"/>
+    <mergeCell ref="B1103:F1103"/>
     <mergeCell ref="A406:F406"/>
     <mergeCell ref="B951:F951"/>
     <mergeCell ref="B130:F130"/>
@@ -21847,6 +22688,7 @@
     <mergeCell ref="B132:F132"/>
     <mergeCell ref="B425:F425"/>
     <mergeCell ref="B430:F430"/>
+    <mergeCell ref="B1107:F1107"/>
     <mergeCell ref="B1045:F1045"/>
     <mergeCell ref="B119:F119"/>
     <mergeCell ref="B290:F290"/>
@@ -21857,10 +22699,13 @@
     <mergeCell ref="B824:F824"/>
     <mergeCell ref="B1017:F1017"/>
     <mergeCell ref="B367:F367"/>
+    <mergeCell ref="B1122:F1122"/>
     <mergeCell ref="B427:F427"/>
+    <mergeCell ref="B1139:F1139"/>
     <mergeCell ref="B112:F112"/>
     <mergeCell ref="B283:F283"/>
     <mergeCell ref="B354:F354"/>
+    <mergeCell ref="B1109:F1109"/>
     <mergeCell ref="B348:F348"/>
     <mergeCell ref="B519:F519"/>
     <mergeCell ref="B419:F419"/>
@@ -21876,6 +22721,7 @@
     <mergeCell ref="B648:F648"/>
     <mergeCell ref="B64:F64"/>
     <mergeCell ref="B51:F51"/>
+    <mergeCell ref="A1126:F1126"/>
     <mergeCell ref="B443:F443"/>
     <mergeCell ref="A196:F196"/>
     <mergeCell ref="B237:F237"/>
@@ -21954,6 +22800,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1064" r:id="rId71"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1079" r:id="rId72"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1094" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1109" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1124" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1139" r:id="rId76"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -21965,7 +22814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J74"/>
+  <dimension ref="A1:J77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -22080,7 +22929,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Security challenges of the green transition in urban und per</t>
+          <t>Défis en matière de sécurité de la transition écologique dan</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -22355,12 +23204,12 @@
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-23</t>
+          <t>HORIZON-CL5-2026-11-D3-04</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Data sharing to support the training and development of AI f</t>
+          <t>De-risking renewable fuel technologies through transnational</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -22395,12 +23244,12 @@
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-06</t>
+          <t>HORIZON-CL5-2026-11-D3-05</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Resource assessment for deep sedimentary and basement reserv</t>
+          <t>Demonstration of solid biofuel supply and conversion to high</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -22435,12 +23284,12 @@
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-14</t>
+          <t>HORIZON-CL5-2026-11-D3-23</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Improved system design for innovative PV applications (EUPI-</t>
+          <t>Data sharing to support the training and development of AI f</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -22475,12 +23324,12 @@
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-05</t>
+          <t>HORIZON-CL5-2026-11-D3-06</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Demonstration of solid biofuel supply and conversion to high</t>
+          <t>Resource assessment for deep sedimentary and basement reserv</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -22515,12 +23364,12 @@
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-04</t>
+          <t>HORIZON-CL5-2026-11-D3-14</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>De-risking renewable fuel technologies through transnational</t>
+          <t>Improved system design for innovative PV applications (EUPI-</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -22555,12 +23404,12 @@
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-27</t>
+          <t>HORIZON-CL5-2027-07-D3-16</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Integrated Approaches for Retrofitting Infrastructures with </t>
+          <t xml:space="preserve">Industrial processes and equipment for innovative, reliable </t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -22595,12 +23444,12 @@
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-26</t>
+          <t>HORIZON-CL5-2027-07-D3-11</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Advanced Distribution Management Systems (ADSM) for more eff</t>
+          <t>Demonstration of hydropower technologies for efficient and f</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -22675,12 +23524,12 @@
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-28</t>
+          <t>HORIZON-CL5-2027-07-D3-26</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Community of practice - Data-Driven Decision-Making in Energ</t>
+          <t>Advanced Distribution Management Systems (ADSM) for more eff</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -22715,12 +23564,12 @@
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-16</t>
+          <t>HORIZON-CL5-2027-07-D3-27</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Industrial processes and equipment for innovative, reliable </t>
+          <t xml:space="preserve">Integrated Approaches for Retrofitting Infrastructures with </t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -22755,12 +23604,12 @@
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-25</t>
+          <t>HORIZON-CL5-2027-07-D3-28</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Advanced TSO control rooms to enhance grid observability, st</t>
+          <t>Community of practice - Data-Driven Decision-Making in Energ</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -22795,12 +23644,12 @@
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-17</t>
+          <t>HORIZON-CL5-2027-07-D3-25</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>PV based electrification of the economy: Designing &amp; optimis</t>
+          <t>Advanced TSO control rooms to enhance grid observability, st</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -22835,12 +23684,12 @@
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-11</t>
+          <t>HORIZON-CL5-2027-07-D3-17</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Demonstration of hydropower technologies for efficient and f</t>
+          <t>PV based electrification of the economy: Designing &amp; optimis</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -23595,12 +24444,12 @@
     <row r="41" ht="28" customHeight="1">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-31</t>
+          <t>HORIZON-CL5-2027-02-D3-08</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support to the implementation of an EU policy framework for </t>
+          <t xml:space="preserve">Co-funding Strategic Energy Technology (SET) Plan renewable </t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
@@ -23635,12 +24484,12 @@
     <row r="42" ht="28" customHeight="1">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-24</t>
+          <t>HORIZON-CL5-2027-02-D3-09</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>Large scale operational validation and upscaling of state-of</t>
+          <t>Innovative technologies and solutions to improve wave and ti</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
@@ -23715,12 +24564,12 @@
     <row r="44" ht="28" customHeight="1">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-15</t>
+          <t>HORIZON-CL5-2027-02-D3-24</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>Production technologies for solar photovoltaics beyond the s</t>
+          <t>Large scale operational validation and upscaling of state-of</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
@@ -23755,12 +24604,12 @@
     <row r="45" ht="28" customHeight="1">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-07</t>
+          <t>HORIZON-CL5-2027-02-D3-31</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>Concentrated solar thermal systems for decarbonising industr</t>
+          <t xml:space="preserve">Support to the implementation of an EU policy framework for </t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
@@ -23795,12 +24644,12 @@
     <row r="46" ht="28" customHeight="1">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-08</t>
+          <t>HORIZON-CL5-2027-02-D3-15</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Co-funding Strategic Energy Technology (SET) Plan renewable </t>
+          <t>Production technologies for solar photovoltaics beyond the s</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
@@ -24407,7 +25256,7 @@
     <row r="64" ht="28" customHeight="1">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>EUS-57677</t>
+          <t>EUS-97378</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
@@ -24443,7 +25292,7 @@
     <row r="65" ht="28" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>EUS-13853</t>
+          <t>EUS-04117</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
@@ -24479,7 +25328,7 @@
     <row r="66" ht="28" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>EUS-25004</t>
+          <t>EUS-87863</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
@@ -24515,7 +25364,7 @@
     <row r="67" ht="28" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>EUS-93927</t>
+          <t>EUS-85070</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
@@ -24551,12 +25400,12 @@
     <row r="68" ht="28" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>EUS-34980</t>
+          <t>EUS-86334</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>I+D.  Red Eureka, o programas financiados por el marco de in</t>
+          <t>Enajenación mediante subasta de diversos materiales que se e</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -24572,7 +25421,7 @@
       <c r="E68" s="6" t="inlineStr"/>
       <c r="F68" s="27" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="G68" s="6" t="inlineStr"/>
@@ -24587,12 +25436,12 @@
     <row r="69" ht="28" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>EUS-01747</t>
+          <t>EUS-05833</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>CEF-E. Línea de infraestructuras energéticas del Mecanismo C</t>
+          <t>I+D.  Red Eureka, o programas financiados por el marco de in</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -24623,12 +25472,12 @@
     <row r="70" ht="28" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>EUS-42478</t>
+          <t>EUS-20593</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta e</t>
+          <t>CEF-E. Línea de infraestructuras energéticas del Mecanismo C</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -24659,12 +25508,12 @@
     <row r="71" ht="28" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>EUS-35761</t>
+          <t>EUS-82373</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>Suministro, implantación, mantenimiento, gestión y operación</t>
+          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta e</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -24695,12 +25544,12 @@
     <row r="72" ht="28" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>EUS-32315</t>
+          <t>EUS-56939</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>Servicio de transporte urbano de viajeros- experiencia pilot</t>
+          <t xml:space="preserve">Adquisición de paraguas corporativos del 90 aniversario del </t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -24731,12 +25580,12 @@
     <row r="73" ht="28" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>EUS-36844</t>
+          <t>EUS-37445</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prestación de servicios de apoyo a la secretaría técnica en </t>
+          <t>Suministro, instalación y puesta en marcha de un conjunto de</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -24767,12 +25616,12 @@
     <row r="74" ht="28" customHeight="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>EUS-88203</t>
+          <t>EUS-17618</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>Mantenimiento limpieza de la red de arquetas y tuberías de s</t>
+          <t>Obras de reparación de la caldera en el colegio Mendiko</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
@@ -24800,8 +25649,116 @@
       <c r="I74" s="6" t="inlineStr"/>
       <c r="J74" s="6" t="inlineStr"/>
     </row>
+    <row r="75" ht="28" customHeight="1">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>EUS-83776</t>
+        </is>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>Suministro, instalación, puesta en marcha y mantenimiento de</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D75" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E75" s="6" t="inlineStr"/>
+      <c r="F75" s="27" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G75" s="6" t="inlineStr"/>
+      <c r="H75" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I75" s="6" t="inlineStr"/>
+      <c r="J75" s="6" t="inlineStr"/>
+    </row>
+    <row r="76" ht="28" customHeight="1">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>EUS-27600</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>Gestión de incidencias en las viviendas dependientes de serv</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E76" s="6" t="inlineStr"/>
+      <c r="F76" s="27" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G76" s="6" t="inlineStr"/>
+      <c r="H76" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I76" s="6" t="inlineStr"/>
+      <c r="J76" s="6" t="inlineStr"/>
+    </row>
+    <row r="77" ht="28" customHeight="1">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>EUS-44604</t>
+        </is>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>Trabajos sobrevenidos de renovación integral de zonas verdes</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="inlineStr"/>
+      <c r="F77" s="27" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G77" s="6" t="inlineStr"/>
+      <c r="H77" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I77" s="6" t="inlineStr"/>
+      <c r="J77" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J74"/>
+  <autoFilter ref="A1:J77"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update funding data 2026-05-12
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Recursos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$83</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$79</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -84,13 +84,13 @@
     <font>
       <name val="Leelawadee UI"/>
       <b val="1"/>
-      <color rgb="00065F46"/>
+      <color rgb="00DC2626"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Leelawadee UI"/>
       <b val="1"/>
-      <color rgb="00DC2626"/>
+      <color rgb="00065F46"/>
       <sz val="10"/>
     </font>
     <font>
@@ -166,17 +166,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FEF2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00065F46"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D1FAE5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEF2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -268,11 +268,11 @@
     <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -312,8 +312,8 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -679,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M83"/>
+  <dimension ref="A1:M85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -707,7 +707,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 11/05/2026 09:01 - 76 convocatorias - 14 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 12/05/2026 08:24 - 78 convocatorias - 17 nuevas</t>
         </is>
       </c>
     </row>
@@ -1289,12 +1289,12 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-04</t>
+          <t>HORIZON-CL5-2026-11-D3-23</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>De-risking renewable fuel technologies through transnational pre-commercial procurement of renewable fuel industrial value chains</t>
+          <t>Data sharing to support the training and development of AI foundation models in the energy sector</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>Pre-commercial Procurement</t>
+          <t>Innovation Actions</t>
         </is>
       </c>
       <c r="I14" s="10" t="inlineStr">
@@ -1334,7 +1334,7 @@
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Public authorities, industry, technology providers, energy producers and consumers profit from de-</t>
+          <t>Expected Outcome:Projects are expected to contribute to all the following expected outcomes:Effective and innovative methods for gathering, sharing and using large data sets in energy applications for</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr"/>
@@ -1352,12 +1352,12 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-05</t>
+          <t>HORIZON-CL5-2026-11-D3-06</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Demonstration of solid biofuel supply and conversion to high efficiency CHP from fully sustainable regional value chains</t>
+          <t>Resource assessment for deep sedimentary and basement reservoirs</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>Innovation Actions</t>
+          <t xml:space="preserve"> Research and Innovation Actions</t>
         </is>
       </c>
       <c r="I15" s="10" t="inlineStr">
@@ -1397,7 +1397,7 @@
       </c>
       <c r="K15" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Fully sustainable regional bioenergy value chains and efficient conversion can play an important role in renewable efficient power and heating generation and for reaching the EU clima</t>
+          <t>Expected Outcome:Deep sedimentary/basement reservoirs are usually characterized by low permeability, high drilling cost and a scarcity of data, as they are typically ignored by hydrocarbon exploration</t>
         </is>
       </c>
       <c r="L15" s="6" t="inlineStr"/>
@@ -1415,12 +1415,12 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-23</t>
+          <t>HORIZON-CL5-2026-11-D3-14</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Data sharing to support the training and development of AI foundation models in the energy sector</t>
+          <t>Improved system design for innovative PV applications (EUPI-PV Partnership)</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
@@ -1460,7 +1460,7 @@
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Projects are expected to contribute to all the following expected outcomes:Effective and innovative methods for gathering, sharing and using large data sets in energy applications for</t>
+          <t>Expected Outcome:Agrivoltaics or the co-location of agricultural activity and PV electricity production is a novel form of PV deployment which could provide farmers with diversified revenue sources an</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr"/>
@@ -1478,12 +1478,12 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-06</t>
+          <t>HORIZON-CL5-2026-11-D3-05</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Resource assessment for deep sedimentary and basement reservoirs</t>
+          <t>Demonstration of solid biofuel supply and conversion to high efficiency CHP from fully sustainable regional value chains</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Research and Innovation Actions</t>
+          <t>Innovation Actions</t>
         </is>
       </c>
       <c r="I17" s="10" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Deep sedimentary/basement reservoirs are usually characterized by low permeability, high drilling cost and a scarcity of data, as they are typically ignored by hydrocarbon exploration</t>
+          <t>Expected Outcome:Fully sustainable regional bioenergy value chains and efficient conversion can play an important role in renewable efficient power and heating generation and for reaching the EU clima</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr"/>
@@ -1541,12 +1541,12 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-14</t>
+          <t>HORIZON-CL5-2026-11-D3-04</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Improved system design for innovative PV applications (EUPI-PV Partnership)</t>
+          <t>De-risking renewable fuel technologies through transnational pre-commercial procurement of renewable fuel industrial value chains</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
@@ -1571,7 +1571,7 @@
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>Innovation Actions</t>
+          <t>Pre-commercial Procurement</t>
         </is>
       </c>
       <c r="I18" s="10" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Agrivoltaics or the co-location of agricultural activity and PV electricity production is a novel form of PV deployment which could provide farmers with diversified revenue sources an</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Public authorities, industry, technology providers, energy producers and consumers profit from de-</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr"/>
@@ -1604,12 +1604,12 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-16</t>
+          <t>HORIZON-CL5-2027-07-D3-27</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Industrial processes and equipment for innovative, reliable and scalable tandem technologies (EUPI-PV Partnership)</t>
+          <t>Integrated Approaches for Retrofitting Infrastructures with Innovative Energy Storage Technologies</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:The REPowerEU plan and the EU Solar Energy Strategy introduced targets for the deployment of solar PV amounting to 600 GWac by 2030. Complying with these targets will be crucial for t</t>
+          <t xml:space="preserve">Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Improved energy security of the energy system by offering cost-effective and efficient solutions for </t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr"/>
@@ -1667,12 +1667,12 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-11</t>
+          <t>HORIZON-CL5-2027-07-D3-26</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Demonstration of hydropower technologies for efficient and forward-looking refurbishment of existing hydropower plants</t>
+          <t>Advanced Distribution Management Systems (ADSM) for more efficient and flexible distribution grids</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="K20" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:For a renewables-based electricity system sufficient flexible and also in the long-run fully sustainable hydropower capacity is pivotal.Project results are expected to contribute to a</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced reliability, resilience, controllability and efficiency of electricity distribution grids. C</t>
         </is>
       </c>
       <c r="L20" s="6" t="inlineStr"/>
@@ -1793,12 +1793,12 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-26</t>
+          <t>HORIZON-CL5-2027-07-D3-28</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Advanced Distribution Management Systems (ADSM) for more efficient and flexible distribution grids</t>
+          <t>Community of practice - Data-Driven Decision-Making in Energy</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>Innovation Actions</t>
+          <t>Coordination and Support Actions</t>
         </is>
       </c>
       <c r="I22" s="10" t="inlineStr">
@@ -1838,7 +1838,7 @@
       </c>
       <c r="K22" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced reliability, resilience, controllability and efficiency of electricity distribution grids. C</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced EU cooperation to generate knowledge sharing on data and analytics used for the planning and</t>
         </is>
       </c>
       <c r="L22" s="6" t="inlineStr"/>
@@ -1856,12 +1856,12 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-27</t>
+          <t>HORIZON-CL5-2027-07-D3-16</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Integrated Approaches for Retrofitting Infrastructures with Innovative Energy Storage Technologies</t>
+          <t>Industrial processes and equipment for innovative, reliable and scalable tandem technologies (EUPI-PV Partnership)</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -1901,7 +1901,7 @@
       </c>
       <c r="K23" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Improved energy security of the energy system by offering cost-effective and efficient solutions for </t>
+          <t>Expected Outcome:The REPowerEU plan and the EU Solar Energy Strategy introduced targets for the deployment of solar PV amounting to 600 GWac by 2030. Complying with these targets will be crucial for t</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr"/>
@@ -1919,12 +1919,12 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-28</t>
+          <t>HORIZON-CL5-2027-07-D3-25</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Community of practice - Data-Driven Decision-Making in Energy</t>
+          <t>Advanced TSO control rooms to enhance grid observability, stability and resilience</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
@@ -1949,7 +1949,7 @@
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>Coordination and Support Actions</t>
+          <t>Innovation Actions</t>
         </is>
       </c>
       <c r="I24" s="10" t="inlineStr">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="K24" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced EU cooperation to generate knowledge sharing on data and analytics used for the planning and</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced reliability, resilience, and efficiency of electricity transmission grids. Grid congestion i</t>
         </is>
       </c>
       <c r="L24" s="6" t="inlineStr"/>
@@ -1982,12 +1982,12 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-25</t>
+          <t>HORIZON-CL5-2027-07-D3-17</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Advanced TSO control rooms to enhance grid observability, stability and resilience</t>
+          <t>PV based electrification of the economy: Designing &amp; optimising PV systems supporting industrial electrification and promoting participation in electricity markets (EUPI-PV Partnership)</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -2027,7 +2027,7 @@
       </c>
       <c r="K25" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced reliability, resilience, and efficiency of electricity transmission grids. Grid congestion i</t>
+          <t>Expected Outcome:Large PV systems such as utility scale PV are evolving towards higher voltage architecture (&amp;gt;=3kV) with the objective to minimize losses and improve system efficiency at lower cost</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr"/>
@@ -2045,12 +2045,12 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-17</t>
+          <t>HORIZON-CL5-2027-07-D3-11</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>PV based electrification of the economy: Designing &amp; optimising PV systems supporting industrial electrification and promoting participation in electricity markets (EUPI-PV Partnership)</t>
+          <t>Demonstration of hydropower technologies for efficient and forward-looking refurbishment of existing hydropower plants</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
@@ -2090,7 +2090,7 @@
       </c>
       <c r="K26" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Large PV systems such as utility scale PV are evolving towards higher voltage architecture (&amp;gt;=3kV) with the objective to minimize losses and improve system efficiency at lower cost</t>
+          <t>Expected Outcome:For a renewables-based electricity system sufficient flexible and also in the long-run fully sustainable hydropower capacity is pivotal.Project results are expected to contribute to a</t>
         </is>
       </c>
       <c r="L26" s="6" t="inlineStr"/>
@@ -3242,12 +3242,12 @@
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-08</t>
+          <t>HORIZON-CL5-2027-02-D3-31</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>Co-funding Strategic Energy Technology (SET) Plan renewable fuel value chains at EU, national, regional, and local level</t>
+          <t>Support to the implementation of an EU policy framework for CO2 transport and storage infrastructure</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
@@ -3272,7 +3272,7 @@
       </c>
       <c r="H45" s="6" t="inlineStr">
         <is>
-          <t>Programme Cofund Actions</t>
+          <t>Coordination and Support Actions</t>
         </is>
       </c>
       <c r="I45" s="10" t="inlineStr">
@@ -3287,7 +3287,7 @@
       </c>
       <c r="K45" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Advance in the realisation of the Strategic Energy Technology (SET) Plan Action of Renewable fuels</t>
+          <t>Expected Outcome:Project results are expected to contribute to the following outcome:Stakeholders involved in the CO2 infrastructure network are in a position to implement the upcoming legislative fra</t>
         </is>
       </c>
       <c r="L45" s="6" t="inlineStr"/>
@@ -3305,12 +3305,12 @@
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-09</t>
+          <t>HORIZON-CL5-2027-02-D3-24</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Innovative technologies and solutions to improve wave and tidal energy systems</t>
+          <t>Large scale operational validation and upscaling of state-of-the-art (Generative) AI tools and models powering a next generation digital energy system</t>
         </is>
       </c>
       <c r="D46" s="6" t="inlineStr">
@@ -3350,7 +3350,7 @@
       </c>
       <c r="K46" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all following expected outcomes:Advance in the realisation of the Strategic Energy Technology (SET) Plan’s research and innovation priori</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Advanced, secure frugal (energy-, resource-, data- and cost-efficient, sustainable) AI tools for real</t>
         </is>
       </c>
       <c r="L46" s="6" t="inlineStr"/>
@@ -3431,12 +3431,12 @@
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-24</t>
+          <t>HORIZON-CL5-2027-02-D3-15</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Large scale operational validation and upscaling of state-of-the-art (Generative) AI tools and models powering a next generation digital energy system</t>
+          <t>Production technologies for solar photovoltaics beyond the state-of-the-art (EUPI-PV Partnership)</t>
         </is>
       </c>
       <c r="D48" s="6" t="inlineStr">
@@ -3476,7 +3476,7 @@
       </c>
       <c r="K48" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Advanced, secure frugal (energy-, resource-, data- and cost-efficient, sustainable) AI tools for real</t>
+          <t>Expected Outcome:The REPowerEU plan and the EU Solar Energy Strategy introduced targets for the deployment of solar PV amounting to 600 GWac by 2030. Complying with these targets will be crucial for t</t>
         </is>
       </c>
       <c r="L48" s="6" t="inlineStr"/>
@@ -3494,12 +3494,12 @@
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-31</t>
+          <t>HORIZON-CL5-2027-02-D3-07</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>Support to the implementation of an EU policy framework for CO2 transport and storage infrastructure</t>
+          <t>Concentrated solar thermal systems for decarbonising industrial processes</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
@@ -3524,7 +3524,7 @@
       </c>
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>Coordination and Support Actions</t>
+          <t>Innovation Actions</t>
         </is>
       </c>
       <c r="I49" s="10" t="inlineStr">
@@ -3539,7 +3539,7 @@
       </c>
       <c r="K49" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to the following outcome:Stakeholders involved in the CO2 infrastructure network are in a position to implement the upcoming legislative fra</t>
+          <t>Expected Outcome:Renewable heating can be directly used to efficiently decarbonise industrial processes. Concentrated solar thermal technologies offer a great potential to supply renewable heat for in</t>
         </is>
       </c>
       <c r="L49" s="6" t="inlineStr"/>
@@ -3557,12 +3557,12 @@
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-15</t>
+          <t>HORIZON-CL5-2027-02-D3-08</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>Production technologies for solar photovoltaics beyond the state-of-the-art (EUPI-PV Partnership)</t>
+          <t>Co-funding Strategic Energy Technology (SET) Plan renewable fuel value chains at EU, national, regional, and local level</t>
         </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>Innovation Actions</t>
+          <t>Programme Cofund Actions</t>
         </is>
       </c>
       <c r="I50" s="10" t="inlineStr">
@@ -3602,7 +3602,7 @@
       </c>
       <c r="K50" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:The REPowerEU plan and the EU Solar Energy Strategy introduced targets for the deployment of solar PV amounting to 600 GWac by 2030. Complying with these targets will be crucial for t</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Advance in the realisation of the Strategic Energy Technology (SET) Plan Action of Renewable fuels</t>
         </is>
       </c>
       <c r="L50" s="6" t="inlineStr"/>
@@ -4407,17 +4407,17 @@
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>BDNS-904269</t>
+          <t>BDNS-904802</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>Ayudas económicas municipales al fomento del empleo estable y de calidad en Vitoria-Gasteiz, para personas mayores de 45  años, para el ejercicio 2026</t>
+          <t>Mondragón Goi Eskola Politeknikoa Enpresa Digitala C12</t>
         </is>
       </c>
       <c r="D68" s="6" t="inlineStr">
         <is>
-          <t>VITORIA-GASTEIZ</t>
+          <t>PAÍS VASCO</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
@@ -4425,14 +4425,10 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="F68" s="6" t="inlineStr">
-        <is>
-          <t>20/09/2026</t>
-        </is>
-      </c>
+      <c r="F68" s="6" t="inlineStr"/>
       <c r="G68" s="6" t="inlineStr">
         <is>
-          <t>600,000.00 EUR</t>
+          <t>465,000.00 EUR</t>
         </is>
       </c>
       <c r="H68" s="6" t="inlineStr">
@@ -4440,50 +4436,110 @@
           <t>Subvencion Nacional</t>
         </is>
       </c>
-      <c r="I68" s="8" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
+      <c r="I68" s="12" t="inlineStr">
+        <is>
+          <t>MUY ALTA</t>
         </is>
       </c>
       <c r="J68" s="6" t="inlineStr"/>
       <c r="K68" s="6" t="inlineStr">
         <is>
-          <t>PYME Y PERSONAS FÍSICAS QUE DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
-        </is>
-      </c>
-      <c r="L68" s="6" t="inlineStr"/>
+          <t>PERSONAS JURÍDICAS QUE NO DESARROLLAN ACTIVIDAD ECONÓMICA. MRR - MECANISMO DE RECUPERACIÓN Y RESILIENCIA. Regiones: ES21 - PAIS VASCO</t>
+        </is>
+      </c>
+      <c r="L68" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
       <c r="M68" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
         </is>
       </c>
     </row>
-    <row r="69" ht="28" customHeight="1">
-      <c r="A69" s="15" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
+    <row r="69" ht="40" customHeight="1">
+      <c r="A69" s="14" t="inlineStr">
+        <is>
+          <t>España</t>
+        </is>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>BDNS-904604</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>CONVENIO DE SUBVENCIÓN NOMINATIVA ENTRE EL AYUNTAMIENTO DE VITORIA-GASTEIZ Y LA ASOCIACIÓN DE REINSERCIÓN SOCIAL SARTU- ÁLAVA PARA EL DESARROLLO DEL PROYECTO SAREGUNE 2026, PARA LA REVITALIZACIÓN E IN</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>VITORIA-GASTEIZ</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="inlineStr">
+        <is>
+          <t>31/12/2026</t>
+        </is>
+      </c>
+      <c r="G69" s="6" t="inlineStr">
+        <is>
+          <t>66,000.00 EUR</t>
+        </is>
+      </c>
+      <c r="H69" s="6" t="inlineStr">
+        <is>
+          <t>Subvencion Nacional</t>
+        </is>
+      </c>
+      <c r="I69" s="12" t="inlineStr">
+        <is>
+          <t>MUY ALTA</t>
+        </is>
+      </c>
+      <c r="J69" s="6" t="inlineStr"/>
+      <c r="K69" s="6" t="inlineStr">
+        <is>
+          <t>PERSONAS JURÍDICAS QUE NO DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
+        </is>
+      </c>
+      <c r="L69" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M69" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
         </is>
       </c>
     </row>
     <row r="70" ht="40" customHeight="1">
-      <c r="A70" s="16" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
+      <c r="A70" s="14" t="inlineStr">
+        <is>
+          <t>España</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>EUS-97378</t>
+          <t>BDNS-904545</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>BANCO DE HIDRÓGENO Y FONDO DE INNOVACIÓN: son parte de los instrumentos mediante los que la UE ha adjudicado nuevas ayudas a proyectos de I+D y producción ecológica de este combustible renovable, impl</t>
+          <t>CONVENIO DE SUBVENCIÓN NOMINATIVA ENTRE EL AYUNTAMIENTO DE VITORIA-GASTEIZ Y LA FUNDACIÓN CATEDRAL DE SANTA MARÍA. PROGRAMA DE VISITAS GUIADAS A LA MURALLA MEDIEVAL AÑO 2026</t>
         </is>
       </c>
       <c r="D70" s="6" t="inlineStr">
         <is>
-          <t>Euskadi</t>
+          <t>VITORIA-GASTEIZ</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
@@ -4491,25 +4547,33 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="F70" s="6" t="inlineStr"/>
-      <c r="G70" s="6" t="inlineStr"/>
+      <c r="F70" s="6" t="inlineStr">
+        <is>
+          <t>31/12/2026</t>
+        </is>
+      </c>
+      <c r="G70" s="6" t="inlineStr">
+        <is>
+          <t>32,000.00 EUR</t>
+        </is>
+      </c>
       <c r="H70" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
-        </is>
-      </c>
-      <c r="I70" s="11" t="inlineStr">
-        <is>
-          <t>ALTA</t>
+          <t>Subvencion Nacional</t>
+        </is>
+      </c>
+      <c r="I70" s="12" t="inlineStr">
+        <is>
+          <t>MUY ALTA</t>
         </is>
       </c>
       <c r="J70" s="6" t="inlineStr"/>
       <c r="K70" s="6" t="inlineStr">
         <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="L70" s="17" t="inlineStr">
+          <t>PERSONAS JURÍDICAS QUE NO DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
+        </is>
+      </c>
+      <c r="L70" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4520,75 +4584,27 @@
         </is>
       </c>
     </row>
-    <row r="71" ht="40" customHeight="1">
+    <row r="71" ht="28" customHeight="1">
       <c r="A71" s="16" t="inlineStr">
         <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="40" customHeight="1">
+      <c r="A72" s="17" t="inlineStr">
+        <is>
           <t>Euskadi</t>
         </is>
       </c>
-      <c r="B71" s="6" t="inlineStr">
-        <is>
-          <t>EUS-04117</t>
-        </is>
-      </c>
-      <c r="C71" s="6" t="inlineStr">
-        <is>
-          <t>NEB, Nueva Bauhaus Europea. Convocatoria para barrios estéticos, inclusivos, sostenibles y con vivienda asequible, con financiación del marco Horizon de I+D y otros programas. Áreas de ecología-inclus</t>
-        </is>
-      </c>
-      <c r="D71" s="6" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
-      <c r="E71" s="7" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F71" s="6" t="inlineStr"/>
-      <c r="G71" s="6" t="inlineStr"/>
-      <c r="H71" s="6" t="inlineStr">
-        <is>
-          <t>Ayuda/Subvencion Euskadi</t>
-        </is>
-      </c>
-      <c r="I71" s="11" t="inlineStr">
-        <is>
-          <t>ALTA</t>
-        </is>
-      </c>
-      <c r="J71" s="6" t="inlineStr"/>
-      <c r="K71" s="6" t="inlineStr">
-        <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
-        </is>
-      </c>
-      <c r="L71" s="17" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="M71" s="9" t="inlineStr">
-        <is>
-          <t>Ver</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="40" customHeight="1">
-      <c r="A72" s="16" t="inlineStr">
-        <is>
-          <t>Euskadi</t>
-        </is>
-      </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>EUS-87863</t>
+          <t>EUS-85014</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>Elige Europa para la Ciencia: primeras 16 carreras apoyadas con la fórmula innovadora de financiar a las universidades de residencia. Inteligencia artificial, biomedicina, robótica, genómica, clima, e</t>
+          <t>Contrato Reservado a Centros Especiales de Empleo, de conformidad con la Disposición Adicional Cuarta de la Ley 9/2017, de 8 de noviembre, de Contratos del Sector Público, para la prestación del servi</t>
         </is>
       </c>
       <c r="D72" s="6" t="inlineStr">
@@ -4605,12 +4621,12 @@
       <c r="G72" s="6" t="inlineStr"/>
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
-        </is>
-      </c>
-      <c r="I72" s="11" t="inlineStr">
-        <is>
-          <t>ALTA</t>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I72" s="12" t="inlineStr">
+        <is>
+          <t>MUY ALTA</t>
         </is>
       </c>
       <c r="J72" s="6" t="inlineStr"/>
@@ -4619,7 +4635,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L72" s="17" t="inlineStr">
+      <c r="L72" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4631,19 +4647,19 @@
       </c>
     </row>
     <row r="73" ht="40" customHeight="1">
-      <c r="A73" s="16" t="inlineStr">
+      <c r="A73" s="17" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>EUS-85070</t>
+          <t>EUS-26962</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>LIFE 2026. Medio ambiente. Ayudas de 4 subprogramas, de naturaleza y biodiversidad, circularidad y calidad de vida, cambio climático y transición energética. Con inscripción abierta para jornadas info</t>
+          <t>BANCO DE HIDRÓGENO Y FONDO DE INNOVACIÓN: son parte de los instrumentos mediante los que la UE ha adjudicado nuevas ayudas a proyectos de I+D y producción ecológica de este combustible renovable, impl</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
@@ -4674,7 +4690,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L73" s="17" t="inlineStr">
+      <c r="L73" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4686,19 +4702,19 @@
       </c>
     </row>
     <row r="74" ht="40" customHeight="1">
-      <c r="A74" s="16" t="inlineStr">
+      <c r="A74" s="17" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>EUS-86334</t>
+          <t>EUS-99909</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>Enajenación mediante subasta de diversos materiales que se encuentran en el almacén municipal para su achatarramiento y tratamiento como residuos sólidos urbanos</t>
+          <t>NEB, Nueva Bauhaus Europea. Convocatoria para barrios estéticos, inclusivos, sostenibles y con vivienda asequible, con financiación del marco Horizon de I+D y otros programas. Áreas de ecología-inclus</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr">
@@ -4715,7 +4731,7 @@
       <c r="G74" s="6" t="inlineStr"/>
       <c r="H74" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="I74" s="11" t="inlineStr">
@@ -4729,7 +4745,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L74" s="17" t="inlineStr">
+      <c r="L74" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4741,19 +4757,19 @@
       </c>
     </row>
     <row r="75" ht="40" customHeight="1">
-      <c r="A75" s="16" t="inlineStr">
+      <c r="A75" s="17" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>EUS-05833</t>
+          <t>EUS-02372</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>I+D.  Red Eureka, o programas financiados por el marco de innovación Horizon, como Eurostars (pymes) PRIMA (Mediterráneo) CETP (Energía) o DUT (Transformación Urbana). Evento del 12.05.26 sobre consor</t>
+          <t>Elige Europa para la Ciencia: primeras 16 carreras apoyadas con la fórmula innovadora de financiar a las universidades de residencia. Inteligencia artificial, biomedicina, robótica, genómica, clima, e</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
@@ -4773,9 +4789,9 @@
           <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
-      <c r="I75" s="8" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
+      <c r="I75" s="11" t="inlineStr">
+        <is>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="J75" s="6" t="inlineStr"/>
@@ -4784,7 +4800,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L75" s="17" t="inlineStr">
+      <c r="L75" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4796,19 +4812,19 @@
       </c>
     </row>
     <row r="76" ht="40" customHeight="1">
-      <c r="A76" s="16" t="inlineStr">
+      <c r="A76" s="17" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>EUS-20593</t>
+          <t>EUS-59698</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>CEF-E. Línea de infraestructuras energéticas del Mecanismo Conectar Europa. Alineado con planes de Redes Transeuropeas (RTE-E) plan de choque anticrisis de la Unión de la Energía (AccelerateEU). Proye</t>
+          <t>LIFE 2026. Medio ambiente. Ayudas de 4 subprogramas, de naturaleza y biodiversidad, circularidad y calidad de vida, cambio climático y transición energética. Con inscripción abierta para jornadas info</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr">
@@ -4828,9 +4844,9 @@
           <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
-      <c r="I76" s="8" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
+      <c r="I76" s="11" t="inlineStr">
+        <is>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="J76" s="6" t="inlineStr"/>
@@ -4839,7 +4855,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L76" s="17" t="inlineStr">
+      <c r="L76" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4851,19 +4867,19 @@
       </c>
     </row>
     <row r="77" ht="40" customHeight="1">
-      <c r="A77" s="16" t="inlineStr">
+      <c r="A77" s="17" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>EUS-82373</t>
+          <t>EUS-09274</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta el 01.10.26. Cribado de enfermedades con inteligencia artificial. Espacio de Datos Sanitarios de la UE. Red de Centros para Seguridad de la I</t>
+          <t>Campaña de información y sensibilización sobre mejora del sistema de recogida selectiva de residuos</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
@@ -4880,12 +4896,12 @@
       <c r="G77" s="6" t="inlineStr"/>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
-        </is>
-      </c>
-      <c r="I77" s="8" t="inlineStr">
-        <is>
-          <t>MEDIA</t>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I77" s="11" t="inlineStr">
+        <is>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="J77" s="6" t="inlineStr"/>
@@ -4894,7 +4910,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L77" s="17" t="inlineStr">
+      <c r="L77" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4906,19 +4922,19 @@
       </c>
     </row>
     <row r="78" ht="40" customHeight="1">
-      <c r="A78" s="16" t="inlineStr">
+      <c r="A78" s="17" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>EUS-56939</t>
+          <t>EUS-77428</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>Adquisición de paraguas corporativos del 90 aniversario del Gobierno Vasco</t>
+          <t>I+D.  Red Eureka, o programas financiados por el marco de innovación Horizon, como Eurostars (pymes) PRIMA (Mediterráneo) CETP (Energía) o DUT (Transformación Urbana). Evento del 12.05.26 sobre consor</t>
         </is>
       </c>
       <c r="D78" s="6" t="inlineStr">
@@ -4935,7 +4951,7 @@
       <c r="G78" s="6" t="inlineStr"/>
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="I78" s="8" t="inlineStr">
@@ -4949,7 +4965,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L78" s="17" t="inlineStr">
+      <c r="L78" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -4961,19 +4977,19 @@
       </c>
     </row>
     <row r="79" ht="40" customHeight="1">
-      <c r="A79" s="16" t="inlineStr">
+      <c r="A79" s="17" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>EUS-37445</t>
+          <t>EUS-23728</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>Suministro, instalación y puesta en marcha de un conjunto de grupos electrógenos y depósitos auxiliares del sistema PEMEL de la red de saneamiento y abastecimiento de Aguas del Añarbe</t>
+          <t>CEF-E. Línea de infraestructuras energéticas del Mecanismo Conectar Europa. Alineado con planes de Redes Transeuropeas (RTE-E) plan de choque anticrisis de la Unión de la Energía (AccelerateEU). Proye</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
@@ -4990,7 +5006,7 @@
       <c r="G79" s="6" t="inlineStr"/>
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="I79" s="8" t="inlineStr">
@@ -5004,7 +5020,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L79" s="17" t="inlineStr">
+      <c r="L79" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -5016,19 +5032,19 @@
       </c>
     </row>
     <row r="80" ht="40" customHeight="1">
-      <c r="A80" s="16" t="inlineStr">
+      <c r="A80" s="17" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>EUS-17618</t>
+          <t>EUS-04696</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>Obras de reparación de la caldera en el colegio Mendiko</t>
+          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta el 01.10.26. Cribado de enfermedades con inteligencia artificial. Espacio de Datos Sanitarios de la UE. Red de Centros para Seguridad de la I</t>
         </is>
       </c>
       <c r="D80" s="6" t="inlineStr">
@@ -5045,7 +5061,7 @@
       <c r="G80" s="6" t="inlineStr"/>
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="I80" s="8" t="inlineStr">
@@ -5059,7 +5075,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L80" s="17" t="inlineStr">
+      <c r="L80" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -5071,19 +5087,19 @@
       </c>
     </row>
     <row r="81" ht="40" customHeight="1">
-      <c r="A81" s="16" t="inlineStr">
+      <c r="A81" s="17" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>EUS-83776</t>
+          <t>EUS-92366</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>Suministro, instalación, puesta en marcha y mantenimiento de un sistema analítico para la determinación de la concentración de compuestos organohalogenados adsorbibles (AOX) en el laboratorio de contr</t>
+          <t>mantenimiento de la sala de calderas de la herri eskola</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
@@ -5114,7 +5130,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L81" s="17" t="inlineStr">
+      <c r="L81" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -5126,19 +5142,19 @@
       </c>
     </row>
     <row r="82" ht="40" customHeight="1">
-      <c r="A82" s="16" t="inlineStr">
+      <c r="A82" s="17" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>EUS-27600</t>
+          <t>EUS-09126</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>Gestión de incidencias en las viviendas dependientes de servicios sociales</t>
+          <t>mantenimiento de la sala de calderas del campo de fútbol de plazeta</t>
         </is>
       </c>
       <c r="D82" s="6" t="inlineStr">
@@ -5169,7 +5185,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L82" s="17" t="inlineStr">
+      <c r="L82" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -5181,19 +5197,19 @@
       </c>
     </row>
     <row r="83" ht="40" customHeight="1">
-      <c r="A83" s="16" t="inlineStr">
+      <c r="A83" s="17" t="inlineStr">
         <is>
           <t>Euskadi</t>
         </is>
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>EUS-44604</t>
+          <t>EUS-15501</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>Trabajos sobrevenidos de renovación integral de zonas verdes aledañas a rampas 1 y 2 bidezabal</t>
+          <t>Cambio del variador del ascensor del frontón astelena por entrada de agua</t>
         </is>
       </c>
       <c r="D83" s="6" t="inlineStr">
@@ -5224,7 +5240,7 @@
           <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
-      <c r="L83" s="17" t="inlineStr">
+      <c r="L83" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
@@ -5235,14 +5251,124 @@
         </is>
       </c>
     </row>
+    <row r="84" ht="40" customHeight="1">
+      <c r="A84" s="17" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>EUS-66632</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="inlineStr">
+        <is>
+          <t>Suministro y instalación de escalera para el acceso al parque de itzio</t>
+        </is>
+      </c>
+      <c r="D84" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E84" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F84" s="6" t="inlineStr"/>
+      <c r="G84" s="6" t="inlineStr"/>
+      <c r="H84" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I84" s="8" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J84" s="6" t="inlineStr"/>
+      <c r="K84" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L84" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M84" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="40" customHeight="1">
+      <c r="A85" s="17" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B85" s="6" t="inlineStr">
+        <is>
+          <t>EUS-69385</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="inlineStr">
+        <is>
+          <t>Limpieza y pintado del muro junto al kiosko de urki</t>
+        </is>
+      </c>
+      <c r="D85" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E85" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F85" s="6" t="inlineStr"/>
+      <c r="G85" s="6" t="inlineStr"/>
+      <c r="H85" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I85" s="8" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J85" s="6" t="inlineStr"/>
+      <c r="K85" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L85" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M85" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:M83"/>
+  <autoFilter ref="A4:M85"/>
   <mergeCells count="5">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A5:M5"/>
     <mergeCell ref="A67:M67"/>
-    <mergeCell ref="A69:M69"/>
     <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A71:M71"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId1"/>
@@ -5307,8 +5433,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M65" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M66" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M68" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M70" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M71" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M69" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M70" r:id="rId64"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M72" r:id="rId65"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M73" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M74" r:id="rId67"/>
@@ -5321,6 +5447,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M81" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M82" r:id="rId75"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M83" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M84" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M85" r:id="rId78"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5332,7 +5460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1139"/>
+  <dimension ref="A1:F1169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7094,7 +7222,7 @@
     <row r="121" ht="30" customHeight="1">
       <c r="A121" s="18" t="inlineStr">
         <is>
-          <t>FICHA 9: HORIZON-CL5-2026-11-D3-04</t>
+          <t>FICHA 9: HORIZON-CL5-2026-11-D3-23</t>
         </is>
       </c>
       <c r="B121" s="19" t="n"/>
@@ -7127,7 +7255,7 @@
       </c>
       <c r="B123" s="21" t="inlineStr">
         <is>
-          <t>De-risking renewable fuel technologies through transnational pre-commercial procurement of renewable fuel industrial value chains</t>
+          <t>Data sharing to support the training and development of AI foundation models in the energy sector</t>
         </is>
       </c>
       <c r="C123" s="22" t="n"/>
@@ -7143,7 +7271,7 @@
       </c>
       <c r="B124" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-04</t>
+          <t>HORIZON-CL5-2026-11-D3-23</t>
         </is>
       </c>
       <c r="C124" s="22" t="n"/>
@@ -7223,7 +7351,7 @@
       </c>
       <c r="B129" s="21" t="inlineStr">
         <is>
-          <t>Pre-commercial Procurement</t>
+          <t>Innovation Actions</t>
         </is>
       </c>
       <c r="C129" s="22" t="n"/>
@@ -7255,7 +7383,7 @@
       </c>
       <c r="B131" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Public authorities, industry, technology providers, energy producers and consumers profit from de-risking of cost-effective essential value chains of those renewable fuel technologies that can contribute to domestic commercial fuel production beyond 2030 customized to their needs, from improved access to better financing exploiting synergies across funding schemes, and from more effective market uptake, business models, increased competitiveness, and commercialization opportunities.Energy prod</t>
+          <t>Expected Outcome:Projects are expected to contribute to all the following expected outcomes:Effective and innovative methods for gathering, sharing and using large data sets in energy applications for the purpose of training AI models while ensuring privacy and security.Advanced and - wherever possible - open-source AI foundation models to support the digitalisation of the energy system, through improved grid observability, forecasting of supply and demand, advanced storage and renewables integration, demand side flexibility and energy efficiency.Enhanced cooperation, knowledge sharing and int</t>
         </is>
       </c>
       <c r="C131" s="22" t="n"/>
@@ -7299,7 +7427,7 @@
       </c>
       <c r="B134" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-04</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-23</t>
         </is>
       </c>
       <c r="C134" s="22" t="n"/>
@@ -7310,7 +7438,7 @@
     <row r="136" ht="30" customHeight="1">
       <c r="A136" s="18" t="inlineStr">
         <is>
-          <t>FICHA 10: HORIZON-CL5-2026-11-D3-05</t>
+          <t>FICHA 10: HORIZON-CL5-2026-11-D3-06</t>
         </is>
       </c>
       <c r="B136" s="19" t="n"/>
@@ -7335,7 +7463,7 @@
       <c r="E137" s="22" t="n"/>
       <c r="F137" s="22" t="n"/>
     </row>
-    <row r="138" ht="45" customHeight="1">
+    <row r="138" ht="20" customHeight="1">
       <c r="A138" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -7343,7 +7471,7 @@
       </c>
       <c r="B138" s="21" t="inlineStr">
         <is>
-          <t>Demonstration of solid biofuel supply and conversion to high efficiency CHP from fully sustainable regional value chains</t>
+          <t>Resource assessment for deep sedimentary and basement reservoirs</t>
         </is>
       </c>
       <c r="C138" s="22" t="n"/>
@@ -7359,7 +7487,7 @@
       </c>
       <c r="B139" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-05</t>
+          <t>HORIZON-CL5-2026-11-D3-06</t>
         </is>
       </c>
       <c r="C139" s="22" t="n"/>
@@ -7439,7 +7567,7 @@
       </c>
       <c r="B144" s="21" t="inlineStr">
         <is>
-          <t>Innovation Actions</t>
+          <t xml:space="preserve"> Research and Innovation Actions</t>
         </is>
       </c>
       <c r="C144" s="22" t="n"/>
@@ -7471,7 +7599,7 @@
       </c>
       <c r="B146" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Fully sustainable regional bioenergy value chains and efficient conversion can play an important role in renewable efficient power and heating generation and for reaching the EU climate and energy targets and contribute to European competitiveness and energy security.Project results are expected to contribute to at all of the following expected outcomes:The demonstration of regional value chains for the use of locally to regionally sourced sustainable and cheap solid biofuel from upgraded biogenic residues and wastes in line with the provisions of the Renewable Energy Directiv</t>
+          <t>Expected Outcome:Deep sedimentary/basement reservoirs are usually characterized by low permeability, high drilling cost and a scarcity of data, as they are typically ignored by hydrocarbon exploration. Major exploration challenges relate to predicting deep sedimentary and basement reservoir structures and properties to identify suitable locations for reservoir-independent approaches, capable of overcoming the low permeability obstacle, such as Enhanced Geothermal Systems (EGS) or closed-loop geothermal systems.Project results are expected to contribute to all of the following expected outcomes</t>
         </is>
       </c>
       <c r="C146" s="22" t="n"/>
@@ -7515,7 +7643,7 @@
       </c>
       <c r="B149" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-05</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-06</t>
         </is>
       </c>
       <c r="C149" s="22" t="n"/>
@@ -7526,7 +7654,7 @@
     <row r="151" ht="30" customHeight="1">
       <c r="A151" s="18" t="inlineStr">
         <is>
-          <t>FICHA 11: HORIZON-CL5-2026-11-D3-23</t>
+          <t>FICHA 11: HORIZON-CL5-2026-11-D3-14</t>
         </is>
       </c>
       <c r="B151" s="19" t="n"/>
@@ -7551,7 +7679,7 @@
       <c r="E152" s="22" t="n"/>
       <c r="F152" s="22" t="n"/>
     </row>
-    <row r="153" ht="45" customHeight="1">
+    <row r="153" ht="20" customHeight="1">
       <c r="A153" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -7559,7 +7687,7 @@
       </c>
       <c r="B153" s="21" t="inlineStr">
         <is>
-          <t>Data sharing to support the training and development of AI foundation models in the energy sector</t>
+          <t>Improved system design for innovative PV applications (EUPI-PV Partnership)</t>
         </is>
       </c>
       <c r="C153" s="22" t="n"/>
@@ -7575,7 +7703,7 @@
       </c>
       <c r="B154" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-23</t>
+          <t>HORIZON-CL5-2026-11-D3-14</t>
         </is>
       </c>
       <c r="C154" s="22" t="n"/>
@@ -7687,7 +7815,7 @@
       </c>
       <c r="B161" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Projects are expected to contribute to all the following expected outcomes:Effective and innovative methods for gathering, sharing and using large data sets in energy applications for the purpose of training AI models while ensuring privacy and security.Advanced and - wherever possible - open-source AI foundation models to support the digitalisation of the energy system, through improved grid observability, forecasting of supply and demand, advanced storage and renewables integration, demand side flexibility and energy efficiency.Enhanced cooperation, knowledge sharing and int</t>
+          <t>Expected Outcome:Agrivoltaics or the co-location of agricultural activity and PV electricity production is a novel form of PV deployment which could provide farmers with diversified revenue sources and ecological benefits, while reducing land use competition, siting restrictions or adverse impacts on biodiversity and agricultural production. Optimizing system designs and business practices will help to enable simultaneous land use creating synergy for both agriculture and electricity production; this can benefit farmers, lower PV costs and enable the European Union to reach the goals of the EU</t>
         </is>
       </c>
       <c r="C161" s="22" t="n"/>
@@ -7731,7 +7859,7 @@
       </c>
       <c r="B164" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-23</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-14</t>
         </is>
       </c>
       <c r="C164" s="22" t="n"/>
@@ -7742,7 +7870,7 @@
     <row r="166" ht="30" customHeight="1">
       <c r="A166" s="18" t="inlineStr">
         <is>
-          <t>FICHA 12: HORIZON-CL5-2026-11-D3-06</t>
+          <t>FICHA 12: HORIZON-CL5-2026-11-D3-05</t>
         </is>
       </c>
       <c r="B166" s="19" t="n"/>
@@ -7767,7 +7895,7 @@
       <c r="E167" s="22" t="n"/>
       <c r="F167" s="22" t="n"/>
     </row>
-    <row r="168" ht="20" customHeight="1">
+    <row r="168" ht="45" customHeight="1">
       <c r="A168" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -7775,7 +7903,7 @@
       </c>
       <c r="B168" s="21" t="inlineStr">
         <is>
-          <t>Resource assessment for deep sedimentary and basement reservoirs</t>
+          <t>Demonstration of solid biofuel supply and conversion to high efficiency CHP from fully sustainable regional value chains</t>
         </is>
       </c>
       <c r="C168" s="22" t="n"/>
@@ -7791,7 +7919,7 @@
       </c>
       <c r="B169" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-06</t>
+          <t>HORIZON-CL5-2026-11-D3-05</t>
         </is>
       </c>
       <c r="C169" s="22" t="n"/>
@@ -7871,7 +7999,7 @@
       </c>
       <c r="B174" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Research and Innovation Actions</t>
+          <t>Innovation Actions</t>
         </is>
       </c>
       <c r="C174" s="22" t="n"/>
@@ -7903,7 +8031,7 @@
       </c>
       <c r="B176" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Deep sedimentary/basement reservoirs are usually characterized by low permeability, high drilling cost and a scarcity of data, as they are typically ignored by hydrocarbon exploration. Major exploration challenges relate to predicting deep sedimentary and basement reservoir structures and properties to identify suitable locations for reservoir-independent approaches, capable of overcoming the low permeability obstacle, such as Enhanced Geothermal Systems (EGS) or closed-loop geothermal systems.Project results are expected to contribute to all of the following expected outcomes</t>
+          <t>Expected Outcome:Fully sustainable regional bioenergy value chains and efficient conversion can play an important role in renewable efficient power and heating generation and for reaching the EU climate and energy targets and contribute to European competitiveness and energy security.Project results are expected to contribute to at all of the following expected outcomes:The demonstration of regional value chains for the use of locally to regionally sourced sustainable and cheap solid biofuel from upgraded biogenic residues and wastes in line with the provisions of the Renewable Energy Directiv</t>
         </is>
       </c>
       <c r="C176" s="22" t="n"/>
@@ -7947,7 +8075,7 @@
       </c>
       <c r="B179" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-06</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-05</t>
         </is>
       </c>
       <c r="C179" s="22" t="n"/>
@@ -7958,7 +8086,7 @@
     <row r="181" ht="30" customHeight="1">
       <c r="A181" s="18" t="inlineStr">
         <is>
-          <t>FICHA 13: HORIZON-CL5-2026-11-D3-14</t>
+          <t>FICHA 13: HORIZON-CL5-2026-11-D3-04</t>
         </is>
       </c>
       <c r="B181" s="19" t="n"/>
@@ -7983,7 +8111,7 @@
       <c r="E182" s="22" t="n"/>
       <c r="F182" s="22" t="n"/>
     </row>
-    <row r="183" ht="20" customHeight="1">
+    <row r="183" ht="45" customHeight="1">
       <c r="A183" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -7991,7 +8119,7 @@
       </c>
       <c r="B183" s="21" t="inlineStr">
         <is>
-          <t>Improved system design for innovative PV applications (EUPI-PV Partnership)</t>
+          <t>De-risking renewable fuel technologies through transnational pre-commercial procurement of renewable fuel industrial value chains</t>
         </is>
       </c>
       <c r="C183" s="22" t="n"/>
@@ -8007,7 +8135,7 @@
       </c>
       <c r="B184" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-14</t>
+          <t>HORIZON-CL5-2026-11-D3-04</t>
         </is>
       </c>
       <c r="C184" s="22" t="n"/>
@@ -8087,7 +8215,7 @@
       </c>
       <c r="B189" s="21" t="inlineStr">
         <is>
-          <t>Innovation Actions</t>
+          <t>Pre-commercial Procurement</t>
         </is>
       </c>
       <c r="C189" s="22" t="n"/>
@@ -8119,7 +8247,7 @@
       </c>
       <c r="B191" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Agrivoltaics or the co-location of agricultural activity and PV electricity production is a novel form of PV deployment which could provide farmers with diversified revenue sources and ecological benefits, while reducing land use competition, siting restrictions or adverse impacts on biodiversity and agricultural production. Optimizing system designs and business practices will help to enable simultaneous land use creating synergy for both agriculture and electricity production; this can benefit farmers, lower PV costs and enable the European Union to reach the goals of the EU</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Public authorities, industry, technology providers, energy producers and consumers profit from de-risking of cost-effective essential value chains of those renewable fuel technologies that can contribute to domestic commercial fuel production beyond 2030 customized to their needs, from improved access to better financing exploiting synergies across funding schemes, and from more effective market uptake, business models, increased competitiveness, and commercialization opportunities.Energy prod</t>
         </is>
       </c>
       <c r="C191" s="22" t="n"/>
@@ -8163,7 +8291,7 @@
       </c>
       <c r="B194" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-14</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2026-11-D3-04</t>
         </is>
       </c>
       <c r="C194" s="22" t="n"/>
@@ -8174,7 +8302,7 @@
     <row r="196" ht="30" customHeight="1">
       <c r="A196" s="18" t="inlineStr">
         <is>
-          <t>FICHA 14: HORIZON-CL5-2027-07-D3-16</t>
+          <t>FICHA 14: HORIZON-CL5-2027-07-D3-27</t>
         </is>
       </c>
       <c r="B196" s="19" t="n"/>
@@ -8207,7 +8335,7 @@
       </c>
       <c r="B198" s="21" t="inlineStr">
         <is>
-          <t>Industrial processes and equipment for innovative, reliable and scalable tandem technologies (EUPI-PV Partnership)</t>
+          <t>Integrated Approaches for Retrofitting Infrastructures with Innovative Energy Storage Technologies</t>
         </is>
       </c>
       <c r="C198" s="22" t="n"/>
@@ -8223,7 +8351,7 @@
       </c>
       <c r="B199" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-16</t>
+          <t>HORIZON-CL5-2027-07-D3-27</t>
         </is>
       </c>
       <c r="C199" s="22" t="n"/>
@@ -8335,7 +8463,7 @@
       </c>
       <c r="B206" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:The REPowerEU plan and the EU Solar Energy Strategy introduced targets for the deployment of solar PV amounting to 600 GWac by 2030. Complying with these targets will be crucial for the European Union to reach its climate targets and free itself from import dependency on fossil fuels and the costs this imposes on Europe’s competitiveness in terms of high energy prices. The Solar Strategy also introduces a target, which has been enshrined into the Net-Zero Industry Act, to re-consolidate the European solar manufacturing sector and scale up European manufacturing capacity across</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Improved energy security of the energy system by offering cost-effective and efficient solutions for additional diverse and flexible energy storage capacities.Improve the sustainability and circularity of energy storage systems.Enhanced economic viability of energy storage by utilizing existing infrastructures.  Scope:Demonstration of novel or improved technological solutions for cost-efficient, circular and sustainable energy storage, which contribute to grid flexibility and make use of existing</t>
         </is>
       </c>
       <c r="C206" s="22" t="n"/>
@@ -8379,7 +8507,7 @@
       </c>
       <c r="B209" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-16</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-27</t>
         </is>
       </c>
       <c r="C209" s="22" t="n"/>
@@ -8390,7 +8518,7 @@
     <row r="211" ht="30" customHeight="1">
       <c r="A211" s="18" t="inlineStr">
         <is>
-          <t>FICHA 15: HORIZON-CL5-2027-07-D3-11</t>
+          <t>FICHA 15: HORIZON-CL5-2027-07-D3-26</t>
         </is>
       </c>
       <c r="B211" s="19" t="n"/>
@@ -8423,7 +8551,7 @@
       </c>
       <c r="B213" s="21" t="inlineStr">
         <is>
-          <t>Demonstration of hydropower technologies for efficient and forward-looking refurbishment of existing hydropower plants</t>
+          <t>Advanced Distribution Management Systems (ADSM) for more efficient and flexible distribution grids</t>
         </is>
       </c>
       <c r="C213" s="22" t="n"/>
@@ -8439,7 +8567,7 @@
       </c>
       <c r="B214" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-11</t>
+          <t>HORIZON-CL5-2027-07-D3-26</t>
         </is>
       </c>
       <c r="C214" s="22" t="n"/>
@@ -8551,7 +8679,7 @@
       </c>
       <c r="B221" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:For a renewables-based electricity system sufficient flexible and also in the long-run fully sustainable hydropower capacity is pivotal.Project results are expected to contribute to all of the following expected outcomes:Enhancing the capacities of the hydropower fleet to contribute with variable renewables base load to a secure and stable electricity system, including by modernising grid integration and hydropower fleet control.Increase technology leadership, competitiveness and technology export potential of European hydropower industry.Address challenges of climate change a</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced reliability, resilience, controllability and efficiency of electricity distribution grids. Congestion in distribution grids is managed effectively;Distribution system operators (DSO) leverage modern digital solutions and employ improved systems to effectively manage their grids and improve interoperability with TSOs and other DSOs;Vendor-agnostic reference architectures, solutions and tools are developed to help advancing the ADSM design and operation and effectively manage a broad range</t>
         </is>
       </c>
       <c r="C221" s="22" t="n"/>
@@ -8595,7 +8723,7 @@
       </c>
       <c r="B224" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-11</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-26</t>
         </is>
       </c>
       <c r="C224" s="22" t="n"/>
@@ -8822,7 +8950,7 @@
     <row r="241" ht="30" customHeight="1">
       <c r="A241" s="18" t="inlineStr">
         <is>
-          <t>FICHA 17: HORIZON-CL5-2027-07-D3-26</t>
+          <t>FICHA 17: HORIZON-CL5-2027-07-D3-28</t>
         </is>
       </c>
       <c r="B241" s="19" t="n"/>
@@ -8847,7 +8975,7 @@
       <c r="E242" s="22" t="n"/>
       <c r="F242" s="22" t="n"/>
     </row>
-    <row r="243" ht="45" customHeight="1">
+    <row r="243" ht="20" customHeight="1">
       <c r="A243" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -8855,7 +8983,7 @@
       </c>
       <c r="B243" s="21" t="inlineStr">
         <is>
-          <t>Advanced Distribution Management Systems (ADSM) for more efficient and flexible distribution grids</t>
+          <t>Community of practice - Data-Driven Decision-Making in Energy</t>
         </is>
       </c>
       <c r="C243" s="22" t="n"/>
@@ -8871,7 +8999,7 @@
       </c>
       <c r="B244" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-26</t>
+          <t>HORIZON-CL5-2027-07-D3-28</t>
         </is>
       </c>
       <c r="C244" s="22" t="n"/>
@@ -8951,7 +9079,7 @@
       </c>
       <c r="B249" s="21" t="inlineStr">
         <is>
-          <t>Innovation Actions</t>
+          <t>Coordination and Support Actions</t>
         </is>
       </c>
       <c r="C249" s="22" t="n"/>
@@ -8983,7 +9111,7 @@
       </c>
       <c r="B251" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced reliability, resilience, controllability and efficiency of electricity distribution grids. Congestion in distribution grids is managed effectively;Distribution system operators (DSO) leverage modern digital solutions and employ improved systems to effectively manage their grids and improve interoperability with TSOs and other DSOs;Vendor-agnostic reference architectures, solutions and tools are developed to help advancing the ADSM design and operation and effectively manage a broad range</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced EU cooperation to generate knowledge sharing on data and analytics used for the planning and operation of European grids, and market integration;Better EU coordination with regard to planning and simulation tools to support the development of electricity grids and integration of RES are made available to the research, academia, grid operators, and key actors in the energy value chains;Coordinated processes to generate new and innovative open-source solutions, software modules etc. that a</t>
         </is>
       </c>
       <c r="C251" s="22" t="n"/>
@@ -9027,7 +9155,7 @@
       </c>
       <c r="B254" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-26</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-28</t>
         </is>
       </c>
       <c r="C254" s="22" t="n"/>
@@ -9038,7 +9166,7 @@
     <row r="256" ht="30" customHeight="1">
       <c r="A256" s="18" t="inlineStr">
         <is>
-          <t>FICHA 18: HORIZON-CL5-2027-07-D3-27</t>
+          <t>FICHA 18: HORIZON-CL5-2027-07-D3-16</t>
         </is>
       </c>
       <c r="B256" s="19" t="n"/>
@@ -9071,7 +9199,7 @@
       </c>
       <c r="B258" s="21" t="inlineStr">
         <is>
-          <t>Integrated Approaches for Retrofitting Infrastructures with Innovative Energy Storage Technologies</t>
+          <t>Industrial processes and equipment for innovative, reliable and scalable tandem technologies (EUPI-PV Partnership)</t>
         </is>
       </c>
       <c r="C258" s="22" t="n"/>
@@ -9087,7 +9215,7 @@
       </c>
       <c r="B259" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-27</t>
+          <t>HORIZON-CL5-2027-07-D3-16</t>
         </is>
       </c>
       <c r="C259" s="22" t="n"/>
@@ -9199,7 +9327,7 @@
       </c>
       <c r="B266" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Improved energy security of the energy system by offering cost-effective and efficient solutions for additional diverse and flexible energy storage capacities.Improve the sustainability and circularity of energy storage systems.Enhanced economic viability of energy storage by utilizing existing infrastructures.  Scope:Demonstration of novel or improved technological solutions for cost-efficient, circular and sustainable energy storage, which contribute to grid flexibility and make use of existing</t>
+          <t>Expected Outcome:The REPowerEU plan and the EU Solar Energy Strategy introduced targets for the deployment of solar PV amounting to 600 GWac by 2030. Complying with these targets will be crucial for the European Union to reach its climate targets and free itself from import dependency on fossil fuels and the costs this imposes on Europe’s competitiveness in terms of high energy prices. The Solar Strategy also introduces a target, which has been enshrined into the Net-Zero Industry Act, to re-consolidate the European solar manufacturing sector and scale up European manufacturing capacity across</t>
         </is>
       </c>
       <c r="C266" s="22" t="n"/>
@@ -9243,7 +9371,7 @@
       </c>
       <c r="B269" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-27</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-16</t>
         </is>
       </c>
       <c r="C269" s="22" t="n"/>
@@ -9254,7 +9382,7 @@
     <row r="271" ht="30" customHeight="1">
       <c r="A271" s="18" t="inlineStr">
         <is>
-          <t>FICHA 19: HORIZON-CL5-2027-07-D3-28</t>
+          <t>FICHA 19: HORIZON-CL5-2027-07-D3-25</t>
         </is>
       </c>
       <c r="B271" s="19" t="n"/>
@@ -9279,7 +9407,7 @@
       <c r="E272" s="22" t="n"/>
       <c r="F272" s="22" t="n"/>
     </row>
-    <row r="273" ht="20" customHeight="1">
+    <row r="273" ht="45" customHeight="1">
       <c r="A273" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -9287,7 +9415,7 @@
       </c>
       <c r="B273" s="21" t="inlineStr">
         <is>
-          <t>Community of practice - Data-Driven Decision-Making in Energy</t>
+          <t>Advanced TSO control rooms to enhance grid observability, stability and resilience</t>
         </is>
       </c>
       <c r="C273" s="22" t="n"/>
@@ -9303,7 +9431,7 @@
       </c>
       <c r="B274" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-28</t>
+          <t>HORIZON-CL5-2027-07-D3-25</t>
         </is>
       </c>
       <c r="C274" s="22" t="n"/>
@@ -9383,7 +9511,7 @@
       </c>
       <c r="B279" s="21" t="inlineStr">
         <is>
-          <t>Coordination and Support Actions</t>
+          <t>Innovation Actions</t>
         </is>
       </c>
       <c r="C279" s="22" t="n"/>
@@ -9415,7 +9543,7 @@
       </c>
       <c r="B281" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced EU cooperation to generate knowledge sharing on data and analytics used for the planning and operation of European grids, and market integration;Better EU coordination with regard to planning and simulation tools to support the development of electricity grids and integration of RES are made available to the research, academia, grid operators, and key actors in the energy value chains;Coordinated processes to generate new and innovative open-source solutions, software modules etc. that a</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced reliability, resilience, and efficiency of electricity transmission grids. Grid congestion is managed efficiently;Enhanced observability of grids and improved forecasting of supply, demand, grid capacity availability, and flexibility;Transmission system operators (TSO) leverage modern digital solutions and employ improved systems to effectively manage their grids and improve interoperability with other TSOs;Vendor-agnostic reference architectures, solutions and tools are developed to hel</t>
         </is>
       </c>
       <c r="C281" s="22" t="n"/>
@@ -9459,7 +9587,7 @@
       </c>
       <c r="B284" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-28</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-25</t>
         </is>
       </c>
       <c r="C284" s="22" t="n"/>
@@ -9470,7 +9598,7 @@
     <row r="286" ht="30" customHeight="1">
       <c r="A286" s="18" t="inlineStr">
         <is>
-          <t>FICHA 20: HORIZON-CL5-2027-07-D3-25</t>
+          <t>FICHA 20: HORIZON-CL5-2027-07-D3-17</t>
         </is>
       </c>
       <c r="B286" s="19" t="n"/>
@@ -9503,7 +9631,7 @@
       </c>
       <c r="B288" s="21" t="inlineStr">
         <is>
-          <t>Advanced TSO control rooms to enhance grid observability, stability and resilience</t>
+          <t>PV based electrification of the economy: Designing &amp; optimising PV systems supporting industrial electrification and promoting participation in electricity markets (EUPI-PV Partnership)</t>
         </is>
       </c>
       <c r="C288" s="22" t="n"/>
@@ -9519,7 +9647,7 @@
       </c>
       <c r="B289" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-25</t>
+          <t>HORIZON-CL5-2027-07-D3-17</t>
         </is>
       </c>
       <c r="C289" s="22" t="n"/>
@@ -9631,7 +9759,7 @@
       </c>
       <c r="B296" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Enhanced reliability, resilience, and efficiency of electricity transmission grids. Grid congestion is managed efficiently;Enhanced observability of grids and improved forecasting of supply, demand, grid capacity availability, and flexibility;Transmission system operators (TSO) leverage modern digital solutions and employ improved systems to effectively manage their grids and improve interoperability with other TSOs;Vendor-agnostic reference architectures, solutions and tools are developed to hel</t>
+          <t>Expected Outcome:Large PV systems such as utility scale PV are evolving towards higher voltage architecture (&amp;gt;=3kV) with the objective to minimize losses and improve system efficiency at lower costs. The intention is to integrate also storage into such (hybrid) PV systems offering flexibility. It is consequently essential to build a blueprint for the implementation of high voltage large PV systems and the development of Direct Current (DC) networks around strategic end users for high voltage demand (industrial sites, servers, electric vehicle charging stations…). Understanding the factors t</t>
         </is>
       </c>
       <c r="C296" s="22" t="n"/>
@@ -9675,7 +9803,7 @@
       </c>
       <c r="B299" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-25</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-17</t>
         </is>
       </c>
       <c r="C299" s="22" t="n"/>
@@ -9686,7 +9814,7 @@
     <row r="301" ht="30" customHeight="1">
       <c r="A301" s="18" t="inlineStr">
         <is>
-          <t>FICHA 21: HORIZON-CL5-2027-07-D3-17</t>
+          <t>FICHA 21: HORIZON-CL5-2027-07-D3-11</t>
         </is>
       </c>
       <c r="B301" s="19" t="n"/>
@@ -9719,7 +9847,7 @@
       </c>
       <c r="B303" s="21" t="inlineStr">
         <is>
-          <t>PV based electrification of the economy: Designing &amp; optimising PV systems supporting industrial electrification and promoting participation in electricity markets (EUPI-PV Partnership)</t>
+          <t>Demonstration of hydropower technologies for efficient and forward-looking refurbishment of existing hydropower plants</t>
         </is>
       </c>
       <c r="C303" s="22" t="n"/>
@@ -9735,7 +9863,7 @@
       </c>
       <c r="B304" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-17</t>
+          <t>HORIZON-CL5-2027-07-D3-11</t>
         </is>
       </c>
       <c r="C304" s="22" t="n"/>
@@ -9847,7 +9975,7 @@
       </c>
       <c r="B311" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Large PV systems such as utility scale PV are evolving towards higher voltage architecture (&amp;gt;=3kV) with the objective to minimize losses and improve system efficiency at lower costs. The intention is to integrate also storage into such (hybrid) PV systems offering flexibility. It is consequently essential to build a blueprint for the implementation of high voltage large PV systems and the development of Direct Current (DC) networks around strategic end users for high voltage demand (industrial sites, servers, electric vehicle charging stations…). Understanding the factors t</t>
+          <t>Expected Outcome:For a renewables-based electricity system sufficient flexible and also in the long-run fully sustainable hydropower capacity is pivotal.Project results are expected to contribute to all of the following expected outcomes:Enhancing the capacities of the hydropower fleet to contribute with variable renewables base load to a secure and stable electricity system, including by modernising grid integration and hydropower fleet control.Increase technology leadership, competitiveness and technology export potential of European hydropower industry.Address challenges of climate change a</t>
         </is>
       </c>
       <c r="C311" s="22" t="n"/>
@@ -9891,7 +10019,7 @@
       </c>
       <c r="B314" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-17</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-07-D3-11</t>
         </is>
       </c>
       <c r="C314" s="22" t="n"/>
@@ -13834,7 +13962,7 @@
     <row r="586" ht="30" customHeight="1">
       <c r="A586" s="18" t="inlineStr">
         <is>
-          <t>FICHA 40: HORIZON-CL5-2027-02-D3-08</t>
+          <t>FICHA 40: HORIZON-CL5-2027-02-D3-31</t>
         </is>
       </c>
       <c r="B586" s="19" t="n"/>
@@ -13867,7 +13995,7 @@
       </c>
       <c r="B588" s="21" t="inlineStr">
         <is>
-          <t>Co-funding Strategic Energy Technology (SET) Plan renewable fuel value chains at EU, national, regional, and local level</t>
+          <t>Support to the implementation of an EU policy framework for CO2 transport and storage infrastructure</t>
         </is>
       </c>
       <c r="C588" s="22" t="n"/>
@@ -13883,7 +14011,7 @@
       </c>
       <c r="B589" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-08</t>
+          <t>HORIZON-CL5-2027-02-D3-31</t>
         </is>
       </c>
       <c r="C589" s="22" t="n"/>
@@ -13963,7 +14091,7 @@
       </c>
       <c r="B594" s="21" t="inlineStr">
         <is>
-          <t>Programme Cofund Actions</t>
+          <t>Coordination and Support Actions</t>
         </is>
       </c>
       <c r="C594" s="22" t="n"/>
@@ -13995,7 +14123,7 @@
       </c>
       <c r="B596" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Advance in the realisation of the Strategic Energy Technology (SET) Plan Action of Renewable fuels and Bioenergy (for the fuels part) is supported, overcoming fragmentation by mobilizing resources and establishing across EU interregional value chains of renewable fuel technologies and by better alignment of public and private R&amp;amp;I priorities and of funding mechanisms.All sector stakeholders benefit from establishment of renewable fuels value chains at EU, national, regional, and local level</t>
+          <t>Expected Outcome:Project results are expected to contribute to the following outcome:Stakeholders involved in the CO2 infrastructure network are in a position to implement the upcoming legislative framework for CO2 infrastructure.  Scope:The project is expected to assist stakeholders involved in the CO2 infrastructure network in implementing the upcoming legislative framework for CO2 infrastructure.Issues to address include market and cost structure, cross-border integration, interoperability and planning, technical harmonisation and investment incentives for new infrastructure, third-party ac</t>
         </is>
       </c>
       <c r="C596" s="22" t="n"/>
@@ -14039,7 +14167,7 @@
       </c>
       <c r="B599" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-08</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-31</t>
         </is>
       </c>
       <c r="C599" s="22" t="n"/>
@@ -14050,7 +14178,7 @@
     <row r="601" ht="30" customHeight="1">
       <c r="A601" s="18" t="inlineStr">
         <is>
-          <t>FICHA 41: HORIZON-CL5-2027-02-D3-09</t>
+          <t>FICHA 41: HORIZON-CL5-2027-02-D3-24</t>
         </is>
       </c>
       <c r="B601" s="19" t="n"/>
@@ -14075,7 +14203,7 @@
       <c r="E602" s="22" t="n"/>
       <c r="F602" s="22" t="n"/>
     </row>
-    <row r="603" ht="20" customHeight="1">
+    <row r="603" ht="45" customHeight="1">
       <c r="A603" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -14083,7 +14211,7 @@
       </c>
       <c r="B603" s="21" t="inlineStr">
         <is>
-          <t>Innovative technologies and solutions to improve wave and tidal energy systems</t>
+          <t>Large scale operational validation and upscaling of state-of-the-art (Generative) AI tools and models powering a next generation digital energy system</t>
         </is>
       </c>
       <c r="C603" s="22" t="n"/>
@@ -14099,7 +14227,7 @@
       </c>
       <c r="B604" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-09</t>
+          <t>HORIZON-CL5-2027-02-D3-24</t>
         </is>
       </c>
       <c r="C604" s="22" t="n"/>
@@ -14211,7 +14339,7 @@
       </c>
       <c r="B611" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all following expected outcomes:Advance in the realisation of the Strategic Energy Technology (SET) Plan’s research and innovation priorities and targets for ocean energy;Energy producers and consumers benefit from increased performance of wave and tidal energy technologies with the focus on efficiency and flexibility, reduced cost, improved reliability and sustainability, operation and maintenance, robustness and security during all stages of the lifetime of an ocean energy farm from installation, operation and maintenance to deco</t>
+          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Advanced, secure frugal (energy-, resource-, data- and cost-efficient, sustainable) AI tools for real-time grid operations (including protection), market operations (if relevant) and consumer empowerment in distributed energy systems.A demonstrated AI development environment integrated with the upgraded digital spine of the energy system and energy-saving consumer applications.Scaled-up capabilities for learning at edge nodes and federated systems using agent-based architectures.A governance fram</t>
         </is>
       </c>
       <c r="C611" s="22" t="n"/>
@@ -14255,7 +14383,7 @@
       </c>
       <c r="B614" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-09</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-24</t>
         </is>
       </c>
       <c r="C614" s="22" t="n"/>
@@ -14482,7 +14610,7 @@
     <row r="631" ht="30" customHeight="1">
       <c r="A631" s="18" t="inlineStr">
         <is>
-          <t>FICHA 43: HORIZON-CL5-2027-02-D3-24</t>
+          <t>FICHA 43: HORIZON-CL5-2027-02-D3-15</t>
         </is>
       </c>
       <c r="B631" s="19" t="n"/>
@@ -14515,7 +14643,7 @@
       </c>
       <c r="B633" s="21" t="inlineStr">
         <is>
-          <t>Large scale operational validation and upscaling of state-of-the-art (Generative) AI tools and models powering a next generation digital energy system</t>
+          <t>Production technologies for solar photovoltaics beyond the state-of-the-art (EUPI-PV Partnership)</t>
         </is>
       </c>
       <c r="C633" s="22" t="n"/>
@@ -14531,7 +14659,7 @@
       </c>
       <c r="B634" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-24</t>
+          <t>HORIZON-CL5-2027-02-D3-15</t>
         </is>
       </c>
       <c r="C634" s="22" t="n"/>
@@ -14643,7 +14771,7 @@
       </c>
       <c r="B641" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all the following expected outcomes:Advanced, secure frugal (energy-, resource-, data- and cost-efficient, sustainable) AI tools for real-time grid operations (including protection), market operations (if relevant) and consumer empowerment in distributed energy systems.A demonstrated AI development environment integrated with the upgraded digital spine of the energy system and energy-saving consumer applications.Scaled-up capabilities for learning at edge nodes and federated systems using agent-based architectures.A governance fram</t>
+          <t>Expected Outcome:The REPowerEU plan and the EU Solar Energy Strategy introduced targets for the deployment of solar PV amounting to 600 GWac by 2030. Complying with these targets will be crucial for the European Union to reach its climate targets and free itself from import dependency on fossil fuels and the costs this imposes on Europe’s competitiveness in terms of high energy prices. The Solar Strategy also introduces a target, which has been enshrined into the Net-Zero Industry Act, to re-consolidate the European solar manufacturing sector and scale up European manufacturing capacity across</t>
         </is>
       </c>
       <c r="C641" s="22" t="n"/>
@@ -14687,7 +14815,7 @@
       </c>
       <c r="B644" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-24</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-15</t>
         </is>
       </c>
       <c r="C644" s="22" t="n"/>
@@ -14698,7 +14826,7 @@
     <row r="646" ht="30" customHeight="1">
       <c r="A646" s="18" t="inlineStr">
         <is>
-          <t>FICHA 44: HORIZON-CL5-2027-02-D3-31</t>
+          <t>FICHA 44: HORIZON-CL5-2027-02-D3-07</t>
         </is>
       </c>
       <c r="B646" s="19" t="n"/>
@@ -14723,7 +14851,7 @@
       <c r="E647" s="22" t="n"/>
       <c r="F647" s="22" t="n"/>
     </row>
-    <row r="648" ht="45" customHeight="1">
+    <row r="648" ht="20" customHeight="1">
       <c r="A648" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -14731,7 +14859,7 @@
       </c>
       <c r="B648" s="21" t="inlineStr">
         <is>
-          <t>Support to the implementation of an EU policy framework for CO2 transport and storage infrastructure</t>
+          <t>Concentrated solar thermal systems for decarbonising industrial processes</t>
         </is>
       </c>
       <c r="C648" s="22" t="n"/>
@@ -14747,7 +14875,7 @@
       </c>
       <c r="B649" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-31</t>
+          <t>HORIZON-CL5-2027-02-D3-07</t>
         </is>
       </c>
       <c r="C649" s="22" t="n"/>
@@ -14827,7 +14955,7 @@
       </c>
       <c r="B654" s="21" t="inlineStr">
         <is>
-          <t>Coordination and Support Actions</t>
+          <t>Innovation Actions</t>
         </is>
       </c>
       <c r="C654" s="22" t="n"/>
@@ -14859,7 +14987,7 @@
       </c>
       <c r="B656" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to the following outcome:Stakeholders involved in the CO2 infrastructure network are in a position to implement the upcoming legislative framework for CO2 infrastructure.  Scope:The project is expected to assist stakeholders involved in the CO2 infrastructure network in implementing the upcoming legislative framework for CO2 infrastructure.Issues to address include market and cost structure, cross-border integration, interoperability and planning, technical harmonisation and investment incentives for new infrastructure, third-party ac</t>
+          <t>Expected Outcome:Renewable heating can be directly used to efficiently decarbonise industrial processes. Concentrated solar thermal technologies offer a great potential to supply renewable heat for industry for temperatures between 150°C - 400°C. Nevertheless, efforts are still required to demonstrate these technologies for a variety of industrial processes.Proposals are expected to contribute to all the following outcomes:Showcase the capacity of concentrated solar thermal systems to largely meet the heat demand of industrial processes and to achieve a yearly solar fraction of at least 50%.In</t>
         </is>
       </c>
       <c r="C656" s="22" t="n"/>
@@ -14903,7 +15031,7 @@
       </c>
       <c r="B659" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-31</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-07</t>
         </is>
       </c>
       <c r="C659" s="22" t="n"/>
@@ -14914,7 +15042,7 @@
     <row r="661" ht="30" customHeight="1">
       <c r="A661" s="18" t="inlineStr">
         <is>
-          <t>FICHA 45: HORIZON-CL5-2027-02-D3-15</t>
+          <t>FICHA 45: HORIZON-CL5-2027-02-D3-08</t>
         </is>
       </c>
       <c r="B661" s="19" t="n"/>
@@ -14947,7 +15075,7 @@
       </c>
       <c r="B663" s="21" t="inlineStr">
         <is>
-          <t>Production technologies for solar photovoltaics beyond the state-of-the-art (EUPI-PV Partnership)</t>
+          <t>Co-funding Strategic Energy Technology (SET) Plan renewable fuel value chains at EU, national, regional, and local level</t>
         </is>
       </c>
       <c r="C663" s="22" t="n"/>
@@ -14963,7 +15091,7 @@
       </c>
       <c r="B664" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-15</t>
+          <t>HORIZON-CL5-2027-02-D3-08</t>
         </is>
       </c>
       <c r="C664" s="22" t="n"/>
@@ -15043,7 +15171,7 @@
       </c>
       <c r="B669" s="21" t="inlineStr">
         <is>
-          <t>Innovation Actions</t>
+          <t>Programme Cofund Actions</t>
         </is>
       </c>
       <c r="C669" s="22" t="n"/>
@@ -15075,7 +15203,7 @@
       </c>
       <c r="B671" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:The REPowerEU plan and the EU Solar Energy Strategy introduced targets for the deployment of solar PV amounting to 600 GWac by 2030. Complying with these targets will be crucial for the European Union to reach its climate targets and free itself from import dependency on fossil fuels and the costs this imposes on Europe’s competitiveness in terms of high energy prices. The Solar Strategy also introduces a target, which has been enshrined into the Net-Zero Industry Act, to re-consolidate the European solar manufacturing sector and scale up European manufacturing capacity across</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Advance in the realisation of the Strategic Energy Technology (SET) Plan Action of Renewable fuels and Bioenergy (for the fuels part) is supported, overcoming fragmentation by mobilizing resources and establishing across EU interregional value chains of renewable fuel technologies and by better alignment of public and private R&amp;amp;I priorities and of funding mechanisms.All sector stakeholders benefit from establishment of renewable fuels value chains at EU, national, regional, and local level</t>
         </is>
       </c>
       <c r="C671" s="22" t="n"/>
@@ -15119,7 +15247,7 @@
       </c>
       <c r="B674" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-15</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-02-D3-08</t>
         </is>
       </c>
       <c r="C674" s="22" t="n"/>
@@ -18478,7 +18606,7 @@
     <row r="916" ht="30" customHeight="1">
       <c r="A916" s="18" t="inlineStr">
         <is>
-          <t>FICHA 62: BDNS-904269</t>
+          <t>FICHA 62: BDNS-904802</t>
         </is>
       </c>
       <c r="B916" s="19" t="n"/>
@@ -18503,7 +18631,7 @@
       <c r="E917" s="22" t="n"/>
       <c r="F917" s="22" t="n"/>
     </row>
-    <row r="918" ht="45" customHeight="1">
+    <row r="918" ht="20" customHeight="1">
       <c r="A918" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -18511,7 +18639,7 @@
       </c>
       <c r="B918" s="21" t="inlineStr">
         <is>
-          <t>Ayudas económicas municipales al fomento del empleo estable y de calidad en Vitoria-Gasteiz, para personas mayores de 45  años, para el ejercicio 2026</t>
+          <t>Mondragón Goi Eskola Politeknikoa Enpresa Digitala C12</t>
         </is>
       </c>
       <c r="C918" s="22" t="n"/>
@@ -18527,7 +18655,7 @@
       </c>
       <c r="B919" s="21" t="inlineStr">
         <is>
-          <t>BDNS-904269</t>
+          <t>BDNS-904802</t>
         </is>
       </c>
       <c r="C919" s="22" t="n"/>
@@ -18543,7 +18671,7 @@
       </c>
       <c r="B920" s="21" t="inlineStr">
         <is>
-          <t>VITORIA-GASTEIZ</t>
+          <t>PAÍS VASCO</t>
         </is>
       </c>
       <c r="C920" s="22" t="n"/>
@@ -18573,11 +18701,7 @@
           <t>Deadline</t>
         </is>
       </c>
-      <c r="B922" s="21" t="inlineStr">
-        <is>
-          <t>20/09/2026</t>
-        </is>
-      </c>
+      <c r="B922" s="21" t="inlineStr"/>
       <c r="C922" s="22" t="n"/>
       <c r="D922" s="22" t="n"/>
       <c r="E922" s="22" t="n"/>
@@ -18591,7 +18715,7 @@
       </c>
       <c r="B923" s="21" t="inlineStr">
         <is>
-          <t>600,000.00 EUR</t>
+          <t>465,000.00 EUR</t>
         </is>
       </c>
       <c r="C923" s="22" t="n"/>
@@ -18623,7 +18747,7 @@
       </c>
       <c r="B925" s="21" t="inlineStr">
         <is>
-          <t>BDNS 904269</t>
+          <t>BDNS 904802</t>
         </is>
       </c>
       <c r="C925" s="22" t="n"/>
@@ -18639,7 +18763,7 @@
       </c>
       <c r="B926" s="21" t="inlineStr">
         <is>
-          <t>PYME Y PERSONAS FÍSICAS QUE DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
+          <t>PERSONAS JURÍDICAS QUE NO DESARROLLAN ACTIVIDAD ECONÓMICA. MRR - MECANISMO DE RECUPERACIÓN Y RESILIENCIA. Regiones: ES21 - PAIS VASCO</t>
         </is>
       </c>
       <c r="C926" s="22" t="n"/>
@@ -18653,7 +18777,11 @@
           <t>Tags</t>
         </is>
       </c>
-      <c r="B927" s="21" t="inlineStr"/>
+      <c r="B927" s="21" t="inlineStr">
+        <is>
+          <t>MRR - MECANISMO DE RECUPERACIÓN Y RESILIENCIA</t>
+        </is>
+      </c>
       <c r="C927" s="22" t="n"/>
       <c r="D927" s="22" t="n"/>
       <c r="E927" s="22" t="n"/>
@@ -18665,9 +18793,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B928" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
+      <c r="B928" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MUY ALTA — </t>
         </is>
       </c>
       <c r="C928" s="22" t="n"/>
@@ -18683,7 +18811,7 @@
       </c>
       <c r="B929" s="23" t="inlineStr">
         <is>
-          <t>https://www.infosubvenciones.es/bdnstrans/GE/es/convocatoria/904269</t>
+          <t>https://www.infosubvenciones.es/bdnstrans/GE/es/convocatoria/904802</t>
         </is>
       </c>
       <c r="C929" s="22" t="n"/>
@@ -18694,7 +18822,7 @@
     <row r="931" ht="30" customHeight="1">
       <c r="A931" s="18" t="inlineStr">
         <is>
-          <t>FICHA 63: EUS-97378</t>
+          <t>FICHA 63: BDNS-904604</t>
         </is>
       </c>
       <c r="B931" s="19" t="n"/>
@@ -18711,7 +18839,7 @@
       </c>
       <c r="B932" s="21" t="inlineStr">
         <is>
-          <t>🟢 Euskadi</t>
+          <t>🇪🇸 España</t>
         </is>
       </c>
       <c r="C932" s="22" t="n"/>
@@ -18727,7 +18855,7 @@
       </c>
       <c r="B933" s="21" t="inlineStr">
         <is>
-          <t>BANCO DE HIDRÓGENO Y FONDO DE INNOVACIÓN: son parte de los instrumentos mediante los que la UE ha adjudicado nuevas ayudas a proyectos de I+D y producción ecológica de este combustible renovable, impl</t>
+          <t>CONVENIO DE SUBVENCIÓN NOMINATIVA ENTRE EL AYUNTAMIENTO DE VITORIA-GASTEIZ Y LA ASOCIACIÓN DE REINSERCIÓN SOCIAL SARTU- ÁLAVA PARA EL DESARROLLO DEL PROYECTO SAREGUNE 2026, PARA LA REVITALIZACIÓN E IN</t>
         </is>
       </c>
       <c r="C933" s="22" t="n"/>
@@ -18743,7 +18871,7 @@
       </c>
       <c r="B934" s="21" t="inlineStr">
         <is>
-          <t>EUS-97378</t>
+          <t>BDNS-904604</t>
         </is>
       </c>
       <c r="C934" s="22" t="n"/>
@@ -18759,7 +18887,7 @@
       </c>
       <c r="B935" s="21" t="inlineStr">
         <is>
-          <t>Euskadi</t>
+          <t>VITORIA-GASTEIZ</t>
         </is>
       </c>
       <c r="C935" s="22" t="n"/>
@@ -18789,7 +18917,11 @@
           <t>Deadline</t>
         </is>
       </c>
-      <c r="B937" s="21" t="inlineStr"/>
+      <c r="B937" s="21" t="inlineStr">
+        <is>
+          <t>31/12/2026</t>
+        </is>
+      </c>
       <c r="C937" s="22" t="n"/>
       <c r="D937" s="22" t="n"/>
       <c r="E937" s="22" t="n"/>
@@ -18803,7 +18935,7 @@
       </c>
       <c r="B938" s="21" t="inlineStr">
         <is>
-          <t>No disponible</t>
+          <t>66,000.00 EUR</t>
         </is>
       </c>
       <c r="C938" s="22" t="n"/>
@@ -18819,7 +18951,7 @@
       </c>
       <c r="B939" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Subvencion Nacional</t>
         </is>
       </c>
       <c r="C939" s="22" t="n"/>
@@ -18833,13 +18965,17 @@
           <t>Call ID</t>
         </is>
       </c>
-      <c r="B940" s="21" t="inlineStr"/>
+      <c r="B940" s="21" t="inlineStr">
+        <is>
+          <t>BDNS 904604</t>
+        </is>
+      </c>
       <c r="C940" s="22" t="n"/>
       <c r="D940" s="22" t="n"/>
       <c r="E940" s="22" t="n"/>
       <c r="F940" s="22" t="n"/>
     </row>
-    <row r="941" ht="20" customHeight="1">
+    <row r="941" ht="45" customHeight="1">
       <c r="A941" s="20" t="inlineStr">
         <is>
           <t>Descripcion</t>
@@ -18847,7 +18983,7 @@
       </c>
       <c r="B941" s="21" t="inlineStr">
         <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+          <t>PERSONAS JURÍDICAS QUE NO DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
         </is>
       </c>
       <c r="C941" s="22" t="n"/>
@@ -18861,11 +18997,7 @@
           <t>Tags</t>
         </is>
       </c>
-      <c r="B942" s="21" t="inlineStr">
-        <is>
-          <t>energia</t>
-        </is>
-      </c>
+      <c r="B942" s="21" t="inlineStr"/>
       <c r="C942" s="22" t="n"/>
       <c r="D942" s="22" t="n"/>
       <c r="E942" s="22" t="n"/>
@@ -18877,9 +19009,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B943" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ALTA — </t>
+      <c r="B943" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MUY ALTA — </t>
         </is>
       </c>
       <c r="C943" s="22" t="n"/>
@@ -18887,7 +19019,7 @@
       <c r="E943" s="22" t="n"/>
       <c r="F943" s="22" t="n"/>
     </row>
-    <row r="944" ht="45" customHeight="1">
+    <row r="944" ht="20" customHeight="1">
       <c r="A944" s="20" t="inlineStr">
         <is>
           <t>Enlace al portal</t>
@@ -18895,7 +19027,7 @@
       </c>
       <c r="B944" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260508cineahidrogenoatafuntsa/web01-tramite/es/</t>
+          <t>https://www.infosubvenciones.es/bdnstrans/GE/es/convocatoria/904604</t>
         </is>
       </c>
       <c r="C944" s="22" t="n"/>
@@ -18906,7 +19038,7 @@
     <row r="946" ht="30" customHeight="1">
       <c r="A946" s="18" t="inlineStr">
         <is>
-          <t>FICHA 64: EUS-04117</t>
+          <t>FICHA 64: BDNS-904545</t>
         </is>
       </c>
       <c r="B946" s="19" t="n"/>
@@ -18923,7 +19055,7 @@
       </c>
       <c r="B947" s="21" t="inlineStr">
         <is>
-          <t>🟢 Euskadi</t>
+          <t>🇪🇸 España</t>
         </is>
       </c>
       <c r="C947" s="22" t="n"/>
@@ -18939,7 +19071,7 @@
       </c>
       <c r="B948" s="21" t="inlineStr">
         <is>
-          <t>NEB, Nueva Bauhaus Europea. Convocatoria para barrios estéticos, inclusivos, sostenibles y con vivienda asequible, con financiación del marco Horizon de I+D y otros programas. Áreas de ecología-inclus</t>
+          <t>CONVENIO DE SUBVENCIÓN NOMINATIVA ENTRE EL AYUNTAMIENTO DE VITORIA-GASTEIZ Y LA FUNDACIÓN CATEDRAL DE SANTA MARÍA. PROGRAMA DE VISITAS GUIADAS A LA MURALLA MEDIEVAL AÑO 2026</t>
         </is>
       </c>
       <c r="C948" s="22" t="n"/>
@@ -18955,7 +19087,7 @@
       </c>
       <c r="B949" s="21" t="inlineStr">
         <is>
-          <t>EUS-04117</t>
+          <t>BDNS-904545</t>
         </is>
       </c>
       <c r="C949" s="22" t="n"/>
@@ -18971,7 +19103,7 @@
       </c>
       <c r="B950" s="21" t="inlineStr">
         <is>
-          <t>Euskadi</t>
+          <t>VITORIA-GASTEIZ</t>
         </is>
       </c>
       <c r="C950" s="22" t="n"/>
@@ -19001,7 +19133,11 @@
           <t>Deadline</t>
         </is>
       </c>
-      <c r="B952" s="21" t="inlineStr"/>
+      <c r="B952" s="21" t="inlineStr">
+        <is>
+          <t>31/12/2026</t>
+        </is>
+      </c>
       <c r="C952" s="22" t="n"/>
       <c r="D952" s="22" t="n"/>
       <c r="E952" s="22" t="n"/>
@@ -19015,7 +19151,7 @@
       </c>
       <c r="B953" s="21" t="inlineStr">
         <is>
-          <t>No disponible</t>
+          <t>32,000.00 EUR</t>
         </is>
       </c>
       <c r="C953" s="22" t="n"/>
@@ -19031,7 +19167,7 @@
       </c>
       <c r="B954" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Subvencion Nacional</t>
         </is>
       </c>
       <c r="C954" s="22" t="n"/>
@@ -19045,13 +19181,17 @@
           <t>Call ID</t>
         </is>
       </c>
-      <c r="B955" s="21" t="inlineStr"/>
+      <c r="B955" s="21" t="inlineStr">
+        <is>
+          <t>BDNS 904545</t>
+        </is>
+      </c>
       <c r="C955" s="22" t="n"/>
       <c r="D955" s="22" t="n"/>
       <c r="E955" s="22" t="n"/>
       <c r="F955" s="22" t="n"/>
     </row>
-    <row r="956" ht="20" customHeight="1">
+    <row r="956" ht="45" customHeight="1">
       <c r="A956" s="20" t="inlineStr">
         <is>
           <t>Descripcion</t>
@@ -19059,7 +19199,7 @@
       </c>
       <c r="B956" s="21" t="inlineStr">
         <is>
-          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+          <t>PERSONAS JURÍDICAS QUE NO DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
         </is>
       </c>
       <c r="C956" s="22" t="n"/>
@@ -19073,11 +19213,7 @@
           <t>Tags</t>
         </is>
       </c>
-      <c r="B957" s="21" t="inlineStr">
-        <is>
-          <t>energia</t>
-        </is>
-      </c>
+      <c r="B957" s="21" t="inlineStr"/>
       <c r="C957" s="22" t="n"/>
       <c r="D957" s="22" t="n"/>
       <c r="E957" s="22" t="n"/>
@@ -19089,9 +19225,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B958" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ALTA — </t>
+      <c r="B958" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MUY ALTA — </t>
         </is>
       </c>
       <c r="C958" s="22" t="n"/>
@@ -19099,7 +19235,7 @@
       <c r="E958" s="22" t="n"/>
       <c r="F958" s="22" t="n"/>
     </row>
-    <row r="959" ht="45" customHeight="1">
+    <row r="959" ht="20" customHeight="1">
       <c r="A959" s="20" t="inlineStr">
         <is>
           <t>Enlace al portal</t>
@@ -19107,7 +19243,7 @@
       </c>
       <c r="B959" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/2605nebauzoetarako3lerroe/web01-tramite/es/</t>
+          <t>https://www.infosubvenciones.es/bdnstrans/GE/es/convocatoria/904545</t>
         </is>
       </c>
       <c r="C959" s="22" t="n"/>
@@ -19118,7 +19254,7 @@
     <row r="961" ht="30" customHeight="1">
       <c r="A961" s="18" t="inlineStr">
         <is>
-          <t>FICHA 65: EUS-87863</t>
+          <t>FICHA 65: EUS-85014</t>
         </is>
       </c>
       <c r="B961" s="19" t="n"/>
@@ -19151,7 +19287,7 @@
       </c>
       <c r="B963" s="21" t="inlineStr">
         <is>
-          <t>Elige Europa para la Ciencia: primeras 16 carreras apoyadas con la fórmula innovadora de financiar a las universidades de residencia. Inteligencia artificial, biomedicina, robótica, genómica, clima, e</t>
+          <t>Contrato Reservado a Centros Especiales de Empleo, de conformidad con la Disposición Adicional Cuarta de la Ley 9/2017, de 8 de noviembre, de Contratos del Sector Público, para la prestación del servi</t>
         </is>
       </c>
       <c r="C963" s="22" t="n"/>
@@ -19167,7 +19303,7 @@
       </c>
       <c r="B964" s="21" t="inlineStr">
         <is>
-          <t>EUS-87863</t>
+          <t>EUS-85014</t>
         </is>
       </c>
       <c r="C964" s="22" t="n"/>
@@ -19243,7 +19379,7 @@
       </c>
       <c r="B969" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C969" s="22" t="n"/>
@@ -19301,9 +19437,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B973" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ALTA — </t>
+      <c r="B973" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MUY ALTA — </t>
         </is>
       </c>
       <c r="C973" s="22" t="n"/>
@@ -19319,7 +19455,7 @@
       </c>
       <c r="B974" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260506aukeratueuropazient/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/contrato-reservado-centros-especiales-empleo-conformidad-disposicion-adicional-cuarta-ley-9-2017-8-noviembre-contratos-del-sector-publico-prestacion-del-servicio-limpieza-viaria-del-municipio-igorre/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C974" s="22" t="n"/>
@@ -19330,7 +19466,7 @@
     <row r="976" ht="30" customHeight="1">
       <c r="A976" s="18" t="inlineStr">
         <is>
-          <t>FICHA 66: EUS-85070</t>
+          <t>FICHA 66: EUS-26962</t>
         </is>
       </c>
       <c r="B976" s="19" t="n"/>
@@ -19363,7 +19499,7 @@
       </c>
       <c r="B978" s="21" t="inlineStr">
         <is>
-          <t>LIFE 2026. Medio ambiente. Ayudas de 4 subprogramas, de naturaleza y biodiversidad, circularidad y calidad de vida, cambio climático y transición energética. Con inscripción abierta para jornadas info</t>
+          <t>BANCO DE HIDRÓGENO Y FONDO DE INNOVACIÓN: son parte de los instrumentos mediante los que la UE ha adjudicado nuevas ayudas a proyectos de I+D y producción ecológica de este combustible renovable, impl</t>
         </is>
       </c>
       <c r="C978" s="22" t="n"/>
@@ -19379,7 +19515,7 @@
       </c>
       <c r="B979" s="21" t="inlineStr">
         <is>
-          <t>EUS-85070</t>
+          <t>EUS-26962</t>
         </is>
       </c>
       <c r="C979" s="22" t="n"/>
@@ -19531,7 +19667,7 @@
       </c>
       <c r="B989" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260421life4lerrotajarduna/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260508cineahidrogenoatafuntsa/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C989" s="22" t="n"/>
@@ -19542,7 +19678,7 @@
     <row r="991" ht="30" customHeight="1">
       <c r="A991" s="18" t="inlineStr">
         <is>
-          <t>FICHA 67: EUS-86334</t>
+          <t>FICHA 67: EUS-99909</t>
         </is>
       </c>
       <c r="B991" s="19" t="n"/>
@@ -19575,7 +19711,7 @@
       </c>
       <c r="B993" s="21" t="inlineStr">
         <is>
-          <t>Enajenación mediante subasta de diversos materiales que se encuentran en el almacén municipal para su achatarramiento y tratamiento como residuos sólidos urbanos</t>
+          <t>NEB, Nueva Bauhaus Europea. Convocatoria para barrios estéticos, inclusivos, sostenibles y con vivienda asequible, con financiación del marco Horizon de I+D y otros programas. Áreas de ecología-inclus</t>
         </is>
       </c>
       <c r="C993" s="22" t="n"/>
@@ -19591,7 +19727,7 @@
       </c>
       <c r="B994" s="21" t="inlineStr">
         <is>
-          <t>EUS-86334</t>
+          <t>EUS-99909</t>
         </is>
       </c>
       <c r="C994" s="22" t="n"/>
@@ -19667,7 +19803,7 @@
       </c>
       <c r="B999" s="21" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C999" s="22" t="n"/>
@@ -19743,7 +19879,7 @@
       </c>
       <c r="B1004" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/enajenacion-mediante-subasta-diversos-materiales-que-se-encuentran-almacen-municipal-su-achatarramiento-y-tratamiento-como-residuos-solidos-urbanos/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/2605nebauzoetarako3lerroe/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1004" s="22" t="n"/>
@@ -19754,7 +19890,7 @@
     <row r="1006" ht="30" customHeight="1">
       <c r="A1006" s="18" t="inlineStr">
         <is>
-          <t>FICHA 68: EUS-05833</t>
+          <t>FICHA 68: EUS-02372</t>
         </is>
       </c>
       <c r="B1006" s="19" t="n"/>
@@ -19787,7 +19923,7 @@
       </c>
       <c r="B1008" s="21" t="inlineStr">
         <is>
-          <t>I+D.  Red Eureka, o programas financiados por el marco de innovación Horizon, como Eurostars (pymes) PRIMA (Mediterráneo) CETP (Energía) o DUT (Transformación Urbana). Evento del 12.05.26 sobre consor</t>
+          <t>Elige Europa para la Ciencia: primeras 16 carreras apoyadas con la fórmula innovadora de financiar a las universidades de residencia. Inteligencia artificial, biomedicina, robótica, genómica, clima, e</t>
         </is>
       </c>
       <c r="C1008" s="22" t="n"/>
@@ -19803,7 +19939,7 @@
       </c>
       <c r="B1009" s="21" t="inlineStr">
         <is>
-          <t>EUS-05833</t>
+          <t>EUS-02372</t>
         </is>
       </c>
       <c r="C1009" s="22" t="n"/>
@@ -19937,9 +20073,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B1018" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
+      <c r="B1018" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALTA — </t>
         </is>
       </c>
       <c r="C1018" s="22" t="n"/>
@@ -19955,7 +20091,7 @@
       </c>
       <c r="B1019" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/2605eurekaeurostarsdutpri/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260506aukeratueuropazient/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1019" s="22" t="n"/>
@@ -19966,7 +20102,7 @@
     <row r="1021" ht="30" customHeight="1">
       <c r="A1021" s="18" t="inlineStr">
         <is>
-          <t>FICHA 69: EUS-20593</t>
+          <t>FICHA 69: EUS-59698</t>
         </is>
       </c>
       <c r="B1021" s="19" t="n"/>
@@ -19999,7 +20135,7 @@
       </c>
       <c r="B1023" s="21" t="inlineStr">
         <is>
-          <t>CEF-E. Línea de infraestructuras energéticas del Mecanismo Conectar Europa. Alineado con planes de Redes Transeuropeas (RTE-E) plan de choque anticrisis de la Unión de la Energía (AccelerateEU). Proye</t>
+          <t>LIFE 2026. Medio ambiente. Ayudas de 4 subprogramas, de naturaleza y biodiversidad, circularidad y calidad de vida, cambio climático y transición energética. Con inscripción abierta para jornadas info</t>
         </is>
       </c>
       <c r="C1023" s="22" t="n"/>
@@ -20015,7 +20151,7 @@
       </c>
       <c r="B1024" s="21" t="inlineStr">
         <is>
-          <t>EUS-20593</t>
+          <t>EUS-59698</t>
         </is>
       </c>
       <c r="C1024" s="22" t="n"/>
@@ -20149,9 +20285,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B1033" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
+      <c r="B1033" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALTA — </t>
         </is>
       </c>
       <c r="C1033" s="22" t="n"/>
@@ -20167,7 +20303,7 @@
       </c>
       <c r="B1034" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/2605ceferteepcipmiacceler/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260421life4lerrotajarduna/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1034" s="22" t="n"/>
@@ -20178,7 +20314,7 @@
     <row r="1036" ht="30" customHeight="1">
       <c r="A1036" s="18" t="inlineStr">
         <is>
-          <t>FICHA 70: EUS-82373</t>
+          <t>FICHA 70: EUS-09274</t>
         </is>
       </c>
       <c r="B1036" s="19" t="n"/>
@@ -20211,7 +20347,7 @@
       </c>
       <c r="B1038" s="21" t="inlineStr">
         <is>
-          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta el 01.10.26. Cribado de enfermedades con inteligencia artificial. Espacio de Datos Sanitarios de la UE. Red de Centros para Seguridad de la I</t>
+          <t>Campaña de información y sensibilización sobre mejora del sistema de recogida selectiva de residuos</t>
         </is>
       </c>
       <c r="C1038" s="22" t="n"/>
@@ -20227,7 +20363,7 @@
       </c>
       <c r="B1039" s="21" t="inlineStr">
         <is>
-          <t>EUS-82373</t>
+          <t>EUS-09274</t>
         </is>
       </c>
       <c r="C1039" s="22" t="n"/>
@@ -20303,7 +20439,7 @@
       </c>
       <c r="B1044" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C1044" s="22" t="n"/>
@@ -20361,9 +20497,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B1048" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MEDIA — </t>
+      <c r="B1048" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALTA — </t>
         </is>
       </c>
       <c r="C1048" s="22" t="n"/>
@@ -20379,7 +20515,7 @@
       </c>
       <c r="B1049" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260422digitaleuropekoak/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/campana-informacion-y-sensibilizacion-mejora-del-sistema-recogida-selectiva-residuos/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1049" s="22" t="n"/>
@@ -20390,7 +20526,7 @@
     <row r="1051" ht="30" customHeight="1">
       <c r="A1051" s="18" t="inlineStr">
         <is>
-          <t>FICHA 71: EUS-56939</t>
+          <t>FICHA 71: EUS-77428</t>
         </is>
       </c>
       <c r="B1051" s="19" t="n"/>
@@ -20415,7 +20551,7 @@
       <c r="E1052" s="22" t="n"/>
       <c r="F1052" s="22" t="n"/>
     </row>
-    <row r="1053" ht="20" customHeight="1">
+    <row r="1053" ht="45" customHeight="1">
       <c r="A1053" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -20423,7 +20559,7 @@
       </c>
       <c r="B1053" s="21" t="inlineStr">
         <is>
-          <t>Adquisición de paraguas corporativos del 90 aniversario del Gobierno Vasco</t>
+          <t>I+D.  Red Eureka, o programas financiados por el marco de innovación Horizon, como Eurostars (pymes) PRIMA (Mediterráneo) CETP (Energía) o DUT (Transformación Urbana). Evento del 12.05.26 sobre consor</t>
         </is>
       </c>
       <c r="C1053" s="22" t="n"/>
@@ -20439,7 +20575,7 @@
       </c>
       <c r="B1054" s="21" t="inlineStr">
         <is>
-          <t>EUS-56939</t>
+          <t>EUS-77428</t>
         </is>
       </c>
       <c r="C1054" s="22" t="n"/>
@@ -20515,7 +20651,7 @@
       </c>
       <c r="B1059" s="21" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C1059" s="22" t="n"/>
@@ -20591,7 +20727,7 @@
       </c>
       <c r="B1064" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/adquisicion-paraguas-corporativos-del-90-aniversario-del-gobierno-vasco/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/2605eurekaeurostarsdutpri/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1064" s="22" t="n"/>
@@ -20602,7 +20738,7 @@
     <row r="1066" ht="30" customHeight="1">
       <c r="A1066" s="18" t="inlineStr">
         <is>
-          <t>FICHA 72: EUS-37445</t>
+          <t>FICHA 72: EUS-23728</t>
         </is>
       </c>
       <c r="B1066" s="19" t="n"/>
@@ -20635,7 +20771,7 @@
       </c>
       <c r="B1068" s="21" t="inlineStr">
         <is>
-          <t>Suministro, instalación y puesta en marcha de un conjunto de grupos electrógenos y depósitos auxiliares del sistema PEMEL de la red de saneamiento y abastecimiento de Aguas del Añarbe</t>
+          <t>CEF-E. Línea de infraestructuras energéticas del Mecanismo Conectar Europa. Alineado con planes de Redes Transeuropeas (RTE-E) plan de choque anticrisis de la Unión de la Energía (AccelerateEU). Proye</t>
         </is>
       </c>
       <c r="C1068" s="22" t="n"/>
@@ -20651,7 +20787,7 @@
       </c>
       <c r="B1069" s="21" t="inlineStr">
         <is>
-          <t>EUS-37445</t>
+          <t>EUS-23728</t>
         </is>
       </c>
       <c r="C1069" s="22" t="n"/>
@@ -20727,7 +20863,7 @@
       </c>
       <c r="B1074" s="21" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C1074" s="22" t="n"/>
@@ -20803,7 +20939,7 @@
       </c>
       <c r="B1079" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-instalacion-y-puesta-marcha-conjunto-grupos-electrogenos-y-depositos-auxiliares-del-sistema-pemel-red-saneamiento-y-abastecimiento-aguas-del-anarbe/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/2605ceferteepcipmiacceler/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1079" s="22" t="n"/>
@@ -20814,7 +20950,7 @@
     <row r="1081" ht="30" customHeight="1">
       <c r="A1081" s="18" t="inlineStr">
         <is>
-          <t>FICHA 73: EUS-17618</t>
+          <t>FICHA 73: EUS-04696</t>
         </is>
       </c>
       <c r="B1081" s="19" t="n"/>
@@ -20839,7 +20975,7 @@
       <c r="E1082" s="22" t="n"/>
       <c r="F1082" s="22" t="n"/>
     </row>
-    <row r="1083" ht="20" customHeight="1">
+    <row r="1083" ht="45" customHeight="1">
       <c r="A1083" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -20847,7 +20983,7 @@
       </c>
       <c r="B1083" s="21" t="inlineStr">
         <is>
-          <t>Obras de reparación de la caldera en el colegio Mendiko</t>
+          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta el 01.10.26. Cribado de enfermedades con inteligencia artificial. Espacio de Datos Sanitarios de la UE. Red de Centros para Seguridad de la I</t>
         </is>
       </c>
       <c r="C1083" s="22" t="n"/>
@@ -20863,7 +20999,7 @@
       </c>
       <c r="B1084" s="21" t="inlineStr">
         <is>
-          <t>EUS-17618</t>
+          <t>EUS-04696</t>
         </is>
       </c>
       <c r="C1084" s="22" t="n"/>
@@ -20939,7 +21075,7 @@
       </c>
       <c r="B1089" s="21" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C1089" s="22" t="n"/>
@@ -21015,7 +21151,7 @@
       </c>
       <c r="B1094" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/obras-reparacion-caldera-colegio-mendiko/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260422digitaleuropekoak/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1094" s="22" t="n"/>
@@ -21026,7 +21162,7 @@
     <row r="1096" ht="30" customHeight="1">
       <c r="A1096" s="18" t="inlineStr">
         <is>
-          <t>FICHA 74: EUS-83776</t>
+          <t>FICHA 74: EUS-92366</t>
         </is>
       </c>
       <c r="B1096" s="19" t="n"/>
@@ -21051,7 +21187,7 @@
       <c r="E1097" s="22" t="n"/>
       <c r="F1097" s="22" t="n"/>
     </row>
-    <row r="1098" ht="45" customHeight="1">
+    <row r="1098" ht="20" customHeight="1">
       <c r="A1098" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -21059,7 +21195,7 @@
       </c>
       <c r="B1098" s="21" t="inlineStr">
         <is>
-          <t>Suministro, instalación, puesta en marcha y mantenimiento de un sistema analítico para la determinación de la concentración de compuestos organohalogenados adsorbibles (AOX) en el laboratorio de contr</t>
+          <t>mantenimiento de la sala de calderas de la herri eskola</t>
         </is>
       </c>
       <c r="C1098" s="22" t="n"/>
@@ -21075,7 +21211,7 @@
       </c>
       <c r="B1099" s="21" t="inlineStr">
         <is>
-          <t>EUS-83776</t>
+          <t>EUS-92366</t>
         </is>
       </c>
       <c r="C1099" s="22" t="n"/>
@@ -21227,7 +21363,7 @@
       </c>
       <c r="B1109" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-instalacion-puesta-marcha-y-mantenimiento-sistema-analitico-determinacion-concentracion-compuestos-organohalogenados-adsorbibles-aox-laboratorio-control-calidad-aguas-residuales-agasa/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/mantenimiento-sala-calderas-herri-eskola/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1109" s="22" t="n"/>
@@ -21238,7 +21374,7 @@
     <row r="1111" ht="30" customHeight="1">
       <c r="A1111" s="18" t="inlineStr">
         <is>
-          <t>FICHA 75: EUS-27600</t>
+          <t>FICHA 75: EUS-09126</t>
         </is>
       </c>
       <c r="B1111" s="19" t="n"/>
@@ -21271,7 +21407,7 @@
       </c>
       <c r="B1113" s="21" t="inlineStr">
         <is>
-          <t>Gestión de incidencias en las viviendas dependientes de servicios sociales</t>
+          <t>mantenimiento de la sala de calderas del campo de fútbol de plazeta</t>
         </is>
       </c>
       <c r="C1113" s="22" t="n"/>
@@ -21287,7 +21423,7 @@
       </c>
       <c r="B1114" s="21" t="inlineStr">
         <is>
-          <t>EUS-27600</t>
+          <t>EUS-09126</t>
         </is>
       </c>
       <c r="C1114" s="22" t="n"/>
@@ -21439,7 +21575,7 @@
       </c>
       <c r="B1124" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/gestion-incidencias-viviendas-dependientes-servicios-sociales/expgegetxo12025002732/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/mantenimiento-sala-calderas-del-campo-futbol-plazeta/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1124" s="22" t="n"/>
@@ -21450,7 +21586,7 @@
     <row r="1126" ht="30" customHeight="1">
       <c r="A1126" s="18" t="inlineStr">
         <is>
-          <t>FICHA 76: EUS-44604</t>
+          <t>FICHA 76: EUS-15501</t>
         </is>
       </c>
       <c r="B1126" s="19" t="n"/>
@@ -21475,7 +21611,7 @@
       <c r="E1127" s="22" t="n"/>
       <c r="F1127" s="22" t="n"/>
     </row>
-    <row r="1128" ht="45" customHeight="1">
+    <row r="1128" ht="20" customHeight="1">
       <c r="A1128" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -21483,7 +21619,7 @@
       </c>
       <c r="B1128" s="21" t="inlineStr">
         <is>
-          <t>Trabajos sobrevenidos de renovación integral de zonas verdes aledañas a rampas 1 y 2 bidezabal</t>
+          <t>Cambio del variador del ascensor del frontón astelena por entrada de agua</t>
         </is>
       </c>
       <c r="C1128" s="22" t="n"/>
@@ -21499,7 +21635,7 @@
       </c>
       <c r="B1129" s="21" t="inlineStr">
         <is>
-          <t>EUS-44604</t>
+          <t>EUS-15501</t>
         </is>
       </c>
       <c r="C1129" s="22" t="n"/>
@@ -21651,7 +21787,7 @@
       </c>
       <c r="B1139" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/trabajos-sobrevenidos-renovacion-integral-zonas-verdes-aledanas-rampas-1-y-2-bidezabal/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/cambio-del-variador-del-ascensor-del-fronton-astelena-entrada-agua/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1139" s="22" t="n"/>
@@ -21659,8 +21795,432 @@
       <c r="E1139" s="22" t="n"/>
       <c r="F1139" s="22" t="n"/>
     </row>
+    <row r="1141" ht="30" customHeight="1">
+      <c r="A1141" s="18" t="inlineStr">
+        <is>
+          <t>FICHA 77: EUS-66632</t>
+        </is>
+      </c>
+      <c r="B1141" s="19" t="n"/>
+      <c r="C1141" s="19" t="n"/>
+      <c r="D1141" s="19" t="n"/>
+      <c r="E1141" s="19" t="n"/>
+      <c r="F1141" s="19" t="n"/>
+    </row>
+    <row r="1142" ht="20" customHeight="1">
+      <c r="A1142" s="20" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1142" s="21" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1142" s="22" t="n"/>
+      <c r="D1142" s="22" t="n"/>
+      <c r="E1142" s="22" t="n"/>
+      <c r="F1142" s="22" t="n"/>
+    </row>
+    <row r="1143" ht="20" customHeight="1">
+      <c r="A1143" s="20" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1143" s="21" t="inlineStr">
+        <is>
+          <t>Suministro y instalación de escalera para el acceso al parque de itzio</t>
+        </is>
+      </c>
+      <c r="C1143" s="22" t="n"/>
+      <c r="D1143" s="22" t="n"/>
+      <c r="E1143" s="22" t="n"/>
+      <c r="F1143" s="22" t="n"/>
+    </row>
+    <row r="1144" ht="20" customHeight="1">
+      <c r="A1144" s="20" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1144" s="21" t="inlineStr">
+        <is>
+          <t>EUS-66632</t>
+        </is>
+      </c>
+      <c r="C1144" s="22" t="n"/>
+      <c r="D1144" s="22" t="n"/>
+      <c r="E1144" s="22" t="n"/>
+      <c r="F1144" s="22" t="n"/>
+    </row>
+    <row r="1145" ht="20" customHeight="1">
+      <c r="A1145" s="20" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1145" s="21" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1145" s="22" t="n"/>
+      <c r="D1145" s="22" t="n"/>
+      <c r="E1145" s="22" t="n"/>
+      <c r="F1145" s="22" t="n"/>
+    </row>
+    <row r="1146" ht="20" customHeight="1">
+      <c r="A1146" s="20" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1146" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1146" s="22" t="n"/>
+      <c r="D1146" s="22" t="n"/>
+      <c r="E1146" s="22" t="n"/>
+      <c r="F1146" s="22" t="n"/>
+    </row>
+    <row r="1147" ht="20" customHeight="1">
+      <c r="A1147" s="20" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1147" s="21" t="inlineStr"/>
+      <c r="C1147" s="22" t="n"/>
+      <c r="D1147" s="22" t="n"/>
+      <c r="E1147" s="22" t="n"/>
+      <c r="F1147" s="22" t="n"/>
+    </row>
+    <row r="1148" ht="20" customHeight="1">
+      <c r="A1148" s="20" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1148" s="21" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1148" s="22" t="n"/>
+      <c r="D1148" s="22" t="n"/>
+      <c r="E1148" s="22" t="n"/>
+      <c r="F1148" s="22" t="n"/>
+    </row>
+    <row r="1149" ht="20" customHeight="1">
+      <c r="A1149" s="20" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1149" s="21" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1149" s="22" t="n"/>
+      <c r="D1149" s="22" t="n"/>
+      <c r="E1149" s="22" t="n"/>
+      <c r="F1149" s="22" t="n"/>
+    </row>
+    <row r="1150" ht="20" customHeight="1">
+      <c r="A1150" s="20" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1150" s="21" t="inlineStr"/>
+      <c r="C1150" s="22" t="n"/>
+      <c r="D1150" s="22" t="n"/>
+      <c r="E1150" s="22" t="n"/>
+      <c r="F1150" s="22" t="n"/>
+    </row>
+    <row r="1151" ht="20" customHeight="1">
+      <c r="A1151" s="20" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1151" s="21" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1151" s="22" t="n"/>
+      <c r="D1151" s="22" t="n"/>
+      <c r="E1151" s="22" t="n"/>
+      <c r="F1151" s="22" t="n"/>
+    </row>
+    <row r="1152" ht="20" customHeight="1">
+      <c r="A1152" s="20" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1152" s="21" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1152" s="22" t="n"/>
+      <c r="D1152" s="22" t="n"/>
+      <c r="E1152" s="22" t="n"/>
+      <c r="F1152" s="22" t="n"/>
+    </row>
+    <row r="1153" ht="20" customHeight="1">
+      <c r="A1153" s="20" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1153" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1153" s="22" t="n"/>
+      <c r="D1153" s="22" t="n"/>
+      <c r="E1153" s="22" t="n"/>
+      <c r="F1153" s="22" t="n"/>
+    </row>
+    <row r="1154" ht="45" customHeight="1">
+      <c r="A1154" s="20" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1154" s="23" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/suministro-y-instalacion-escalera-acceso-al-parque-itzio/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1154" s="22" t="n"/>
+      <c r="D1154" s="22" t="n"/>
+      <c r="E1154" s="22" t="n"/>
+      <c r="F1154" s="22" t="n"/>
+    </row>
+    <row r="1156" ht="30" customHeight="1">
+      <c r="A1156" s="18" t="inlineStr">
+        <is>
+          <t>FICHA 78: EUS-69385</t>
+        </is>
+      </c>
+      <c r="B1156" s="19" t="n"/>
+      <c r="C1156" s="19" t="n"/>
+      <c r="D1156" s="19" t="n"/>
+      <c r="E1156" s="19" t="n"/>
+      <c r="F1156" s="19" t="n"/>
+    </row>
+    <row r="1157" ht="20" customHeight="1">
+      <c r="A1157" s="20" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1157" s="21" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+      <c r="C1157" s="22" t="n"/>
+      <c r="D1157" s="22" t="n"/>
+      <c r="E1157" s="22" t="n"/>
+      <c r="F1157" s="22" t="n"/>
+    </row>
+    <row r="1158" ht="20" customHeight="1">
+      <c r="A1158" s="20" t="inlineStr">
+        <is>
+          <t>Titulo</t>
+        </is>
+      </c>
+      <c r="B1158" s="21" t="inlineStr">
+        <is>
+          <t>Limpieza y pintado del muro junto al kiosko de urki</t>
+        </is>
+      </c>
+      <c r="C1158" s="22" t="n"/>
+      <c r="D1158" s="22" t="n"/>
+      <c r="E1158" s="22" t="n"/>
+      <c r="F1158" s="22" t="n"/>
+    </row>
+    <row r="1159" ht="20" customHeight="1">
+      <c r="A1159" s="20" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1159" s="21" t="inlineStr">
+        <is>
+          <t>EUS-69385</t>
+        </is>
+      </c>
+      <c r="C1159" s="22" t="n"/>
+      <c r="D1159" s="22" t="n"/>
+      <c r="E1159" s="22" t="n"/>
+      <c r="F1159" s="22" t="n"/>
+    </row>
+    <row r="1160" ht="20" customHeight="1">
+      <c r="A1160" s="20" t="inlineStr">
+        <is>
+          <t>Programa</t>
+        </is>
+      </c>
+      <c r="B1160" s="21" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="C1160" s="22" t="n"/>
+      <c r="D1160" s="22" t="n"/>
+      <c r="E1160" s="22" t="n"/>
+      <c r="F1160" s="22" t="n"/>
+    </row>
+    <row r="1161" ht="20" customHeight="1">
+      <c r="A1161" s="20" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="B1161" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="C1161" s="22" t="n"/>
+      <c r="D1161" s="22" t="n"/>
+      <c r="E1161" s="22" t="n"/>
+      <c r="F1161" s="22" t="n"/>
+    </row>
+    <row r="1162" ht="20" customHeight="1">
+      <c r="A1162" s="20" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B1162" s="21" t="inlineStr"/>
+      <c r="C1162" s="22" t="n"/>
+      <c r="D1162" s="22" t="n"/>
+      <c r="E1162" s="22" t="n"/>
+      <c r="F1162" s="22" t="n"/>
+    </row>
+    <row r="1163" ht="20" customHeight="1">
+      <c r="A1163" s="20" t="inlineStr">
+        <is>
+          <t>Presupuesto (EUR)</t>
+        </is>
+      </c>
+      <c r="B1163" s="21" t="inlineStr">
+        <is>
+          <t>No disponible</t>
+        </is>
+      </c>
+      <c r="C1163" s="22" t="n"/>
+      <c r="D1163" s="22" t="n"/>
+      <c r="E1163" s="22" t="n"/>
+      <c r="F1163" s="22" t="n"/>
+    </row>
+    <row r="1164" ht="20" customHeight="1">
+      <c r="A1164" s="20" t="inlineStr">
+        <is>
+          <t>Tipo de Accion</t>
+        </is>
+      </c>
+      <c r="B1164" s="21" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="C1164" s="22" t="n"/>
+      <c r="D1164" s="22" t="n"/>
+      <c r="E1164" s="22" t="n"/>
+      <c r="F1164" s="22" t="n"/>
+    </row>
+    <row r="1165" ht="20" customHeight="1">
+      <c r="A1165" s="20" t="inlineStr">
+        <is>
+          <t>Call ID</t>
+        </is>
+      </c>
+      <c r="B1165" s="21" t="inlineStr"/>
+      <c r="C1165" s="22" t="n"/>
+      <c r="D1165" s="22" t="n"/>
+      <c r="E1165" s="22" t="n"/>
+      <c r="F1165" s="22" t="n"/>
+    </row>
+    <row r="1166" ht="20" customHeight="1">
+      <c r="A1166" s="20" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="B1166" s="21" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="C1166" s="22" t="n"/>
+      <c r="D1166" s="22" t="n"/>
+      <c r="E1166" s="22" t="n"/>
+      <c r="F1166" s="22" t="n"/>
+    </row>
+    <row r="1167" ht="20" customHeight="1">
+      <c r="A1167" s="20" t="inlineStr">
+        <is>
+          <t>Tags</t>
+        </is>
+      </c>
+      <c r="B1167" s="21" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
+      <c r="C1167" s="22" t="n"/>
+      <c r="D1167" s="22" t="n"/>
+      <c r="E1167" s="22" t="n"/>
+      <c r="F1167" s="22" t="n"/>
+    </row>
+    <row r="1168" ht="20" customHeight="1">
+      <c r="A1168" s="20" t="inlineStr">
+        <is>
+          <t>Relevancia Bilbao</t>
+        </is>
+      </c>
+      <c r="B1168" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
+        </is>
+      </c>
+      <c r="C1168" s="22" t="n"/>
+      <c r="D1168" s="22" t="n"/>
+      <c r="E1168" s="22" t="n"/>
+      <c r="F1168" s="22" t="n"/>
+    </row>
+    <row r="1169" ht="45" customHeight="1">
+      <c r="A1169" s="20" t="inlineStr">
+        <is>
+          <t>Enlace al portal</t>
+        </is>
+      </c>
+      <c r="B1169" s="23" t="inlineStr">
+        <is>
+          <t>https://www.euskadi.eus/anuncio_contratacion/limpieza-y-pintado-del-muro-junto-al-kiosko-urki/web01-tramite/es/</t>
+        </is>
+      </c>
+      <c r="C1169" s="22" t="n"/>
+      <c r="D1169" s="22" t="n"/>
+      <c r="E1169" s="22" t="n"/>
+      <c r="F1169" s="22" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="1064">
+  <mergeCells count="1092">
     <mergeCell ref="B679:F679"/>
     <mergeCell ref="B666:F666"/>
     <mergeCell ref="B964:F964"/>
@@ -21704,6 +22264,7 @@
     <mergeCell ref="B342:F342"/>
     <mergeCell ref="B578:F578"/>
     <mergeCell ref="A541:F541"/>
+    <mergeCell ref="B1148:F1148"/>
     <mergeCell ref="B1099:F1099"/>
     <mergeCell ref="B515:F515"/>
     <mergeCell ref="B1128:F1128"/>
@@ -21719,6 +22280,7 @@
     <mergeCell ref="B369:F369"/>
     <mergeCell ref="B667:F667"/>
     <mergeCell ref="B418:F418"/>
+    <mergeCell ref="B1142:F1142"/>
     <mergeCell ref="B356:F356"/>
     <mergeCell ref="B160:F160"/>
     <mergeCell ref="B489:F489"/>
@@ -21802,6 +22364,7 @@
     <mergeCell ref="A346:F346"/>
     <mergeCell ref="B904:F904"/>
     <mergeCell ref="B635:F635"/>
+    <mergeCell ref="A1141:F1141"/>
     <mergeCell ref="B141:F141"/>
     <mergeCell ref="B439:F439"/>
     <mergeCell ref="A136:F136"/>
@@ -21854,6 +22417,7 @@
     <mergeCell ref="B1055:F1055"/>
     <mergeCell ref="B536:F536"/>
     <mergeCell ref="B834:F834"/>
+    <mergeCell ref="B1143:F1143"/>
     <mergeCell ref="B899:F899"/>
     <mergeCell ref="B752:F752"/>
     <mergeCell ref="B1070:F1070"/>
@@ -21873,6 +22437,7 @@
     <mergeCell ref="B1044:F1044"/>
     <mergeCell ref="B156:F156"/>
     <mergeCell ref="B327:F327"/>
+    <mergeCell ref="B1144:F1144"/>
     <mergeCell ref="B454:F454"/>
     <mergeCell ref="B625:F625"/>
     <mergeCell ref="B923:F923"/>
@@ -21893,6 +22458,7 @@
     <mergeCell ref="B562:F562"/>
     <mergeCell ref="B689:F689"/>
     <mergeCell ref="B1121:F1121"/>
+    <mergeCell ref="B1146:F1146"/>
     <mergeCell ref="B1123:F1123"/>
     <mergeCell ref="B86:F86"/>
     <mergeCell ref="B912:F912"/>
@@ -21981,6 +22547,7 @@
     <mergeCell ref="A226:F226"/>
     <mergeCell ref="B1124:F1124"/>
     <mergeCell ref="B394:F394"/>
+    <mergeCell ref="B1162:F1162"/>
     <mergeCell ref="B692:F692"/>
     <mergeCell ref="A931:F931"/>
     <mergeCell ref="B486:F486"/>
@@ -22003,6 +22570,7 @@
     <mergeCell ref="B185:F185"/>
     <mergeCell ref="A826:F826"/>
     <mergeCell ref="B483:F483"/>
+    <mergeCell ref="B1165:F1165"/>
     <mergeCell ref="B581:F581"/>
     <mergeCell ref="B1048:F1048"/>
     <mergeCell ref="B475:F475"/>
@@ -22029,17 +22597,20 @@
     <mergeCell ref="B1117:F1117"/>
     <mergeCell ref="B107:F107"/>
     <mergeCell ref="B1104:F1104"/>
+    <mergeCell ref="B1160:F1160"/>
     <mergeCell ref="B641:F641"/>
     <mergeCell ref="B57:F57"/>
     <mergeCell ref="B883:F883"/>
     <mergeCell ref="B908:F908"/>
     <mergeCell ref="B171:F171"/>
+    <mergeCell ref="B1168:F1168"/>
     <mergeCell ref="B407:F407"/>
     <mergeCell ref="A646:F646"/>
     <mergeCell ref="B972:F972"/>
     <mergeCell ref="B9:F9"/>
     <mergeCell ref="B463:F463"/>
     <mergeCell ref="B438:F438"/>
+    <mergeCell ref="B1145:F1145"/>
     <mergeCell ref="B359:F359"/>
     <mergeCell ref="B207:F207"/>
     <mergeCell ref="B788:F788"/>
@@ -22055,6 +22626,7 @@
     <mergeCell ref="B1061:F1061"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="B1097:F1097"/>
+    <mergeCell ref="B1153:F1153"/>
     <mergeCell ref="A46:F46"/>
     <mergeCell ref="B507:F507"/>
     <mergeCell ref="B62:F62"/>
@@ -22070,6 +22642,7 @@
     <mergeCell ref="B857:F857"/>
     <mergeCell ref="B1063:F1063"/>
     <mergeCell ref="B1090:F1090"/>
+    <mergeCell ref="B1161:F1161"/>
     <mergeCell ref="B807:F807"/>
     <mergeCell ref="B1000:F1000"/>
     <mergeCell ref="B39:F39"/>
@@ -22104,6 +22677,7 @@
     <mergeCell ref="B428:F428"/>
     <mergeCell ref="B1118:F1118"/>
     <mergeCell ref="B284:F284"/>
+    <mergeCell ref="B1167:F1167"/>
     <mergeCell ref="B222:F222"/>
     <mergeCell ref="B344:F344"/>
     <mergeCell ref="B415:F415"/>
@@ -22164,6 +22738,8 @@
     <mergeCell ref="B808:F808"/>
     <mergeCell ref="B879:F879"/>
     <mergeCell ref="B897:F897"/>
+    <mergeCell ref="B1164:F1164"/>
+    <mergeCell ref="B1158:F1158"/>
     <mergeCell ref="B403:F403"/>
     <mergeCell ref="B574:F574"/>
     <mergeCell ref="B745:F745"/>
@@ -22171,6 +22747,7 @@
     <mergeCell ref="B55:F55"/>
     <mergeCell ref="B1003:F1003"/>
     <mergeCell ref="B169:F169"/>
+    <mergeCell ref="B1166:F1166"/>
     <mergeCell ref="A706:F706"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B129:F129"/>
@@ -22228,6 +22805,7 @@
     <mergeCell ref="A721:F721"/>
     <mergeCell ref="A31:F31"/>
     <mergeCell ref="B747:F747"/>
+    <mergeCell ref="B1152:F1152"/>
     <mergeCell ref="B668:F668"/>
     <mergeCell ref="B84:F84"/>
     <mergeCell ref="A736:F736"/>
@@ -22320,6 +22898,7 @@
     <mergeCell ref="B830:F830"/>
     <mergeCell ref="A871:F871"/>
     <mergeCell ref="B895:F895"/>
+    <mergeCell ref="A1156:F1156"/>
     <mergeCell ref="B232:F232"/>
     <mergeCell ref="B321:F321"/>
     <mergeCell ref="B215:F215"/>
@@ -22421,6 +23000,7 @@
     <mergeCell ref="B756:F756"/>
     <mergeCell ref="B992:F992"/>
     <mergeCell ref="A811:F811"/>
+    <mergeCell ref="B1150:F1150"/>
     <mergeCell ref="B329:F329"/>
     <mergeCell ref="B627:F627"/>
     <mergeCell ref="B49:F49"/>
@@ -22468,6 +23048,7 @@
     <mergeCell ref="B845:F845"/>
     <mergeCell ref="B261:F261"/>
     <mergeCell ref="B1087:F1087"/>
+    <mergeCell ref="B1149:F1149"/>
     <mergeCell ref="B184:F184"/>
     <mergeCell ref="B1062:F1062"/>
     <mergeCell ref="A301:F301"/>
@@ -22488,6 +23069,7 @@
     <mergeCell ref="B250:F250"/>
     <mergeCell ref="B927:F927"/>
     <mergeCell ref="B44:F44"/>
+    <mergeCell ref="B1163:F1163"/>
     <mergeCell ref="B408:F408"/>
     <mergeCell ref="B464:F464"/>
     <mergeCell ref="A916:F916"/>
@@ -22554,6 +23136,8 @@
     <mergeCell ref="B1024:F1024"/>
     <mergeCell ref="B396:F396"/>
     <mergeCell ref="B567:F567"/>
+    <mergeCell ref="B1151:F1151"/>
+    <mergeCell ref="B1157:F1157"/>
     <mergeCell ref="B632:F632"/>
     <mergeCell ref="B803:F803"/>
     <mergeCell ref="B996:F996"/>
@@ -22564,6 +23148,7 @@
     <mergeCell ref="B267:F267"/>
     <mergeCell ref="B798:F798"/>
     <mergeCell ref="B1088:F1088"/>
+    <mergeCell ref="B1159:F1159"/>
     <mergeCell ref="B398:F398"/>
     <mergeCell ref="B569:F569"/>
     <mergeCell ref="A466:F466"/>
@@ -22573,6 +23158,7 @@
     <mergeCell ref="B269:F269"/>
     <mergeCell ref="B187:F187"/>
     <mergeCell ref="B485:F485"/>
+    <mergeCell ref="B1154:F1154"/>
     <mergeCell ref="B124:F124"/>
     <mergeCell ref="B251:F251"/>
     <mergeCell ref="B806:F806"/>
@@ -22582,6 +23168,7 @@
     <mergeCell ref="B487:F487"/>
     <mergeCell ref="B1077:F1077"/>
     <mergeCell ref="B343:F343"/>
+    <mergeCell ref="B1169:F1169"/>
     <mergeCell ref="B414:F414"/>
     <mergeCell ref="B474:F474"/>
     <mergeCell ref="B772:F772"/>
@@ -22625,6 +23212,7 @@
     <mergeCell ref="B1101:F1101"/>
     <mergeCell ref="B582:F582"/>
     <mergeCell ref="B849:F849"/>
+    <mergeCell ref="B1147:F1147"/>
     <mergeCell ref="B1132:F1132"/>
     <mergeCell ref="B73:F73"/>
     <mergeCell ref="B371:F371"/>
@@ -22803,6 +23391,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1109" r:id="rId74"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1124" r:id="rId75"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1139" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1154" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B1169" r:id="rId78"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -22814,7 +23404,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J77"/>
+  <dimension ref="A1:J79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -23204,12 +23794,12 @@
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-04</t>
+          <t>HORIZON-CL5-2026-11-D3-23</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>De-risking renewable fuel technologies through transnational</t>
+          <t>Data sharing to support the training and development of AI f</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -23244,12 +23834,12 @@
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-05</t>
+          <t>HORIZON-CL5-2026-11-D3-06</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Demonstration of solid biofuel supply and conversion to high</t>
+          <t>Resource assessment for deep sedimentary and basement reserv</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -23284,12 +23874,12 @@
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-23</t>
+          <t>HORIZON-CL5-2026-11-D3-14</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Data sharing to support the training and development of AI f</t>
+          <t>Improved system design for innovative PV applications (EUPI-</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -23324,12 +23914,12 @@
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-06</t>
+          <t>HORIZON-CL5-2026-11-D3-05</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Resource assessment for deep sedimentary and basement reserv</t>
+          <t>Demonstration of solid biofuel supply and conversion to high</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -23364,12 +23954,12 @@
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2026-11-D3-14</t>
+          <t>HORIZON-CL5-2026-11-D3-04</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Improved system design for innovative PV applications (EUPI-</t>
+          <t>De-risking renewable fuel technologies through transnational</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -23404,12 +23994,12 @@
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-16</t>
+          <t>HORIZON-CL5-2027-07-D3-27</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Industrial processes and equipment for innovative, reliable </t>
+          <t xml:space="preserve">Integrated Approaches for Retrofitting Infrastructures with </t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -23444,12 +24034,12 @@
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-11</t>
+          <t>HORIZON-CL5-2027-07-D3-26</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Demonstration of hydropower technologies for efficient and f</t>
+          <t>Advanced Distribution Management Systems (ADSM) for more eff</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -23524,12 +24114,12 @@
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-26</t>
+          <t>HORIZON-CL5-2027-07-D3-28</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Advanced Distribution Management Systems (ADSM) for more eff</t>
+          <t>Community of practice - Data-Driven Decision-Making in Energ</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -23564,12 +24154,12 @@
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-27</t>
+          <t>HORIZON-CL5-2027-07-D3-16</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Integrated Approaches for Retrofitting Infrastructures with </t>
+          <t xml:space="preserve">Industrial processes and equipment for innovative, reliable </t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -23604,12 +24194,12 @@
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-28</t>
+          <t>HORIZON-CL5-2027-07-D3-25</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Community of practice - Data-Driven Decision-Making in Energ</t>
+          <t>Advanced TSO control rooms to enhance grid observability, st</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -23644,12 +24234,12 @@
     <row r="21" ht="28" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-25</t>
+          <t>HORIZON-CL5-2027-07-D3-17</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Advanced TSO control rooms to enhance grid observability, st</t>
+          <t>PV based electrification of the economy: Designing &amp; optimis</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -23684,12 +24274,12 @@
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-07-D3-17</t>
+          <t>HORIZON-CL5-2027-07-D3-11</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>PV based electrification of the economy: Designing &amp; optimis</t>
+          <t>Demonstration of hydropower technologies for efficient and f</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -24444,12 +25034,12 @@
     <row r="41" ht="28" customHeight="1">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-08</t>
+          <t>HORIZON-CL5-2027-02-D3-31</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Co-funding Strategic Energy Technology (SET) Plan renewable </t>
+          <t xml:space="preserve">Support to the implementation of an EU policy framework for </t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
@@ -24484,12 +25074,12 @@
     <row r="42" ht="28" customHeight="1">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-09</t>
+          <t>HORIZON-CL5-2027-02-D3-24</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>Innovative technologies and solutions to improve wave and ti</t>
+          <t>Large scale operational validation and upscaling of state-of</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
@@ -24564,12 +25154,12 @@
     <row r="44" ht="28" customHeight="1">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-24</t>
+          <t>HORIZON-CL5-2027-02-D3-15</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>Large scale operational validation and upscaling of state-of</t>
+          <t>Production technologies for solar photovoltaics beyond the s</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
@@ -24604,12 +25194,12 @@
     <row r="45" ht="28" customHeight="1">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-31</t>
+          <t>HORIZON-CL5-2027-02-D3-07</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Support to the implementation of an EU policy framework for </t>
+          <t>Concentrated solar thermal systems for decarbonising industr</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
@@ -24644,12 +25234,12 @@
     <row r="46" ht="28" customHeight="1">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-02-D3-15</t>
+          <t>HORIZON-CL5-2027-02-D3-08</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>Production technologies for solar photovoltaics beyond the s</t>
+          <t xml:space="preserve">Co-funding Strategic Energy Technology (SET) Plan renewable </t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
@@ -25216,17 +25806,17 @@
     <row r="63" ht="28" customHeight="1">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>BDNS-904269</t>
+          <t>BDNS-904802</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ayudas económicas municipales al fomento del empleo estable </t>
+          <t>Mondragón Goi Eskola Politeknikoa Enpresa Digitala C12</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>VITORIA-GASTEIZ</t>
+          <t>PAÍS VASCO</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
@@ -25234,14 +25824,10 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="E63" s="6" t="inlineStr">
-        <is>
-          <t>20/09/2026</t>
-        </is>
-      </c>
+      <c r="E63" s="6" t="inlineStr"/>
       <c r="F63" s="27" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>MUY ALTA</t>
         </is>
       </c>
       <c r="G63" s="6" t="inlineStr"/>
@@ -25256,17 +25842,17 @@
     <row r="64" ht="28" customHeight="1">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>EUS-97378</t>
+          <t>BDNS-904604</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>BANCO DE HIDRÓGENO Y FONDO DE INNOVACIÓN: son parte de los i</t>
+          <t>CONVENIO DE SUBVENCIÓN NOMINATIVA ENTRE EL AYUNTAMIENTO DE V</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>Euskadi</t>
+          <t>VITORIA-GASTEIZ</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
@@ -25274,10 +25860,14 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="E64" s="6" t="inlineStr"/>
+      <c r="E64" s="6" t="inlineStr">
+        <is>
+          <t>31/12/2026</t>
+        </is>
+      </c>
       <c r="F64" s="27" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>MUY ALTA</t>
         </is>
       </c>
       <c r="G64" s="6" t="inlineStr"/>
@@ -25292,17 +25882,17 @@
     <row r="65" ht="28" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>EUS-04117</t>
+          <t>BDNS-904545</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>NEB, Nueva Bauhaus Europea. Convocatoria para barrios estéti</t>
+          <t>CONVENIO DE SUBVENCIÓN NOMINATIVA ENTRE EL AYUNTAMIENTO DE V</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>Euskadi</t>
+          <t>VITORIA-GASTEIZ</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
@@ -25310,10 +25900,14 @@
           <t>Open</t>
         </is>
       </c>
-      <c r="E65" s="6" t="inlineStr"/>
+      <c r="E65" s="6" t="inlineStr">
+        <is>
+          <t>31/12/2026</t>
+        </is>
+      </c>
       <c r="F65" s="27" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>MUY ALTA</t>
         </is>
       </c>
       <c r="G65" s="6" t="inlineStr"/>
@@ -25328,12 +25922,12 @@
     <row r="66" ht="28" customHeight="1">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>EUS-87863</t>
+          <t>EUS-85014</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Elige Europa para la Ciencia: primeras 16 carreras apoyadas </t>
+          <t>Contrato Reservado a Centros Especiales de Empleo, de confor</t>
         </is>
       </c>
       <c r="C66" s="6" t="inlineStr">
@@ -25349,7 +25943,7 @@
       <c r="E66" s="6" t="inlineStr"/>
       <c r="F66" s="27" t="inlineStr">
         <is>
-          <t>ALTA</t>
+          <t>MUY ALTA</t>
         </is>
       </c>
       <c r="G66" s="6" t="inlineStr"/>
@@ -25364,12 +25958,12 @@
     <row r="67" ht="28" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>EUS-85070</t>
+          <t>EUS-26962</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>LIFE 2026. Medio ambiente. Ayudas de 4 subprogramas, de natu</t>
+          <t>BANCO DE HIDRÓGENO Y FONDO DE INNOVACIÓN: son parte de los i</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
@@ -25400,12 +25994,12 @@
     <row r="68" ht="28" customHeight="1">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>EUS-86334</t>
+          <t>EUS-99909</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>Enajenación mediante subasta de diversos materiales que se e</t>
+          <t>NEB, Nueva Bauhaus Europea. Convocatoria para barrios estéti</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
@@ -25436,12 +26030,12 @@
     <row r="69" ht="28" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>EUS-05833</t>
+          <t>EUS-02372</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>I+D.  Red Eureka, o programas financiados por el marco de in</t>
+          <t xml:space="preserve">Elige Europa para la Ciencia: primeras 16 carreras apoyadas </t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -25457,7 +26051,7 @@
       <c r="E69" s="6" t="inlineStr"/>
       <c r="F69" s="27" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="G69" s="6" t="inlineStr"/>
@@ -25472,12 +26066,12 @@
     <row r="70" ht="28" customHeight="1">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>EUS-20593</t>
+          <t>EUS-59698</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>CEF-E. Línea de infraestructuras energéticas del Mecanismo C</t>
+          <t>LIFE 2026. Medio ambiente. Ayudas de 4 subprogramas, de natu</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
@@ -25493,7 +26087,7 @@
       <c r="E70" s="6" t="inlineStr"/>
       <c r="F70" s="27" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="G70" s="6" t="inlineStr"/>
@@ -25508,12 +26102,12 @@
     <row r="71" ht="28" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>EUS-82373</t>
+          <t>EUS-09274</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta e</t>
+          <t>Campaña de información y sensibilización sobre mejora del si</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -25529,7 +26123,7 @@
       <c r="E71" s="6" t="inlineStr"/>
       <c r="F71" s="27" t="inlineStr">
         <is>
-          <t>MEDIA</t>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="G71" s="6" t="inlineStr"/>
@@ -25544,12 +26138,12 @@
     <row r="72" ht="28" customHeight="1">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>EUS-56939</t>
+          <t>EUS-77428</t>
         </is>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Adquisición de paraguas corporativos del 90 aniversario del </t>
+          <t>I+D.  Red Eureka, o programas financiados por el marco de in</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
@@ -25580,12 +26174,12 @@
     <row r="73" ht="28" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>EUS-37445</t>
+          <t>EUS-23728</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>Suministro, instalación y puesta en marcha de un conjunto de</t>
+          <t>CEF-E. Línea de infraestructuras energéticas del Mecanismo C</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -25616,12 +26210,12 @@
     <row r="74" ht="28" customHeight="1">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>EUS-17618</t>
+          <t>EUS-04696</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>Obras de reparación de la caldera en el colegio Mendiko</t>
+          <t>Digital Europe y Plan Continente IA: 7 convocatorias hasta e</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
@@ -25652,12 +26246,12 @@
     <row r="75" ht="28" customHeight="1">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>EUS-83776</t>
+          <t>EUS-92366</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>Suministro, instalación, puesta en marcha y mantenimiento de</t>
+          <t>mantenimiento de la sala de calderas de la herri eskola</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
@@ -25688,12 +26282,12 @@
     <row r="76" ht="28" customHeight="1">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>EUS-27600</t>
+          <t>EUS-09126</t>
         </is>
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>Gestión de incidencias en las viviendas dependientes de serv</t>
+          <t xml:space="preserve">mantenimiento de la sala de calderas del campo de fútbol de </t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
@@ -25724,12 +26318,12 @@
     <row r="77" ht="28" customHeight="1">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>EUS-44604</t>
+          <t>EUS-15501</t>
         </is>
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>Trabajos sobrevenidos de renovación integral de zonas verdes</t>
+          <t>Cambio del variador del ascensor del frontón astelena por en</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
@@ -25757,8 +26351,80 @@
       <c r="I77" s="6" t="inlineStr"/>
       <c r="J77" s="6" t="inlineStr"/>
     </row>
+    <row r="78" ht="28" customHeight="1">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>EUS-66632</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>Suministro y instalación de escalera para el acceso al parqu</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E78" s="6" t="inlineStr"/>
+      <c r="F78" s="27" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G78" s="6" t="inlineStr"/>
+      <c r="H78" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I78" s="6" t="inlineStr"/>
+      <c r="J78" s="6" t="inlineStr"/>
+    </row>
+    <row r="79" ht="28" customHeight="1">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t>EUS-69385</t>
+        </is>
+      </c>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>Limpieza y pintado del muro junto al kiosko de urki</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E79" s="6" t="inlineStr"/>
+      <c r="F79" s="27" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="G79" s="6" t="inlineStr"/>
+      <c r="H79" s="6" t="inlineStr">
+        <is>
+          <t>Por revisar</t>
+        </is>
+      </c>
+      <c r="I79" s="6" t="inlineStr"/>
+      <c r="J79" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J77"/>
+  <autoFilter ref="A1:J79"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Update funding data 2026-05-13
</commit_message>
<xml_diff>
--- a/docs/resultados_convocatorias.xlsx
+++ b/docs/resultados_convocatorias.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Recursos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$85</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumen'!$A$4:$M$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Seguimiento'!$A$1:$J$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -679,7 +679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M85"/>
+  <dimension ref="A1:M92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -707,7 +707,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 12/05/2026 08:24 - 78 convocatorias - 17 nuevas</t>
+          <t>Mision Climatica - Neutralidad 2030 - Actualizado: 13/05/2026 08:32 - 85 convocatorias - 22 nuevas</t>
         </is>
       </c>
     </row>
@@ -2108,12 +2108,12 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
+          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
@@ -2153,7 +2153,7 @@
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Euro</t>
+          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and inter</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr"/>
@@ -2297,12 +2297,12 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -2327,7 +2327,7 @@
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Research and Innovation Actions</t>
+          <t>Programme Cofund Actions</t>
         </is>
       </c>
       <c r="I30" s="10" t="inlineStr">
@@ -2342,7 +2342,7 @@
       </c>
       <c r="K30" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to info</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is estab</t>
         </is>
       </c>
       <c r="L30" s="6" t="inlineStr"/>
@@ -2360,12 +2360,12 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-08</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
@@ -2405,7 +2405,7 @@
       </c>
       <c r="K31" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and inter</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorpo</t>
         </is>
       </c>
       <c r="L31" s="6" t="inlineStr"/>
@@ -2423,12 +2423,12 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
@@ -2453,7 +2453,7 @@
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>Programme Cofund Actions</t>
+          <t xml:space="preserve"> Research and Innovation Actions</t>
         </is>
       </c>
       <c r="I32" s="10" t="inlineStr">
@@ -2468,7 +2468,7 @@
       </c>
       <c r="K32" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is estab</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to info</t>
         </is>
       </c>
       <c r="L32" s="6" t="inlineStr"/>
@@ -2486,12 +2486,12 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
@@ -2531,7 +2531,7 @@
       </c>
       <c r="K33" s="6" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorpo</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Euro</t>
         </is>
       </c>
       <c r="L33" s="6" t="inlineStr"/>
@@ -4447,11 +4447,7 @@
           <t>PERSONAS JURÍDICAS QUE NO DESARROLLAN ACTIVIDAD ECONÓMICA. MRR - MECANISMO DE RECUPERACIÓN Y RESILIENCIA. Regiones: ES21 - PAIS VASCO</t>
         </is>
       </c>
-      <c r="L68" s="15" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
+      <c r="L68" s="6" t="inlineStr"/>
       <c r="M68" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
@@ -4466,12 +4462,12 @@
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>BDNS-904604</t>
+          <t>BDNS-905090</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>CONVENIO DE SUBVENCIÓN NOMINATIVA ENTRE EL AYUNTAMIENTO DE VITORIA-GASTEIZ Y LA ASOCIACIÓN DE REINSERCIÓN SOCIAL SARTU- ÁLAVA PARA EL DESARROLLO DEL PROYECTO SAREGUNE 2026, PARA LA REVITALIZACIÓN E IN</t>
+          <t>Ayudas dirigidas al desarrollo de proyectos de descarbonización 2026</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
@@ -4486,12 +4482,12 @@
       </c>
       <c r="F69" s="6" t="inlineStr">
         <is>
-          <t>31/12/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="G69" s="6" t="inlineStr">
         <is>
-          <t>66,000.00 EUR</t>
+          <t>600,000.00 EUR</t>
         </is>
       </c>
       <c r="H69" s="6" t="inlineStr">
@@ -4499,9 +4495,9 @@
           <t>Subvencion Nacional</t>
         </is>
       </c>
-      <c r="I69" s="12" t="inlineStr">
-        <is>
-          <t>MUY ALTA</t>
+      <c r="I69" s="8" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
         </is>
       </c>
       <c r="J69" s="6" t="inlineStr"/>
@@ -4521,73 +4517,65 @@
         </is>
       </c>
     </row>
-    <row r="70" ht="40" customHeight="1">
-      <c r="A70" s="14" t="inlineStr">
-        <is>
-          <t>España</t>
-        </is>
-      </c>
-      <c r="B70" s="6" t="inlineStr">
-        <is>
-          <t>BDNS-904545</t>
-        </is>
-      </c>
-      <c r="C70" s="6" t="inlineStr">
-        <is>
-          <t>CONVENIO DE SUBVENCIÓN NOMINATIVA ENTRE EL AYUNTAMIENTO DE VITORIA-GASTEIZ Y LA FUNDACIÓN CATEDRAL DE SANTA MARÍA. PROGRAMA DE VISITAS GUIADAS A LA MURALLA MEDIEVAL AÑO 2026</t>
-        </is>
-      </c>
-      <c r="D70" s="6" t="inlineStr">
-        <is>
-          <t>VITORIA-GASTEIZ</t>
-        </is>
-      </c>
-      <c r="E70" s="7" t="inlineStr">
+    <row r="70" ht="28" customHeight="1">
+      <c r="A70" s="16" t="inlineStr">
+        <is>
+          <t>🟢 Euskadi</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="40" customHeight="1">
+      <c r="A71" s="17" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>EUS-60487</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I+D, Horizon: evento informativo sobre la financiación en cascada o fórmula usada por el programa marco de innovación de la UE Horizon para dar inclusividad a pymes en grandes consorcios tecnológicos </t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="F70" s="6" t="inlineStr">
-        <is>
-          <t>31/12/2026</t>
-        </is>
-      </c>
-      <c r="G70" s="6" t="inlineStr">
-        <is>
-          <t>32,000.00 EUR</t>
-        </is>
-      </c>
-      <c r="H70" s="6" t="inlineStr">
-        <is>
-          <t>Subvencion Nacional</t>
-        </is>
-      </c>
-      <c r="I70" s="12" t="inlineStr">
-        <is>
-          <t>MUY ALTA</t>
-        </is>
-      </c>
-      <c r="J70" s="6" t="inlineStr"/>
-      <c r="K70" s="6" t="inlineStr">
-        <is>
-          <t>PERSONAS JURÍDICAS QUE NO DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
-        </is>
-      </c>
-      <c r="L70" s="15" t="inlineStr">
+      <c r="F71" s="6" t="inlineStr"/>
+      <c r="G71" s="6" t="inlineStr"/>
+      <c r="H71" s="6" t="inlineStr">
+        <is>
+          <t>Ayuda/Subvencion Euskadi</t>
+        </is>
+      </c>
+      <c r="I71" s="11" t="inlineStr">
+        <is>
+          <t>ALTA</t>
+        </is>
+      </c>
+      <c r="J71" s="6" t="inlineStr"/>
+      <c r="K71" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L71" s="15" t="inlineStr">
         <is>
           <t>NUEVA</t>
         </is>
       </c>
-      <c r="M70" s="9" t="inlineStr">
+      <c r="M71" s="9" t="inlineStr">
         <is>
           <t>Ver</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="28" customHeight="1">
-      <c r="A71" s="16" t="inlineStr">
-        <is>
-          <t>🟢 Euskadi</t>
         </is>
       </c>
     </row>
@@ -4599,12 +4587,12 @@
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>EUS-85014</t>
+          <t>EUS-76876</t>
         </is>
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>Contrato Reservado a Centros Especiales de Empleo, de conformidad con la Disposición Adicional Cuarta de la Ley 9/2017, de 8 de noviembre, de Contratos del Sector Público, para la prestación del servi</t>
+          <t>BANCO DE HIDRÓGENO Y FONDO DE INNOVACIÓN: son parte de los instrumentos mediante los que la UE ha adjudicado nuevas ayudas a proyectos de I+D y producción ecológica de este combustible renovable, impl</t>
         </is>
       </c>
       <c r="D72" s="6" t="inlineStr">
@@ -4621,12 +4609,12 @@
       <c r="G72" s="6" t="inlineStr"/>
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
-        </is>
-      </c>
-      <c r="I72" s="12" t="inlineStr">
-        <is>
-          <t>MUY ALTA</t>
+          <t>Ayuda/Subvencion Euskadi</t>
+        </is>
+      </c>
+      <c r="I72" s="11" t="inlineStr">
+        <is>
+          <t>ALTA</t>
         </is>
       </c>
       <c r="J72" s="6" t="inlineStr"/>
@@ -4654,12 +4642,12 @@
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>EUS-26962</t>
+          <t>EUS-34926</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>BANCO DE HIDRÓGENO Y FONDO DE INNOVACIÓN: son parte de los instrumentos mediante los que la UE ha adjudicado nuevas ayudas a proyectos de I+D y producción ecológica de este combustible renovable, impl</t>
+          <t>NEB, Nueva Bauhaus Europea. Convocatoria para barrios estéticos, inclusivos, sostenibles y con vivienda asequible, con financiación del marco Horizon de I+D y otros programas. Áreas de ecología-inclus</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
@@ -4709,12 +4697,12 @@
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>EUS-99909</t>
+          <t>EUS-71324</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>NEB, Nueva Bauhaus Europea. Convocatoria para barrios estéticos, inclusivos, sostenibles y con vivienda asequible, con financiación del marco Horizon de I+D y otros programas. Áreas de ecología-inclus</t>
+          <t>Elige Europa para la Ciencia: primeras 16 carreras apoyadas con la fórmula innovadora de financiar a las universidades de residencia. Inteligencia artificial, biomedicina, robótica, genómica, clima, e</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr">
@@ -4764,12 +4752,12 @@
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>EUS-02372</t>
+          <t>EUS-25492</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>Elige Europa para la Ciencia: primeras 16 carreras apoyadas con la fórmula innovadora de financiar a las universidades de residencia. Inteligencia artificial, biomedicina, robótica, genómica, clima, e</t>
+          <t>LIFE 2026. Medio ambiente. Ayudas de 4 subprogramas, de naturaleza y biodiversidad, circularidad y calidad de vida, cambio climático y transición energética. Con inscripción abierta para jornadas info</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
@@ -4819,12 +4807,12 @@
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>EUS-59698</t>
+          <t>EUS-67282</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>LIFE 2026. Medio ambiente. Ayudas de 4 subprogramas, de naturaleza y biodiversidad, circularidad y calidad de vida, cambio climático y transición energética. Con inscripción abierta para jornadas info</t>
+          <t>Sustitucion de sistemas de climatizacion y ventilación</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr">
@@ -4841,7 +4829,7 @@
       <c r="G76" s="6" t="inlineStr"/>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="I76" s="11" t="inlineStr">
@@ -4874,7 +4862,7 @@
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>EUS-09274</t>
+          <t>EUS-76748</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
@@ -4929,7 +4917,7 @@
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>EUS-77428</t>
+          <t>EUS-72997</t>
         </is>
       </c>
       <c r="C78" s="6" t="inlineStr">
@@ -4984,7 +4972,7 @@
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>EUS-23728</t>
+          <t>EUS-73348</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
@@ -5039,7 +5027,7 @@
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>EUS-04696</t>
+          <t>EUS-95747</t>
         </is>
       </c>
       <c r="C80" s="6" t="inlineStr">
@@ -5094,12 +5082,12 @@
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>EUS-92366</t>
+          <t>EUS-99974</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>mantenimiento de la sala de calderas de la herri eskola</t>
+          <t>Servicios para la redacción documento de actuación medioambiental que ofrezca las bases para la redacción de un mapa de riesgos, plan de acción y medidas específicaspara abordar los aspectos ambiental</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
@@ -5149,12 +5137,12 @@
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>EUS-09126</t>
+          <t>EUS-96634</t>
         </is>
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>mantenimiento de la sala de calderas del campo de fútbol de plazeta</t>
+          <t>Reparacion de recogida de pluviales</t>
         </is>
       </c>
       <c r="D82" s="6" t="inlineStr">
@@ -5204,12 +5192,12 @@
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>EUS-15501</t>
+          <t>EUS-61983</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>Cambio del variador del ascensor del frontón astelena por entrada de agua</t>
+          <t>Limpieza e inspeccion de colectores</t>
         </is>
       </c>
       <c r="D83" s="6" t="inlineStr">
@@ -5259,12 +5247,12 @@
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>EUS-66632</t>
+          <t>EUS-12793</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>Suministro y instalación de escalera para el acceso al parque de itzio</t>
+          <t>Licitación del servicio de seguridad y vigilancia en viviendas y edificios gestionados por Alokabide</t>
         </is>
       </c>
       <c r="D84" s="6" t="inlineStr">
@@ -5314,12 +5302,12 @@
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>EUS-69385</t>
+          <t>EUS-23993</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>Limpieza y pintado del muro junto al kiosko de urki</t>
+          <t>Proyecto de las redes de saneamiento, pluviales y abastecimiento</t>
         </is>
       </c>
       <c r="D85" s="6" t="inlineStr">
@@ -5361,14 +5349,395 @@
         </is>
       </c>
     </row>
+    <row r="86" ht="40" customHeight="1">
+      <c r="A86" s="17" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B86" s="6" t="inlineStr">
+        <is>
+          <t>EUS-52457</t>
+        </is>
+      </c>
+      <c r="C86" s="6" t="inlineStr">
+        <is>
+          <t>Suministro de zapatos para trabajadora de la limpieza errebal alb 1253</t>
+        </is>
+      </c>
+      <c r="D86" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E86" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F86" s="6" t="inlineStr"/>
+      <c r="G86" s="6" t="inlineStr"/>
+      <c r="H86" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I86" s="8" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J86" s="6" t="inlineStr"/>
+      <c r="K86" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L86" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M86" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="40" customHeight="1">
+      <c r="A87" s="17" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B87" s="6" t="inlineStr">
+        <is>
+          <t>EUS-68392</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="inlineStr">
+        <is>
+          <t>Servicio de desratizacion y desinsectacion anual de los edificios culturales</t>
+        </is>
+      </c>
+      <c r="D87" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E87" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F87" s="6" t="inlineStr"/>
+      <c r="G87" s="6" t="inlineStr"/>
+      <c r="H87" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I87" s="8" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J87" s="6" t="inlineStr"/>
+      <c r="K87" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L87" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M87" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="40" customHeight="1">
+      <c r="A88" s="17" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B88" s="6" t="inlineStr">
+        <is>
+          <t>EUS-39270</t>
+        </is>
+      </c>
+      <c r="C88" s="6" t="inlineStr">
+        <is>
+          <t>Servicio de contratacion artistica de 4 bertsolaris para las fiestas de Amorebieta-Etxano</t>
+        </is>
+      </c>
+      <c r="D88" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E88" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F88" s="6" t="inlineStr"/>
+      <c r="G88" s="6" t="inlineStr"/>
+      <c r="H88" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I88" s="8" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J88" s="6" t="inlineStr"/>
+      <c r="K88" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L88" s="6" t="inlineStr"/>
+      <c r="M88" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="40" customHeight="1">
+      <c r="A89" s="17" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B89" s="6" t="inlineStr">
+        <is>
+          <t>EUS-71120</t>
+        </is>
+      </c>
+      <c r="C89" s="6" t="inlineStr">
+        <is>
+          <t>Prestación de servicios de conducción y mantenimiento de los edificios e instalaciones del Museo Cristóbal Balenciaga de Getaria</t>
+        </is>
+      </c>
+      <c r="D89" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E89" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F89" s="6" t="inlineStr"/>
+      <c r="G89" s="6" t="inlineStr"/>
+      <c r="H89" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I89" s="8" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J89" s="6" t="inlineStr"/>
+      <c r="K89" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L89" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M89" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="40" customHeight="1">
+      <c r="A90" s="17" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B90" s="6" t="inlineStr">
+        <is>
+          <t>EUS-07463</t>
+        </is>
+      </c>
+      <c r="C90" s="6" t="inlineStr">
+        <is>
+          <t>Contratación de los Servicios de transporte dentro de las campañas del servicio de deporte  (curso 2026-2028)</t>
+        </is>
+      </c>
+      <c r="D90" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E90" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F90" s="6" t="inlineStr"/>
+      <c r="G90" s="6" t="inlineStr"/>
+      <c r="H90" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I90" s="8" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J90" s="6" t="inlineStr"/>
+      <c r="K90" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L90" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M90" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="40" customHeight="1">
+      <c r="A91" s="17" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B91" s="6" t="inlineStr">
+        <is>
+          <t>EUS-79287</t>
+        </is>
+      </c>
+      <c r="C91" s="6" t="inlineStr">
+        <is>
+          <t>Anteproyecto de red de aguas, saneamiento, pluviales y abastecimiento</t>
+        </is>
+      </c>
+      <c r="D91" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E91" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F91" s="6" t="inlineStr"/>
+      <c r="G91" s="6" t="inlineStr"/>
+      <c r="H91" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I91" s="8" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J91" s="6" t="inlineStr"/>
+      <c r="K91" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L91" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M91" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="40" customHeight="1">
+      <c r="A92" s="17" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="B92" s="6" t="inlineStr">
+        <is>
+          <t>EUS-22621</t>
+        </is>
+      </c>
+      <c r="C92" s="6" t="inlineStr">
+        <is>
+          <t>Mejora de cubiertas naves con bandas adhesivas</t>
+        </is>
+      </c>
+      <c r="D92" s="6" t="inlineStr">
+        <is>
+          <t>Euskadi</t>
+        </is>
+      </c>
+      <c r="E92" s="7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F92" s="6" t="inlineStr"/>
+      <c r="G92" s="6" t="inlineStr"/>
+      <c r="H92" s="6" t="inlineStr">
+        <is>
+          <t>Licitacion Euskadi</t>
+        </is>
+      </c>
+      <c r="I92" s="8" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
+        </is>
+      </c>
+      <c r="J92" s="6" t="inlineStr"/>
+      <c r="K92" s="6" t="inlineStr">
+        <is>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
+        </is>
+      </c>
+      <c r="L92" s="15" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="M92" s="9" t="inlineStr">
+        <is>
+          <t>Ver</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:M85"/>
+  <autoFilter ref="A4:M92"/>
   <mergeCells count="5">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="A5:M5"/>
     <mergeCell ref="A67:M67"/>
+    <mergeCell ref="A70:M70"/>
     <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A71:M71"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId1"/>
@@ -5434,7 +5803,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M66" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M68" r:id="rId62"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M69" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M70" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M71" r:id="rId64"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M72" r:id="rId65"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M73" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M74" r:id="rId67"/>
@@ -5449,6 +5818,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M83" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M84" r:id="rId77"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M85" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M86" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M87" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M88" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M89" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M90" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M91" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M92" r:id="rId85"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5460,7 +5836,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1169"/>
+  <dimension ref="A1:F1274"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10030,7 +10406,7 @@
     <row r="316" ht="30" customHeight="1">
       <c r="A316" s="18" t="inlineStr">
         <is>
-          <t>FICHA 22: HORIZON-CL5-2027-01-D1-07</t>
+          <t>FICHA 22: HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="B316" s="19" t="n"/>
@@ -10055,7 +10431,7 @@
       <c r="E317" s="22" t="n"/>
       <c r="F317" s="22" t="n"/>
     </row>
-    <row r="318" ht="45" customHeight="1">
+    <row r="318" ht="20" customHeight="1">
       <c r="A318" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -10063,7 +10439,7 @@
       </c>
       <c r="B318" s="21" t="inlineStr">
         <is>
-          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
+          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
         </is>
       </c>
       <c r="C318" s="22" t="n"/>
@@ -10079,7 +10455,7 @@
       </c>
       <c r="B319" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-07</t>
+          <t>HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="C319" s="22" t="n"/>
@@ -10191,7 +10567,7 @@
       </c>
       <c r="B326" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Europe and globally, as well as the interaction between different hazards, their cumulative and/or cascading effects.Enhanced seamless prediction and projection modelling and attribution capabilities for extreme events and their likelihood to support preparedness, response and resilience to climate change by EU and national and regional actors. The EU Union Preparedness Strategy, the EU Adaptation Str</t>
+          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and interactions with ecosystems, leading to improved Earth system models;Future climate change scenarios produced in light of past changes in the Earth system, in particular warm climates/high sea-level situations, and abrupt transitions;Identification of thresholds in Earth system components and better characterisation of driving mechanisms and feedbacks that may be responsible for non-linear behaviours,</t>
         </is>
       </c>
       <c r="C326" s="22" t="n"/>
@@ -10235,7 +10611,7 @@
       </c>
       <c r="B329" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-07</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-08</t>
         </is>
       </c>
       <c r="C329" s="22" t="n"/>
@@ -10678,7 +11054,7 @@
     <row r="361" ht="30" customHeight="1">
       <c r="A361" s="18" t="inlineStr">
         <is>
-          <t>FICHA 25: HORIZON-CL5-2027-01-D1-09</t>
+          <t>FICHA 25: HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="B361" s="19" t="n"/>
@@ -10703,7 +11079,7 @@
       <c r="E362" s="22" t="n"/>
       <c r="F362" s="22" t="n"/>
     </row>
-    <row r="363" ht="45" customHeight="1">
+    <row r="363" ht="20" customHeight="1">
       <c r="A363" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -10711,7 +11087,7 @@
       </c>
       <c r="B363" s="21" t="inlineStr">
         <is>
-          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
+          <t>Africa-EU CO-FUND action on climate</t>
         </is>
       </c>
       <c r="C363" s="22" t="n"/>
@@ -10727,7 +11103,7 @@
       </c>
       <c r="B364" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-09</t>
+          <t>HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C364" s="22" t="n"/>
@@ -10807,7 +11183,7 @@
       </c>
       <c r="B369" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Research and Innovation Actions</t>
+          <t>Programme Cofund Actions</t>
         </is>
       </c>
       <c r="C369" s="22" t="n"/>
@@ -10839,7 +11215,7 @@
       </c>
       <c r="B371" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to inform mitigation action and policy improvements, ensuring a fair transition and social acceptability;Methodologies are developed and improved for ex-ante assessment and ex-post evaluation of greenhouse gas emission reductions from climate policies and measures;Strengthened collaboration and established networks between researchers, policy experts and government officials involved in designing and eva</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is established through development and implementation of the Climate Action pillar of the EU-AU Research and Innovation Partnership on Climate Change and Sustainable Energy (CCSE),[1] in co-design between African and European partners;Reduced fragmentation by aligning the EU, national and multilateral R&amp;amp;I efforts with increased leverage and impact of funding;African scientific, policy and practice com</t>
         </is>
       </c>
       <c r="C371" s="22" t="n"/>
@@ -10883,7 +11259,7 @@
       </c>
       <c r="B374" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-09</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-11</t>
         </is>
       </c>
       <c r="C374" s="22" t="n"/>
@@ -10894,7 +11270,7 @@
     <row r="376" ht="30" customHeight="1">
       <c r="A376" s="18" t="inlineStr">
         <is>
-          <t>FICHA 26: HORIZON-CL5-2027-01-D1-08</t>
+          <t>FICHA 26: HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="B376" s="19" t="n"/>
@@ -10927,7 +11303,7 @@
       </c>
       <c r="B378" s="21" t="inlineStr">
         <is>
-          <t>Palaeoclimate science for a better understanding of Earth system dynamics</t>
+          <t>Understanding and avoiding maladaptation to climate change</t>
         </is>
       </c>
       <c r="C378" s="22" t="n"/>
@@ -10943,7 +11319,7 @@
       </c>
       <c r="B379" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-08</t>
+          <t>HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C379" s="22" t="n"/>
@@ -11055,7 +11431,7 @@
       </c>
       <c r="B386" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to some of the following outcomes:Better process understanding of past climate changes at different time scales, their variability and interactions with ecosystems, leading to improved Earth system models;Future climate change scenarios produced in light of past changes in the Earth system, in particular warm climates/high sea-level situations, and abrupt transitions;Identification of thresholds in Earth system components and better characterisation of driving mechanisms and feedbacks that may be responsible for non-linear behaviours,</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorporation into main EU repositories, such as Climate-ADAPT or the portal of the EU Mission on Adaptation to Climate Change;The risk and adaptation assessment frameworks are improved by better integrating the maladaptation dimension;Guidelines and tools for maladaptation prevention and correction strategies are made available to adaptation stakeholders at relevant scales and inform the design and impl</t>
         </is>
       </c>
       <c r="C386" s="22" t="n"/>
@@ -11099,7 +11475,7 @@
       </c>
       <c r="B389" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-08</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-10</t>
         </is>
       </c>
       <c r="C389" s="22" t="n"/>
@@ -11110,7 +11486,7 @@
     <row r="391" ht="30" customHeight="1">
       <c r="A391" s="18" t="inlineStr">
         <is>
-          <t>FICHA 27: HORIZON-CL5-2027-01-D1-11</t>
+          <t>FICHA 27: HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="B391" s="19" t="n"/>
@@ -11135,7 +11511,7 @@
       <c r="E392" s="22" t="n"/>
       <c r="F392" s="22" t="n"/>
     </row>
-    <row r="393" ht="20" customHeight="1">
+    <row r="393" ht="45" customHeight="1">
       <c r="A393" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -11143,7 +11519,7 @@
       </c>
       <c r="B393" s="21" t="inlineStr">
         <is>
-          <t>Africa-EU CO-FUND action on climate</t>
+          <t>Assessing the performance of policy instruments to inform climate change mitigation action</t>
         </is>
       </c>
       <c r="C393" s="22" t="n"/>
@@ -11159,7 +11535,7 @@
       </c>
       <c r="B394" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-11</t>
+          <t>HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C394" s="22" t="n"/>
@@ -11239,7 +11615,7 @@
       </c>
       <c r="B399" s="21" t="inlineStr">
         <is>
-          <t>Programme Cofund Actions</t>
+          <t xml:space="preserve"> Research and Innovation Actions</t>
         </is>
       </c>
       <c r="C399" s="22" t="n"/>
@@ -11271,7 +11647,7 @@
       </c>
       <c r="B401" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:A long-term collaboration on climate change research between the EU and the African Union is established through development and implementation of the Climate Action pillar of the EU-AU Research and Innovation Partnership on Climate Change and Sustainable Energy (CCSE),[1] in co-design between African and European partners;Reduced fragmentation by aligning the EU, national and multilateral R&amp;amp;I efforts with increased leverage and impact of funding;African scientific, policy and practice com</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Enhanced knowledge of the effectiveness of policy instruments on EU and Member State level to inform mitigation action and policy improvements, ensuring a fair transition and social acceptability;Methodologies are developed and improved for ex-ante assessment and ex-post evaluation of greenhouse gas emission reductions from climate policies and measures;Strengthened collaboration and established networks between researchers, policy experts and government officials involved in designing and eva</t>
         </is>
       </c>
       <c r="C401" s="22" t="n"/>
@@ -11315,7 +11691,7 @@
       </c>
       <c r="B404" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-11</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-09</t>
         </is>
       </c>
       <c r="C404" s="22" t="n"/>
@@ -11326,7 +11702,7 @@
     <row r="406" ht="30" customHeight="1">
       <c r="A406" s="18" t="inlineStr">
         <is>
-          <t>FICHA 28: HORIZON-CL5-2027-01-D1-10</t>
+          <t>FICHA 28: HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="B406" s="19" t="n"/>
@@ -11351,7 +11727,7 @@
       <c r="E407" s="22" t="n"/>
       <c r="F407" s="22" t="n"/>
     </row>
-    <row r="408" ht="20" customHeight="1">
+    <row r="408" ht="45" customHeight="1">
       <c r="A408" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -11359,7 +11735,7 @@
       </c>
       <c r="B408" s="21" t="inlineStr">
         <is>
-          <t>Understanding and avoiding maladaptation to climate change</t>
+          <t>Advancing understanding, modelling and prediction of extreme events in a changing climate</t>
         </is>
       </c>
       <c r="C408" s="22" t="n"/>
@@ -11375,7 +11751,7 @@
       </c>
       <c r="B409" s="21" t="inlineStr">
         <is>
-          <t>HORIZON-CL5-2027-01-D1-10</t>
+          <t>HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C409" s="22" t="n"/>
@@ -11487,7 +11863,7 @@
       </c>
       <c r="B416" s="21" t="inlineStr">
         <is>
-          <t>Expected Outcome:Project results are expected to contribute to all of the following outcomes:Existing evidence on maladaptation is retrieved comprehensively, and new knowledge is generated for incorporation into main EU repositories, such as Climate-ADAPT or the portal of the EU Mission on Adaptation to Climate Change;The risk and adaptation assessment frameworks are improved by better integrating the maladaptation dimension;Guidelines and tools for maladaptation prevention and correction strategies are made available to adaptation stakeholders at relevant scales and inform the design and impl</t>
+          <t>Expected Outcome:Project results are expected to contribute to all of the following expected outcomes:Improved understanding of past and present extreme events in the context of climate change in Europe and globally, as well as the interaction between different hazards, their cumulative and/or cascading effects.Enhanced seamless prediction and projection modelling and attribution capabilities for extreme events and their likelihood to support preparedness, response and resilience to climate change by EU and national and regional actors. The EU Union Preparedness Strategy, the EU Adaptation Str</t>
         </is>
       </c>
       <c r="C416" s="22" t="n"/>
@@ -11531,7 +11907,7 @@
       </c>
       <c r="B419" s="23" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-10</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-CL5-2027-01-D1-07</t>
         </is>
       </c>
       <c r="C419" s="22" t="n"/>
@@ -18822,7 +19198,7 @@
     <row r="931" ht="30" customHeight="1">
       <c r="A931" s="18" t="inlineStr">
         <is>
-          <t>FICHA 63: BDNS-904604</t>
+          <t>FICHA 63: BDNS-905090</t>
         </is>
       </c>
       <c r="B931" s="19" t="n"/>
@@ -18847,7 +19223,7 @@
       <c r="E932" s="22" t="n"/>
       <c r="F932" s="22" t="n"/>
     </row>
-    <row r="933" ht="45" customHeight="1">
+    <row r="933" ht="20" customHeight="1">
       <c r="A933" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -18855,7 +19231,7 @@
       </c>
       <c r="B933" s="21" t="inlineStr">
         <is>
-          <t>CONVENIO DE SUBVENCIÓN NOMINATIVA ENTRE EL AYUNTAMIENTO DE VITORIA-GASTEIZ Y LA ASOCIACIÓN DE REINSERCIÓN SOCIAL SARTU- ÁLAVA PARA EL DESARROLLO DEL PROYECTO SAREGUNE 2026, PARA LA REVITALIZACIÓN E IN</t>
+          <t>Ayudas dirigidas al desarrollo de proyectos de descarbonización 2026</t>
         </is>
       </c>
       <c r="C933" s="22" t="n"/>
@@ -18871,7 +19247,7 @@
       </c>
       <c r="B934" s="21" t="inlineStr">
         <is>
-          <t>BDNS-904604</t>
+          <t>BDNS-905090</t>
         </is>
       </c>
       <c r="C934" s="22" t="n"/>
@@ -18919,7 +19295,7 @@
       </c>
       <c r="B937" s="21" t="inlineStr">
         <is>
-          <t>31/12/2026</t>
+          <t>18/09/2026</t>
         </is>
       </c>
       <c r="C937" s="22" t="n"/>
@@ -18935,7 +19311,7 @@
       </c>
       <c r="B938" s="21" t="inlineStr">
         <is>
-          <t>66,000.00 EUR</t>
+          <t>600,000.00 EUR</t>
         </is>
       </c>
       <c r="C938" s="22" t="n"/>
@@ -18967,7 +19343,7 @@
       </c>
       <c r="B940" s="21" t="inlineStr">
         <is>
-          <t>BDNS 904604</t>
+          <t>BDNS 905090</t>
         </is>
       </c>
       <c r="C940" s="22" t="n"/>
@@ -19009,9 +19385,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B943" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MUY ALTA — </t>
+      <c r="B943" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MEDIA — </t>
         </is>
       </c>
       <c r="C943" s="22" t="n"/>
@@ -19027,7 +19403,7 @@
       </c>
       <c r="B944" s="23" t="inlineStr">
         <is>
-          <t>https://www.infosubvenciones.es/bdnstrans/GE/es/convocatoria/904604</t>
+          <t>https://www.infosubvenciones.es/bdnstrans/GE/es/convocatoria/905090</t>
         </is>
       </c>
       <c r="C944" s="22" t="n"/>
@@ -19038,7 +19414,7 @@
     <row r="946" ht="30" customHeight="1">
       <c r="A946" s="18" t="inlineStr">
         <is>
-          <t>FICHA 64: BDNS-904545</t>
+          <t>FICHA 64: EUS-60487</t>
         </is>
       </c>
       <c r="B946" s="19" t="n"/>
@@ -19055,7 +19431,7 @@
       </c>
       <c r="B947" s="21" t="inlineStr">
         <is>
-          <t>🇪🇸 España</t>
+          <t>🟢 Euskadi</t>
         </is>
       </c>
       <c r="C947" s="22" t="n"/>
@@ -19071,7 +19447,7 @@
       </c>
       <c r="B948" s="21" t="inlineStr">
         <is>
-          <t>CONVENIO DE SUBVENCIÓN NOMINATIVA ENTRE EL AYUNTAMIENTO DE VITORIA-GASTEIZ Y LA FUNDACIÓN CATEDRAL DE SANTA MARÍA. PROGRAMA DE VISITAS GUIADAS A LA MURALLA MEDIEVAL AÑO 2026</t>
+          <t xml:space="preserve">I+D, Horizon: evento informativo sobre la financiación en cascada o fórmula usada por el programa marco de innovación de la UE Horizon para dar inclusividad a pymes en grandes consorcios tecnológicos </t>
         </is>
       </c>
       <c r="C948" s="22" t="n"/>
@@ -19087,7 +19463,7 @@
       </c>
       <c r="B949" s="21" t="inlineStr">
         <is>
-          <t>BDNS-904545</t>
+          <t>EUS-60487</t>
         </is>
       </c>
       <c r="C949" s="22" t="n"/>
@@ -19103,7 +19479,7 @@
       </c>
       <c r="B950" s="21" t="inlineStr">
         <is>
-          <t>VITORIA-GASTEIZ</t>
+          <t>Euskadi</t>
         </is>
       </c>
       <c r="C950" s="22" t="n"/>
@@ -19133,11 +19509,7 @@
           <t>Deadline</t>
         </is>
       </c>
-      <c r="B952" s="21" t="inlineStr">
-        <is>
-          <t>31/12/2026</t>
-        </is>
-      </c>
+      <c r="B952" s="21" t="inlineStr"/>
       <c r="C952" s="22" t="n"/>
       <c r="D952" s="22" t="n"/>
       <c r="E952" s="22" t="n"/>
@@ -19151,7 +19523,7 @@
       </c>
       <c r="B953" s="21" t="inlineStr">
         <is>
-          <t>32,000.00 EUR</t>
+          <t>No disponible</t>
         </is>
       </c>
       <c r="C953" s="22" t="n"/>
@@ -19167,7 +19539,7 @@
       </c>
       <c r="B954" s="21" t="inlineStr">
         <is>
-          <t>Subvencion Nacional</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C954" s="22" t="n"/>
@@ -19181,17 +19553,13 @@
           <t>Call ID</t>
         </is>
       </c>
-      <c r="B955" s="21" t="inlineStr">
-        <is>
-          <t>BDNS 904545</t>
-        </is>
-      </c>
+      <c r="B955" s="21" t="inlineStr"/>
       <c r="C955" s="22" t="n"/>
       <c r="D955" s="22" t="n"/>
       <c r="E955" s="22" t="n"/>
       <c r="F955" s="22" t="n"/>
     </row>
-    <row r="956" ht="45" customHeight="1">
+    <row r="956" ht="20" customHeight="1">
       <c r="A956" s="20" t="inlineStr">
         <is>
           <t>Descripcion</t>
@@ -19199,7 +19567,7 @@
       </c>
       <c r="B956" s="21" t="inlineStr">
         <is>
-          <t>PERSONAS JURÍDICAS QUE NO DESARROLLAN ACTIVIDAD ECONÓMICA. . Regiones: ES211 - Araba/Álava</t>
+          <t>Gobierno Vasco / Sector Publico Euskadi</t>
         </is>
       </c>
       <c r="C956" s="22" t="n"/>
@@ -19213,7 +19581,11 @@
           <t>Tags</t>
         </is>
       </c>
-      <c r="B957" s="21" t="inlineStr"/>
+      <c r="B957" s="21" t="inlineStr">
+        <is>
+          <t>energia</t>
+        </is>
+      </c>
       <c r="C957" s="22" t="n"/>
       <c r="D957" s="22" t="n"/>
       <c r="E957" s="22" t="n"/>
@@ -19225,9 +19597,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B958" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MUY ALTA — </t>
+      <c r="B958" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALTA — </t>
         </is>
       </c>
       <c r="C958" s="22" t="n"/>
@@ -19235,7 +19607,7 @@
       <c r="E958" s="22" t="n"/>
       <c r="F958" s="22" t="n"/>
     </row>
-    <row r="959" ht="20" customHeight="1">
+    <row r="959" ht="45" customHeight="1">
       <c r="A959" s="20" t="inlineStr">
         <is>
           <t>Enlace al portal</t>
@@ -19243,7 +19615,7 @@
       </c>
       <c r="B959" s="23" t="inlineStr">
         <is>
-          <t>https://www.infosubvenciones.es/bdnstrans/GE/es/convocatoria/904545</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260512horizonekitaldiinfo/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C959" s="22" t="n"/>
@@ -19254,7 +19626,7 @@
     <row r="961" ht="30" customHeight="1">
       <c r="A961" s="18" t="inlineStr">
         <is>
-          <t>FICHA 65: EUS-85014</t>
+          <t>FICHA 65: EUS-76876</t>
         </is>
       </c>
       <c r="B961" s="19" t="n"/>
@@ -19287,7 +19659,7 @@
       </c>
       <c r="B963" s="21" t="inlineStr">
         <is>
-          <t>Contrato Reservado a Centros Especiales de Empleo, de conformidad con la Disposición Adicional Cuarta de la Ley 9/2017, de 8 de noviembre, de Contratos del Sector Público, para la prestación del servi</t>
+          <t>BANCO DE HIDRÓGENO Y FONDO DE INNOVACIÓN: son parte de los instrumentos mediante los que la UE ha adjudicado nuevas ayudas a proyectos de I+D y producción ecológica de este combustible renovable, impl</t>
         </is>
       </c>
       <c r="C963" s="22" t="n"/>
@@ -19303,7 +19675,7 @@
       </c>
       <c r="B964" s="21" t="inlineStr">
         <is>
-          <t>EUS-85014</t>
+          <t>EUS-76876</t>
         </is>
       </c>
       <c r="C964" s="22" t="n"/>
@@ -19379,7 +19751,7 @@
       </c>
       <c r="B969" s="21" t="inlineStr">
         <is>
-          <t>Licitacion Euskadi</t>
+          <t>Ayuda/Subvencion Euskadi</t>
         </is>
       </c>
       <c r="C969" s="22" t="n"/>
@@ -19437,9 +19809,9 @@
           <t>Relevancia Bilbao</t>
         </is>
       </c>
-      <c r="B973" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MUY ALTA — </t>
+      <c r="B973" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ALTA — </t>
         </is>
       </c>
       <c r="C973" s="22" t="n"/>
@@ -19455,7 +19827,7 @@
       </c>
       <c r="B974" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/anuncio_contratacion/contrato-reservado-centros-especiales-empleo-conformidad-disposicion-adicional-cuarta-ley-9-2017-8-noviembre-contratos-del-sector-publico-prestacion-del-servicio-limpieza-viaria-del-municipio-igorre/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260508cineahidrogenoatafuntsa/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C974" s="22" t="n"/>
@@ -19466,7 +19838,7 @@
     <row r="976" ht="30" customHeight="1">
       <c r="A976" s="18" t="inlineStr">
         <is>
-          <t>FICHA 66: EUS-26962</t>
+          <t>FICHA 66: EUS-34926</t>
         </is>
       </c>
       <c r="B976" s="19" t="n"/>
@@ -19499,7 +19871,7 @@
       </c>
       <c r="B978" s="21" t="inlineStr">
         <is>
-          <t>BANCO DE HIDRÓGENO Y FONDO DE INNOVACIÓN: son parte de los instrumentos mediante los que la UE ha adjudicado nuevas ayudas a proyectos de I+D y producción ecológica de este combustible renovable, impl</t>
+          <t>NEB, Nueva Bauhaus Europea. Convocatoria para barrios estéticos, inclusivos, sostenibles y con vivienda asequible, con financiación del marco Horizon de I+D y otros programas. Áreas de ecología-inclus</t>
         </is>
       </c>
       <c r="C978" s="22" t="n"/>
@@ -19515,7 +19887,7 @@
       </c>
       <c r="B979" s="21" t="inlineStr">
         <is>
-          <t>EUS-26962</t>
+          <t>EUS-34926</t>
         </is>
       </c>
       <c r="C979" s="22" t="n"/>
@@ -19667,7 +20039,7 @@
       </c>
       <c r="B989" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260508cineahidrogenoatafuntsa/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/2605nebauzoetarako3lerroe/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C989" s="22" t="n"/>
@@ -19678,7 +20050,7 @@
     <row r="991" ht="30" customHeight="1">
       <c r="A991" s="18" t="inlineStr">
         <is>
-          <t>FICHA 67: EUS-99909</t>
+          <t>FICHA 67: EUS-71324</t>
         </is>
       </c>
       <c r="B991" s="19" t="n"/>
@@ -19711,7 +20083,7 @@
       </c>
       <c r="B993" s="21" t="inlineStr">
         <is>
-          <t>NEB, Nueva Bauhaus Europea. Convocatoria para barrios estéticos, inclusivos, sostenibles y con vivienda asequible, con financiación del marco Horizon de I+D y otros programas. Áreas de ecología-inclus</t>
+          <t>Elige Europa para la Ciencia: primeras 16 carreras apoyadas con la fórmula innovadora de financiar a las universidades de residencia. Inteligencia artificial, biomedicina, robótica, genómica, clima, e</t>
         </is>
       </c>
       <c r="C993" s="22" t="n"/>
@@ -19727,7 +20099,7 @@
       </c>
       <c r="B994" s="21" t="inlineStr">
         <is>
-          <t>EUS-99909</t>
+          <t>EUS-71324</t>
         </is>
       </c>
       <c r="C994" s="22" t="n"/>
@@ -19879,7 +20251,7 @@
       </c>
       <c r="B1004" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/2605nebauzoetarako3lerroe/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260506aukeratueuropazient/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1004" s="22" t="n"/>
@@ -19890,7 +20262,7 @@
     <row r="1006" ht="30" customHeight="1">
       <c r="A1006" s="18" t="inlineStr">
         <is>
-          <t>FICHA 68: EUS-02372</t>
+          <t>FICHA 68: EUS-25492</t>
         </is>
       </c>
       <c r="B1006" s="19" t="n"/>
@@ -19923,7 +20295,7 @@
       </c>
       <c r="B1008" s="21" t="inlineStr">
         <is>
-          <t>Elige Europa para la Ciencia: primeras 16 carreras apoyadas con la fórmula innovadora de financiar a las universidades de residencia. Inteligencia artificial, biomedicina, robótica, genómica, clima, e</t>
+          <t>LIFE 2026. Medio ambiente. Ayudas de 4 subprogramas, de naturaleza y biodiversidad, circularidad y calidad de vida, cambio climático y transición energética. Con inscripción abierta para jornadas info</t>
         </is>
       </c>
       <c r="C1008" s="22" t="n"/>
@@ -19939,7 +20311,7 @@
       </c>
       <c r="B1009" s="21" t="inlineStr">
         <is>
-          <t>EUS-02372</t>
+          <t>EUS-25492</t>
         </is>
       </c>
       <c r="C1009" s="22" t="n"/>
@@ -20091,7 +20463,7 @@
       </c>
       <c r="B1019" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260506aukeratueuropazient/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260421life4lerrotajarduna/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1019" s="22" t="n"/>
@@ -20102,7 +20474,7 @@
     <row r="1021" ht="30" customHeight="1">
       <c r="A1021" s="18" t="inlineStr">
         <is>
-          <t>FICHA 69: EUS-59698</t>
+          <t>FICHA 69: EUS-67282</t>
         </is>
       </c>
       <c r="B1021" s="19" t="n"/>
@@ -20127,7 +20499,7 @@
       <c r="E1022" s="22" t="n"/>
       <c r="F1022" s="22" t="n"/>
     </row>
-    <row r="1023" ht="45" customHeight="1">
+    <row r="1023" ht="20" customHeight="1">
       <c r="A1023" s="20" t="inlineStr">
         <is>
           <t>Titulo</t>
@@ -20135,7 +20507,7 @@
       </c>
       <c r="B1023" s="21" t="inlineStr">
         <is>
-          <t>LIFE 2026. Medio ambiente. Ayudas de 4 subprogramas, de naturaleza y biodiversidad, circularidad y calidad de vida, cambio climático y transición energética. Con inscripción abierta para jornadas info</t>
+          <t>Sustitucion de sistemas de climatizacion y ventilación</t>
         </is>
       </c>
       <c r="C1023" s="22" t="n"/>
@@ -20151,7 +20523,7 @@
       </c>
       <c r="B1024" s="21" t="inlineStr">
         <is>
-          <t>EUS-59698</t>
+          <t>EUS-67282</t>
         </is>
       </c>
       <c r="C1024" s="22" t="n"/>
@@ -20227,7 +20599,7 @@
       </c>
       <c r="B1029" s="21" t="inlineStr">
         <is>
-          <t>Ayuda/Subvencion Euskadi</t>
+          <t>Licitacion Euskadi</t>
         </is>
       </c>
       <c r="C1029" s="22" t="n"/>
@@ -20303,7 +20675,7 @@
       </c>
       <c r="B1034" s="23" t="inlineStr">
         <is>
-          <t>https://www.euskadi.eus/ayuda_subvencion/2026/260421life4lerrotajarduna/web01-tramite/es/</t>
+          <t>https://www.euskadi.eus/anuncio_contratacion/sustitucion-sistemas-climatizacion-y-ventilacion/web01-tramite/es/</t>
         </is>
       </c>
       <c r="C1034" s="22" t="n"/>
@@ -20314,7 +20686,7 @@
     <row r="1036" ht="30" customHeight="1">
       <c r="A1036" s="18" t="inlineStr">
         <is>
-          <t>FICHA 70: EUS-09274</t>
+          <t>FICHA 70: EUS-76748</t>
         </is>
       </c>
       <c r="B1036" s="19" t="n"/>
@@ -20363,7 +20735,7 @@
       </c>
       <c r="B1039" s="21" t="inlineStr">
         <is>
-          <t>EUS-09274</t>
+          <t>EUS-76748</t>
         </is>
       </c>
       <c r="C1039" s="22" t="n"/>
@@ -20526,7 +20898,7 @@
     <row r="1051" ht="30" customHeight="1">
       <c r="A1051" s="18" t="inlineStr">
         <is>
-          <t>FICHA 71: EUS-77428</t>
+          <t>FICHA 71: EUS-72997</t>
         </is>
       </c>
       <c r="B1051" s="19" t="n"/>
@@ -20575,7 +20947,7 @@
       </c>
       <c r="B1054" s="21" t="inlineStr">
         <is>
-          <t>EUS-77428</t>
+          <t>EUS-72997</t>
         </is>
       </c>
       <c r="C1054" s="22" t="n"/>
@@ -20738,7 +21110,7 @@
     <row r="1066" ht="30" customHeight="1">
       <c r="A1066" s="18" t="inlineStr">
         <is>
-          <t>FICHA 72: EUS-23728</t>
+          <t>FICHA 72: EUS-73348</t>
         </is>
       </c>
       <c r="B1066" s="19" t="n"/>
@@ -20787,7 +21159,7 @@
       </c>
       <c r="B1069" s="21" t="inlineStr">
         <is>
-          <t>EUS-23728</t>
+          <t>EUS-73348</t>
         </is>
       </c>
       <c r="C1069" s="22" t="n"/>
@@ -20950,7 +21322,7 @@
     <row r="10